<commit_message>
Agregar 6 proyectos nuevos y 8 cambios de fase (2026-07-23)
- LNG (1 nuevo): Sabine Pass LNG Expansion (Train 7 + reliquefacción)
- Mining (2 nuevos): South West Arkansas Lithium Project (Smackover Lithium), Bagdad Mine Concentrator Expansion (Freeport-McMoRan)
- Data Centers (2 nuevos): PowerPlay AI "Greater Abilene", Liberty Energy/PowerBridge "Alpha Digital Campus"

Cambios de fase: Saguaro Energía LNG (pausado por orden judicial), Corpus Christi Stage 3 (FERC autoriza Train 7), Texas LNG Brownsville (inversión HPS/BlackRock), El Pilar Copper Project (permisos asegurados, US$551M), Hermosa Critical Minerals (ROD final USFS), Project Jupiter (audiencia NMED oct-2026).

Se regenera proyectos.xlsx (una hoja por industria) con el acumulado completo.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YLKArezdQJfAqyTik1hNM8
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -20,10 +20,18 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
@@ -49,8 +57,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -419,47 +428,47 @@
   <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -493,7 +502,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>[Fluor newsroom](https://newsroom.fluor.com/news-releases/news-details/2026/Fluor-Awarded-Contract-to-Engineer-and-Design-the-America-First-Refining-Facility-in-Brownsville-Texas/default.aspx)</t>
+          <t>https://newsroom.fluor.com/news-releases/news-details/2026/Fluor-Awarded-Contract-to-Engineer-and-Design-the-America-First-Refining-Facility-in-Brownsville-Texas/default.aspx</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -530,7 +539,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>[AllStream Insiders](https://allstreaminsiders.com/us-exxonmobil-may-build-cracker-pe-plant-in-texas-with-an-8-6-billion-investment/)</t>
+          <t>https://allstreaminsiders.com/us-exxonmobil-may-build-cracker-pe-plant-in-texas-with-an-8-6-billion-investment/</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -567,7 +576,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>[BIC Magazine](https://www.bicmagazine.com/departments/operations/cpchem-golden-triangle-polymers-facility-startup-phase/)</t>
+          <t>https://www.bicmagazine.com/departments/operations/cpchem-golden-triangle-polymers-facility-startup-phase/</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -604,7 +613,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>[Construction Front](https://constructionfront.com/2025-04-13-technip-energies-to-deliver-blue-point-worlds-largest-low-carbon-ammonia-facility-in-louisiana/)</t>
+          <t>https://constructionfront.com/2025-04-13-technip-energies-to-deliver-blue-point-worlds-largest-low-carbon-ammonia-facility-in-louisiana/</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -641,7 +650,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>[East Daley](https://eastdaley.com/media-and-news/the-race-is-on-to-build-permian-processing)</t>
+          <t>https://eastdaley.com/media-and-news/the-race-is-on-to-build-permian-processing</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -678,7 +687,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>[Techint](https://www.techint.com/en/our-projects/dos-bocas-refinery)</t>
+          <t>https://www.techint.com/en/our-projects/dos-bocas-refinery</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -715,7 +724,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>[OGJ](https://www.ogj.com/refining-processing/refining/optimization/article/17279334/pemex-to-proceed-with-dos-bocas-refinery-project)</t>
+          <t>https://www.ogj.com/refining-processing/refining/optimization/article/17279334/pemex-to-proceed-with-dos-bocas-refinery-project</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -752,7 +761,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>[Forbes México](https://forbes.com.mx/pemex-invertira-5300-millones-de-dolares-para-reactivar-la-industria-petroquimica/)</t>
+          <t>https://forbes.com.mx/pemex-invertira-5300-millones-de-dolares-para-reactivar-la-industria-petroquimica/</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -789,7 +798,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>[Forbes México](https://forbes.com.mx/pemex-invertira-5300-millones-de-dolares-para-reactivar-la-industria-petroquimica/)</t>
+          <t>https://forbes.com.mx/pemex-invertira-5300-millones-de-dolares-para-reactivar-la-industria-petroquimica/</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -826,7 +835,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>[Forbes México](https://forbes.com.mx/asi-es-la-inversion-de-1553-mdd-por-parte-de-pemex-en-una-planta-de-fertilizantes-en-veracruz/)</t>
+          <t>https://forbes.com.mx/asi-es-la-inversion-de-1553-mdd-por-parte-de-pemex-en-una-planta-de-fertilizantes-en-veracruz/</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -863,7 +872,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>[Tribuna](https://tribuna.com.mx/mexico/2026/06/05/sheinbaum-anuncia-inversion-de-93-mil-mdp-para-reactivar-la-industria-petroquimica-y-de-fertilizantes-en-veracruz_560837/)</t>
+          <t>https://tribuna.com.mx/mexico/2026/06/05/sheinbaum-anuncia-inversion-de-93-mil-mdp-para-reactivar-la-industria-petroquimica-y-de-fertilizantes-en-veracruz_560837/</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -900,7 +909,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>[PV Magazine México](https://www.pv-magazine-mexico.com/2026/04/28/inician-en-sinaloa-la-construccion-de-la-mayor-planta-de-metanol-ultrabajo-en-carbono-a-partir-de-hidrogeno-verde/)</t>
+          <t>https://www.pv-magazine-mexico.com/2026/04/28/inician-en-sinaloa-la-construccion-de-la-mayor-planta-de-metanol-ultrabajo-en-carbono-a-partir-de-hidrogeno-verde/</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -937,7 +946,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>[H2 View](https://www.h2-view.com/story/first-ammonia-project-on-track-for-2026-fid-despite-topsoe-deal-collapse/2138792.article/)</t>
+          <t>https://www.h2-view.com/story/first-ammonia-project-on-track-for-2026-fid-despite-topsoe-deal-collapse/2138792.article/</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -974,7 +983,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>[Debate](https://www.debate.com.mx/economia/secretaria-de-economia-complejo-de-amoniaco-en-topolobampo-prioritario-para-el-gobierno-de-mexico-20260713-0092.html)</t>
+          <t>https://www.debate.com.mx/economia/secretaria-de-economia-complejo-de-amoniaco-en-topolobampo-prioritario-para-el-gobierno-de-mexico-20260713-0092.html</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1011,7 +1020,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>[ICIS](https://www.icis.com/explore/resources/news/2025/11/13/11155109/lake-charles-methanol-ii-awards-feed-fid-expected-in-q2-2026/)</t>
+          <t>https://www.icis.com/explore/resources/news/2025/11/13/11155109/lake-charles-methanol-ii-awards-feed-fid-expected-in-q2-2026/</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1048,7 +1057,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>[Diario del Istmo](https://diariodelistmo.com/nacional/este-es-el-avance-que-lleva-la-planta-coquizadora-en-la-refineria-de-salina-cruz/50642321)</t>
+          <t>https://diariodelistmo.com/nacional/este-es-el-avance-que-lleva-la-planta-coquizadora-en-la-refineria-de-salina-cruz/50642321</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1085,7 +1094,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/petrochemicals/06032026/shintech-announces-us34-billion-at-louisiana-petrochemicals-complex/)</t>
+          <t>https://www.hydrocarbonengineering.com/petrochemicals/06032026/shintech-announces-us34-billion-at-louisiana-petrochemicals-complex/</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1122,7 +1131,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>[Alchempro](https://www.alchempro.com/news/chemicals-news/ineos-backs-1-7-bn-low-carbon-methanol-project-in-texas-city-310108-newsdetails.htm)</t>
+          <t>https://www.alchempro.com/news/chemicals-news/ineos-backs-1-7-bn-low-carbon-methanol-project-in-texas-city-310108-newsdetails.htm</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1159,7 +1168,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/petrochemicals/13072026/oxea-confirms-fid-for-major-capacity-expansion/)</t>
+          <t>https://www.hydrocarbonengineering.com/petrochemicals/13072026/oxea-confirms-fid-for-major-capacity-expansion/</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1196,7 +1205,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>[OGJ](https://www.ogj.com/refining-processing/gas-processing/news/55320579/targa-advances-permian-gas-pipeline-processing-expansion)</t>
+          <t>https://www.ogj.com/refining-processing/gas-processing/news/55320579/targa-advances-permian-gas-pipeline-processing-expansion</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1233,7 +1242,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>[Business Wire](https://www.businesswire.com/news/home/20250806663187/en/Enterprise-Agrees-to-Acquire-Occidentals-Gas-Gathering-Affiliate-Enters-Into-Natural-Gas-Processing-Agreement-Announces-New-Midland-Basin-Natural-Gas-Processing-Plant)</t>
+          <t>https://www.businesswire.com/news/home/20250806663187/en/Enterprise-Agrees-to-Acquire-Occidentals-Gas-Gathering-Affiliate-Enters-Into-Natural-Gas-Processing-Agreement-Announces-New-Midland-Basin-Natural-Gas-Processing-Plant</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1270,7 +1279,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>[Natural Gas Intel](https://naturalgasintel.com/news/mplx-scales-up-for-power-hungry-future-with-natural-gas-focused-growth-plan/)</t>
+          <t>https://naturalgasintel.com/news/mplx-scales-up-for-power-hungry-future-with-natural-gas-focused-growth-plan/</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1307,7 +1316,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>[East Daley](https://eastdaley.com/daley-note/mplx-acquires-northwind-for-2-375b-acquires-more-ngls-for-jv-project)</t>
+          <t>https://eastdaley.com/daley-note/mplx-acquires-northwind-for-2-375b-acquires-more-ngls-for-jv-project</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1344,7 +1353,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>[Grand Forks Herald](https://www.grandforksherald.com/news/local/northern-plains-nitrogen-proposal-receiving-more-attention-amid-global-fertilizer-pressure)</t>
+          <t>https://www.grandforksherald.com/news/local/northern-plains-nitrogen-proposal-receiving-more-attention-amid-global-fertilizer-pressure</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1381,7 +1390,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>[Phillips 66](https://www.phillips66.com/newsroom/iron-mesa-safely-enters-next-phase-of-construction/)</t>
+          <t>https://www.phillips66.com/newsroom/iron-mesa-safely-enters-next-phase-of-construction/</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1418,7 +1427,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>[Targa Resources](https://www.targaresources.com/news-releases/news-release-details/targa-resources-corp-announces-permian-growth-projects-and)</t>
+          <t>https://www.targaresources.com/news-releases/news-release-details/targa-resources-corp-announces-permian-growth-projects-and</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1455,7 +1464,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>[Elefante Blanco](https://elefanteblanco.mx/2026/01/02/pemex-abre-30-licitaciones-para-obras-en-la-refineria-madero/)</t>
+          <t>https://elefanteblanco.mx/2026/01/02/pemex-abre-30-licitaciones-para-obras-en-la-refineria-madero/</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1492,7 +1501,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>[La Jornada](https://www.jornada.com.mx/noticia/2026/06/08/economia/da-inicio-ejecucion-de-planta-de-fertilizantes-en-durango-por-parte-de-fermachem)</t>
+          <t>https://www.jornada.com.mx/noticia/2026/06/08/economia/da-inicio-ejecucion-de-planta-de-fertilizantes-en-durango-por-parte-de-fermachem</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1529,7 +1538,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>[Downstream Calendar](https://downstreamcalendar.com/mcdermott-secures-feed-contract-for-ascension-clean-energy-project/)</t>
+          <t>https://downstreamcalendar.com/mcdermott-secures-feed-contract-for-ascension-clean-energy-project/</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1566,7 +1575,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>[Business Wire](https://www.businesswire.com/news/home/20260517310811/en/Phillips-66-announces-Zeus-Gas-Plant-and-a-third-Coastal-Bend-Fractionator)</t>
+          <t>https://www.businesswire.com/news/home/20260517310811/en/Phillips-66-announces-Zeus-Gas-Plant-and-a-third-Coastal-Bend-Fractionator</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1603,7 +1612,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>[USDA](https://www.usda.gov/about-usda/news/press-releases/2026/07/01/secretary-rollins-announces-500-million-fertilizer-investment-and-expansion-program-strengthen)</t>
+          <t>https://www.usda.gov/about-usda/news/press-releases/2026/07/01/secretary-rollins-announces-500-million-fertilizer-investment-and-expansion-program-strengthen</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1623,50 +1632,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -1700,7 +1709,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>[Bechtel](https://www.bechtel.com/press-releases/nextdecade-executes-epc-contract-with-bechtel-for-train-4-at-the-rio-grande-lng-facility/)</t>
+          <t>https://www.bechtel.com/press-releases/nextdecade-executes-epc-contract-with-bechtel-for-train-4-at-the-rio-grande-lng-facility/</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -1737,7 +1746,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>[Bechtel](https://www.bechtel.com/press-releases/sempra-infrastructure-announces-epc-contract-with-bechtel-for-port-arthur-lng-phase-2/)</t>
+          <t>https://www.bechtel.com/press-releases/sempra-infrastructure-announces-epc-contract-with-bechtel-for-port-arthur-lng-phase-2/</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -1774,7 +1783,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>[Woodside](https://www.woodside.com/what-we-do/growth-projects/woodside-louisiana-lng)</t>
+          <t>https://www.woodside.com/what-we-do/growth-projects/woodside-louisiana-lng</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -1811,7 +1820,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>[GEM.wiki](https://www.gem.wiki/CP2_LNG_Terminal)</t>
+          <t>https://www.gem.wiki/CP2_LNG_Terminal</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -1848,7 +1857,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>[Offshore Energy](https://www.offshore-energy.biz/kbr-zachry-to-work-on-ventures-plaquemines-lng/)</t>
+          <t>https://www.offshore-energy.biz/kbr-zachry-to-work-on-ventures-plaquemines-lng/</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -1885,7 +1894,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>[LNG Prime](https://lngprime.com/contracts-and-tenders/golden-pass-lng-contractors-ink-revised-epc-deal-for-second-and-third-train/169104/)</t>
+          <t>https://lngprime.com/contracts-and-tenders/golden-pass-lng-contractors-ink-revised-epc-deal-for-second-and-third-train/169104/</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1917,17 +1926,17 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Construcción (98%)</t>
+          <t>Construcción (FERC autorizó introducción de gas combustible en Train 7, 17-jul-2026; primera producción de LNG esperada ago-2026, servicio comercial sep-2026)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>[LNG Prime](https://lngprime.com/americas/chenieres-corpus-christi-stage-3-project-98-percent-complete/190871/)</t>
+          <t>https://pgjonline.com/news/2026/july/corpus-christi-lng-train-7-cleared-to-introduce-fuel-gas-by-ferc</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-23</t>
         </is>
       </c>
     </row>
@@ -1959,7 +1968,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/06/03/3306350/0/en/delfin-midstream-announces-5-billion-final-investment-decision-for-first-flng-vessel.html)</t>
+          <t>https://www.globenewswire.com/news-release/2026/06/03/3306350/0/en/delfin-midstream-announces-5-billion-final-investment-decision-for-first-flng-vessel.html</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1991,17 +2000,17 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Ingeniería/Pre-FID con retrasos</t>
+          <t>Pre-FID PAUSADO (suspensión judicial desde abr-2026 por demanda ambiental sobre ballenas en el Mar de Cortés; presión de activistas contra financiadores JPMorgan/Santander, 17-jul-2026; definición de autorización pendiente para 2026)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>[IEEFA](https://ieefa.org/resources/mexico-pacific-limited-delays-turmoil-and-permitting-errors-have-stymied-mexicos-largest)</t>
+          <t>https://dossierpolitico.com/2026/07/17/activistas-entregan-90-mil-firmas-para-frenar-proyecto-saguaro-energia-en-sonora/</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-23</t>
         </is>
       </c>
     </row>
@@ -2033,7 +2042,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>[GEM Wiki](https://www.gem.wiki/New_Fortress_Altamira_FLNG_Terminal)</t>
+          <t>https://www.gem.wiki/New_Fortress_Altamira_FLNG_Terminal</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -2065,17 +2074,17 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Construcción (LNTP otorgado a Kiewit 4-jul-2026 para compra de equipo de entrega larga, ingeniería EPC y geotécnico; FID prevista fin de 2026)</t>
+          <t>Construcción (LNTP otorgado a Kiewit 4-jul-2026; HPS Investment Partners/BlackRock invirtió US$500M para obras tempranas, visto como paso final previo a FID; FID prevista fin de 2026)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>[OGJ](https://www.ogj.com/pipelines-transportation/lng/news/55388908/texas-lng-advances-pre-fid-project-with-limited-notice-to-proceed)</t>
+          <t>https://www.naturalgasintel.com/news/glenfarne-lands-investment-for-early-work-on-texas-lng-ahead-of-fid/</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-23</t>
         </is>
       </c>
     </row>
@@ -2107,7 +2116,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>[PGJ](https://pgjonline.com/news/2026/july/commonwealth-lng-awards-main-automation-contract-for-louisiana-export-terminal)</t>
+          <t>https://pgjonline.com/news/2026/july/commonwealth-lng-awards-main-automation-contract-for-louisiana-export-terminal</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -2144,7 +2153,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>[Houston Public Media](https://www.houstonpublicmedia.org/articles/galveston-county/2026/07/14/557086/galveston-pelican-island-lng/)</t>
+          <t>https://www.houstonpublicmedia.org/articles/galveston-county/2026/07/14/557086/galveston-pelican-island-lng/</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -2181,7 +2190,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>[Sempra](https://www.sempra.com/newsroom/press-releases/sempra-infrastructures-eca-lng-phase-1-exports-first-lng-cargo-mexicos)</t>
+          <t>https://www.sempra.com/newsroom/press-releases/sempra-infrastructures-eca-lng-phase-1-exports-first-lng-cargo-mexicos</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -2218,7 +2227,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>[LNG Prime](https://lngprime.com/americas/gato-negro-eyes-fid-on-mexico-lng-plant-in-late-2026/165906/)</t>
+          <t>https://lngprime.com/americas/gato-negro-eyes-fid-on-mexico-lng-plant-in-late-2026/165906/</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -2255,7 +2264,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/amigo-lng-awards-landmark-epc-contract-to-dubai-based-drydocks-world-for-worlds-largest-flng-facility-302537739.html)</t>
+          <t>https://www.prnewswire.com/news-releases/amigo-lng-awards-landmark-epc-contract-to-dubai-based-drydocks-world-for-worlds-largest-flng-facility-302537739.html</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -2292,7 +2301,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>[KBR](https://www.kbr.com/en/insights-news/press-release/kbr-awarded-feed-coastal-bend-lng-project)</t>
+          <t>https://www.kbr.com/en/insights-news/press-release/kbr-awarded-feed-coastal-bend-lng-project</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2329,7 +2338,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>[FERC](https://www.ferc.gov/gulfstream-lng-terminal-project)</t>
+          <t>https://www.ferc.gov/gulfstream-lng-terminal-project</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2366,7 +2375,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>[Glenfarne](https://glenfarnegroup.com/glenfarne-announces-major-phase-one-alaska-lng-milestones-with-construction-line-pipe-supply-and-in-state-gas-agreements/)</t>
+          <t>https://glenfarnegroup.com/glenfarne-announces-major-phase-one-alaska-lng-milestones-with-construction-line-pipe-supply-and-in-state-gas-agreements/</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2403,7 +2412,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>[PGJ](https://pgjonline.com/news/2026/july/311-mile-sonora-gas-pipeline-project-advances-in-mexico)</t>
+          <t>https://pgjonline.com/news/2026/july/311-mile-sonora-gas-pipeline-project-advances-in-mexico</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2440,7 +2449,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>[OGJ](https://www.ogj.com/pipelines-transportation/pipelines/news/55322537/arm-energy-takes-fid-on-23-billion-mustang-express-pipeline)</t>
+          <t>https://www.ogj.com/pipelines-transportation/pipelines/news/55322537/arm-energy-takes-fid-on-23-billion-mustang-express-pipeline</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2477,7 +2486,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>[Mexico Business News](https://mexicobusiness.news/energy/news/ursus-energy-scales-investment-us21-billion)</t>
+          <t>https://mexicobusiness.news/energy/news/ursus-energy-scales-investment-us21-billion</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2514,7 +2523,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/15/3327983/0/en/Delfin-Midstream-Partners-With-EIG-s-MidOcean-Energy-to-Advance-Second-FLNG-Vessel-Issues-Limited-Notice-to-Proceed-to-Siemens-Energy.html)</t>
+          <t>https://www.globenewswire.com/news-release/2026/07/15/3327983/0/en/Delfin-Midstream-Partners-With-EIG-s-MidOcean-Energy-to-Advance-Second-FLNG-Vessel-Issues-Limited-Notice-to-Proceed-to-Siemens-Energy.html</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2551,7 +2560,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>[Natural Gas Intel](https://www.naturalgasintel.com/news/texas-gateway-open-season-expands-haynesville-natural-gas-links-amid-lng-growth/)</t>
+          <t>https://www.naturalgasintel.com/news/texas-gateway-open-season-expands-haynesville-natural-gas-links-amid-lng-growth/</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2588,7 +2597,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>[World Oil](https://worldoil.com/news/2026/7/6/argent-lng-awards-engineering-contract-for-port-fourchon-lng-project/)</t>
+          <t>https://worldoil.com/news/2026/7/6/argent-lng-awards-engineering-contract-for-port-fourchon-lng-project/</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2625,7 +2634,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>[Federal Register](https://www.federalregister.gov/documents/2026/04/17/2026-07517/deepwater-port-license-application-st-lng-deepwater-port-development-project-draft-environmental)</t>
+          <t>https://www.federalregister.gov/documents/2026/04/17/2026-07517/deepwater-port-license-application-st-lng-deepwater-port-development-project-draft-environmental</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -2662,7 +2671,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>[Natural Gas Intel](https://naturalgasintel.com/news/kinder-morgan-greenlights-7b-in-natural-gas-pipeline-projects-amid-regulatory-speedup/)</t>
+          <t>https://naturalgasintel.com/news/kinder-morgan-greenlights-7b-in-natural-gas-pipeline-projects-amid-regulatory-speedup/</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -2699,7 +2708,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>[Natural Gas Intel](https://naturalgasintel.com/news/kinder-morgan-greenlights-7b-in-natural-gas-pipeline-projects-amid-regulatory-speedup/)</t>
+          <t>https://naturalgasintel.com/news/kinder-morgan-greenlights-7b-in-natural-gas-pipeline-projects-amid-regulatory-speedup/</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2736,12 +2745,49 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>[LNG Prime](https://lngprime.com/americas/kinder-morgan-seeks-doe-extension-for-gulf-lng-export-project/184334/)</t>
+          <t>https://lngprime.com/americas/kinder-morgan-seeks-doe-extension-for-gulf-lng-export-project/184334/</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
           <t>2026-07-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Sabine Pass LNG Expansion (Train 7 + unidad de re-licuefacción de boil-off gas)</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Cameron Parish, Luisiana, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Cheniere Energy Partners</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Bechtel (EPC); Baker Hughes (equipo mayor)</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Construcción/Procura de equipo mayor (EPC firmado 28-may-2026; Baker Hughes recibió pedido de 7 turbinas de gas PGT25+ G4 y 15 compresores centrífugos, ~6 MTPA adicionales; construcción plena prevista inicios de 2027)</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>https://investors.bakerhughes.com/news/press-releases/news-details/2026/Baker-Hughes-Secures-Substantial-Equipment-and-Services-Awards-for-Chenieres-Sabine-Pass-LNG-Facility/default.aspx</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
         </is>
       </c>
     </row>
@@ -2756,50 +2802,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -2833,7 +2879,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>[Mining Weekly](https://www.miningweekly.com/article/ivanhoe-electric-pencils-in-2026-construction-start-at-arizona-copper-mine-2025-06-25)</t>
+          <t>https://www.miningweekly.com/article/ivanhoe-electric-pencils-in-2026-construction-start-at-arizona-copper-mine-2025-06-25</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -2870,7 +2916,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>[SEC/Hudbay](https://www.sec.gov/Archives/edgar/data/1322422/000106299326001973/exhibit99-2.htm)</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1322422/000106299326001973/exhibit99-2.htm</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -2907,7 +2953,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>[SEC](https://www.sec.gov/Archives/edgar/data/863064/000086306426000019/ex12d16mr_resolutionland.htm)</t>
+          <t>https://www.sec.gov/Archives/edgar/data/863064/000086306426000019/ex12d16mr_resolutionland.htm</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -2944,7 +2990,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>[Nevada Appeal](https://www.nevadaappeal.com/news/2026/mar/26/lithium-americas-900-construction-workers-at-thacker-pass-mine/)</t>
+          <t>https://www.nevadaappeal.com/news/2026/mar/26/lithium-americas-900-construction-workers-at-thacker-pass-mine/</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -2981,7 +3027,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>[Mining.com](https://www.mining.com/teck-agnico-team-up-at-san-nicolas-copper-project-in-mexico/)</t>
+          <t>https://www.mining.com/teck-agnico-team-up-at-san-nicolas-copper-project-in-mexico/</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -3018,7 +3064,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>[Energy Magazine MX](https://energymagazine.mx/2025/10/grupo-mexico-espera-autorizacion-federal-para-continuar-proyectos-mineros-por-10-mil-200-mdd/)</t>
+          <t>https://energymagazine.mx/2025/10/grupo-mexico-espera-autorizacion-federal-para-continuar-proyectos-mineros-por-10-mil-200-mdd/</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -3040,7 +3086,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Grupo México</t>
+          <t>Grupo México / Southern Copper Corporation</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -3050,17 +3096,17 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Ingeniería básica completada / trámite ambiental</t>
+          <t>Permisos ambientales asegurados (proyecto revaluado en US$551 millones; preparación de sitio inicia sep-2026, construcción plena 2027, primer cobre ~2028)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>[Mexico Mining Center](https://www.mexicominingcenter.com/grupo-mexico-compra-mina-el-pilar/)</t>
+          <t>https://www.bnamericas.com/en/news/southern-copper-wins-permits-for-us551mn-el-pilar-in-mexico</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-23</t>
         </is>
       </c>
     </row>
@@ -3092,7 +3138,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>[M3 Engineering](https://m3eng.com/portfolio/buenavista-del-cobre-concentradora-no-2/)</t>
+          <t>https://m3eng.com/portfolio/buenavista-del-cobre-concentradora-no-2/</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -3129,7 +3175,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>[Minería en Línea](https://mineriaenlinea.com/2026/04/torex-gold-alcanza-velocidad-de-crucero-en-media-luna-9-meses-adelante-de-cronograma/)</t>
+          <t>https://mineriaenlinea.com/2026/04/torex-gold-alcanza-velocidad-de-crucero-en-media-luna-9-meses-adelante-de-cronograma/</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -3166,7 +3212,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>[Mining.com](https://www.mining.com/nevada-copper-unveils-restart-and-financing-plan-for-pumpkin-hollow/)</t>
+          <t>https://www.mining.com/nevada-copper-unveils-restart-and-financing-plan-for-pumpkin-hollow/</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -3198,17 +3244,17 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Construcción (Record of Decision final emitido por USFS 14-jul-2026; ~50% avance en porción privada; autorización operativa prevista sep-2026)</t>
+          <t>Construcción (Record of Decision final emitido por USFS 7-jul-2026, cerrando revisión NEPA de infraestructura en Coronado National Forest; primer proyecto minero aceptado en programa federal FAST-41; ~50% avance en porción privada; primer concentrado ahora proyectado H1-2028, antes H1-2027)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>[Chamber Business News](https://chamberbusinessnews.com/2026/07/14/hermosa-critical-minerals-mining-project-reaches-major-federal-permitting-milestone/)</t>
+          <t>https://www.usda.gov/about-usda/news/press-releases/2026/07/07/usda-advances-trump-administration-effort-boost-us-mineral-energy-production</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-23</t>
         </is>
       </c>
     </row>
@@ -3240,7 +3286,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/perpetua-resources-advances-construction-of-the-stibnite-gold-project-302787012.html)</t>
+          <t>https://www.prnewswire.com/news-releases/perpetua-resources-advances-construction-of-the-stibnite-gold-project-302787012.html</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -3277,7 +3323,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>[Silver Tiger Metals](https://silvertigermetals.com/news/2026/silver-tiger-metals-awards-engineering-procurement-and-construction-management-contract-and-provides-construction-update)</t>
+          <t>https://silvertigermetals.com/news/2026/silver-tiger-metals-awards-engineering-procurement-and-construction-management-contract-and-provides-construction-update</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -3314,7 +3360,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/vizsla-silver-awards-epcm-and-mine-design-contracts-for-the-development-of-the-panuco-silver-gold-project-302750621.html)</t>
+          <t>https://www.prnewswire.com/news-releases/vizsla-silver-awards-epcm-and-mine-design-contracts-for-the-development-of-the-panuco-silver-gold-project-302750621.html</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -3351,7 +3397,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>[Orla Mining](https://orlamining.com/news/orla-announces-results-of-updated-feasibility-study-for-south-railroad-project/)</t>
+          <t>https://orlamining.com/news/orla-announces-results-of-updated-feasibility-study-for-south-railroad-project/</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -3388,7 +3434,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>[Mining Weekly](https://www.miningweekly.com/article/minera-alamos-confirms-low-cost-near-term-mining-possible-at-copperstone-in-arizona-2026-05-28)</t>
+          <t>https://www.miningweekly.com/article/minera-alamos-confirms-low-cost-near-term-mining-possible-at-copperstone-in-arizona-2026-05-28</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -3425,7 +3471,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>[Wyoming News](https://www.wyomingnews.com/rawlinstimes/plans-move-forward-for-ck-gold-project-as-developers-target-2026-construction-start/article_b2bb147e-2f92-4ca2-bf86-fcc9983917a7.html)</t>
+          <t>https://www.wyomingnews.com/rawlinstimes/plans-move-forward-for-ck-gold-project-as-developers-target-2026-construction-start/article_b2bb147e-2f92-4ca2-bf86-fcc9983917a7.html</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -3462,7 +3508,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>[First Majestic](https://www.juniorminingnetwork.com/junior-miner-news/press-releases/1082-tsx/ag/206222-first-majestic-receives-construction-permits-for-santo-nino-and-navidad-advances-development-across-the-santa-elena-district.html)</t>
+          <t>https://www.juniorminingnetwork.com/junior-miner-news/press-releases/1082-tsx/ag/206222-first-majestic-receives-construction-permits-for-santo-nino-and-navidad-advances-development-across-the-santa-elena-district.html</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -3499,7 +3545,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>[SEC/Americas Gold and Silver](https://www.sec.gov/Archives/edgar/data/0001286973/000106299326002645/exhibit99-2.htm)</t>
+          <t>https://www.sec.gov/Archives/edgar/data/0001286973/000106299326002645/exhibit99-2.htm</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -3536,7 +3582,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>[Kitco](https://www.kitco.com/news/off-the-wire/2026-06-08/minera-frisco-restarts-two-mexico-mines-plans-new-silver-unit)</t>
+          <t>https://www.kitco.com/news/off-the-wire/2026-06-08/minera-frisco-restarts-two-mexico-mines-plans-new-silver-unit</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -3573,7 +3619,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/trilogy-metals-announces-publication-of-federal-and-state-permitting-schedule-for-arctic-project-establishing-defined-timeline-toward-a-record-of-decision-by-september-2028-302827083.html)</t>
+          <t>https://www.prnewswire.com/news-releases/trilogy-metals-announces-publication-of-federal-and-state-permitting-schedule-for-arctic-project-establishing-defined-timeline-toward-a-record-of-decision-by-september-2028-302827083.html</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -3610,7 +3656,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>[Northern Miner](https://www.northernminer.com/news/gogold-approved-to-build-227m-mine-in-mexico/1003891932/)</t>
+          <t>https://www.northernminer.com/news/gogold-approved-to-build-227m-mine-in-mexico/1003891932/</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -3647,7 +3693,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>[BNamericas](https://www.bnamericas.com/en/news/discovery-advances-permitting-financing-at-us606mn-cordero-in-mexico)</t>
+          <t>https://www.bnamericas.com/en/news/discovery-advances-permitting-financing-at-us606mn-cordero-in-mexico</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -3684,7 +3730,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>[Resource World](https://resourceworld.com/tocvan-ventures-eyes-mexican-gold-pour-by-q4-2026/)</t>
+          <t>https://resourceworld.com/tocvan-ventures-eyes-mexican-gold-pour-by-q4-2026/</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -3721,7 +3767,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>[Fresnillo plc](https://www.fresnilloplc.com/portfolio/exploration/orisyvo/)</t>
+          <t>https://www.fresnilloplc.com/portfolio/exploration/orisyvo/</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -3758,7 +3804,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>[Mining.com](https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/)</t>
+          <t>https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -3795,7 +3841,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>[Mining.com](https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/)</t>
+          <t>https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -3832,7 +3878,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>[Mining.com](https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/)</t>
+          <t>https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -3869,7 +3915,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>[IM Mining](https://im-mining.com/2026/06/29/metso-to-supply-additional-crushing-package-for-grupo-mexico-la-caridad-copper-concentrator/)</t>
+          <t>https://im-mining.com/2026/06/29/metso-to-supply-additional-crushing-package-for-grupo-mexico-la-caridad-copper-concentrator/</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -3906,7 +3952,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/05/21/3299182)</t>
+          <t>https://www.globenewswire.com/news-release/2026/05/21/3299182</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3943,7 +3989,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>[Mexico Business News](https://mexicobusiness.news/mining/news/grupo-mexicos-asarco-may-reopen-united-states)</t>
+          <t>https://mexicobusiness.news/mining/news/grupo-mexicos-asarco-may-reopen-united-states</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -3980,7 +4026,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>[Minera Alamos](https://mineraalamos.com/our-assets/cerro-de-oro-project/)</t>
+          <t>https://mineraalamos.com/our-assets/cerro-de-oro-project/</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -4017,7 +4063,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>[Global Mining Review](https://www.globalminingreview.com/mining/11022025/antler-copper-project-achieves-critical-federal-permitting-milestone/)</t>
+          <t>https://www.globalminingreview.com/mining/11022025/antler-copper-project-achieves-critical-federal-permitting-milestone/</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -4054,12 +4100,86 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>[BLM](https://www.blm.gov/press-release/blm-approves-lisbon-valley-copper-mine-expansion-utah)</t>
+          <t>https://www.blm.gov/press-release/blm-approves-lisbon-valley-copper-mine-expansion-utah</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
           <t>2026-07-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>South West Arkansas Lithium Project (Central Processing Facility)</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Sur de Arkansas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Smackover Lithium (JV Standard Lithium / Equinor)</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>S&amp;B Engineers and Constructors (EPCC); Hatch Ltd. (ingeniería de diseño/comisionamiento)</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Ingeniería de detalle/procura temprana (contrato EPCC otorgado, NTP limitado activo; FID esperada en 2026; planta diseñada para 22,500 tpa de carbonato de litio grado batería)</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>https://investingnews.com/smackover-lithium-announces-the-award-of-last-key-construction-contract-for-the-south-west-arkansas-project-ahead-of-final-investment-decision/</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Bagdad Mine Concentrator Expansion</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Yavapai County, Arizona, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Freeport-McMoRan</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Pre-FID/ingeniería avanzada (estudio para más que duplicar capacidad del concentrador, +200-250 Mlb/año cobre; capex incremental estimado ~US$3,500 millones bajo revisión; US$150M asignados en 2026 para ingeniería y obras tempranas; decisión de inversión esperada 2S-2026)</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/0000831259/000083125926000033/a2q2026exhibit991.htm</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
         </is>
       </c>
     </row>
@@ -4074,50 +4194,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -4151,7 +4271,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/vantage-breaks-ground-on-texas-gigawatt-data-center-campus-for-openai/)</t>
+          <t>https://www.datacenterdynamics.com/en/news/vantage-breaks-ground-on-texas-gigawatt-data-center-campus-for-openai/</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -4188,7 +4308,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>[Epoch AI](https://epoch.ai/publications/openai-stargate-where-the-us-sites-stand)</t>
+          <t>https://epoch.ai/publications/openai-stargate-where-the-us-sites-stand</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -4225,7 +4345,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/crusoe-tops-out-final-building-at-openai-stargate-data-center-campus-in-abilene-texas/)</t>
+          <t>https://www.datacenterdynamics.com/en/news/crusoe-tops-out-final-building-at-openai-stargate-data-center-campus-in-abilene-texas/</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -4262,7 +4382,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>[CNBC](https://www.cnbc.com/2026/06/22/chevron-cvx-microsoft-msft-natural-gas-data-center.html)</t>
+          <t>https://www.cnbc.com/2026/06/22/chevron-cvx-microsoft-msft-natural-gas-data-center.html</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -4299,7 +4419,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>[Gobierno de México](https://www.gob.mx/presidencia/prensa/plan-mexico-avanza-se-anuncia-inversion-de-4-mil-800-mdd-de-cloudhq-para-la-construccion-de-6-centros-de-datos-en-queretaro)</t>
+          <t>https://www.gob.mx/presidencia/prensa/plan-mexico-avanza-se-anuncia-inversion-de-4-mil-800-mdd-de-cloudhq-para-la-construccion-de-6-centros-de-datos-en-queretaro</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -4336,7 +4456,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>[UCS](https://www.ucs.org/about/news/judge-orders-meta-explain-new-gas-demand-hyperscale-louisiana-data-center)</t>
+          <t>https://www.ucs.org/about/news/judge-orders-meta-explain-new-gas-demand-hyperscale-louisiana-data-center</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -4373,7 +4493,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55305086/nv1-and-the-nevada-hyperscale-boom-vantage-data-centers-bets-3b-on-the-ai-future)</t>
+          <t>https://www.datacenterfrontier.com/site-selection/article/55305086/nv1-and-the-nevada-hyperscale-boom-vantage-data-centers-bets-3b-on-the-ai-future</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -4410,7 +4530,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/cloudburst-breaks-ground-on-gigawatt-scale-data-center-campus-in-texas/)</t>
+          <t>https://www.datacenterdynamics.com/en/news/cloudburst-breaks-ground-on-gigawatt-scale-data-center-campus-in-texas/</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -4447,7 +4567,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/prometheus-hyperscale-details-plans-for-dallas-data-center-campus/)</t>
+          <t>https://www.datacenterdynamics.com/en/news/prometheus-hyperscale-details-plans-for-dallas-data-center-campus/</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -4484,7 +4604,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>[Business Wire](https://www.businesswire.com/news/home/20260126236053/en/Pacifico-Energy-Secures-7.65-GW-Power-Generation-Permit-for-GW-Ranch-Project)</t>
+          <t>https://www.businesswire.com/news/home/20260126236053/en/Pacifico-Energy-Secures-7.65-GW-Power-Generation-Permit-for-GW-Ranch-Project</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -4521,7 +4641,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/amazon-looks-to-build-large-scale-data-center-campus-next-to-nuclear-plant-in-texas/)</t>
+          <t>https://www.datacenterdynamics.com/en/news/amazon-looks-to-build-large-scale-data-center-campus-next-to-nuclear-plant-in-texas/</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -4558,7 +4678,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>[Mexico News Daily](https://mexiconewsdaily.com/business/durango-data-center-fertilizer-plant-investment-fermaca/)</t>
+          <t>https://mexiconewsdaily.com/business/durango-data-center-fertilizer-plant-investment-fermaca/</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -4595,7 +4715,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/circe-energy-secures-2gw-of-natural-gas-capacity-for-west-texas-data-center-campus/)</t>
+          <t>https://www.datacenterdynamics.com/en/news/circe-energy-secures-2gw-of-natural-gas-capacity-for-west-texas-data-center-campus/</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -4612,7 +4732,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Santa Teresa, Doña Ana County, Nuevo México, EE.UU.</t>
+          <t>Santa Teresa/Sunland Park, Doña Ana County, Nuevo México, EE.UU.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -4627,197 +4747,197 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Construcción activa con riesgo regulatorio (Comisionado de Tierras de NM rechazó dos veces el derecho de vía en terrenos estatales para el gasoducto "Green Chile" de Energy Transfer, 15/16-jul-2026, tras la previa aprobación de BLM en tierra federal; meta de entrada en servicio ago-2026 en riesgo, posible retraso a 2027)</t>
+          <t>Construcción activa con riesgo regulatorio (Comisionada de Tierras de NM rechazó por segunda vez el derecho de vía en terrenos estatales para el gasoducto "Green Chile" de Energy Transfer, 14-jul-2026; NMED pospuso la decisión final sobre permisos de calidad de aire de las dos plantas de gas gemelas y programó audiencia pública para 19-oct-2026; meta de entrada en servicio ago-2026 en riesgo)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/new-mexico-regulators-reject-natural-gas-pipeline-for-oracles-25gw-project-jupiter-data-center/)</t>
+          <t>https://sourcenm.com/2026/07/16/new-mexico-land-commissioner-blocks-project-jupiter-related-pipeline-from-building-on-state-land/</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>New Era Energy &amp; Digital Hub</t>
+          <t>PowerPlay AI "Greater Abilene" Data Center</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Lea County, Nuevo México, EE.UU.</t>
+          <t>Área metropolitana de Abilene, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>New Era Energy &amp; Digital</t>
+          <t>PowerPlay AI (JV con socio Neocloud cotizado en Nasdaq, sin nombre público)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>IPP en proceso de RFP (aún sin seleccionar)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Planeación temprana (opción de terreno)</t>
+          <t>Ejecución activa post-adquisición de terreno (400MW behind-the-meter iniciales; arranque objetivo 2028)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>[PowerMag](https://www.powermag.com/nuclear-natural-gas-power-generation-planned-for-massive-new-mexico-data-center-site/)</t>
+          <t>https://www.prnewswire.com/news-releases/powerplay-ai-announces-400-mw-behind-the-meter-ai-data-center-development-in-greater-abilene-with-nasdaq-listed-neocloud-joint-venture-partner-302829610.html</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-23</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Texas Critical Data Centers (TCDC) Campus</t>
+          <t>Liberty Energy/PowerBridge "Alpha Digital Campus"</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Ector County (cerca de Odessa), Texas, EE.UU.</t>
+          <t>Condado de Reeves, Texas, EE.UU. (cerca del hub de gas Waha)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>New Era Energy &amp; Digital</t>
+          <t>PowerBridge LLC</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Stream Data Centers (JV vía LOI); Thunderhead Energy Solutions (carta de acuerdo no vinculante para ~250MW de gen. de gas behind-the-meter)</t>
+          <t>Liberty Power Innovations (subsidiaria de Liberty Energy, JV)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Ingeniería Fase Two (438 acres totales; permiso de aire en trámite; construcción total prevista en 2026, primeros 100MW dic-2026)</t>
+          <t>JV firmada/desarrollo temprano (~3,400 acres; primera fase &gt;300MW, primera entrega de energía prevista 4T2027; campus completo 2GW)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55289667/powering-ai-in-the-permian-texas-critical-data-centers-sustainable-energy-play)</t>
+          <t>https://www.datacenterdynamics.com/en/news/liberty-energy-powerbridge-form-jv-to-power-planned-2gw-data-center-in-west-texas/</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-23</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Stargate Lordstown</t>
+          <t>New Era Energy &amp; Digital Hub</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Lordstown, Ohio, EE.UU.</t>
+          <t>Lea County, Nuevo México, EE.UU.</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>OpenAI / Oracle / SoftBank</t>
+          <t>New Era Energy &amp; Digital</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>SB Energy (SoftBank)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Construcción (rompimiento de tierra)</t>
+          <t>Planeación temprana (opción de terreno)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>[OpenAI](https://openai.com/index/five-new-stargate-sites/)</t>
+          <t>https://www.powermag.com/nuclear-natural-gas-power-generation-planned-for-massive-new-mexico-data-center-site/</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Stargate Wisconsin</t>
+          <t>Texas Critical Data Centers (TCDC) Campus</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Wisconsin, EE.UU. (ubicación exacta no divulgada)</t>
+          <t>Ector County (cerca de Odessa), Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>OpenAI / Oracle / SoftBank</t>
+          <t>New Era Energy &amp; Digital</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Vantage Data Centers (en sociedad con Oracle)</t>
+          <t>Stream Data Centers (JV vía LOI); Thunderhead Energy Solutions (carta de acuerdo no vinculante para ~250MW de gen. de gas behind-the-meter)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Planeación/desarrollo temprano</t>
+          <t>Ingeniería Fase Two (438 acres totales; permiso de aire en trámite; construcción total prevista en 2026, primeros 100MW dic-2026)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>[OpenAI](https://openai.com/index/five-new-stargate-sites/)</t>
+          <t>https://www.datacenterfrontier.com/site-selection/article/55289667/powering-ai-in-the-permian-texas-critical-data-centers-sustainable-energy-play</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>AWS Región Digital Querétaro</t>
+          <t>Stargate Lordstown</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Querétaro, México</t>
+          <t>Lordstown, Ohio, EE.UU.</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Amazon Web Services (AWS)</t>
+          <t>OpenAI / Oracle / SoftBank</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>SB Energy (SoftBank)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Construcción/desarrollo (anunciado 2025, en curso)</t>
+          <t>Construcción (rompimiento de tierra)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>[Mexico News Daily](https://mexiconewsdaily.com/business/aws-invest-5b-mexico-data-region/)</t>
+          <t>https://openai.com/index/five-new-stargate-sites/</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -4829,106 +4949,106 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Stargate Michigan (Saline Barn Campus)</t>
+          <t>Stargate Wisconsin</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Saline Township, Michigan, EE.UU.</t>
+          <t>Wisconsin, EE.UU. (ubicación exacta no divulgada)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>OpenAI / Oracle (desarrollador: Related Digital)</t>
+          <t>OpenAI / Oracle / SoftBank</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Walbridge</t>
+          <t>Vantage Data Centers (en sociedad con Oracle)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Construcción</t>
+          <t>Planeación/desarrollo temprano</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/oracle-and-openai-start-construction-on-stargate-data-center-campus-in-saline-township-michigan/)</t>
+          <t>https://openai.com/index/five-new-stargate-sites/</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-14</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Applied Digital AI Factory Campuses (Polaris Forge, Ellendale/Harwood; nuevo campus Oliver County)</t>
+          <t>AWS Región Digital Querétaro</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>North Dakota, EE.UU.</t>
+          <t>Querétaro, México</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Applied Digital / Base Electron</t>
+          <t>Amazon Web Services (AWS)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Babcock &amp; Wilcox (generación); Siemens Energy (turbinas de vapor)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Construcción (Polaris Forge 1 Edificio 2 Fase 1 alcanzó Ready-for-Service 1-jul-2026, 175MW operativos; acuerdo de uso de caminos firmado 10-jul-2026 para tercer campus cerca de Center, Oliver County)</t>
+          <t>Construcción/desarrollo (anunciado 2025, en curso)</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>[Valley News Live](https://www.valleynewslive.com/2026/07/13/applied-digital-expands-north-dakota-eyes-oliver-county-third-data-center/)</t>
+          <t>https://mexiconewsdaily.com/business/aws-invest-5b-mexico-data-region/</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-14</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>AI-GDC / Cipre Holding "Green Data Center"</t>
+          <t>Stargate Michigan (Saline Barn Campus)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>San Pedro Garza García, Nuevo León, México</t>
+          <t>Saline Township, Michigan, EE.UU.</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>AI-GDC + Cipre Holding (Nvidia, socio tecnológico)</t>
+          <t>OpenAI / Oracle (desarrollador: Related Digital)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Walbridge</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Planeación/desarrollo temprano</t>
+          <t>Construcción</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>[Energy Magazine MX](https://energymagazine.mx/2026/01/el-data-center-verde-que-encendio-la-polemica-asi-sera-el-proyecto-de-ia-en-nuevo-leon-que-usara-tecnologia-de-nvidia/)</t>
+          <t>https://www.datacenterdynamics.com/en/news/oracle-and-openai-start-construction-on-stargate-data-center-campus-in-saline-township-michigan/</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -4940,54 +5060,54 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CleanArc Data Centers VA1 Campus</t>
+          <t>Applied Digital AI Factory Campuses (Polaris Forge, Ellendale/Harwood; nuevo campus Oliver County)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Caroline County, Virginia, EE.UU.</t>
+          <t>North Dakota, EE.UU.</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>CleanArc Data Centers</t>
+          <t>Applied Digital / Base Electron</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Babcock &amp; Wilcox (generación); Siemens Energy (turbinas de vapor)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Construcción</t>
+          <t>Construcción (Polaris Forge 1 Edificio 2 Fase 1 alcanzó Ready-for-Service 1-jul-2026, 175MW operativos; acuerdo de uso de caminos firmado 10-jul-2026 para tercer campus cerca de Center, Oliver County)</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>[Construction Dive](https://www.constructiondive.com/news/data-center-cleanarc-breaks-ground-virginia-campus/806489/)</t>
+          <t>https://www.valleynewslive.com/2026/07/13/applied-digital-expands-north-dakota-eyes-oliver-county-third-data-center/</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Joule Energy and Data Center Campus</t>
+          <t>AI-GDC / Cipre Holding "Green Data Center"</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Millard County (Holden), Utah, EE.UU.</t>
+          <t>San Pedro Garza García, Nuevo León, México</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Joule Capital Partners</t>
+          <t>AI-GDC + Cipre Holding (Nvidia, socio tecnológico)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -4997,12 +5117,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Construcción</t>
+          <t>Planeación/desarrollo temprano</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>[KSL](https://www.ksl.com/article/51402125/groundbreaking-for-new-millard-county-artificial-intelligence-data-center)</t>
+          <t>https://energymagazine.mx/2026/01/el-data-center-verde-que-encendio-la-polemica-asi-sera-el-proyecto-de-ia-en-nuevo-leon-que-usara-tecnologia-de-nvidia/</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -5014,17 +5134,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Amazon Montgomery County Campus</t>
+          <t>CleanArc Data Centers VA1 Campus</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>New Florence, Montgomery County, Missouri, EE.UU.</t>
+          <t>Caroline County, Virginia, EE.UU.</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>CleanArc Data Centers</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -5034,12 +5154,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Anuncio/permisos</t>
+          <t>Construcción</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>[Governor.mo.gov](https://governor.mo.gov/press-releases/archive/amazon-investing-10-billion-montgomery-county)</t>
+          <t>https://www.constructiondive.com/news/data-center-cleanarc-breaks-ground-virginia-campus/806489/</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -5051,17 +5171,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Google Montgomery County Campus</t>
+          <t>Joule Energy and Data Center Campus</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>New Florence, Montgomery County, Missouri, EE.UU.</t>
+          <t>Millard County (Holden), Utah, EE.UU.</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Joule Capital Partners</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -5071,12 +5191,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Anuncio/permisos</t>
+          <t>Construcción</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>[STLPR](https://www.stlpr.org/government-politics-issues/2026-05-21/missouri-governor-google-announce-15-billion-data-center-montgomery-county)</t>
+          <t>https://www.ksl.com/article/51402125/groundbreaking-for-new-millard-county-artificial-intelligence-data-center</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -5088,17 +5208,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Big Digital Energy / 10NetZero AI Datacenter Campus</t>
+          <t>Amazon Montgomery County Campus</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Hood County, Texas, EE.UU.</t>
+          <t>New Florence, Montgomery County, Missouri, EE.UU.</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Big Digital Energy + 10NetZero (JV)</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -5108,12 +5228,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Planeación/adquisición de sitio</t>
+          <t>Anuncio/permisos</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/06/3322404/0/en/big-digital-energy-announces-partnership-with-10netzero-to-acquire-power-ready-hood-county-texas-site-for-ai-datacenter-development.html)</t>
+          <t>https://governor.mo.gov/press-releases/archive/amazon-investing-10-billion-montgomery-county</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -5125,54 +5245,54 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Williams "Project Socrates"</t>
+          <t>Google Montgomery County Campus</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>New Albany, Ohio, EE.UU.</t>
+          <t>New Florence, Montgomery County, Missouri, EE.UU.</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Meta (vía Sidecat, LLC)</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Williams Companies / Will-Power</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Construcción (financiamiento de USD 5.34 mil millones de Blackstone/Apollo/KKR cerrado jul-2026 por 49% de participación no controladora en 5 proyectos Power Innovation de Williams; Socrates Norte/Sur, 400MW combinados, en servicio 3T/4T2026)</t>
+          <t>Anuncio/permisos</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/)</t>
+          <t>https://www.stlpr.org/government-politics-issues/2026-05-21/missouri-governor-google-announce-15-billion-data-center-montgomery-county</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-15</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Meta El Paso Campus (expansión)</t>
+          <t>Big Digital Energy / 10NetZero AI Datacenter Campus</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>El Paso, Texas, EE.UU.</t>
+          <t>Hood County, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>Big Digital Energy + 10NetZero (JV)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -5182,12 +5302,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Permisos</t>
+          <t>Planeación/adquisición de sitio</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/meta-files-to-expand-campus-in-el-paso-texas-with-12-new-buildings/)</t>
+          <t>https://www.globenewswire.com/news-release/2026/07/06/3322404/0/en/big-digital-energy-announces-partnership-with-10netzero-to-acquire-power-ready-hood-county-texas-site-for-ai-datacenter-development.html</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -5199,143 +5319,143 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>SB Energy/SoftBank PORTS Technology Campus</t>
+          <t>Williams "Project Socrates"</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Pike County, Ohio, EE.UU.</t>
+          <t>New Albany, Ohio, EE.UU.</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>SB Energy (SoftBank) / DOE / AEP Ohio</t>
+          <t>Meta (vía Sidecat, LLC)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Williams Companies / Will-Power</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Planeación/desarrollo temprano</t>
+          <t>Construcción (financiamiento de USD 5.34 mil millones de Blackstone/Apollo/KKR cerrado jul-2026 por 49% de participación no controladora en 5 proyectos Power Innovation de Williams; Socrates Norte/Sur, 400MW combinados, en servicio 3T/4T2026)</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/softbank-eyes-10gw-data-center-at-former-doe-nuclear-enrichment-site-in-ohio/)</t>
+          <t>https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Williams "Apollo" Power Generation Project</t>
+          <t>Meta El Paso Campus (expansión)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Wood County (Middleton Township), Ohio, EE.UU.</t>
+          <t>El Paso, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Meta Platforms (planta: Will-Power OH, LLC / Williams Companies)</t>
+          <t>Meta</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Williams Companies</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Construcción (aprobado por Ohio Power Siting Board feb-2026; financiamiento de USD 5.34 mil millones cerrado con Blackstone/Apollo/KKR jul-2026)</t>
+          <t>Permisos</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/)</t>
+          <t>https://www.datacenterdynamics.com/en/news/meta-files-to-expand-campus-in-el-paso-texas-with-12-new-buildings/</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-15</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Williams "Aquila" Power Project</t>
+          <t>SB Energy/SoftBank PORTS Technology Campus</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Utah, EE.UU. (condado no revelado)</t>
+          <t>Pike County, Ohio, EE.UU.</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Cliente de centro de datos no revelado (planta: Williams Companies)</t>
+          <t>SB Energy (SoftBank) / DOE / AEP Ohio</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Williams Companies</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Construcción/desarrollo (520MW; entrada en servicio prevista H1 2027; parte del financiamiento de USD 5.34 mil millones de Blackstone/Apollo/KKR)</t>
+          <t>Planeación/desarrollo temprano</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>[Williams Companies](https://www.williams.com/2026/07/13/williams-announces-5-34-billion-investment-in-power-innovation-joint-venture-from-blackstone/)</t>
+          <t>https://www.datacenterdynamics.com/en/news/softbank-eyes-10gw-data-center-at-former-doe-nuclear-enrichment-site-in-ohio/</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-15</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CleanCore/HST Technologies West Texas Data Center Campus</t>
+          <t>Williams "Apollo" Power Generation Project</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>West Texas, EE.UU. (condado no revelado)</t>
+          <t>Wood County (Middleton Township), Ohio, EE.UU.</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>CleanCore Solutions (ZONE) / HST Technologies (JV)</t>
+          <t>Meta Platforms (planta: Will-Power OH, LLC / Williams Companies)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Williams Companies</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Cierre de transacción (200MW fase inicial, jul-2026; expansión a 500MW+ prevista para 2030)</t>
+          <t>Construcción (aprobado por Ohio Power Siting Board feb-2026; financiamiento de USD 5.34 mil millones cerrado con Blackstone/Apollo/KKR jul-2026)</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/cleancore-solutions-zone-announces-closing-of-first-data-center-project-establishing-its-critical-infrastructure-buildout-for-the-ai-economy-302821421.html)</t>
+          <t>https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -5347,54 +5467,54 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Crusoe/Tallgrass AI Data Center Campus (Project Jade)</t>
+          <t>Williams "Aquila" Power Project</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Condado de Laramie, Wyoming, EE.UU.</t>
+          <t>Utah, EE.UU. (condado no revelado)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Crusoe Energy / Tallgrass</t>
+          <t>Cliente de centro de datos no revelado (planta: Williams Companies)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Williams Companies</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Desarrollo PAUSADO (Crusoe pausó actividades en jun-2026 a solicitud de su cliente; afecta también la generación de gas asociada BFC Power/Cheyenne Power Hub; aprobado ene-2026, 1.8GW inicial escalable a 10GW)</t>
+          <t>Construcción/desarrollo (520MW; entrada en servicio prevista H1 2027; parte del financiamiento de USD 5.34 mil millones de Blackstone/Apollo/KKR)</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>[Bloomberg](https://www.bloomberg.com/news/articles/2026-06-09/crusoe-touts-5-gigawatts-worth-of-data-centers-deals-pauses-wyoming-site)</t>
+          <t>https://www.williams.com/2026/07/13/williams-announces-5-34-billion-investment-in-power-innovation-joint-venture-from-blackstone/</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-16</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Core Scientific Pecos Campus (expansión IA)</t>
+          <t>CleanCore/HST Technologies West Texas Data Center Campus</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Pecos, Reeves County, Texas, EE.UU.</t>
+          <t>West Texas, EE.UU. (condado no revelado)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Core Scientific</t>
+          <t>CleanCore Solutions (ZONE) / HST Technologies (JV)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -5404,12 +5524,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Construcción (primera nave de datos en construcción vertical; expansión a 1.5GW bruto; primera capacidad prevista inicios de 2027)</t>
+          <t>Cierre de transacción (200MW fase inicial, jul-2026; expansión a 500MW+ prevista para 2030)</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>[HPCwire](https://www.hpcwire.com/off-the-wire/core-scientific-plans-expansion-to-1-5gw-of-gross-power-at-pecos-texas-campus/)</t>
+          <t>https://www.prnewswire.com/news-releases/cleancore-solutions-zone-announces-closing-of-first-data-center-project-establishing-its-critical-infrastructure-buildout-for-the-ai-economy-302821421.html</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -5421,17 +5541,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Stratos Project / Wonder Valley</t>
+          <t>Crusoe/Tallgrass AI Data Center Campus (Project Jade)</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Condado de Box Elder (Hansel Valley), Utah, EE.UU.</t>
+          <t>Condado de Laramie, Wyoming, EE.UU.</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>O'Leary Digital (Kevin O'Leary)</t>
+          <t>Crusoe Energy / Tallgrass</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -5441,71 +5561,71 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Permisos/desarrollo temprano (aprobado por comisión del condado may-2026; hasta 9GW planeados; alimentado por gasoducto Ruby; obras tempranas previstas otoño 2026)</t>
+          <t>Desarrollo PAUSADO (Crusoe pausó actividades en jun-2026 a solicitud de su cliente; afecta también la generación de gas asociada BFC Power/Cheyenne Power Hub; aprobado ene-2026, 1.8GW inicial escalable a 10GW)</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>[Utah News Dispatch](https://utahnewsdispatch.com/2026/05/19/renderings-show-massive-data-center-box-elder-utah-permits-could-take-years/)</t>
+          <t>https://www.bloomberg.com/news/articles/2026-06-09/crusoe-touts-5-gigawatts-worth-of-data-centers-deals-pauses-wyoming-site</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Fermi America Project Matador</t>
+          <t>Core Scientific Pecos Campus (expansión IA)</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Carson County (Amarillo), Texas, EE.UU.</t>
+          <t>Pecos, Reeves County, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Fermi America</t>
+          <t>Core Scientific</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Primoris Services Corporation (balance of plant, turbinas de gas)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Construcción (excavación de isla de turbinas completada; EPC firmado)</t>
+          <t>Construcción (primera nave de datos en construcción vertical; expansión a 1.5GW bruto; primera capacidad prevista inicios de 2027)</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/fermi-selects-primoris-services-corporation-to-engineer-and-construct-balance-of-plant-for-first-six-sgt-800-gas-turbines-of-phase-one-power-buildout-302814505.html)</t>
+          <t>https://www.hpcwire.com/off-the-wire/core-scientific-plans-expansion-to-1-5gw-of-gross-power-at-pecos-texas-campus/</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-16</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>NextEra Texas Power Generation Hub</t>
+          <t>Stratos Project / Wonder Valley</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Anderson County, Texas, EE.UU.</t>
+          <t>Condado de Box Elder (Hansel Valley), Utah, EE.UU.</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>NextEra Energy Resources</t>
+          <t>O'Leary Digital (Kevin O'Leary)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -5515,71 +5635,71 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Aprobado/planeación (5.2GW a gas; primera fase en línea 2028; data center asociado aún no contratado)</t>
+          <t>Permisos/desarrollo temprano (aprobado por comisión del condado may-2026; hasta 9GW planeados; alimentado por gasoducto Ruby; obras tempranas previstas otoño 2026)</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>[KLTV](https://www.kltv.com/2026/03/20/president-trump-approves-16-billion-natural-gas-generator-be-installed-anderson-county/)</t>
+          <t>https://utahnewsdispatch.com/2026/05/19/renderings-show-massive-data-center-box-elder-utah-permits-could-take-years/</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-16</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Mon Power/FirstEnergy Gas Plant (Maidsville Energy Center)</t>
+          <t>Fermi America Project Matador</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Monongalia County, Virginia Occidental, EE.UU.</t>
+          <t>Carson County (Amarillo), Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Mon Power (FirstEnergy)</t>
+          <t>Fermi America</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Primoris Services Corporation (balance of plant, turbinas de gas)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Planeación/regulatorio (USD 2.4 mil millones, 1,200MW; audiencia probatoria concluida 16/17-jul-2026 ante PSC; Mon Power confirmó pláticas con 3 desarrolladores de data centers no identificados; op. comercial prevista 31-dic-2031)</t>
+          <t>Construcción (excavación de isla de turbinas completada; EPC firmado)</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>[WV MetroNews](https://wvmetronews.com/2026/07/16/mon-power-president-says-data-centers-will-end-up-paying-for-natural-gas-powered-power-plant/)</t>
+          <t>https://www.prnewswire.com/news-releases/fermi-selects-primoris-services-corporation-to-engineer-and-construct-balance-of-plant-for-first-six-sgt-800-gas-turbines-of-phase-one-power-buildout-302814505.html</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-17</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>IEP Greene County Data Center &amp; Power Plant</t>
+          <t>NextEra Texas Power Generation Hub</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Greene County, Pensilvania, EE.UU.</t>
+          <t>Anderson County, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>International Electric Power</t>
+          <t>NextEra Energy Resources</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -5589,12 +5709,12 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Permisos (aprobación preliminar de desarrollo de terreno; planta CCGT de 944MW; COD previsto Q1 2029)</t>
+          <t>Aprobado/planeación (5.2GW a gas; primera fase en línea 2028; data center asociado aún no contratado)</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>[Utility Dive](https://www.utilitydive.com/news/iep-plans-944-mw-behind-the-meter-gas-plant-in-pennsylvania-to-power-data-c/758830/)</t>
+          <t>https://www.kltv.com/2026/03/20/president-trump-approves-16-billion-natural-gas-generator-be-installed-anderson-county/</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -5606,17 +5726,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>AWS "Project Eagle"</t>
+          <t>Mon Power/FirstEnergy Gas Plant (Maidsville Energy Center)</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Boling, Wharton County, Texas, EE.UU. (SO de Houston)</t>
+          <t>Monongalia County, Virginia Occidental, EE.UU.</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Amazon Web Services</t>
+          <t>Mon Power (FirstEnergy)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -5626,34 +5746,34 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Permisos (presentados ante TDLR; construcción de 4 edificios, USD 1.2 mil millones, inicia 1-ago-2026)</t>
+          <t>Planeación/regulatorio (USD 2.4 mil millones, 1,200MW; audiencia probatoria concluida 16/17-jul-2026 ante PSC; Mon Power confirmó pláticas con 3 desarrolladores de data centers no identificados; op. comercial prevista 31-dic-2031)</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/aws-files-for-12bn-data-center-campus-outside-houston-texas/)</t>
+          <t>https://wvmetronews.com/2026/07/16/mon-power-president-says-data-centers-will-end-up-paying-for-natural-gas-powered-power-plant/</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Crusoe/Lancium Childress Data Center Campus</t>
+          <t>IEP Greene County Data Center &amp; Power Plant</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Condado de Childress, Texas, EE.UU.</t>
+          <t>Greene County, Pensilvania, EE.UU.</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Crusoe (operador) / Lancium (infraestructura energética)</t>
+          <t>International Electric Power</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -5663,49 +5783,49 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Anuncio/planeación (construcción prevista 3T2026; campus de 1.0-1.4GW)</t>
+          <t>Permisos (aprobación preliminar de desarrollo de terreno; planta CCGT de 944MW; COD previsto Q1 2029)</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>[Crusoe](https://www.crusoe.ai/resources/newsroom/crusoe-and-lancium-announce-1-gigawatt-ai-data-center-campus-in-childress-texas)</t>
+          <t>https://www.utilitydive.com/news/iep-plans-944-mw-behind-the-meter-gas-plant-in-pennsylvania-to-power-data-c/758830/</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-17</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Williams "Neo" Power Innovation Project</t>
+          <t>AWS "Project Eagle"</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Ohio, EE.UU. (sitio exacto no revelado)</t>
+          <t>Boling, Wharton County, Texas, EE.UU. (SO de Houston)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Cliente de centro de datos no revelado</t>
+          <t>Amazon Web Services</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Williams Companies</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Planeación/desarrollo (682MW; en servicio 2S2028; parte del financiamiento de USD 5.34 mil millones de Blackstone/Apollo/KKR)</t>
+          <t>Permisos (presentados ante TDLR; construcción de 4 edificios, USD 1.2 mil millones, inicia 1-ago-2026)</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/)</t>
+          <t>https://www.datacenterdynamics.com/en/news/aws-files-for-12bn-data-center-campus-outside-houston-texas/</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -5717,106 +5837,106 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Williams "Socrates the Younger" Power Innovation Project</t>
+          <t>Crusoe/Lancium Childress Data Center Campus</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>New Albany, Ohio, EE.UU. (adyacente a Project Socrates)</t>
+          <t>Condado de Childress, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Meta Platforms (vía Sidecat, LLC)</t>
+          <t>Crusoe (operador) / Lancium (infraestructura energética)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Williams Companies</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Construcción (aprobada por Ohio Power Siting Board 9-jun-2026; 340MW; en servicio 2S2028; parte del financiamiento de USD 5.34 mil millones de Blackstone/Apollo/KKR)</t>
+          <t>Anuncio/planeación (construcción prevista 3T2026; campus de 1.0-1.4GW)</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>[PowerMag](https://www.powermag.com/new-200-mw-gas-fired-plant-in-ohio-will-power-meta-data-center/)</t>
+          <t>https://www.crusoe.ai/resources/newsroom/crusoe-and-lancium-announce-1-gigawatt-ai-data-center-campus-in-childress-texas</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Crusoe/Google "Goodnight Campus"</t>
+          <t>Williams "Neo" Power Innovation Project</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Condado de Armstrong (Claude), Texas, EE.UU.</t>
+          <t>Ohio, EE.UU. (sitio exacto no revelado)</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Google (negociación de arrendamiento) / Crusoe Energy (desarrollador)</t>
+          <t>Cliente de centro de datos no revelado</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Williams Companies</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Construcción (4 de 7 edificios en obra; campus de USD 29 mil millones, ~1,030MW; planta de gas propia de 933MW en trámite ante TCEQ, respaldada por parque eólico Goodnight de 265.5MW)</t>
+          <t>Planeación/desarrollo (682MW; en servicio 2S2028; parte del financiamiento de USD 5.34 mil millones de Blackstone/Apollo/KKR)</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>[Aterio](https://www.aterio.io/blog/crusoe-launches-usd29b-goodnight-campus-in-claude-mirroring-openai-s-stargate)</t>
+          <t>https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>VoltaGrid/Serverfarm Covington</t>
+          <t>Williams "Socrates the Younger" Power Innovation Project</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Condado de Newton (Covington), Georgia, EE.UU.</t>
+          <t>New Albany, Ohio, EE.UU. (adyacente a Project Socrates)</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Serverfarm</t>
+          <t>Meta Platforms (vía Sidecat, LLC)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>VoltaGrid (planta de energía "pop-up", 33 motores de combustión interna)</t>
+          <t>Williams Companies</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Construcción DETENIDA (orden de suspensión de la agencia ambiental de Georgia -EPD- por construir sin permisos, 2-jul-2026)</t>
+          <t>Construcción (aprobada por Ohio Power Siting Board 9-jun-2026; 340MW; en servicio 2S2028; parte del financiamiento de USD 5.34 mil millones de Blackstone/Apollo/KKR)</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>[AJC](https://www.ajc.com/business/2026/07/officials-order-georgia-data-centers-pop-up-power-plant-to-halt-construction/)</t>
+          <t>https://www.powermag.com/new-200-mw-gas-fired-plant-in-ohio-will-power-meta-data-center/</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -5828,17 +5948,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Stark Power/Sagebrush Infrastructure Partners (SAGE)</t>
+          <t>Crusoe/Google "Goodnight Campus"</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Múltiples sitios, EE.UU. Central (ubicaciones no reveladas)</t>
+          <t>Condado de Armstrong (Claude), Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Stark Power (adquirió SAGE, 8-jun-2026)</t>
+          <t>Google (negociación de arrendamiento) / Crusoe Energy (desarrollador)</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -5848,12 +5968,12 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Adquisición/planeación temprana (portafolio de 5 campus hyperscale con generación de gas co-localizada, 5.6GW agregados)</t>
+          <t>Construcción (4 de 7 edificios en obra; campus de USD 29 mil millones, ~1,030MW; planta de gas propia de 933MW en trámite ante TCEQ, respaldada por parque eólico Goodnight de 265.5MW)</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/stark-power-lands-56gw-data-center-development-portfolio-in-sagebrush-acquisition/)</t>
+          <t>https://www.aterio.io/blog/crusoe-launches-usd29b-goodnight-campus-in-claude-mirroring-openai-s-stargate</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -5865,106 +5985,106 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Homer City Energy Campus</t>
+          <t>VoltaGrid/Serverfarm Covington</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Condado de Indiana, Pensilvania, EE.UU.</t>
+          <t>Condado de Newton (Covington), Georgia, EE.UU.</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Homer City Redevelopment (HCR)</t>
+          <t>Serverfarm</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Kiewit Power Constructors Co.; turbinas GE Vernova (7x 7HA.02 con capacidad de hidrógeno)</t>
+          <t>VoltaGrid (planta de energía "pop-up", 33 motores de combustión interna)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Construcción (excavación/demolición completadas; planta de gas de 4.5GW, la más grande planeada en EE.UU.; primeras entregas de turbinas 2026, operación comercial 2027)</t>
+          <t>Construcción DETENIDA (orden de suspensión de la agencia ambiental de Georgia -EPD- por construir sin permisos, 2-jul-2026)</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55281341/pennsylvanias-homer-city-energy-campus-a-brownfield-transformed-for-data-center-innovation)</t>
+          <t>https://www.ajc.com/business/2026/07/officials-order-georgia-data-centers-pop-up-power-plant-to-halt-construction/</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-21</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Nebius Vineland AI Data Center Campus</t>
+          <t>Stark Power/Sagebrush Infrastructure Partners (SAGE)</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Vineland, Nueva Jersey, EE.UU.</t>
+          <t>Múltiples sitios, EE.UU. Central (ubicaciones no reveladas)</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Nebius Group (cómputo entregado a Microsoft bajo acuerdo de USD 17.4 mil millones)</t>
+          <t>Stark Power (adquirió SAGE, 8-jun-2026)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>No especificado (motores reciprocantes de gas Bergen, ~30 unidades)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Construcción/Permisos (planta de gas de hasta 400MW enfrenta retrasos por Ley de Justicia Ambiental de NJ; meta de entrega nov-2026 en riesgo)</t>
+          <t>Adquisición/planeación temprana (portafolio de 5 campus hyperscale con generación de gas co-localizada, 5.6GW agregados)</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>[Data Center Knowledge](https://www.datacenterknowledge.com/data-center-site-selection/nebius-plans-300-mw-data-center-in-new-jersey-amid-us-expansion)</t>
+          <t>https://www.datacenterdynamics.com/en/news/stark-power-lands-56gw-data-center-development-portfolio-in-sagebrush-acquisition/</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-21</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>TerraVolt Infrastructure AI Data Center Campus</t>
+          <t>Homer City Energy Campus</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Sureste de Idaho, EE.UU. (sobre gasoducto Northwest Natural Gas Pipeline)</t>
+          <t>Condado de Indiana, Pensilvania, EE.UU.</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>TerraVolt Infrastructure, Inc. (subsidiaria de CalEthos, Inc.)</t>
+          <t>Homer City Redevelopment (HCR)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Kiewit Power Constructors Co.; turbinas GE Vernova (7x 7HA.02 con capacidad de hidrógeno)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Ingeniería/Planeación (acuerdo de suministro de gas natural firmado, 55,000 MMBtu/día, para planta on-site de 200-240MW)</t>
+          <t>Construcción (excavación/demolición completadas; planta de gas de 4.5GW, la más grande planeada en EE.UU.; primeras entregas de turbinas 2026, operación comercial 2027)</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/terravolt-inks-natural-gas-supply-deal-for-onsite-power-plant-at-planned-data-center-campus-in-idaho/)</t>
+          <t>https://www.datacenterfrontier.com/site-selection/article/55281341/pennsylvanias-homer-city-energy-campus-a-brownfield-transformed-for-data-center-innovation</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -5976,35 +6096,109 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
+          <t>Nebius Vineland AI Data Center Campus</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Vineland, Nueva Jersey, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Nebius Group (cómputo entregado a Microsoft bajo acuerdo de USD 17.4 mil millones)</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>No especificado (motores reciprocantes de gas Bergen, ~30 unidades)</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Construcción/Permisos (planta de gas de hasta 400MW enfrenta retrasos por Ley de Justicia Ambiental de NJ; meta de entrega nov-2026 en riesgo)</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>https://www.datacenterknowledge.com/data-center-site-selection/nebius-plans-300-mw-data-center-in-new-jersey-amid-us-expansion</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>TerraVolt Infrastructure AI Data Center Campus</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Sureste de Idaho, EE.UU. (sobre gasoducto Northwest Natural Gas Pipeline)</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>TerraVolt Infrastructure, Inc. (subsidiaria de CalEthos, Inc.)</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Ingeniería/Planeación (acuerdo de suministro de gas natural firmado, 55,000 MMBtu/día, para planta on-site de 200-240MW)</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>https://www.datacenterdynamics.com/en/news/terravolt-inks-natural-gas-supply-deal-for-onsite-power-plant-at-planned-data-center-campus-in-idaho/</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
           <t>CyrusOne SAT14A</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr">
+      <c r="B54" t="inlineStr">
         <is>
           <t>Castroville, San Antonio, Texas, EE.UU.</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="C54" t="inlineStr">
         <is>
           <t>CyrusOne (sin arrendatario asignado aún)</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>No especificado</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
         <is>
           <t>Ingeniería/Permisos (6to campus en San Antonio, 11vo en Texas; USD 500 millones, 460,000 pies²; inicio de construcción previsto dic-2026)</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/cyrusone-announces-sixth-data-center-campus-in-san-antonio-texas/)</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>https://www.datacenterdynamics.com/en/news/cyrusone-announces-sixth-data-center-campus-in-san-antonio-texas/</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
         <is>
           <t>2026-07-22</t>
         </is>

</xml_diff>

<commit_message>
Agregar 6 proyectos nuevos y 8 cambios de fase (2026-07-23) (#7)
- LNG (1 nuevo): Sabine Pass LNG Expansion (Train 7 + reliquefacción)
- Mining (2 nuevos): South West Arkansas Lithium Project (Smackover Lithium), Bagdad Mine Concentrator Expansion (Freeport-McMoRan)
- Data Centers (2 nuevos): PowerPlay AI "Greater Abilene", Liberty Energy/PowerBridge "Alpha Digital Campus"

Cambios de fase: Saguaro Energía LNG (pausado por orden judicial), Corpus Christi Stage 3 (FERC autoriza Train 7), Texas LNG Brownsville (inversión HPS/BlackRock), El Pilar Copper Project (permisos asegurados, US$551M), Hermosa Critical Minerals (ROD final USFS), Project Jupiter (audiencia NMED oct-2026).

Se regenera proyectos.xlsx (una hoja por industria) con el acumulado completo.


Claude-Session: https://claude.ai/code/session_01YLKArezdQJfAqyTik1hNM8

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -20,10 +20,18 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
@@ -49,8 +57,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -419,47 +428,47 @@
   <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -493,7 +502,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>[Fluor newsroom](https://newsroom.fluor.com/news-releases/news-details/2026/Fluor-Awarded-Contract-to-Engineer-and-Design-the-America-First-Refining-Facility-in-Brownsville-Texas/default.aspx)</t>
+          <t>https://newsroom.fluor.com/news-releases/news-details/2026/Fluor-Awarded-Contract-to-Engineer-and-Design-the-America-First-Refining-Facility-in-Brownsville-Texas/default.aspx</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -530,7 +539,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>[AllStream Insiders](https://allstreaminsiders.com/us-exxonmobil-may-build-cracker-pe-plant-in-texas-with-an-8-6-billion-investment/)</t>
+          <t>https://allstreaminsiders.com/us-exxonmobil-may-build-cracker-pe-plant-in-texas-with-an-8-6-billion-investment/</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -567,7 +576,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>[BIC Magazine](https://www.bicmagazine.com/departments/operations/cpchem-golden-triangle-polymers-facility-startup-phase/)</t>
+          <t>https://www.bicmagazine.com/departments/operations/cpchem-golden-triangle-polymers-facility-startup-phase/</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -604,7 +613,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>[Construction Front](https://constructionfront.com/2025-04-13-technip-energies-to-deliver-blue-point-worlds-largest-low-carbon-ammonia-facility-in-louisiana/)</t>
+          <t>https://constructionfront.com/2025-04-13-technip-energies-to-deliver-blue-point-worlds-largest-low-carbon-ammonia-facility-in-louisiana/</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -641,7 +650,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>[East Daley](https://eastdaley.com/media-and-news/the-race-is-on-to-build-permian-processing)</t>
+          <t>https://eastdaley.com/media-and-news/the-race-is-on-to-build-permian-processing</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -678,7 +687,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>[Techint](https://www.techint.com/en/our-projects/dos-bocas-refinery)</t>
+          <t>https://www.techint.com/en/our-projects/dos-bocas-refinery</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -715,7 +724,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>[OGJ](https://www.ogj.com/refining-processing/refining/optimization/article/17279334/pemex-to-proceed-with-dos-bocas-refinery-project)</t>
+          <t>https://www.ogj.com/refining-processing/refining/optimization/article/17279334/pemex-to-proceed-with-dos-bocas-refinery-project</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -752,7 +761,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>[Forbes México](https://forbes.com.mx/pemex-invertira-5300-millones-de-dolares-para-reactivar-la-industria-petroquimica/)</t>
+          <t>https://forbes.com.mx/pemex-invertira-5300-millones-de-dolares-para-reactivar-la-industria-petroquimica/</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -789,7 +798,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>[Forbes México](https://forbes.com.mx/pemex-invertira-5300-millones-de-dolares-para-reactivar-la-industria-petroquimica/)</t>
+          <t>https://forbes.com.mx/pemex-invertira-5300-millones-de-dolares-para-reactivar-la-industria-petroquimica/</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -826,7 +835,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>[Forbes México](https://forbes.com.mx/asi-es-la-inversion-de-1553-mdd-por-parte-de-pemex-en-una-planta-de-fertilizantes-en-veracruz/)</t>
+          <t>https://forbes.com.mx/asi-es-la-inversion-de-1553-mdd-por-parte-de-pemex-en-una-planta-de-fertilizantes-en-veracruz/</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -863,7 +872,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>[Tribuna](https://tribuna.com.mx/mexico/2026/06/05/sheinbaum-anuncia-inversion-de-93-mil-mdp-para-reactivar-la-industria-petroquimica-y-de-fertilizantes-en-veracruz_560837/)</t>
+          <t>https://tribuna.com.mx/mexico/2026/06/05/sheinbaum-anuncia-inversion-de-93-mil-mdp-para-reactivar-la-industria-petroquimica-y-de-fertilizantes-en-veracruz_560837/</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -900,7 +909,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>[PV Magazine México](https://www.pv-magazine-mexico.com/2026/04/28/inician-en-sinaloa-la-construccion-de-la-mayor-planta-de-metanol-ultrabajo-en-carbono-a-partir-de-hidrogeno-verde/)</t>
+          <t>https://www.pv-magazine-mexico.com/2026/04/28/inician-en-sinaloa-la-construccion-de-la-mayor-planta-de-metanol-ultrabajo-en-carbono-a-partir-de-hidrogeno-verde/</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -937,7 +946,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>[H2 View](https://www.h2-view.com/story/first-ammonia-project-on-track-for-2026-fid-despite-topsoe-deal-collapse/2138792.article/)</t>
+          <t>https://www.h2-view.com/story/first-ammonia-project-on-track-for-2026-fid-despite-topsoe-deal-collapse/2138792.article/</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -974,7 +983,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>[Debate](https://www.debate.com.mx/economia/secretaria-de-economia-complejo-de-amoniaco-en-topolobampo-prioritario-para-el-gobierno-de-mexico-20260713-0092.html)</t>
+          <t>https://www.debate.com.mx/economia/secretaria-de-economia-complejo-de-amoniaco-en-topolobampo-prioritario-para-el-gobierno-de-mexico-20260713-0092.html</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1011,7 +1020,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>[ICIS](https://www.icis.com/explore/resources/news/2025/11/13/11155109/lake-charles-methanol-ii-awards-feed-fid-expected-in-q2-2026/)</t>
+          <t>https://www.icis.com/explore/resources/news/2025/11/13/11155109/lake-charles-methanol-ii-awards-feed-fid-expected-in-q2-2026/</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1048,7 +1057,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>[Diario del Istmo](https://diariodelistmo.com/nacional/este-es-el-avance-que-lleva-la-planta-coquizadora-en-la-refineria-de-salina-cruz/50642321)</t>
+          <t>https://diariodelistmo.com/nacional/este-es-el-avance-que-lleva-la-planta-coquizadora-en-la-refineria-de-salina-cruz/50642321</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1085,7 +1094,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/petrochemicals/06032026/shintech-announces-us34-billion-at-louisiana-petrochemicals-complex/)</t>
+          <t>https://www.hydrocarbonengineering.com/petrochemicals/06032026/shintech-announces-us34-billion-at-louisiana-petrochemicals-complex/</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1122,7 +1131,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>[Alchempro](https://www.alchempro.com/news/chemicals-news/ineos-backs-1-7-bn-low-carbon-methanol-project-in-texas-city-310108-newsdetails.htm)</t>
+          <t>https://www.alchempro.com/news/chemicals-news/ineos-backs-1-7-bn-low-carbon-methanol-project-in-texas-city-310108-newsdetails.htm</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1159,7 +1168,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/petrochemicals/13072026/oxea-confirms-fid-for-major-capacity-expansion/)</t>
+          <t>https://www.hydrocarbonengineering.com/petrochemicals/13072026/oxea-confirms-fid-for-major-capacity-expansion/</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1196,7 +1205,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>[OGJ](https://www.ogj.com/refining-processing/gas-processing/news/55320579/targa-advances-permian-gas-pipeline-processing-expansion)</t>
+          <t>https://www.ogj.com/refining-processing/gas-processing/news/55320579/targa-advances-permian-gas-pipeline-processing-expansion</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1233,7 +1242,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>[Business Wire](https://www.businesswire.com/news/home/20250806663187/en/Enterprise-Agrees-to-Acquire-Occidentals-Gas-Gathering-Affiliate-Enters-Into-Natural-Gas-Processing-Agreement-Announces-New-Midland-Basin-Natural-Gas-Processing-Plant)</t>
+          <t>https://www.businesswire.com/news/home/20250806663187/en/Enterprise-Agrees-to-Acquire-Occidentals-Gas-Gathering-Affiliate-Enters-Into-Natural-Gas-Processing-Agreement-Announces-New-Midland-Basin-Natural-Gas-Processing-Plant</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1270,7 +1279,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>[Natural Gas Intel](https://naturalgasintel.com/news/mplx-scales-up-for-power-hungry-future-with-natural-gas-focused-growth-plan/)</t>
+          <t>https://naturalgasintel.com/news/mplx-scales-up-for-power-hungry-future-with-natural-gas-focused-growth-plan/</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1307,7 +1316,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>[East Daley](https://eastdaley.com/daley-note/mplx-acquires-northwind-for-2-375b-acquires-more-ngls-for-jv-project)</t>
+          <t>https://eastdaley.com/daley-note/mplx-acquires-northwind-for-2-375b-acquires-more-ngls-for-jv-project</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1344,7 +1353,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>[Grand Forks Herald](https://www.grandforksherald.com/news/local/northern-plains-nitrogen-proposal-receiving-more-attention-amid-global-fertilizer-pressure)</t>
+          <t>https://www.grandforksherald.com/news/local/northern-plains-nitrogen-proposal-receiving-more-attention-amid-global-fertilizer-pressure</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1381,7 +1390,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>[Phillips 66](https://www.phillips66.com/newsroom/iron-mesa-safely-enters-next-phase-of-construction/)</t>
+          <t>https://www.phillips66.com/newsroom/iron-mesa-safely-enters-next-phase-of-construction/</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1418,7 +1427,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>[Targa Resources](https://www.targaresources.com/news-releases/news-release-details/targa-resources-corp-announces-permian-growth-projects-and)</t>
+          <t>https://www.targaresources.com/news-releases/news-release-details/targa-resources-corp-announces-permian-growth-projects-and</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1455,7 +1464,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>[Elefante Blanco](https://elefanteblanco.mx/2026/01/02/pemex-abre-30-licitaciones-para-obras-en-la-refineria-madero/)</t>
+          <t>https://elefanteblanco.mx/2026/01/02/pemex-abre-30-licitaciones-para-obras-en-la-refineria-madero/</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1492,7 +1501,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>[La Jornada](https://www.jornada.com.mx/noticia/2026/06/08/economia/da-inicio-ejecucion-de-planta-de-fertilizantes-en-durango-por-parte-de-fermachem)</t>
+          <t>https://www.jornada.com.mx/noticia/2026/06/08/economia/da-inicio-ejecucion-de-planta-de-fertilizantes-en-durango-por-parte-de-fermachem</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1529,7 +1538,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>[Downstream Calendar](https://downstreamcalendar.com/mcdermott-secures-feed-contract-for-ascension-clean-energy-project/)</t>
+          <t>https://downstreamcalendar.com/mcdermott-secures-feed-contract-for-ascension-clean-energy-project/</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1566,7 +1575,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>[Business Wire](https://www.businesswire.com/news/home/20260517310811/en/Phillips-66-announces-Zeus-Gas-Plant-and-a-third-Coastal-Bend-Fractionator)</t>
+          <t>https://www.businesswire.com/news/home/20260517310811/en/Phillips-66-announces-Zeus-Gas-Plant-and-a-third-Coastal-Bend-Fractionator</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1603,7 +1612,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>[USDA](https://www.usda.gov/about-usda/news/press-releases/2026/07/01/secretary-rollins-announces-500-million-fertilizer-investment-and-expansion-program-strengthen)</t>
+          <t>https://www.usda.gov/about-usda/news/press-releases/2026/07/01/secretary-rollins-announces-500-million-fertilizer-investment-and-expansion-program-strengthen</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1623,50 +1632,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -1700,7 +1709,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>[Bechtel](https://www.bechtel.com/press-releases/nextdecade-executes-epc-contract-with-bechtel-for-train-4-at-the-rio-grande-lng-facility/)</t>
+          <t>https://www.bechtel.com/press-releases/nextdecade-executes-epc-contract-with-bechtel-for-train-4-at-the-rio-grande-lng-facility/</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -1737,7 +1746,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>[Bechtel](https://www.bechtel.com/press-releases/sempra-infrastructure-announces-epc-contract-with-bechtel-for-port-arthur-lng-phase-2/)</t>
+          <t>https://www.bechtel.com/press-releases/sempra-infrastructure-announces-epc-contract-with-bechtel-for-port-arthur-lng-phase-2/</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -1774,7 +1783,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>[Woodside](https://www.woodside.com/what-we-do/growth-projects/woodside-louisiana-lng)</t>
+          <t>https://www.woodside.com/what-we-do/growth-projects/woodside-louisiana-lng</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -1811,7 +1820,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>[GEM.wiki](https://www.gem.wiki/CP2_LNG_Terminal)</t>
+          <t>https://www.gem.wiki/CP2_LNG_Terminal</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -1848,7 +1857,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>[Offshore Energy](https://www.offshore-energy.biz/kbr-zachry-to-work-on-ventures-plaquemines-lng/)</t>
+          <t>https://www.offshore-energy.biz/kbr-zachry-to-work-on-ventures-plaquemines-lng/</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -1885,7 +1894,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>[LNG Prime](https://lngprime.com/contracts-and-tenders/golden-pass-lng-contractors-ink-revised-epc-deal-for-second-and-third-train/169104/)</t>
+          <t>https://lngprime.com/contracts-and-tenders/golden-pass-lng-contractors-ink-revised-epc-deal-for-second-and-third-train/169104/</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1917,17 +1926,17 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Construcción (98%)</t>
+          <t>Construcción (FERC autorizó introducción de gas combustible en Train 7, 17-jul-2026; primera producción de LNG esperada ago-2026, servicio comercial sep-2026)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>[LNG Prime](https://lngprime.com/americas/chenieres-corpus-christi-stage-3-project-98-percent-complete/190871/)</t>
+          <t>https://pgjonline.com/news/2026/july/corpus-christi-lng-train-7-cleared-to-introduce-fuel-gas-by-ferc</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-23</t>
         </is>
       </c>
     </row>
@@ -1959,7 +1968,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/06/03/3306350/0/en/delfin-midstream-announces-5-billion-final-investment-decision-for-first-flng-vessel.html)</t>
+          <t>https://www.globenewswire.com/news-release/2026/06/03/3306350/0/en/delfin-midstream-announces-5-billion-final-investment-decision-for-first-flng-vessel.html</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1991,17 +2000,17 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Ingeniería/Pre-FID con retrasos</t>
+          <t>Pre-FID PAUSADO (suspensión judicial desde abr-2026 por demanda ambiental sobre ballenas en el Mar de Cortés; presión de activistas contra financiadores JPMorgan/Santander, 17-jul-2026; definición de autorización pendiente para 2026)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>[IEEFA](https://ieefa.org/resources/mexico-pacific-limited-delays-turmoil-and-permitting-errors-have-stymied-mexicos-largest)</t>
+          <t>https://dossierpolitico.com/2026/07/17/activistas-entregan-90-mil-firmas-para-frenar-proyecto-saguaro-energia-en-sonora/</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-23</t>
         </is>
       </c>
     </row>
@@ -2033,7 +2042,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>[GEM Wiki](https://www.gem.wiki/New_Fortress_Altamira_FLNG_Terminal)</t>
+          <t>https://www.gem.wiki/New_Fortress_Altamira_FLNG_Terminal</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -2065,17 +2074,17 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Construcción (LNTP otorgado a Kiewit 4-jul-2026 para compra de equipo de entrega larga, ingeniería EPC y geotécnico; FID prevista fin de 2026)</t>
+          <t>Construcción (LNTP otorgado a Kiewit 4-jul-2026; HPS Investment Partners/BlackRock invirtió US$500M para obras tempranas, visto como paso final previo a FID; FID prevista fin de 2026)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>[OGJ](https://www.ogj.com/pipelines-transportation/lng/news/55388908/texas-lng-advances-pre-fid-project-with-limited-notice-to-proceed)</t>
+          <t>https://www.naturalgasintel.com/news/glenfarne-lands-investment-for-early-work-on-texas-lng-ahead-of-fid/</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-23</t>
         </is>
       </c>
     </row>
@@ -2107,7 +2116,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>[PGJ](https://pgjonline.com/news/2026/july/commonwealth-lng-awards-main-automation-contract-for-louisiana-export-terminal)</t>
+          <t>https://pgjonline.com/news/2026/july/commonwealth-lng-awards-main-automation-contract-for-louisiana-export-terminal</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -2144,7 +2153,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>[Houston Public Media](https://www.houstonpublicmedia.org/articles/galveston-county/2026/07/14/557086/galveston-pelican-island-lng/)</t>
+          <t>https://www.houstonpublicmedia.org/articles/galveston-county/2026/07/14/557086/galveston-pelican-island-lng/</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -2181,7 +2190,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>[Sempra](https://www.sempra.com/newsroom/press-releases/sempra-infrastructures-eca-lng-phase-1-exports-first-lng-cargo-mexicos)</t>
+          <t>https://www.sempra.com/newsroom/press-releases/sempra-infrastructures-eca-lng-phase-1-exports-first-lng-cargo-mexicos</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -2218,7 +2227,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>[LNG Prime](https://lngprime.com/americas/gato-negro-eyes-fid-on-mexico-lng-plant-in-late-2026/165906/)</t>
+          <t>https://lngprime.com/americas/gato-negro-eyes-fid-on-mexico-lng-plant-in-late-2026/165906/</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -2255,7 +2264,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/amigo-lng-awards-landmark-epc-contract-to-dubai-based-drydocks-world-for-worlds-largest-flng-facility-302537739.html)</t>
+          <t>https://www.prnewswire.com/news-releases/amigo-lng-awards-landmark-epc-contract-to-dubai-based-drydocks-world-for-worlds-largest-flng-facility-302537739.html</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -2292,7 +2301,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>[KBR](https://www.kbr.com/en/insights-news/press-release/kbr-awarded-feed-coastal-bend-lng-project)</t>
+          <t>https://www.kbr.com/en/insights-news/press-release/kbr-awarded-feed-coastal-bend-lng-project</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2329,7 +2338,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>[FERC](https://www.ferc.gov/gulfstream-lng-terminal-project)</t>
+          <t>https://www.ferc.gov/gulfstream-lng-terminal-project</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2366,7 +2375,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>[Glenfarne](https://glenfarnegroup.com/glenfarne-announces-major-phase-one-alaska-lng-milestones-with-construction-line-pipe-supply-and-in-state-gas-agreements/)</t>
+          <t>https://glenfarnegroup.com/glenfarne-announces-major-phase-one-alaska-lng-milestones-with-construction-line-pipe-supply-and-in-state-gas-agreements/</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2403,7 +2412,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>[PGJ](https://pgjonline.com/news/2026/july/311-mile-sonora-gas-pipeline-project-advances-in-mexico)</t>
+          <t>https://pgjonline.com/news/2026/july/311-mile-sonora-gas-pipeline-project-advances-in-mexico</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2440,7 +2449,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>[OGJ](https://www.ogj.com/pipelines-transportation/pipelines/news/55322537/arm-energy-takes-fid-on-23-billion-mustang-express-pipeline)</t>
+          <t>https://www.ogj.com/pipelines-transportation/pipelines/news/55322537/arm-energy-takes-fid-on-23-billion-mustang-express-pipeline</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2477,7 +2486,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>[Mexico Business News](https://mexicobusiness.news/energy/news/ursus-energy-scales-investment-us21-billion)</t>
+          <t>https://mexicobusiness.news/energy/news/ursus-energy-scales-investment-us21-billion</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2514,7 +2523,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/15/3327983/0/en/Delfin-Midstream-Partners-With-EIG-s-MidOcean-Energy-to-Advance-Second-FLNG-Vessel-Issues-Limited-Notice-to-Proceed-to-Siemens-Energy.html)</t>
+          <t>https://www.globenewswire.com/news-release/2026/07/15/3327983/0/en/Delfin-Midstream-Partners-With-EIG-s-MidOcean-Energy-to-Advance-Second-FLNG-Vessel-Issues-Limited-Notice-to-Proceed-to-Siemens-Energy.html</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2551,7 +2560,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>[Natural Gas Intel](https://www.naturalgasintel.com/news/texas-gateway-open-season-expands-haynesville-natural-gas-links-amid-lng-growth/)</t>
+          <t>https://www.naturalgasintel.com/news/texas-gateway-open-season-expands-haynesville-natural-gas-links-amid-lng-growth/</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2588,7 +2597,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>[World Oil](https://worldoil.com/news/2026/7/6/argent-lng-awards-engineering-contract-for-port-fourchon-lng-project/)</t>
+          <t>https://worldoil.com/news/2026/7/6/argent-lng-awards-engineering-contract-for-port-fourchon-lng-project/</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2625,7 +2634,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>[Federal Register](https://www.federalregister.gov/documents/2026/04/17/2026-07517/deepwater-port-license-application-st-lng-deepwater-port-development-project-draft-environmental)</t>
+          <t>https://www.federalregister.gov/documents/2026/04/17/2026-07517/deepwater-port-license-application-st-lng-deepwater-port-development-project-draft-environmental</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -2662,7 +2671,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>[Natural Gas Intel](https://naturalgasintel.com/news/kinder-morgan-greenlights-7b-in-natural-gas-pipeline-projects-amid-regulatory-speedup/)</t>
+          <t>https://naturalgasintel.com/news/kinder-morgan-greenlights-7b-in-natural-gas-pipeline-projects-amid-regulatory-speedup/</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -2699,7 +2708,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>[Natural Gas Intel](https://naturalgasintel.com/news/kinder-morgan-greenlights-7b-in-natural-gas-pipeline-projects-amid-regulatory-speedup/)</t>
+          <t>https://naturalgasintel.com/news/kinder-morgan-greenlights-7b-in-natural-gas-pipeline-projects-amid-regulatory-speedup/</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2736,12 +2745,49 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>[LNG Prime](https://lngprime.com/americas/kinder-morgan-seeks-doe-extension-for-gulf-lng-export-project/184334/)</t>
+          <t>https://lngprime.com/americas/kinder-morgan-seeks-doe-extension-for-gulf-lng-export-project/184334/</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
           <t>2026-07-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Sabine Pass LNG Expansion (Train 7 + unidad de re-licuefacción de boil-off gas)</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Cameron Parish, Luisiana, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Cheniere Energy Partners</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Bechtel (EPC); Baker Hughes (equipo mayor)</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Construcción/Procura de equipo mayor (EPC firmado 28-may-2026; Baker Hughes recibió pedido de 7 turbinas de gas PGT25+ G4 y 15 compresores centrífugos, ~6 MTPA adicionales; construcción plena prevista inicios de 2027)</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>https://investors.bakerhughes.com/news/press-releases/news-details/2026/Baker-Hughes-Secures-Substantial-Equipment-and-Services-Awards-for-Chenieres-Sabine-Pass-LNG-Facility/default.aspx</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
         </is>
       </c>
     </row>
@@ -2756,50 +2802,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -2833,7 +2879,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>[Mining Weekly](https://www.miningweekly.com/article/ivanhoe-electric-pencils-in-2026-construction-start-at-arizona-copper-mine-2025-06-25)</t>
+          <t>https://www.miningweekly.com/article/ivanhoe-electric-pencils-in-2026-construction-start-at-arizona-copper-mine-2025-06-25</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -2870,7 +2916,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>[SEC/Hudbay](https://www.sec.gov/Archives/edgar/data/1322422/000106299326001973/exhibit99-2.htm)</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1322422/000106299326001973/exhibit99-2.htm</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -2907,7 +2953,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>[SEC](https://www.sec.gov/Archives/edgar/data/863064/000086306426000019/ex12d16mr_resolutionland.htm)</t>
+          <t>https://www.sec.gov/Archives/edgar/data/863064/000086306426000019/ex12d16mr_resolutionland.htm</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -2944,7 +2990,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>[Nevada Appeal](https://www.nevadaappeal.com/news/2026/mar/26/lithium-americas-900-construction-workers-at-thacker-pass-mine/)</t>
+          <t>https://www.nevadaappeal.com/news/2026/mar/26/lithium-americas-900-construction-workers-at-thacker-pass-mine/</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -2981,7 +3027,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>[Mining.com](https://www.mining.com/teck-agnico-team-up-at-san-nicolas-copper-project-in-mexico/)</t>
+          <t>https://www.mining.com/teck-agnico-team-up-at-san-nicolas-copper-project-in-mexico/</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -3018,7 +3064,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>[Energy Magazine MX](https://energymagazine.mx/2025/10/grupo-mexico-espera-autorizacion-federal-para-continuar-proyectos-mineros-por-10-mil-200-mdd/)</t>
+          <t>https://energymagazine.mx/2025/10/grupo-mexico-espera-autorizacion-federal-para-continuar-proyectos-mineros-por-10-mil-200-mdd/</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -3040,7 +3086,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Grupo México</t>
+          <t>Grupo México / Southern Copper Corporation</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -3050,17 +3096,17 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Ingeniería básica completada / trámite ambiental</t>
+          <t>Permisos ambientales asegurados (proyecto revaluado en US$551 millones; preparación de sitio inicia sep-2026, construcción plena 2027, primer cobre ~2028)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>[Mexico Mining Center](https://www.mexicominingcenter.com/grupo-mexico-compra-mina-el-pilar/)</t>
+          <t>https://www.bnamericas.com/en/news/southern-copper-wins-permits-for-us551mn-el-pilar-in-mexico</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-23</t>
         </is>
       </c>
     </row>
@@ -3092,7 +3138,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>[M3 Engineering](https://m3eng.com/portfolio/buenavista-del-cobre-concentradora-no-2/)</t>
+          <t>https://m3eng.com/portfolio/buenavista-del-cobre-concentradora-no-2/</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -3129,7 +3175,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>[Minería en Línea](https://mineriaenlinea.com/2026/04/torex-gold-alcanza-velocidad-de-crucero-en-media-luna-9-meses-adelante-de-cronograma/)</t>
+          <t>https://mineriaenlinea.com/2026/04/torex-gold-alcanza-velocidad-de-crucero-en-media-luna-9-meses-adelante-de-cronograma/</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -3166,7 +3212,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>[Mining.com](https://www.mining.com/nevada-copper-unveils-restart-and-financing-plan-for-pumpkin-hollow/)</t>
+          <t>https://www.mining.com/nevada-copper-unveils-restart-and-financing-plan-for-pumpkin-hollow/</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -3198,17 +3244,17 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Construcción (Record of Decision final emitido por USFS 14-jul-2026; ~50% avance en porción privada; autorización operativa prevista sep-2026)</t>
+          <t>Construcción (Record of Decision final emitido por USFS 7-jul-2026, cerrando revisión NEPA de infraestructura en Coronado National Forest; primer proyecto minero aceptado en programa federal FAST-41; ~50% avance en porción privada; primer concentrado ahora proyectado H1-2028, antes H1-2027)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>[Chamber Business News](https://chamberbusinessnews.com/2026/07/14/hermosa-critical-minerals-mining-project-reaches-major-federal-permitting-milestone/)</t>
+          <t>https://www.usda.gov/about-usda/news/press-releases/2026/07/07/usda-advances-trump-administration-effort-boost-us-mineral-energy-production</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-23</t>
         </is>
       </c>
     </row>
@@ -3240,7 +3286,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/perpetua-resources-advances-construction-of-the-stibnite-gold-project-302787012.html)</t>
+          <t>https://www.prnewswire.com/news-releases/perpetua-resources-advances-construction-of-the-stibnite-gold-project-302787012.html</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -3277,7 +3323,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>[Silver Tiger Metals](https://silvertigermetals.com/news/2026/silver-tiger-metals-awards-engineering-procurement-and-construction-management-contract-and-provides-construction-update)</t>
+          <t>https://silvertigermetals.com/news/2026/silver-tiger-metals-awards-engineering-procurement-and-construction-management-contract-and-provides-construction-update</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -3314,7 +3360,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/vizsla-silver-awards-epcm-and-mine-design-contracts-for-the-development-of-the-panuco-silver-gold-project-302750621.html)</t>
+          <t>https://www.prnewswire.com/news-releases/vizsla-silver-awards-epcm-and-mine-design-contracts-for-the-development-of-the-panuco-silver-gold-project-302750621.html</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -3351,7 +3397,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>[Orla Mining](https://orlamining.com/news/orla-announces-results-of-updated-feasibility-study-for-south-railroad-project/)</t>
+          <t>https://orlamining.com/news/orla-announces-results-of-updated-feasibility-study-for-south-railroad-project/</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -3388,7 +3434,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>[Mining Weekly](https://www.miningweekly.com/article/minera-alamos-confirms-low-cost-near-term-mining-possible-at-copperstone-in-arizona-2026-05-28)</t>
+          <t>https://www.miningweekly.com/article/minera-alamos-confirms-low-cost-near-term-mining-possible-at-copperstone-in-arizona-2026-05-28</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -3425,7 +3471,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>[Wyoming News](https://www.wyomingnews.com/rawlinstimes/plans-move-forward-for-ck-gold-project-as-developers-target-2026-construction-start/article_b2bb147e-2f92-4ca2-bf86-fcc9983917a7.html)</t>
+          <t>https://www.wyomingnews.com/rawlinstimes/plans-move-forward-for-ck-gold-project-as-developers-target-2026-construction-start/article_b2bb147e-2f92-4ca2-bf86-fcc9983917a7.html</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -3462,7 +3508,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>[First Majestic](https://www.juniorminingnetwork.com/junior-miner-news/press-releases/1082-tsx/ag/206222-first-majestic-receives-construction-permits-for-santo-nino-and-navidad-advances-development-across-the-santa-elena-district.html)</t>
+          <t>https://www.juniorminingnetwork.com/junior-miner-news/press-releases/1082-tsx/ag/206222-first-majestic-receives-construction-permits-for-santo-nino-and-navidad-advances-development-across-the-santa-elena-district.html</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -3499,7 +3545,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>[SEC/Americas Gold and Silver](https://www.sec.gov/Archives/edgar/data/0001286973/000106299326002645/exhibit99-2.htm)</t>
+          <t>https://www.sec.gov/Archives/edgar/data/0001286973/000106299326002645/exhibit99-2.htm</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -3536,7 +3582,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>[Kitco](https://www.kitco.com/news/off-the-wire/2026-06-08/minera-frisco-restarts-two-mexico-mines-plans-new-silver-unit)</t>
+          <t>https://www.kitco.com/news/off-the-wire/2026-06-08/minera-frisco-restarts-two-mexico-mines-plans-new-silver-unit</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -3573,7 +3619,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/trilogy-metals-announces-publication-of-federal-and-state-permitting-schedule-for-arctic-project-establishing-defined-timeline-toward-a-record-of-decision-by-september-2028-302827083.html)</t>
+          <t>https://www.prnewswire.com/news-releases/trilogy-metals-announces-publication-of-federal-and-state-permitting-schedule-for-arctic-project-establishing-defined-timeline-toward-a-record-of-decision-by-september-2028-302827083.html</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -3610,7 +3656,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>[Northern Miner](https://www.northernminer.com/news/gogold-approved-to-build-227m-mine-in-mexico/1003891932/)</t>
+          <t>https://www.northernminer.com/news/gogold-approved-to-build-227m-mine-in-mexico/1003891932/</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -3647,7 +3693,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>[BNamericas](https://www.bnamericas.com/en/news/discovery-advances-permitting-financing-at-us606mn-cordero-in-mexico)</t>
+          <t>https://www.bnamericas.com/en/news/discovery-advances-permitting-financing-at-us606mn-cordero-in-mexico</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -3684,7 +3730,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>[Resource World](https://resourceworld.com/tocvan-ventures-eyes-mexican-gold-pour-by-q4-2026/)</t>
+          <t>https://resourceworld.com/tocvan-ventures-eyes-mexican-gold-pour-by-q4-2026/</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -3721,7 +3767,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>[Fresnillo plc](https://www.fresnilloplc.com/portfolio/exploration/orisyvo/)</t>
+          <t>https://www.fresnilloplc.com/portfolio/exploration/orisyvo/</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -3758,7 +3804,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>[Mining.com](https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/)</t>
+          <t>https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -3795,7 +3841,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>[Mining.com](https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/)</t>
+          <t>https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -3832,7 +3878,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>[Mining.com](https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/)</t>
+          <t>https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -3869,7 +3915,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>[IM Mining](https://im-mining.com/2026/06/29/metso-to-supply-additional-crushing-package-for-grupo-mexico-la-caridad-copper-concentrator/)</t>
+          <t>https://im-mining.com/2026/06/29/metso-to-supply-additional-crushing-package-for-grupo-mexico-la-caridad-copper-concentrator/</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -3906,7 +3952,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/05/21/3299182)</t>
+          <t>https://www.globenewswire.com/news-release/2026/05/21/3299182</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3943,7 +3989,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>[Mexico Business News](https://mexicobusiness.news/mining/news/grupo-mexicos-asarco-may-reopen-united-states)</t>
+          <t>https://mexicobusiness.news/mining/news/grupo-mexicos-asarco-may-reopen-united-states</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -3980,7 +4026,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>[Minera Alamos](https://mineraalamos.com/our-assets/cerro-de-oro-project/)</t>
+          <t>https://mineraalamos.com/our-assets/cerro-de-oro-project/</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -4017,7 +4063,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>[Global Mining Review](https://www.globalminingreview.com/mining/11022025/antler-copper-project-achieves-critical-federal-permitting-milestone/)</t>
+          <t>https://www.globalminingreview.com/mining/11022025/antler-copper-project-achieves-critical-federal-permitting-milestone/</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -4054,12 +4100,86 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>[BLM](https://www.blm.gov/press-release/blm-approves-lisbon-valley-copper-mine-expansion-utah)</t>
+          <t>https://www.blm.gov/press-release/blm-approves-lisbon-valley-copper-mine-expansion-utah</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
           <t>2026-07-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>South West Arkansas Lithium Project (Central Processing Facility)</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Sur de Arkansas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Smackover Lithium (JV Standard Lithium / Equinor)</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>S&amp;B Engineers and Constructors (EPCC); Hatch Ltd. (ingeniería de diseño/comisionamiento)</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Ingeniería de detalle/procura temprana (contrato EPCC otorgado, NTP limitado activo; FID esperada en 2026; planta diseñada para 22,500 tpa de carbonato de litio grado batería)</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>https://investingnews.com/smackover-lithium-announces-the-award-of-last-key-construction-contract-for-the-south-west-arkansas-project-ahead-of-final-investment-decision/</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Bagdad Mine Concentrator Expansion</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Yavapai County, Arizona, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Freeport-McMoRan</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Pre-FID/ingeniería avanzada (estudio para más que duplicar capacidad del concentrador, +200-250 Mlb/año cobre; capex incremental estimado ~US$3,500 millones bajo revisión; US$150M asignados en 2026 para ingeniería y obras tempranas; decisión de inversión esperada 2S-2026)</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/0000831259/000083125926000033/a2q2026exhibit991.htm</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
         </is>
       </c>
     </row>
@@ -4074,50 +4194,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -4151,7 +4271,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/vantage-breaks-ground-on-texas-gigawatt-data-center-campus-for-openai/)</t>
+          <t>https://www.datacenterdynamics.com/en/news/vantage-breaks-ground-on-texas-gigawatt-data-center-campus-for-openai/</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -4188,7 +4308,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>[Epoch AI](https://epoch.ai/publications/openai-stargate-where-the-us-sites-stand)</t>
+          <t>https://epoch.ai/publications/openai-stargate-where-the-us-sites-stand</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -4225,7 +4345,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/crusoe-tops-out-final-building-at-openai-stargate-data-center-campus-in-abilene-texas/)</t>
+          <t>https://www.datacenterdynamics.com/en/news/crusoe-tops-out-final-building-at-openai-stargate-data-center-campus-in-abilene-texas/</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -4262,7 +4382,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>[CNBC](https://www.cnbc.com/2026/06/22/chevron-cvx-microsoft-msft-natural-gas-data-center.html)</t>
+          <t>https://www.cnbc.com/2026/06/22/chevron-cvx-microsoft-msft-natural-gas-data-center.html</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -4299,7 +4419,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>[Gobierno de México](https://www.gob.mx/presidencia/prensa/plan-mexico-avanza-se-anuncia-inversion-de-4-mil-800-mdd-de-cloudhq-para-la-construccion-de-6-centros-de-datos-en-queretaro)</t>
+          <t>https://www.gob.mx/presidencia/prensa/plan-mexico-avanza-se-anuncia-inversion-de-4-mil-800-mdd-de-cloudhq-para-la-construccion-de-6-centros-de-datos-en-queretaro</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -4336,7 +4456,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>[UCS](https://www.ucs.org/about/news/judge-orders-meta-explain-new-gas-demand-hyperscale-louisiana-data-center)</t>
+          <t>https://www.ucs.org/about/news/judge-orders-meta-explain-new-gas-demand-hyperscale-louisiana-data-center</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -4373,7 +4493,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55305086/nv1-and-the-nevada-hyperscale-boom-vantage-data-centers-bets-3b-on-the-ai-future)</t>
+          <t>https://www.datacenterfrontier.com/site-selection/article/55305086/nv1-and-the-nevada-hyperscale-boom-vantage-data-centers-bets-3b-on-the-ai-future</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -4410,7 +4530,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/cloudburst-breaks-ground-on-gigawatt-scale-data-center-campus-in-texas/)</t>
+          <t>https://www.datacenterdynamics.com/en/news/cloudburst-breaks-ground-on-gigawatt-scale-data-center-campus-in-texas/</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -4447,7 +4567,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/prometheus-hyperscale-details-plans-for-dallas-data-center-campus/)</t>
+          <t>https://www.datacenterdynamics.com/en/news/prometheus-hyperscale-details-plans-for-dallas-data-center-campus/</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -4484,7 +4604,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>[Business Wire](https://www.businesswire.com/news/home/20260126236053/en/Pacifico-Energy-Secures-7.65-GW-Power-Generation-Permit-for-GW-Ranch-Project)</t>
+          <t>https://www.businesswire.com/news/home/20260126236053/en/Pacifico-Energy-Secures-7.65-GW-Power-Generation-Permit-for-GW-Ranch-Project</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -4521,7 +4641,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/amazon-looks-to-build-large-scale-data-center-campus-next-to-nuclear-plant-in-texas/)</t>
+          <t>https://www.datacenterdynamics.com/en/news/amazon-looks-to-build-large-scale-data-center-campus-next-to-nuclear-plant-in-texas/</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -4558,7 +4678,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>[Mexico News Daily](https://mexiconewsdaily.com/business/durango-data-center-fertilizer-plant-investment-fermaca/)</t>
+          <t>https://mexiconewsdaily.com/business/durango-data-center-fertilizer-plant-investment-fermaca/</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -4595,7 +4715,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/circe-energy-secures-2gw-of-natural-gas-capacity-for-west-texas-data-center-campus/)</t>
+          <t>https://www.datacenterdynamics.com/en/news/circe-energy-secures-2gw-of-natural-gas-capacity-for-west-texas-data-center-campus/</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -4612,7 +4732,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Santa Teresa, Doña Ana County, Nuevo México, EE.UU.</t>
+          <t>Santa Teresa/Sunland Park, Doña Ana County, Nuevo México, EE.UU.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -4627,197 +4747,197 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Construcción activa con riesgo regulatorio (Comisionado de Tierras de NM rechazó dos veces el derecho de vía en terrenos estatales para el gasoducto "Green Chile" de Energy Transfer, 15/16-jul-2026, tras la previa aprobación de BLM en tierra federal; meta de entrada en servicio ago-2026 en riesgo, posible retraso a 2027)</t>
+          <t>Construcción activa con riesgo regulatorio (Comisionada de Tierras de NM rechazó por segunda vez el derecho de vía en terrenos estatales para el gasoducto "Green Chile" de Energy Transfer, 14-jul-2026; NMED pospuso la decisión final sobre permisos de calidad de aire de las dos plantas de gas gemelas y programó audiencia pública para 19-oct-2026; meta de entrada en servicio ago-2026 en riesgo)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/new-mexico-regulators-reject-natural-gas-pipeline-for-oracles-25gw-project-jupiter-data-center/)</t>
+          <t>https://sourcenm.com/2026/07/16/new-mexico-land-commissioner-blocks-project-jupiter-related-pipeline-from-building-on-state-land/</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>New Era Energy &amp; Digital Hub</t>
+          <t>PowerPlay AI "Greater Abilene" Data Center</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Lea County, Nuevo México, EE.UU.</t>
+          <t>Área metropolitana de Abilene, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>New Era Energy &amp; Digital</t>
+          <t>PowerPlay AI (JV con socio Neocloud cotizado en Nasdaq, sin nombre público)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>IPP en proceso de RFP (aún sin seleccionar)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Planeación temprana (opción de terreno)</t>
+          <t>Ejecución activa post-adquisición de terreno (400MW behind-the-meter iniciales; arranque objetivo 2028)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>[PowerMag](https://www.powermag.com/nuclear-natural-gas-power-generation-planned-for-massive-new-mexico-data-center-site/)</t>
+          <t>https://www.prnewswire.com/news-releases/powerplay-ai-announces-400-mw-behind-the-meter-ai-data-center-development-in-greater-abilene-with-nasdaq-listed-neocloud-joint-venture-partner-302829610.html</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-23</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Texas Critical Data Centers (TCDC) Campus</t>
+          <t>Liberty Energy/PowerBridge "Alpha Digital Campus"</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Ector County (cerca de Odessa), Texas, EE.UU.</t>
+          <t>Condado de Reeves, Texas, EE.UU. (cerca del hub de gas Waha)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>New Era Energy &amp; Digital</t>
+          <t>PowerBridge LLC</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Stream Data Centers (JV vía LOI); Thunderhead Energy Solutions (carta de acuerdo no vinculante para ~250MW de gen. de gas behind-the-meter)</t>
+          <t>Liberty Power Innovations (subsidiaria de Liberty Energy, JV)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Ingeniería Fase Two (438 acres totales; permiso de aire en trámite; construcción total prevista en 2026, primeros 100MW dic-2026)</t>
+          <t>JV firmada/desarrollo temprano (~3,400 acres; primera fase &gt;300MW, primera entrega de energía prevista 4T2027; campus completo 2GW)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55289667/powering-ai-in-the-permian-texas-critical-data-centers-sustainable-energy-play)</t>
+          <t>https://www.datacenterdynamics.com/en/news/liberty-energy-powerbridge-form-jv-to-power-planned-2gw-data-center-in-west-texas/</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-23</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Stargate Lordstown</t>
+          <t>New Era Energy &amp; Digital Hub</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Lordstown, Ohio, EE.UU.</t>
+          <t>Lea County, Nuevo México, EE.UU.</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>OpenAI / Oracle / SoftBank</t>
+          <t>New Era Energy &amp; Digital</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>SB Energy (SoftBank)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Construcción (rompimiento de tierra)</t>
+          <t>Planeación temprana (opción de terreno)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>[OpenAI](https://openai.com/index/five-new-stargate-sites/)</t>
+          <t>https://www.powermag.com/nuclear-natural-gas-power-generation-planned-for-massive-new-mexico-data-center-site/</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Stargate Wisconsin</t>
+          <t>Texas Critical Data Centers (TCDC) Campus</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Wisconsin, EE.UU. (ubicación exacta no divulgada)</t>
+          <t>Ector County (cerca de Odessa), Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>OpenAI / Oracle / SoftBank</t>
+          <t>New Era Energy &amp; Digital</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Vantage Data Centers (en sociedad con Oracle)</t>
+          <t>Stream Data Centers (JV vía LOI); Thunderhead Energy Solutions (carta de acuerdo no vinculante para ~250MW de gen. de gas behind-the-meter)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Planeación/desarrollo temprano</t>
+          <t>Ingeniería Fase Two (438 acres totales; permiso de aire en trámite; construcción total prevista en 2026, primeros 100MW dic-2026)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>[OpenAI](https://openai.com/index/five-new-stargate-sites/)</t>
+          <t>https://www.datacenterfrontier.com/site-selection/article/55289667/powering-ai-in-the-permian-texas-critical-data-centers-sustainable-energy-play</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>AWS Región Digital Querétaro</t>
+          <t>Stargate Lordstown</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Querétaro, México</t>
+          <t>Lordstown, Ohio, EE.UU.</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Amazon Web Services (AWS)</t>
+          <t>OpenAI / Oracle / SoftBank</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>SB Energy (SoftBank)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Construcción/desarrollo (anunciado 2025, en curso)</t>
+          <t>Construcción (rompimiento de tierra)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>[Mexico News Daily](https://mexiconewsdaily.com/business/aws-invest-5b-mexico-data-region/)</t>
+          <t>https://openai.com/index/five-new-stargate-sites/</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -4829,106 +4949,106 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Stargate Michigan (Saline Barn Campus)</t>
+          <t>Stargate Wisconsin</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Saline Township, Michigan, EE.UU.</t>
+          <t>Wisconsin, EE.UU. (ubicación exacta no divulgada)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>OpenAI / Oracle (desarrollador: Related Digital)</t>
+          <t>OpenAI / Oracle / SoftBank</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Walbridge</t>
+          <t>Vantage Data Centers (en sociedad con Oracle)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Construcción</t>
+          <t>Planeación/desarrollo temprano</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/oracle-and-openai-start-construction-on-stargate-data-center-campus-in-saline-township-michigan/)</t>
+          <t>https://openai.com/index/five-new-stargate-sites/</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-14</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Applied Digital AI Factory Campuses (Polaris Forge, Ellendale/Harwood; nuevo campus Oliver County)</t>
+          <t>AWS Región Digital Querétaro</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>North Dakota, EE.UU.</t>
+          <t>Querétaro, México</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Applied Digital / Base Electron</t>
+          <t>Amazon Web Services (AWS)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Babcock &amp; Wilcox (generación); Siemens Energy (turbinas de vapor)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Construcción (Polaris Forge 1 Edificio 2 Fase 1 alcanzó Ready-for-Service 1-jul-2026, 175MW operativos; acuerdo de uso de caminos firmado 10-jul-2026 para tercer campus cerca de Center, Oliver County)</t>
+          <t>Construcción/desarrollo (anunciado 2025, en curso)</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>[Valley News Live](https://www.valleynewslive.com/2026/07/13/applied-digital-expands-north-dakota-eyes-oliver-county-third-data-center/)</t>
+          <t>https://mexiconewsdaily.com/business/aws-invest-5b-mexico-data-region/</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-14</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>AI-GDC / Cipre Holding "Green Data Center"</t>
+          <t>Stargate Michigan (Saline Barn Campus)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>San Pedro Garza García, Nuevo León, México</t>
+          <t>Saline Township, Michigan, EE.UU.</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>AI-GDC + Cipre Holding (Nvidia, socio tecnológico)</t>
+          <t>OpenAI / Oracle (desarrollador: Related Digital)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Walbridge</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Planeación/desarrollo temprano</t>
+          <t>Construcción</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>[Energy Magazine MX](https://energymagazine.mx/2026/01/el-data-center-verde-que-encendio-la-polemica-asi-sera-el-proyecto-de-ia-en-nuevo-leon-que-usara-tecnologia-de-nvidia/)</t>
+          <t>https://www.datacenterdynamics.com/en/news/oracle-and-openai-start-construction-on-stargate-data-center-campus-in-saline-township-michigan/</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -4940,54 +5060,54 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CleanArc Data Centers VA1 Campus</t>
+          <t>Applied Digital AI Factory Campuses (Polaris Forge, Ellendale/Harwood; nuevo campus Oliver County)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Caroline County, Virginia, EE.UU.</t>
+          <t>North Dakota, EE.UU.</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>CleanArc Data Centers</t>
+          <t>Applied Digital / Base Electron</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Babcock &amp; Wilcox (generación); Siemens Energy (turbinas de vapor)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Construcción</t>
+          <t>Construcción (Polaris Forge 1 Edificio 2 Fase 1 alcanzó Ready-for-Service 1-jul-2026, 175MW operativos; acuerdo de uso de caminos firmado 10-jul-2026 para tercer campus cerca de Center, Oliver County)</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>[Construction Dive](https://www.constructiondive.com/news/data-center-cleanarc-breaks-ground-virginia-campus/806489/)</t>
+          <t>https://www.valleynewslive.com/2026/07/13/applied-digital-expands-north-dakota-eyes-oliver-county-third-data-center/</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Joule Energy and Data Center Campus</t>
+          <t>AI-GDC / Cipre Holding "Green Data Center"</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Millard County (Holden), Utah, EE.UU.</t>
+          <t>San Pedro Garza García, Nuevo León, México</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Joule Capital Partners</t>
+          <t>AI-GDC + Cipre Holding (Nvidia, socio tecnológico)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -4997,12 +5117,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Construcción</t>
+          <t>Planeación/desarrollo temprano</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>[KSL](https://www.ksl.com/article/51402125/groundbreaking-for-new-millard-county-artificial-intelligence-data-center)</t>
+          <t>https://energymagazine.mx/2026/01/el-data-center-verde-que-encendio-la-polemica-asi-sera-el-proyecto-de-ia-en-nuevo-leon-que-usara-tecnologia-de-nvidia/</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -5014,17 +5134,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Amazon Montgomery County Campus</t>
+          <t>CleanArc Data Centers VA1 Campus</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>New Florence, Montgomery County, Missouri, EE.UU.</t>
+          <t>Caroline County, Virginia, EE.UU.</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>CleanArc Data Centers</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -5034,12 +5154,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Anuncio/permisos</t>
+          <t>Construcción</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>[Governor.mo.gov](https://governor.mo.gov/press-releases/archive/amazon-investing-10-billion-montgomery-county)</t>
+          <t>https://www.constructiondive.com/news/data-center-cleanarc-breaks-ground-virginia-campus/806489/</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -5051,17 +5171,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Google Montgomery County Campus</t>
+          <t>Joule Energy and Data Center Campus</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>New Florence, Montgomery County, Missouri, EE.UU.</t>
+          <t>Millard County (Holden), Utah, EE.UU.</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Joule Capital Partners</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -5071,12 +5191,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Anuncio/permisos</t>
+          <t>Construcción</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>[STLPR](https://www.stlpr.org/government-politics-issues/2026-05-21/missouri-governor-google-announce-15-billion-data-center-montgomery-county)</t>
+          <t>https://www.ksl.com/article/51402125/groundbreaking-for-new-millard-county-artificial-intelligence-data-center</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -5088,17 +5208,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Big Digital Energy / 10NetZero AI Datacenter Campus</t>
+          <t>Amazon Montgomery County Campus</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Hood County, Texas, EE.UU.</t>
+          <t>New Florence, Montgomery County, Missouri, EE.UU.</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Big Digital Energy + 10NetZero (JV)</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -5108,12 +5228,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Planeación/adquisición de sitio</t>
+          <t>Anuncio/permisos</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/06/3322404/0/en/big-digital-energy-announces-partnership-with-10netzero-to-acquire-power-ready-hood-county-texas-site-for-ai-datacenter-development.html)</t>
+          <t>https://governor.mo.gov/press-releases/archive/amazon-investing-10-billion-montgomery-county</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -5125,54 +5245,54 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Williams "Project Socrates"</t>
+          <t>Google Montgomery County Campus</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>New Albany, Ohio, EE.UU.</t>
+          <t>New Florence, Montgomery County, Missouri, EE.UU.</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Meta (vía Sidecat, LLC)</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Williams Companies / Will-Power</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Construcción (financiamiento de USD 5.34 mil millones de Blackstone/Apollo/KKR cerrado jul-2026 por 49% de participación no controladora en 5 proyectos Power Innovation de Williams; Socrates Norte/Sur, 400MW combinados, en servicio 3T/4T2026)</t>
+          <t>Anuncio/permisos</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/)</t>
+          <t>https://www.stlpr.org/government-politics-issues/2026-05-21/missouri-governor-google-announce-15-billion-data-center-montgomery-county</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-15</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Meta El Paso Campus (expansión)</t>
+          <t>Big Digital Energy / 10NetZero AI Datacenter Campus</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>El Paso, Texas, EE.UU.</t>
+          <t>Hood County, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>Big Digital Energy + 10NetZero (JV)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -5182,12 +5302,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Permisos</t>
+          <t>Planeación/adquisición de sitio</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/meta-files-to-expand-campus-in-el-paso-texas-with-12-new-buildings/)</t>
+          <t>https://www.globenewswire.com/news-release/2026/07/06/3322404/0/en/big-digital-energy-announces-partnership-with-10netzero-to-acquire-power-ready-hood-county-texas-site-for-ai-datacenter-development.html</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -5199,143 +5319,143 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>SB Energy/SoftBank PORTS Technology Campus</t>
+          <t>Williams "Project Socrates"</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Pike County, Ohio, EE.UU.</t>
+          <t>New Albany, Ohio, EE.UU.</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>SB Energy (SoftBank) / DOE / AEP Ohio</t>
+          <t>Meta (vía Sidecat, LLC)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Williams Companies / Will-Power</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Planeación/desarrollo temprano</t>
+          <t>Construcción (financiamiento de USD 5.34 mil millones de Blackstone/Apollo/KKR cerrado jul-2026 por 49% de participación no controladora en 5 proyectos Power Innovation de Williams; Socrates Norte/Sur, 400MW combinados, en servicio 3T/4T2026)</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/softbank-eyes-10gw-data-center-at-former-doe-nuclear-enrichment-site-in-ohio/)</t>
+          <t>https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Williams "Apollo" Power Generation Project</t>
+          <t>Meta El Paso Campus (expansión)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Wood County (Middleton Township), Ohio, EE.UU.</t>
+          <t>El Paso, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Meta Platforms (planta: Will-Power OH, LLC / Williams Companies)</t>
+          <t>Meta</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Williams Companies</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Construcción (aprobado por Ohio Power Siting Board feb-2026; financiamiento de USD 5.34 mil millones cerrado con Blackstone/Apollo/KKR jul-2026)</t>
+          <t>Permisos</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/)</t>
+          <t>https://www.datacenterdynamics.com/en/news/meta-files-to-expand-campus-in-el-paso-texas-with-12-new-buildings/</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-15</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Williams "Aquila" Power Project</t>
+          <t>SB Energy/SoftBank PORTS Technology Campus</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Utah, EE.UU. (condado no revelado)</t>
+          <t>Pike County, Ohio, EE.UU.</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Cliente de centro de datos no revelado (planta: Williams Companies)</t>
+          <t>SB Energy (SoftBank) / DOE / AEP Ohio</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Williams Companies</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Construcción/desarrollo (520MW; entrada en servicio prevista H1 2027; parte del financiamiento de USD 5.34 mil millones de Blackstone/Apollo/KKR)</t>
+          <t>Planeación/desarrollo temprano</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>[Williams Companies](https://www.williams.com/2026/07/13/williams-announces-5-34-billion-investment-in-power-innovation-joint-venture-from-blackstone/)</t>
+          <t>https://www.datacenterdynamics.com/en/news/softbank-eyes-10gw-data-center-at-former-doe-nuclear-enrichment-site-in-ohio/</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-15</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CleanCore/HST Technologies West Texas Data Center Campus</t>
+          <t>Williams "Apollo" Power Generation Project</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>West Texas, EE.UU. (condado no revelado)</t>
+          <t>Wood County (Middleton Township), Ohio, EE.UU.</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>CleanCore Solutions (ZONE) / HST Technologies (JV)</t>
+          <t>Meta Platforms (planta: Will-Power OH, LLC / Williams Companies)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Williams Companies</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Cierre de transacción (200MW fase inicial, jul-2026; expansión a 500MW+ prevista para 2030)</t>
+          <t>Construcción (aprobado por Ohio Power Siting Board feb-2026; financiamiento de USD 5.34 mil millones cerrado con Blackstone/Apollo/KKR jul-2026)</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/cleancore-solutions-zone-announces-closing-of-first-data-center-project-establishing-its-critical-infrastructure-buildout-for-the-ai-economy-302821421.html)</t>
+          <t>https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -5347,54 +5467,54 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Crusoe/Tallgrass AI Data Center Campus (Project Jade)</t>
+          <t>Williams "Aquila" Power Project</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Condado de Laramie, Wyoming, EE.UU.</t>
+          <t>Utah, EE.UU. (condado no revelado)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Crusoe Energy / Tallgrass</t>
+          <t>Cliente de centro de datos no revelado (planta: Williams Companies)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Williams Companies</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Desarrollo PAUSADO (Crusoe pausó actividades en jun-2026 a solicitud de su cliente; afecta también la generación de gas asociada BFC Power/Cheyenne Power Hub; aprobado ene-2026, 1.8GW inicial escalable a 10GW)</t>
+          <t>Construcción/desarrollo (520MW; entrada en servicio prevista H1 2027; parte del financiamiento de USD 5.34 mil millones de Blackstone/Apollo/KKR)</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>[Bloomberg](https://www.bloomberg.com/news/articles/2026-06-09/crusoe-touts-5-gigawatts-worth-of-data-centers-deals-pauses-wyoming-site)</t>
+          <t>https://www.williams.com/2026/07/13/williams-announces-5-34-billion-investment-in-power-innovation-joint-venture-from-blackstone/</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-16</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Core Scientific Pecos Campus (expansión IA)</t>
+          <t>CleanCore/HST Technologies West Texas Data Center Campus</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Pecos, Reeves County, Texas, EE.UU.</t>
+          <t>West Texas, EE.UU. (condado no revelado)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Core Scientific</t>
+          <t>CleanCore Solutions (ZONE) / HST Technologies (JV)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -5404,12 +5524,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Construcción (primera nave de datos en construcción vertical; expansión a 1.5GW bruto; primera capacidad prevista inicios de 2027)</t>
+          <t>Cierre de transacción (200MW fase inicial, jul-2026; expansión a 500MW+ prevista para 2030)</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>[HPCwire](https://www.hpcwire.com/off-the-wire/core-scientific-plans-expansion-to-1-5gw-of-gross-power-at-pecos-texas-campus/)</t>
+          <t>https://www.prnewswire.com/news-releases/cleancore-solutions-zone-announces-closing-of-first-data-center-project-establishing-its-critical-infrastructure-buildout-for-the-ai-economy-302821421.html</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -5421,17 +5541,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Stratos Project / Wonder Valley</t>
+          <t>Crusoe/Tallgrass AI Data Center Campus (Project Jade)</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Condado de Box Elder (Hansel Valley), Utah, EE.UU.</t>
+          <t>Condado de Laramie, Wyoming, EE.UU.</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>O'Leary Digital (Kevin O'Leary)</t>
+          <t>Crusoe Energy / Tallgrass</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -5441,71 +5561,71 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Permisos/desarrollo temprano (aprobado por comisión del condado may-2026; hasta 9GW planeados; alimentado por gasoducto Ruby; obras tempranas previstas otoño 2026)</t>
+          <t>Desarrollo PAUSADO (Crusoe pausó actividades en jun-2026 a solicitud de su cliente; afecta también la generación de gas asociada BFC Power/Cheyenne Power Hub; aprobado ene-2026, 1.8GW inicial escalable a 10GW)</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>[Utah News Dispatch](https://utahnewsdispatch.com/2026/05/19/renderings-show-massive-data-center-box-elder-utah-permits-could-take-years/)</t>
+          <t>https://www.bloomberg.com/news/articles/2026-06-09/crusoe-touts-5-gigawatts-worth-of-data-centers-deals-pauses-wyoming-site</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Fermi America Project Matador</t>
+          <t>Core Scientific Pecos Campus (expansión IA)</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Carson County (Amarillo), Texas, EE.UU.</t>
+          <t>Pecos, Reeves County, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Fermi America</t>
+          <t>Core Scientific</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Primoris Services Corporation (balance of plant, turbinas de gas)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Construcción (excavación de isla de turbinas completada; EPC firmado)</t>
+          <t>Construcción (primera nave de datos en construcción vertical; expansión a 1.5GW bruto; primera capacidad prevista inicios de 2027)</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/fermi-selects-primoris-services-corporation-to-engineer-and-construct-balance-of-plant-for-first-six-sgt-800-gas-turbines-of-phase-one-power-buildout-302814505.html)</t>
+          <t>https://www.hpcwire.com/off-the-wire/core-scientific-plans-expansion-to-1-5gw-of-gross-power-at-pecos-texas-campus/</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-16</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>NextEra Texas Power Generation Hub</t>
+          <t>Stratos Project / Wonder Valley</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Anderson County, Texas, EE.UU.</t>
+          <t>Condado de Box Elder (Hansel Valley), Utah, EE.UU.</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>NextEra Energy Resources</t>
+          <t>O'Leary Digital (Kevin O'Leary)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -5515,71 +5635,71 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Aprobado/planeación (5.2GW a gas; primera fase en línea 2028; data center asociado aún no contratado)</t>
+          <t>Permisos/desarrollo temprano (aprobado por comisión del condado may-2026; hasta 9GW planeados; alimentado por gasoducto Ruby; obras tempranas previstas otoño 2026)</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>[KLTV](https://www.kltv.com/2026/03/20/president-trump-approves-16-billion-natural-gas-generator-be-installed-anderson-county/)</t>
+          <t>https://utahnewsdispatch.com/2026/05/19/renderings-show-massive-data-center-box-elder-utah-permits-could-take-years/</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-16</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Mon Power/FirstEnergy Gas Plant (Maidsville Energy Center)</t>
+          <t>Fermi America Project Matador</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Monongalia County, Virginia Occidental, EE.UU.</t>
+          <t>Carson County (Amarillo), Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Mon Power (FirstEnergy)</t>
+          <t>Fermi America</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Primoris Services Corporation (balance of plant, turbinas de gas)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Planeación/regulatorio (USD 2.4 mil millones, 1,200MW; audiencia probatoria concluida 16/17-jul-2026 ante PSC; Mon Power confirmó pláticas con 3 desarrolladores de data centers no identificados; op. comercial prevista 31-dic-2031)</t>
+          <t>Construcción (excavación de isla de turbinas completada; EPC firmado)</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>[WV MetroNews](https://wvmetronews.com/2026/07/16/mon-power-president-says-data-centers-will-end-up-paying-for-natural-gas-powered-power-plant/)</t>
+          <t>https://www.prnewswire.com/news-releases/fermi-selects-primoris-services-corporation-to-engineer-and-construct-balance-of-plant-for-first-six-sgt-800-gas-turbines-of-phase-one-power-buildout-302814505.html</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-17</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>IEP Greene County Data Center &amp; Power Plant</t>
+          <t>NextEra Texas Power Generation Hub</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Greene County, Pensilvania, EE.UU.</t>
+          <t>Anderson County, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>International Electric Power</t>
+          <t>NextEra Energy Resources</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -5589,12 +5709,12 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Permisos (aprobación preliminar de desarrollo de terreno; planta CCGT de 944MW; COD previsto Q1 2029)</t>
+          <t>Aprobado/planeación (5.2GW a gas; primera fase en línea 2028; data center asociado aún no contratado)</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>[Utility Dive](https://www.utilitydive.com/news/iep-plans-944-mw-behind-the-meter-gas-plant-in-pennsylvania-to-power-data-c/758830/)</t>
+          <t>https://www.kltv.com/2026/03/20/president-trump-approves-16-billion-natural-gas-generator-be-installed-anderson-county/</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -5606,17 +5726,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>AWS "Project Eagle"</t>
+          <t>Mon Power/FirstEnergy Gas Plant (Maidsville Energy Center)</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Boling, Wharton County, Texas, EE.UU. (SO de Houston)</t>
+          <t>Monongalia County, Virginia Occidental, EE.UU.</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Amazon Web Services</t>
+          <t>Mon Power (FirstEnergy)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -5626,34 +5746,34 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Permisos (presentados ante TDLR; construcción de 4 edificios, USD 1.2 mil millones, inicia 1-ago-2026)</t>
+          <t>Planeación/regulatorio (USD 2.4 mil millones, 1,200MW; audiencia probatoria concluida 16/17-jul-2026 ante PSC; Mon Power confirmó pláticas con 3 desarrolladores de data centers no identificados; op. comercial prevista 31-dic-2031)</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/aws-files-for-12bn-data-center-campus-outside-houston-texas/)</t>
+          <t>https://wvmetronews.com/2026/07/16/mon-power-president-says-data-centers-will-end-up-paying-for-natural-gas-powered-power-plant/</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Crusoe/Lancium Childress Data Center Campus</t>
+          <t>IEP Greene County Data Center &amp; Power Plant</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Condado de Childress, Texas, EE.UU.</t>
+          <t>Greene County, Pensilvania, EE.UU.</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Crusoe (operador) / Lancium (infraestructura energética)</t>
+          <t>International Electric Power</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -5663,49 +5783,49 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Anuncio/planeación (construcción prevista 3T2026; campus de 1.0-1.4GW)</t>
+          <t>Permisos (aprobación preliminar de desarrollo de terreno; planta CCGT de 944MW; COD previsto Q1 2029)</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>[Crusoe](https://www.crusoe.ai/resources/newsroom/crusoe-and-lancium-announce-1-gigawatt-ai-data-center-campus-in-childress-texas)</t>
+          <t>https://www.utilitydive.com/news/iep-plans-944-mw-behind-the-meter-gas-plant-in-pennsylvania-to-power-data-c/758830/</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-17</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Williams "Neo" Power Innovation Project</t>
+          <t>AWS "Project Eagle"</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Ohio, EE.UU. (sitio exacto no revelado)</t>
+          <t>Boling, Wharton County, Texas, EE.UU. (SO de Houston)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Cliente de centro de datos no revelado</t>
+          <t>Amazon Web Services</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Williams Companies</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Planeación/desarrollo (682MW; en servicio 2S2028; parte del financiamiento de USD 5.34 mil millones de Blackstone/Apollo/KKR)</t>
+          <t>Permisos (presentados ante TDLR; construcción de 4 edificios, USD 1.2 mil millones, inicia 1-ago-2026)</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/)</t>
+          <t>https://www.datacenterdynamics.com/en/news/aws-files-for-12bn-data-center-campus-outside-houston-texas/</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -5717,106 +5837,106 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Williams "Socrates the Younger" Power Innovation Project</t>
+          <t>Crusoe/Lancium Childress Data Center Campus</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>New Albany, Ohio, EE.UU. (adyacente a Project Socrates)</t>
+          <t>Condado de Childress, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Meta Platforms (vía Sidecat, LLC)</t>
+          <t>Crusoe (operador) / Lancium (infraestructura energética)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Williams Companies</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Construcción (aprobada por Ohio Power Siting Board 9-jun-2026; 340MW; en servicio 2S2028; parte del financiamiento de USD 5.34 mil millones de Blackstone/Apollo/KKR)</t>
+          <t>Anuncio/planeación (construcción prevista 3T2026; campus de 1.0-1.4GW)</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>[PowerMag](https://www.powermag.com/new-200-mw-gas-fired-plant-in-ohio-will-power-meta-data-center/)</t>
+          <t>https://www.crusoe.ai/resources/newsroom/crusoe-and-lancium-announce-1-gigawatt-ai-data-center-campus-in-childress-texas</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Crusoe/Google "Goodnight Campus"</t>
+          <t>Williams "Neo" Power Innovation Project</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Condado de Armstrong (Claude), Texas, EE.UU.</t>
+          <t>Ohio, EE.UU. (sitio exacto no revelado)</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Google (negociación de arrendamiento) / Crusoe Energy (desarrollador)</t>
+          <t>Cliente de centro de datos no revelado</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Williams Companies</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Construcción (4 de 7 edificios en obra; campus de USD 29 mil millones, ~1,030MW; planta de gas propia de 933MW en trámite ante TCEQ, respaldada por parque eólico Goodnight de 265.5MW)</t>
+          <t>Planeación/desarrollo (682MW; en servicio 2S2028; parte del financiamiento de USD 5.34 mil millones de Blackstone/Apollo/KKR)</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>[Aterio](https://www.aterio.io/blog/crusoe-launches-usd29b-goodnight-campus-in-claude-mirroring-openai-s-stargate)</t>
+          <t>https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>VoltaGrid/Serverfarm Covington</t>
+          <t>Williams "Socrates the Younger" Power Innovation Project</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Condado de Newton (Covington), Georgia, EE.UU.</t>
+          <t>New Albany, Ohio, EE.UU. (adyacente a Project Socrates)</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Serverfarm</t>
+          <t>Meta Platforms (vía Sidecat, LLC)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>VoltaGrid (planta de energía "pop-up", 33 motores de combustión interna)</t>
+          <t>Williams Companies</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Construcción DETENIDA (orden de suspensión de la agencia ambiental de Georgia -EPD- por construir sin permisos, 2-jul-2026)</t>
+          <t>Construcción (aprobada por Ohio Power Siting Board 9-jun-2026; 340MW; en servicio 2S2028; parte del financiamiento de USD 5.34 mil millones de Blackstone/Apollo/KKR)</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>[AJC](https://www.ajc.com/business/2026/07/officials-order-georgia-data-centers-pop-up-power-plant-to-halt-construction/)</t>
+          <t>https://www.powermag.com/new-200-mw-gas-fired-plant-in-ohio-will-power-meta-data-center/</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -5828,17 +5948,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Stark Power/Sagebrush Infrastructure Partners (SAGE)</t>
+          <t>Crusoe/Google "Goodnight Campus"</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Múltiples sitios, EE.UU. Central (ubicaciones no reveladas)</t>
+          <t>Condado de Armstrong (Claude), Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Stark Power (adquirió SAGE, 8-jun-2026)</t>
+          <t>Google (negociación de arrendamiento) / Crusoe Energy (desarrollador)</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -5848,12 +5968,12 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Adquisición/planeación temprana (portafolio de 5 campus hyperscale con generación de gas co-localizada, 5.6GW agregados)</t>
+          <t>Construcción (4 de 7 edificios en obra; campus de USD 29 mil millones, ~1,030MW; planta de gas propia de 933MW en trámite ante TCEQ, respaldada por parque eólico Goodnight de 265.5MW)</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/stark-power-lands-56gw-data-center-development-portfolio-in-sagebrush-acquisition/)</t>
+          <t>https://www.aterio.io/blog/crusoe-launches-usd29b-goodnight-campus-in-claude-mirroring-openai-s-stargate</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -5865,106 +5985,106 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Homer City Energy Campus</t>
+          <t>VoltaGrid/Serverfarm Covington</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Condado de Indiana, Pensilvania, EE.UU.</t>
+          <t>Condado de Newton (Covington), Georgia, EE.UU.</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Homer City Redevelopment (HCR)</t>
+          <t>Serverfarm</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Kiewit Power Constructors Co.; turbinas GE Vernova (7x 7HA.02 con capacidad de hidrógeno)</t>
+          <t>VoltaGrid (planta de energía "pop-up", 33 motores de combustión interna)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Construcción (excavación/demolición completadas; planta de gas de 4.5GW, la más grande planeada en EE.UU.; primeras entregas de turbinas 2026, operación comercial 2027)</t>
+          <t>Construcción DETENIDA (orden de suspensión de la agencia ambiental de Georgia -EPD- por construir sin permisos, 2-jul-2026)</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55281341/pennsylvanias-homer-city-energy-campus-a-brownfield-transformed-for-data-center-innovation)</t>
+          <t>https://www.ajc.com/business/2026/07/officials-order-georgia-data-centers-pop-up-power-plant-to-halt-construction/</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-21</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Nebius Vineland AI Data Center Campus</t>
+          <t>Stark Power/Sagebrush Infrastructure Partners (SAGE)</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Vineland, Nueva Jersey, EE.UU.</t>
+          <t>Múltiples sitios, EE.UU. Central (ubicaciones no reveladas)</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Nebius Group (cómputo entregado a Microsoft bajo acuerdo de USD 17.4 mil millones)</t>
+          <t>Stark Power (adquirió SAGE, 8-jun-2026)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>No especificado (motores reciprocantes de gas Bergen, ~30 unidades)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Construcción/Permisos (planta de gas de hasta 400MW enfrenta retrasos por Ley de Justicia Ambiental de NJ; meta de entrega nov-2026 en riesgo)</t>
+          <t>Adquisición/planeación temprana (portafolio de 5 campus hyperscale con generación de gas co-localizada, 5.6GW agregados)</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>[Data Center Knowledge](https://www.datacenterknowledge.com/data-center-site-selection/nebius-plans-300-mw-data-center-in-new-jersey-amid-us-expansion)</t>
+          <t>https://www.datacenterdynamics.com/en/news/stark-power-lands-56gw-data-center-development-portfolio-in-sagebrush-acquisition/</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-21</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>TerraVolt Infrastructure AI Data Center Campus</t>
+          <t>Homer City Energy Campus</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Sureste de Idaho, EE.UU. (sobre gasoducto Northwest Natural Gas Pipeline)</t>
+          <t>Condado de Indiana, Pensilvania, EE.UU.</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>TerraVolt Infrastructure, Inc. (subsidiaria de CalEthos, Inc.)</t>
+          <t>Homer City Redevelopment (HCR)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Kiewit Power Constructors Co.; turbinas GE Vernova (7x 7HA.02 con capacidad de hidrógeno)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Ingeniería/Planeación (acuerdo de suministro de gas natural firmado, 55,000 MMBtu/día, para planta on-site de 200-240MW)</t>
+          <t>Construcción (excavación/demolición completadas; planta de gas de 4.5GW, la más grande planeada en EE.UU.; primeras entregas de turbinas 2026, operación comercial 2027)</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/terravolt-inks-natural-gas-supply-deal-for-onsite-power-plant-at-planned-data-center-campus-in-idaho/)</t>
+          <t>https://www.datacenterfrontier.com/site-selection/article/55281341/pennsylvanias-homer-city-energy-campus-a-brownfield-transformed-for-data-center-innovation</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -5976,35 +6096,109 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
+          <t>Nebius Vineland AI Data Center Campus</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Vineland, Nueva Jersey, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Nebius Group (cómputo entregado a Microsoft bajo acuerdo de USD 17.4 mil millones)</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>No especificado (motores reciprocantes de gas Bergen, ~30 unidades)</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Construcción/Permisos (planta de gas de hasta 400MW enfrenta retrasos por Ley de Justicia Ambiental de NJ; meta de entrega nov-2026 en riesgo)</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>https://www.datacenterknowledge.com/data-center-site-selection/nebius-plans-300-mw-data-center-in-new-jersey-amid-us-expansion</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>TerraVolt Infrastructure AI Data Center Campus</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Sureste de Idaho, EE.UU. (sobre gasoducto Northwest Natural Gas Pipeline)</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>TerraVolt Infrastructure, Inc. (subsidiaria de CalEthos, Inc.)</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Ingeniería/Planeación (acuerdo de suministro de gas natural firmado, 55,000 MMBtu/día, para planta on-site de 200-240MW)</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>https://www.datacenterdynamics.com/en/news/terravolt-inks-natural-gas-supply-deal-for-onsite-power-plant-at-planned-data-center-campus-in-idaho/</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
           <t>CyrusOne SAT14A</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr">
+      <c r="B54" t="inlineStr">
         <is>
           <t>Castroville, San Antonio, Texas, EE.UU.</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="C54" t="inlineStr">
         <is>
           <t>CyrusOne (sin arrendatario asignado aún)</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>No especificado</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
         <is>
           <t>Ingeniería/Permisos (6to campus en San Antonio, 11vo en Texas; USD 500 millones, 460,000 pies²; inicio de construcción previsto dic-2026)</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/cyrusone-announces-sixth-data-center-campus-in-san-antonio-texas/)</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>https://www.datacenterdynamics.com/en/news/cyrusone-announces-sixth-data-center-campus-in-san-antonio-texas/</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
         <is>
           <t>2026-07-22</t>
         </is>

</xml_diff>

<commit_message>
Agregar 12 proyectos nuevos y 3 cambios de fase (2026-07-24)
Petroquímica: Wabash Low-Carbon Ammonia Project.
LNG: Corpus Christi Stage 4, Freeport LNG Train 4, Gasoducto Coatzacoalcos II;
actualizaciones de fase en Golden Pass LNG y ST LNG Deepwater Port.
Mining: Elk Creek Critical Minerals, Goldfield Project, Cactus Mine, Doby George
Gold Project, Metates Project.
Data Centers: EdgeConneX PowerConneX New Albany, xAI Colossus 2/3 (Southaven),
Applied Digital Delta Forge 1; actualización de fase en Fermi America Project Matador.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FbFqSFuzuNzfzdxHWN1Thd
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -425,16 +425,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
     <col width="55" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -502,7 +502,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://newsroom.fluor.com/news-releases/news-details/2026/Fluor-Awarded-Contract-to-Engineer-and-Design-the-America-First-Refining-Facility-in-Brownsville-Texas/default.aspx</t>
+          <t>[Fluor newsroom](https://newsroom.fluor.com/news-releases/news-details/2026/Fluor-Awarded-Contract-to-Engineer-and-Design-the-America-First-Refining-Facility-in-Brownsville-Texas/default.aspx)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -539,7 +539,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://allstreaminsiders.com/us-exxonmobil-may-build-cracker-pe-plant-in-texas-with-an-8-6-billion-investment/</t>
+          <t>[AllStream Insiders](https://allstreaminsiders.com/us-exxonmobil-may-build-cracker-pe-plant-in-texas-with-an-8-6-billion-investment/)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -576,7 +576,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.bicmagazine.com/departments/operations/cpchem-golden-triangle-polymers-facility-startup-phase/</t>
+          <t>[BIC Magazine](https://www.bicmagazine.com/departments/operations/cpchem-golden-triangle-polymers-facility-startup-phase/)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -613,7 +613,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://constructionfront.com/2025-04-13-technip-energies-to-deliver-blue-point-worlds-largest-low-carbon-ammonia-facility-in-louisiana/</t>
+          <t>[Construction Front](https://constructionfront.com/2025-04-13-technip-energies-to-deliver-blue-point-worlds-largest-low-carbon-ammonia-facility-in-louisiana/)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -650,7 +650,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://eastdaley.com/media-and-news/the-race-is-on-to-build-permian-processing</t>
+          <t>[East Daley](https://eastdaley.com/media-and-news/the-race-is-on-to-build-permian-processing)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -687,7 +687,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.techint.com/en/our-projects/dos-bocas-refinery</t>
+          <t>[Techint](https://www.techint.com/en/our-projects/dos-bocas-refinery)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -724,7 +724,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://www.ogj.com/refining-processing/refining/optimization/article/17279334/pemex-to-proceed-with-dos-bocas-refinery-project</t>
+          <t>[OGJ](https://www.ogj.com/refining-processing/refining/optimization/article/17279334/pemex-to-proceed-with-dos-bocas-refinery-project)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -761,7 +761,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://forbes.com.mx/pemex-invertira-5300-millones-de-dolares-para-reactivar-la-industria-petroquimica/</t>
+          <t>[Forbes México](https://forbes.com.mx/pemex-invertira-5300-millones-de-dolares-para-reactivar-la-industria-petroquimica/)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -798,7 +798,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://forbes.com.mx/pemex-invertira-5300-millones-de-dolares-para-reactivar-la-industria-petroquimica/</t>
+          <t>[Forbes México](https://forbes.com.mx/pemex-invertira-5300-millones-de-dolares-para-reactivar-la-industria-petroquimica/)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -835,7 +835,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://forbes.com.mx/asi-es-la-inversion-de-1553-mdd-por-parte-de-pemex-en-una-planta-de-fertilizantes-en-veracruz/</t>
+          <t>[Forbes México](https://forbes.com.mx/asi-es-la-inversion-de-1553-mdd-por-parte-de-pemex-en-una-planta-de-fertilizantes-en-veracruz/)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -872,7 +872,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://tribuna.com.mx/mexico/2026/06/05/sheinbaum-anuncia-inversion-de-93-mil-mdp-para-reactivar-la-industria-petroquimica-y-de-fertilizantes-en-veracruz_560837/</t>
+          <t>[Tribuna](https://tribuna.com.mx/mexico/2026/06/05/sheinbaum-anuncia-inversion-de-93-mil-mdp-para-reactivar-la-industria-petroquimica-y-de-fertilizantes-en-veracruz_560837/)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -909,7 +909,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://www.pv-magazine-mexico.com/2026/04/28/inician-en-sinaloa-la-construccion-de-la-mayor-planta-de-metanol-ultrabajo-en-carbono-a-partir-de-hidrogeno-verde/</t>
+          <t>[PV Magazine México](https://www.pv-magazine-mexico.com/2026/04/28/inician-en-sinaloa-la-construccion-de-la-mayor-planta-de-metanol-ultrabajo-en-carbono-a-partir-de-hidrogeno-verde/)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://www.h2-view.com/story/first-ammonia-project-on-track-for-2026-fid-despite-topsoe-deal-collapse/2138792.article/</t>
+          <t>[H2 View](https://www.h2-view.com/story/first-ammonia-project-on-track-for-2026-fid-despite-topsoe-deal-collapse/2138792.article/)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -983,7 +983,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://www.debate.com.mx/economia/secretaria-de-economia-complejo-de-amoniaco-en-topolobampo-prioritario-para-el-gobierno-de-mexico-20260713-0092.html</t>
+          <t>[Debate](https://www.debate.com.mx/economia/secretaria-de-economia-complejo-de-amoniaco-en-topolobampo-prioritario-para-el-gobierno-de-mexico-20260713-0092.html)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1020,7 +1020,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://www.icis.com/explore/resources/news/2025/11/13/11155109/lake-charles-methanol-ii-awards-feed-fid-expected-in-q2-2026/</t>
+          <t>[ICIS](https://www.icis.com/explore/resources/news/2025/11/13/11155109/lake-charles-methanol-ii-awards-feed-fid-expected-in-q2-2026/)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://diariodelistmo.com/nacional/este-es-el-avance-que-lleva-la-planta-coquizadora-en-la-refineria-de-salina-cruz/50642321</t>
+          <t>[Diario del Istmo](https://diariodelistmo.com/nacional/este-es-el-avance-que-lleva-la-planta-coquizadora-en-la-refineria-de-salina-cruz/50642321)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1094,7 +1094,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://www.hydrocarbonengineering.com/petrochemicals/06032026/shintech-announces-us34-billion-at-louisiana-petrochemicals-complex/</t>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/petrochemicals/06032026/shintech-announces-us34-billion-at-louisiana-petrochemicals-complex/)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1131,7 +1131,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://www.alchempro.com/news/chemicals-news/ineos-backs-1-7-bn-low-carbon-methanol-project-in-texas-city-310108-newsdetails.htm</t>
+          <t>[Alchempro](https://www.alchempro.com/news/chemicals-news/ineos-backs-1-7-bn-low-carbon-methanol-project-in-texas-city-310108-newsdetails.htm)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1168,7 +1168,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://www.hydrocarbonengineering.com/petrochemicals/13072026/oxea-confirms-fid-for-major-capacity-expansion/</t>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/petrochemicals/13072026/oxea-confirms-fid-for-major-capacity-expansion/)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1205,7 +1205,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://www.ogj.com/refining-processing/gas-processing/news/55320579/targa-advances-permian-gas-pipeline-processing-expansion</t>
+          <t>[OGJ](https://www.ogj.com/refining-processing/gas-processing/news/55320579/targa-advances-permian-gas-pipeline-processing-expansion)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1242,7 +1242,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://www.businesswire.com/news/home/20250806663187/en/Enterprise-Agrees-to-Acquire-Occidentals-Gas-Gathering-Affiliate-Enters-Into-Natural-Gas-Processing-Agreement-Announces-New-Midland-Basin-Natural-Gas-Processing-Plant</t>
+          <t>[Business Wire](https://www.businesswire.com/news/home/20250806663187/en/Enterprise-Agrees-to-Acquire-Occidentals-Gas-Gathering-Affiliate-Enters-Into-Natural-Gas-Processing-Agreement-Announces-New-Midland-Basin-Natural-Gas-Processing-Plant)</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1279,7 +1279,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://naturalgasintel.com/news/mplx-scales-up-for-power-hungry-future-with-natural-gas-focused-growth-plan/</t>
+          <t>[Natural Gas Intel](https://naturalgasintel.com/news/mplx-scales-up-for-power-hungry-future-with-natural-gas-focused-growth-plan/)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1316,7 +1316,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://eastdaley.com/daley-note/mplx-acquires-northwind-for-2-375b-acquires-more-ngls-for-jv-project</t>
+          <t>[East Daley](https://eastdaley.com/daley-note/mplx-acquires-northwind-for-2-375b-acquires-more-ngls-for-jv-project)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1353,7 +1353,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://www.grandforksherald.com/news/local/northern-plains-nitrogen-proposal-receiving-more-attention-amid-global-fertilizer-pressure</t>
+          <t>[Grand Forks Herald](https://www.grandforksherald.com/news/local/northern-plains-nitrogen-proposal-receiving-more-attention-amid-global-fertilizer-pressure)</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1390,7 +1390,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://www.phillips66.com/newsroom/iron-mesa-safely-enters-next-phase-of-construction/</t>
+          <t>[Phillips 66](https://www.phillips66.com/newsroom/iron-mesa-safely-enters-next-phase-of-construction/)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://www.targaresources.com/news-releases/news-release-details/targa-resources-corp-announces-permian-growth-projects-and</t>
+          <t>[Targa Resources](https://www.targaresources.com/news-releases/news-release-details/targa-resources-corp-announces-permian-growth-projects-and)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1464,7 +1464,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://elefanteblanco.mx/2026/01/02/pemex-abre-30-licitaciones-para-obras-en-la-refineria-madero/</t>
+          <t>[Elefante Blanco](https://elefanteblanco.mx/2026/01/02/pemex-abre-30-licitaciones-para-obras-en-la-refineria-madero/)</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1501,7 +1501,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://www.jornada.com.mx/noticia/2026/06/08/economia/da-inicio-ejecucion-de-planta-de-fertilizantes-en-durango-por-parte-de-fermachem</t>
+          <t>[La Jornada](https://www.jornada.com.mx/noticia/2026/06/08/economia/da-inicio-ejecucion-de-planta-de-fertilizantes-en-durango-por-parte-de-fermachem)</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1538,7 +1538,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://downstreamcalendar.com/mcdermott-secures-feed-contract-for-ascension-clean-energy-project/</t>
+          <t>[Downstream Calendar](https://downstreamcalendar.com/mcdermott-secures-feed-contract-for-ascension-clean-energy-project/)</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1575,7 +1575,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://www.businesswire.com/news/home/20260517310811/en/Phillips-66-announces-Zeus-Gas-Plant-and-a-third-Coastal-Bend-Fractionator</t>
+          <t>[Business Wire](https://www.businesswire.com/news/home/20260517310811/en/Phillips-66-announces-Zeus-Gas-Plant-and-a-third-Coastal-Bend-Fractionator)</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1612,12 +1612,49 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://www.usda.gov/about-usda/news/press-releases/2026/07/01/secretary-rollins-announces-500-million-fertilizer-investment-and-expansion-program-strengthen</t>
+          <t>[USDA](https://www.usda.gov/about-usda/news/press-releases/2026/07/01/secretary-rollins-announces-500-million-fertilizer-investment-and-expansion-program-strengthen)</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
           <t>2026-07-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Wabash Low-Carbon Ammonia Project</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>West Terre Haute, Indiana, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Wabash Valley Resources</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Samsung E&amp;C (contrato EPF ~US$475 millones)</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Construcción (groundbreaking 5-ene-2026; amoniaco bajo en carbono 500,000 ton/año con captura de 1.67 millones ton CO2/año; meta de finalización 2029)</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/clean-fuels/06012026/samsung-ea-announces-groundbreaking-of-low-carbon-ammonia-plant/)</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
         </is>
       </c>
     </row>
@@ -1632,16 +1669,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
     <col width="55" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1709,7 +1746,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://www.bechtel.com/press-releases/nextdecade-executes-epc-contract-with-bechtel-for-train-4-at-the-rio-grande-lng-facility/</t>
+          <t>[Bechtel](https://www.bechtel.com/press-releases/nextdecade-executes-epc-contract-with-bechtel-for-train-4-at-the-rio-grande-lng-facility/)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -1746,7 +1783,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://www.bechtel.com/press-releases/sempra-infrastructure-announces-epc-contract-with-bechtel-for-port-arthur-lng-phase-2/</t>
+          <t>[Bechtel](https://www.bechtel.com/press-releases/sempra-infrastructure-announces-epc-contract-with-bechtel-for-port-arthur-lng-phase-2/)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -1783,7 +1820,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.woodside.com/what-we-do/growth-projects/woodside-louisiana-lng</t>
+          <t>[Woodside](https://www.woodside.com/what-we-do/growth-projects/woodside-louisiana-lng)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -1820,7 +1857,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.gem.wiki/CP2_LNG_Terminal</t>
+          <t>[GEM.wiki](https://www.gem.wiki/CP2_LNG_Terminal)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -1857,7 +1894,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.offshore-energy.biz/kbr-zachry-to-work-on-ventures-plaquemines-lng/</t>
+          <t>[Offshore Energy](https://www.offshore-energy.biz/kbr-zachry-to-work-on-ventures-plaquemines-lng/)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -1889,17 +1926,17 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Construcción</t>
+          <t>Construcción/Producción (Train 1: primer LNG mar-2026, primer cargamento exportado 22-abr-2026; Train 2 objetivo 2S2026; Train 3 objetivo 1S2027)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://lngprime.com/contracts-and-tenders/golden-pass-lng-contractors-ink-revised-epc-deal-for-second-and-third-train/169104/</t>
+          <t>[Port Arthur News](https://panews.com/2026/04/24/golden-pass-lng-makes-history-with-first-export-from-sabine-pass-terminal/)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-24</t>
         </is>
       </c>
     </row>
@@ -1931,7 +1968,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://pgjonline.com/news/2026/july/corpus-christi-lng-train-7-cleared-to-introduce-fuel-gas-by-ferc</t>
+          <t>[PGJ](https://pgjonline.com/news/2026/july/corpus-christi-lng-train-7-cleared-to-introduce-fuel-gas-by-ferc)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1968,7 +2005,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2026/06/03/3306350/0/en/delfin-midstream-announces-5-billion-final-investment-decision-for-first-flng-vessel.html</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/06/03/3306350/0/en/delfin-midstream-announces-5-billion-final-investment-decision-for-first-flng-vessel.html)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -2005,7 +2042,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://dossierpolitico.com/2026/07/17/activistas-entregan-90-mil-firmas-para-frenar-proyecto-saguaro-energia-en-sonora/</t>
+          <t>[Dossier Político](https://dossierpolitico.com/2026/07/17/activistas-entregan-90-mil-firmas-para-frenar-proyecto-saguaro-energia-en-sonora/)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -2042,7 +2079,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://www.gem.wiki/New_Fortress_Altamira_FLNG_Terminal</t>
+          <t>[GEM Wiki](https://www.gem.wiki/New_Fortress_Altamira_FLNG_Terminal)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -2079,7 +2116,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://www.naturalgasintel.com/news/glenfarne-lands-investment-for-early-work-on-texas-lng-ahead-of-fid/</t>
+          <t>[Natural Gas Intel](https://www.naturalgasintel.com/news/glenfarne-lands-investment-for-early-work-on-texas-lng-ahead-of-fid/)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -2116,7 +2153,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://pgjonline.com/news/2026/july/commonwealth-lng-awards-main-automation-contract-for-louisiana-export-terminal</t>
+          <t>[PGJ](https://pgjonline.com/news/2026/july/commonwealth-lng-awards-main-automation-contract-for-louisiana-export-terminal)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -2153,7 +2190,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://www.houstonpublicmedia.org/articles/galveston-county/2026/07/14/557086/galveston-pelican-island-lng/</t>
+          <t>[Houston Public Media](https://www.houstonpublicmedia.org/articles/galveston-county/2026/07/14/557086/galveston-pelican-island-lng/)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -2190,7 +2227,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://www.sempra.com/newsroom/press-releases/sempra-infrastructures-eca-lng-phase-1-exports-first-lng-cargo-mexicos</t>
+          <t>[Sempra](https://www.sempra.com/newsroom/press-releases/sempra-infrastructures-eca-lng-phase-1-exports-first-lng-cargo-mexicos)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -2227,7 +2264,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://lngprime.com/americas/gato-negro-eyes-fid-on-mexico-lng-plant-in-late-2026/165906/</t>
+          <t>[LNG Prime](https://lngprime.com/americas/gato-negro-eyes-fid-on-mexico-lng-plant-in-late-2026/165906/)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -2264,7 +2301,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/amigo-lng-awards-landmark-epc-contract-to-dubai-based-drydocks-world-for-worlds-largest-flng-facility-302537739.html</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/amigo-lng-awards-landmark-epc-contract-to-dubai-based-drydocks-world-for-worlds-largest-flng-facility-302537739.html)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -2301,7 +2338,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://www.kbr.com/en/insights-news/press-release/kbr-awarded-feed-coastal-bend-lng-project</t>
+          <t>[KBR](https://www.kbr.com/en/insights-news/press-release/kbr-awarded-feed-coastal-bend-lng-project)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2338,7 +2375,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://www.ferc.gov/gulfstream-lng-terminal-project</t>
+          <t>[FERC](https://www.ferc.gov/gulfstream-lng-terminal-project)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2375,7 +2412,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://glenfarnegroup.com/glenfarne-announces-major-phase-one-alaska-lng-milestones-with-construction-line-pipe-supply-and-in-state-gas-agreements/</t>
+          <t>[Glenfarne](https://glenfarnegroup.com/glenfarne-announces-major-phase-one-alaska-lng-milestones-with-construction-line-pipe-supply-and-in-state-gas-agreements/)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2412,7 +2449,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://pgjonline.com/news/2026/july/311-mile-sonora-gas-pipeline-project-advances-in-mexico</t>
+          <t>[PGJ](https://pgjonline.com/news/2026/july/311-mile-sonora-gas-pipeline-project-advances-in-mexico)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2449,7 +2486,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://www.ogj.com/pipelines-transportation/pipelines/news/55322537/arm-energy-takes-fid-on-23-billion-mustang-express-pipeline</t>
+          <t>[OGJ](https://www.ogj.com/pipelines-transportation/pipelines/news/55322537/arm-energy-takes-fid-on-23-billion-mustang-express-pipeline)</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2486,7 +2523,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://mexicobusiness.news/energy/news/ursus-energy-scales-investment-us21-billion</t>
+          <t>[Mexico Business News](https://mexicobusiness.news/energy/news/ursus-energy-scales-investment-us21-billion)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2523,7 +2560,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2026/07/15/3327983/0/en/Delfin-Midstream-Partners-With-EIG-s-MidOcean-Energy-to-Advance-Second-FLNG-Vessel-Issues-Limited-Notice-to-Proceed-to-Siemens-Energy.html</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/15/3327983/0/en/Delfin-Midstream-Partners-With-EIG-s-MidOcean-Energy-to-Advance-Second-FLNG-Vessel-Issues-Limited-Notice-to-Proceed-to-Siemens-Energy.html)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2560,7 +2597,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://www.naturalgasintel.com/news/texas-gateway-open-season-expands-haynesville-natural-gas-links-amid-lng-growth/</t>
+          <t>[Natural Gas Intel](https://www.naturalgasintel.com/news/texas-gateway-open-season-expands-haynesville-natural-gas-links-amid-lng-growth/)</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2597,7 +2634,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://worldoil.com/news/2026/7/6/argent-lng-awards-engineering-contract-for-port-fourchon-lng-project/</t>
+          <t>[World Oil](https://worldoil.com/news/2026/7/6/argent-lng-awards-engineering-contract-for-port-fourchon-lng-project/)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2629,17 +2666,17 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Permitting/Pre-FID (Draft EIS publicado abr-2026)</t>
+          <t>Permitting/Pre-FID (EIS Final publicado 24-jul-2026, avanzando desde Draft EIS de abr-2026; capacidad 8.4 Mtpa)</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://www.federalregister.gov/documents/2026/04/17/2026-07517/deepwater-port-license-application-st-lng-deepwater-port-development-project-draft-environmental</t>
+          <t>[Federal Register](https://www.federalregister.gov/documents/2026/07/24/2026-14963/deepwater-port-license-application-st-lng-deepwater-port-development-project-final-environmental)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-24</t>
         </is>
       </c>
     </row>
@@ -2671,7 +2708,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://naturalgasintel.com/news/kinder-morgan-greenlights-7b-in-natural-gas-pipeline-projects-amid-regulatory-speedup/</t>
+          <t>[Natural Gas Intel](https://naturalgasintel.com/news/kinder-morgan-greenlights-7b-in-natural-gas-pipeline-projects-amid-regulatory-speedup/)</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -2708,7 +2745,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://naturalgasintel.com/news/kinder-morgan-greenlights-7b-in-natural-gas-pipeline-projects-amid-regulatory-speedup/</t>
+          <t>[Natural Gas Intel](https://naturalgasintel.com/news/kinder-morgan-greenlights-7b-in-natural-gas-pipeline-projects-amid-regulatory-speedup/)</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2745,7 +2782,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://lngprime.com/americas/kinder-morgan-seeks-doe-extension-for-gulf-lng-export-project/184334/</t>
+          <t>[LNG Prime](https://lngprime.com/americas/kinder-morgan-seeks-doe-extension-for-gulf-lng-export-project/184334/)</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2782,12 +2819,123 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://investors.bakerhughes.com/news/press-releases/news-details/2026/Baker-Hughes-Secures-Substantial-Equipment-and-Services-Awards-for-Chenieres-Sabine-Pass-LNG-Facility/default.aspx</t>
+          <t>[Baker Hughes](https://investors.bakerhughes.com/news/press-releases/news-details/2026/Baker-Hughes-Secures-Substantial-Equipment-and-Services-Awards-for-Chenieres-Sabine-Pass-LNG-Facility/default.aspx)</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
           <t>2026-07-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Corpus Christi Stage 4</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>San Patricio County / Corpus Christi, Texas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Cheniere Energy</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Permitting (solicitud FERC en proceso desde 17-feb-2026; DOE revisando solicitud de exportación; EIS borrador esperado sep-2026; incluye gasoducto de alimentación CCPL de 42"/26 millas)</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>[Federal Register](https://www.federalregister.gov/documents/2026/05/05/2026-08654/cheniere-corpus-christi-pipeline-lp-corpus-christi-liquefaction-stage-iv-llc-corpus-christi)</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Freeport LNG Train 4</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Freeport, Texas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Freeport LNG Development, L.P.</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Pre-FID (FERC extendió plazo de puesta en servicio a ago-2028; capacidad 5.1 Mtpa)</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>[Natural Gas Intel](https://www.naturalgasintel.com/news/ferc-approves-extension-for-freeport-lngs-fourth-train-expansion-project/)</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Gasoducto Coatzacoalcos II (alimenta PODEBI Coatzacoalcos II)</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Coatzacoalcos, Veracruz, México</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>CFE / CENAGAS</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Por definir (licitación pública, adjudicación 15-jul-2026)</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Bidding/Construcción inminente (9.69 km en dos etapas; inversión ~US$177 millones; plazo de ejecución 17 meses)</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>[Proyectos México](https://www.proyectosmexico.gob.mx/proyecto_inversion/1076-gasoducto-coatzacoalcos-ii/)</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
         </is>
       </c>
     </row>
@@ -2802,16 +2950,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
     <col width="55" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2879,7 +3027,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://www.miningweekly.com/article/ivanhoe-electric-pencils-in-2026-construction-start-at-arizona-copper-mine-2025-06-25</t>
+          <t>[Mining Weekly](https://www.miningweekly.com/article/ivanhoe-electric-pencils-in-2026-construction-start-at-arizona-copper-mine-2025-06-25)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -2916,7 +3064,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1322422/000106299326001973/exhibit99-2.htm</t>
+          <t>[SEC/Hudbay](https://www.sec.gov/Archives/edgar/data/1322422/000106299326001973/exhibit99-2.htm)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -2953,7 +3101,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/863064/000086306426000019/ex12d16mr_resolutionland.htm</t>
+          <t>[SEC](https://www.sec.gov/Archives/edgar/data/863064/000086306426000019/ex12d16mr_resolutionland.htm)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -2990,7 +3138,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.nevadaappeal.com/news/2026/mar/26/lithium-americas-900-construction-workers-at-thacker-pass-mine/</t>
+          <t>[Nevada Appeal](https://www.nevadaappeal.com/news/2026/mar/26/lithium-americas-900-construction-workers-at-thacker-pass-mine/)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -3027,7 +3175,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.mining.com/teck-agnico-team-up-at-san-nicolas-copper-project-in-mexico/</t>
+          <t>[Mining.com](https://www.mining.com/teck-agnico-team-up-at-san-nicolas-copper-project-in-mexico/)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -3064,7 +3212,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://energymagazine.mx/2025/10/grupo-mexico-espera-autorizacion-federal-para-continuar-proyectos-mineros-por-10-mil-200-mdd/</t>
+          <t>[Energy Magazine MX](https://energymagazine.mx/2025/10/grupo-mexico-espera-autorizacion-federal-para-continuar-proyectos-mineros-por-10-mil-200-mdd/)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -3101,7 +3249,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://www.bnamericas.com/en/news/southern-copper-wins-permits-for-us551mn-el-pilar-in-mexico</t>
+          <t>[BNamericas](https://www.bnamericas.com/en/news/southern-copper-wins-permits-for-us551mn-el-pilar-in-mexico)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -3138,7 +3286,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://m3eng.com/portfolio/buenavista-del-cobre-concentradora-no-2/</t>
+          <t>[M3 Engineering](https://m3eng.com/portfolio/buenavista-del-cobre-concentradora-no-2/)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -3175,7 +3323,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://mineriaenlinea.com/2026/04/torex-gold-alcanza-velocidad-de-crucero-en-media-luna-9-meses-adelante-de-cronograma/</t>
+          <t>[Minería en Línea](https://mineriaenlinea.com/2026/04/torex-gold-alcanza-velocidad-de-crucero-en-media-luna-9-meses-adelante-de-cronograma/)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -3212,7 +3360,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://www.mining.com/nevada-copper-unveils-restart-and-financing-plan-for-pumpkin-hollow/</t>
+          <t>[Mining.com](https://www.mining.com/nevada-copper-unveils-restart-and-financing-plan-for-pumpkin-hollow/)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -3249,7 +3397,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://www.usda.gov/about-usda/news/press-releases/2026/07/07/usda-advances-trump-administration-effort-boost-us-mineral-energy-production</t>
+          <t>[USDA](https://www.usda.gov/about-usda/news/press-releases/2026/07/07/usda-advances-trump-administration-effort-boost-us-mineral-energy-production)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -3286,7 +3434,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/perpetua-resources-advances-construction-of-the-stibnite-gold-project-302787012.html</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/perpetua-resources-advances-construction-of-the-stibnite-gold-project-302787012.html)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -3323,7 +3471,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://silvertigermetals.com/news/2026/silver-tiger-metals-awards-engineering-procurement-and-construction-management-contract-and-provides-construction-update</t>
+          <t>[Silver Tiger Metals](https://silvertigermetals.com/news/2026/silver-tiger-metals-awards-engineering-procurement-and-construction-management-contract-and-provides-construction-update)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -3360,7 +3508,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/vizsla-silver-awards-epcm-and-mine-design-contracts-for-the-development-of-the-panuco-silver-gold-project-302750621.html</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/vizsla-silver-awards-epcm-and-mine-design-contracts-for-the-development-of-the-panuco-silver-gold-project-302750621.html)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -3397,7 +3545,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://orlamining.com/news/orla-announces-results-of-updated-feasibility-study-for-south-railroad-project/</t>
+          <t>[Orla Mining](https://orlamining.com/news/orla-announces-results-of-updated-feasibility-study-for-south-railroad-project/)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -3434,7 +3582,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://www.miningweekly.com/article/minera-alamos-confirms-low-cost-near-term-mining-possible-at-copperstone-in-arizona-2026-05-28</t>
+          <t>[Mining Weekly](https://www.miningweekly.com/article/minera-alamos-confirms-low-cost-near-term-mining-possible-at-copperstone-in-arizona-2026-05-28)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -3471,7 +3619,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://www.wyomingnews.com/rawlinstimes/plans-move-forward-for-ck-gold-project-as-developers-target-2026-construction-start/article_b2bb147e-2f92-4ca2-bf86-fcc9983917a7.html</t>
+          <t>[Wyoming News](https://www.wyomingnews.com/rawlinstimes/plans-move-forward-for-ck-gold-project-as-developers-target-2026-construction-start/article_b2bb147e-2f92-4ca2-bf86-fcc9983917a7.html)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -3508,7 +3656,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://www.juniorminingnetwork.com/junior-miner-news/press-releases/1082-tsx/ag/206222-first-majestic-receives-construction-permits-for-santo-nino-and-navidad-advances-development-across-the-santa-elena-district.html</t>
+          <t>[First Majestic](https://www.juniorminingnetwork.com/junior-miner-news/press-releases/1082-tsx/ag/206222-first-majestic-receives-construction-permits-for-santo-nino-and-navidad-advances-development-across-the-santa-elena-district.html)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -3545,7 +3693,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/0001286973/000106299326002645/exhibit99-2.htm</t>
+          <t>[SEC/Americas Gold and Silver](https://www.sec.gov/Archives/edgar/data/0001286973/000106299326002645/exhibit99-2.htm)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -3582,7 +3730,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://www.kitco.com/news/off-the-wire/2026-06-08/minera-frisco-restarts-two-mexico-mines-plans-new-silver-unit</t>
+          <t>[Kitco](https://www.kitco.com/news/off-the-wire/2026-06-08/minera-frisco-restarts-two-mexico-mines-plans-new-silver-unit)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -3619,7 +3767,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/trilogy-metals-announces-publication-of-federal-and-state-permitting-schedule-for-arctic-project-establishing-defined-timeline-toward-a-record-of-decision-by-september-2028-302827083.html</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/trilogy-metals-announces-publication-of-federal-and-state-permitting-schedule-for-arctic-project-establishing-defined-timeline-toward-a-record-of-decision-by-september-2028-302827083.html)</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -3656,7 +3804,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://www.northernminer.com/news/gogold-approved-to-build-227m-mine-in-mexico/1003891932/</t>
+          <t>[Northern Miner](https://www.northernminer.com/news/gogold-approved-to-build-227m-mine-in-mexico/1003891932/)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -3693,7 +3841,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://www.bnamericas.com/en/news/discovery-advances-permitting-financing-at-us606mn-cordero-in-mexico</t>
+          <t>[BNamericas](https://www.bnamericas.com/en/news/discovery-advances-permitting-financing-at-us606mn-cordero-in-mexico)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -3730,7 +3878,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://resourceworld.com/tocvan-ventures-eyes-mexican-gold-pour-by-q4-2026/</t>
+          <t>[Resource World](https://resourceworld.com/tocvan-ventures-eyes-mexican-gold-pour-by-q4-2026/)</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -3767,7 +3915,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://www.fresnilloplc.com/portfolio/exploration/orisyvo/</t>
+          <t>[Fresnillo plc](https://www.fresnilloplc.com/portfolio/exploration/orisyvo/)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -3804,7 +3952,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/</t>
+          <t>[Mining.com](https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -3841,7 +3989,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/</t>
+          <t>[Mining.com](https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/)</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -3878,7 +4026,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/</t>
+          <t>[Mining.com](https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/)</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -3915,7 +4063,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://im-mining.com/2026/06/29/metso-to-supply-additional-crushing-package-for-grupo-mexico-la-caridad-copper-concentrator/</t>
+          <t>[IM Mining](https://im-mining.com/2026/06/29/metso-to-supply-additional-crushing-package-for-grupo-mexico-la-caridad-copper-concentrator/)</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -3952,7 +4100,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2026/05/21/3299182</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/05/21/3299182)</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3989,7 +4137,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://mexicobusiness.news/mining/news/grupo-mexicos-asarco-may-reopen-united-states</t>
+          <t>[Mexico Business News](https://mexicobusiness.news/mining/news/grupo-mexicos-asarco-may-reopen-united-states)</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -4026,7 +4174,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>https://mineraalamos.com/our-assets/cerro-de-oro-project/</t>
+          <t>[Minera Alamos](https://mineraalamos.com/our-assets/cerro-de-oro-project/)</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -4063,7 +4211,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>https://www.globalminingreview.com/mining/11022025/antler-copper-project-achieves-critical-federal-permitting-milestone/</t>
+          <t>[Global Mining Review](https://www.globalminingreview.com/mining/11022025/antler-copper-project-achieves-critical-federal-permitting-milestone/)</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -4100,7 +4248,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>https://www.blm.gov/press-release/blm-approves-lisbon-valley-copper-mine-expansion-utah</t>
+          <t>[BLM](https://www.blm.gov/press-release/blm-approves-lisbon-valley-copper-mine-expansion-utah)</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -4137,7 +4285,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>https://investingnews.com/smackover-lithium-announces-the-award-of-last-key-construction-contract-for-the-south-west-arkansas-project-ahead-of-final-investment-decision/</t>
+          <t>[InvestingNews](https://investingnews.com/smackover-lithium-announces-the-award-of-last-key-construction-contract-for-the-south-west-arkansas-project-ahead-of-final-investment-decision/)</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -4174,12 +4322,197 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/0000831259/000083125926000033/a2q2026exhibit991.htm</t>
+          <t>[SEC/Freeport-McMoRan](https://www.sec.gov/Archives/edgar/data/0000831259/000083125926000033/a2q2026exhibit991.htm)</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
           <t>2026-07-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Elk Creek Critical Minerals Project</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Elk Creek, Nebraska, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>NioCorp Developments Ltd.</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Construcción (portal de mina de doble rampa, ~US$44.6 millones, iniciado feb/mar-2026; proyecto de niobio/escandio/titanio con planta de superficie que requerirá tubería de proceso)</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>[NioCorp](https://niocorp.com/niocorp-launches-construction-of-elk-creek-critical-minerals-project-mine-portal/)</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Goldfield Project</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Goldfield, Nevada, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Centerra Gold Inc.</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Ingeniería/Construcción temprana (ingeniería de detalle y procura de largo plazo en 2026; construcción mayor de pila de lixiviación y circuitos de trituración/procesamiento en 2027; primera producción fin de 2028)</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>[E&amp;MJ](https://www.e-mj.com/breaking-news/centerra-advances-goldfield-project-in-nevada/)</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Cactus Mine (distrito Copper World/Arizona Sonoran)</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Casa Grande, Arizona, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Hudbay Minerals (adquisición de Arizona Sonoran Copper Co. anunciada 2-mar-2026)</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Desarrollo/Feasibility (planta SX-EW de cátodos de cobre, ~103,000 t Cu/año proyectadas; Hudbay busca fusionarlo con el distrito Copper World adyacente ya rastreado)</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/03/02/3247157/0/en/hudbay-to-acquire-arizona-sonoran-creating-the-third-largest-copper-district-in-north-america.html)</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Doby George Gold Project (Distrito Aura)</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>~120 km al norte de Elko, Nevada, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Western Exploration Inc.</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>No especificado (WSP realiza feasibility study; Stantec y Kappes Cassidy en estudios ambientales)</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Feasibility/Permitting (PEA positiva 2025; Mine Plan of Operations en preparación; proyecto de lixiviación en pilas de óxidos)</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>[Western Exploration](https://www.westernexploration.com/news-and-updates/news/news-details/2026/Western-Exploration-Outlines-2026-Program-to-Advance-Doby-George-Permitting-and-Expand-Gravel-Creek-Resources-2026-aaotfYHcV7/default.aspx)</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Metates Project</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Durango, México</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Chesapeake Gold Corp.</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Feasibility (prefeasibility study objetivo 2026; pruebas metalúrgicas de lixiviación de sulfuros y estudios ambientales de línea base en curso; uno de los mayores depósitos de oro-plata no desarrollados de América)</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>[Chesapeake Gold Corp.](https://chesapeakegold.com/metates/)</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
         </is>
       </c>
     </row>
@@ -4194,16 +4527,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
     <col width="55" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4271,7 +4604,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/vantage-breaks-ground-on-texas-gigawatt-data-center-campus-for-openai/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/vantage-breaks-ground-on-texas-gigawatt-data-center-campus-for-openai/)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -4308,7 +4641,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://epoch.ai/publications/openai-stargate-where-the-us-sites-stand</t>
+          <t>[Epoch AI](https://epoch.ai/publications/openai-stargate-where-the-us-sites-stand)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -4345,7 +4678,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/crusoe-tops-out-final-building-at-openai-stargate-data-center-campus-in-abilene-texas/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/crusoe-tops-out-final-building-at-openai-stargate-data-center-campus-in-abilene-texas/)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -4382,7 +4715,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.cnbc.com/2026/06/22/chevron-cvx-microsoft-msft-natural-gas-data-center.html</t>
+          <t>[CNBC](https://www.cnbc.com/2026/06/22/chevron-cvx-microsoft-msft-natural-gas-data-center.html)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -4419,7 +4752,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.gob.mx/presidencia/prensa/plan-mexico-avanza-se-anuncia-inversion-de-4-mil-800-mdd-de-cloudhq-para-la-construccion-de-6-centros-de-datos-en-queretaro</t>
+          <t>[Gobierno de México](https://www.gob.mx/presidencia/prensa/plan-mexico-avanza-se-anuncia-inversion-de-4-mil-800-mdd-de-cloudhq-para-la-construccion-de-6-centros-de-datos-en-queretaro)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -4456,7 +4789,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.ucs.org/about/news/judge-orders-meta-explain-new-gas-demand-hyperscale-louisiana-data-center</t>
+          <t>[UCS](https://www.ucs.org/about/news/judge-orders-meta-explain-new-gas-demand-hyperscale-louisiana-data-center)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -4493,7 +4826,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://www.datacenterfrontier.com/site-selection/article/55305086/nv1-and-the-nevada-hyperscale-boom-vantage-data-centers-bets-3b-on-the-ai-future</t>
+          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55305086/nv1-and-the-nevada-hyperscale-boom-vantage-data-centers-bets-3b-on-the-ai-future)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -4530,7 +4863,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/cloudburst-breaks-ground-on-gigawatt-scale-data-center-campus-in-texas/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/cloudburst-breaks-ground-on-gigawatt-scale-data-center-campus-in-texas/)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -4567,7 +4900,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/prometheus-hyperscale-details-plans-for-dallas-data-center-campus/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/prometheus-hyperscale-details-plans-for-dallas-data-center-campus/)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -4604,7 +4937,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://www.businesswire.com/news/home/20260126236053/en/Pacifico-Energy-Secures-7.65-GW-Power-Generation-Permit-for-GW-Ranch-Project</t>
+          <t>[Business Wire](https://www.businesswire.com/news/home/20260126236053/en/Pacifico-Energy-Secures-7.65-GW-Power-Generation-Permit-for-GW-Ranch-Project)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -4641,7 +4974,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/amazon-looks-to-build-large-scale-data-center-campus-next-to-nuclear-plant-in-texas/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/amazon-looks-to-build-large-scale-data-center-campus-next-to-nuclear-plant-in-texas/)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -4678,7 +5011,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://mexiconewsdaily.com/business/durango-data-center-fertilizer-plant-investment-fermaca/</t>
+          <t>[Mexico News Daily](https://mexiconewsdaily.com/business/durango-data-center-fertilizer-plant-investment-fermaca/)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -4715,7 +5048,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/circe-energy-secures-2gw-of-natural-gas-capacity-for-west-texas-data-center-campus/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/circe-energy-secures-2gw-of-natural-gas-capacity-for-west-texas-data-center-campus/)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -4752,7 +5085,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://sourcenm.com/2026/07/16/new-mexico-land-commissioner-blocks-project-jupiter-related-pipeline-from-building-on-state-land/</t>
+          <t>[Source NM](https://sourcenm.com/2026/07/16/new-mexico-land-commissioner-blocks-project-jupiter-related-pipeline-from-building-on-state-land/)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -4789,7 +5122,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/powerplay-ai-announces-400-mw-behind-the-meter-ai-data-center-development-in-greater-abilene-with-nasdaq-listed-neocloud-joint-venture-partner-302829610.html</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/powerplay-ai-announces-400-mw-behind-the-meter-ai-data-center-development-in-greater-abilene-with-nasdaq-listed-neocloud-joint-venture-partner-302829610.html)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -4826,7 +5159,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/liberty-energy-powerbridge-form-jv-to-power-planned-2gw-data-center-in-west-texas/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/liberty-energy-powerbridge-form-jv-to-power-planned-2gw-data-center-in-west-texas/)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -4863,7 +5196,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://www.powermag.com/nuclear-natural-gas-power-generation-planned-for-massive-new-mexico-data-center-site/</t>
+          <t>[PowerMag](https://www.powermag.com/nuclear-natural-gas-power-generation-planned-for-massive-new-mexico-data-center-site/)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -4900,7 +5233,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://www.datacenterfrontier.com/site-selection/article/55289667/powering-ai-in-the-permian-texas-critical-data-centers-sustainable-energy-play</t>
+          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55289667/powering-ai-in-the-permian-texas-critical-data-centers-sustainable-energy-play)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -4937,7 +5270,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://openai.com/index/five-new-stargate-sites/</t>
+          <t>[OpenAI](https://openai.com/index/five-new-stargate-sites/)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -4974,7 +5307,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://openai.com/index/five-new-stargate-sites/</t>
+          <t>[OpenAI](https://openai.com/index/five-new-stargate-sites/)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -5011,7 +5344,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://mexiconewsdaily.com/business/aws-invest-5b-mexico-data-region/</t>
+          <t>[Mexico News Daily](https://mexiconewsdaily.com/business/aws-invest-5b-mexico-data-region/)</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -5048,7 +5381,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/oracle-and-openai-start-construction-on-stargate-data-center-campus-in-saline-township-michigan/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/oracle-and-openai-start-construction-on-stargate-data-center-campus-in-saline-township-michigan/)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -5085,7 +5418,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://www.valleynewslive.com/2026/07/13/applied-digital-expands-north-dakota-eyes-oliver-county-third-data-center/</t>
+          <t>[Valley News Live](https://www.valleynewslive.com/2026/07/13/applied-digital-expands-north-dakota-eyes-oliver-county-third-data-center/)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -5122,7 +5455,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://energymagazine.mx/2026/01/el-data-center-verde-que-encendio-la-polemica-asi-sera-el-proyecto-de-ia-en-nuevo-leon-que-usara-tecnologia-de-nvidia/</t>
+          <t>[Energy Magazine MX](https://energymagazine.mx/2026/01/el-data-center-verde-que-encendio-la-polemica-asi-sera-el-proyecto-de-ia-en-nuevo-leon-que-usara-tecnologia-de-nvidia/)</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -5159,7 +5492,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://www.constructiondive.com/news/data-center-cleanarc-breaks-ground-virginia-campus/806489/</t>
+          <t>[Construction Dive](https://www.constructiondive.com/news/data-center-cleanarc-breaks-ground-virginia-campus/806489/)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -5196,7 +5529,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://www.ksl.com/article/51402125/groundbreaking-for-new-millard-county-artificial-intelligence-data-center</t>
+          <t>[KSL](https://www.ksl.com/article/51402125/groundbreaking-for-new-millard-county-artificial-intelligence-data-center)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -5233,7 +5566,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://governor.mo.gov/press-releases/archive/amazon-investing-10-billion-montgomery-county</t>
+          <t>[Governor.mo.gov](https://governor.mo.gov/press-releases/archive/amazon-investing-10-billion-montgomery-county)</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -5270,7 +5603,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://www.stlpr.org/government-politics-issues/2026-05-21/missouri-governor-google-announce-15-billion-data-center-montgomery-county</t>
+          <t>[STLPR](https://www.stlpr.org/government-politics-issues/2026-05-21/missouri-governor-google-announce-15-billion-data-center-montgomery-county)</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -5307,7 +5640,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2026/07/06/3322404/0/en/big-digital-energy-announces-partnership-with-10netzero-to-acquire-power-ready-hood-county-texas-site-for-ai-datacenter-development.html</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/06/3322404/0/en/big-digital-energy-announces-partnership-with-10netzero-to-acquire-power-ready-hood-county-texas-site-for-ai-datacenter-development.html)</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -5344,7 +5677,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/)</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -5381,7 +5714,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/meta-files-to-expand-campus-in-el-paso-texas-with-12-new-buildings/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/meta-files-to-expand-campus-in-el-paso-texas-with-12-new-buildings/)</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -5418,7 +5751,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/softbank-eyes-10gw-data-center-at-former-doe-nuclear-enrichment-site-in-ohio/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/softbank-eyes-10gw-data-center-at-former-doe-nuclear-enrichment-site-in-ohio/)</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -5455,7 +5788,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/)</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -5492,7 +5825,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>https://www.williams.com/2026/07/13/williams-announces-5-34-billion-investment-in-power-innovation-joint-venture-from-blackstone/</t>
+          <t>[Williams Companies](https://www.williams.com/2026/07/13/williams-announces-5-34-billion-investment-in-power-innovation-joint-venture-from-blackstone/)</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -5529,7 +5862,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/cleancore-solutions-zone-announces-closing-of-first-data-center-project-establishing-its-critical-infrastructure-buildout-for-the-ai-economy-302821421.html</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/cleancore-solutions-zone-announces-closing-of-first-data-center-project-establishing-its-critical-infrastructure-buildout-for-the-ai-economy-302821421.html)</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -5566,7 +5899,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>https://www.bloomberg.com/news/articles/2026-06-09/crusoe-touts-5-gigawatts-worth-of-data-centers-deals-pauses-wyoming-site</t>
+          <t>[Bloomberg](https://www.bloomberg.com/news/articles/2026-06-09/crusoe-touts-5-gigawatts-worth-of-data-centers-deals-pauses-wyoming-site)</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -5603,7 +5936,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>https://www.hpcwire.com/off-the-wire/core-scientific-plans-expansion-to-1-5gw-of-gross-power-at-pecos-texas-campus/</t>
+          <t>[HPCwire](https://www.hpcwire.com/off-the-wire/core-scientific-plans-expansion-to-1-5gw-of-gross-power-at-pecos-texas-campus/)</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -5640,7 +5973,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>https://utahnewsdispatch.com/2026/05/19/renderings-show-massive-data-center-box-elder-utah-permits-could-take-years/</t>
+          <t>[Utah News Dispatch](https://utahnewsdispatch.com/2026/05/19/renderings-show-massive-data-center-box-elder-utah-permits-could-take-years/)</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -5667,22 +6000,22 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Primoris Services Corporation (balance of plant, turbinas de gas)</t>
+          <t>Primoris Services Corporation (balance of plant, turbinas de gas); Siemens Energy (suministro de turbinas)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Construcción (excavación de isla de turbinas completada; EPC firmado)</t>
+          <t>Construcción (excavación de isla de turbinas completada; EPC firmado; 3 turbinas de gas Siemens Energy SGT6-5000F, hasta 780MW ciclo simple, llegaron al Puerto de Houston 21-jul-2026 con destino al sitio; meta de 1GW en línea a fines de 2026)</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/fermi-selects-primoris-services-corporation-to-engineer-and-construct-balance-of-plant-for-first-six-sgt-800-gas-turbines-of-phase-one-power-buildout-302814505.html</t>
+          <t>[StockTitan](https://www.stocktitan.net/news/FRMI/fermi-announces-first-siemens-turbines-arrive-at-port-of-qg7ienp885jk.html)</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-24</t>
         </is>
       </c>
     </row>
@@ -5714,7 +6047,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>https://www.kltv.com/2026/03/20/president-trump-approves-16-billion-natural-gas-generator-be-installed-anderson-county/</t>
+          <t>[KLTV](https://www.kltv.com/2026/03/20/president-trump-approves-16-billion-natural-gas-generator-be-installed-anderson-county/)</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -5751,7 +6084,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>https://wvmetronews.com/2026/07/16/mon-power-president-says-data-centers-will-end-up-paying-for-natural-gas-powered-power-plant/</t>
+          <t>[WV MetroNews](https://wvmetronews.com/2026/07/16/mon-power-president-says-data-centers-will-end-up-paying-for-natural-gas-powered-power-plant/)</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -5788,7 +6121,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>https://www.utilitydive.com/news/iep-plans-944-mw-behind-the-meter-gas-plant-in-pennsylvania-to-power-data-c/758830/</t>
+          <t>[Utility Dive](https://www.utilitydive.com/news/iep-plans-944-mw-behind-the-meter-gas-plant-in-pennsylvania-to-power-data-c/758830/)</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -5825,7 +6158,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/aws-files-for-12bn-data-center-campus-outside-houston-texas/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/aws-files-for-12bn-data-center-campus-outside-houston-texas/)</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -5862,7 +6195,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>https://www.crusoe.ai/resources/newsroom/crusoe-and-lancium-announce-1-gigawatt-ai-data-center-campus-in-childress-texas</t>
+          <t>[Crusoe](https://www.crusoe.ai/resources/newsroom/crusoe-and-lancium-announce-1-gigawatt-ai-data-center-campus-in-childress-texas)</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -5899,7 +6232,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/)</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -5936,7 +6269,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>https://www.powermag.com/new-200-mw-gas-fired-plant-in-ohio-will-power-meta-data-center/</t>
+          <t>[PowerMag](https://www.powermag.com/new-200-mw-gas-fired-plant-in-ohio-will-power-meta-data-center/)</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -5973,7 +6306,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>https://www.aterio.io/blog/crusoe-launches-usd29b-goodnight-campus-in-claude-mirroring-openai-s-stargate</t>
+          <t>[Aterio](https://www.aterio.io/blog/crusoe-launches-usd29b-goodnight-campus-in-claude-mirroring-openai-s-stargate)</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -6010,7 +6343,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>https://www.ajc.com/business/2026/07/officials-order-georgia-data-centers-pop-up-power-plant-to-halt-construction/</t>
+          <t>[AJC](https://www.ajc.com/business/2026/07/officials-order-georgia-data-centers-pop-up-power-plant-to-halt-construction/)</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -6047,7 +6380,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/stark-power-lands-56gw-data-center-development-portfolio-in-sagebrush-acquisition/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/stark-power-lands-56gw-data-center-development-portfolio-in-sagebrush-acquisition/)</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -6084,7 +6417,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>https://www.datacenterfrontier.com/site-selection/article/55281341/pennsylvanias-homer-city-energy-campus-a-brownfield-transformed-for-data-center-innovation</t>
+          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55281341/pennsylvanias-homer-city-energy-campus-a-brownfield-transformed-for-data-center-innovation)</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -6121,7 +6454,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>https://www.datacenterknowledge.com/data-center-site-selection/nebius-plans-300-mw-data-center-in-new-jersey-amid-us-expansion</t>
+          <t>[Data Center Knowledge](https://www.datacenterknowledge.com/data-center-site-selection/nebius-plans-300-mw-data-center-in-new-jersey-amid-us-expansion)</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -6158,7 +6491,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/terravolt-inks-natural-gas-supply-deal-for-onsite-power-plant-at-planned-data-center-campus-in-idaho/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/terravolt-inks-natural-gas-supply-deal-for-onsite-power-plant-at-planned-data-center-campus-in-idaho/)</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -6195,12 +6528,123 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/cyrusone-announces-sixth-data-center-campus-in-san-antonio-texas/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/cyrusone-announces-sixth-data-center-campus-in-san-antonio-texas/)</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
           <t>2026-07-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>EdgeConneX PowerConneX New Albany Energy Center (I y II)</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>New Albany, Licking County, Ohio, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>EdgeConneX (propiedad de EQT Infrastructure)</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>No especificado (desarrollado vía afiliada PowerConneX)</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Construcción (PowerConneX I, 120MW, certificado OPSB 22-jul-2025, construcción iniciada sep-2025, operación comercial posible 3T2026; PowerConneX II, 216MW, solicitado ante OPSB, operación comercial objetivo 2T2027)</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>[Data Center Dynamics](https://www.datacenterdynamics.com/en/news/edgeconnex-plans-120mw-gas-plant-to-power-ohio-data-center/)</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>xAI Colossus 2/Colossus 3 ("MACROHARDRR")</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Southaven, Misisipi / Memphis, Tennessee, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>xAI</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Operando parcialmente/en expansión con crisis regulatoria activa (59 turbinas de gas natural operando en Southaven, la mayoría sin permisos federales de Clean Air Act; demanda de NAACP/Southern Environmental Law Center/Earthjustice desde abr-2026; capacidad total del sitio creciendo hacia 2GW+ en tres edificios)</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>[Technology.org](https://www.technology.org/2026/07/15/xai-59-unpermitted-gas-turbines-southaven-colossus-2/)</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Applied Digital "Delta Forge 1" (planta de gas dedicada Cleco 756MW)</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Rapides Parish, Luisiana, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Applied Digital</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Cleco Power (planta de gas dedicada de 756MW)</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Construcción (campus de USD 3.6 mil millones/430MW, la mayor carga individual jamás atendida por Cleco; rompimiento de tierra ene-2026; operaciones iniciales objetivo mediados de 2027)</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>[Data Center Dynamics](https://www.datacenterdynamics.com/en/news/cleco-to-construct-756mw-natural-gas-plant-to-serve-applied-digitals-data-center-in-rapides-parish-louisiana-report/)</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Agregar 12 proyectos nuevos y 3 cambios de fase (2026-07-24) (#8)
Petroquímica: Wabash Low-Carbon Ammonia Project.
LNG: Corpus Christi Stage 4, Freeport LNG Train 4, Gasoducto Coatzacoalcos II;
actualizaciones de fase en Golden Pass LNG y ST LNG Deepwater Port.
Mining: Elk Creek Critical Minerals, Goldfield Project, Cactus Mine, Doby George
Gold Project, Metates Project.
Data Centers: EdgeConneX PowerConneX New Albany, xAI Colossus 2/3 (Southaven),
Applied Digital Delta Forge 1; actualización de fase en Fermi America Project Matador.


Claude-Session: https://claude.ai/code/session_01FbFqSFuzuNzfzdxHWN1Thd

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -425,16 +425,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
     <col width="55" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -502,7 +502,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://newsroom.fluor.com/news-releases/news-details/2026/Fluor-Awarded-Contract-to-Engineer-and-Design-the-America-First-Refining-Facility-in-Brownsville-Texas/default.aspx</t>
+          <t>[Fluor newsroom](https://newsroom.fluor.com/news-releases/news-details/2026/Fluor-Awarded-Contract-to-Engineer-and-Design-the-America-First-Refining-Facility-in-Brownsville-Texas/default.aspx)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -539,7 +539,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://allstreaminsiders.com/us-exxonmobil-may-build-cracker-pe-plant-in-texas-with-an-8-6-billion-investment/</t>
+          <t>[AllStream Insiders](https://allstreaminsiders.com/us-exxonmobil-may-build-cracker-pe-plant-in-texas-with-an-8-6-billion-investment/)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -576,7 +576,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.bicmagazine.com/departments/operations/cpchem-golden-triangle-polymers-facility-startup-phase/</t>
+          <t>[BIC Magazine](https://www.bicmagazine.com/departments/operations/cpchem-golden-triangle-polymers-facility-startup-phase/)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -613,7 +613,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://constructionfront.com/2025-04-13-technip-energies-to-deliver-blue-point-worlds-largest-low-carbon-ammonia-facility-in-louisiana/</t>
+          <t>[Construction Front](https://constructionfront.com/2025-04-13-technip-energies-to-deliver-blue-point-worlds-largest-low-carbon-ammonia-facility-in-louisiana/)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -650,7 +650,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://eastdaley.com/media-and-news/the-race-is-on-to-build-permian-processing</t>
+          <t>[East Daley](https://eastdaley.com/media-and-news/the-race-is-on-to-build-permian-processing)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -687,7 +687,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.techint.com/en/our-projects/dos-bocas-refinery</t>
+          <t>[Techint](https://www.techint.com/en/our-projects/dos-bocas-refinery)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -724,7 +724,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://www.ogj.com/refining-processing/refining/optimization/article/17279334/pemex-to-proceed-with-dos-bocas-refinery-project</t>
+          <t>[OGJ](https://www.ogj.com/refining-processing/refining/optimization/article/17279334/pemex-to-proceed-with-dos-bocas-refinery-project)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -761,7 +761,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://forbes.com.mx/pemex-invertira-5300-millones-de-dolares-para-reactivar-la-industria-petroquimica/</t>
+          <t>[Forbes México](https://forbes.com.mx/pemex-invertira-5300-millones-de-dolares-para-reactivar-la-industria-petroquimica/)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -798,7 +798,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://forbes.com.mx/pemex-invertira-5300-millones-de-dolares-para-reactivar-la-industria-petroquimica/</t>
+          <t>[Forbes México](https://forbes.com.mx/pemex-invertira-5300-millones-de-dolares-para-reactivar-la-industria-petroquimica/)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -835,7 +835,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://forbes.com.mx/asi-es-la-inversion-de-1553-mdd-por-parte-de-pemex-en-una-planta-de-fertilizantes-en-veracruz/</t>
+          <t>[Forbes México](https://forbes.com.mx/asi-es-la-inversion-de-1553-mdd-por-parte-de-pemex-en-una-planta-de-fertilizantes-en-veracruz/)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -872,7 +872,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://tribuna.com.mx/mexico/2026/06/05/sheinbaum-anuncia-inversion-de-93-mil-mdp-para-reactivar-la-industria-petroquimica-y-de-fertilizantes-en-veracruz_560837/</t>
+          <t>[Tribuna](https://tribuna.com.mx/mexico/2026/06/05/sheinbaum-anuncia-inversion-de-93-mil-mdp-para-reactivar-la-industria-petroquimica-y-de-fertilizantes-en-veracruz_560837/)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -909,7 +909,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://www.pv-magazine-mexico.com/2026/04/28/inician-en-sinaloa-la-construccion-de-la-mayor-planta-de-metanol-ultrabajo-en-carbono-a-partir-de-hidrogeno-verde/</t>
+          <t>[PV Magazine México](https://www.pv-magazine-mexico.com/2026/04/28/inician-en-sinaloa-la-construccion-de-la-mayor-planta-de-metanol-ultrabajo-en-carbono-a-partir-de-hidrogeno-verde/)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://www.h2-view.com/story/first-ammonia-project-on-track-for-2026-fid-despite-topsoe-deal-collapse/2138792.article/</t>
+          <t>[H2 View](https://www.h2-view.com/story/first-ammonia-project-on-track-for-2026-fid-despite-topsoe-deal-collapse/2138792.article/)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -983,7 +983,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://www.debate.com.mx/economia/secretaria-de-economia-complejo-de-amoniaco-en-topolobampo-prioritario-para-el-gobierno-de-mexico-20260713-0092.html</t>
+          <t>[Debate](https://www.debate.com.mx/economia/secretaria-de-economia-complejo-de-amoniaco-en-topolobampo-prioritario-para-el-gobierno-de-mexico-20260713-0092.html)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1020,7 +1020,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://www.icis.com/explore/resources/news/2025/11/13/11155109/lake-charles-methanol-ii-awards-feed-fid-expected-in-q2-2026/</t>
+          <t>[ICIS](https://www.icis.com/explore/resources/news/2025/11/13/11155109/lake-charles-methanol-ii-awards-feed-fid-expected-in-q2-2026/)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://diariodelistmo.com/nacional/este-es-el-avance-que-lleva-la-planta-coquizadora-en-la-refineria-de-salina-cruz/50642321</t>
+          <t>[Diario del Istmo](https://diariodelistmo.com/nacional/este-es-el-avance-que-lleva-la-planta-coquizadora-en-la-refineria-de-salina-cruz/50642321)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1094,7 +1094,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://www.hydrocarbonengineering.com/petrochemicals/06032026/shintech-announces-us34-billion-at-louisiana-petrochemicals-complex/</t>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/petrochemicals/06032026/shintech-announces-us34-billion-at-louisiana-petrochemicals-complex/)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1131,7 +1131,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://www.alchempro.com/news/chemicals-news/ineos-backs-1-7-bn-low-carbon-methanol-project-in-texas-city-310108-newsdetails.htm</t>
+          <t>[Alchempro](https://www.alchempro.com/news/chemicals-news/ineos-backs-1-7-bn-low-carbon-methanol-project-in-texas-city-310108-newsdetails.htm)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1168,7 +1168,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://www.hydrocarbonengineering.com/petrochemicals/13072026/oxea-confirms-fid-for-major-capacity-expansion/</t>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/petrochemicals/13072026/oxea-confirms-fid-for-major-capacity-expansion/)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1205,7 +1205,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://www.ogj.com/refining-processing/gas-processing/news/55320579/targa-advances-permian-gas-pipeline-processing-expansion</t>
+          <t>[OGJ](https://www.ogj.com/refining-processing/gas-processing/news/55320579/targa-advances-permian-gas-pipeline-processing-expansion)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1242,7 +1242,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://www.businesswire.com/news/home/20250806663187/en/Enterprise-Agrees-to-Acquire-Occidentals-Gas-Gathering-Affiliate-Enters-Into-Natural-Gas-Processing-Agreement-Announces-New-Midland-Basin-Natural-Gas-Processing-Plant</t>
+          <t>[Business Wire](https://www.businesswire.com/news/home/20250806663187/en/Enterprise-Agrees-to-Acquire-Occidentals-Gas-Gathering-Affiliate-Enters-Into-Natural-Gas-Processing-Agreement-Announces-New-Midland-Basin-Natural-Gas-Processing-Plant)</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1279,7 +1279,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://naturalgasintel.com/news/mplx-scales-up-for-power-hungry-future-with-natural-gas-focused-growth-plan/</t>
+          <t>[Natural Gas Intel](https://naturalgasintel.com/news/mplx-scales-up-for-power-hungry-future-with-natural-gas-focused-growth-plan/)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1316,7 +1316,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://eastdaley.com/daley-note/mplx-acquires-northwind-for-2-375b-acquires-more-ngls-for-jv-project</t>
+          <t>[East Daley](https://eastdaley.com/daley-note/mplx-acquires-northwind-for-2-375b-acquires-more-ngls-for-jv-project)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1353,7 +1353,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://www.grandforksherald.com/news/local/northern-plains-nitrogen-proposal-receiving-more-attention-amid-global-fertilizer-pressure</t>
+          <t>[Grand Forks Herald](https://www.grandforksherald.com/news/local/northern-plains-nitrogen-proposal-receiving-more-attention-amid-global-fertilizer-pressure)</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1390,7 +1390,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://www.phillips66.com/newsroom/iron-mesa-safely-enters-next-phase-of-construction/</t>
+          <t>[Phillips 66](https://www.phillips66.com/newsroom/iron-mesa-safely-enters-next-phase-of-construction/)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://www.targaresources.com/news-releases/news-release-details/targa-resources-corp-announces-permian-growth-projects-and</t>
+          <t>[Targa Resources](https://www.targaresources.com/news-releases/news-release-details/targa-resources-corp-announces-permian-growth-projects-and)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1464,7 +1464,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://elefanteblanco.mx/2026/01/02/pemex-abre-30-licitaciones-para-obras-en-la-refineria-madero/</t>
+          <t>[Elefante Blanco](https://elefanteblanco.mx/2026/01/02/pemex-abre-30-licitaciones-para-obras-en-la-refineria-madero/)</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1501,7 +1501,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://www.jornada.com.mx/noticia/2026/06/08/economia/da-inicio-ejecucion-de-planta-de-fertilizantes-en-durango-por-parte-de-fermachem</t>
+          <t>[La Jornada](https://www.jornada.com.mx/noticia/2026/06/08/economia/da-inicio-ejecucion-de-planta-de-fertilizantes-en-durango-por-parte-de-fermachem)</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1538,7 +1538,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://downstreamcalendar.com/mcdermott-secures-feed-contract-for-ascension-clean-energy-project/</t>
+          <t>[Downstream Calendar](https://downstreamcalendar.com/mcdermott-secures-feed-contract-for-ascension-clean-energy-project/)</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1575,7 +1575,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://www.businesswire.com/news/home/20260517310811/en/Phillips-66-announces-Zeus-Gas-Plant-and-a-third-Coastal-Bend-Fractionator</t>
+          <t>[Business Wire](https://www.businesswire.com/news/home/20260517310811/en/Phillips-66-announces-Zeus-Gas-Plant-and-a-third-Coastal-Bend-Fractionator)</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1612,12 +1612,49 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://www.usda.gov/about-usda/news/press-releases/2026/07/01/secretary-rollins-announces-500-million-fertilizer-investment-and-expansion-program-strengthen</t>
+          <t>[USDA](https://www.usda.gov/about-usda/news/press-releases/2026/07/01/secretary-rollins-announces-500-million-fertilizer-investment-and-expansion-program-strengthen)</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
           <t>2026-07-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Wabash Low-Carbon Ammonia Project</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>West Terre Haute, Indiana, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Wabash Valley Resources</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Samsung E&amp;C (contrato EPF ~US$475 millones)</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Construcción (groundbreaking 5-ene-2026; amoniaco bajo en carbono 500,000 ton/año con captura de 1.67 millones ton CO2/año; meta de finalización 2029)</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/clean-fuels/06012026/samsung-ea-announces-groundbreaking-of-low-carbon-ammonia-plant/)</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
         </is>
       </c>
     </row>
@@ -1632,16 +1669,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
     <col width="55" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1709,7 +1746,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://www.bechtel.com/press-releases/nextdecade-executes-epc-contract-with-bechtel-for-train-4-at-the-rio-grande-lng-facility/</t>
+          <t>[Bechtel](https://www.bechtel.com/press-releases/nextdecade-executes-epc-contract-with-bechtel-for-train-4-at-the-rio-grande-lng-facility/)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -1746,7 +1783,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://www.bechtel.com/press-releases/sempra-infrastructure-announces-epc-contract-with-bechtel-for-port-arthur-lng-phase-2/</t>
+          <t>[Bechtel](https://www.bechtel.com/press-releases/sempra-infrastructure-announces-epc-contract-with-bechtel-for-port-arthur-lng-phase-2/)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -1783,7 +1820,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.woodside.com/what-we-do/growth-projects/woodside-louisiana-lng</t>
+          <t>[Woodside](https://www.woodside.com/what-we-do/growth-projects/woodside-louisiana-lng)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -1820,7 +1857,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.gem.wiki/CP2_LNG_Terminal</t>
+          <t>[GEM.wiki](https://www.gem.wiki/CP2_LNG_Terminal)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -1857,7 +1894,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.offshore-energy.biz/kbr-zachry-to-work-on-ventures-plaquemines-lng/</t>
+          <t>[Offshore Energy](https://www.offshore-energy.biz/kbr-zachry-to-work-on-ventures-plaquemines-lng/)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -1889,17 +1926,17 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Construcción</t>
+          <t>Construcción/Producción (Train 1: primer LNG mar-2026, primer cargamento exportado 22-abr-2026; Train 2 objetivo 2S2026; Train 3 objetivo 1S2027)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://lngprime.com/contracts-and-tenders/golden-pass-lng-contractors-ink-revised-epc-deal-for-second-and-third-train/169104/</t>
+          <t>[Port Arthur News](https://panews.com/2026/04/24/golden-pass-lng-makes-history-with-first-export-from-sabine-pass-terminal/)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-24</t>
         </is>
       </c>
     </row>
@@ -1931,7 +1968,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://pgjonline.com/news/2026/july/corpus-christi-lng-train-7-cleared-to-introduce-fuel-gas-by-ferc</t>
+          <t>[PGJ](https://pgjonline.com/news/2026/july/corpus-christi-lng-train-7-cleared-to-introduce-fuel-gas-by-ferc)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1968,7 +2005,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2026/06/03/3306350/0/en/delfin-midstream-announces-5-billion-final-investment-decision-for-first-flng-vessel.html</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/06/03/3306350/0/en/delfin-midstream-announces-5-billion-final-investment-decision-for-first-flng-vessel.html)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -2005,7 +2042,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://dossierpolitico.com/2026/07/17/activistas-entregan-90-mil-firmas-para-frenar-proyecto-saguaro-energia-en-sonora/</t>
+          <t>[Dossier Político](https://dossierpolitico.com/2026/07/17/activistas-entregan-90-mil-firmas-para-frenar-proyecto-saguaro-energia-en-sonora/)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -2042,7 +2079,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://www.gem.wiki/New_Fortress_Altamira_FLNG_Terminal</t>
+          <t>[GEM Wiki](https://www.gem.wiki/New_Fortress_Altamira_FLNG_Terminal)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -2079,7 +2116,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://www.naturalgasintel.com/news/glenfarne-lands-investment-for-early-work-on-texas-lng-ahead-of-fid/</t>
+          <t>[Natural Gas Intel](https://www.naturalgasintel.com/news/glenfarne-lands-investment-for-early-work-on-texas-lng-ahead-of-fid/)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -2116,7 +2153,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://pgjonline.com/news/2026/july/commonwealth-lng-awards-main-automation-contract-for-louisiana-export-terminal</t>
+          <t>[PGJ](https://pgjonline.com/news/2026/july/commonwealth-lng-awards-main-automation-contract-for-louisiana-export-terminal)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -2153,7 +2190,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://www.houstonpublicmedia.org/articles/galveston-county/2026/07/14/557086/galveston-pelican-island-lng/</t>
+          <t>[Houston Public Media](https://www.houstonpublicmedia.org/articles/galveston-county/2026/07/14/557086/galveston-pelican-island-lng/)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -2190,7 +2227,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://www.sempra.com/newsroom/press-releases/sempra-infrastructures-eca-lng-phase-1-exports-first-lng-cargo-mexicos</t>
+          <t>[Sempra](https://www.sempra.com/newsroom/press-releases/sempra-infrastructures-eca-lng-phase-1-exports-first-lng-cargo-mexicos)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -2227,7 +2264,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://lngprime.com/americas/gato-negro-eyes-fid-on-mexico-lng-plant-in-late-2026/165906/</t>
+          <t>[LNG Prime](https://lngprime.com/americas/gato-negro-eyes-fid-on-mexico-lng-plant-in-late-2026/165906/)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -2264,7 +2301,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/amigo-lng-awards-landmark-epc-contract-to-dubai-based-drydocks-world-for-worlds-largest-flng-facility-302537739.html</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/amigo-lng-awards-landmark-epc-contract-to-dubai-based-drydocks-world-for-worlds-largest-flng-facility-302537739.html)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -2301,7 +2338,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://www.kbr.com/en/insights-news/press-release/kbr-awarded-feed-coastal-bend-lng-project</t>
+          <t>[KBR](https://www.kbr.com/en/insights-news/press-release/kbr-awarded-feed-coastal-bend-lng-project)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2338,7 +2375,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://www.ferc.gov/gulfstream-lng-terminal-project</t>
+          <t>[FERC](https://www.ferc.gov/gulfstream-lng-terminal-project)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2375,7 +2412,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://glenfarnegroup.com/glenfarne-announces-major-phase-one-alaska-lng-milestones-with-construction-line-pipe-supply-and-in-state-gas-agreements/</t>
+          <t>[Glenfarne](https://glenfarnegroup.com/glenfarne-announces-major-phase-one-alaska-lng-milestones-with-construction-line-pipe-supply-and-in-state-gas-agreements/)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2412,7 +2449,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://pgjonline.com/news/2026/july/311-mile-sonora-gas-pipeline-project-advances-in-mexico</t>
+          <t>[PGJ](https://pgjonline.com/news/2026/july/311-mile-sonora-gas-pipeline-project-advances-in-mexico)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2449,7 +2486,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://www.ogj.com/pipelines-transportation/pipelines/news/55322537/arm-energy-takes-fid-on-23-billion-mustang-express-pipeline</t>
+          <t>[OGJ](https://www.ogj.com/pipelines-transportation/pipelines/news/55322537/arm-energy-takes-fid-on-23-billion-mustang-express-pipeline)</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2486,7 +2523,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://mexicobusiness.news/energy/news/ursus-energy-scales-investment-us21-billion</t>
+          <t>[Mexico Business News](https://mexicobusiness.news/energy/news/ursus-energy-scales-investment-us21-billion)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2523,7 +2560,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2026/07/15/3327983/0/en/Delfin-Midstream-Partners-With-EIG-s-MidOcean-Energy-to-Advance-Second-FLNG-Vessel-Issues-Limited-Notice-to-Proceed-to-Siemens-Energy.html</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/15/3327983/0/en/Delfin-Midstream-Partners-With-EIG-s-MidOcean-Energy-to-Advance-Second-FLNG-Vessel-Issues-Limited-Notice-to-Proceed-to-Siemens-Energy.html)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2560,7 +2597,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://www.naturalgasintel.com/news/texas-gateway-open-season-expands-haynesville-natural-gas-links-amid-lng-growth/</t>
+          <t>[Natural Gas Intel](https://www.naturalgasintel.com/news/texas-gateway-open-season-expands-haynesville-natural-gas-links-amid-lng-growth/)</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2597,7 +2634,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://worldoil.com/news/2026/7/6/argent-lng-awards-engineering-contract-for-port-fourchon-lng-project/</t>
+          <t>[World Oil](https://worldoil.com/news/2026/7/6/argent-lng-awards-engineering-contract-for-port-fourchon-lng-project/)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2629,17 +2666,17 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Permitting/Pre-FID (Draft EIS publicado abr-2026)</t>
+          <t>Permitting/Pre-FID (EIS Final publicado 24-jul-2026, avanzando desde Draft EIS de abr-2026; capacidad 8.4 Mtpa)</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://www.federalregister.gov/documents/2026/04/17/2026-07517/deepwater-port-license-application-st-lng-deepwater-port-development-project-draft-environmental</t>
+          <t>[Federal Register](https://www.federalregister.gov/documents/2026/07/24/2026-14963/deepwater-port-license-application-st-lng-deepwater-port-development-project-final-environmental)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-24</t>
         </is>
       </c>
     </row>
@@ -2671,7 +2708,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://naturalgasintel.com/news/kinder-morgan-greenlights-7b-in-natural-gas-pipeline-projects-amid-regulatory-speedup/</t>
+          <t>[Natural Gas Intel](https://naturalgasintel.com/news/kinder-morgan-greenlights-7b-in-natural-gas-pipeline-projects-amid-regulatory-speedup/)</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -2708,7 +2745,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://naturalgasintel.com/news/kinder-morgan-greenlights-7b-in-natural-gas-pipeline-projects-amid-regulatory-speedup/</t>
+          <t>[Natural Gas Intel](https://naturalgasintel.com/news/kinder-morgan-greenlights-7b-in-natural-gas-pipeline-projects-amid-regulatory-speedup/)</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2745,7 +2782,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://lngprime.com/americas/kinder-morgan-seeks-doe-extension-for-gulf-lng-export-project/184334/</t>
+          <t>[LNG Prime](https://lngprime.com/americas/kinder-morgan-seeks-doe-extension-for-gulf-lng-export-project/184334/)</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2782,12 +2819,123 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://investors.bakerhughes.com/news/press-releases/news-details/2026/Baker-Hughes-Secures-Substantial-Equipment-and-Services-Awards-for-Chenieres-Sabine-Pass-LNG-Facility/default.aspx</t>
+          <t>[Baker Hughes](https://investors.bakerhughes.com/news/press-releases/news-details/2026/Baker-Hughes-Secures-Substantial-Equipment-and-Services-Awards-for-Chenieres-Sabine-Pass-LNG-Facility/default.aspx)</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
           <t>2026-07-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Corpus Christi Stage 4</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>San Patricio County / Corpus Christi, Texas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Cheniere Energy</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Permitting (solicitud FERC en proceso desde 17-feb-2026; DOE revisando solicitud de exportación; EIS borrador esperado sep-2026; incluye gasoducto de alimentación CCPL de 42"/26 millas)</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>[Federal Register](https://www.federalregister.gov/documents/2026/05/05/2026-08654/cheniere-corpus-christi-pipeline-lp-corpus-christi-liquefaction-stage-iv-llc-corpus-christi)</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Freeport LNG Train 4</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Freeport, Texas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Freeport LNG Development, L.P.</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Pre-FID (FERC extendió plazo de puesta en servicio a ago-2028; capacidad 5.1 Mtpa)</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>[Natural Gas Intel](https://www.naturalgasintel.com/news/ferc-approves-extension-for-freeport-lngs-fourth-train-expansion-project/)</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Gasoducto Coatzacoalcos II (alimenta PODEBI Coatzacoalcos II)</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Coatzacoalcos, Veracruz, México</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>CFE / CENAGAS</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Por definir (licitación pública, adjudicación 15-jul-2026)</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Bidding/Construcción inminente (9.69 km en dos etapas; inversión ~US$177 millones; plazo de ejecución 17 meses)</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>[Proyectos México](https://www.proyectosmexico.gob.mx/proyecto_inversion/1076-gasoducto-coatzacoalcos-ii/)</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
         </is>
       </c>
     </row>
@@ -2802,16 +2950,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
     <col width="55" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2879,7 +3027,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://www.miningweekly.com/article/ivanhoe-electric-pencils-in-2026-construction-start-at-arizona-copper-mine-2025-06-25</t>
+          <t>[Mining Weekly](https://www.miningweekly.com/article/ivanhoe-electric-pencils-in-2026-construction-start-at-arizona-copper-mine-2025-06-25)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -2916,7 +3064,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1322422/000106299326001973/exhibit99-2.htm</t>
+          <t>[SEC/Hudbay](https://www.sec.gov/Archives/edgar/data/1322422/000106299326001973/exhibit99-2.htm)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -2953,7 +3101,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/863064/000086306426000019/ex12d16mr_resolutionland.htm</t>
+          <t>[SEC](https://www.sec.gov/Archives/edgar/data/863064/000086306426000019/ex12d16mr_resolutionland.htm)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -2990,7 +3138,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.nevadaappeal.com/news/2026/mar/26/lithium-americas-900-construction-workers-at-thacker-pass-mine/</t>
+          <t>[Nevada Appeal](https://www.nevadaappeal.com/news/2026/mar/26/lithium-americas-900-construction-workers-at-thacker-pass-mine/)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -3027,7 +3175,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.mining.com/teck-agnico-team-up-at-san-nicolas-copper-project-in-mexico/</t>
+          <t>[Mining.com](https://www.mining.com/teck-agnico-team-up-at-san-nicolas-copper-project-in-mexico/)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -3064,7 +3212,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://energymagazine.mx/2025/10/grupo-mexico-espera-autorizacion-federal-para-continuar-proyectos-mineros-por-10-mil-200-mdd/</t>
+          <t>[Energy Magazine MX](https://energymagazine.mx/2025/10/grupo-mexico-espera-autorizacion-federal-para-continuar-proyectos-mineros-por-10-mil-200-mdd/)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -3101,7 +3249,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://www.bnamericas.com/en/news/southern-copper-wins-permits-for-us551mn-el-pilar-in-mexico</t>
+          <t>[BNamericas](https://www.bnamericas.com/en/news/southern-copper-wins-permits-for-us551mn-el-pilar-in-mexico)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -3138,7 +3286,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://m3eng.com/portfolio/buenavista-del-cobre-concentradora-no-2/</t>
+          <t>[M3 Engineering](https://m3eng.com/portfolio/buenavista-del-cobre-concentradora-no-2/)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -3175,7 +3323,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://mineriaenlinea.com/2026/04/torex-gold-alcanza-velocidad-de-crucero-en-media-luna-9-meses-adelante-de-cronograma/</t>
+          <t>[Minería en Línea](https://mineriaenlinea.com/2026/04/torex-gold-alcanza-velocidad-de-crucero-en-media-luna-9-meses-adelante-de-cronograma/)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -3212,7 +3360,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://www.mining.com/nevada-copper-unveils-restart-and-financing-plan-for-pumpkin-hollow/</t>
+          <t>[Mining.com](https://www.mining.com/nevada-copper-unveils-restart-and-financing-plan-for-pumpkin-hollow/)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -3249,7 +3397,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://www.usda.gov/about-usda/news/press-releases/2026/07/07/usda-advances-trump-administration-effort-boost-us-mineral-energy-production</t>
+          <t>[USDA](https://www.usda.gov/about-usda/news/press-releases/2026/07/07/usda-advances-trump-administration-effort-boost-us-mineral-energy-production)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -3286,7 +3434,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/perpetua-resources-advances-construction-of-the-stibnite-gold-project-302787012.html</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/perpetua-resources-advances-construction-of-the-stibnite-gold-project-302787012.html)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -3323,7 +3471,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://silvertigermetals.com/news/2026/silver-tiger-metals-awards-engineering-procurement-and-construction-management-contract-and-provides-construction-update</t>
+          <t>[Silver Tiger Metals](https://silvertigermetals.com/news/2026/silver-tiger-metals-awards-engineering-procurement-and-construction-management-contract-and-provides-construction-update)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -3360,7 +3508,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/vizsla-silver-awards-epcm-and-mine-design-contracts-for-the-development-of-the-panuco-silver-gold-project-302750621.html</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/vizsla-silver-awards-epcm-and-mine-design-contracts-for-the-development-of-the-panuco-silver-gold-project-302750621.html)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -3397,7 +3545,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://orlamining.com/news/orla-announces-results-of-updated-feasibility-study-for-south-railroad-project/</t>
+          <t>[Orla Mining](https://orlamining.com/news/orla-announces-results-of-updated-feasibility-study-for-south-railroad-project/)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -3434,7 +3582,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://www.miningweekly.com/article/minera-alamos-confirms-low-cost-near-term-mining-possible-at-copperstone-in-arizona-2026-05-28</t>
+          <t>[Mining Weekly](https://www.miningweekly.com/article/minera-alamos-confirms-low-cost-near-term-mining-possible-at-copperstone-in-arizona-2026-05-28)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -3471,7 +3619,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://www.wyomingnews.com/rawlinstimes/plans-move-forward-for-ck-gold-project-as-developers-target-2026-construction-start/article_b2bb147e-2f92-4ca2-bf86-fcc9983917a7.html</t>
+          <t>[Wyoming News](https://www.wyomingnews.com/rawlinstimes/plans-move-forward-for-ck-gold-project-as-developers-target-2026-construction-start/article_b2bb147e-2f92-4ca2-bf86-fcc9983917a7.html)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -3508,7 +3656,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://www.juniorminingnetwork.com/junior-miner-news/press-releases/1082-tsx/ag/206222-first-majestic-receives-construction-permits-for-santo-nino-and-navidad-advances-development-across-the-santa-elena-district.html</t>
+          <t>[First Majestic](https://www.juniorminingnetwork.com/junior-miner-news/press-releases/1082-tsx/ag/206222-first-majestic-receives-construction-permits-for-santo-nino-and-navidad-advances-development-across-the-santa-elena-district.html)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -3545,7 +3693,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/0001286973/000106299326002645/exhibit99-2.htm</t>
+          <t>[SEC/Americas Gold and Silver](https://www.sec.gov/Archives/edgar/data/0001286973/000106299326002645/exhibit99-2.htm)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -3582,7 +3730,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://www.kitco.com/news/off-the-wire/2026-06-08/minera-frisco-restarts-two-mexico-mines-plans-new-silver-unit</t>
+          <t>[Kitco](https://www.kitco.com/news/off-the-wire/2026-06-08/minera-frisco-restarts-two-mexico-mines-plans-new-silver-unit)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -3619,7 +3767,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/trilogy-metals-announces-publication-of-federal-and-state-permitting-schedule-for-arctic-project-establishing-defined-timeline-toward-a-record-of-decision-by-september-2028-302827083.html</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/trilogy-metals-announces-publication-of-federal-and-state-permitting-schedule-for-arctic-project-establishing-defined-timeline-toward-a-record-of-decision-by-september-2028-302827083.html)</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -3656,7 +3804,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://www.northernminer.com/news/gogold-approved-to-build-227m-mine-in-mexico/1003891932/</t>
+          <t>[Northern Miner](https://www.northernminer.com/news/gogold-approved-to-build-227m-mine-in-mexico/1003891932/)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -3693,7 +3841,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://www.bnamericas.com/en/news/discovery-advances-permitting-financing-at-us606mn-cordero-in-mexico</t>
+          <t>[BNamericas](https://www.bnamericas.com/en/news/discovery-advances-permitting-financing-at-us606mn-cordero-in-mexico)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -3730,7 +3878,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://resourceworld.com/tocvan-ventures-eyes-mexican-gold-pour-by-q4-2026/</t>
+          <t>[Resource World](https://resourceworld.com/tocvan-ventures-eyes-mexican-gold-pour-by-q4-2026/)</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -3767,7 +3915,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://www.fresnilloplc.com/portfolio/exploration/orisyvo/</t>
+          <t>[Fresnillo plc](https://www.fresnilloplc.com/portfolio/exploration/orisyvo/)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -3804,7 +3952,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/</t>
+          <t>[Mining.com](https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -3841,7 +3989,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/</t>
+          <t>[Mining.com](https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/)</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -3878,7 +4026,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/</t>
+          <t>[Mining.com](https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/)</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -3915,7 +4063,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://im-mining.com/2026/06/29/metso-to-supply-additional-crushing-package-for-grupo-mexico-la-caridad-copper-concentrator/</t>
+          <t>[IM Mining](https://im-mining.com/2026/06/29/metso-to-supply-additional-crushing-package-for-grupo-mexico-la-caridad-copper-concentrator/)</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -3952,7 +4100,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2026/05/21/3299182</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/05/21/3299182)</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3989,7 +4137,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://mexicobusiness.news/mining/news/grupo-mexicos-asarco-may-reopen-united-states</t>
+          <t>[Mexico Business News](https://mexicobusiness.news/mining/news/grupo-mexicos-asarco-may-reopen-united-states)</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -4026,7 +4174,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>https://mineraalamos.com/our-assets/cerro-de-oro-project/</t>
+          <t>[Minera Alamos](https://mineraalamos.com/our-assets/cerro-de-oro-project/)</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -4063,7 +4211,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>https://www.globalminingreview.com/mining/11022025/antler-copper-project-achieves-critical-federal-permitting-milestone/</t>
+          <t>[Global Mining Review](https://www.globalminingreview.com/mining/11022025/antler-copper-project-achieves-critical-federal-permitting-milestone/)</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -4100,7 +4248,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>https://www.blm.gov/press-release/blm-approves-lisbon-valley-copper-mine-expansion-utah</t>
+          <t>[BLM](https://www.blm.gov/press-release/blm-approves-lisbon-valley-copper-mine-expansion-utah)</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -4137,7 +4285,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>https://investingnews.com/smackover-lithium-announces-the-award-of-last-key-construction-contract-for-the-south-west-arkansas-project-ahead-of-final-investment-decision/</t>
+          <t>[InvestingNews](https://investingnews.com/smackover-lithium-announces-the-award-of-last-key-construction-contract-for-the-south-west-arkansas-project-ahead-of-final-investment-decision/)</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -4174,12 +4322,197 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/0000831259/000083125926000033/a2q2026exhibit991.htm</t>
+          <t>[SEC/Freeport-McMoRan](https://www.sec.gov/Archives/edgar/data/0000831259/000083125926000033/a2q2026exhibit991.htm)</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
           <t>2026-07-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Elk Creek Critical Minerals Project</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Elk Creek, Nebraska, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>NioCorp Developments Ltd.</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Construcción (portal de mina de doble rampa, ~US$44.6 millones, iniciado feb/mar-2026; proyecto de niobio/escandio/titanio con planta de superficie que requerirá tubería de proceso)</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>[NioCorp](https://niocorp.com/niocorp-launches-construction-of-elk-creek-critical-minerals-project-mine-portal/)</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Goldfield Project</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Goldfield, Nevada, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Centerra Gold Inc.</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Ingeniería/Construcción temprana (ingeniería de detalle y procura de largo plazo en 2026; construcción mayor de pila de lixiviación y circuitos de trituración/procesamiento en 2027; primera producción fin de 2028)</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>[E&amp;MJ](https://www.e-mj.com/breaking-news/centerra-advances-goldfield-project-in-nevada/)</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Cactus Mine (distrito Copper World/Arizona Sonoran)</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Casa Grande, Arizona, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Hudbay Minerals (adquisición de Arizona Sonoran Copper Co. anunciada 2-mar-2026)</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Desarrollo/Feasibility (planta SX-EW de cátodos de cobre, ~103,000 t Cu/año proyectadas; Hudbay busca fusionarlo con el distrito Copper World adyacente ya rastreado)</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/03/02/3247157/0/en/hudbay-to-acquire-arizona-sonoran-creating-the-third-largest-copper-district-in-north-america.html)</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Doby George Gold Project (Distrito Aura)</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>~120 km al norte de Elko, Nevada, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Western Exploration Inc.</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>No especificado (WSP realiza feasibility study; Stantec y Kappes Cassidy en estudios ambientales)</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Feasibility/Permitting (PEA positiva 2025; Mine Plan of Operations en preparación; proyecto de lixiviación en pilas de óxidos)</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>[Western Exploration](https://www.westernexploration.com/news-and-updates/news/news-details/2026/Western-Exploration-Outlines-2026-Program-to-Advance-Doby-George-Permitting-and-Expand-Gravel-Creek-Resources-2026-aaotfYHcV7/default.aspx)</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Metates Project</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Durango, México</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Chesapeake Gold Corp.</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Feasibility (prefeasibility study objetivo 2026; pruebas metalúrgicas de lixiviación de sulfuros y estudios ambientales de línea base en curso; uno de los mayores depósitos de oro-plata no desarrollados de América)</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>[Chesapeake Gold Corp.](https://chesapeakegold.com/metates/)</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
         </is>
       </c>
     </row>
@@ -4194,16 +4527,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
     <col width="55" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4271,7 +4604,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/vantage-breaks-ground-on-texas-gigawatt-data-center-campus-for-openai/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/vantage-breaks-ground-on-texas-gigawatt-data-center-campus-for-openai/)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -4308,7 +4641,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://epoch.ai/publications/openai-stargate-where-the-us-sites-stand</t>
+          <t>[Epoch AI](https://epoch.ai/publications/openai-stargate-where-the-us-sites-stand)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -4345,7 +4678,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/crusoe-tops-out-final-building-at-openai-stargate-data-center-campus-in-abilene-texas/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/crusoe-tops-out-final-building-at-openai-stargate-data-center-campus-in-abilene-texas/)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -4382,7 +4715,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.cnbc.com/2026/06/22/chevron-cvx-microsoft-msft-natural-gas-data-center.html</t>
+          <t>[CNBC](https://www.cnbc.com/2026/06/22/chevron-cvx-microsoft-msft-natural-gas-data-center.html)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -4419,7 +4752,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.gob.mx/presidencia/prensa/plan-mexico-avanza-se-anuncia-inversion-de-4-mil-800-mdd-de-cloudhq-para-la-construccion-de-6-centros-de-datos-en-queretaro</t>
+          <t>[Gobierno de México](https://www.gob.mx/presidencia/prensa/plan-mexico-avanza-se-anuncia-inversion-de-4-mil-800-mdd-de-cloudhq-para-la-construccion-de-6-centros-de-datos-en-queretaro)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -4456,7 +4789,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.ucs.org/about/news/judge-orders-meta-explain-new-gas-demand-hyperscale-louisiana-data-center</t>
+          <t>[UCS](https://www.ucs.org/about/news/judge-orders-meta-explain-new-gas-demand-hyperscale-louisiana-data-center)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -4493,7 +4826,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://www.datacenterfrontier.com/site-selection/article/55305086/nv1-and-the-nevada-hyperscale-boom-vantage-data-centers-bets-3b-on-the-ai-future</t>
+          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55305086/nv1-and-the-nevada-hyperscale-boom-vantage-data-centers-bets-3b-on-the-ai-future)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -4530,7 +4863,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/cloudburst-breaks-ground-on-gigawatt-scale-data-center-campus-in-texas/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/cloudburst-breaks-ground-on-gigawatt-scale-data-center-campus-in-texas/)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -4567,7 +4900,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/prometheus-hyperscale-details-plans-for-dallas-data-center-campus/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/prometheus-hyperscale-details-plans-for-dallas-data-center-campus/)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -4604,7 +4937,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://www.businesswire.com/news/home/20260126236053/en/Pacifico-Energy-Secures-7.65-GW-Power-Generation-Permit-for-GW-Ranch-Project</t>
+          <t>[Business Wire](https://www.businesswire.com/news/home/20260126236053/en/Pacifico-Energy-Secures-7.65-GW-Power-Generation-Permit-for-GW-Ranch-Project)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -4641,7 +4974,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/amazon-looks-to-build-large-scale-data-center-campus-next-to-nuclear-plant-in-texas/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/amazon-looks-to-build-large-scale-data-center-campus-next-to-nuclear-plant-in-texas/)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -4678,7 +5011,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://mexiconewsdaily.com/business/durango-data-center-fertilizer-plant-investment-fermaca/</t>
+          <t>[Mexico News Daily](https://mexiconewsdaily.com/business/durango-data-center-fertilizer-plant-investment-fermaca/)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -4715,7 +5048,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/circe-energy-secures-2gw-of-natural-gas-capacity-for-west-texas-data-center-campus/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/circe-energy-secures-2gw-of-natural-gas-capacity-for-west-texas-data-center-campus/)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -4752,7 +5085,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://sourcenm.com/2026/07/16/new-mexico-land-commissioner-blocks-project-jupiter-related-pipeline-from-building-on-state-land/</t>
+          <t>[Source NM](https://sourcenm.com/2026/07/16/new-mexico-land-commissioner-blocks-project-jupiter-related-pipeline-from-building-on-state-land/)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -4789,7 +5122,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/powerplay-ai-announces-400-mw-behind-the-meter-ai-data-center-development-in-greater-abilene-with-nasdaq-listed-neocloud-joint-venture-partner-302829610.html</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/powerplay-ai-announces-400-mw-behind-the-meter-ai-data-center-development-in-greater-abilene-with-nasdaq-listed-neocloud-joint-venture-partner-302829610.html)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -4826,7 +5159,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/liberty-energy-powerbridge-form-jv-to-power-planned-2gw-data-center-in-west-texas/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/liberty-energy-powerbridge-form-jv-to-power-planned-2gw-data-center-in-west-texas/)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -4863,7 +5196,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://www.powermag.com/nuclear-natural-gas-power-generation-planned-for-massive-new-mexico-data-center-site/</t>
+          <t>[PowerMag](https://www.powermag.com/nuclear-natural-gas-power-generation-planned-for-massive-new-mexico-data-center-site/)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -4900,7 +5233,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://www.datacenterfrontier.com/site-selection/article/55289667/powering-ai-in-the-permian-texas-critical-data-centers-sustainable-energy-play</t>
+          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55289667/powering-ai-in-the-permian-texas-critical-data-centers-sustainable-energy-play)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -4937,7 +5270,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://openai.com/index/five-new-stargate-sites/</t>
+          <t>[OpenAI](https://openai.com/index/five-new-stargate-sites/)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -4974,7 +5307,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://openai.com/index/five-new-stargate-sites/</t>
+          <t>[OpenAI](https://openai.com/index/five-new-stargate-sites/)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -5011,7 +5344,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://mexiconewsdaily.com/business/aws-invest-5b-mexico-data-region/</t>
+          <t>[Mexico News Daily](https://mexiconewsdaily.com/business/aws-invest-5b-mexico-data-region/)</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -5048,7 +5381,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/oracle-and-openai-start-construction-on-stargate-data-center-campus-in-saline-township-michigan/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/oracle-and-openai-start-construction-on-stargate-data-center-campus-in-saline-township-michigan/)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -5085,7 +5418,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://www.valleynewslive.com/2026/07/13/applied-digital-expands-north-dakota-eyes-oliver-county-third-data-center/</t>
+          <t>[Valley News Live](https://www.valleynewslive.com/2026/07/13/applied-digital-expands-north-dakota-eyes-oliver-county-third-data-center/)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -5122,7 +5455,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://energymagazine.mx/2026/01/el-data-center-verde-que-encendio-la-polemica-asi-sera-el-proyecto-de-ia-en-nuevo-leon-que-usara-tecnologia-de-nvidia/</t>
+          <t>[Energy Magazine MX](https://energymagazine.mx/2026/01/el-data-center-verde-que-encendio-la-polemica-asi-sera-el-proyecto-de-ia-en-nuevo-leon-que-usara-tecnologia-de-nvidia/)</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -5159,7 +5492,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://www.constructiondive.com/news/data-center-cleanarc-breaks-ground-virginia-campus/806489/</t>
+          <t>[Construction Dive](https://www.constructiondive.com/news/data-center-cleanarc-breaks-ground-virginia-campus/806489/)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -5196,7 +5529,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://www.ksl.com/article/51402125/groundbreaking-for-new-millard-county-artificial-intelligence-data-center</t>
+          <t>[KSL](https://www.ksl.com/article/51402125/groundbreaking-for-new-millard-county-artificial-intelligence-data-center)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -5233,7 +5566,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://governor.mo.gov/press-releases/archive/amazon-investing-10-billion-montgomery-county</t>
+          <t>[Governor.mo.gov](https://governor.mo.gov/press-releases/archive/amazon-investing-10-billion-montgomery-county)</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -5270,7 +5603,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://www.stlpr.org/government-politics-issues/2026-05-21/missouri-governor-google-announce-15-billion-data-center-montgomery-county</t>
+          <t>[STLPR](https://www.stlpr.org/government-politics-issues/2026-05-21/missouri-governor-google-announce-15-billion-data-center-montgomery-county)</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -5307,7 +5640,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2026/07/06/3322404/0/en/big-digital-energy-announces-partnership-with-10netzero-to-acquire-power-ready-hood-county-texas-site-for-ai-datacenter-development.html</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/06/3322404/0/en/big-digital-energy-announces-partnership-with-10netzero-to-acquire-power-ready-hood-county-texas-site-for-ai-datacenter-development.html)</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -5344,7 +5677,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/)</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -5381,7 +5714,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/meta-files-to-expand-campus-in-el-paso-texas-with-12-new-buildings/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/meta-files-to-expand-campus-in-el-paso-texas-with-12-new-buildings/)</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -5418,7 +5751,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/softbank-eyes-10gw-data-center-at-former-doe-nuclear-enrichment-site-in-ohio/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/softbank-eyes-10gw-data-center-at-former-doe-nuclear-enrichment-site-in-ohio/)</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -5455,7 +5788,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/)</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -5492,7 +5825,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>https://www.williams.com/2026/07/13/williams-announces-5-34-billion-investment-in-power-innovation-joint-venture-from-blackstone/</t>
+          <t>[Williams Companies](https://www.williams.com/2026/07/13/williams-announces-5-34-billion-investment-in-power-innovation-joint-venture-from-blackstone/)</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -5529,7 +5862,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/cleancore-solutions-zone-announces-closing-of-first-data-center-project-establishing-its-critical-infrastructure-buildout-for-the-ai-economy-302821421.html</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/cleancore-solutions-zone-announces-closing-of-first-data-center-project-establishing-its-critical-infrastructure-buildout-for-the-ai-economy-302821421.html)</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -5566,7 +5899,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>https://www.bloomberg.com/news/articles/2026-06-09/crusoe-touts-5-gigawatts-worth-of-data-centers-deals-pauses-wyoming-site</t>
+          <t>[Bloomberg](https://www.bloomberg.com/news/articles/2026-06-09/crusoe-touts-5-gigawatts-worth-of-data-centers-deals-pauses-wyoming-site)</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -5603,7 +5936,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>https://www.hpcwire.com/off-the-wire/core-scientific-plans-expansion-to-1-5gw-of-gross-power-at-pecos-texas-campus/</t>
+          <t>[HPCwire](https://www.hpcwire.com/off-the-wire/core-scientific-plans-expansion-to-1-5gw-of-gross-power-at-pecos-texas-campus/)</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -5640,7 +5973,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>https://utahnewsdispatch.com/2026/05/19/renderings-show-massive-data-center-box-elder-utah-permits-could-take-years/</t>
+          <t>[Utah News Dispatch](https://utahnewsdispatch.com/2026/05/19/renderings-show-massive-data-center-box-elder-utah-permits-could-take-years/)</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -5667,22 +6000,22 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Primoris Services Corporation (balance of plant, turbinas de gas)</t>
+          <t>Primoris Services Corporation (balance of plant, turbinas de gas); Siemens Energy (suministro de turbinas)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Construcción (excavación de isla de turbinas completada; EPC firmado)</t>
+          <t>Construcción (excavación de isla de turbinas completada; EPC firmado; 3 turbinas de gas Siemens Energy SGT6-5000F, hasta 780MW ciclo simple, llegaron al Puerto de Houston 21-jul-2026 con destino al sitio; meta de 1GW en línea a fines de 2026)</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/fermi-selects-primoris-services-corporation-to-engineer-and-construct-balance-of-plant-for-first-six-sgt-800-gas-turbines-of-phase-one-power-buildout-302814505.html</t>
+          <t>[StockTitan](https://www.stocktitan.net/news/FRMI/fermi-announces-first-siemens-turbines-arrive-at-port-of-qg7ienp885jk.html)</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-24</t>
         </is>
       </c>
     </row>
@@ -5714,7 +6047,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>https://www.kltv.com/2026/03/20/president-trump-approves-16-billion-natural-gas-generator-be-installed-anderson-county/</t>
+          <t>[KLTV](https://www.kltv.com/2026/03/20/president-trump-approves-16-billion-natural-gas-generator-be-installed-anderson-county/)</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -5751,7 +6084,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>https://wvmetronews.com/2026/07/16/mon-power-president-says-data-centers-will-end-up-paying-for-natural-gas-powered-power-plant/</t>
+          <t>[WV MetroNews](https://wvmetronews.com/2026/07/16/mon-power-president-says-data-centers-will-end-up-paying-for-natural-gas-powered-power-plant/)</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -5788,7 +6121,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>https://www.utilitydive.com/news/iep-plans-944-mw-behind-the-meter-gas-plant-in-pennsylvania-to-power-data-c/758830/</t>
+          <t>[Utility Dive](https://www.utilitydive.com/news/iep-plans-944-mw-behind-the-meter-gas-plant-in-pennsylvania-to-power-data-c/758830/)</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -5825,7 +6158,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/aws-files-for-12bn-data-center-campus-outside-houston-texas/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/aws-files-for-12bn-data-center-campus-outside-houston-texas/)</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -5862,7 +6195,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>https://www.crusoe.ai/resources/newsroom/crusoe-and-lancium-announce-1-gigawatt-ai-data-center-campus-in-childress-texas</t>
+          <t>[Crusoe](https://www.crusoe.ai/resources/newsroom/crusoe-and-lancium-announce-1-gigawatt-ai-data-center-campus-in-childress-texas)</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -5899,7 +6232,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/)</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -5936,7 +6269,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>https://www.powermag.com/new-200-mw-gas-fired-plant-in-ohio-will-power-meta-data-center/</t>
+          <t>[PowerMag](https://www.powermag.com/new-200-mw-gas-fired-plant-in-ohio-will-power-meta-data-center/)</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -5973,7 +6306,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>https://www.aterio.io/blog/crusoe-launches-usd29b-goodnight-campus-in-claude-mirroring-openai-s-stargate</t>
+          <t>[Aterio](https://www.aterio.io/blog/crusoe-launches-usd29b-goodnight-campus-in-claude-mirroring-openai-s-stargate)</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -6010,7 +6343,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>https://www.ajc.com/business/2026/07/officials-order-georgia-data-centers-pop-up-power-plant-to-halt-construction/</t>
+          <t>[AJC](https://www.ajc.com/business/2026/07/officials-order-georgia-data-centers-pop-up-power-plant-to-halt-construction/)</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -6047,7 +6380,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/stark-power-lands-56gw-data-center-development-portfolio-in-sagebrush-acquisition/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/stark-power-lands-56gw-data-center-development-portfolio-in-sagebrush-acquisition/)</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -6084,7 +6417,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>https://www.datacenterfrontier.com/site-selection/article/55281341/pennsylvanias-homer-city-energy-campus-a-brownfield-transformed-for-data-center-innovation</t>
+          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55281341/pennsylvanias-homer-city-energy-campus-a-brownfield-transformed-for-data-center-innovation)</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -6121,7 +6454,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>https://www.datacenterknowledge.com/data-center-site-selection/nebius-plans-300-mw-data-center-in-new-jersey-amid-us-expansion</t>
+          <t>[Data Center Knowledge](https://www.datacenterknowledge.com/data-center-site-selection/nebius-plans-300-mw-data-center-in-new-jersey-amid-us-expansion)</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -6158,7 +6491,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/terravolt-inks-natural-gas-supply-deal-for-onsite-power-plant-at-planned-data-center-campus-in-idaho/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/terravolt-inks-natural-gas-supply-deal-for-onsite-power-plant-at-planned-data-center-campus-in-idaho/)</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -6195,12 +6528,123 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/cyrusone-announces-sixth-data-center-campus-in-san-antonio-texas/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/cyrusone-announces-sixth-data-center-campus-in-san-antonio-texas/)</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
           <t>2026-07-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>EdgeConneX PowerConneX New Albany Energy Center (I y II)</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>New Albany, Licking County, Ohio, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>EdgeConneX (propiedad de EQT Infrastructure)</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>No especificado (desarrollado vía afiliada PowerConneX)</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Construcción (PowerConneX I, 120MW, certificado OPSB 22-jul-2025, construcción iniciada sep-2025, operación comercial posible 3T2026; PowerConneX II, 216MW, solicitado ante OPSB, operación comercial objetivo 2T2027)</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>[Data Center Dynamics](https://www.datacenterdynamics.com/en/news/edgeconnex-plans-120mw-gas-plant-to-power-ohio-data-center/)</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>xAI Colossus 2/Colossus 3 ("MACROHARDRR")</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Southaven, Misisipi / Memphis, Tennessee, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>xAI</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Operando parcialmente/en expansión con crisis regulatoria activa (59 turbinas de gas natural operando en Southaven, la mayoría sin permisos federales de Clean Air Act; demanda de NAACP/Southern Environmental Law Center/Earthjustice desde abr-2026; capacidad total del sitio creciendo hacia 2GW+ en tres edificios)</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>[Technology.org](https://www.technology.org/2026/07/15/xai-59-unpermitted-gas-turbines-southaven-colossus-2/)</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Applied Digital "Delta Forge 1" (planta de gas dedicada Cleco 756MW)</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Rapides Parish, Luisiana, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Applied Digital</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Cleco Power (planta de gas dedicada de 756MW)</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Construcción (campus de USD 3.6 mil millones/430MW, la mayor carga individual jamás atendida por Cleco; rompimiento de tierra ene-2026; operaciones iniciales objetivo mediados de 2027)</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>[Data Center Dynamics](https://www.datacenterdynamics.com/en/news/cleco-to-construct-756mw-natural-gas-plant-to-serve-applied-digitals-data-center-in-rapides-parish-louisiana-report/)</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Agregar 6 proyectos nuevos y 12 cambios de fase (2026-07-28)
Nuevos:
- Petroquímica: Green Fuels Operating - Refinería Duncan (Oklahoma)
- LNG: CP2 LNG Fase 3 (Louisiana)
- Mining: Pathfinder Tonopah (Nevada), La Colorada Mine expansión (Sonora)
- Data Centers: Anthropic/Nexus Hubbard Campus (Texas), Stillwater Technology Park (Georgia)

Cambios de fase: CF Industries Blue Point, Fertinal-ProAgro, Rio Grande LNG,
Corpus Christi Stage 3, Los Ricos South Mine, Copper World Complex,
Resolution Copper, Stargate Frontier Campus, SB Energy PORTS Technology
Campus, Fermaca Digital City, Prometheus Hyperscale Dallas, EdgeConneX
PowerConneX New Albany.

Se regeneró proyectos.xlsx con el acumulado completo (una hoja por industria).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012WFngDt9cuLNAQtoEh1sN8
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -35,6 +35,7 @@
     </font>
     <font>
       <name val="Arial"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="3">
@@ -66,7 +67,7 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -436,16 +437,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -513,7 +514,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>https://newsroom.fluor.com/news-releases/news-details/2026/Fluor-Awarded-Contract-to-Engineer-and-Design-the-America-First-Refining-Facility-in-Brownsville-Texas/default.aspx</t>
+          <t>[Fluor newsroom](https://newsroom.fluor.com/news-releases/news-details/2026/Fluor-Awarded-Contract-to-Engineer-and-Design-the-America-First-Refining-Facility-in-Brownsville-Texas/default.aspx)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -550,7 +551,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>https://allstreaminsiders.com/us-exxonmobil-may-build-cracker-pe-plant-in-texas-with-an-8-6-billion-investment/</t>
+          <t>[AllStream Insiders](https://allstreaminsiders.com/us-exxonmobil-may-build-cracker-pe-plant-in-texas-with-an-8-6-billion-investment/)</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -587,7 +588,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>https://www.bicmagazine.com/departments/operations/cpchem-golden-triangle-polymers-facility-startup-phase/</t>
+          <t>[BIC Magazine](https://www.bicmagazine.com/departments/operations/cpchem-golden-triangle-polymers-facility-startup-phase/)</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -619,17 +620,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Construcción</t>
+          <t>Construcción (impulso federal de permisos anunciado may-2026 con finalización esperada en 45 días; CF Industries confirma inicio de construcción en 2026)</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>https://constructionfront.com/2025-04-13-technip-energies-to-deliver-blue-point-worlds-largest-low-carbon-ammonia-facility-in-louisiana/</t>
+          <t>[Construction Front](https://constructionfront.com/2025-04-13-technip-energies-to-deliver-blue-point-worlds-largest-low-carbon-ammonia-facility-in-louisiana/); [FuelCellsWorks](https://fuelcellsworks.com/2026/05/07/h2/cf-industries-targets-construction-start-this-year-on-blue-hydrogen-and-ammonia-complex)</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
@@ -661,7 +662,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>https://eastdaley.com/media-and-news/the-race-is-on-to-build-permian-processing</t>
+          <t>[East Daley](https://eastdaley.com/media-and-news/the-race-is-on-to-build-permian-processing)</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -698,7 +699,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>https://www.techint.com/en/our-projects/dos-bocas-refinery</t>
+          <t>[Techint](https://www.techint.com/en/our-projects/dos-bocas-refinery)</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -735,7 +736,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>https://www.ogj.com/refining-processing/refining/optimization/article/17279334/pemex-to-proceed-with-dos-bocas-refinery-project</t>
+          <t>[OGJ](https://www.ogj.com/refining-processing/refining/optimization/article/17279334/pemex-to-proceed-with-dos-bocas-refinery-project)</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -772,7 +773,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>https://forbes.com.mx/pemex-invertira-5300-millones-de-dolares-para-reactivar-la-industria-petroquimica/</t>
+          <t>[Forbes México](https://forbes.com.mx/pemex-invertira-5300-millones-de-dolares-para-reactivar-la-industria-petroquimica/)</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -809,7 +810,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>https://forbes.com.mx/pemex-invertira-5300-millones-de-dolares-para-reactivar-la-industria-petroquimica/</t>
+          <t>[Forbes México](https://forbes.com.mx/pemex-invertira-5300-millones-de-dolares-para-reactivar-la-industria-petroquimica/)</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -846,7 +847,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>https://forbes.com.mx/asi-es-la-inversion-de-1553-mdd-por-parte-de-pemex-en-una-planta-de-fertilizantes-en-veracruz/</t>
+          <t>[Forbes México](https://forbes.com.mx/asi-es-la-inversion-de-1553-mdd-por-parte-de-pemex-en-una-planta-de-fertilizantes-en-veracruz/)</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -878,17 +879,17 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/rehabilitación</t>
+          <t>Ingeniería/rehabilitación (incorporado al plan de reactivación petroquímica de Pemex, jun-2026; 13,700 millones de pesos asignados para los complejos Lázaro Cárdenas y ProAgro; meta de 2.4 millones ton/año de urea y fertilizantes fosfatados)</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>https://tribuna.com.mx/mexico/2026/06/05/sheinbaum-anuncia-inversion-de-93-mil-mdp-para-reactivar-la-industria-petroquimica-y-de-fertilizantes-en-veracruz_560837/</t>
+          <t>[Tribuna](https://tribuna.com.mx/mexico/2026/06/05/sheinbaum-anuncia-inversion-de-93-mil-mdp-para-reactivar-la-industria-petroquimica-y-de-fertilizantes-en-veracruz_560837/); [Contralínea](https://contralinea.com.mx/interno/semana/presentan-plan-con-inversion-de-93-mil-mdp-para-rescatar-la-petroquimica-nacional/)</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
@@ -920,7 +921,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>https://www.pv-magazine-mexico.com/2026/04/28/inician-en-sinaloa-la-construccion-de-la-mayor-planta-de-metanol-ultrabajo-en-carbono-a-partir-de-hidrogeno-verde/</t>
+          <t>[PV Magazine México](https://www.pv-magazine-mexico.com/2026/04/28/inician-en-sinaloa-la-construccion-de-la-mayor-planta-de-metanol-ultrabajo-en-carbono-a-partir-de-hidrogeno-verde/)</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -957,7 +958,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>https://www.h2-view.com/story/first-ammonia-project-on-track-for-2026-fid-despite-topsoe-deal-collapse/2138792.article/</t>
+          <t>[H2 View](https://www.h2-view.com/story/first-ammonia-project-on-track-for-2026-fid-despite-topsoe-deal-collapse/2138792.article/)</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -994,7 +995,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>https://www.debate.com.mx/economia/secretaria-de-economia-complejo-de-amoniaco-en-topolobampo-prioritario-para-el-gobierno-de-mexico-20260713-0092.html</t>
+          <t>[Debate](https://www.debate.com.mx/economia/secretaria-de-economia-complejo-de-amoniaco-en-topolobampo-prioritario-para-el-gobierno-de-mexico-20260713-0092.html)</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -1031,7 +1032,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>https://www.icis.com/explore/resources/news/2025/11/13/11155109/lake-charles-methanol-ii-awards-feed-fid-expected-in-q2-2026/</t>
+          <t>[ICIS](https://www.icis.com/explore/resources/news/2025/11/13/11155109/lake-charles-methanol-ii-awards-feed-fid-expected-in-q2-2026/)</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -1068,7 +1069,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>https://diariodelistmo.com/nacional/este-es-el-avance-que-lleva-la-planta-coquizadora-en-la-refineria-de-salina-cruz/50642321</t>
+          <t>[Diario del Istmo](https://diariodelistmo.com/nacional/este-es-el-avance-que-lleva-la-planta-coquizadora-en-la-refineria-de-salina-cruz/50642321)</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -1105,7 +1106,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>https://www.hydrocarbonengineering.com/petrochemicals/06032026/shintech-announces-us34-billion-at-louisiana-petrochemicals-complex/</t>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/petrochemicals/06032026/shintech-announces-us34-billion-at-louisiana-petrochemicals-complex/)</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -1142,7 +1143,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>https://www.alchempro.com/news/chemicals-news/ineos-backs-1-7-bn-low-carbon-methanol-project-in-texas-city-310108-newsdetails.htm</t>
+          <t>[Alchempro](https://www.alchempro.com/news/chemicals-news/ineos-backs-1-7-bn-low-carbon-methanol-project-in-texas-city-310108-newsdetails.htm)</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -1179,7 +1180,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>https://www.hydrocarbonengineering.com/petrochemicals/13072026/oxea-confirms-fid-for-major-capacity-expansion/</t>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/petrochemicals/13072026/oxea-confirms-fid-for-major-capacity-expansion/)</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -1216,7 +1217,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>https://www.ogj.com/refining-processing/gas-processing/news/55320579/targa-advances-permian-gas-pipeline-processing-expansion</t>
+          <t>[OGJ](https://www.ogj.com/refining-processing/gas-processing/news/55320579/targa-advances-permian-gas-pipeline-processing-expansion)</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -1253,7 +1254,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>https://www.businesswire.com/news/home/20250806663187/en/Enterprise-Agrees-to-Acquire-Occidentals-Gas-Gathering-Affiliate-Enters-Into-Natural-Gas-Processing-Agreement-Announces-New-Midland-Basin-Natural-Gas-Processing-Plant</t>
+          <t>[Business Wire](https://www.businesswire.com/news/home/20250806663187/en/Enterprise-Agrees-to-Acquire-Occidentals-Gas-Gathering-Affiliate-Enters-Into-Natural-Gas-Processing-Agreement-Announces-New-Midland-Basin-Natural-Gas-Processing-Plant)</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -1290,7 +1291,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>https://naturalgasintel.com/news/mplx-scales-up-for-power-hungry-future-with-natural-gas-focused-growth-plan/</t>
+          <t>[Natural Gas Intel](https://naturalgasintel.com/news/mplx-scales-up-for-power-hungry-future-with-natural-gas-focused-growth-plan/)</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -1327,7 +1328,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>https://eastdaley.com/daley-note/mplx-acquires-northwind-for-2-375b-acquires-more-ngls-for-jv-project</t>
+          <t>[East Daley](https://eastdaley.com/daley-note/mplx-acquires-northwind-for-2-375b-acquires-more-ngls-for-jv-project)</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -1364,7 +1365,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>https://www.grandforksherald.com/news/local/northern-plains-nitrogen-proposal-receiving-more-attention-amid-global-fertilizer-pressure</t>
+          <t>[Grand Forks Herald](https://www.grandforksherald.com/news/local/northern-plains-nitrogen-proposal-receiving-more-attention-amid-global-fertilizer-pressure)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -1401,7 +1402,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>https://www.phillips66.com/newsroom/iron-mesa-safely-enters-next-phase-of-construction/</t>
+          <t>[Phillips 66](https://www.phillips66.com/newsroom/iron-mesa-safely-enters-next-phase-of-construction/)</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -1438,7 +1439,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>https://www.targaresources.com/news-releases/news-release-details/targa-resources-corp-announces-permian-growth-projects-and</t>
+          <t>[Targa Resources](https://www.targaresources.com/news-releases/news-release-details/targa-resources-corp-announces-permian-growth-projects-and)</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -1475,7 +1476,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>https://elefanteblanco.mx/2026/01/02/pemex-abre-30-licitaciones-para-obras-en-la-refineria-madero/</t>
+          <t>[Elefante Blanco](https://elefanteblanco.mx/2026/01/02/pemex-abre-30-licitaciones-para-obras-en-la-refineria-madero/)</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -1512,7 +1513,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>https://www.jornada.com.mx/noticia/2026/06/08/economia/da-inicio-ejecucion-de-planta-de-fertilizantes-en-durango-por-parte-de-fermachem</t>
+          <t>[La Jornada](https://www.jornada.com.mx/noticia/2026/06/08/economia/da-inicio-ejecucion-de-planta-de-fertilizantes-en-durango-por-parte-de-fermachem)</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -1549,7 +1550,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>https://downstreamcalendar.com/mcdermott-secures-feed-contract-for-ascension-clean-energy-project/</t>
+          <t>[Downstream Calendar](https://downstreamcalendar.com/mcdermott-secures-feed-contract-for-ascension-clean-energy-project/)</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -1586,7 +1587,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>https://www.businesswire.com/news/home/20260517310811/en/Phillips-66-announces-Zeus-Gas-Plant-and-a-third-Coastal-Bend-Fractionator</t>
+          <t>[Business Wire](https://www.businesswire.com/news/home/20260517310811/en/Phillips-66-announces-Zeus-Gas-Plant-and-a-third-Coastal-Bend-Fractionator)</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -1623,7 +1624,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>https://www.usda.gov/about-usda/news/press-releases/2026/07/01/secretary-rollins-announces-500-million-fertilizer-investment-and-expansion-program-strengthen</t>
+          <t>[USDA](https://www.usda.gov/about-usda/news/press-releases/2026/07/01/secretary-rollins-announces-500-million-fertilizer-investment-and-expansion-program-strengthen)</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -1660,12 +1661,49 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>https://www.hydrocarbonengineering.com/clean-fuels/06012026/samsung-ea-announces-groundbreaking-of-low-carbon-ammonia-plant/</t>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/clean-fuels/06012026/samsung-ea-announces-groundbreaking-of-low-carbon-ammonia-plant/)</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
           <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Green Fuels Operating — Refinería Duncan</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Duncan, Stephens County, Oklahoma, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Green Fuels Operating</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Construcción (groundbreaking 29-may-2026; inversión US$400 millones; capacidad inicial 30,000 bbl/d, expandible a 50,000 bbl/d, sobre sitio de refinería histórica de los años 1920)</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/refining/03062026/green-fuels-hosts-groundbreaking-ceremony-for-new-refinery/)</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
@@ -1680,16 +1718,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1752,17 +1790,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Construcción</t>
+          <t>Construcción (FERC aprobó inicio de construcción de Trenes 4 y 5 en mar-2026; NextDecade evalúa un 6to tren para superar 36 mtpa; gasoducto de alimentación Rio Bravo Pipeline —138 millas, JV Whitewater/MPLX/Enbridge— en camino a entrar en servicio 2S2026)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>https://www.bechtel.com/press-releases/nextdecade-executes-epc-contract-with-bechtel-for-train-4-at-the-rio-grande-lng-facility/</t>
+          <t>[Bechtel](https://www.bechtel.com/press-releases/nextdecade-executes-epc-contract-with-bechtel-for-train-4-at-the-rio-grande-lng-facility/); [Natural Gas Intel](https://naturalgasintel.com/news/nextdecade-targets-more-than-36-mty-with-rio-grande-lng-upscale-sixth-train-expansion/)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
@@ -1794,7 +1832,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>https://www.bechtel.com/press-releases/sempra-infrastructure-announces-epc-contract-with-bechtel-for-port-arthur-lng-phase-2/</t>
+          <t>[Bechtel](https://www.bechtel.com/press-releases/sempra-infrastructure-announces-epc-contract-with-bechtel-for-port-arthur-lng-phase-2/)</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -1831,7 +1869,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>https://www.woodside.com/what-we-do/growth-projects/woodside-louisiana-lng</t>
+          <t>[Woodside](https://www.woodside.com/what-we-do/growth-projects/woodside-louisiana-lng)</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1868,7 +1906,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>https://www.gem.wiki/CP2_LNG_Terminal</t>
+          <t>[GEM.wiki](https://www.gem.wiki/CP2_LNG_Terminal)</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -1905,7 +1943,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>https://www.offshore-energy.biz/kbr-zachry-to-work-on-ventures-plaquemines-lng/</t>
+          <t>[Offshore Energy](https://www.offshore-energy.biz/kbr-zachry-to-work-on-ventures-plaquemines-lng/)</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1942,7 +1980,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>https://panews.com/2026/04/24/golden-pass-lng-makes-history-with-first-export-from-sabine-pass-terminal/</t>
+          <t>[Port Arthur News](https://panews.com/2026/04/24/golden-pass-lng-makes-history-with-first-export-from-sabine-pass-terminal/)</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -1974,17 +2012,17 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Construcción (FERC autorizó introducción de gas combustible en Train 7, 17-jul-2026; primera producción de LNG esperada ago-2026, servicio comercial sep-2026)</t>
+          <t>Construcción (FERC autorizó introducción de gas combustible en Train 7, 17-jul-2026; primera producción de LNG esperada ago-2026, servicio comercial sep-2026; Trenes 5 y 6 completados mar/jun-2026; expansión completa de 7 trenes 85.4% de avance, prevista para fin de 2026)</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>https://pgjonline.com/news/2026/july/corpus-christi-lng-train-7-cleared-to-introduce-fuel-gas-by-ferc</t>
+          <t>[PGJ](https://pgjonline.com/news/2026/july/corpus-christi-lng-train-7-cleared-to-introduce-fuel-gas-by-ferc); [LNG Prime](https://lngprime.com/americas/chenieres-corpus-christi-expansion-project-85-4-percent-complete/155448/)</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
@@ -2016,7 +2054,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2026/06/03/3306350/0/en/delfin-midstream-announces-5-billion-final-investment-decision-for-first-flng-vessel.html</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/06/03/3306350/0/en/delfin-midstream-announces-5-billion-final-investment-decision-for-first-flng-vessel.html)</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -2053,7 +2091,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>https://dossierpolitico.com/2026/07/17/activistas-entregan-90-mil-firmas-para-frenar-proyecto-saguaro-energia-en-sonora/</t>
+          <t>[Dossier Político](https://dossierpolitico.com/2026/07/17/activistas-entregan-90-mil-firmas-para-frenar-proyecto-saguaro-energia-en-sonora/)</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -2090,7 +2128,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>https://www.gem.wiki/New_Fortress_Altamira_FLNG_Terminal</t>
+          <t>[GEM Wiki](https://www.gem.wiki/New_Fortress_Altamira_FLNG_Terminal)</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -2127,7 +2165,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>https://www.naturalgasintel.com/news/glenfarne-lands-investment-for-early-work-on-texas-lng-ahead-of-fid/</t>
+          <t>[Natural Gas Intel](https://www.naturalgasintel.com/news/glenfarne-lands-investment-for-early-work-on-texas-lng-ahead-of-fid/)</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -2164,7 +2202,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>https://pgjonline.com/news/2026/july/commonwealth-lng-awards-main-automation-contract-for-louisiana-export-terminal</t>
+          <t>[PGJ](https://pgjonline.com/news/2026/july/commonwealth-lng-awards-main-automation-contract-for-louisiana-export-terminal)</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -2201,7 +2239,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>https://www.houstonpublicmedia.org/articles/galveston-county/2026/07/14/557086/galveston-pelican-island-lng/</t>
+          <t>[Houston Public Media](https://www.houstonpublicmedia.org/articles/galveston-county/2026/07/14/557086/galveston-pelican-island-lng/)</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -2238,7 +2276,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>https://www.sempra.com/newsroom/press-releases/sempra-infrastructures-eca-lng-phase-1-exports-first-lng-cargo-mexicos</t>
+          <t>[Sempra](https://www.sempra.com/newsroom/press-releases/sempra-infrastructures-eca-lng-phase-1-exports-first-lng-cargo-mexicos)</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -2275,7 +2313,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>https://lngprime.com/americas/gato-negro-eyes-fid-on-mexico-lng-plant-in-late-2026/165906/</t>
+          <t>[LNG Prime](https://lngprime.com/americas/gato-negro-eyes-fid-on-mexico-lng-plant-in-late-2026/165906/)</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -2312,7 +2350,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/amigo-lng-awards-landmark-epc-contract-to-dubai-based-drydocks-world-for-worlds-largest-flng-facility-302537739.html</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/amigo-lng-awards-landmark-epc-contract-to-dubai-based-drydocks-world-for-worlds-largest-flng-facility-302537739.html)</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -2349,7 +2387,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>https://www.kbr.com/en/insights-news/press-release/kbr-awarded-feed-coastal-bend-lng-project</t>
+          <t>[KBR](https://www.kbr.com/en/insights-news/press-release/kbr-awarded-feed-coastal-bend-lng-project)</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -2386,7 +2424,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>https://www.ferc.gov/gulfstream-lng-terminal-project</t>
+          <t>[FERC](https://www.ferc.gov/gulfstream-lng-terminal-project)</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -2423,7 +2461,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>https://alaskabeacon.com/2026/07/17/hilcorp-killed-alaska-lng-bill-some-legislators-say-but-governor-calls-the-claim-bullst/</t>
+          <t>[Alaska Beacon](https://alaskabeacon.com/2026/07/17/hilcorp-killed-alaska-lng-bill-some-legislators-say-but-governor-calls-the-claim-bullst/)</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -2460,7 +2498,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>https://pgjonline.com/news/2026/july/311-mile-sonora-gas-pipeline-project-advances-in-mexico</t>
+          <t>[PGJ](https://pgjonline.com/news/2026/july/311-mile-sonora-gas-pipeline-project-advances-in-mexico)</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -2497,7 +2535,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>https://www.ogj.com/pipelines-transportation/pipelines/news/55322537/arm-energy-takes-fid-on-23-billion-mustang-express-pipeline</t>
+          <t>[OGJ](https://www.ogj.com/pipelines-transportation/pipelines/news/55322537/arm-energy-takes-fid-on-23-billion-mustang-express-pipeline)</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -2534,7 +2572,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>https://mexicobusiness.news/energy/news/ursus-energy-scales-investment-us21-billion</t>
+          <t>[Mexico Business News](https://mexicobusiness.news/energy/news/ursus-energy-scales-investment-us21-billion)</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -2571,7 +2609,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2026/07/15/3327983/0/en/Delfin-Midstream-Partners-With-EIG-s-MidOcean-Energy-to-Advance-Second-FLNG-Vessel-Issues-Limited-Notice-to-Proceed-to-Siemens-Energy.html</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/15/3327983/0/en/Delfin-Midstream-Partners-With-EIG-s-MidOcean-Energy-to-Advance-Second-FLNG-Vessel-Issues-Limited-Notice-to-Proceed-to-Siemens-Energy.html)</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -2608,7 +2646,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>https://www.naturalgasintel.com/news/texas-gateway-open-season-expands-haynesville-natural-gas-links-amid-lng-growth/</t>
+          <t>[Natural Gas Intel](https://www.naturalgasintel.com/news/texas-gateway-open-season-expands-haynesville-natural-gas-links-amid-lng-growth/)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -2645,7 +2683,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>https://worldoil.com/news/2026/7/24/doe-approves-20-year-export-authorization-for-argent-lng-project/</t>
+          <t>[World Oil](https://worldoil.com/news/2026/7/24/doe-approves-20-year-export-authorization-for-argent-lng-project/)</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -2682,7 +2720,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>https://www.federalregister.gov/documents/2026/07/24/2026-14963/deepwater-port-license-application-st-lng-deepwater-port-development-project-final-environmental</t>
+          <t>[Federal Register](https://www.federalregister.gov/documents/2026/07/24/2026-14963/deepwater-port-license-application-st-lng-deepwater-port-development-project-final-environmental)</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -2719,7 +2757,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>https://naturalgasintel.com/news/kinder-morgan-greenlights-7b-in-natural-gas-pipeline-projects-amid-regulatory-speedup/</t>
+          <t>[Natural Gas Intel](https://naturalgasintel.com/news/kinder-morgan-greenlights-7b-in-natural-gas-pipeline-projects-amid-regulatory-speedup/)</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -2756,7 +2794,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>https://naturalgasintel.com/news/kinder-morgan-greenlights-7b-in-natural-gas-pipeline-projects-amid-regulatory-speedup/</t>
+          <t>[Natural Gas Intel](https://naturalgasintel.com/news/kinder-morgan-greenlights-7b-in-natural-gas-pipeline-projects-amid-regulatory-speedup/)</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -2793,7 +2831,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>https://lngprime.com/americas/kinder-morgan-seeks-doe-extension-for-gulf-lng-export-project/184334/</t>
+          <t>[LNG Prime](https://lngprime.com/americas/kinder-morgan-seeks-doe-extension-for-gulf-lng-export-project/184334/)</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -2830,7 +2868,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>https://investors.bakerhughes.com/news/press-releases/news-details/2026/Baker-Hughes-Secures-Substantial-Equipment-and-Services-Awards-for-Chenieres-Sabine-Pass-LNG-Facility/default.aspx</t>
+          <t>[Baker Hughes](https://investors.bakerhughes.com/news/press-releases/news-details/2026/Baker-Hughes-Secures-Substantial-Equipment-and-Services-Awards-for-Chenieres-Sabine-Pass-LNG-Facility/default.aspx)</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -2867,7 +2905,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>https://www.federalregister.gov/documents/2026/05/05/2026-08654/cheniere-corpus-christi-pipeline-lp-corpus-christi-liquefaction-stage-iv-llc-corpus-christi</t>
+          <t>[Federal Register](https://www.federalregister.gov/documents/2026/05/05/2026-08654/cheniere-corpus-christi-pipeline-lp-corpus-christi-liquefaction-stage-iv-llc-corpus-christi)</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -2904,7 +2942,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>https://www.federalregister.gov/documents/2026/07/24/2026-15040/freeport-lng-development-lp-flng-liquefaction-llc-flng-liquefaction-2-llc-flng-liquefaction-3-llc</t>
+          <t>[Federal Register](https://www.federalregister.gov/documents/2026/07/24/2026-15040/freeport-lng-development-lp-flng-liquefaction-llc-flng-liquefaction-2-llc-flng-liquefaction-3-llc)</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -2941,7 +2979,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>https://www.proyectosmexico.gob.mx/proyecto_inversion/1076-gasoducto-coatzacoalcos-ii/</t>
+          <t>[Proyectos México](https://www.proyectosmexico.gob.mx/proyecto_inversion/1076-gasoducto-coatzacoalcos-ii/)</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -2978,12 +3016,49 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>https://www.lngindustry.com/liquefaction/24072026/stabilis-solutions-receives-lor-from-us-coast-guard/</t>
+          <t>[LNG Industry](https://www.lngindustry.com/liquefaction/24072026/stabilis-solutions-receives-lor-from-us-coast-guard/)</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
           <t>2026-07-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>CP2 LNG Fase 3</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Cameron Parish, Luisiana, EE.UU. (adyacente al complejo CP2 Fase 1/2)</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Venture Global Inc.</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>No especificado (pendiente FID)</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Permitting (FERC exoneró proceso de pre-filing 16-abr-2026; solicitud formal presentada 26-may-2026; Notice of Application publicado 12-jun-2026; 6 bloques de licuefacción adicionales/12 trenes, planta de energía de 720MW, tercer atracadero marino; eleva capacidad pico del complejo de 28 a 35 mtpa)</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>[Federal Register](https://www.federalregister.gov/documents/2026/06/12/2026-11881/venture-global-cp2-lng-llc-venture-global-cp-express-llc-notice-of-application-and-establishing)</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
@@ -2998,16 +3073,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3075,7 +3150,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>https://www.miningweekly.com/article/ivanhoe-electric-pencils-in-2026-construction-start-at-arizona-copper-mine-2025-06-25</t>
+          <t>[Mining Weekly](https://www.miningweekly.com/article/ivanhoe-electric-pencils-in-2026-construction-start-at-arizona-copper-mine-2025-06-25)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -3107,17 +3182,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/Feasibility (DFS &gt;85% completo)</t>
+          <t>Ingeniería/Feasibility (DFS &gt;85% completo; colocación de bonos municipales por US$52 millones completada 24-jun-2026 para financiar el proyecto, ya totalmente permisado para iniciar construcción)</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1322422/000106299326001973/exhibit99-2.htm</t>
+          <t>[SEC/Hudbay](https://www.sec.gov/Archives/edgar/data/1322422/000106299326001973/exhibit99-2.htm); [GlobeNewswire](https://www.globenewswire.com/news-release/2026/06/24/3317147/0/en/hudbay-completes-offering-of-us-52-million-of-4-50-municipal-bonds-for-copper-world.html)</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
@@ -3144,17 +3219,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería temprana post intercambio de tierras (marzo 2026)</t>
+          <t>Ingeniería temprana post intercambio de tierras (marzo 2026); firmó Master Supply Agreement (1-jul-2026) con Johnson Controls Inc. y United Association Local 469 (sindicato de plomeros/pipefitters) para mantenimiento de instalaciones y soporte operativo en sitio</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/863064/000086306426000019/ex12d16mr_resolutionland.htm</t>
+          <t>[SEC](https://www.sec.gov/Archives/edgar/data/863064/000086306426000019/ex12d16mr_resolutionland.htm); [Resolution Copper](https://resolutioncopper.com/resolution-copper-and-united-association-local-469-enter-into-master-supply-agreement-supporting-operations-in-arizona/)</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
@@ -3186,7 +3261,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>https://www.nevadaappeal.com/news/2026/mar/26/lithium-americas-900-construction-workers-at-thacker-pass-mine/</t>
+          <t>[Nevada Appeal](https://www.nevadaappeal.com/news/2026/mar/26/lithium-americas-900-construction-workers-at-thacker-pass-mine/)</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -3223,7 +3298,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>https://www.mining.com/teck-agnico-team-up-at-san-nicolas-copper-project-in-mexico/</t>
+          <t>[Mining.com](https://www.mining.com/teck-agnico-team-up-at-san-nicolas-copper-project-in-mexico/)</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -3260,7 +3335,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>https://energymagazine.mx/2025/10/grupo-mexico-espera-autorizacion-federal-para-continuar-proyectos-mineros-por-10-mil-200-mdd/</t>
+          <t>[Energy Magazine MX](https://energymagazine.mx/2025/10/grupo-mexico-espera-autorizacion-federal-para-continuar-proyectos-mineros-por-10-mil-200-mdd/)</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -3297,7 +3372,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>https://www.bnamericas.com/en/news/southern-copper-wins-permits-for-us551mn-el-pilar-in-mexico</t>
+          <t>[BNamericas](https://www.bnamericas.com/en/news/southern-copper-wins-permits-for-us551mn-el-pilar-in-mexico)</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -3334,7 +3409,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>https://m3eng.com/portfolio/buenavista-del-cobre-concentradora-no-2/</t>
+          <t>[M3 Engineering](https://m3eng.com/portfolio/buenavista-del-cobre-concentradora-no-2/)</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -3371,7 +3446,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>https://mineriaenlinea.com/2026/04/torex-gold-alcanza-velocidad-de-crucero-en-media-luna-9-meses-adelante-de-cronograma/</t>
+          <t>[Minería en Línea](https://mineriaenlinea.com/2026/04/torex-gold-alcanza-velocidad-de-crucero-en-media-luna-9-meses-adelante-de-cronograma/)</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -3408,7 +3483,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>https://www.mining.com/nevada-copper-unveils-restart-and-financing-plan-for-pumpkin-hollow/</t>
+          <t>[Mining.com](https://www.mining.com/nevada-copper-unveils-restart-and-financing-plan-for-pumpkin-hollow/)</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -3445,7 +3520,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>https://www.usda.gov/about-usda/news/press-releases/2026/07/07/usda-advances-trump-administration-effort-boost-us-mineral-energy-production</t>
+          <t>[USDA](https://www.usda.gov/about-usda/news/press-releases/2026/07/07/usda-advances-trump-administration-effort-boost-us-mineral-energy-production)</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -3482,7 +3557,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/perpetua-resources-advances-construction-of-the-stibnite-gold-project-302787012.html</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/perpetua-resources-advances-construction-of-the-stibnite-gold-project-302787012.html)</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -3519,7 +3594,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>https://silvertigermetals.com/news/2026/silver-tiger-metals-awards-engineering-procurement-and-construction-management-contract-and-provides-construction-update</t>
+          <t>[Silver Tiger Metals](https://silvertigermetals.com/news/2026/silver-tiger-metals-awards-engineering-procurement-and-construction-management-contract-and-provides-construction-update)</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -3556,7 +3631,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/vizsla-silver-awards-epcm-and-mine-design-contracts-for-the-development-of-the-panuco-silver-gold-project-302750621.html</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/vizsla-silver-awards-epcm-and-mine-design-contracts-for-the-development-of-the-panuco-silver-gold-project-302750621.html)</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -3593,7 +3668,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>https://orlamining.com/news/orla-announces-results-of-updated-feasibility-study-for-south-railroad-project/</t>
+          <t>[Orla Mining](https://orlamining.com/news/orla-announces-results-of-updated-feasibility-study-for-south-railroad-project/)</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -3630,7 +3705,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>https://www.miningweekly.com/article/minera-alamos-confirms-low-cost-near-term-mining-possible-at-copperstone-in-arizona-2026-05-28</t>
+          <t>[Mining Weekly](https://www.miningweekly.com/article/minera-alamos-confirms-low-cost-near-term-mining-possible-at-copperstone-in-arizona-2026-05-28)</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -3667,7 +3742,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>https://www.wyomingnews.com/rawlinstimes/plans-move-forward-for-ck-gold-project-as-developers-target-2026-construction-start/article_b2bb147e-2f92-4ca2-bf86-fcc9983917a7.html</t>
+          <t>[Wyoming News](https://www.wyomingnews.com/rawlinstimes/plans-move-forward-for-ck-gold-project-as-developers-target-2026-construction-start/article_b2bb147e-2f92-4ca2-bf86-fcc9983917a7.html)</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -3704,7 +3779,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>https://www.juniorminingnetwork.com/junior-miner-news/press-releases/1082-tsx/ag/206222-first-majestic-receives-construction-permits-for-santo-nino-and-navidad-advances-development-across-the-santa-elena-district.html</t>
+          <t>[First Majestic](https://www.juniorminingnetwork.com/junior-miner-news/press-releases/1082-tsx/ag/206222-first-majestic-receives-construction-permits-for-santo-nino-and-navidad-advances-development-across-the-santa-elena-district.html)</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -3741,7 +3816,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/0001286973/000106299326002645/exhibit99-2.htm</t>
+          <t>[SEC/Americas Gold and Silver](https://www.sec.gov/Archives/edgar/data/0001286973/000106299326002645/exhibit99-2.htm)</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -3778,7 +3853,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>https://www.kitco.com/news/off-the-wire/2026-06-08/minera-frisco-restarts-two-mexico-mines-plans-new-silver-unit</t>
+          <t>[Kitco](https://www.kitco.com/news/off-the-wire/2026-06-08/minera-frisco-restarts-two-mexico-mines-plans-new-silver-unit)</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -3815,7 +3890,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/trilogy-metals-announces-publication-of-federal-and-state-permitting-schedule-for-arctic-project-establishing-defined-timeline-toward-a-record-of-decision-by-september-2028-302827083.html</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/trilogy-metals-announces-publication-of-federal-and-state-permitting-schedule-for-arctic-project-establishing-defined-timeline-toward-a-record-of-decision-by-september-2028-302827083.html)</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -3847,17 +3922,17 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Construcción aprobada (permisos SEMARNAT jun-2026)</t>
+          <t>Construcción aprobada por el consejo (permisos SEMARNAT completos jun-2026; presupuesto ~US$227 millones; ventana de construcción de ~24 meses; primer vertido de metal previsto mediados de 2028)</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>https://www.northernminer.com/news/gogold-approved-to-build-227m-mine-in-mexico/1003891932/</t>
+          <t>[Northern Miner](https://www.northernminer.com/news/gogold-approved-to-build-227m-mine-in-mexico/1003891932/); [Newsfile](https://www.newsfilecorp.com/release/300455/GoGold-Achieves-Major-Milestone-Final-Remaining-Permits-Secured-and-Construction-Approved-for-Los-Ricos-South-Underground-Mine)</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
@@ -3889,7 +3964,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>https://www.bnamericas.com/en/news/discovery-advances-permitting-financing-at-us606mn-cordero-in-mexico</t>
+          <t>[BNamericas](https://www.bnamericas.com/en/news/discovery-advances-permitting-financing-at-us606mn-cordero-in-mexico)</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -3926,7 +4001,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>https://resourceworld.com/tocvan-ventures-eyes-mexican-gold-pour-by-q4-2026/</t>
+          <t>[Resource World](https://resourceworld.com/tocvan-ventures-eyes-mexican-gold-pour-by-q4-2026/)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -3963,7 +4038,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>https://www.fresnilloplc.com/portfolio/exploration/orisyvo/</t>
+          <t>[Fresnillo plc](https://www.fresnilloplc.com/portfolio/exploration/orisyvo/)</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -4000,7 +4075,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/</t>
+          <t>[Mining.com](https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/)</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -4037,7 +4112,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/</t>
+          <t>[Mining.com](https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/)</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -4074,7 +4149,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/</t>
+          <t>[Mining.com](https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/)</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -4111,7 +4186,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>https://im-mining.com/2026/06/29/metso-to-supply-additional-crushing-package-for-grupo-mexico-la-caridad-copper-concentrator/</t>
+          <t>[IM Mining](https://im-mining.com/2026/06/29/metso-to-supply-additional-crushing-package-for-grupo-mexico-la-caridad-copper-concentrator/)</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -4148,7 +4223,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2026/05/21/3299182</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/05/21/3299182)</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -4185,7 +4260,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>https://mexicobusiness.news/mining/news/grupo-mexicos-asarco-may-reopen-united-states</t>
+          <t>[Mexico Business News](https://mexicobusiness.news/mining/news/grupo-mexicos-asarco-may-reopen-united-states)</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -4222,7 +4297,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>https://mineraalamos.com/our-assets/cerro-de-oro-project/</t>
+          <t>[Minera Alamos](https://mineraalamos.com/our-assets/cerro-de-oro-project/)</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -4259,7 +4334,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>https://www.globalminingreview.com/mining/11022025/antler-copper-project-achieves-critical-federal-permitting-milestone/</t>
+          <t>[Global Mining Review](https://www.globalminingreview.com/mining/11022025/antler-copper-project-achieves-critical-federal-permitting-milestone/)</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -4296,7 +4371,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>https://www.blm.gov/press-release/blm-approves-lisbon-valley-copper-mine-expansion-utah</t>
+          <t>[BLM](https://www.blm.gov/press-release/blm-approves-lisbon-valley-copper-mine-expansion-utah)</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -4333,7 +4408,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>https://investingnews.com/smackover-lithium-announces-the-award-of-last-key-construction-contract-for-the-south-west-arkansas-project-ahead-of-final-investment-decision/</t>
+          <t>[InvestingNews](https://investingnews.com/smackover-lithium-announces-the-award-of-last-key-construction-contract-for-the-south-west-arkansas-project-ahead-of-final-investment-decision/)</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -4370,7 +4445,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/0000831259/000083125926000033/a2q2026exhibit991.htm</t>
+          <t>[SEC/Freeport-McMoRan](https://www.sec.gov/Archives/edgar/data/0000831259/000083125926000033/a2q2026exhibit991.htm)</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -4407,7 +4482,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>https://niocorp.com/niocorp-launches-construction-of-elk-creek-critical-minerals-project-mine-portal/</t>
+          <t>[NioCorp](https://niocorp.com/niocorp-launches-construction-of-elk-creek-critical-minerals-project-mine-portal/)</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -4444,7 +4519,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>https://www.e-mj.com/breaking-news/centerra-advances-goldfield-project-in-nevada/</t>
+          <t>[E&amp;MJ](https://www.e-mj.com/breaking-news/centerra-advances-goldfield-project-in-nevada/)</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -4481,7 +4556,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2026/03/02/3247157/0/en/hudbay-to-acquire-arizona-sonoran-creating-the-third-largest-copper-district-in-north-america.html</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/03/02/3247157/0/en/hudbay-to-acquire-arizona-sonoran-creating-the-third-largest-copper-district-in-north-america.html)</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -4518,7 +4593,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>https://www.westernexploration.com/news-and-updates/news/news-details/2026/Western-Exploration-Outlines-2026-Program-to-Advance-Doby-George-Permitting-and-Expand-Gravel-Creek-Resources-2026-aaotfYHcV7/default.aspx</t>
+          <t>[Western Exploration](https://www.westernexploration.com/news-and-updates/news/news-details/2026/Western-Exploration-Outlines-2026-Program-to-Advance-Doby-George-Permitting-and-Expand-Gravel-Creek-Resources-2026-aaotfYHcV7/default.aspx)</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -4555,7 +4630,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>https://chesapeakegold.com/metates/</t>
+          <t>[Chesapeake Gold Corp.](https://chesapeakegold.com/metates/)</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -4567,72 +4642,146 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Libby Project (Cabinet Mountains)</t>
+          <t>Pathfinder Tonopah (cobre-molibdeno-plata)</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Condado de Lincoln, Montana, EE.UU.</t>
+          <t>Tonopah, Nevada, EE.UU.</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Hecla Mining Company</t>
+          <t>Pathfinder Minerals (Pathfinder Tonopah)</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Bowman (permisos ambientales, FEED, planta piloto)</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Permitting federal completado para exploración subterránea (extensión de ~1 milla del socavón Libby Adit; recurso potencial 1,500 millones lb de cobre y 183 millones oz de plata; pendiente permiso de descarga de agua de MT DEQ)</t>
+          <t>Permitting/FEED (avanzando hacia estudio de factibilidad definitivo; carta de interés no vinculante de EXIM Bank por US$896 millones para financiamiento, programa "Make More in America")</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>https://thewesternnews.com/news/2026/jul/24/libby-mining-project-takes-another-step-forward-with-federal-ok/</t>
+          <t>[Mining Technology](https://www.mining-technology.com/news/pathfinder-896m-loi-us-exim-copper-mine/)</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
+          <t>La Colorada Mine — Expansión Veta Madre/Veta Madre Plus</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Sonora, México</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Heliostar Metals</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Permisos completos obtenidos (2026); waste stripping programado 3T2026; producción de zona expandida esperada 1S2027</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>[Mexico Business News](https://mexicobusiness.news/mining/news/heliostar-advances-la-colorada-pit-permits-drill-data)</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Libby Project (Cabinet Mountains)</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Condado de Lincoln, Montana, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Hecla Mining Company</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Permitting federal completado para exploración subterránea (extensión de ~1 milla del socavón Libby Adit; recurso potencial 1,500 millones lb de cobre y 183 millones oz de plata; pendiente permiso de descarga de agua de MT DEQ)</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>[The Western News](https://thewesternnews.com/news/2026/jul/24/libby-mining-project-takes-another-step-forward-with-federal-ok/)</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
           <t>Donlin Gold</t>
         </is>
       </c>
-      <c r="B44" s="2" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>Alaska, EE.UU.</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr">
         <is>
           <t>NovaGold Corporation (adquiriendo 100%, compra de participación del 40% de Paulson Advisers)</t>
         </is>
       </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>No especificado</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr">
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
         <is>
           <t>Totalmente permisado / consolidación de propiedad (acuerdo de US$4.2 mil millones, cierre previsto 4T2026); aún sin decisión de construcción (FID)</t>
         </is>
       </c>
-      <c r="F44" s="2" t="inlineStr">
-        <is>
-          <t>https://www.miningnewsnorth.com/story/2026/07/24/news/donlin-gold-partners-form-new-novagold/9781.html</t>
-        </is>
-      </c>
-      <c r="G44" s="2" t="inlineStr">
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>[Mining News North](https://www.miningnewsnorth.com/story/2026/07/24/news/donlin-gold-partners-form-new-novagold/9781.html)</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
         <is>
           <t>2026-07-27</t>
         </is>
@@ -4649,16 +4798,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G59"/>
+  <dimension ref="A1:G61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4721,17 +4870,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Construcción</t>
+          <t>Construcción (rompimiento de tierra formal completado; 1,200 acres/10 edificios/1.4GW; VoltaGrid aprobado para operar 210 generadores de gas industrial, 700MW combinados, permitiendo operación fuera de la red pública; primera instalación en servicio 2S2026)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/vantage-breaks-ground-on-texas-gigawatt-data-center-campus-for-openai/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/vantage-breaks-ground-on-texas-gigawatt-data-center-campus-for-openai/); [Construction Owners](https://www.constructionowners.com/news/oracle-and-openai-to-power-new-texas-data-center-off-the-grid)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
@@ -4763,7 +4912,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>https://epoch.ai/publications/openai-stargate-where-the-us-sites-stand</t>
+          <t>[Epoch AI](https://epoch.ai/publications/openai-stargate-where-the-us-sites-stand)</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -4800,7 +4949,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/crusoe-tops-out-final-building-at-openai-stargate-data-center-campus-in-abilene-texas/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/crusoe-tops-out-final-building-at-openai-stargate-data-center-campus-in-abilene-texas/)</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -4837,7 +4986,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>https://www.cnbc.com/2026/06/22/chevron-cvx-microsoft-msft-natural-gas-data-center.html</t>
+          <t>[CNBC](https://www.cnbc.com/2026/06/22/chevron-cvx-microsoft-msft-natural-gas-data-center.html)</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -4874,7 +5023,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>https://www.gob.mx/presidencia/prensa/plan-mexico-avanza-se-anuncia-inversion-de-4-mil-800-mdd-de-cloudhq-para-la-construccion-de-6-centros-de-datos-en-queretaro</t>
+          <t>[Gobierno de México](https://www.gob.mx/presidencia/prensa/plan-mexico-avanza-se-anuncia-inversion-de-4-mil-800-mdd-de-cloudhq-para-la-construccion-de-6-centros-de-datos-en-queretaro)</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -4911,7 +5060,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>https://www.ucs.org/about/news/judge-orders-meta-explain-new-gas-demand-hyperscale-louisiana-data-center</t>
+          <t>[UCS](https://www.ucs.org/about/news/judge-orders-meta-explain-new-gas-demand-hyperscale-louisiana-data-center)</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -4948,7 +5097,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterfrontier.com/site-selection/article/55305086/nv1-and-the-nevada-hyperscale-boom-vantage-data-centers-bets-3b-on-the-ai-future</t>
+          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55305086/nv1-and-the-nevada-hyperscale-boom-vantage-data-centers-bets-3b-on-the-ai-future)</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -4985,7 +5134,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/cloudburst-breaks-ground-on-gigawatt-scale-data-center-campus-in-texas/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/cloudburst-breaks-ground-on-gigawatt-scale-data-center-campus-in-texas/)</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -5002,7 +5151,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Kaufman County, Texas, EE.UU.</t>
+          <t>Entre Talty y Post Oak Bend City, Kaufman County, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -5017,17 +5166,17 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/construcción temprana</t>
+          <t>Ingeniería/construcción temprana (campus de 200MW/4 edificios; estrategia behind-the-meter con motores de gas Jenbacher J620 + almacenamiento en baterías de Engie; primera instalación 2026, fases hasta 2028)</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/prometheus-hyperscale-details-plans-for-dallas-data-center-campus/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/prometheus-hyperscale-details-plans-for-dallas-data-center-campus/)</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
@@ -5059,7 +5208,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>https://www.businesswire.com/news/home/20260126236053/en/Pacifico-Energy-Secures-7.65-GW-Power-Generation-Permit-for-GW-Ranch-Project</t>
+          <t>[Business Wire](https://www.businesswire.com/news/home/20260126236053/en/Pacifico-Energy-Secures-7.65-GW-Power-Generation-Permit-for-GW-Ranch-Project)</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -5096,7 +5245,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/amazon-looks-to-build-large-scale-data-center-campus-next-to-nuclear-plant-in-texas/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/amazon-looks-to-build-large-scale-data-center-campus-next-to-nuclear-plant-in-texas/)</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -5128,17 +5277,17 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Permisos/negociación avanzada (construcción inminente)</t>
+          <t>Permisos/negociación avanzada (inversión total US$3.7 mil millones: US$2.7B centro de datos + US$1B planta de fertilizantes Fermachem; gasoducto de 160km desde Texas; planta de ciclo combinado on-site de 350MW para alimentar data center de 250MW; Congreso de Durango aprobó donación de 50 hectáreas)</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>https://mexiconewsdaily.com/business/durango-data-center-fertilizer-plant-investment-fermaca/</t>
+          <t>[Mexico News Daily](https://mexiconewsdaily.com/business/durango-data-center-fertilizer-plant-investment-fermaca/); [DCD](https://www.datacenterdynamics.com/en/news/250mw-natural-gas-powered-data-center-campus-announced-in-durango-mexico/)</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
@@ -5170,7 +5319,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/circe-energy-secures-2gw-of-natural-gas-capacity-for-west-texas-data-center-campus/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/circe-energy-secures-2gw-of-natural-gas-capacity-for-west-texas-data-center-campus/)</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -5207,7 +5356,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>https://sourcenm.com/2026/07/16/new-mexico-land-commissioner-blocks-project-jupiter-related-pipeline-from-building-on-state-land/</t>
+          <t>[Source NM](https://sourcenm.com/2026/07/16/new-mexico-land-commissioner-blocks-project-jupiter-related-pipeline-from-building-on-state-land/)</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -5244,7 +5393,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/powerplay-ai-announces-400-mw-behind-the-meter-ai-data-center-development-in-greater-abilene-with-nasdaq-listed-neocloud-joint-venture-partner-302829610.html</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/powerplay-ai-announces-400-mw-behind-the-meter-ai-data-center-development-in-greater-abilene-with-nasdaq-listed-neocloud-joint-venture-partner-302829610.html)</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -5281,7 +5430,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/liberty-energy-powerbridge-form-jv-to-power-planned-2gw-data-center-in-west-texas/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/liberty-energy-powerbridge-form-jv-to-power-planned-2gw-data-center-in-west-texas/)</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -5318,7 +5467,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>https://www.powermag.com/nuclear-natural-gas-power-generation-planned-for-massive-new-mexico-data-center-site/</t>
+          <t>[PowerMag](https://www.powermag.com/nuclear-natural-gas-power-generation-planned-for-massive-new-mexico-data-center-site/)</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -5355,7 +5504,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterfrontier.com/site-selection/article/55289667/powering-ai-in-the-permian-texas-critical-data-centers-sustainable-energy-play</t>
+          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55289667/powering-ai-in-the-permian-texas-critical-data-centers-sustainable-energy-play)</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -5392,7 +5541,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>https://openai.com/index/five-new-stargate-sites/</t>
+          <t>[OpenAI](https://openai.com/index/five-new-stargate-sites/)</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -5429,7 +5578,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>https://openai.com/index/five-new-stargate-sites/</t>
+          <t>[OpenAI](https://openai.com/index/five-new-stargate-sites/)</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -5466,7 +5615,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>https://mexiconewsdaily.com/business/aws-invest-5b-mexico-data-region/</t>
+          <t>[Mexico News Daily](https://mexiconewsdaily.com/business/aws-invest-5b-mexico-data-region/)</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -5503,7 +5652,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/oracle-and-openai-start-construction-on-stargate-data-center-campus-in-saline-township-michigan/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/oracle-and-openai-start-construction-on-stargate-data-center-campus-in-saline-township-michigan/)</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -5540,7 +5689,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>https://www.valleynewslive.com/2026/07/13/applied-digital-expands-north-dakota-eyes-oliver-county-third-data-center/</t>
+          <t>[Valley News Live](https://www.valleynewslive.com/2026/07/13/applied-digital-expands-north-dakota-eyes-oliver-county-third-data-center/)</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -5577,7 +5726,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>https://energymagazine.mx/2026/01/el-data-center-verde-que-encendio-la-polemica-asi-sera-el-proyecto-de-ia-en-nuevo-leon-que-usara-tecnologia-de-nvidia/</t>
+          <t>[Energy Magazine MX](https://energymagazine.mx/2026/01/el-data-center-verde-que-encendio-la-polemica-asi-sera-el-proyecto-de-ia-en-nuevo-leon-que-usara-tecnologia-de-nvidia/)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -5614,7 +5763,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>https://www.constructiondive.com/news/data-center-cleanarc-breaks-ground-virginia-campus/806489/</t>
+          <t>[Construction Dive](https://www.constructiondive.com/news/data-center-cleanarc-breaks-ground-virginia-campus/806489/)</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -5651,7 +5800,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>https://www.ksl.com/article/51402125/groundbreaking-for-new-millard-county-artificial-intelligence-data-center</t>
+          <t>[KSL](https://www.ksl.com/article/51402125/groundbreaking-for-new-millard-county-artificial-intelligence-data-center)</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -5688,7 +5837,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>https://governor.mo.gov/press-releases/archive/amazon-investing-10-billion-montgomery-county</t>
+          <t>[Governor.mo.gov](https://governor.mo.gov/press-releases/archive/amazon-investing-10-billion-montgomery-county)</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -5725,7 +5874,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>https://www.stlpr.org/government-politics-issues/2026-05-21/missouri-governor-google-announce-15-billion-data-center-montgomery-county</t>
+          <t>[STLPR](https://www.stlpr.org/government-politics-issues/2026-05-21/missouri-governor-google-announce-15-billion-data-center-montgomery-county)</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -5762,7 +5911,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2026/07/06/3322404/0/en/big-digital-energy-announces-partnership-with-10netzero-to-acquire-power-ready-hood-county-texas-site-for-ai-datacenter-development.html</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/06/3322404/0/en/big-digital-energy-announces-partnership-with-10netzero-to-acquire-power-ready-hood-county-texas-site-for-ai-datacenter-development.html)</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -5799,7 +5948,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/)</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -5836,7 +5985,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/meta-files-to-expand-campus-in-el-paso-texas-with-12-new-buildings/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/meta-files-to-expand-campus-in-el-paso-texas-with-12-new-buildings/)</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -5868,17 +6017,17 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Planeación/desarrollo temprano</t>
+          <t>Planeación avanzada (SB Energy construirá 9.2GW de generación a gas natural, financiamiento de US$33.3 mil millones por SoftBank, más US$4.2 mil millones en transmisión; 26-jul-2026 trascendió que Nvidia negocia garantía financiera de hasta US$250 mil millones para que OpenAI arriende el sitio, primera fase de 800MW en 2028)</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/softbank-eyes-10gw-data-center-at-former-doe-nuclear-enrichment-site-in-ohio/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/softbank-eyes-10gw-data-center-at-former-doe-nuclear-enrichment-site-in-ohio/); [Bloomberg](https://www.bloomberg.com/news/articles/2026-07-26/nvidia-in-talks-on-250-billion-backing-for-openai-hub-wsj-says)</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
@@ -5910,7 +6059,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/)</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -5947,7 +6096,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>https://www.williams.com/2026/07/13/williams-announces-5-34-billion-investment-in-power-innovation-joint-venture-from-blackstone/</t>
+          <t>[Williams Companies](https://www.williams.com/2026/07/13/williams-announces-5-34-billion-investment-in-power-innovation-joint-venture-from-blackstone/)</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -5984,7 +6133,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/cleancore-solutions-zone-announces-closing-of-first-data-center-project-establishing-its-critical-infrastructure-buildout-for-the-ai-economy-302821421.html</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/cleancore-solutions-zone-announces-closing-of-first-data-center-project-establishing-its-critical-infrastructure-buildout-for-the-ai-economy-302821421.html)</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -6021,7 +6170,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>https://www.bloomberg.com/news/articles/2026-06-09/crusoe-touts-5-gigawatts-worth-of-data-centers-deals-pauses-wyoming-site</t>
+          <t>[Bloomberg](https://www.bloomberg.com/news/articles/2026-06-09/crusoe-touts-5-gigawatts-worth-of-data-centers-deals-pauses-wyoming-site)</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -6058,7 +6207,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>https://www.hpcwire.com/off-the-wire/core-scientific-plans-expansion-to-1-5gw-of-gross-power-at-pecos-texas-campus/</t>
+          <t>[HPCwire](https://www.hpcwire.com/off-the-wire/core-scientific-plans-expansion-to-1-5gw-of-gross-power-at-pecos-texas-campus/)</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -6095,7 +6244,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>https://utahnewsdispatch.com/2026/05/19/renderings-show-massive-data-center-box-elder-utah-permits-could-take-years/</t>
+          <t>[Utah News Dispatch](https://utahnewsdispatch.com/2026/05/19/renderings-show-massive-data-center-box-elder-utah-permits-could-take-years/)</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -6132,7 +6281,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>https://www.stocktitan.net/news/FRMI/fermi-announces-first-siemens-turbines-arrive-at-port-of-qg7ienp885jk.html</t>
+          <t>[StockTitan](https://www.stocktitan.net/news/FRMI/fermi-announces-first-siemens-turbines-arrive-at-port-of-qg7ienp885jk.html)</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -6169,7 +6318,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>https://www.kltv.com/2026/03/20/president-trump-approves-16-billion-natural-gas-generator-be-installed-anderson-county/</t>
+          <t>[KLTV](https://www.kltv.com/2026/03/20/president-trump-approves-16-billion-natural-gas-generator-be-installed-anderson-county/)</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -6206,7 +6355,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>https://wvmetronews.com/2026/07/16/mon-power-president-says-data-centers-will-end-up-paying-for-natural-gas-powered-power-plant/</t>
+          <t>[WV MetroNews](https://wvmetronews.com/2026/07/16/mon-power-president-says-data-centers-will-end-up-paying-for-natural-gas-powered-power-plant/)</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -6243,7 +6392,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>https://www.utilitydive.com/news/iep-plans-944-mw-behind-the-meter-gas-plant-in-pennsylvania-to-power-data-c/758830/</t>
+          <t>[Utility Dive](https://www.utilitydive.com/news/iep-plans-944-mw-behind-the-meter-gas-plant-in-pennsylvania-to-power-data-c/758830/)</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -6280,7 +6429,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/aws-files-for-12bn-data-center-campus-outside-houston-texas/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/aws-files-for-12bn-data-center-campus-outside-houston-texas/)</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -6317,7 +6466,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>https://www.crusoe.ai/resources/newsroom/crusoe-and-lancium-announce-1-gigawatt-ai-data-center-campus-in-childress-texas</t>
+          <t>[Crusoe](https://www.crusoe.ai/resources/newsroom/crusoe-and-lancium-announce-1-gigawatt-ai-data-center-campus-in-childress-texas)</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -6354,7 +6503,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/)</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -6391,7 +6540,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>https://www.powermag.com/new-200-mw-gas-fired-plant-in-ohio-will-power-meta-data-center/</t>
+          <t>[PowerMag](https://www.powermag.com/new-200-mw-gas-fired-plant-in-ohio-will-power-meta-data-center/)</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -6428,7 +6577,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>https://www.aterio.io/blog/crusoe-launches-usd29b-goodnight-campus-in-claude-mirroring-openai-s-stargate</t>
+          <t>[Aterio](https://www.aterio.io/blog/crusoe-launches-usd29b-goodnight-campus-in-claude-mirroring-openai-s-stargate)</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -6465,7 +6614,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>https://www.ajc.com/business/2026/07/officials-order-georgia-data-centers-pop-up-power-plant-to-halt-construction/</t>
+          <t>[AJC](https://www.ajc.com/business/2026/07/officials-order-georgia-data-centers-pop-up-power-plant-to-halt-construction/)</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -6502,7 +6651,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/stark-power-lands-56gw-data-center-development-portfolio-in-sagebrush-acquisition/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/stark-power-lands-56gw-data-center-development-portfolio-in-sagebrush-acquisition/)</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -6539,7 +6688,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterfrontier.com/site-selection/article/55281341/pennsylvanias-homer-city-energy-campus-a-brownfield-transformed-for-data-center-innovation</t>
+          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55281341/pennsylvanias-homer-city-energy-campus-a-brownfield-transformed-for-data-center-innovation)</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -6576,7 +6725,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterknowledge.com/data-center-site-selection/nebius-plans-300-mw-data-center-in-new-jersey-amid-us-expansion</t>
+          <t>[Data Center Knowledge](https://www.datacenterknowledge.com/data-center-site-selection/nebius-plans-300-mw-data-center-in-new-jersey-amid-us-expansion)</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -6613,7 +6762,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/terravolt-inks-natural-gas-supply-deal-for-onsite-power-plant-at-planned-data-center-campus-in-idaho/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/terravolt-inks-natural-gas-supply-deal-for-onsite-power-plant-at-planned-data-center-campus-in-idaho/)</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -6650,7 +6799,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/cyrusone-announces-sixth-data-center-campus-in-san-antonio-texas/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/cyrusone-announces-sixth-data-center-campus-in-san-antonio-texas/)</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -6662,7 +6811,7 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>EdgeConneX PowerConneX New Albany Energy Center (I y II)</t>
+          <t>EdgeConneX PowerConneX New Albany Energy Center (I, II y III)</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -6682,17 +6831,17 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Construcción (PowerConneX I, 120MW, certificado OPSB 22-jul-2025, construcción iniciada sep-2025, operación comercial posible 3T2026; PowerConneX II, 216MW, solicitado ante OPSB, operación comercial objetivo 2T2027)</t>
+          <t>Construcción (PowerConneX I, 120MW, certificado OPSB 22-jul-2025, construcción iniciada sep-2025, operación comercial posible 3T2026; PowerConneX II, 216MW, solicitado ante OPSB, operación comercial objetivo 2T2027; PowerConneX III, 430MW, notificación previa ante OPSB abr-2026, elevando capacidad total del sitio a ~766MW de gas)</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/edgeconnex-plans-120mw-gas-plant-to-power-ohio-data-center/</t>
+          <t>[Data Center Dynamics](https://www.datacenterdynamics.com/en/news/edgeconnex-plans-120mw-gas-plant-to-power-ohio-data-center/); [BeBeez](https://bebeez.eu/2026/04/14/edgeconnex-affiliate-proposes-430mw-natural-gas-plant-to-power-data-center-campus-in-new-albany-ohio/)</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
@@ -6724,7 +6873,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>https://www.technology.org/2026/07/15/xai-59-unpermitted-gas-turbines-southaven-colossus-2/</t>
+          <t>[Technology.org](https://www.technology.org/2026/07/15/xai-59-unpermitted-gas-turbines-southaven-colossus-2/)</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -6761,7 +6910,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/cleco-to-construct-756mw-natural-gas-plant-to-serve-applied-digitals-data-center-in-rapides-parish-louisiana-report/</t>
+          <t>[Data Center Dynamics](https://www.datacenterdynamics.com/en/news/cleco-to-construct-756mw-natural-gas-plant-to-serve-applied-digitals-data-center-in-rapides-parish-louisiana-report/)</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -6798,7 +6947,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>https://kentuckylantern.com/2026/07/22/developer-proposes-hyperscale-data-center-at-the-site-at-former-eastern-kentucky-steel-mill/</t>
+          <t>[Kentucky Lantern](https://kentuckylantern.com/2026/07/22/developer-proposes-hyperscale-data-center-at-the-site-at-former-eastern-kentucky-steel-mill/)</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -6835,12 +6984,86 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/qts-to-build-11-data-centers-on-lancium-campus-in-hall-county-texas/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/qts-to-build-11-data-centers-on-lancium-campus-in-hall-county-texas/)</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
           <t>2026-07-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Anthropic/Nexus Hubbard Campus</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Hubbard, Condado de Hill, Texas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Anthropic (operado por Nexus Data Centers; respaldo financiero de Google)</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>Construcción iniciada (primera fase 500-612MW prevista 2026, ampliable a ~7.2-7.7GW; planta de gas natural behind-the-meter cerca de gasoducto principal)</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/600mw-natural-gas-powered-data-center-campus-proposed-in-hubbard-texas/); [Construction Review](https://constructionreviewonline.com/5bn-anthropic-data-center-in-texas-receives-critical-financial-backing-from-google/)</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>Stillwater Technology Park</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>Lovejoy, Condado de Clayton, Georgia, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>Stillwater Development, LLC (cliente hyperscaler final no revelado)</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>Permisos ("development of regional impact" presentado ante el estado; hasta 15 edificios, 1.25GW, US$13 mil millones; generación de energía aún no confirmada, contempla interconexión con Central Georgia EMC)</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/gigawatt-scale-data-center-campus-planned-outside-atlanta-georgia/)</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Agregar 6 proyectos nuevos y 12 cambios de fase (2026-07-28) (#10)
Nuevos:
- Petroquímica: Green Fuels Operating - Refinería Duncan (Oklahoma)
- LNG: CP2 LNG Fase 3 (Louisiana)
- Mining: Pathfinder Tonopah (Nevada), La Colorada Mine expansión (Sonora)
- Data Centers: Anthropic/Nexus Hubbard Campus (Texas), Stillwater Technology Park (Georgia)

Cambios de fase: CF Industries Blue Point, Fertinal-ProAgro, Rio Grande LNG,
Corpus Christi Stage 3, Los Ricos South Mine, Copper World Complex,
Resolution Copper, Stargate Frontier Campus, SB Energy PORTS Technology
Campus, Fermaca Digital City, Prometheus Hyperscale Dallas, EdgeConneX
PowerConneX New Albany.

Se regeneró proyectos.xlsx con el acumulado completo (una hoja por industria).


Claude-Session: https://claude.ai/code/session_012WFngDt9cuLNAQtoEh1sN8

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -35,6 +35,7 @@
     </font>
     <font>
       <name val="Arial"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="3">
@@ -66,7 +67,7 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -436,16 +437,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -513,7 +514,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>https://newsroom.fluor.com/news-releases/news-details/2026/Fluor-Awarded-Contract-to-Engineer-and-Design-the-America-First-Refining-Facility-in-Brownsville-Texas/default.aspx</t>
+          <t>[Fluor newsroom](https://newsroom.fluor.com/news-releases/news-details/2026/Fluor-Awarded-Contract-to-Engineer-and-Design-the-America-First-Refining-Facility-in-Brownsville-Texas/default.aspx)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -550,7 +551,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>https://allstreaminsiders.com/us-exxonmobil-may-build-cracker-pe-plant-in-texas-with-an-8-6-billion-investment/</t>
+          <t>[AllStream Insiders](https://allstreaminsiders.com/us-exxonmobil-may-build-cracker-pe-plant-in-texas-with-an-8-6-billion-investment/)</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -587,7 +588,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>https://www.bicmagazine.com/departments/operations/cpchem-golden-triangle-polymers-facility-startup-phase/</t>
+          <t>[BIC Magazine](https://www.bicmagazine.com/departments/operations/cpchem-golden-triangle-polymers-facility-startup-phase/)</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -619,17 +620,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Construcción</t>
+          <t>Construcción (impulso federal de permisos anunciado may-2026 con finalización esperada en 45 días; CF Industries confirma inicio de construcción en 2026)</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>https://constructionfront.com/2025-04-13-technip-energies-to-deliver-blue-point-worlds-largest-low-carbon-ammonia-facility-in-louisiana/</t>
+          <t>[Construction Front](https://constructionfront.com/2025-04-13-technip-energies-to-deliver-blue-point-worlds-largest-low-carbon-ammonia-facility-in-louisiana/); [FuelCellsWorks](https://fuelcellsworks.com/2026/05/07/h2/cf-industries-targets-construction-start-this-year-on-blue-hydrogen-and-ammonia-complex)</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
@@ -661,7 +662,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>https://eastdaley.com/media-and-news/the-race-is-on-to-build-permian-processing</t>
+          <t>[East Daley](https://eastdaley.com/media-and-news/the-race-is-on-to-build-permian-processing)</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -698,7 +699,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>https://www.techint.com/en/our-projects/dos-bocas-refinery</t>
+          <t>[Techint](https://www.techint.com/en/our-projects/dos-bocas-refinery)</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -735,7 +736,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>https://www.ogj.com/refining-processing/refining/optimization/article/17279334/pemex-to-proceed-with-dos-bocas-refinery-project</t>
+          <t>[OGJ](https://www.ogj.com/refining-processing/refining/optimization/article/17279334/pemex-to-proceed-with-dos-bocas-refinery-project)</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -772,7 +773,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>https://forbes.com.mx/pemex-invertira-5300-millones-de-dolares-para-reactivar-la-industria-petroquimica/</t>
+          <t>[Forbes México](https://forbes.com.mx/pemex-invertira-5300-millones-de-dolares-para-reactivar-la-industria-petroquimica/)</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -809,7 +810,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>https://forbes.com.mx/pemex-invertira-5300-millones-de-dolares-para-reactivar-la-industria-petroquimica/</t>
+          <t>[Forbes México](https://forbes.com.mx/pemex-invertira-5300-millones-de-dolares-para-reactivar-la-industria-petroquimica/)</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -846,7 +847,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>https://forbes.com.mx/asi-es-la-inversion-de-1553-mdd-por-parte-de-pemex-en-una-planta-de-fertilizantes-en-veracruz/</t>
+          <t>[Forbes México](https://forbes.com.mx/asi-es-la-inversion-de-1553-mdd-por-parte-de-pemex-en-una-planta-de-fertilizantes-en-veracruz/)</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -878,17 +879,17 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/rehabilitación</t>
+          <t>Ingeniería/rehabilitación (incorporado al plan de reactivación petroquímica de Pemex, jun-2026; 13,700 millones de pesos asignados para los complejos Lázaro Cárdenas y ProAgro; meta de 2.4 millones ton/año de urea y fertilizantes fosfatados)</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>https://tribuna.com.mx/mexico/2026/06/05/sheinbaum-anuncia-inversion-de-93-mil-mdp-para-reactivar-la-industria-petroquimica-y-de-fertilizantes-en-veracruz_560837/</t>
+          <t>[Tribuna](https://tribuna.com.mx/mexico/2026/06/05/sheinbaum-anuncia-inversion-de-93-mil-mdp-para-reactivar-la-industria-petroquimica-y-de-fertilizantes-en-veracruz_560837/); [Contralínea](https://contralinea.com.mx/interno/semana/presentan-plan-con-inversion-de-93-mil-mdp-para-rescatar-la-petroquimica-nacional/)</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
@@ -920,7 +921,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>https://www.pv-magazine-mexico.com/2026/04/28/inician-en-sinaloa-la-construccion-de-la-mayor-planta-de-metanol-ultrabajo-en-carbono-a-partir-de-hidrogeno-verde/</t>
+          <t>[PV Magazine México](https://www.pv-magazine-mexico.com/2026/04/28/inician-en-sinaloa-la-construccion-de-la-mayor-planta-de-metanol-ultrabajo-en-carbono-a-partir-de-hidrogeno-verde/)</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -957,7 +958,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>https://www.h2-view.com/story/first-ammonia-project-on-track-for-2026-fid-despite-topsoe-deal-collapse/2138792.article/</t>
+          <t>[H2 View](https://www.h2-view.com/story/first-ammonia-project-on-track-for-2026-fid-despite-topsoe-deal-collapse/2138792.article/)</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -994,7 +995,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>https://www.debate.com.mx/economia/secretaria-de-economia-complejo-de-amoniaco-en-topolobampo-prioritario-para-el-gobierno-de-mexico-20260713-0092.html</t>
+          <t>[Debate](https://www.debate.com.mx/economia/secretaria-de-economia-complejo-de-amoniaco-en-topolobampo-prioritario-para-el-gobierno-de-mexico-20260713-0092.html)</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -1031,7 +1032,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>https://www.icis.com/explore/resources/news/2025/11/13/11155109/lake-charles-methanol-ii-awards-feed-fid-expected-in-q2-2026/</t>
+          <t>[ICIS](https://www.icis.com/explore/resources/news/2025/11/13/11155109/lake-charles-methanol-ii-awards-feed-fid-expected-in-q2-2026/)</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -1068,7 +1069,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>https://diariodelistmo.com/nacional/este-es-el-avance-que-lleva-la-planta-coquizadora-en-la-refineria-de-salina-cruz/50642321</t>
+          <t>[Diario del Istmo](https://diariodelistmo.com/nacional/este-es-el-avance-que-lleva-la-planta-coquizadora-en-la-refineria-de-salina-cruz/50642321)</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -1105,7 +1106,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>https://www.hydrocarbonengineering.com/petrochemicals/06032026/shintech-announces-us34-billion-at-louisiana-petrochemicals-complex/</t>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/petrochemicals/06032026/shintech-announces-us34-billion-at-louisiana-petrochemicals-complex/)</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -1142,7 +1143,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>https://www.alchempro.com/news/chemicals-news/ineos-backs-1-7-bn-low-carbon-methanol-project-in-texas-city-310108-newsdetails.htm</t>
+          <t>[Alchempro](https://www.alchempro.com/news/chemicals-news/ineos-backs-1-7-bn-low-carbon-methanol-project-in-texas-city-310108-newsdetails.htm)</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -1179,7 +1180,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>https://www.hydrocarbonengineering.com/petrochemicals/13072026/oxea-confirms-fid-for-major-capacity-expansion/</t>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/petrochemicals/13072026/oxea-confirms-fid-for-major-capacity-expansion/)</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -1216,7 +1217,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>https://www.ogj.com/refining-processing/gas-processing/news/55320579/targa-advances-permian-gas-pipeline-processing-expansion</t>
+          <t>[OGJ](https://www.ogj.com/refining-processing/gas-processing/news/55320579/targa-advances-permian-gas-pipeline-processing-expansion)</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -1253,7 +1254,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>https://www.businesswire.com/news/home/20250806663187/en/Enterprise-Agrees-to-Acquire-Occidentals-Gas-Gathering-Affiliate-Enters-Into-Natural-Gas-Processing-Agreement-Announces-New-Midland-Basin-Natural-Gas-Processing-Plant</t>
+          <t>[Business Wire](https://www.businesswire.com/news/home/20250806663187/en/Enterprise-Agrees-to-Acquire-Occidentals-Gas-Gathering-Affiliate-Enters-Into-Natural-Gas-Processing-Agreement-Announces-New-Midland-Basin-Natural-Gas-Processing-Plant)</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -1290,7 +1291,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>https://naturalgasintel.com/news/mplx-scales-up-for-power-hungry-future-with-natural-gas-focused-growth-plan/</t>
+          <t>[Natural Gas Intel](https://naturalgasintel.com/news/mplx-scales-up-for-power-hungry-future-with-natural-gas-focused-growth-plan/)</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -1327,7 +1328,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>https://eastdaley.com/daley-note/mplx-acquires-northwind-for-2-375b-acquires-more-ngls-for-jv-project</t>
+          <t>[East Daley](https://eastdaley.com/daley-note/mplx-acquires-northwind-for-2-375b-acquires-more-ngls-for-jv-project)</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -1364,7 +1365,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>https://www.grandforksherald.com/news/local/northern-plains-nitrogen-proposal-receiving-more-attention-amid-global-fertilizer-pressure</t>
+          <t>[Grand Forks Herald](https://www.grandforksherald.com/news/local/northern-plains-nitrogen-proposal-receiving-more-attention-amid-global-fertilizer-pressure)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -1401,7 +1402,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>https://www.phillips66.com/newsroom/iron-mesa-safely-enters-next-phase-of-construction/</t>
+          <t>[Phillips 66](https://www.phillips66.com/newsroom/iron-mesa-safely-enters-next-phase-of-construction/)</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -1438,7 +1439,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>https://www.targaresources.com/news-releases/news-release-details/targa-resources-corp-announces-permian-growth-projects-and</t>
+          <t>[Targa Resources](https://www.targaresources.com/news-releases/news-release-details/targa-resources-corp-announces-permian-growth-projects-and)</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -1475,7 +1476,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>https://elefanteblanco.mx/2026/01/02/pemex-abre-30-licitaciones-para-obras-en-la-refineria-madero/</t>
+          <t>[Elefante Blanco](https://elefanteblanco.mx/2026/01/02/pemex-abre-30-licitaciones-para-obras-en-la-refineria-madero/)</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -1512,7 +1513,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>https://www.jornada.com.mx/noticia/2026/06/08/economia/da-inicio-ejecucion-de-planta-de-fertilizantes-en-durango-por-parte-de-fermachem</t>
+          <t>[La Jornada](https://www.jornada.com.mx/noticia/2026/06/08/economia/da-inicio-ejecucion-de-planta-de-fertilizantes-en-durango-por-parte-de-fermachem)</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -1549,7 +1550,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>https://downstreamcalendar.com/mcdermott-secures-feed-contract-for-ascension-clean-energy-project/</t>
+          <t>[Downstream Calendar](https://downstreamcalendar.com/mcdermott-secures-feed-contract-for-ascension-clean-energy-project/)</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -1586,7 +1587,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>https://www.businesswire.com/news/home/20260517310811/en/Phillips-66-announces-Zeus-Gas-Plant-and-a-third-Coastal-Bend-Fractionator</t>
+          <t>[Business Wire](https://www.businesswire.com/news/home/20260517310811/en/Phillips-66-announces-Zeus-Gas-Plant-and-a-third-Coastal-Bend-Fractionator)</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -1623,7 +1624,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>https://www.usda.gov/about-usda/news/press-releases/2026/07/01/secretary-rollins-announces-500-million-fertilizer-investment-and-expansion-program-strengthen</t>
+          <t>[USDA](https://www.usda.gov/about-usda/news/press-releases/2026/07/01/secretary-rollins-announces-500-million-fertilizer-investment-and-expansion-program-strengthen)</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -1660,12 +1661,49 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>https://www.hydrocarbonengineering.com/clean-fuels/06012026/samsung-ea-announces-groundbreaking-of-low-carbon-ammonia-plant/</t>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/clean-fuels/06012026/samsung-ea-announces-groundbreaking-of-low-carbon-ammonia-plant/)</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
           <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Green Fuels Operating — Refinería Duncan</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Duncan, Stephens County, Oklahoma, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Green Fuels Operating</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Construcción (groundbreaking 29-may-2026; inversión US$400 millones; capacidad inicial 30,000 bbl/d, expandible a 50,000 bbl/d, sobre sitio de refinería histórica de los años 1920)</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/refining/03062026/green-fuels-hosts-groundbreaking-ceremony-for-new-refinery/)</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
@@ -1680,16 +1718,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1752,17 +1790,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Construcción</t>
+          <t>Construcción (FERC aprobó inicio de construcción de Trenes 4 y 5 en mar-2026; NextDecade evalúa un 6to tren para superar 36 mtpa; gasoducto de alimentación Rio Bravo Pipeline —138 millas, JV Whitewater/MPLX/Enbridge— en camino a entrar en servicio 2S2026)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>https://www.bechtel.com/press-releases/nextdecade-executes-epc-contract-with-bechtel-for-train-4-at-the-rio-grande-lng-facility/</t>
+          <t>[Bechtel](https://www.bechtel.com/press-releases/nextdecade-executes-epc-contract-with-bechtel-for-train-4-at-the-rio-grande-lng-facility/); [Natural Gas Intel](https://naturalgasintel.com/news/nextdecade-targets-more-than-36-mty-with-rio-grande-lng-upscale-sixth-train-expansion/)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
@@ -1794,7 +1832,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>https://www.bechtel.com/press-releases/sempra-infrastructure-announces-epc-contract-with-bechtel-for-port-arthur-lng-phase-2/</t>
+          <t>[Bechtel](https://www.bechtel.com/press-releases/sempra-infrastructure-announces-epc-contract-with-bechtel-for-port-arthur-lng-phase-2/)</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -1831,7 +1869,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>https://www.woodside.com/what-we-do/growth-projects/woodside-louisiana-lng</t>
+          <t>[Woodside](https://www.woodside.com/what-we-do/growth-projects/woodside-louisiana-lng)</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1868,7 +1906,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>https://www.gem.wiki/CP2_LNG_Terminal</t>
+          <t>[GEM.wiki](https://www.gem.wiki/CP2_LNG_Terminal)</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -1905,7 +1943,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>https://www.offshore-energy.biz/kbr-zachry-to-work-on-ventures-plaquemines-lng/</t>
+          <t>[Offshore Energy](https://www.offshore-energy.biz/kbr-zachry-to-work-on-ventures-plaquemines-lng/)</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1942,7 +1980,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>https://panews.com/2026/04/24/golden-pass-lng-makes-history-with-first-export-from-sabine-pass-terminal/</t>
+          <t>[Port Arthur News](https://panews.com/2026/04/24/golden-pass-lng-makes-history-with-first-export-from-sabine-pass-terminal/)</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -1974,17 +2012,17 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Construcción (FERC autorizó introducción de gas combustible en Train 7, 17-jul-2026; primera producción de LNG esperada ago-2026, servicio comercial sep-2026)</t>
+          <t>Construcción (FERC autorizó introducción de gas combustible en Train 7, 17-jul-2026; primera producción de LNG esperada ago-2026, servicio comercial sep-2026; Trenes 5 y 6 completados mar/jun-2026; expansión completa de 7 trenes 85.4% de avance, prevista para fin de 2026)</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>https://pgjonline.com/news/2026/july/corpus-christi-lng-train-7-cleared-to-introduce-fuel-gas-by-ferc</t>
+          <t>[PGJ](https://pgjonline.com/news/2026/july/corpus-christi-lng-train-7-cleared-to-introduce-fuel-gas-by-ferc); [LNG Prime](https://lngprime.com/americas/chenieres-corpus-christi-expansion-project-85-4-percent-complete/155448/)</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
@@ -2016,7 +2054,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2026/06/03/3306350/0/en/delfin-midstream-announces-5-billion-final-investment-decision-for-first-flng-vessel.html</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/06/03/3306350/0/en/delfin-midstream-announces-5-billion-final-investment-decision-for-first-flng-vessel.html)</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -2053,7 +2091,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>https://dossierpolitico.com/2026/07/17/activistas-entregan-90-mil-firmas-para-frenar-proyecto-saguaro-energia-en-sonora/</t>
+          <t>[Dossier Político](https://dossierpolitico.com/2026/07/17/activistas-entregan-90-mil-firmas-para-frenar-proyecto-saguaro-energia-en-sonora/)</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -2090,7 +2128,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>https://www.gem.wiki/New_Fortress_Altamira_FLNG_Terminal</t>
+          <t>[GEM Wiki](https://www.gem.wiki/New_Fortress_Altamira_FLNG_Terminal)</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -2127,7 +2165,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>https://www.naturalgasintel.com/news/glenfarne-lands-investment-for-early-work-on-texas-lng-ahead-of-fid/</t>
+          <t>[Natural Gas Intel](https://www.naturalgasintel.com/news/glenfarne-lands-investment-for-early-work-on-texas-lng-ahead-of-fid/)</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -2164,7 +2202,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>https://pgjonline.com/news/2026/july/commonwealth-lng-awards-main-automation-contract-for-louisiana-export-terminal</t>
+          <t>[PGJ](https://pgjonline.com/news/2026/july/commonwealth-lng-awards-main-automation-contract-for-louisiana-export-terminal)</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -2201,7 +2239,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>https://www.houstonpublicmedia.org/articles/galveston-county/2026/07/14/557086/galveston-pelican-island-lng/</t>
+          <t>[Houston Public Media](https://www.houstonpublicmedia.org/articles/galveston-county/2026/07/14/557086/galveston-pelican-island-lng/)</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -2238,7 +2276,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>https://www.sempra.com/newsroom/press-releases/sempra-infrastructures-eca-lng-phase-1-exports-first-lng-cargo-mexicos</t>
+          <t>[Sempra](https://www.sempra.com/newsroom/press-releases/sempra-infrastructures-eca-lng-phase-1-exports-first-lng-cargo-mexicos)</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -2275,7 +2313,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>https://lngprime.com/americas/gato-negro-eyes-fid-on-mexico-lng-plant-in-late-2026/165906/</t>
+          <t>[LNG Prime](https://lngprime.com/americas/gato-negro-eyes-fid-on-mexico-lng-plant-in-late-2026/165906/)</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -2312,7 +2350,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/amigo-lng-awards-landmark-epc-contract-to-dubai-based-drydocks-world-for-worlds-largest-flng-facility-302537739.html</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/amigo-lng-awards-landmark-epc-contract-to-dubai-based-drydocks-world-for-worlds-largest-flng-facility-302537739.html)</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -2349,7 +2387,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>https://www.kbr.com/en/insights-news/press-release/kbr-awarded-feed-coastal-bend-lng-project</t>
+          <t>[KBR](https://www.kbr.com/en/insights-news/press-release/kbr-awarded-feed-coastal-bend-lng-project)</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -2386,7 +2424,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>https://www.ferc.gov/gulfstream-lng-terminal-project</t>
+          <t>[FERC](https://www.ferc.gov/gulfstream-lng-terminal-project)</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -2423,7 +2461,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>https://alaskabeacon.com/2026/07/17/hilcorp-killed-alaska-lng-bill-some-legislators-say-but-governor-calls-the-claim-bullst/</t>
+          <t>[Alaska Beacon](https://alaskabeacon.com/2026/07/17/hilcorp-killed-alaska-lng-bill-some-legislators-say-but-governor-calls-the-claim-bullst/)</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -2460,7 +2498,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>https://pgjonline.com/news/2026/july/311-mile-sonora-gas-pipeline-project-advances-in-mexico</t>
+          <t>[PGJ](https://pgjonline.com/news/2026/july/311-mile-sonora-gas-pipeline-project-advances-in-mexico)</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -2497,7 +2535,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>https://www.ogj.com/pipelines-transportation/pipelines/news/55322537/arm-energy-takes-fid-on-23-billion-mustang-express-pipeline</t>
+          <t>[OGJ](https://www.ogj.com/pipelines-transportation/pipelines/news/55322537/arm-energy-takes-fid-on-23-billion-mustang-express-pipeline)</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -2534,7 +2572,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>https://mexicobusiness.news/energy/news/ursus-energy-scales-investment-us21-billion</t>
+          <t>[Mexico Business News](https://mexicobusiness.news/energy/news/ursus-energy-scales-investment-us21-billion)</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -2571,7 +2609,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2026/07/15/3327983/0/en/Delfin-Midstream-Partners-With-EIG-s-MidOcean-Energy-to-Advance-Second-FLNG-Vessel-Issues-Limited-Notice-to-Proceed-to-Siemens-Energy.html</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/15/3327983/0/en/Delfin-Midstream-Partners-With-EIG-s-MidOcean-Energy-to-Advance-Second-FLNG-Vessel-Issues-Limited-Notice-to-Proceed-to-Siemens-Energy.html)</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -2608,7 +2646,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>https://www.naturalgasintel.com/news/texas-gateway-open-season-expands-haynesville-natural-gas-links-amid-lng-growth/</t>
+          <t>[Natural Gas Intel](https://www.naturalgasintel.com/news/texas-gateway-open-season-expands-haynesville-natural-gas-links-amid-lng-growth/)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -2645,7 +2683,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>https://worldoil.com/news/2026/7/24/doe-approves-20-year-export-authorization-for-argent-lng-project/</t>
+          <t>[World Oil](https://worldoil.com/news/2026/7/24/doe-approves-20-year-export-authorization-for-argent-lng-project/)</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -2682,7 +2720,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>https://www.federalregister.gov/documents/2026/07/24/2026-14963/deepwater-port-license-application-st-lng-deepwater-port-development-project-final-environmental</t>
+          <t>[Federal Register](https://www.federalregister.gov/documents/2026/07/24/2026-14963/deepwater-port-license-application-st-lng-deepwater-port-development-project-final-environmental)</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -2719,7 +2757,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>https://naturalgasintel.com/news/kinder-morgan-greenlights-7b-in-natural-gas-pipeline-projects-amid-regulatory-speedup/</t>
+          <t>[Natural Gas Intel](https://naturalgasintel.com/news/kinder-morgan-greenlights-7b-in-natural-gas-pipeline-projects-amid-regulatory-speedup/)</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -2756,7 +2794,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>https://naturalgasintel.com/news/kinder-morgan-greenlights-7b-in-natural-gas-pipeline-projects-amid-regulatory-speedup/</t>
+          <t>[Natural Gas Intel](https://naturalgasintel.com/news/kinder-morgan-greenlights-7b-in-natural-gas-pipeline-projects-amid-regulatory-speedup/)</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -2793,7 +2831,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>https://lngprime.com/americas/kinder-morgan-seeks-doe-extension-for-gulf-lng-export-project/184334/</t>
+          <t>[LNG Prime](https://lngprime.com/americas/kinder-morgan-seeks-doe-extension-for-gulf-lng-export-project/184334/)</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -2830,7 +2868,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>https://investors.bakerhughes.com/news/press-releases/news-details/2026/Baker-Hughes-Secures-Substantial-Equipment-and-Services-Awards-for-Chenieres-Sabine-Pass-LNG-Facility/default.aspx</t>
+          <t>[Baker Hughes](https://investors.bakerhughes.com/news/press-releases/news-details/2026/Baker-Hughes-Secures-Substantial-Equipment-and-Services-Awards-for-Chenieres-Sabine-Pass-LNG-Facility/default.aspx)</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -2867,7 +2905,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>https://www.federalregister.gov/documents/2026/05/05/2026-08654/cheniere-corpus-christi-pipeline-lp-corpus-christi-liquefaction-stage-iv-llc-corpus-christi</t>
+          <t>[Federal Register](https://www.federalregister.gov/documents/2026/05/05/2026-08654/cheniere-corpus-christi-pipeline-lp-corpus-christi-liquefaction-stage-iv-llc-corpus-christi)</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -2904,7 +2942,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>https://www.federalregister.gov/documents/2026/07/24/2026-15040/freeport-lng-development-lp-flng-liquefaction-llc-flng-liquefaction-2-llc-flng-liquefaction-3-llc</t>
+          <t>[Federal Register](https://www.federalregister.gov/documents/2026/07/24/2026-15040/freeport-lng-development-lp-flng-liquefaction-llc-flng-liquefaction-2-llc-flng-liquefaction-3-llc)</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -2941,7 +2979,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>https://www.proyectosmexico.gob.mx/proyecto_inversion/1076-gasoducto-coatzacoalcos-ii/</t>
+          <t>[Proyectos México](https://www.proyectosmexico.gob.mx/proyecto_inversion/1076-gasoducto-coatzacoalcos-ii/)</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -2978,12 +3016,49 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>https://www.lngindustry.com/liquefaction/24072026/stabilis-solutions-receives-lor-from-us-coast-guard/</t>
+          <t>[LNG Industry](https://www.lngindustry.com/liquefaction/24072026/stabilis-solutions-receives-lor-from-us-coast-guard/)</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
           <t>2026-07-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>CP2 LNG Fase 3</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Cameron Parish, Luisiana, EE.UU. (adyacente al complejo CP2 Fase 1/2)</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Venture Global Inc.</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>No especificado (pendiente FID)</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Permitting (FERC exoneró proceso de pre-filing 16-abr-2026; solicitud formal presentada 26-may-2026; Notice of Application publicado 12-jun-2026; 6 bloques de licuefacción adicionales/12 trenes, planta de energía de 720MW, tercer atracadero marino; eleva capacidad pico del complejo de 28 a 35 mtpa)</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>[Federal Register](https://www.federalregister.gov/documents/2026/06/12/2026-11881/venture-global-cp2-lng-llc-venture-global-cp-express-llc-notice-of-application-and-establishing)</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
@@ -2998,16 +3073,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3075,7 +3150,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>https://www.miningweekly.com/article/ivanhoe-electric-pencils-in-2026-construction-start-at-arizona-copper-mine-2025-06-25</t>
+          <t>[Mining Weekly](https://www.miningweekly.com/article/ivanhoe-electric-pencils-in-2026-construction-start-at-arizona-copper-mine-2025-06-25)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -3107,17 +3182,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/Feasibility (DFS &gt;85% completo)</t>
+          <t>Ingeniería/Feasibility (DFS &gt;85% completo; colocación de bonos municipales por US$52 millones completada 24-jun-2026 para financiar el proyecto, ya totalmente permisado para iniciar construcción)</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1322422/000106299326001973/exhibit99-2.htm</t>
+          <t>[SEC/Hudbay](https://www.sec.gov/Archives/edgar/data/1322422/000106299326001973/exhibit99-2.htm); [GlobeNewswire](https://www.globenewswire.com/news-release/2026/06/24/3317147/0/en/hudbay-completes-offering-of-us-52-million-of-4-50-municipal-bonds-for-copper-world.html)</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
@@ -3144,17 +3219,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería temprana post intercambio de tierras (marzo 2026)</t>
+          <t>Ingeniería temprana post intercambio de tierras (marzo 2026); firmó Master Supply Agreement (1-jul-2026) con Johnson Controls Inc. y United Association Local 469 (sindicato de plomeros/pipefitters) para mantenimiento de instalaciones y soporte operativo en sitio</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/863064/000086306426000019/ex12d16mr_resolutionland.htm</t>
+          <t>[SEC](https://www.sec.gov/Archives/edgar/data/863064/000086306426000019/ex12d16mr_resolutionland.htm); [Resolution Copper](https://resolutioncopper.com/resolution-copper-and-united-association-local-469-enter-into-master-supply-agreement-supporting-operations-in-arizona/)</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
@@ -3186,7 +3261,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>https://www.nevadaappeal.com/news/2026/mar/26/lithium-americas-900-construction-workers-at-thacker-pass-mine/</t>
+          <t>[Nevada Appeal](https://www.nevadaappeal.com/news/2026/mar/26/lithium-americas-900-construction-workers-at-thacker-pass-mine/)</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -3223,7 +3298,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>https://www.mining.com/teck-agnico-team-up-at-san-nicolas-copper-project-in-mexico/</t>
+          <t>[Mining.com](https://www.mining.com/teck-agnico-team-up-at-san-nicolas-copper-project-in-mexico/)</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -3260,7 +3335,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>https://energymagazine.mx/2025/10/grupo-mexico-espera-autorizacion-federal-para-continuar-proyectos-mineros-por-10-mil-200-mdd/</t>
+          <t>[Energy Magazine MX](https://energymagazine.mx/2025/10/grupo-mexico-espera-autorizacion-federal-para-continuar-proyectos-mineros-por-10-mil-200-mdd/)</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -3297,7 +3372,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>https://www.bnamericas.com/en/news/southern-copper-wins-permits-for-us551mn-el-pilar-in-mexico</t>
+          <t>[BNamericas](https://www.bnamericas.com/en/news/southern-copper-wins-permits-for-us551mn-el-pilar-in-mexico)</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -3334,7 +3409,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>https://m3eng.com/portfolio/buenavista-del-cobre-concentradora-no-2/</t>
+          <t>[M3 Engineering](https://m3eng.com/portfolio/buenavista-del-cobre-concentradora-no-2/)</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -3371,7 +3446,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>https://mineriaenlinea.com/2026/04/torex-gold-alcanza-velocidad-de-crucero-en-media-luna-9-meses-adelante-de-cronograma/</t>
+          <t>[Minería en Línea](https://mineriaenlinea.com/2026/04/torex-gold-alcanza-velocidad-de-crucero-en-media-luna-9-meses-adelante-de-cronograma/)</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -3408,7 +3483,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>https://www.mining.com/nevada-copper-unveils-restart-and-financing-plan-for-pumpkin-hollow/</t>
+          <t>[Mining.com](https://www.mining.com/nevada-copper-unveils-restart-and-financing-plan-for-pumpkin-hollow/)</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -3445,7 +3520,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>https://www.usda.gov/about-usda/news/press-releases/2026/07/07/usda-advances-trump-administration-effort-boost-us-mineral-energy-production</t>
+          <t>[USDA](https://www.usda.gov/about-usda/news/press-releases/2026/07/07/usda-advances-trump-administration-effort-boost-us-mineral-energy-production)</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -3482,7 +3557,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/perpetua-resources-advances-construction-of-the-stibnite-gold-project-302787012.html</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/perpetua-resources-advances-construction-of-the-stibnite-gold-project-302787012.html)</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -3519,7 +3594,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>https://silvertigermetals.com/news/2026/silver-tiger-metals-awards-engineering-procurement-and-construction-management-contract-and-provides-construction-update</t>
+          <t>[Silver Tiger Metals](https://silvertigermetals.com/news/2026/silver-tiger-metals-awards-engineering-procurement-and-construction-management-contract-and-provides-construction-update)</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -3556,7 +3631,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/vizsla-silver-awards-epcm-and-mine-design-contracts-for-the-development-of-the-panuco-silver-gold-project-302750621.html</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/vizsla-silver-awards-epcm-and-mine-design-contracts-for-the-development-of-the-panuco-silver-gold-project-302750621.html)</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -3593,7 +3668,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>https://orlamining.com/news/orla-announces-results-of-updated-feasibility-study-for-south-railroad-project/</t>
+          <t>[Orla Mining](https://orlamining.com/news/orla-announces-results-of-updated-feasibility-study-for-south-railroad-project/)</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -3630,7 +3705,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>https://www.miningweekly.com/article/minera-alamos-confirms-low-cost-near-term-mining-possible-at-copperstone-in-arizona-2026-05-28</t>
+          <t>[Mining Weekly](https://www.miningweekly.com/article/minera-alamos-confirms-low-cost-near-term-mining-possible-at-copperstone-in-arizona-2026-05-28)</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -3667,7 +3742,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>https://www.wyomingnews.com/rawlinstimes/plans-move-forward-for-ck-gold-project-as-developers-target-2026-construction-start/article_b2bb147e-2f92-4ca2-bf86-fcc9983917a7.html</t>
+          <t>[Wyoming News](https://www.wyomingnews.com/rawlinstimes/plans-move-forward-for-ck-gold-project-as-developers-target-2026-construction-start/article_b2bb147e-2f92-4ca2-bf86-fcc9983917a7.html)</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -3704,7 +3779,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>https://www.juniorminingnetwork.com/junior-miner-news/press-releases/1082-tsx/ag/206222-first-majestic-receives-construction-permits-for-santo-nino-and-navidad-advances-development-across-the-santa-elena-district.html</t>
+          <t>[First Majestic](https://www.juniorminingnetwork.com/junior-miner-news/press-releases/1082-tsx/ag/206222-first-majestic-receives-construction-permits-for-santo-nino-and-navidad-advances-development-across-the-santa-elena-district.html)</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -3741,7 +3816,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/0001286973/000106299326002645/exhibit99-2.htm</t>
+          <t>[SEC/Americas Gold and Silver](https://www.sec.gov/Archives/edgar/data/0001286973/000106299326002645/exhibit99-2.htm)</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -3778,7 +3853,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>https://www.kitco.com/news/off-the-wire/2026-06-08/minera-frisco-restarts-two-mexico-mines-plans-new-silver-unit</t>
+          <t>[Kitco](https://www.kitco.com/news/off-the-wire/2026-06-08/minera-frisco-restarts-two-mexico-mines-plans-new-silver-unit)</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -3815,7 +3890,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/trilogy-metals-announces-publication-of-federal-and-state-permitting-schedule-for-arctic-project-establishing-defined-timeline-toward-a-record-of-decision-by-september-2028-302827083.html</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/trilogy-metals-announces-publication-of-federal-and-state-permitting-schedule-for-arctic-project-establishing-defined-timeline-toward-a-record-of-decision-by-september-2028-302827083.html)</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -3847,17 +3922,17 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Construcción aprobada (permisos SEMARNAT jun-2026)</t>
+          <t>Construcción aprobada por el consejo (permisos SEMARNAT completos jun-2026; presupuesto ~US$227 millones; ventana de construcción de ~24 meses; primer vertido de metal previsto mediados de 2028)</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>https://www.northernminer.com/news/gogold-approved-to-build-227m-mine-in-mexico/1003891932/</t>
+          <t>[Northern Miner](https://www.northernminer.com/news/gogold-approved-to-build-227m-mine-in-mexico/1003891932/); [Newsfile](https://www.newsfilecorp.com/release/300455/GoGold-Achieves-Major-Milestone-Final-Remaining-Permits-Secured-and-Construction-Approved-for-Los-Ricos-South-Underground-Mine)</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
@@ -3889,7 +3964,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>https://www.bnamericas.com/en/news/discovery-advances-permitting-financing-at-us606mn-cordero-in-mexico</t>
+          <t>[BNamericas](https://www.bnamericas.com/en/news/discovery-advances-permitting-financing-at-us606mn-cordero-in-mexico)</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -3926,7 +4001,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>https://resourceworld.com/tocvan-ventures-eyes-mexican-gold-pour-by-q4-2026/</t>
+          <t>[Resource World](https://resourceworld.com/tocvan-ventures-eyes-mexican-gold-pour-by-q4-2026/)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -3963,7 +4038,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>https://www.fresnilloplc.com/portfolio/exploration/orisyvo/</t>
+          <t>[Fresnillo plc](https://www.fresnilloplc.com/portfolio/exploration/orisyvo/)</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -4000,7 +4075,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/</t>
+          <t>[Mining.com](https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/)</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -4037,7 +4112,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/</t>
+          <t>[Mining.com](https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/)</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -4074,7 +4149,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/</t>
+          <t>[Mining.com](https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/)</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -4111,7 +4186,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>https://im-mining.com/2026/06/29/metso-to-supply-additional-crushing-package-for-grupo-mexico-la-caridad-copper-concentrator/</t>
+          <t>[IM Mining](https://im-mining.com/2026/06/29/metso-to-supply-additional-crushing-package-for-grupo-mexico-la-caridad-copper-concentrator/)</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -4148,7 +4223,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2026/05/21/3299182</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/05/21/3299182)</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -4185,7 +4260,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>https://mexicobusiness.news/mining/news/grupo-mexicos-asarco-may-reopen-united-states</t>
+          <t>[Mexico Business News](https://mexicobusiness.news/mining/news/grupo-mexicos-asarco-may-reopen-united-states)</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -4222,7 +4297,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>https://mineraalamos.com/our-assets/cerro-de-oro-project/</t>
+          <t>[Minera Alamos](https://mineraalamos.com/our-assets/cerro-de-oro-project/)</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -4259,7 +4334,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>https://www.globalminingreview.com/mining/11022025/antler-copper-project-achieves-critical-federal-permitting-milestone/</t>
+          <t>[Global Mining Review](https://www.globalminingreview.com/mining/11022025/antler-copper-project-achieves-critical-federal-permitting-milestone/)</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -4296,7 +4371,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>https://www.blm.gov/press-release/blm-approves-lisbon-valley-copper-mine-expansion-utah</t>
+          <t>[BLM](https://www.blm.gov/press-release/blm-approves-lisbon-valley-copper-mine-expansion-utah)</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -4333,7 +4408,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>https://investingnews.com/smackover-lithium-announces-the-award-of-last-key-construction-contract-for-the-south-west-arkansas-project-ahead-of-final-investment-decision/</t>
+          <t>[InvestingNews](https://investingnews.com/smackover-lithium-announces-the-award-of-last-key-construction-contract-for-the-south-west-arkansas-project-ahead-of-final-investment-decision/)</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -4370,7 +4445,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/0000831259/000083125926000033/a2q2026exhibit991.htm</t>
+          <t>[SEC/Freeport-McMoRan](https://www.sec.gov/Archives/edgar/data/0000831259/000083125926000033/a2q2026exhibit991.htm)</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -4407,7 +4482,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>https://niocorp.com/niocorp-launches-construction-of-elk-creek-critical-minerals-project-mine-portal/</t>
+          <t>[NioCorp](https://niocorp.com/niocorp-launches-construction-of-elk-creek-critical-minerals-project-mine-portal/)</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -4444,7 +4519,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>https://www.e-mj.com/breaking-news/centerra-advances-goldfield-project-in-nevada/</t>
+          <t>[E&amp;MJ](https://www.e-mj.com/breaking-news/centerra-advances-goldfield-project-in-nevada/)</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -4481,7 +4556,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2026/03/02/3247157/0/en/hudbay-to-acquire-arizona-sonoran-creating-the-third-largest-copper-district-in-north-america.html</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/03/02/3247157/0/en/hudbay-to-acquire-arizona-sonoran-creating-the-third-largest-copper-district-in-north-america.html)</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -4518,7 +4593,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>https://www.westernexploration.com/news-and-updates/news/news-details/2026/Western-Exploration-Outlines-2026-Program-to-Advance-Doby-George-Permitting-and-Expand-Gravel-Creek-Resources-2026-aaotfYHcV7/default.aspx</t>
+          <t>[Western Exploration](https://www.westernexploration.com/news-and-updates/news/news-details/2026/Western-Exploration-Outlines-2026-Program-to-Advance-Doby-George-Permitting-and-Expand-Gravel-Creek-Resources-2026-aaotfYHcV7/default.aspx)</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -4555,7 +4630,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>https://chesapeakegold.com/metates/</t>
+          <t>[Chesapeake Gold Corp.](https://chesapeakegold.com/metates/)</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -4567,72 +4642,146 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Libby Project (Cabinet Mountains)</t>
+          <t>Pathfinder Tonopah (cobre-molibdeno-plata)</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Condado de Lincoln, Montana, EE.UU.</t>
+          <t>Tonopah, Nevada, EE.UU.</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Hecla Mining Company</t>
+          <t>Pathfinder Minerals (Pathfinder Tonopah)</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Bowman (permisos ambientales, FEED, planta piloto)</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Permitting federal completado para exploración subterránea (extensión de ~1 milla del socavón Libby Adit; recurso potencial 1,500 millones lb de cobre y 183 millones oz de plata; pendiente permiso de descarga de agua de MT DEQ)</t>
+          <t>Permitting/FEED (avanzando hacia estudio de factibilidad definitivo; carta de interés no vinculante de EXIM Bank por US$896 millones para financiamiento, programa "Make More in America")</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>https://thewesternnews.com/news/2026/jul/24/libby-mining-project-takes-another-step-forward-with-federal-ok/</t>
+          <t>[Mining Technology](https://www.mining-technology.com/news/pathfinder-896m-loi-us-exim-copper-mine/)</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
+          <t>La Colorada Mine — Expansión Veta Madre/Veta Madre Plus</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Sonora, México</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Heliostar Metals</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Permisos completos obtenidos (2026); waste stripping programado 3T2026; producción de zona expandida esperada 1S2027</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>[Mexico Business News](https://mexicobusiness.news/mining/news/heliostar-advances-la-colorada-pit-permits-drill-data)</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Libby Project (Cabinet Mountains)</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Condado de Lincoln, Montana, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Hecla Mining Company</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Permitting federal completado para exploración subterránea (extensión de ~1 milla del socavón Libby Adit; recurso potencial 1,500 millones lb de cobre y 183 millones oz de plata; pendiente permiso de descarga de agua de MT DEQ)</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>[The Western News](https://thewesternnews.com/news/2026/jul/24/libby-mining-project-takes-another-step-forward-with-federal-ok/)</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
           <t>Donlin Gold</t>
         </is>
       </c>
-      <c r="B44" s="2" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>Alaska, EE.UU.</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr">
         <is>
           <t>NovaGold Corporation (adquiriendo 100%, compra de participación del 40% de Paulson Advisers)</t>
         </is>
       </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>No especificado</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr">
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
         <is>
           <t>Totalmente permisado / consolidación de propiedad (acuerdo de US$4.2 mil millones, cierre previsto 4T2026); aún sin decisión de construcción (FID)</t>
         </is>
       </c>
-      <c r="F44" s="2" t="inlineStr">
-        <is>
-          <t>https://www.miningnewsnorth.com/story/2026/07/24/news/donlin-gold-partners-form-new-novagold/9781.html</t>
-        </is>
-      </c>
-      <c r="G44" s="2" t="inlineStr">
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>[Mining News North](https://www.miningnewsnorth.com/story/2026/07/24/news/donlin-gold-partners-form-new-novagold/9781.html)</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
         <is>
           <t>2026-07-27</t>
         </is>
@@ -4649,16 +4798,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G59"/>
+  <dimension ref="A1:G61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4721,17 +4870,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Construcción</t>
+          <t>Construcción (rompimiento de tierra formal completado; 1,200 acres/10 edificios/1.4GW; VoltaGrid aprobado para operar 210 generadores de gas industrial, 700MW combinados, permitiendo operación fuera de la red pública; primera instalación en servicio 2S2026)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/vantage-breaks-ground-on-texas-gigawatt-data-center-campus-for-openai/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/vantage-breaks-ground-on-texas-gigawatt-data-center-campus-for-openai/); [Construction Owners](https://www.constructionowners.com/news/oracle-and-openai-to-power-new-texas-data-center-off-the-grid)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
@@ -4763,7 +4912,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>https://epoch.ai/publications/openai-stargate-where-the-us-sites-stand</t>
+          <t>[Epoch AI](https://epoch.ai/publications/openai-stargate-where-the-us-sites-stand)</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -4800,7 +4949,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/crusoe-tops-out-final-building-at-openai-stargate-data-center-campus-in-abilene-texas/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/crusoe-tops-out-final-building-at-openai-stargate-data-center-campus-in-abilene-texas/)</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -4837,7 +4986,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>https://www.cnbc.com/2026/06/22/chevron-cvx-microsoft-msft-natural-gas-data-center.html</t>
+          <t>[CNBC](https://www.cnbc.com/2026/06/22/chevron-cvx-microsoft-msft-natural-gas-data-center.html)</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -4874,7 +5023,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>https://www.gob.mx/presidencia/prensa/plan-mexico-avanza-se-anuncia-inversion-de-4-mil-800-mdd-de-cloudhq-para-la-construccion-de-6-centros-de-datos-en-queretaro</t>
+          <t>[Gobierno de México](https://www.gob.mx/presidencia/prensa/plan-mexico-avanza-se-anuncia-inversion-de-4-mil-800-mdd-de-cloudhq-para-la-construccion-de-6-centros-de-datos-en-queretaro)</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -4911,7 +5060,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>https://www.ucs.org/about/news/judge-orders-meta-explain-new-gas-demand-hyperscale-louisiana-data-center</t>
+          <t>[UCS](https://www.ucs.org/about/news/judge-orders-meta-explain-new-gas-demand-hyperscale-louisiana-data-center)</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -4948,7 +5097,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterfrontier.com/site-selection/article/55305086/nv1-and-the-nevada-hyperscale-boom-vantage-data-centers-bets-3b-on-the-ai-future</t>
+          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55305086/nv1-and-the-nevada-hyperscale-boom-vantage-data-centers-bets-3b-on-the-ai-future)</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -4985,7 +5134,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/cloudburst-breaks-ground-on-gigawatt-scale-data-center-campus-in-texas/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/cloudburst-breaks-ground-on-gigawatt-scale-data-center-campus-in-texas/)</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -5002,7 +5151,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Kaufman County, Texas, EE.UU.</t>
+          <t>Entre Talty y Post Oak Bend City, Kaufman County, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -5017,17 +5166,17 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/construcción temprana</t>
+          <t>Ingeniería/construcción temprana (campus de 200MW/4 edificios; estrategia behind-the-meter con motores de gas Jenbacher J620 + almacenamiento en baterías de Engie; primera instalación 2026, fases hasta 2028)</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/prometheus-hyperscale-details-plans-for-dallas-data-center-campus/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/prometheus-hyperscale-details-plans-for-dallas-data-center-campus/)</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
@@ -5059,7 +5208,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>https://www.businesswire.com/news/home/20260126236053/en/Pacifico-Energy-Secures-7.65-GW-Power-Generation-Permit-for-GW-Ranch-Project</t>
+          <t>[Business Wire](https://www.businesswire.com/news/home/20260126236053/en/Pacifico-Energy-Secures-7.65-GW-Power-Generation-Permit-for-GW-Ranch-Project)</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -5096,7 +5245,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/amazon-looks-to-build-large-scale-data-center-campus-next-to-nuclear-plant-in-texas/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/amazon-looks-to-build-large-scale-data-center-campus-next-to-nuclear-plant-in-texas/)</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -5128,17 +5277,17 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Permisos/negociación avanzada (construcción inminente)</t>
+          <t>Permisos/negociación avanzada (inversión total US$3.7 mil millones: US$2.7B centro de datos + US$1B planta de fertilizantes Fermachem; gasoducto de 160km desde Texas; planta de ciclo combinado on-site de 350MW para alimentar data center de 250MW; Congreso de Durango aprobó donación de 50 hectáreas)</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>https://mexiconewsdaily.com/business/durango-data-center-fertilizer-plant-investment-fermaca/</t>
+          <t>[Mexico News Daily](https://mexiconewsdaily.com/business/durango-data-center-fertilizer-plant-investment-fermaca/); [DCD](https://www.datacenterdynamics.com/en/news/250mw-natural-gas-powered-data-center-campus-announced-in-durango-mexico/)</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
@@ -5170,7 +5319,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/circe-energy-secures-2gw-of-natural-gas-capacity-for-west-texas-data-center-campus/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/circe-energy-secures-2gw-of-natural-gas-capacity-for-west-texas-data-center-campus/)</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -5207,7 +5356,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>https://sourcenm.com/2026/07/16/new-mexico-land-commissioner-blocks-project-jupiter-related-pipeline-from-building-on-state-land/</t>
+          <t>[Source NM](https://sourcenm.com/2026/07/16/new-mexico-land-commissioner-blocks-project-jupiter-related-pipeline-from-building-on-state-land/)</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -5244,7 +5393,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/powerplay-ai-announces-400-mw-behind-the-meter-ai-data-center-development-in-greater-abilene-with-nasdaq-listed-neocloud-joint-venture-partner-302829610.html</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/powerplay-ai-announces-400-mw-behind-the-meter-ai-data-center-development-in-greater-abilene-with-nasdaq-listed-neocloud-joint-venture-partner-302829610.html)</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -5281,7 +5430,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/liberty-energy-powerbridge-form-jv-to-power-planned-2gw-data-center-in-west-texas/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/liberty-energy-powerbridge-form-jv-to-power-planned-2gw-data-center-in-west-texas/)</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -5318,7 +5467,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>https://www.powermag.com/nuclear-natural-gas-power-generation-planned-for-massive-new-mexico-data-center-site/</t>
+          <t>[PowerMag](https://www.powermag.com/nuclear-natural-gas-power-generation-planned-for-massive-new-mexico-data-center-site/)</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -5355,7 +5504,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterfrontier.com/site-selection/article/55289667/powering-ai-in-the-permian-texas-critical-data-centers-sustainable-energy-play</t>
+          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55289667/powering-ai-in-the-permian-texas-critical-data-centers-sustainable-energy-play)</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -5392,7 +5541,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>https://openai.com/index/five-new-stargate-sites/</t>
+          <t>[OpenAI](https://openai.com/index/five-new-stargate-sites/)</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -5429,7 +5578,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>https://openai.com/index/five-new-stargate-sites/</t>
+          <t>[OpenAI](https://openai.com/index/five-new-stargate-sites/)</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -5466,7 +5615,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>https://mexiconewsdaily.com/business/aws-invest-5b-mexico-data-region/</t>
+          <t>[Mexico News Daily](https://mexiconewsdaily.com/business/aws-invest-5b-mexico-data-region/)</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -5503,7 +5652,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/oracle-and-openai-start-construction-on-stargate-data-center-campus-in-saline-township-michigan/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/oracle-and-openai-start-construction-on-stargate-data-center-campus-in-saline-township-michigan/)</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -5540,7 +5689,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>https://www.valleynewslive.com/2026/07/13/applied-digital-expands-north-dakota-eyes-oliver-county-third-data-center/</t>
+          <t>[Valley News Live](https://www.valleynewslive.com/2026/07/13/applied-digital-expands-north-dakota-eyes-oliver-county-third-data-center/)</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -5577,7 +5726,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>https://energymagazine.mx/2026/01/el-data-center-verde-que-encendio-la-polemica-asi-sera-el-proyecto-de-ia-en-nuevo-leon-que-usara-tecnologia-de-nvidia/</t>
+          <t>[Energy Magazine MX](https://energymagazine.mx/2026/01/el-data-center-verde-que-encendio-la-polemica-asi-sera-el-proyecto-de-ia-en-nuevo-leon-que-usara-tecnologia-de-nvidia/)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -5614,7 +5763,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>https://www.constructiondive.com/news/data-center-cleanarc-breaks-ground-virginia-campus/806489/</t>
+          <t>[Construction Dive](https://www.constructiondive.com/news/data-center-cleanarc-breaks-ground-virginia-campus/806489/)</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -5651,7 +5800,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>https://www.ksl.com/article/51402125/groundbreaking-for-new-millard-county-artificial-intelligence-data-center</t>
+          <t>[KSL](https://www.ksl.com/article/51402125/groundbreaking-for-new-millard-county-artificial-intelligence-data-center)</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -5688,7 +5837,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>https://governor.mo.gov/press-releases/archive/amazon-investing-10-billion-montgomery-county</t>
+          <t>[Governor.mo.gov](https://governor.mo.gov/press-releases/archive/amazon-investing-10-billion-montgomery-county)</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -5725,7 +5874,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>https://www.stlpr.org/government-politics-issues/2026-05-21/missouri-governor-google-announce-15-billion-data-center-montgomery-county</t>
+          <t>[STLPR](https://www.stlpr.org/government-politics-issues/2026-05-21/missouri-governor-google-announce-15-billion-data-center-montgomery-county)</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -5762,7 +5911,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>https://www.globenewswire.com/news-release/2026/07/06/3322404/0/en/big-digital-energy-announces-partnership-with-10netzero-to-acquire-power-ready-hood-county-texas-site-for-ai-datacenter-development.html</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/06/3322404/0/en/big-digital-energy-announces-partnership-with-10netzero-to-acquire-power-ready-hood-county-texas-site-for-ai-datacenter-development.html)</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -5799,7 +5948,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/)</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -5836,7 +5985,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/meta-files-to-expand-campus-in-el-paso-texas-with-12-new-buildings/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/meta-files-to-expand-campus-in-el-paso-texas-with-12-new-buildings/)</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -5868,17 +6017,17 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Planeación/desarrollo temprano</t>
+          <t>Planeación avanzada (SB Energy construirá 9.2GW de generación a gas natural, financiamiento de US$33.3 mil millones por SoftBank, más US$4.2 mil millones en transmisión; 26-jul-2026 trascendió que Nvidia negocia garantía financiera de hasta US$250 mil millones para que OpenAI arriende el sitio, primera fase de 800MW en 2028)</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/softbank-eyes-10gw-data-center-at-former-doe-nuclear-enrichment-site-in-ohio/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/softbank-eyes-10gw-data-center-at-former-doe-nuclear-enrichment-site-in-ohio/); [Bloomberg](https://www.bloomberg.com/news/articles/2026-07-26/nvidia-in-talks-on-250-billion-backing-for-openai-hub-wsj-says)</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
@@ -5910,7 +6059,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/)</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -5947,7 +6096,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>https://www.williams.com/2026/07/13/williams-announces-5-34-billion-investment-in-power-innovation-joint-venture-from-blackstone/</t>
+          <t>[Williams Companies](https://www.williams.com/2026/07/13/williams-announces-5-34-billion-investment-in-power-innovation-joint-venture-from-blackstone/)</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -5984,7 +6133,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/cleancore-solutions-zone-announces-closing-of-first-data-center-project-establishing-its-critical-infrastructure-buildout-for-the-ai-economy-302821421.html</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/cleancore-solutions-zone-announces-closing-of-first-data-center-project-establishing-its-critical-infrastructure-buildout-for-the-ai-economy-302821421.html)</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -6021,7 +6170,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>https://www.bloomberg.com/news/articles/2026-06-09/crusoe-touts-5-gigawatts-worth-of-data-centers-deals-pauses-wyoming-site</t>
+          <t>[Bloomberg](https://www.bloomberg.com/news/articles/2026-06-09/crusoe-touts-5-gigawatts-worth-of-data-centers-deals-pauses-wyoming-site)</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -6058,7 +6207,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>https://www.hpcwire.com/off-the-wire/core-scientific-plans-expansion-to-1-5gw-of-gross-power-at-pecos-texas-campus/</t>
+          <t>[HPCwire](https://www.hpcwire.com/off-the-wire/core-scientific-plans-expansion-to-1-5gw-of-gross-power-at-pecos-texas-campus/)</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -6095,7 +6244,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>https://utahnewsdispatch.com/2026/05/19/renderings-show-massive-data-center-box-elder-utah-permits-could-take-years/</t>
+          <t>[Utah News Dispatch](https://utahnewsdispatch.com/2026/05/19/renderings-show-massive-data-center-box-elder-utah-permits-could-take-years/)</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -6132,7 +6281,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>https://www.stocktitan.net/news/FRMI/fermi-announces-first-siemens-turbines-arrive-at-port-of-qg7ienp885jk.html</t>
+          <t>[StockTitan](https://www.stocktitan.net/news/FRMI/fermi-announces-first-siemens-turbines-arrive-at-port-of-qg7ienp885jk.html)</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -6169,7 +6318,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>https://www.kltv.com/2026/03/20/president-trump-approves-16-billion-natural-gas-generator-be-installed-anderson-county/</t>
+          <t>[KLTV](https://www.kltv.com/2026/03/20/president-trump-approves-16-billion-natural-gas-generator-be-installed-anderson-county/)</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -6206,7 +6355,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>https://wvmetronews.com/2026/07/16/mon-power-president-says-data-centers-will-end-up-paying-for-natural-gas-powered-power-plant/</t>
+          <t>[WV MetroNews](https://wvmetronews.com/2026/07/16/mon-power-president-says-data-centers-will-end-up-paying-for-natural-gas-powered-power-plant/)</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -6243,7 +6392,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>https://www.utilitydive.com/news/iep-plans-944-mw-behind-the-meter-gas-plant-in-pennsylvania-to-power-data-c/758830/</t>
+          <t>[Utility Dive](https://www.utilitydive.com/news/iep-plans-944-mw-behind-the-meter-gas-plant-in-pennsylvania-to-power-data-c/758830/)</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -6280,7 +6429,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/aws-files-for-12bn-data-center-campus-outside-houston-texas/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/aws-files-for-12bn-data-center-campus-outside-houston-texas/)</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -6317,7 +6466,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>https://www.crusoe.ai/resources/newsroom/crusoe-and-lancium-announce-1-gigawatt-ai-data-center-campus-in-childress-texas</t>
+          <t>[Crusoe](https://www.crusoe.ai/resources/newsroom/crusoe-and-lancium-announce-1-gigawatt-ai-data-center-campus-in-childress-texas)</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -6354,7 +6503,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/)</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -6391,7 +6540,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>https://www.powermag.com/new-200-mw-gas-fired-plant-in-ohio-will-power-meta-data-center/</t>
+          <t>[PowerMag](https://www.powermag.com/new-200-mw-gas-fired-plant-in-ohio-will-power-meta-data-center/)</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -6428,7 +6577,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>https://www.aterio.io/blog/crusoe-launches-usd29b-goodnight-campus-in-claude-mirroring-openai-s-stargate</t>
+          <t>[Aterio](https://www.aterio.io/blog/crusoe-launches-usd29b-goodnight-campus-in-claude-mirroring-openai-s-stargate)</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -6465,7 +6614,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>https://www.ajc.com/business/2026/07/officials-order-georgia-data-centers-pop-up-power-plant-to-halt-construction/</t>
+          <t>[AJC](https://www.ajc.com/business/2026/07/officials-order-georgia-data-centers-pop-up-power-plant-to-halt-construction/)</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -6502,7 +6651,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/stark-power-lands-56gw-data-center-development-portfolio-in-sagebrush-acquisition/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/stark-power-lands-56gw-data-center-development-portfolio-in-sagebrush-acquisition/)</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -6539,7 +6688,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterfrontier.com/site-selection/article/55281341/pennsylvanias-homer-city-energy-campus-a-brownfield-transformed-for-data-center-innovation</t>
+          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55281341/pennsylvanias-homer-city-energy-campus-a-brownfield-transformed-for-data-center-innovation)</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -6576,7 +6725,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterknowledge.com/data-center-site-selection/nebius-plans-300-mw-data-center-in-new-jersey-amid-us-expansion</t>
+          <t>[Data Center Knowledge](https://www.datacenterknowledge.com/data-center-site-selection/nebius-plans-300-mw-data-center-in-new-jersey-amid-us-expansion)</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -6613,7 +6762,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/terravolt-inks-natural-gas-supply-deal-for-onsite-power-plant-at-planned-data-center-campus-in-idaho/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/terravolt-inks-natural-gas-supply-deal-for-onsite-power-plant-at-planned-data-center-campus-in-idaho/)</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -6650,7 +6799,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/cyrusone-announces-sixth-data-center-campus-in-san-antonio-texas/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/cyrusone-announces-sixth-data-center-campus-in-san-antonio-texas/)</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -6662,7 +6811,7 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>EdgeConneX PowerConneX New Albany Energy Center (I y II)</t>
+          <t>EdgeConneX PowerConneX New Albany Energy Center (I, II y III)</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -6682,17 +6831,17 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Construcción (PowerConneX I, 120MW, certificado OPSB 22-jul-2025, construcción iniciada sep-2025, operación comercial posible 3T2026; PowerConneX II, 216MW, solicitado ante OPSB, operación comercial objetivo 2T2027)</t>
+          <t>Construcción (PowerConneX I, 120MW, certificado OPSB 22-jul-2025, construcción iniciada sep-2025, operación comercial posible 3T2026; PowerConneX II, 216MW, solicitado ante OPSB, operación comercial objetivo 2T2027; PowerConneX III, 430MW, notificación previa ante OPSB abr-2026, elevando capacidad total del sitio a ~766MW de gas)</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/edgeconnex-plans-120mw-gas-plant-to-power-ohio-data-center/</t>
+          <t>[Data Center Dynamics](https://www.datacenterdynamics.com/en/news/edgeconnex-plans-120mw-gas-plant-to-power-ohio-data-center/); [BeBeez](https://bebeez.eu/2026/04/14/edgeconnex-affiliate-proposes-430mw-natural-gas-plant-to-power-data-center-campus-in-new-albany-ohio/)</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
@@ -6724,7 +6873,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>https://www.technology.org/2026/07/15/xai-59-unpermitted-gas-turbines-southaven-colossus-2/</t>
+          <t>[Technology.org](https://www.technology.org/2026/07/15/xai-59-unpermitted-gas-turbines-southaven-colossus-2/)</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -6761,7 +6910,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/cleco-to-construct-756mw-natural-gas-plant-to-serve-applied-digitals-data-center-in-rapides-parish-louisiana-report/</t>
+          <t>[Data Center Dynamics](https://www.datacenterdynamics.com/en/news/cleco-to-construct-756mw-natural-gas-plant-to-serve-applied-digitals-data-center-in-rapides-parish-louisiana-report/)</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -6798,7 +6947,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>https://kentuckylantern.com/2026/07/22/developer-proposes-hyperscale-data-center-at-the-site-at-former-eastern-kentucky-steel-mill/</t>
+          <t>[Kentucky Lantern](https://kentuckylantern.com/2026/07/22/developer-proposes-hyperscale-data-center-at-the-site-at-former-eastern-kentucky-steel-mill/)</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -6835,12 +6984,86 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>https://www.datacenterdynamics.com/en/news/qts-to-build-11-data-centers-on-lancium-campus-in-hall-county-texas/</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/qts-to-build-11-data-centers-on-lancium-campus-in-hall-county-texas/)</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
           <t>2026-07-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Anthropic/Nexus Hubbard Campus</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Hubbard, Condado de Hill, Texas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Anthropic (operado por Nexus Data Centers; respaldo financiero de Google)</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>Construcción iniciada (primera fase 500-612MW prevista 2026, ampliable a ~7.2-7.7GW; planta de gas natural behind-the-meter cerca de gasoducto principal)</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/600mw-natural-gas-powered-data-center-campus-proposed-in-hubbard-texas/); [Construction Review](https://constructionreviewonline.com/5bn-anthropic-data-center-in-texas-receives-critical-financial-backing-from-google/)</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>Stillwater Technology Park</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>Lovejoy, Condado de Clayton, Georgia, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>Stillwater Development, LLC (cliente hyperscaler final no revelado)</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>Permisos ("development of regional impact" presentado ante el estado; hasta 15 edificios, 1.25GW, US$13 mil millones; generación de energía aún no confirmada, contempla interconexión con Central Georgia EMC)</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/gigawatt-scale-data-center-campus-planned-outside-atlanta-georgia/)</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Agregar 7 proyectos nuevos (2026-08-03)
Petroquímica (2): Enterprise Products Plant 12/Athena 2, Targa Roadrunner III/Copperhead II
LNG (1): Gasoducto Trident (Kinder Morgan, alimenta Golden Pass LNG)
Mining (2): Black Butte Copper Project, Planta de Litio Red River (US Army)
Data Centers (2): Savannah River Site AI Data Center, Pacifico Cedar Creek Power Campus

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014rEZC87YNCrJEYf5DoXH7Q
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -416,14 +416,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
-    <col width="35" customWidth="1" min="3" max="3"/>
-    <col width="35" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
@@ -1868,6 +1868,80 @@
       <c r="G39" t="inlineStr">
         <is>
           <t>2026-07-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Enterprise Products — Plant 12 (Delaware Basin) y Athena 2 (Midland Basin)</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Cuenca Delaware y Cuenca Midland, Texas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Enterprise Products Partners L.P.</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Enterprise Products (propietario-constructor)</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Construcción (sancionadas, divulgadas en resultados 2T2026 el 30-jul-2026; Plant 12 Delaware Basin ~300 MMcf/d en servicio 4T2027; Athena 2 Midland Basin en servicio 3T2027)</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>[Enterprise Reports Second Quarter 2026 Earnings](https://ir.enterpriseproducts.com/news-releases/news-release-details/enterprise-reports-second-quarter-2026-earnings)</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Targa Resources Roadrunner III / Copperhead II (plantas de gas)</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Cuenca Delaware (Permian), Texas/Nuevo México, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Targa Resources Corp.</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Targa Resources (propietario-constructor)</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Construcción (aprobadas may-2026; Roadrunner III 265 MMcf/d, Copperhead II 275 MMcf/d; en servicio previsto 1T2028)</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>[PGJ](https://pgjonline.com/news/2026/may/targa-expands-permian-gas-processing-delaware-express-pipeline-capacity)</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
         </is>
       </c>
     </row>
@@ -1882,14 +1956,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
-    <col width="35" customWidth="1" min="3" max="3"/>
-    <col width="35" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
@@ -3297,6 +3371,43 @@
       <c r="G38" t="inlineStr">
         <is>
           <t>2026-07-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Gasoducto Trident (alimenta Golden Pass LNG)</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Katy a Port Arthur, Texas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Kinder Morgan, Inc.</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Construcción (tendido/soldadura de tubería en curso en Waller County; ~216-220 millas, 42"/48", US$1.7-1.8 mil millones; en servicio Fase 1 previsto 1T2027)</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>[Storage Terminals Magazine](https://storageterminalsmag.com/kinder-morgans-trident-pipeline-project-enters-active-construction-phase-in-southeast-texas/); [Natural Gas Intel](https://www.naturalgasintel.com/news/kinder-morgan-greenlights-7b-in-natural-gas-pipeline-projects-amid-regulatory-speedup/)</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
         </is>
       </c>
     </row>
@@ -3311,14 +3422,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
-    <col width="35" customWidth="1" min="3" max="3"/>
-    <col width="35" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
@@ -5170,6 +5281,80 @@
       <c r="G50" t="inlineStr">
         <is>
           <t>2026-07-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Black Butte Copper Project</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Meagher County, Montana, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Sandfire Resources America Inc. (Sandfire Resources)</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Por definir (PFS elaborado por DM Consulting)</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Feasibility (PFS actualizado presentado 28-jul-2026 con nuevas reservas Lowry, vida de mina de 12 años; mina subterránea de cobre de alta ley)</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/29/3334925/0/en/sandfire-resources-america-files-black-butte-copper-project-preliminary-feasibility-study.html)</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Planta de Procesamiento de Litio Red River (US Army)</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Bowie County, Texas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Pentágono / Departamento del Ejército de EE.UU.</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>EnergyX (desarrollador-operador)</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Acuerdo de arrendamiento condicional otorgado (confirmado 25-jun-2026; 5to sitio del programa de minerales críticos en bases del Ejército, junto con Tooele, Pine Bluff/Anniston; construcción prevista desde 2027)</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>[Texarkana Gazette](https://www.texarkanagazette.com/news/2026/jun/30/army-awards-lithium-company-energyx-conditional/)</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
         </is>
       </c>
     </row>
@@ -5184,14 +5369,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G68"/>
+  <dimension ref="A1:G70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
-    <col width="35" customWidth="1" min="3" max="3"/>
-    <col width="35" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
@@ -7712,6 +7897,80 @@
         </is>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Savannah River Site AI Data Center &amp; Energy Campus</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Aiken, Carolina del Sur, EE.UU. (sitio federal DOE/NNSA)</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>DOE/NNSA (sitio federal)</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Amentum (desarrollador seleccionado) / DC BLOX (socio de infraestructura)</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Negociación de arrendamiento por fases (seleccionado ~20-23 jul-2026; campus de ~1GW con ~2GW de generación dedicada in-situ, iniciando con gas natural como puente hacia energía nuclear futura)</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/doe-selects-amentum-dc-blox-to-develop-behind-the-meter-ai-data-center-at-savannah-river-site-in-south-carolina/); [Energy.gov](https://www.energy.gov/nnsa/articles/nnsa-selects-amentum-ai-data-center-and-energy-project-savannah-river-site)</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Pacifico Cedar Creek Power Campus</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Cedar Creek, Bastrop County, Texas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Pacifico Energy (Pacifico Cedar Creek LLC); inquilino de centro de datos aún no revelado</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Permisos/incentivos en revisión (solicitud de incentivos ante el Contralor de Texas presentada 24-jun-2026; campus de 2,842 acres; planta de gas natural on-site de 710MW para servir ~490MW de carga de centro de datos, esquema behind-the-meter)</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>[Community Impact](https://communityimpact.com/bastrop-cedar-creek/business/new-22b-cedar-creek-data-center-project-abatements-under-review/)</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Agregar 7 proyectos nuevos y actualizar Excel (2026-08-03) (#14)
Petroquímica (2): Enterprise Products Plant 12/Athena 2, Targa Roadrunner III/Copperhead II
LNG (1): Gasoducto Trident (Kinder Morgan, alimenta Golden Pass LNG)
Mining (2): Black Butte Copper Project, Planta de Litio Red River (US Army)
Data Centers (2): Savannah River Site AI Data Center, Pacifico Cedar Creek Power Campus


Claude-Session: https://claude.ai/code/session_014rEZC87YNCrJEYf5DoXH7Q

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -416,14 +416,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
-    <col width="35" customWidth="1" min="3" max="3"/>
-    <col width="35" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
@@ -1868,6 +1868,80 @@
       <c r="G39" t="inlineStr">
         <is>
           <t>2026-07-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Enterprise Products — Plant 12 (Delaware Basin) y Athena 2 (Midland Basin)</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Cuenca Delaware y Cuenca Midland, Texas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Enterprise Products Partners L.P.</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Enterprise Products (propietario-constructor)</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Construcción (sancionadas, divulgadas en resultados 2T2026 el 30-jul-2026; Plant 12 Delaware Basin ~300 MMcf/d en servicio 4T2027; Athena 2 Midland Basin en servicio 3T2027)</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>[Enterprise Reports Second Quarter 2026 Earnings](https://ir.enterpriseproducts.com/news-releases/news-release-details/enterprise-reports-second-quarter-2026-earnings)</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Targa Resources Roadrunner III / Copperhead II (plantas de gas)</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Cuenca Delaware (Permian), Texas/Nuevo México, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Targa Resources Corp.</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Targa Resources (propietario-constructor)</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Construcción (aprobadas may-2026; Roadrunner III 265 MMcf/d, Copperhead II 275 MMcf/d; en servicio previsto 1T2028)</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>[PGJ](https://pgjonline.com/news/2026/may/targa-expands-permian-gas-processing-delaware-express-pipeline-capacity)</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
         </is>
       </c>
     </row>
@@ -1882,14 +1956,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
-    <col width="35" customWidth="1" min="3" max="3"/>
-    <col width="35" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
@@ -3297,6 +3371,43 @@
       <c r="G38" t="inlineStr">
         <is>
           <t>2026-07-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Gasoducto Trident (alimenta Golden Pass LNG)</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Katy a Port Arthur, Texas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Kinder Morgan, Inc.</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Construcción (tendido/soldadura de tubería en curso en Waller County; ~216-220 millas, 42"/48", US$1.7-1.8 mil millones; en servicio Fase 1 previsto 1T2027)</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>[Storage Terminals Magazine](https://storageterminalsmag.com/kinder-morgans-trident-pipeline-project-enters-active-construction-phase-in-southeast-texas/); [Natural Gas Intel](https://www.naturalgasintel.com/news/kinder-morgan-greenlights-7b-in-natural-gas-pipeline-projects-amid-regulatory-speedup/)</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
         </is>
       </c>
     </row>
@@ -3311,14 +3422,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
-    <col width="35" customWidth="1" min="3" max="3"/>
-    <col width="35" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
@@ -5170,6 +5281,80 @@
       <c r="G50" t="inlineStr">
         <is>
           <t>2026-07-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Black Butte Copper Project</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Meagher County, Montana, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Sandfire Resources America Inc. (Sandfire Resources)</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Por definir (PFS elaborado por DM Consulting)</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Feasibility (PFS actualizado presentado 28-jul-2026 con nuevas reservas Lowry, vida de mina de 12 años; mina subterránea de cobre de alta ley)</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/29/3334925/0/en/sandfire-resources-america-files-black-butte-copper-project-preliminary-feasibility-study.html)</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Planta de Procesamiento de Litio Red River (US Army)</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Bowie County, Texas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Pentágono / Departamento del Ejército de EE.UU.</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>EnergyX (desarrollador-operador)</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Acuerdo de arrendamiento condicional otorgado (confirmado 25-jun-2026; 5to sitio del programa de minerales críticos en bases del Ejército, junto con Tooele, Pine Bluff/Anniston; construcción prevista desde 2027)</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>[Texarkana Gazette](https://www.texarkanagazette.com/news/2026/jun/30/army-awards-lithium-company-energyx-conditional/)</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
         </is>
       </c>
     </row>
@@ -5184,14 +5369,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G68"/>
+  <dimension ref="A1:G70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
-    <col width="35" customWidth="1" min="3" max="3"/>
-    <col width="35" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
@@ -7712,6 +7897,80 @@
         </is>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Savannah River Site AI Data Center &amp; Energy Campus</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Aiken, Carolina del Sur, EE.UU. (sitio federal DOE/NNSA)</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>DOE/NNSA (sitio federal)</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Amentum (desarrollador seleccionado) / DC BLOX (socio de infraestructura)</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Negociación de arrendamiento por fases (seleccionado ~20-23 jul-2026; campus de ~1GW con ~2GW de generación dedicada in-situ, iniciando con gas natural como puente hacia energía nuclear futura)</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/doe-selects-amentum-dc-blox-to-develop-behind-the-meter-ai-data-center-at-savannah-river-site-in-south-carolina/); [Energy.gov](https://www.energy.gov/nnsa/articles/nnsa-selects-amentum-ai-data-center-and-energy-project-savannah-river-site)</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Pacifico Cedar Creek Power Campus</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Cedar Creek, Bastrop County, Texas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Pacifico Energy (Pacifico Cedar Creek LLC); inquilino de centro de datos aún no revelado</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Permisos/incentivos en revisión (solicitud de incentivos ante el Contralor de Texas presentada 24-jun-2026; campus de 2,842 acres; planta de gas natural on-site de 710MW para servir ~490MW de carga de centro de datos, esquema behind-the-meter)</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>[Community Impact](https://communityimpact.com/bastrop-cedar-creek/business/new-22b-cedar-creek-data-center-project-abatements-under-review/)</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Agregar 4 proyectos nuevos y actualizar Excel (2026-08-04)
- Petroquímica: Southern Energy Renewables (metanol/SAF, St. Charles Parish, LA)
- Mining: Camino Rojo proyecto subterráneo (Orla Mining, Zacatecas) y Cerro Caliche Gold Project (Sonoro Gold, Sonora)
- Data Centers: Bosque County Data Center Campus (ECP/KKR/CyrusOne/Calpine, Texas)

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DQUm6RR9hLaH9erYPCQsfu
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -20,10 +20,18 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
@@ -49,8 +57,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -416,50 +425,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -1942,6 +1951,43 @@
       <c r="G41" t="inlineStr">
         <is>
           <t>2026-08-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Southern Energy Renewables — Complejo de Metanol y SAF</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>St. Charles Parish (Killona), Luisiana, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Southern Energy Renewables</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Planeación/pre-construcción (inversión US$1,400 millones; convierte biomasa de desecho de madera en metanol verde y combustible de aviación sostenible; construcción prevista a iniciar fines de 2027, producción prevista fines de 2029)</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>[Hydrocarbon Processing](https://www.hydrocarbonprocessing.com/news/2026/03/southern-energy-renewables-announce-14-b-methanol-and-saf-complex-in-louisiana/); [Louisiana Economic Development](https://www.opportunitylouisiana.gov/news/southern-energy-renewables-announce-1-4-billion-methanol-and-sustainable-aviation-fuel-facility-in-st-charles-parish)</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
         </is>
       </c>
     </row>
@@ -1959,47 +2005,47 @@
   <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -3422,50 +3468,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -5355,6 +5401,80 @@
       <c r="G52" t="inlineStr">
         <is>
           <t>2026-08-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Camino Rojo — Proyecto Subterráneo (extensión)</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Zacatecas, México</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Orla Mining Ltd.</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Permisos completos/inicio de desarrollo subterráneo (SEMARNAT aprobó MIA 18-mar-2026, habilitando minado del resto del tajo de óxidos y construcción de rampa de exploración subterránea; inicio de obras de acceso subterráneo previsto 2S2026; PEA de proyecto subterráneo indica VPN de US$1,300 millones)</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>[Mining.com](https://www.mining.com/orla-secures-final-permit-to-advance-underground-mining-at-camino-rojo/); [Orla Mining](https://orlamining.com/news/orla-mining-receives-permits-to-extend-operations-in-mexico-supporting-companys-long-term-commitment-to-camino-rojo/)</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Cerro Caliche Gold Project</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Sonora, México</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Sonoro Gold Corp.</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>EPC por definir (en negociación con múltiples empresas EPC de China)</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Permisos/estructuración de financiamiento EPC (plataforma consolidada de 3,924 hectáreas en 25 concesiones; finalización de permisos esperada 1T2026; 4 empresas EPC chinas evaluando financiamiento de deuda y desarrollo)</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>[Sonoro Gold Corp.](https://sonorogold.com/wp-content/uploads/2026/03/2026.03.01_Sonoro-Gold-Corporate-Presentation.pdf); [Mexico Mining Center](https://www.mexicominingcenter.com/sonoro-continues-discussions-with-china-based-epc-companies-and-potential-equity-investors/)</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
         </is>
       </c>
     </row>
@@ -5369,50 +5489,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G70"/>
+  <dimension ref="A1:G71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -7968,6 +8088,43 @@
       <c r="G70" t="inlineStr">
         <is>
           <t>2026-08-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Bosque County Data Center Campus</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Condado de Bosque, Texas, EE.UU. (~30 millas al sur de Dallas-Fort Worth)</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Energy Capital Partners (ECP) / KKR (asociación estratégica de US$50 mil millones)</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>CyrusOne (JV de construcción/operación); Calpine Corp. (suministro de energía dedicada desde Thad Hill Energy Center)</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Construcción (primera inversión de la asociación estratégica ECP-KKR; campus de ~700,000 pies², inversión total cercana a US$4,000 millones, capacidad inicial de TI de 144MW sobre 190MW total; operación prevista 4T2026)</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>[Data Centre Magazine](https://datacentremagazine.com/news/ecp-and-kkr-to-build-4bn-190mw-hyperscale-data-centre); [Connect CRE](https://www.connectcre.com/stories/energy-capital-kkr-joint-forces-on-bosque-county-data-center/)</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Agregar 4 proyectos nuevos y actualizar Excel (2026-08-04) (#15)
- Petroquímica: Southern Energy Renewables (metanol/SAF, St. Charles Parish, LA)
- Mining: Camino Rojo proyecto subterráneo (Orla Mining, Zacatecas) y Cerro Caliche Gold Project (Sonoro Gold, Sonora)
- Data Centers: Bosque County Data Center Campus (ECP/KKR/CyrusOne/Calpine, Texas)


Claude-Session: https://claude.ai/code/session_01DQUm6RR9hLaH9erYPCQsfu

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -20,10 +20,18 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
@@ -49,8 +57,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -416,50 +425,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -1942,6 +1951,43 @@
       <c r="G41" t="inlineStr">
         <is>
           <t>2026-08-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Southern Energy Renewables — Complejo de Metanol y SAF</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>St. Charles Parish (Killona), Luisiana, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Southern Energy Renewables</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Planeación/pre-construcción (inversión US$1,400 millones; convierte biomasa de desecho de madera en metanol verde y combustible de aviación sostenible; construcción prevista a iniciar fines de 2027, producción prevista fines de 2029)</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>[Hydrocarbon Processing](https://www.hydrocarbonprocessing.com/news/2026/03/southern-energy-renewables-announce-14-b-methanol-and-saf-complex-in-louisiana/); [Louisiana Economic Development](https://www.opportunitylouisiana.gov/news/southern-energy-renewables-announce-1-4-billion-methanol-and-sustainable-aviation-fuel-facility-in-st-charles-parish)</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
         </is>
       </c>
     </row>
@@ -1959,47 +2005,47 @@
   <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -3422,50 +3468,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -5355,6 +5401,80 @@
       <c r="G52" t="inlineStr">
         <is>
           <t>2026-08-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Camino Rojo — Proyecto Subterráneo (extensión)</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Zacatecas, México</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Orla Mining Ltd.</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Permisos completos/inicio de desarrollo subterráneo (SEMARNAT aprobó MIA 18-mar-2026, habilitando minado del resto del tajo de óxidos y construcción de rampa de exploración subterránea; inicio de obras de acceso subterráneo previsto 2S2026; PEA de proyecto subterráneo indica VPN de US$1,300 millones)</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>[Mining.com](https://www.mining.com/orla-secures-final-permit-to-advance-underground-mining-at-camino-rojo/); [Orla Mining](https://orlamining.com/news/orla-mining-receives-permits-to-extend-operations-in-mexico-supporting-companys-long-term-commitment-to-camino-rojo/)</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Cerro Caliche Gold Project</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Sonora, México</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Sonoro Gold Corp.</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>EPC por definir (en negociación con múltiples empresas EPC de China)</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Permisos/estructuración de financiamiento EPC (plataforma consolidada de 3,924 hectáreas en 25 concesiones; finalización de permisos esperada 1T2026; 4 empresas EPC chinas evaluando financiamiento de deuda y desarrollo)</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>[Sonoro Gold Corp.](https://sonorogold.com/wp-content/uploads/2026/03/2026.03.01_Sonoro-Gold-Corporate-Presentation.pdf); [Mexico Mining Center](https://www.mexicominingcenter.com/sonoro-continues-discussions-with-china-based-epc-companies-and-potential-equity-investors/)</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
         </is>
       </c>
     </row>
@@ -5369,50 +5489,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G70"/>
+  <dimension ref="A1:G71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -7968,6 +8088,43 @@
       <c r="G70" t="inlineStr">
         <is>
           <t>2026-08-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Bosque County Data Center Campus</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Condado de Bosque, Texas, EE.UU. (~30 millas al sur de Dallas-Fort Worth)</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Energy Capital Partners (ECP) / KKR (asociación estratégica de US$50 mil millones)</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>CyrusOne (JV de construcción/operación); Calpine Corp. (suministro de energía dedicada desde Thad Hill Energy Center)</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Construcción (primera inversión de la asociación estratégica ECP-KKR; campus de ~700,000 pies², inversión total cercana a US$4,000 millones, capacidad inicial de TI de 144MW sobre 190MW total; operación prevista 4T2026)</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>[Data Centre Magazine](https://datacentremagazine.com/news/ecp-and-kkr-to-build-4bn-190mw-hyperscale-data-centre); [Connect CRE](https://www.connectcre.com/stories/energy-capital-kkr-joint-forces-on-bosque-county-data-center/)</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Agregar 2 proyectos nuevos y 1 cambio de fase (2026-08-05)
- Mining: Bunker Hill Mine (Idaho, reinicio + planta de relleno en pasta)
- Mining: NewRange Copper Nickel / NorthMet (Minnesota, rediseño/permitting)
- Mining: Tamarack Nickel-Copper-Cobalt — actualizado con sitio de planta
  de proceso (Beulah, ND)

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LtG2tuXt4GQhSXHBiZp95N
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -20,18 +20,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <b val="1"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
@@ -57,9 +49,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -428,47 +419,47 @@
   <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -2005,47 +1996,47 @@
   <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -3468,50 +3459,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:G56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -5264,7 +5255,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Aitkin County, Minnesota (mina) / sitio de planta de proceso por definir (Mercer County, Dakota del Norte vs. Eagle Mine/Humboldt Mill, Michigan), EE.UU.</t>
+          <t>Aitkin County, Minnesota (mina) / Beulah, Dakota del Norte (planta de proceso — Beulah Minerals Processing Facility), EE.UU.</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -5279,34 +5270,34 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Permitting/Feasibility (EIS en scoping, comentarios cierran 14-sep-2026; estudio de factibilidad —incl. decisión de sitio de planta— esperado 2S2026; entendimiento informal de offtake con Tesla)</t>
+          <t>Permitting/Feasibility (Talon firmó acuerdo de opción de terreno con Westmoreland Mining, 28-jul-2026, por ~256 acres cerca de Beulah, ND, para la Beulah Minerals Processing Facility —planta de procesamiento de concentrado níquel-cobre respaldada por subvención DOE de US$114.8 millones—; EIS de la mina en scoping, comentarios cierran 14-sep-2026; entendimiento informal de offtake con Tesla)</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>[North Dakota Monitor](https://northdakotamonitor.com/2026/07/28/plans-for-north-dakota-nickel-processing-unclear-as-company-also-evaluates-michigan-site/)</t>
+          <t>[Talon Metals](https://talonmetals.com/talon-metals-and-westmoreland-mining-sign-land-agreement-to-progress-north-dakota-minerals-processing-facility/)</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>White Mesa Mill — Expansión de Tierras Raras Pesadas</t>
+          <t>Bunker Hill Mine — Reinicio + Planta de Relleno en Pasta</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Blanding, Utah, EE.UU.</t>
+          <t>Kellogg/Wardner, Idaho, EE.UU. (Distrito Minero Coeur d'Alene)</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Energy Fuels Inc.</t>
+          <t>Bunker Hill Mining Corp.</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -5316,163 +5307,237 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Construcción (planta comercial de tierras raras pesadas —disprosio/terbio— iniciada 29-jul-2026; capex ~US$104 millones, para uso en imanes/defensa/vehículos eléctricos)</t>
+          <t>Construcción/Comisionamiento (primer embarque de concentrado a la fundición Trail de Teck tras 45+ años de cierre; nueva planta de proceso de 1,800 tpd comisionada; planta de relleno en pasta en sitio Wardner sustancialmente completa, comisionamiento final previsto ~3 semanas tras el anuncio; meta de producción comercial plena fin de 2026)</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>[Energy Fuels](https://investors.energyfuels.com/2026-07-29-Commercial-Scale-Heavy-Rare-Earth-Plant-Now-Under-Construction-in-Utah); [PR Newswire](https://www.prnewswire.com/news-releases/commercial-scale-heavy-rare-earth-plant-now-under-construction-in-utah-302837314.html)</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/31/3337077/0/en/bunker-hill-ships-first-concentrate-to-trail-smelter-and-announces-drawdown-of-standby-facility.html)</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Black Butte Copper Project</t>
+          <t>NewRange Copper Nickel (Proyecto NorthMet) — Rediseño Mayor</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Meagher County, Montana, EE.UU.</t>
+          <t>Babbitt/Hoyt Lakes, Minnesota, EE.UU. (Iron Range)</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Sandfire Resources America Inc. (Sandfire Resources)</t>
+          <t>NewRange Copper Nickel (JV PolyMet/Glencore + Teck)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Por definir (PFS elaborado por DM Consulting)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Feasibility (PFS actualizado presentado 28-jul-2026 con nuevas reservas Lowry, vida de mina de 12 años; mina subterránea de cobre de alta ley)</t>
+          <t>Permitting (rediseño mayor elimina la represa de jales propuesta —roca estéril se almacenaría en tajos de mineral de hierro existentes—; solicitud de permiso de humedales Sección 404/Clean Water Act presentada ante USACE; revisión ambiental suplementaria (SEIS) solicitada a Minnesota DNR)</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/29/3334925/0/en/sandfire-resources-america-files-black-butte-copper-project-preliminary-feasibility-study.html)</t>
+          <t>[MPR News](https://www.mprnews.org/story/2026/07/30/newrange-copper-nickel-proposes-major-changes-to-copper-mine-plan)</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Planta de Procesamiento de Litio Red River (US Army)</t>
+          <t>White Mesa Mill — Expansión de Tierras Raras Pesadas</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Bowie County, Texas, EE.UU.</t>
+          <t>Blanding, Utah, EE.UU.</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Pentágono / Departamento del Ejército de EE.UU.</t>
+          <t>Energy Fuels Inc.</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>EnergyX (desarrollador-operador)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Acuerdo de arrendamiento condicional otorgado (confirmado 25-jun-2026; 5to sitio del programa de minerales críticos en bases del Ejército, junto con Tooele, Pine Bluff/Anniston; construcción prevista desde 2027)</t>
+          <t>Construcción (planta comercial de tierras raras pesadas —disprosio/terbio— iniciada 29-jul-2026; capex ~US$104 millones, para uso en imanes/defensa/vehículos eléctricos)</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>[Texarkana Gazette](https://www.texarkanagazette.com/news/2026/jun/30/army-awards-lithium-company-energyx-conditional/)</t>
+          <t>[Energy Fuels](https://investors.energyfuels.com/2026-07-29-Commercial-Scale-Heavy-Rare-Earth-Plant-Now-Under-Construction-in-Utah); [PR Newswire](https://www.prnewswire.com/news-releases/commercial-scale-heavy-rare-earth-plant-now-under-construction-in-utah-302837314.html)</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-07-30</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Camino Rojo — Proyecto Subterráneo (extensión)</t>
+          <t>Black Butte Copper Project</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Zacatecas, México</t>
+          <t>Meagher County, Montana, EE.UU.</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Orla Mining Ltd.</t>
+          <t>Sandfire Resources America Inc. (Sandfire Resources)</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Por definir (PFS elaborado por DM Consulting)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Permisos completos/inicio de desarrollo subterráneo (SEMARNAT aprobó MIA 18-mar-2026, habilitando minado del resto del tajo de óxidos y construcción de rampa de exploración subterránea; inicio de obras de acceso subterráneo previsto 2S2026; PEA de proyecto subterráneo indica VPN de US$1,300 millones)</t>
+          <t>Feasibility (PFS actualizado presentado 28-jul-2026 con nuevas reservas Lowry, vida de mina de 12 años; mina subterránea de cobre de alta ley)</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>[Mining.com](https://www.mining.com/orla-secures-final-permit-to-advance-underground-mining-at-camino-rojo/); [Orla Mining](https://orlamining.com/news/orla-mining-receives-permits-to-extend-operations-in-mexico-supporting-companys-long-term-commitment-to-camino-rojo/)</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/29/3334925/0/en/sandfire-resources-america-files-black-butte-copper-project-preliminary-feasibility-study.html)</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-03</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
+          <t>Planta de Procesamiento de Litio Red River (US Army)</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Bowie County, Texas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Pentágono / Departamento del Ejército de EE.UU.</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>EnergyX (desarrollador-operador)</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Acuerdo de arrendamiento condicional otorgado (confirmado 25-jun-2026; 5to sitio del programa de minerales críticos en bases del Ejército, junto con Tooele, Pine Bluff/Anniston; construcción prevista desde 2027)</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>[Texarkana Gazette](https://www.texarkanagazette.com/news/2026/jun/30/army-awards-lithium-company-energyx-conditional/)</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Camino Rojo — Proyecto Subterráneo (extensión)</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Zacatecas, México</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Orla Mining Ltd.</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Permisos completos/inicio de desarrollo subterráneo (SEMARNAT aprobó MIA 18-mar-2026, habilitando minado del resto del tajo de óxidos y construcción de rampa de exploración subterránea; inicio de obras de acceso subterráneo previsto 2S2026; PEA de proyecto subterráneo indica VPN de US$1,300 millones)</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>[Mining.com](https://www.mining.com/orla-secures-final-permit-to-advance-underground-mining-at-camino-rojo/); [Orla Mining](https://orlamining.com/news/orla-mining-receives-permits-to-extend-operations-in-mexico-supporting-companys-long-term-commitment-to-camino-rojo/)</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
           <t>Cerro Caliche Gold Project</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B56" t="inlineStr">
         <is>
           <t>Sonora, México</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C56" t="inlineStr">
         <is>
           <t>Sonoro Gold Corp.</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr">
+      <c r="D56" t="inlineStr">
         <is>
           <t>EPC por definir (en negociación con múltiples empresas EPC de China)</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
+      <c r="E56" t="inlineStr">
         <is>
           <t>Permisos/estructuración de financiamiento EPC (plataforma consolidada de 3,924 hectáreas en 25 concesiones; finalización de permisos esperada 1T2026; 4 empresas EPC chinas evaluando financiamiento de deuda y desarrollo)</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr">
+      <c r="F56" t="inlineStr">
         <is>
           <t>[Sonoro Gold Corp.](https://sonorogold.com/wp-content/uploads/2026/03/2026.03.01_Sonoro-Gold-Corporate-Presentation.pdf); [Mexico Mining Center](https://www.mexicominingcenter.com/sonoro-continues-discussions-with-china-based-epc-companies-and-potential-equity-investors/)</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr">
+      <c r="G56" t="inlineStr">
         <is>
           <t>2026-08-04</t>
         </is>
@@ -5492,47 +5557,47 @@
   <dimension ref="A1:G71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>

</xml_diff>

<commit_message>
Agregar 12 proyectos nuevos y 2 cambios de fase (2026-08-10)
Nuevos: Gasoducto TTC Connector (LNG); Lone Tree Plant, Round Mountain
Phase X, Bald Mountain Redbird 2, Bear Lodge Rare Earth, Cobre
Angangueo, Cobre Chalchihuites, Modernización Empalme (Mining);
Galaxy Digital Project Merlin, Nexus Fulcrum Gas Plant (Data
Centers). Actualizaciones de fase: GW Ranch Power Campus (Amazon
confirmado como inquilino), VoltaGrid/Serverfarm Covington
(construcción reanudada).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ArQ4Pz8sq54DrJPjfCETqj
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -416,15 +416,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -801,217 +801,217 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Rehab. Fertinal-ProAgro (urea y fosfatos)</t>
+          <t>Proyecto Escolín (amoniaco/urea)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Lázaro Cárdenas, Michoacán, México</t>
+          <t>Poza Rica, Veracruz, México</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Pemex</t>
+          <t>Pemex Transformación Industrial</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Mota-Engil México (EPC confirmado; plazo de construcción 33 meses)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Ingeniería/rehabilitación (incorporado al plan de reactivación petroquímica de Pemex, jun-2026; 13,700 millones de pesos asignados para los complejos Lázaro Cárdenas y ProAgro; meta de 2.4 millones ton/año de urea y fertilizantes fosfatados)</t>
+          <t>Ingeniería/inicio de construcción (inversión confirmada US$1,553 millones)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>[Tribuna](https://tribuna.com.mx/mexico/2026/06/05/sheinbaum-anuncia-inversion-de-93-mil-mdp-para-reactivar-la-industria-petroquimica-y-de-fertilizantes-en-veracruz_560837/); [Contralínea](https://contralinea.com.mx/interno/semana/presentan-plan-con-inversion-de-93-mil-mdp-para-rescatar-la-petroquimica-nacional/)</t>
+          <t>[Forbes México](https://forbes.com.mx/asi-es-la-inversion-de-1553-mdd-por-parte-de-pemex-en-una-planta-de-fertilizantes-en-veracruz/)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Pacífico Mexinol (metanol ultra bajo carbono)</t>
+          <t>Rehab. Fertinal-ProAgro (urea y fosfatos)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Topolobampo, Sinaloa, México</t>
+          <t>Lázaro Cárdenas, Michoacán, México</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Transition Industries</t>
+          <t>Pemex</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Siemens Energy / Techint E&amp;C (FEED electrolizador)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Construcción (iniciada abr-2026)</t>
+          <t>Ingeniería/rehabilitación (incorporado al plan de reactivación petroquímica de Pemex, jun-2026; 13,700 millones de pesos asignados para los complejos Lázaro Cárdenas y ProAgro; meta de 2.4 millones ton/año de urea y fertilizantes fosfatados)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>[PV Magazine México](https://www.pv-magazine-mexico.com/2026/04/28/inician-en-sinaloa-la-construccion-de-la-mayor-planta-de-metanol-ultrabajo-en-carbono-a-partir-de-hidrogeno-verde/)</t>
+          <t>[Tribuna](https://tribuna.com.mx/mexico/2026/06/05/sheinbaum-anuncia-inversion-de-93-mil-mdp-para-reactivar-la-industria-petroquimica-y-de-fertilizantes-en-veracruz_560837/); [Contralínea](https://contralinea.com.mx/interno/semana/presentan-plan-con-inversion-de-93-mil-mdp-para-rescatar-la-petroquimica-nacional/)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>First Ammonia (amoniaco verde)</t>
+          <t>Pacífico Mexinol (metanol ultra bajo carbono)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Victoria, Texas, EE.UU.</t>
+          <t>Topolobampo, Sinaloa, México</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>First Ammonia / Cox Group USA</t>
+          <t>Transition Industries</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Worley (FEED)</t>
+          <t>Siemens Energy / Techint E&amp;C (FEED electrolizador)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Ingeniería (FEED completo) / FID prevista 2026</t>
+          <t>Construcción (iniciada abr-2026)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>[H2 View](https://www.h2-view.com/story/first-ammonia-project-on-track-for-2026-fid-despite-topsoe-deal-collapse/2138792.article/)</t>
+          <t>[PV Magazine México](https://www.pv-magazine-mexico.com/2026/04/28/inician-en-sinaloa-la-construccion-de-la-mayor-planta-de-metanol-ultrabajo-en-carbono-a-partir-de-hidrogeno-verde/)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-10</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Planta de Amoniaco Topolobampo (GPO)</t>
+          <t>First Ammonia (amoniaco verde)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Topolobampo, Sinaloa, México</t>
+          <t>Victoria, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Gas y Petroquímica de Occidente (GPO) / Proman AG</t>
+          <t>First Ammonia / Cox Group USA</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Worley (FEED)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Construcción (avance ~80% confirmado por Secretaría de Economía jul-2026; op. comercial H1 2027)</t>
+          <t>Ingeniería (FEED completo) / FID prevista 2026</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>[Debate](https://www.debate.com.mx/economia/secretaria-de-economia-complejo-de-amoniaco-en-topolobampo-prioritario-para-el-gobierno-de-mexico-20260713-0092.html)</t>
+          <t>[H2 View](https://www.h2-view.com/story/first-ammonia-project-on-track-for-2026-fid-despite-topsoe-deal-collapse/2138792.article/)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Lake Charles Methanol II</t>
+          <t>Planta de Amoniaco Topolobampo (GPO)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Lake Charles, Luisiana, EE.UU.</t>
+          <t>Topolobampo, Sinaloa, México</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Lake Charles Methanol II LLC</t>
+          <t>Gas y Petroquímica de Occidente (GPO) / Proman AG</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Zachry Group (FEED)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Ingeniería (FEED) / FID prevista</t>
+          <t>Construcción (avance ~80% confirmado por Secretaría de Economía jul-2026; op. comercial H1 2027)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>[ICIS](https://www.icis.com/explore/resources/news/2025/11/13/11155109/lake-charles-methanol-ii-awards-feed-fid-expected-in-q2-2026/)</t>
+          <t>[Debate](https://www.debate.com.mx/economia/secretaria-de-economia-complejo-de-amoniaco-en-topolobampo-prioritario-para-el-gobierno-de-mexico-20260713-0092.html)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Planta Coquizadora Salina Cruz</t>
+          <t>Lake Charles Methanol II</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Salina Cruz, Oaxaca, México</t>
+          <t>Lake Charles, Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Pemex</t>
+          <t>Lake Charles Methanol II LLC</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>ICA Fluor</t>
+          <t>Zachry Group (FEED)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Construcción (~74% avance)</t>
+          <t>Ingeniería (FEED) / FID prevista</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>[Diario del Istmo](https://diariodelistmo.com/nacional/este-es-el-avance-que-lleva-la-planta-coquizadora-en-la-refineria-de-salina-cruz/50642321)</t>
+          <t>[ICIS](https://www.icis.com/explore/resources/news/2025/11/13/11155109/lake-charles-methanol-ii-awards-feed-fid-expected-in-q2-2026/)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1023,54 +1023,54 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Shintech Louisiana — Expansión Plaquemine (2do craqueador de etileno + 4ta unidad cloro-álcali/VCM)</t>
+          <t>Planta Coquizadora Salina Cruz</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Plaquemine, Iberville Parish, Luisiana, EE.UU.</t>
+          <t>Salina Cruz, Oaxaca, México</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Shintech Louisiana, LLC</t>
+          <t>Pemex</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>ICA Fluor</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Ingeniería/planeación (construcción por fases, 1a fase prevista 2030)</t>
+          <t>Construcción (~74% avance)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/petrochemicals/06032026/shintech-announces-us34-billion-at-louisiana-petrochemicals-complex/)</t>
+          <t>[Diario del Istmo](https://diariodelistmo.com/nacional/este-es-el-avance-que-lleva-la-planta-coquizadora-en-la-refineria-de-salina-cruz/50642321)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Sandpiper Chemicals (metanol bajo carbono)</t>
+          <t>Shintech Louisiana — Expansión Plaquemine (2do craqueador de etileno + 4ta unidad cloro-álcali/VCM)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Texas City, Texas, EE.UU.</t>
+          <t>Plaquemine, Iberville Parish, Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Sandpiper Chemicals, LLC / INEOS Acetyls (colaboración estratégica, abr-2026)</t>
+          <t>Shintech Louisiana, LLC</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1080,86 +1080,86 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Ingeniería (FEED en curso desde 2T2026; US$1,700 millones, 1.1 MMtpa; INEOS Acetyls tomará 300,000 ton/año para su unidad de ácido acético) / FID prevista 2027, primera producción ~2030</t>
+          <t>Ingeniería/planeación (construcción por fases, 1a fase prevista 2030)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>[INEOS](https://www.ineos.com/news/shared-news/ineos-acetyls-and-sandpiper-chemicals-announce-strategic-collaboration-for-the-development-of-a-low-carbon-methanol-project-in-texas-city-texas/)</t>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/petrochemicals/06032026/shintech-announces-us34-billion-at-louisiana-petrochemicals-complex/)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-14</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>OXEA Bay City Capacity Expansion + Air Liquide POX Syngas Unit</t>
+          <t>Sandpiper Chemicals (metanol bajo carbono)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Bay City, Matagorda County, Texas, EE.UU.</t>
+          <t>Texas City, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>OXEA (oxo chemicals) / Air Liquide (unidad de syngas)</t>
+          <t>Sandpiper Chemicals, LLC / INEOS Acetyls (colaboración estratégica, abr-2026)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Air Liquide (unidad propia); OXEA no especificado</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Construcción (FID confirmado 13-jul-2026; preparación de sitio 3T2026; finalización fines de 2028)</t>
+          <t>Ingeniería (FEED en curso desde 2T2026; US$1,700 millones, 1.1 MMtpa; INEOS Acetyls tomará 300,000 ton/año para su unidad de ácido acético) / FID prevista 2027, primera producción ~2030</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/petrochemicals/13072026/oxea-confirms-fid-for-major-capacity-expansion/)</t>
+          <t>[INEOS](https://www.ineos.com/news/shared-news/ineos-acetyls-and-sandpiper-chemicals-announce-strategic-collaboration-for-the-development-of-a-low-carbon-methanol-project-in-texas-city-texas/)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-29</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Targa Resources East Driver Gas Processing Plant</t>
+          <t>OXEA Bay City Capacity Expansion + Air Liquide POX Syngas Unit</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Condado de Midland, Texas, EE.UU.</t>
+          <t>Bay City, Matagorda County, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Targa Resources Corp.</t>
+          <t>OXEA (oxo chemicals) / Air Liquide (unidad de syngas)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Targa Resources (propietario-constructor)</t>
+          <t>Air Liquide (unidad propia); OXEA no especificado</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Construcción (planta criogénica 275 MMcf/d; arranque previsto 3T2026)</t>
+          <t>Construcción (FID confirmado 13-jul-2026; preparación de sitio 3T2026; finalización fines de 2028)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>[OGJ](https://www.ogj.com/refining-processing/gas-processing/news/55320579/targa-advances-permian-gas-pipeline-processing-expansion)</t>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/petrochemicals/13072026/oxea-confirms-fid-for-major-capacity-expansion/)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1171,32 +1171,32 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Enterprise Products "Athena" Natural Gas Processing Plant</t>
+          <t>Targa Resources East Driver Gas Processing Plant</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Cuenca Midland (cuatro condados), Texas, EE.UU.</t>
+          <t>Condado de Midland, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Enterprise Products Partners L.P.</t>
+          <t>Targa Resources Corp.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Enterprise Products (propietario-constructor)</t>
+          <t>Targa Resources (propietario-constructor)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Construcción (300 MMcf/d + hasta 40,000 bpd de NGLs; en servicio 4T2026)</t>
+          <t>Construcción (planta criogénica 275 MMcf/d; arranque previsto 3T2026)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>[Business Wire](https://www.businesswire.com/news/home/20250806663187/en/Enterprise-Agrees-to-Acquire-Occidentals-Gas-Gathering-Affiliate-Enters-Into-Natural-Gas-Processing-Agreement-Announces-New-Midland-Basin-Natural-Gas-Processing-Plant)</t>
+          <t>[OGJ](https://www.ogj.com/refining-processing/gas-processing/news/55320579/targa-advances-permian-gas-pipeline-processing-expansion)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1208,32 +1208,32 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>MPLX Secretariat II Gas Processing Plant</t>
+          <t>Enterprise Products "Athena" Natural Gas Processing Plant</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Cuenca Pérmica (subcuenca Delaware), Texas/Nuevo México, EE.UU.</t>
+          <t>Cuenca Midland (cuatro condados), Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>MPLX LP</t>
+          <t>Enterprise Products Partners L.P.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>MPLX (propietario-constructor)</t>
+          <t>Enterprise Products (propietario-constructor)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Planeada/desarrollo (300 MMcf/d; en servicio 2S2028)</t>
+          <t>Construcción (300 MMcf/d + hasta 40,000 bpd de NGLs; en servicio 4T2026)</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>[Natural Gas Intel](https://naturalgasintel.com/news/mplx-scales-up-for-power-hungry-future-with-natural-gas-focused-growth-plan/)</t>
+          <t>[Business Wire](https://www.businesswire.com/news/home/20250806663187/en/Enterprise-Agrees-to-Acquire-Occidentals-Gas-Gathering-Affiliate-Enters-Into-Natural-Gas-Processing-Agreement-Announces-New-Midland-Basin-Natural-Gas-Processing-Plant)</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1245,12 +1245,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>MPLX Titan Complex (Northwind) — Expansión de Tratamiento de Gas Amargo</t>
+          <t>MPLX Secretariat II Gas Processing Plant</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Condado de Lea, Nuevo México / frontera TX-NM, EE.UU.</t>
+          <t>Cuenca Pérmica (subcuenca Delaware), Texas/Nuevo México, EE.UU.</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1265,12 +1265,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Construcción (expansión de capacidad &gt;400 MMcf/d; plenamente operativo 4T2026)</t>
+          <t>Planeada/desarrollo (300 MMcf/d; en servicio 2S2028)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>[East Daley](https://eastdaley.com/daley-note/mplx-acquires-northwind-for-2-375b-acquires-more-ngls-for-jv-project)</t>
+          <t>[Natural Gas Intel](https://naturalgasintel.com/news/mplx-scales-up-for-power-hungry-future-with-natural-gas-focused-growth-plan/)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1282,32 +1282,32 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Northern Plains Nitrogen (urea/amoniaco)</t>
+          <t>MPLX Titan Complex (Northwind) — Expansión de Tratamiento de Gas Amargo</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Grand Forks, Dakota del Norte, EE.UU.</t>
+          <t>Condado de Lea, Nuevo México / frontera TX-NM, EE.UU.</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Northern Plains Nitrogen LLC</t>
+          <t>MPLX LP</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>EPC no designado</t>
+          <t>MPLX (propietario-constructor)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Pre-FEED completo / FID buscada 4T2026</t>
+          <t>Construcción (expansión de capacidad &gt;400 MMcf/d; plenamente operativo 4T2026)</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>[Grand Forks Herald](https://www.grandforksherald.com/news/local/northern-plains-nitrogen-proposal-receiving-more-attention-amid-global-fertilizer-pressure)</t>
+          <t>[East Daley](https://eastdaley.com/daley-note/mplx-acquires-northwind-for-2-375b-acquires-more-ngls-for-jv-project)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1319,54 +1319,54 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Iron Mesa (planta de gas)</t>
+          <t>Northern Plains Nitrogen (urea/amoniaco)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Goldsmith, Ector County, Texas, EE.UU.</t>
+          <t>Grand Forks, Dakota del Norte, EE.UU.</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Phillips 66</t>
+          <t>Northern Plains Nitrogen LLC</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>EPC no designado</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Construcción (arranque previsto Q1 2027)</t>
+          <t>Pre-FEED completo / FID buscada 4T2026</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>[Phillips 66](https://www.phillips66.com/newsroom/iron-mesa-safely-enters-next-phase-of-construction/)</t>
+          <t>[Grand Forks Herald](https://www.grandforksherald.com/news/local/northern-plains-nitrogen-proposal-receiving-more-attention-amid-global-fertilizer-pressure)</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Yeti II (planta de gas)</t>
+          <t>Iron Mesa (planta de gas)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Cuenca Delaware (Permian), Texas/Nuevo México, EE.UU.</t>
+          <t>Goldsmith, Ector County, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Targa Resources</t>
+          <t>Phillips 66</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1376,12 +1376,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Ingeniería/planeación (en línea previsto Q4 2027)</t>
+          <t>Construcción (arranque previsto Q1 2027)</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>[Targa Resources](https://www.targaresources.com/news-releases/news-release-details/targa-resources-corp-announces-permian-growth-projects-and)</t>
+          <t>[Phillips 66](https://www.phillips66.com/newsroom/iron-mesa-safely-enters-next-phase-of-construction/)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1393,32 +1393,32 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Refinería Francisco I. Madero (rehabilitación)</t>
+          <t>Yeti II (planta de gas)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Ciudad Madero, Tamaulipas, México</t>
+          <t>Cuenca Delaware (Permian), Texas/Nuevo México, EE.UU.</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Pemex</t>
+          <t>Targa Resources</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Múltiples contratistas por licitar (30+ licitaciones)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Licitación/bidding</t>
+          <t>Ingeniería/planeación (en línea previsto Q4 2027)</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>[Elefante Blanco](https://elefanteblanco.mx/2026/01/02/pemex-abre-30-licitaciones-para-obras-en-la-refineria-madero/)</t>
+          <t>[Targa Resources](https://www.targaresources.com/news-releases/news-release-details/targa-resources-corp-announces-permian-growth-projects-and)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1430,69 +1430,69 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Fermachem Planta de Urea/Amoniaco</t>
+          <t>Refinería Francisco I. Madero (rehabilitación)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Ejido Sapioris, Lerdo, Durango, México</t>
+          <t>Ciudad Madero, Tamaulipas, México</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Fermaca Dreams (Fermachem)</t>
+          <t>Pemex</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Técnicas Reunidas (licencia/tecnología KBR-Stamicarbon)</t>
+          <t>Múltiples contratistas por licitar (30+ licitaciones)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Construcción (ejecución iniciada jun-2026)</t>
+          <t>Licitación/bidding</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>[La Jornada](https://www.jornada.com.mx/noticia/2026/06/08/economia/da-inicio-ejecucion-de-planta-de-fertilizantes-en-durango-por-parte-de-fermachem)</t>
+          <t>[Elefante Blanco](https://elefanteblanco.mx/2026/01/02/pemex-abre-30-licitaciones-para-obras-en-la-refineria-madero/)</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-15</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Ascension Clean Energy (ACE) — amoniaco azul</t>
+          <t>Fermachem Planta de Urea/Amoniaco</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Donaldsonville, Ascension Parish, Luisiana, EE.UU.</t>
+          <t>Ejido Sapioris, Lerdo, Durango, México</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Clean Hydrogen Works</t>
+          <t>Fermaca Dreams (Fermachem)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>McDermott (FEED)</t>
+          <t>Técnicas Reunidas (licencia/tecnología KBR-Stamicarbon)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Ingeniería (FEED) / Pre-FID</t>
+          <t>Construcción (ejecución iniciada jun-2026)</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>[Downstream Calendar](https://downstreamcalendar.com/mcdermott-secures-feed-contract-for-ascension-clean-energy-project/)</t>
+          <t>[La Jornada](https://www.jornada.com.mx/noticia/2026/06/08/economia/da-inicio-ejecucion-de-planta-de-fertilizantes-en-durango-por-parte-de-fermachem)</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1504,32 +1504,32 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Zeus Gas Plant + 3ra Fraccionadora Coastal Bend</t>
+          <t>Ascension Clean Energy (ACE) — amoniaco azul</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Cuenca Pérmica, Texas / Robstown, Texas, EE.UU.</t>
+          <t>Donaldsonville, Ascension Parish, Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Phillips 66</t>
+          <t>Clean Hydrogen Works</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>McDermott (FEED)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Ingeniería (sancionado; en línea 2028)</t>
+          <t>Ingeniería (FEED) / Pre-FID</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>[Business Wire](https://www.businesswire.com/news/home/20260517310811/en/Phillips-66-announces-Zeus-Gas-Plant-and-a-third-Coastal-Bend-Fractionator)</t>
+          <t>[Downstream Calendar](https://downstreamcalendar.com/mcdermott-secures-feed-contract-for-ascension-clean-energy-project/)</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1541,128 +1541,128 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Project Meadowlark (complejo de amoniaco azul/UAN/ATS/DEF)</t>
+          <t>Zeus Gas Plant + 3ra Fraccionadora Coastal Bend</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Gothenburg, Nebraska, EE.UU.</t>
+          <t>Cuenca Pérmica, Texas / Robstown, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>J. Westling &amp; Co. (JWC Gburg, LLC)</t>
+          <t>Phillips 66</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>No especificado (tecnología licenciada Topsoe SynCOR Ammonia); contrato EPC/fabricación asegurado</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Ingeniería/Permisos (permiso de aire emitido, sitio zonificado; obras civiles previstas 2027, operación comercial 2029)</t>
+          <t>Ingeniería (sancionado; en línea 2028)</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>[USDA](https://www.usda.gov/about-usda/news/press-releases/2026/07/01/secretary-rollins-announces-500-million-fertilizer-investment-and-expansion-program-strengthen)</t>
+          <t>[Business Wire](https://www.businesswire.com/news/home/20260517310811/en/Phillips-66-announces-Zeus-Gas-Plant-and-a-third-Coastal-Bend-Fractionator)</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-17</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Wabash Low-Carbon Ammonia Project</t>
+          <t>Project Meadowlark (complejo de amoniaco azul/UAN/ATS/DEF)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>West Terre Haute, Indiana, EE.UU.</t>
+          <t>Gothenburg, Nebraska, EE.UU.</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Wabash Valley Resources</t>
+          <t>J. Westling &amp; Co. (JWC Gburg, LLC)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Samsung E&amp;C (contrato EPF ~US$475 millones)</t>
+          <t>No especificado (tecnología licenciada Topsoe SynCOR Ammonia); contrato EPC/fabricación asegurado</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Construcción (groundbreaking 5-ene-2026; amoniaco bajo en carbono 500,000 ton/año con captura de 1.67 millones ton CO2/año; meta de finalización 2029)</t>
+          <t>Ingeniería/Permisos (permiso de aire emitido, sitio zonificado; obras civiles previstas 2027, operación comercial 2029)</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/clean-fuels/06012026/samsung-ea-announces-groundbreaking-of-low-carbon-ammonia-plant/)</t>
+          <t>[USDA](https://www.usda.gov/about-usda/news/press-releases/2026/07/01/secretary-rollins-announces-500-million-fertilizer-investment-and-expansion-program-strengthen)</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Green Fuels Operating — Refinería Duncan</t>
+          <t>Wabash Low-Carbon Ammonia Project</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Duncan, Stephens County, Oklahoma, EE.UU.</t>
+          <t>West Terre Haute, Indiana, EE.UU.</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Green Fuels Operating</t>
+          <t>Wabash Valley Resources</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Samsung E&amp;C (contrato EPF ~US$475 millones)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Construcción (groundbreaking 29-may-2026; inversión US$400 millones; capacidad inicial 30,000 bbl/d, expandible a 50,000 bbl/d, sobre sitio de refinería histórica de los años 1920)</t>
+          <t>Construcción (groundbreaking 5-ene-2026; amoniaco bajo en carbono 500,000 ton/año con captura de 1.67 millones ton CO2/año; meta de finalización 2029)</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/refining/03062026/green-fuels-hosts-groundbreaking-ceremony-for-new-refinery/)</t>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/clean-fuels/06012026/samsung-ea-announces-groundbreaking-of-low-carbon-ammonia-plant/)</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-24</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Energy Transfer Mustang Draw I &amp; II (plantas de gas)</t>
+          <t>Green Fuels Operating — Refinería Duncan</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Cuenca Midland, Texas, EE.UU.</t>
+          <t>Duncan, Stephens County, Oklahoma, EE.UU.</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Energy Transfer LP</t>
+          <t>Green Fuels Operating</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1672,34 +1672,34 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Construcción (Mustang Draw I en comisionamiento, servicio pleno ~jun-2026; Mustang Draw II en construcción, en servicio 4T2026; 275 MMcf/d cada una)</t>
+          <t>Construcción (groundbreaking 29-may-2026; inversión US$400 millones; capacidad inicial 30,000 bbl/d, expandible a 50,000 bbl/d, sobre sitio de refinería histórica de los años 1920)</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>[Energy Transfer](https://www.energytransfer.com/project-highlights/)</t>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/refining/03062026/green-fuels-hosts-groundbreaking-ceremony-for-new-refinery/)</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ONEOK Bighorn / Cutter / Shadowfax (plantas de gas)</t>
+          <t>Energy Transfer Mustang Draw I &amp; II (plantas de gas)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Cuenca Delaware (Bighorn), Texas / Cuenca Powder River (Cutter), Wyoming / Cuenca Midland (Shadowfax reubicada), Texas, EE.UU.</t>
+          <t>Cuenca Midland, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ONEOK Inc.</t>
+          <t>Energy Transfer LP</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1709,12 +1709,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Construcción (Bighorn US$365 millones/300 MMcf/d tratamiento alto CO2, meta mediados 2027; Cutter 60 MMcf/d en construcción, meta 4T2026; Shadowfax 150 MMcf/d reubicación completada 1T2026, en rampa)</t>
+          <t>Construcción (Mustang Draw I en comisionamiento, servicio pleno ~jun-2026; Mustang Draw II en construcción, en servicio 4T2026; 275 MMcf/d cada una)</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>[Inspectioneering](https://inspectioneering.com/news/2025-08-07/11702/oneok-greenlights-new-365m-delaware-basin-gas-plant)</t>
+          <t>[Energy Transfer](https://www.energytransfer.com/project-highlights/)</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1726,32 +1726,32 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>MPLX Harmon Creek III (planta de gas + de-etanizadora)</t>
+          <t>ONEOK Bighorn / Cutter / Shadowfax (plantas de gas)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Región Marcellus/Utica, noreste de EE.UU. (ubicación exacta no especificada)</t>
+          <t>Cuenca Delaware (Bighorn), Texas / Cuenca Powder River (Cutter), Wyoming / Cuenca Midland (Shadowfax reubicada), Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>MPLX LP</t>
+          <t>ONEOK Inc.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>MPLX (propietario-constructor)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Construcción (300 MMcf/d + de-etanizadora 40 Mbpd; en servicio 3T2026)</t>
+          <t>Construcción (Bighorn US$365 millones/300 MMcf/d tratamiento alto CO2, meta mediados 2027; Cutter 60 MMcf/d en construcción, meta 4T2026; Shadowfax 150 MMcf/d reubicación completada 1T2026, en rampa)</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>[Natural Gas Intel](https://www.naturalgasintel.com/news/mplx-scales-up-for-power-hungry-future-with-natural-gas-focused-growth-plan/)</t>
+          <t>[Inspectioneering](https://inspectioneering.com/news/2025-08-07/11702/oneok-greenlights-new-365m-delaware-basin-gas-plant)</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1763,86 +1763,86 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Rehab. Complejo Cosoleacaque (amoniaco) + Complejo Morelos (etano-etileno)</t>
+          <t>MPLX Harmon Creek III (planta de gas + de-etanizadora)</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Cosoleacaque y Complejo Morelos, Veracruz, México</t>
+          <t>Región Marcellus/Utica, noreste de EE.UU. (ubicación exacta no especificada)</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Pemex Transformación Industrial</t>
+          <t>MPLX LP</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Mota-Engil México (plantas VI/VII y TASP Pajaritos); ICA (paquete relacionado)</t>
+          <t>MPLX (propietario-constructor)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Ingeniería/planeación (parte del plan de reactivación petroquímica de Pemex de 93,000 mdp anunciado jun-2026; 13,000 mdp para 2 plantas de amoniaco en Cosoleacaque, meta 957,000 ton/año; Complejo Morelos incluido en programa de rehabilitación etano-etileno de 30,000 mdp/5 plantas, meta 520,000 ton/año de polietilenos/óxido de etileno/glicoles; contratos de rehabilitación y confiabilidad adjudicados dic-2025, confirmados ene-2026)</t>
+          <t>Construcción (300 MMcf/d + de-etanizadora 40 Mbpd; en servicio 3T2026)</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>[Contralínea](https://contralinea.com.mx/interno/semana/presentan-plan-con-inversion-de-93-mil-mdp-para-rescatar-la-petroquimica-nacional/); [El Diario de Juárez](https://diario.mx/nacional/2026/jan/22/adjudica-pemex-contratos-a-favoritas-1102601.html)</t>
+          <t>[Natural Gas Intel](https://www.naturalgasintel.com/news/mplx-scales-up-for-power-hungry-future-with-natural-gas-focused-growth-plan/)</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-07-29</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Enterprise Products — Nuevas Plantas de Gas Permian (Plant 11 Midland / Plant 13 Delaware) + NGL Frac 15 Mont Belvieu</t>
+          <t>Rehab. Complejo Cosoleacaque (amoniaco) + Complejo Morelos (etano-etileno)</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Cuenca Midland y Cuenca Delaware, Texas, EE.UU. / Mont Belvieu, Texas, EE.UU.</t>
+          <t>Cosoleacaque y Complejo Morelos, Veracruz, México</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Enterprise Products Partners L.P.</t>
+          <t>Pemex Transformación Industrial</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Enterprise Products (propietario-constructor)</t>
+          <t>Mota-Engil México (plantas VI/VII y TASP Pajaritos); ICA (paquete relacionado)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Construcción (sancionadas/aprobadas en resultados 2T2026: Plant 11 Midland Basin 300 MMcf/d en servicio 1T2029; Plant 13 Delaware Basin 300 MMcf/d en servicio 3T2028; NGL Frac 15 en Mont Belvieu 150 MBPD en servicio 1T2028; gasto de capital de crecimiento 2026 aumentado en más de US$700 millones por estas sanciones)</t>
+          <t>Ingeniería/planeación (parte del plan de reactivación petroquímica de Pemex de 93,000 mdp anunciado jun-2026; 13,000 mdp para 2 plantas de amoniaco en Cosoleacaque, meta 957,000 ton/año; Complejo Morelos incluido en programa de rehabilitación etano-etileno de 30,000 mdp/5 plantas, meta 520,000 ton/año de polietilenos/óxido de etileno/glicoles; contratos de rehabilitación y confiabilidad adjudicados dic-2025, confirmados ene-2026)</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>[Enterprise Reports Second Quarter 2026 Earnings](https://ir.enterpriseproducts.com/news-releases/news-release-details/enterprise-reports-second-quarter-2026-earnings)</t>
+          <t>[Contralínea](https://contralinea.com.mx/interno/semana/presentan-plan-con-inversion-de-93-mil-mdp-para-rescatar-la-petroquimica-nacional/); [El Diario de Juárez](https://diario.mx/nacional/2026/jan/22/adjudica-pemex-contratos-a-favoritas-1102601.html)</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-06</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Enterprise Products — Plant 12 (Delaware Basin) y Athena 2 (Midland Basin)</t>
+          <t>Enterprise Products — Nuevas Plantas de Gas Permian (Plant 11 Midland / Plant 13 Delaware) + NGL Frac 15 Mont Belvieu</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Cuenca Delaware y Cuenca Midland, Texas, EE.UU.</t>
+          <t>Cuenca Midland y Cuenca Delaware, Texas, EE.UU. / Mont Belvieu, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1857,7 +1857,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Construcción (sancionadas, divulgadas en resultados 2T2026 el 30-jul-2026; Plant 12 Delaware Basin ~300 MMcf/d en servicio 4T2027; Athena 2 Midland Basin en servicio 3T2027)</t>
+          <t>Construcción (sancionadas/aprobadas en resultados 2T2026: Plant 11 Midland Basin 300 MMcf/d en servicio 1T2029; Plant 13 Delaware Basin 300 MMcf/d en servicio 3T2028; NGL Frac 15 en Mont Belvieu 150 MBPD en servicio 1T2028; gasto de capital de crecimiento 2026 aumentado en más de US$700 millones por estas sanciones)</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -1867,39 +1867,39 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-07-31</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Targa Resources Roadrunner III / Copperhead II (plantas de gas)</t>
+          <t>Enterprise Products — Plant 12 (Delaware Basin) y Athena 2 (Midland Basin)</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Cuenca Delaware (Permian), Texas/Nuevo México, EE.UU.</t>
+          <t>Cuenca Delaware y Cuenca Midland, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Targa Resources Corp.</t>
+          <t>Enterprise Products Partners L.P.</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Targa Resources (propietario-constructor)</t>
+          <t>Enterprise Products (propietario-constructor)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Construcción (aprobadas may-2026; Roadrunner III 265 MMcf/d, Copperhead II 275 MMcf/d; en servicio previsto 1T2028)</t>
+          <t>Construcción (sancionadas, divulgadas en resultados 2T2026 el 30-jul-2026; Plant 12 Delaware Basin ~300 MMcf/d en servicio 4T2027; Athena 2 Midland Basin en servicio 3T2027)</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>[PGJ](https://pgjonline.com/news/2026/may/targa-expands-permian-gas-processing-delaware-express-pipeline-capacity)</t>
+          <t>[Enterprise Reports Second Quarter 2026 Earnings](https://ir.enterpriseproducts.com/news-releases/news-release-details/enterprise-reports-second-quarter-2026-earnings)</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -1911,54 +1911,54 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Southern Energy Renewables — Complejo de Metanol y SAF</t>
+          <t>Targa Resources Roadrunner III / Copperhead II (plantas de gas)</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>St. Charles Parish (Killona), Luisiana, EE.UU.</t>
+          <t>Cuenca Delaware (Permian), Texas/Nuevo México, EE.UU.</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Southern Energy Renewables</t>
+          <t>Targa Resources Corp.</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Targa Resources (propietario-constructor)</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Planeación/pre-construcción (inversión US$1,400 millones; convierte biomasa de desecho de madera en metanol verde y combustible de aviación sostenible; construcción prevista a iniciar fines de 2027, producción prevista fines de 2029)</t>
+          <t>Construcción (aprobadas may-2026; Roadrunner III 265 MMcf/d, Copperhead II 275 MMcf/d; en servicio previsto 1T2028)</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>[Hydrocarbon Processing](https://www.hydrocarbonprocessing.com/news/2026/03/southern-energy-renewables-announce-14-b-methanol-and-saf-complex-in-louisiana/); [Louisiana Economic Development](https://www.opportunitylouisiana.gov/news/southern-energy-renewables-announce-1-4-billion-methanol-and-sustainable-aviation-fuel-facility-in-st-charles-parish)</t>
+          <t>[PGJ](https://pgjonline.com/news/2026/may/targa-expands-permian-gas-processing-delaware-express-pipeline-capacity)</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-03</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Atlas Agro — Pacific Green Fertilizer Plant</t>
+          <t>Southern Energy Renewables — Complejo de Metanol y SAF</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Richland, Washington, EE.UU.</t>
+          <t>St. Charles Parish (Killona), Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Atlas Agro</t>
+          <t>Southern Energy Renewables</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1968,49 +1968,49 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Ingeniería/FEED (diseño ~70% completo, USD 315 millones de capital levantado, permisos en proceso; planta de fertilizante nitrato ~0.7 Mt/año, inversión USD 1,100-1,500 millones; debe iniciar construcción antes de fines de 2027 para calificar a créditos fiscales federales; construcción estimada en 36 meses)</t>
+          <t>Planeación/pre-construcción (inversión US$1,400 millones; convierte biomasa de desecho de madera en metanol verde y combustible de aviación sostenible; construcción prevista a iniciar fines de 2027, producción prevista fines de 2029)</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>[Tri-Cities Area Journal of Business](https://www.tricitiesbusinessnews.com/articles/atlas-agro-plant-nears-decision-point); [Washington State Standard](https://washingtonstatestandard.com/2025/10/30/plan-for-1-5b-fertilizer-plant-in-central-wa-still-alive-despite-loss-of-federal-funds/)</t>
+          <t>[Hydrocarbon Processing](https://www.hydrocarbonprocessing.com/news/2026/03/southern-energy-renewables-announce-14-b-methanol-and-saf-complex-in-louisiana/); [Louisiana Economic Development](https://www.opportunitylouisiana.gov/news/southern-energy-renewables-announce-1-4-billion-methanol-and-sustainable-aviation-fuel-facility-in-st-charles-parish)</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-04</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Hydrogen City (complejo Power-to-X / e-metanol)</t>
+          <t>Atlas Agro — Pacific Green Fertilizer Plant</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Piedras Pintas Salt Dome, Condado de Duval, sur de Texas, EE.UU.</t>
+          <t>Richland, Washington, EE.UU.</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Green Hydrogen International (GHI)</t>
+          <t>Atlas Agro</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>ABB (automatización/control, vía MOU)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Ingeniería/FEED (inversión USD 6,000-10,000 millones; electrolizador de 2.2 GW; producirá 1.4 Mt/año de e-metanol y capturará ~2 Mt/año de CO2; construcción planeada desde 2026, primera producción estimada 2030)</t>
+          <t>Ingeniería/FEED (diseño ~70% completo, USD 315 millones de capital levantado, permisos en proceso; planta de fertilizante nitrato ~0.7 Mt/año, inversión USD 1,100-1,500 millones; debe iniciar construcción antes de fines de 2027 para calificar a créditos fiscales federales; construcción estimada en 36 meses)</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>[The Engineer](https://www.theengineer.co.uk/content/news/abb-joins-team-for-22gw-hydrogen-city-project-in-texas); [Energy Capital HTX](https://energycapitalhtx.com/green-hydrogen-city-abb-mou)</t>
+          <t>[Tri-Cities Area Journal of Business](https://www.tricitiesbusinessnews.com/articles/atlas-agro-plant-nears-decision-point); [Washington State Standard](https://washingtonstatestandard.com/2025/10/30/plan-for-1-5b-fertilizer-plant-in-central-wa-still-alive-despite-loss-of-federal-funds/)</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2022,35 +2022,72 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t>Hydrogen City (complejo Power-to-X / e-metanol)</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Piedras Pintas Salt Dome, Condado de Duval, sur de Texas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Green Hydrogen International (GHI)</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>ABB (automatización/control, vía MOU)</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Ingeniería/FEED (inversión USD 6,000-10,000 millones; electrolizador de 2.2 GW; producirá 1.4 Mt/año de e-metanol y capturará ~2 Mt/año de CO2; construcción planeada desde 2026, primera producción estimada 2030)</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>[The Engineer](https://www.theengineer.co.uk/content/news/abb-joins-team-for-22gw-hydrogen-city-project-in-texas); [Energy Capital HTX](https://energycapitalhtx.com/green-hydrogen-city-abb-mou)</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t>Targa Resources Falcon II Gas Processing Plant</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B45" t="inlineStr">
         <is>
           <t>Cuenca Delaware, Permian Basin, Texas, EE.UU.</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>Targa Resources Corp.</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D45" t="inlineStr">
         <is>
           <t>Targa Resources (propietario-constructor)</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
+      <c r="E45" t="inlineStr">
         <is>
           <t>Construcción/Comisionamiento (planta criogénica 275 MMcf/d; arranque adelantado a 1T2026, dos trimestres antes de lo previsto)</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="F45" t="inlineStr">
         <is>
           <t>[Oil &amp; Gas Journal](https://www.ogj.com/refining-processing/gas-processing/capacities/article/55240691/targa-advances-expansion-plans-for-permian-basin-gas-processing)</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
+      <c r="G45" t="inlineStr">
         <is>
           <t>2026-08-06</t>
         </is>
@@ -2067,15 +2104,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -3556,6 +3593,43 @@
       <c r="G40" t="inlineStr">
         <is>
           <t>2026-08-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Gasoducto TTC Connector (alimenta Freeport LNG)</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Condados de Colorado y Wharton, Texas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Desarrollador: TTC Connector, LLC; opción de compra: Enbridge Inc.; cliente de capacidad: bp</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Construcción (25 millas/300 MMpc/d; en servicio previsto fines de 2026)</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>[LNG Industry](https://www.lngindustry.com/liquid-natural-gas/07082026/enbridge-signs-option-to-acquire-ttc-connector/)</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
@@ -3570,15 +3644,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G70"/>
+  <dimension ref="A1:G77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -6169,6 +6243,265 @@
       <c r="G70" t="inlineStr">
         <is>
           <t>2026-08-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Lone Tree Plant (Refurbishment Autoclave/CIL)</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Lovelock, Nevada, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>i-80 Gold Corp</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Hatch (EPCM)</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Construcción (obras tempranas y movilización de contratistas en curso; construcción mayor prevista 4T2026)</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/i-80-gold-provides-update-on-lone-tree-plant-refurbishment-project-remains-on-schedule-and-on-budget-302836341.html)</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Round Mountain Phase X — Planta de Paste Backfill</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Nye County, Nevada, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Kinross Gold Corporation</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>No especificado (paquetes de equipo móvil, ventiladores y planta CRF ya adjudicados)</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Construcción/Ingeniería detallada</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/29/3335652/0/en/Kinross-reports-strong-2026-second-quarter-results.html)</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Bald Mountain Redbird 2 — Planta SART (ácido/lixiviación)</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>White Pine County, Nevada, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Kinross Gold Corporation</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Contratista de ingeniería detallada ya seleccionado, no revelado en la fuente</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Ingeniería (básica ~50% completa)</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/29/3335652/0/en/Kinross-reports-strong-2026-second-quarter-results.html)</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Bear Lodge Rare Earth Project</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Crook County, Wyoming, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Rare Element Resources Ltd. (afiliada de General Atomics/Synchron)</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Permitting (designación FAST-41; aviso NEPA publicado en Federal Register 29-jul-2026)</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>[Federal Register](https://www.federalregister.gov/documents/2026/07/29/2026-15255/black-hills-national-forest-wyoming-bear-lodge-rare-earth-project)</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Proyecto de Cobre Angangueo</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Angangueo, Michoacán, México</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Southern Copper Corporation (Grupo México)</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Pre-desarrollo (en negociación de permisos con gobierno federal)</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>[Minería en Línea](https://mineriaenlinea.com/2026/07/southern-copper-obtiene-permisos-ambientales-para-el-pilar-produccion-a-partir-de-2029/)</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Proyecto de Cobre Chalchihuites</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Chalchihuites, Zacatecas, México</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Southern Copper Corporation (Grupo México)</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Pre-desarrollo (en negociación de permisos)</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>[Minería en Línea](https://mineriaenlinea.com/2026/07/southern-copper-obtiene-permisos-ambientales-para-el-pilar-produccion-a-partir-de-2029/)</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Modernización Complejo Metalúrgico Empalme</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Empalme, Sonora, México</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Southern Copper Corporation (Grupo México)</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Pre-desarrollo (en negociación de permisos; fundición existente a modernizar)</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>[Minería en Línea](https://mineriaenlinea.com/2026/07/southern-copper-obtiene-permisos-ambientales-para-el-pilar-produccion-a-partir-de-2029/)</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
@@ -6183,15 +6516,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G79"/>
+  <dimension ref="A1:G81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -6578,7 +6911,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Pacifico Energy</t>
+          <t>Pacifico Energy; inquilino confirmado: Amazon (AWS)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -6588,17 +6921,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Permisos obtenidos/inicio construcción (TCEQ otorgó permiso de aire para 7.65GW de generación a gas, el más grande emitido en EE.UU. hasta la fecha; Fase 1 de 1GW prevista en operación 1S2027)</t>
+          <t>Construcción de edificios de centro de datos iniciada (TCEQ ya había otorgado permiso de aire para 7.65GW de generación a gas; Amazon presentó a inicios de ago-2026 permisos de construcción para 3 edificios de centro de datos —"Pecos County Data Center", Buildings A/B/C, ~189,060 pies² c/u, ~US$300M c/u—; construcción de edificios prevista ago-dic 2026; Fase 1 de 1GW de generación prevista en operación 1S2027)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>[Business Wire](https://www.businesswire.com/news/home/20260126236053/en/Pacifico-Energy-Secures-7.65-GW-Power-Generation-Permit-for-GW-Ranch-Project)</t>
+          <t>[Business Wire](https://www.businesswire.com/news/home/20260126236053/en/Pacifico-Energy-Secures-7.65-GW-Power-Generation-Permit-for-GW-Ranch-Project); [US Data Center Projects](https://usdatacenterprojects.com/texas/amazon-files-plans-for-new-data-center-buildings-in-texas-across-three-sites)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
@@ -7994,17 +8327,17 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Construcción DETENIDA (orden de suspensión de la agencia ambiental de Georgia -EPD- por construir sin permisos, 2-jul-2026)</t>
+          <t>Construcción REANUDADA (tras orden de suspensión de la agencia ambiental de Georgia -EPD- del 2-jul-2026 por construir sin permisos; a 31-jul-2026 la construcción de la planta de 90MW está en marcha de nuevo, con 6 de 33 motores a gas ya instalados)</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>[AJC](https://www.ajc.com/business/2026/07/officials-order-georgia-data-centers-pop-up-power-plant-to-halt-construction/)</t>
+          <t>[AJC](https://www.ajc.com/business/2026/07/officials-order-georgia-data-centers-pop-up-power-plant-to-halt-construction/); [Inside Climate News](https://insideclimatenews.org/news/31072026/georgia-data-center-private-power-plant/)</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
@@ -9115,6 +9448,80 @@
       <c r="G79" t="inlineStr">
         <is>
           <t>2026-08-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Galaxy Digital Project Merlin</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>McGregor, Condado de McLennan, Texas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Galaxy Digital</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Planeación/permitting inicial (500 acres adquiridos; acuerdo de desarrollo aprobado por el ayuntamiento de McGregor 24-jun-2026; subestación eléctrica propia en construcción; enfriamiento de circuito cerrado, sin planta de gas on-site confirmada; Fase 1 de 74MW prevista 2028)</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/galaxy-expands-data-center-footprint-with-acquisition-of-500-acre-campus-in-mcgregor-texas-302836014.html)</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Nexus Fulcrum Gas Plant (TRIC)</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Tahoe-Reno Industrial Center, Condado de Storey, Nevada, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Nexus Fulcrum LLC (abastecerá al hub industrial/de centros de datos de TRIC, donde operan Switch, Google, Tract, entre otros)</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Permitting (solicitud regulatoria presentada ante reguladores estatales de energía de Nevada para planta de gas natural de 510MW)</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>[The Nevada Independent](https://thenevadaindependent.com/article/nevada-data-center-rush-drives-request-for-a-novel-type-of-gas-power-plant)</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Agregar 12 proyectos nuevos y 2 cambios de fase (2026-08-10) (#19)
Nuevos: Gasoducto TTC Connector (LNG); Lone Tree Plant, Round Mountain
Phase X, Bald Mountain Redbird 2, Bear Lodge Rare Earth, Cobre
Angangueo, Cobre Chalchihuites, Modernización Empalme (Mining);
Galaxy Digital Project Merlin, Nexus Fulcrum Gas Plant (Data
Centers). Actualizaciones de fase: GW Ranch Power Campus (Amazon
confirmado como inquilino), VoltaGrid/Serverfarm Covington
(construcción reanudada).


Claude-Session: https://claude.ai/code/session_01ArQ4Pz8sq54DrJPjfCETqj

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -416,15 +416,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -801,217 +801,217 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Rehab. Fertinal-ProAgro (urea y fosfatos)</t>
+          <t>Proyecto Escolín (amoniaco/urea)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Lázaro Cárdenas, Michoacán, México</t>
+          <t>Poza Rica, Veracruz, México</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Pemex</t>
+          <t>Pemex Transformación Industrial</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Mota-Engil México (EPC confirmado; plazo de construcción 33 meses)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Ingeniería/rehabilitación (incorporado al plan de reactivación petroquímica de Pemex, jun-2026; 13,700 millones de pesos asignados para los complejos Lázaro Cárdenas y ProAgro; meta de 2.4 millones ton/año de urea y fertilizantes fosfatados)</t>
+          <t>Ingeniería/inicio de construcción (inversión confirmada US$1,553 millones)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>[Tribuna](https://tribuna.com.mx/mexico/2026/06/05/sheinbaum-anuncia-inversion-de-93-mil-mdp-para-reactivar-la-industria-petroquimica-y-de-fertilizantes-en-veracruz_560837/); [Contralínea](https://contralinea.com.mx/interno/semana/presentan-plan-con-inversion-de-93-mil-mdp-para-rescatar-la-petroquimica-nacional/)</t>
+          <t>[Forbes México](https://forbes.com.mx/asi-es-la-inversion-de-1553-mdd-por-parte-de-pemex-en-una-planta-de-fertilizantes-en-veracruz/)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Pacífico Mexinol (metanol ultra bajo carbono)</t>
+          <t>Rehab. Fertinal-ProAgro (urea y fosfatos)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Topolobampo, Sinaloa, México</t>
+          <t>Lázaro Cárdenas, Michoacán, México</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Transition Industries</t>
+          <t>Pemex</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Siemens Energy / Techint E&amp;C (FEED electrolizador)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Construcción (iniciada abr-2026)</t>
+          <t>Ingeniería/rehabilitación (incorporado al plan de reactivación petroquímica de Pemex, jun-2026; 13,700 millones de pesos asignados para los complejos Lázaro Cárdenas y ProAgro; meta de 2.4 millones ton/año de urea y fertilizantes fosfatados)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>[PV Magazine México](https://www.pv-magazine-mexico.com/2026/04/28/inician-en-sinaloa-la-construccion-de-la-mayor-planta-de-metanol-ultrabajo-en-carbono-a-partir-de-hidrogeno-verde/)</t>
+          <t>[Tribuna](https://tribuna.com.mx/mexico/2026/06/05/sheinbaum-anuncia-inversion-de-93-mil-mdp-para-reactivar-la-industria-petroquimica-y-de-fertilizantes-en-veracruz_560837/); [Contralínea](https://contralinea.com.mx/interno/semana/presentan-plan-con-inversion-de-93-mil-mdp-para-rescatar-la-petroquimica-nacional/)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>First Ammonia (amoniaco verde)</t>
+          <t>Pacífico Mexinol (metanol ultra bajo carbono)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Victoria, Texas, EE.UU.</t>
+          <t>Topolobampo, Sinaloa, México</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>First Ammonia / Cox Group USA</t>
+          <t>Transition Industries</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Worley (FEED)</t>
+          <t>Siemens Energy / Techint E&amp;C (FEED electrolizador)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Ingeniería (FEED completo) / FID prevista 2026</t>
+          <t>Construcción (iniciada abr-2026)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>[H2 View](https://www.h2-view.com/story/first-ammonia-project-on-track-for-2026-fid-despite-topsoe-deal-collapse/2138792.article/)</t>
+          <t>[PV Magazine México](https://www.pv-magazine-mexico.com/2026/04/28/inician-en-sinaloa-la-construccion-de-la-mayor-planta-de-metanol-ultrabajo-en-carbono-a-partir-de-hidrogeno-verde/)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-10</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Planta de Amoniaco Topolobampo (GPO)</t>
+          <t>First Ammonia (amoniaco verde)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Topolobampo, Sinaloa, México</t>
+          <t>Victoria, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Gas y Petroquímica de Occidente (GPO) / Proman AG</t>
+          <t>First Ammonia / Cox Group USA</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Worley (FEED)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Construcción (avance ~80% confirmado por Secretaría de Economía jul-2026; op. comercial H1 2027)</t>
+          <t>Ingeniería (FEED completo) / FID prevista 2026</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>[Debate](https://www.debate.com.mx/economia/secretaria-de-economia-complejo-de-amoniaco-en-topolobampo-prioritario-para-el-gobierno-de-mexico-20260713-0092.html)</t>
+          <t>[H2 View](https://www.h2-view.com/story/first-ammonia-project-on-track-for-2026-fid-despite-topsoe-deal-collapse/2138792.article/)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Lake Charles Methanol II</t>
+          <t>Planta de Amoniaco Topolobampo (GPO)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Lake Charles, Luisiana, EE.UU.</t>
+          <t>Topolobampo, Sinaloa, México</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Lake Charles Methanol II LLC</t>
+          <t>Gas y Petroquímica de Occidente (GPO) / Proman AG</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Zachry Group (FEED)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Ingeniería (FEED) / FID prevista</t>
+          <t>Construcción (avance ~80% confirmado por Secretaría de Economía jul-2026; op. comercial H1 2027)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>[ICIS](https://www.icis.com/explore/resources/news/2025/11/13/11155109/lake-charles-methanol-ii-awards-feed-fid-expected-in-q2-2026/)</t>
+          <t>[Debate](https://www.debate.com.mx/economia/secretaria-de-economia-complejo-de-amoniaco-en-topolobampo-prioritario-para-el-gobierno-de-mexico-20260713-0092.html)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Planta Coquizadora Salina Cruz</t>
+          <t>Lake Charles Methanol II</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Salina Cruz, Oaxaca, México</t>
+          <t>Lake Charles, Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Pemex</t>
+          <t>Lake Charles Methanol II LLC</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>ICA Fluor</t>
+          <t>Zachry Group (FEED)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Construcción (~74% avance)</t>
+          <t>Ingeniería (FEED) / FID prevista</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>[Diario del Istmo](https://diariodelistmo.com/nacional/este-es-el-avance-que-lleva-la-planta-coquizadora-en-la-refineria-de-salina-cruz/50642321)</t>
+          <t>[ICIS](https://www.icis.com/explore/resources/news/2025/11/13/11155109/lake-charles-methanol-ii-awards-feed-fid-expected-in-q2-2026/)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1023,54 +1023,54 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Shintech Louisiana — Expansión Plaquemine (2do craqueador de etileno + 4ta unidad cloro-álcali/VCM)</t>
+          <t>Planta Coquizadora Salina Cruz</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Plaquemine, Iberville Parish, Luisiana, EE.UU.</t>
+          <t>Salina Cruz, Oaxaca, México</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Shintech Louisiana, LLC</t>
+          <t>Pemex</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>ICA Fluor</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Ingeniería/planeación (construcción por fases, 1a fase prevista 2030)</t>
+          <t>Construcción (~74% avance)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/petrochemicals/06032026/shintech-announces-us34-billion-at-louisiana-petrochemicals-complex/)</t>
+          <t>[Diario del Istmo](https://diariodelistmo.com/nacional/este-es-el-avance-que-lleva-la-planta-coquizadora-en-la-refineria-de-salina-cruz/50642321)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Sandpiper Chemicals (metanol bajo carbono)</t>
+          <t>Shintech Louisiana — Expansión Plaquemine (2do craqueador de etileno + 4ta unidad cloro-álcali/VCM)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Texas City, Texas, EE.UU.</t>
+          <t>Plaquemine, Iberville Parish, Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Sandpiper Chemicals, LLC / INEOS Acetyls (colaboración estratégica, abr-2026)</t>
+          <t>Shintech Louisiana, LLC</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1080,86 +1080,86 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Ingeniería (FEED en curso desde 2T2026; US$1,700 millones, 1.1 MMtpa; INEOS Acetyls tomará 300,000 ton/año para su unidad de ácido acético) / FID prevista 2027, primera producción ~2030</t>
+          <t>Ingeniería/planeación (construcción por fases, 1a fase prevista 2030)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>[INEOS](https://www.ineos.com/news/shared-news/ineos-acetyls-and-sandpiper-chemicals-announce-strategic-collaboration-for-the-development-of-a-low-carbon-methanol-project-in-texas-city-texas/)</t>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/petrochemicals/06032026/shintech-announces-us34-billion-at-louisiana-petrochemicals-complex/)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-14</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>OXEA Bay City Capacity Expansion + Air Liquide POX Syngas Unit</t>
+          <t>Sandpiper Chemicals (metanol bajo carbono)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Bay City, Matagorda County, Texas, EE.UU.</t>
+          <t>Texas City, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>OXEA (oxo chemicals) / Air Liquide (unidad de syngas)</t>
+          <t>Sandpiper Chemicals, LLC / INEOS Acetyls (colaboración estratégica, abr-2026)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Air Liquide (unidad propia); OXEA no especificado</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Construcción (FID confirmado 13-jul-2026; preparación de sitio 3T2026; finalización fines de 2028)</t>
+          <t>Ingeniería (FEED en curso desde 2T2026; US$1,700 millones, 1.1 MMtpa; INEOS Acetyls tomará 300,000 ton/año para su unidad de ácido acético) / FID prevista 2027, primera producción ~2030</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/petrochemicals/13072026/oxea-confirms-fid-for-major-capacity-expansion/)</t>
+          <t>[INEOS](https://www.ineos.com/news/shared-news/ineos-acetyls-and-sandpiper-chemicals-announce-strategic-collaboration-for-the-development-of-a-low-carbon-methanol-project-in-texas-city-texas/)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-29</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Targa Resources East Driver Gas Processing Plant</t>
+          <t>OXEA Bay City Capacity Expansion + Air Liquide POX Syngas Unit</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Condado de Midland, Texas, EE.UU.</t>
+          <t>Bay City, Matagorda County, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Targa Resources Corp.</t>
+          <t>OXEA (oxo chemicals) / Air Liquide (unidad de syngas)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Targa Resources (propietario-constructor)</t>
+          <t>Air Liquide (unidad propia); OXEA no especificado</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Construcción (planta criogénica 275 MMcf/d; arranque previsto 3T2026)</t>
+          <t>Construcción (FID confirmado 13-jul-2026; preparación de sitio 3T2026; finalización fines de 2028)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>[OGJ](https://www.ogj.com/refining-processing/gas-processing/news/55320579/targa-advances-permian-gas-pipeline-processing-expansion)</t>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/petrochemicals/13072026/oxea-confirms-fid-for-major-capacity-expansion/)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1171,32 +1171,32 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Enterprise Products "Athena" Natural Gas Processing Plant</t>
+          <t>Targa Resources East Driver Gas Processing Plant</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Cuenca Midland (cuatro condados), Texas, EE.UU.</t>
+          <t>Condado de Midland, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Enterprise Products Partners L.P.</t>
+          <t>Targa Resources Corp.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Enterprise Products (propietario-constructor)</t>
+          <t>Targa Resources (propietario-constructor)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Construcción (300 MMcf/d + hasta 40,000 bpd de NGLs; en servicio 4T2026)</t>
+          <t>Construcción (planta criogénica 275 MMcf/d; arranque previsto 3T2026)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>[Business Wire](https://www.businesswire.com/news/home/20250806663187/en/Enterprise-Agrees-to-Acquire-Occidentals-Gas-Gathering-Affiliate-Enters-Into-Natural-Gas-Processing-Agreement-Announces-New-Midland-Basin-Natural-Gas-Processing-Plant)</t>
+          <t>[OGJ](https://www.ogj.com/refining-processing/gas-processing/news/55320579/targa-advances-permian-gas-pipeline-processing-expansion)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1208,32 +1208,32 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>MPLX Secretariat II Gas Processing Plant</t>
+          <t>Enterprise Products "Athena" Natural Gas Processing Plant</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Cuenca Pérmica (subcuenca Delaware), Texas/Nuevo México, EE.UU.</t>
+          <t>Cuenca Midland (cuatro condados), Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>MPLX LP</t>
+          <t>Enterprise Products Partners L.P.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>MPLX (propietario-constructor)</t>
+          <t>Enterprise Products (propietario-constructor)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Planeada/desarrollo (300 MMcf/d; en servicio 2S2028)</t>
+          <t>Construcción (300 MMcf/d + hasta 40,000 bpd de NGLs; en servicio 4T2026)</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>[Natural Gas Intel](https://naturalgasintel.com/news/mplx-scales-up-for-power-hungry-future-with-natural-gas-focused-growth-plan/)</t>
+          <t>[Business Wire](https://www.businesswire.com/news/home/20250806663187/en/Enterprise-Agrees-to-Acquire-Occidentals-Gas-Gathering-Affiliate-Enters-Into-Natural-Gas-Processing-Agreement-Announces-New-Midland-Basin-Natural-Gas-Processing-Plant)</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1245,12 +1245,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>MPLX Titan Complex (Northwind) — Expansión de Tratamiento de Gas Amargo</t>
+          <t>MPLX Secretariat II Gas Processing Plant</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Condado de Lea, Nuevo México / frontera TX-NM, EE.UU.</t>
+          <t>Cuenca Pérmica (subcuenca Delaware), Texas/Nuevo México, EE.UU.</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1265,12 +1265,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Construcción (expansión de capacidad &gt;400 MMcf/d; plenamente operativo 4T2026)</t>
+          <t>Planeada/desarrollo (300 MMcf/d; en servicio 2S2028)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>[East Daley](https://eastdaley.com/daley-note/mplx-acquires-northwind-for-2-375b-acquires-more-ngls-for-jv-project)</t>
+          <t>[Natural Gas Intel](https://naturalgasintel.com/news/mplx-scales-up-for-power-hungry-future-with-natural-gas-focused-growth-plan/)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1282,32 +1282,32 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Northern Plains Nitrogen (urea/amoniaco)</t>
+          <t>MPLX Titan Complex (Northwind) — Expansión de Tratamiento de Gas Amargo</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Grand Forks, Dakota del Norte, EE.UU.</t>
+          <t>Condado de Lea, Nuevo México / frontera TX-NM, EE.UU.</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Northern Plains Nitrogen LLC</t>
+          <t>MPLX LP</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>EPC no designado</t>
+          <t>MPLX (propietario-constructor)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Pre-FEED completo / FID buscada 4T2026</t>
+          <t>Construcción (expansión de capacidad &gt;400 MMcf/d; plenamente operativo 4T2026)</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>[Grand Forks Herald](https://www.grandforksherald.com/news/local/northern-plains-nitrogen-proposal-receiving-more-attention-amid-global-fertilizer-pressure)</t>
+          <t>[East Daley](https://eastdaley.com/daley-note/mplx-acquires-northwind-for-2-375b-acquires-more-ngls-for-jv-project)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1319,54 +1319,54 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Iron Mesa (planta de gas)</t>
+          <t>Northern Plains Nitrogen (urea/amoniaco)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Goldsmith, Ector County, Texas, EE.UU.</t>
+          <t>Grand Forks, Dakota del Norte, EE.UU.</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Phillips 66</t>
+          <t>Northern Plains Nitrogen LLC</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>EPC no designado</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Construcción (arranque previsto Q1 2027)</t>
+          <t>Pre-FEED completo / FID buscada 4T2026</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>[Phillips 66](https://www.phillips66.com/newsroom/iron-mesa-safely-enters-next-phase-of-construction/)</t>
+          <t>[Grand Forks Herald](https://www.grandforksherald.com/news/local/northern-plains-nitrogen-proposal-receiving-more-attention-amid-global-fertilizer-pressure)</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Yeti II (planta de gas)</t>
+          <t>Iron Mesa (planta de gas)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Cuenca Delaware (Permian), Texas/Nuevo México, EE.UU.</t>
+          <t>Goldsmith, Ector County, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Targa Resources</t>
+          <t>Phillips 66</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1376,12 +1376,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Ingeniería/planeación (en línea previsto Q4 2027)</t>
+          <t>Construcción (arranque previsto Q1 2027)</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>[Targa Resources](https://www.targaresources.com/news-releases/news-release-details/targa-resources-corp-announces-permian-growth-projects-and)</t>
+          <t>[Phillips 66](https://www.phillips66.com/newsroom/iron-mesa-safely-enters-next-phase-of-construction/)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1393,32 +1393,32 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Refinería Francisco I. Madero (rehabilitación)</t>
+          <t>Yeti II (planta de gas)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Ciudad Madero, Tamaulipas, México</t>
+          <t>Cuenca Delaware (Permian), Texas/Nuevo México, EE.UU.</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Pemex</t>
+          <t>Targa Resources</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Múltiples contratistas por licitar (30+ licitaciones)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Licitación/bidding</t>
+          <t>Ingeniería/planeación (en línea previsto Q4 2027)</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>[Elefante Blanco](https://elefanteblanco.mx/2026/01/02/pemex-abre-30-licitaciones-para-obras-en-la-refineria-madero/)</t>
+          <t>[Targa Resources](https://www.targaresources.com/news-releases/news-release-details/targa-resources-corp-announces-permian-growth-projects-and)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1430,69 +1430,69 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Fermachem Planta de Urea/Amoniaco</t>
+          <t>Refinería Francisco I. Madero (rehabilitación)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Ejido Sapioris, Lerdo, Durango, México</t>
+          <t>Ciudad Madero, Tamaulipas, México</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Fermaca Dreams (Fermachem)</t>
+          <t>Pemex</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Técnicas Reunidas (licencia/tecnología KBR-Stamicarbon)</t>
+          <t>Múltiples contratistas por licitar (30+ licitaciones)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Construcción (ejecución iniciada jun-2026)</t>
+          <t>Licitación/bidding</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>[La Jornada](https://www.jornada.com.mx/noticia/2026/06/08/economia/da-inicio-ejecucion-de-planta-de-fertilizantes-en-durango-por-parte-de-fermachem)</t>
+          <t>[Elefante Blanco](https://elefanteblanco.mx/2026/01/02/pemex-abre-30-licitaciones-para-obras-en-la-refineria-madero/)</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-15</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Ascension Clean Energy (ACE) — amoniaco azul</t>
+          <t>Fermachem Planta de Urea/Amoniaco</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Donaldsonville, Ascension Parish, Luisiana, EE.UU.</t>
+          <t>Ejido Sapioris, Lerdo, Durango, México</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Clean Hydrogen Works</t>
+          <t>Fermaca Dreams (Fermachem)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>McDermott (FEED)</t>
+          <t>Técnicas Reunidas (licencia/tecnología KBR-Stamicarbon)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Ingeniería (FEED) / Pre-FID</t>
+          <t>Construcción (ejecución iniciada jun-2026)</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>[Downstream Calendar](https://downstreamcalendar.com/mcdermott-secures-feed-contract-for-ascension-clean-energy-project/)</t>
+          <t>[La Jornada](https://www.jornada.com.mx/noticia/2026/06/08/economia/da-inicio-ejecucion-de-planta-de-fertilizantes-en-durango-por-parte-de-fermachem)</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1504,32 +1504,32 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Zeus Gas Plant + 3ra Fraccionadora Coastal Bend</t>
+          <t>Ascension Clean Energy (ACE) — amoniaco azul</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Cuenca Pérmica, Texas / Robstown, Texas, EE.UU.</t>
+          <t>Donaldsonville, Ascension Parish, Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Phillips 66</t>
+          <t>Clean Hydrogen Works</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>McDermott (FEED)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Ingeniería (sancionado; en línea 2028)</t>
+          <t>Ingeniería (FEED) / Pre-FID</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>[Business Wire](https://www.businesswire.com/news/home/20260517310811/en/Phillips-66-announces-Zeus-Gas-Plant-and-a-third-Coastal-Bend-Fractionator)</t>
+          <t>[Downstream Calendar](https://downstreamcalendar.com/mcdermott-secures-feed-contract-for-ascension-clean-energy-project/)</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1541,128 +1541,128 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Project Meadowlark (complejo de amoniaco azul/UAN/ATS/DEF)</t>
+          <t>Zeus Gas Plant + 3ra Fraccionadora Coastal Bend</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Gothenburg, Nebraska, EE.UU.</t>
+          <t>Cuenca Pérmica, Texas / Robstown, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>J. Westling &amp; Co. (JWC Gburg, LLC)</t>
+          <t>Phillips 66</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>No especificado (tecnología licenciada Topsoe SynCOR Ammonia); contrato EPC/fabricación asegurado</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Ingeniería/Permisos (permiso de aire emitido, sitio zonificado; obras civiles previstas 2027, operación comercial 2029)</t>
+          <t>Ingeniería (sancionado; en línea 2028)</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>[USDA](https://www.usda.gov/about-usda/news/press-releases/2026/07/01/secretary-rollins-announces-500-million-fertilizer-investment-and-expansion-program-strengthen)</t>
+          <t>[Business Wire](https://www.businesswire.com/news/home/20260517310811/en/Phillips-66-announces-Zeus-Gas-Plant-and-a-third-Coastal-Bend-Fractionator)</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-17</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Wabash Low-Carbon Ammonia Project</t>
+          <t>Project Meadowlark (complejo de amoniaco azul/UAN/ATS/DEF)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>West Terre Haute, Indiana, EE.UU.</t>
+          <t>Gothenburg, Nebraska, EE.UU.</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Wabash Valley Resources</t>
+          <t>J. Westling &amp; Co. (JWC Gburg, LLC)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Samsung E&amp;C (contrato EPF ~US$475 millones)</t>
+          <t>No especificado (tecnología licenciada Topsoe SynCOR Ammonia); contrato EPC/fabricación asegurado</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Construcción (groundbreaking 5-ene-2026; amoniaco bajo en carbono 500,000 ton/año con captura de 1.67 millones ton CO2/año; meta de finalización 2029)</t>
+          <t>Ingeniería/Permisos (permiso de aire emitido, sitio zonificado; obras civiles previstas 2027, operación comercial 2029)</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/clean-fuels/06012026/samsung-ea-announces-groundbreaking-of-low-carbon-ammonia-plant/)</t>
+          <t>[USDA](https://www.usda.gov/about-usda/news/press-releases/2026/07/01/secretary-rollins-announces-500-million-fertilizer-investment-and-expansion-program-strengthen)</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Green Fuels Operating — Refinería Duncan</t>
+          <t>Wabash Low-Carbon Ammonia Project</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Duncan, Stephens County, Oklahoma, EE.UU.</t>
+          <t>West Terre Haute, Indiana, EE.UU.</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Green Fuels Operating</t>
+          <t>Wabash Valley Resources</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Samsung E&amp;C (contrato EPF ~US$475 millones)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Construcción (groundbreaking 29-may-2026; inversión US$400 millones; capacidad inicial 30,000 bbl/d, expandible a 50,000 bbl/d, sobre sitio de refinería histórica de los años 1920)</t>
+          <t>Construcción (groundbreaking 5-ene-2026; amoniaco bajo en carbono 500,000 ton/año con captura de 1.67 millones ton CO2/año; meta de finalización 2029)</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/refining/03062026/green-fuels-hosts-groundbreaking-ceremony-for-new-refinery/)</t>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/clean-fuels/06012026/samsung-ea-announces-groundbreaking-of-low-carbon-ammonia-plant/)</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-24</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Energy Transfer Mustang Draw I &amp; II (plantas de gas)</t>
+          <t>Green Fuels Operating — Refinería Duncan</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Cuenca Midland, Texas, EE.UU.</t>
+          <t>Duncan, Stephens County, Oklahoma, EE.UU.</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Energy Transfer LP</t>
+          <t>Green Fuels Operating</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1672,34 +1672,34 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Construcción (Mustang Draw I en comisionamiento, servicio pleno ~jun-2026; Mustang Draw II en construcción, en servicio 4T2026; 275 MMcf/d cada una)</t>
+          <t>Construcción (groundbreaking 29-may-2026; inversión US$400 millones; capacidad inicial 30,000 bbl/d, expandible a 50,000 bbl/d, sobre sitio de refinería histórica de los años 1920)</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>[Energy Transfer](https://www.energytransfer.com/project-highlights/)</t>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/refining/03062026/green-fuels-hosts-groundbreaking-ceremony-for-new-refinery/)</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ONEOK Bighorn / Cutter / Shadowfax (plantas de gas)</t>
+          <t>Energy Transfer Mustang Draw I &amp; II (plantas de gas)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Cuenca Delaware (Bighorn), Texas / Cuenca Powder River (Cutter), Wyoming / Cuenca Midland (Shadowfax reubicada), Texas, EE.UU.</t>
+          <t>Cuenca Midland, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ONEOK Inc.</t>
+          <t>Energy Transfer LP</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1709,12 +1709,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Construcción (Bighorn US$365 millones/300 MMcf/d tratamiento alto CO2, meta mediados 2027; Cutter 60 MMcf/d en construcción, meta 4T2026; Shadowfax 150 MMcf/d reubicación completada 1T2026, en rampa)</t>
+          <t>Construcción (Mustang Draw I en comisionamiento, servicio pleno ~jun-2026; Mustang Draw II en construcción, en servicio 4T2026; 275 MMcf/d cada una)</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>[Inspectioneering](https://inspectioneering.com/news/2025-08-07/11702/oneok-greenlights-new-365m-delaware-basin-gas-plant)</t>
+          <t>[Energy Transfer](https://www.energytransfer.com/project-highlights/)</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1726,32 +1726,32 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>MPLX Harmon Creek III (planta de gas + de-etanizadora)</t>
+          <t>ONEOK Bighorn / Cutter / Shadowfax (plantas de gas)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Región Marcellus/Utica, noreste de EE.UU. (ubicación exacta no especificada)</t>
+          <t>Cuenca Delaware (Bighorn), Texas / Cuenca Powder River (Cutter), Wyoming / Cuenca Midland (Shadowfax reubicada), Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>MPLX LP</t>
+          <t>ONEOK Inc.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>MPLX (propietario-constructor)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Construcción (300 MMcf/d + de-etanizadora 40 Mbpd; en servicio 3T2026)</t>
+          <t>Construcción (Bighorn US$365 millones/300 MMcf/d tratamiento alto CO2, meta mediados 2027; Cutter 60 MMcf/d en construcción, meta 4T2026; Shadowfax 150 MMcf/d reubicación completada 1T2026, en rampa)</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>[Natural Gas Intel](https://www.naturalgasintel.com/news/mplx-scales-up-for-power-hungry-future-with-natural-gas-focused-growth-plan/)</t>
+          <t>[Inspectioneering](https://inspectioneering.com/news/2025-08-07/11702/oneok-greenlights-new-365m-delaware-basin-gas-plant)</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1763,86 +1763,86 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Rehab. Complejo Cosoleacaque (amoniaco) + Complejo Morelos (etano-etileno)</t>
+          <t>MPLX Harmon Creek III (planta de gas + de-etanizadora)</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Cosoleacaque y Complejo Morelos, Veracruz, México</t>
+          <t>Región Marcellus/Utica, noreste de EE.UU. (ubicación exacta no especificada)</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Pemex Transformación Industrial</t>
+          <t>MPLX LP</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Mota-Engil México (plantas VI/VII y TASP Pajaritos); ICA (paquete relacionado)</t>
+          <t>MPLX (propietario-constructor)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Ingeniería/planeación (parte del plan de reactivación petroquímica de Pemex de 93,000 mdp anunciado jun-2026; 13,000 mdp para 2 plantas de amoniaco en Cosoleacaque, meta 957,000 ton/año; Complejo Morelos incluido en programa de rehabilitación etano-etileno de 30,000 mdp/5 plantas, meta 520,000 ton/año de polietilenos/óxido de etileno/glicoles; contratos de rehabilitación y confiabilidad adjudicados dic-2025, confirmados ene-2026)</t>
+          <t>Construcción (300 MMcf/d + de-etanizadora 40 Mbpd; en servicio 3T2026)</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>[Contralínea](https://contralinea.com.mx/interno/semana/presentan-plan-con-inversion-de-93-mil-mdp-para-rescatar-la-petroquimica-nacional/); [El Diario de Juárez](https://diario.mx/nacional/2026/jan/22/adjudica-pemex-contratos-a-favoritas-1102601.html)</t>
+          <t>[Natural Gas Intel](https://www.naturalgasintel.com/news/mplx-scales-up-for-power-hungry-future-with-natural-gas-focused-growth-plan/)</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-07-29</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Enterprise Products — Nuevas Plantas de Gas Permian (Plant 11 Midland / Plant 13 Delaware) + NGL Frac 15 Mont Belvieu</t>
+          <t>Rehab. Complejo Cosoleacaque (amoniaco) + Complejo Morelos (etano-etileno)</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Cuenca Midland y Cuenca Delaware, Texas, EE.UU. / Mont Belvieu, Texas, EE.UU.</t>
+          <t>Cosoleacaque y Complejo Morelos, Veracruz, México</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Enterprise Products Partners L.P.</t>
+          <t>Pemex Transformación Industrial</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Enterprise Products (propietario-constructor)</t>
+          <t>Mota-Engil México (plantas VI/VII y TASP Pajaritos); ICA (paquete relacionado)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Construcción (sancionadas/aprobadas en resultados 2T2026: Plant 11 Midland Basin 300 MMcf/d en servicio 1T2029; Plant 13 Delaware Basin 300 MMcf/d en servicio 3T2028; NGL Frac 15 en Mont Belvieu 150 MBPD en servicio 1T2028; gasto de capital de crecimiento 2026 aumentado en más de US$700 millones por estas sanciones)</t>
+          <t>Ingeniería/planeación (parte del plan de reactivación petroquímica de Pemex de 93,000 mdp anunciado jun-2026; 13,000 mdp para 2 plantas de amoniaco en Cosoleacaque, meta 957,000 ton/año; Complejo Morelos incluido en programa de rehabilitación etano-etileno de 30,000 mdp/5 plantas, meta 520,000 ton/año de polietilenos/óxido de etileno/glicoles; contratos de rehabilitación y confiabilidad adjudicados dic-2025, confirmados ene-2026)</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>[Enterprise Reports Second Quarter 2026 Earnings](https://ir.enterpriseproducts.com/news-releases/news-release-details/enterprise-reports-second-quarter-2026-earnings)</t>
+          <t>[Contralínea](https://contralinea.com.mx/interno/semana/presentan-plan-con-inversion-de-93-mil-mdp-para-rescatar-la-petroquimica-nacional/); [El Diario de Juárez](https://diario.mx/nacional/2026/jan/22/adjudica-pemex-contratos-a-favoritas-1102601.html)</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-06</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Enterprise Products — Plant 12 (Delaware Basin) y Athena 2 (Midland Basin)</t>
+          <t>Enterprise Products — Nuevas Plantas de Gas Permian (Plant 11 Midland / Plant 13 Delaware) + NGL Frac 15 Mont Belvieu</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Cuenca Delaware y Cuenca Midland, Texas, EE.UU.</t>
+          <t>Cuenca Midland y Cuenca Delaware, Texas, EE.UU. / Mont Belvieu, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1857,7 +1857,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Construcción (sancionadas, divulgadas en resultados 2T2026 el 30-jul-2026; Plant 12 Delaware Basin ~300 MMcf/d en servicio 4T2027; Athena 2 Midland Basin en servicio 3T2027)</t>
+          <t>Construcción (sancionadas/aprobadas en resultados 2T2026: Plant 11 Midland Basin 300 MMcf/d en servicio 1T2029; Plant 13 Delaware Basin 300 MMcf/d en servicio 3T2028; NGL Frac 15 en Mont Belvieu 150 MBPD en servicio 1T2028; gasto de capital de crecimiento 2026 aumentado en más de US$700 millones por estas sanciones)</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -1867,39 +1867,39 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-07-31</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Targa Resources Roadrunner III / Copperhead II (plantas de gas)</t>
+          <t>Enterprise Products — Plant 12 (Delaware Basin) y Athena 2 (Midland Basin)</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Cuenca Delaware (Permian), Texas/Nuevo México, EE.UU.</t>
+          <t>Cuenca Delaware y Cuenca Midland, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Targa Resources Corp.</t>
+          <t>Enterprise Products Partners L.P.</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Targa Resources (propietario-constructor)</t>
+          <t>Enterprise Products (propietario-constructor)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Construcción (aprobadas may-2026; Roadrunner III 265 MMcf/d, Copperhead II 275 MMcf/d; en servicio previsto 1T2028)</t>
+          <t>Construcción (sancionadas, divulgadas en resultados 2T2026 el 30-jul-2026; Plant 12 Delaware Basin ~300 MMcf/d en servicio 4T2027; Athena 2 Midland Basin en servicio 3T2027)</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>[PGJ](https://pgjonline.com/news/2026/may/targa-expands-permian-gas-processing-delaware-express-pipeline-capacity)</t>
+          <t>[Enterprise Reports Second Quarter 2026 Earnings](https://ir.enterpriseproducts.com/news-releases/news-release-details/enterprise-reports-second-quarter-2026-earnings)</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -1911,54 +1911,54 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Southern Energy Renewables — Complejo de Metanol y SAF</t>
+          <t>Targa Resources Roadrunner III / Copperhead II (plantas de gas)</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>St. Charles Parish (Killona), Luisiana, EE.UU.</t>
+          <t>Cuenca Delaware (Permian), Texas/Nuevo México, EE.UU.</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Southern Energy Renewables</t>
+          <t>Targa Resources Corp.</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Targa Resources (propietario-constructor)</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Planeación/pre-construcción (inversión US$1,400 millones; convierte biomasa de desecho de madera en metanol verde y combustible de aviación sostenible; construcción prevista a iniciar fines de 2027, producción prevista fines de 2029)</t>
+          <t>Construcción (aprobadas may-2026; Roadrunner III 265 MMcf/d, Copperhead II 275 MMcf/d; en servicio previsto 1T2028)</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>[Hydrocarbon Processing](https://www.hydrocarbonprocessing.com/news/2026/03/southern-energy-renewables-announce-14-b-methanol-and-saf-complex-in-louisiana/); [Louisiana Economic Development](https://www.opportunitylouisiana.gov/news/southern-energy-renewables-announce-1-4-billion-methanol-and-sustainable-aviation-fuel-facility-in-st-charles-parish)</t>
+          <t>[PGJ](https://pgjonline.com/news/2026/may/targa-expands-permian-gas-processing-delaware-express-pipeline-capacity)</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-03</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Atlas Agro — Pacific Green Fertilizer Plant</t>
+          <t>Southern Energy Renewables — Complejo de Metanol y SAF</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Richland, Washington, EE.UU.</t>
+          <t>St. Charles Parish (Killona), Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Atlas Agro</t>
+          <t>Southern Energy Renewables</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1968,49 +1968,49 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Ingeniería/FEED (diseño ~70% completo, USD 315 millones de capital levantado, permisos en proceso; planta de fertilizante nitrato ~0.7 Mt/año, inversión USD 1,100-1,500 millones; debe iniciar construcción antes de fines de 2027 para calificar a créditos fiscales federales; construcción estimada en 36 meses)</t>
+          <t>Planeación/pre-construcción (inversión US$1,400 millones; convierte biomasa de desecho de madera en metanol verde y combustible de aviación sostenible; construcción prevista a iniciar fines de 2027, producción prevista fines de 2029)</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>[Tri-Cities Area Journal of Business](https://www.tricitiesbusinessnews.com/articles/atlas-agro-plant-nears-decision-point); [Washington State Standard](https://washingtonstatestandard.com/2025/10/30/plan-for-1-5b-fertilizer-plant-in-central-wa-still-alive-despite-loss-of-federal-funds/)</t>
+          <t>[Hydrocarbon Processing](https://www.hydrocarbonprocessing.com/news/2026/03/southern-energy-renewables-announce-14-b-methanol-and-saf-complex-in-louisiana/); [Louisiana Economic Development](https://www.opportunitylouisiana.gov/news/southern-energy-renewables-announce-1-4-billion-methanol-and-sustainable-aviation-fuel-facility-in-st-charles-parish)</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-04</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Hydrogen City (complejo Power-to-X / e-metanol)</t>
+          <t>Atlas Agro — Pacific Green Fertilizer Plant</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Piedras Pintas Salt Dome, Condado de Duval, sur de Texas, EE.UU.</t>
+          <t>Richland, Washington, EE.UU.</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Green Hydrogen International (GHI)</t>
+          <t>Atlas Agro</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>ABB (automatización/control, vía MOU)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Ingeniería/FEED (inversión USD 6,000-10,000 millones; electrolizador de 2.2 GW; producirá 1.4 Mt/año de e-metanol y capturará ~2 Mt/año de CO2; construcción planeada desde 2026, primera producción estimada 2030)</t>
+          <t>Ingeniería/FEED (diseño ~70% completo, USD 315 millones de capital levantado, permisos en proceso; planta de fertilizante nitrato ~0.7 Mt/año, inversión USD 1,100-1,500 millones; debe iniciar construcción antes de fines de 2027 para calificar a créditos fiscales federales; construcción estimada en 36 meses)</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>[The Engineer](https://www.theengineer.co.uk/content/news/abb-joins-team-for-22gw-hydrogen-city-project-in-texas); [Energy Capital HTX](https://energycapitalhtx.com/green-hydrogen-city-abb-mou)</t>
+          <t>[Tri-Cities Area Journal of Business](https://www.tricitiesbusinessnews.com/articles/atlas-agro-plant-nears-decision-point); [Washington State Standard](https://washingtonstatestandard.com/2025/10/30/plan-for-1-5b-fertilizer-plant-in-central-wa-still-alive-despite-loss-of-federal-funds/)</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2022,35 +2022,72 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t>Hydrogen City (complejo Power-to-X / e-metanol)</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Piedras Pintas Salt Dome, Condado de Duval, sur de Texas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Green Hydrogen International (GHI)</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>ABB (automatización/control, vía MOU)</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Ingeniería/FEED (inversión USD 6,000-10,000 millones; electrolizador de 2.2 GW; producirá 1.4 Mt/año de e-metanol y capturará ~2 Mt/año de CO2; construcción planeada desde 2026, primera producción estimada 2030)</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>[The Engineer](https://www.theengineer.co.uk/content/news/abb-joins-team-for-22gw-hydrogen-city-project-in-texas); [Energy Capital HTX](https://energycapitalhtx.com/green-hydrogen-city-abb-mou)</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t>Targa Resources Falcon II Gas Processing Plant</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B45" t="inlineStr">
         <is>
           <t>Cuenca Delaware, Permian Basin, Texas, EE.UU.</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>Targa Resources Corp.</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D45" t="inlineStr">
         <is>
           <t>Targa Resources (propietario-constructor)</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
+      <c r="E45" t="inlineStr">
         <is>
           <t>Construcción/Comisionamiento (planta criogénica 275 MMcf/d; arranque adelantado a 1T2026, dos trimestres antes de lo previsto)</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="F45" t="inlineStr">
         <is>
           <t>[Oil &amp; Gas Journal](https://www.ogj.com/refining-processing/gas-processing/capacities/article/55240691/targa-advances-expansion-plans-for-permian-basin-gas-processing)</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
+      <c r="G45" t="inlineStr">
         <is>
           <t>2026-08-06</t>
         </is>
@@ -2067,15 +2104,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -3556,6 +3593,43 @@
       <c r="G40" t="inlineStr">
         <is>
           <t>2026-08-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Gasoducto TTC Connector (alimenta Freeport LNG)</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Condados de Colorado y Wharton, Texas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Desarrollador: TTC Connector, LLC; opción de compra: Enbridge Inc.; cliente de capacidad: bp</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Construcción (25 millas/300 MMpc/d; en servicio previsto fines de 2026)</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>[LNG Industry](https://www.lngindustry.com/liquid-natural-gas/07082026/enbridge-signs-option-to-acquire-ttc-connector/)</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
@@ -3570,15 +3644,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G70"/>
+  <dimension ref="A1:G77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -6169,6 +6243,265 @@
       <c r="G70" t="inlineStr">
         <is>
           <t>2026-08-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Lone Tree Plant (Refurbishment Autoclave/CIL)</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Lovelock, Nevada, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>i-80 Gold Corp</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Hatch (EPCM)</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Construcción (obras tempranas y movilización de contratistas en curso; construcción mayor prevista 4T2026)</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/i-80-gold-provides-update-on-lone-tree-plant-refurbishment-project-remains-on-schedule-and-on-budget-302836341.html)</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Round Mountain Phase X — Planta de Paste Backfill</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Nye County, Nevada, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Kinross Gold Corporation</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>No especificado (paquetes de equipo móvil, ventiladores y planta CRF ya adjudicados)</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Construcción/Ingeniería detallada</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/29/3335652/0/en/Kinross-reports-strong-2026-second-quarter-results.html)</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Bald Mountain Redbird 2 — Planta SART (ácido/lixiviación)</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>White Pine County, Nevada, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Kinross Gold Corporation</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Contratista de ingeniería detallada ya seleccionado, no revelado en la fuente</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Ingeniería (básica ~50% completa)</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/29/3335652/0/en/Kinross-reports-strong-2026-second-quarter-results.html)</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Bear Lodge Rare Earth Project</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Crook County, Wyoming, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Rare Element Resources Ltd. (afiliada de General Atomics/Synchron)</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Permitting (designación FAST-41; aviso NEPA publicado en Federal Register 29-jul-2026)</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>[Federal Register](https://www.federalregister.gov/documents/2026/07/29/2026-15255/black-hills-national-forest-wyoming-bear-lodge-rare-earth-project)</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Proyecto de Cobre Angangueo</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Angangueo, Michoacán, México</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Southern Copper Corporation (Grupo México)</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Pre-desarrollo (en negociación de permisos con gobierno federal)</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>[Minería en Línea](https://mineriaenlinea.com/2026/07/southern-copper-obtiene-permisos-ambientales-para-el-pilar-produccion-a-partir-de-2029/)</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Proyecto de Cobre Chalchihuites</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Chalchihuites, Zacatecas, México</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Southern Copper Corporation (Grupo México)</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Pre-desarrollo (en negociación de permisos)</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>[Minería en Línea](https://mineriaenlinea.com/2026/07/southern-copper-obtiene-permisos-ambientales-para-el-pilar-produccion-a-partir-de-2029/)</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Modernización Complejo Metalúrgico Empalme</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Empalme, Sonora, México</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Southern Copper Corporation (Grupo México)</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Pre-desarrollo (en negociación de permisos; fundición existente a modernizar)</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>[Minería en Línea](https://mineriaenlinea.com/2026/07/southern-copper-obtiene-permisos-ambientales-para-el-pilar-produccion-a-partir-de-2029/)</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
@@ -6183,15 +6516,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G79"/>
+  <dimension ref="A1:G81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -6578,7 +6911,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Pacifico Energy</t>
+          <t>Pacifico Energy; inquilino confirmado: Amazon (AWS)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -6588,17 +6921,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Permisos obtenidos/inicio construcción (TCEQ otorgó permiso de aire para 7.65GW de generación a gas, el más grande emitido en EE.UU. hasta la fecha; Fase 1 de 1GW prevista en operación 1S2027)</t>
+          <t>Construcción de edificios de centro de datos iniciada (TCEQ ya había otorgado permiso de aire para 7.65GW de generación a gas; Amazon presentó a inicios de ago-2026 permisos de construcción para 3 edificios de centro de datos —"Pecos County Data Center", Buildings A/B/C, ~189,060 pies² c/u, ~US$300M c/u—; construcción de edificios prevista ago-dic 2026; Fase 1 de 1GW de generación prevista en operación 1S2027)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>[Business Wire](https://www.businesswire.com/news/home/20260126236053/en/Pacifico-Energy-Secures-7.65-GW-Power-Generation-Permit-for-GW-Ranch-Project)</t>
+          <t>[Business Wire](https://www.businesswire.com/news/home/20260126236053/en/Pacifico-Energy-Secures-7.65-GW-Power-Generation-Permit-for-GW-Ranch-Project); [US Data Center Projects](https://usdatacenterprojects.com/texas/amazon-files-plans-for-new-data-center-buildings-in-texas-across-three-sites)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
@@ -7994,17 +8327,17 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Construcción DETENIDA (orden de suspensión de la agencia ambiental de Georgia -EPD- por construir sin permisos, 2-jul-2026)</t>
+          <t>Construcción REANUDADA (tras orden de suspensión de la agencia ambiental de Georgia -EPD- del 2-jul-2026 por construir sin permisos; a 31-jul-2026 la construcción de la planta de 90MW está en marcha de nuevo, con 6 de 33 motores a gas ya instalados)</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>[AJC](https://www.ajc.com/business/2026/07/officials-order-georgia-data-centers-pop-up-power-plant-to-halt-construction/)</t>
+          <t>[AJC](https://www.ajc.com/business/2026/07/officials-order-georgia-data-centers-pop-up-power-plant-to-halt-construction/); [Inside Climate News](https://insideclimatenews.org/news/31072026/georgia-data-center-private-power-plant/)</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
@@ -9115,6 +9448,80 @@
       <c r="G79" t="inlineStr">
         <is>
           <t>2026-08-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Galaxy Digital Project Merlin</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>McGregor, Condado de McLennan, Texas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Galaxy Digital</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Planeación/permitting inicial (500 acres adquiridos; acuerdo de desarrollo aprobado por el ayuntamiento de McGregor 24-jun-2026; subestación eléctrica propia en construcción; enfriamiento de circuito cerrado, sin planta de gas on-site confirmada; Fase 1 de 74MW prevista 2028)</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/galaxy-expands-data-center-footprint-with-acquisition-of-500-acre-campus-in-mcgregor-texas-302836014.html)</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Nexus Fulcrum Gas Plant (TRIC)</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Tahoe-Reno Industrial Center, Condado de Storey, Nevada, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Nexus Fulcrum LLC (abastecerá al hub industrial/de centros de datos de TRIC, donde operan Switch, Google, Tract, entre otros)</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Permitting (solicitud regulatoria presentada ante reguladores estatales de energía de Nevada para planta de gas natural de 510MW)</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>[The Nevada Independent](https://thenevadaindependent.com/article/nevada-data-center-rush-drives-request-for-a-novel-type-of-gas-power-plant)</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Agregar 4 proyectos nuevos y 8 cambios de fase (2026-08-11)
Petroquimica: CF Industries Blue Point (inicio construccion), MPLX
Harmon Creek III (arranque), ONEOK Bighorn/Cutter/Shadowfax
(expansion/reubicacion).
LNG: Delfin FLNG 1 (contrato de estudios submarinos), Alaska LNG
(nueva sesion legislativa especial).
Mining: 3 proyectos nuevos de minerales criticos (Coosa Graphite,
Global Advanced Metals Tantalio/Niobio, Boron Americas Fort Cady),
Resolution Copper (contratos de exploracion), Santa Cruz Copper
(financiamiento EXIM ampliado).
Data Centers: Dove Creek Technology Campus (nuevo), GW Ranch Power
Campus (permiso de aire TCEQ confirmado).

Proyectos.xlsx regenerado con el acumulado completo (44 Petroquimica,
40 LNG, 79 Mining, 81 Data Centers).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6DeVZBn5b37Hwr88vxai9
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -20,10 +20,18 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
@@ -49,8 +57,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -420,46 +429,46 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -493,7 +502,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>[Fluor newsroom](https://newsroom.fluor.com/news-releases/news-details/2026/Fluor-Awarded-Contract-to-Engineer-and-Design-the-America-First-Refining-Facility-in-Brownsville-Texas/default.aspx); [Tech Times](https://www.techtimes.com/articles/323235/20260805/trumps-flagship-texas-refinery-races-permit-deadline-after-326b-grid-loan.htm)</t>
+          <t>Fluor newsroom (https://newsroom.fluor.com/news-releases/news-details/2026/Fluor-Awarded-Contract-to-Engineer-and-Design-the-America-First-Refining-Facility-in-Brownsville-Texas/default.aspx); Tech Times (https://www.techtimes.com/articles/323235/20260805/trumps-flagship-texas-refinery-races-permit-deadline-after-326b-grid-loan.htm)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -505,69 +514,69 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ExxonMobil Coastal Plain (cracker + PE)</t>
+          <t>CF Industries Blue Point (amoniaco bajo carbono)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Calhoun County, Texas, EE.UU.</t>
+          <t>Ascension Parish, Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ExxonMobil</t>
+          <t>CF Industries / JERA / Mitsui &amp; Co.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Technip Energies</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Ingeniería/FEED</t>
+          <t>Construcción (Luisiana y el U.S. Army Corps of Engineers emitieron en jul-2026 los permisos de construcción civil necesarios; CF Industries confirmó en su reporte 2T2026 —8-K, 5-ago-2026— el inicio de construcción en ago-2026 de la planta de amoniaco bajo carbono, ~708,000-1.4 MTPA, ~US$3.7-4,000 millones; producción prevista 2029)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>[AllStream Insiders](https://allstreaminsiders.com/us-exxonmobil-may-build-cracker-pe-plant-in-texas-with-an-8-6-billion-investment/)</t>
+          <t>FuelCellsWorks (https://fuelcellsworks.com/2026/08/06/clean-energy/cf-industries-to-begin-construction-of-3-7bn-louisiana-blue-ammonia-plant); gasworld (https://www.gasworld.com/story/cf-industries-to-begin-construction-of-4bn-louisiana-blue-ammonia-project/2256572.article/)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Golden Triangle Polymers</t>
+          <t>ExxonMobil Coastal Plain (cracker + PE)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Orange, Texas, EE.UU.</t>
+          <t>Calhoun County, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Chevron Phillips Chemical (CPChem) / QatarEnergy</t>
+          <t>ExxonMobil</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>ZDJV (Zachry/DL USA); JKJV (JGC America/Kiewit)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Construcción (comisionamiento)</t>
+          <t>Ingeniería/FEED</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>[BIC Magazine](https://www.bicmagazine.com/departments/operations/cpchem-golden-triangle-polymers-facility-startup-phase/)</t>
+          <t>AllStream Insiders (https://allstreaminsiders.com/us-exxonmobil-may-build-cracker-pe-plant-in-texas-with-an-8-6-billion-investment/)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -579,37 +588,37 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CF Industries Blue Point (amoniaco bajo carbono)</t>
+          <t>Golden Triangle Polymers</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Ascension Parish, Luisiana, EE.UU.</t>
+          <t>Orange, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>CF Industries / JERA / Mitsui &amp; Co.</t>
+          <t>Chevron Phillips Chemical (CPChem) / QatarEnergy</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Technip Energies</t>
+          <t>ZDJV (Zachry/DL USA); JKJV (JGC America/Kiewit)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Construcción (impulso federal de permisos anunciado may-2026 con finalización esperada en 45 días; CF Industries confirma inicio de construcción en 2026)</t>
+          <t>Construcción (comisionamiento)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>[Construction Front](https://constructionfront.com/2025-04-13-technip-energies-to-deliver-blue-point-worlds-largest-low-carbon-ammonia-facility-in-louisiana/); [FuelCellsWorks](https://fuelcellsworks.com/2026/05/07/h2/cf-industries-targets-construction-start-this-year-on-blue-hydrogen-and-ammonia-complex)</t>
+          <t>BIC Magazine (https://www.bicmagazine.com/departments/operations/cpchem-golden-triangle-polymers-facility-startup-phase/)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-10</t>
         </is>
       </c>
     </row>
@@ -641,7 +650,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>[East Daley](https://eastdaley.com/media-and-news/the-race-is-on-to-build-permian-processing)</t>
+          <t>East Daley (https://eastdaley.com/media-and-news/the-race-is-on-to-build-permian-processing)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -678,7 +687,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>[Techint](https://www.techint.com/en/our-projects/dos-bocas-refinery)</t>
+          <t>Techint (https://www.techint.com/en/our-projects/dos-bocas-refinery)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -715,7 +724,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>[OGJ](https://www.ogj.com/refining-processing/refining/optimization/article/17279334/pemex-to-proceed-with-dos-bocas-refinery-project)</t>
+          <t>OGJ (https://www.ogj.com/refining-processing/refining/optimization/article/17279334/pemex-to-proceed-with-dos-bocas-refinery-project)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -752,7 +761,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>[Forbes México](https://forbes.com.mx/pemex-invertira-5300-millones-de-dolares-para-reactivar-la-industria-petroquimica/)</t>
+          <t>Forbes México (https://forbes.com.mx/pemex-invertira-5300-millones-de-dolares-para-reactivar-la-industria-petroquimica/)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -789,7 +798,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>[Forbes México](https://forbes.com.mx/pemex-invertira-5300-millones-de-dolares-para-reactivar-la-industria-petroquimica/)</t>
+          <t>Forbes México (https://forbes.com.mx/pemex-invertira-5300-millones-de-dolares-para-reactivar-la-industria-petroquimica/)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -826,7 +835,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>[Forbes México](https://forbes.com.mx/asi-es-la-inversion-de-1553-mdd-por-parte-de-pemex-en-una-planta-de-fertilizantes-en-veracruz/)</t>
+          <t>Forbes México (https://forbes.com.mx/asi-es-la-inversion-de-1553-mdd-por-parte-de-pemex-en-una-planta-de-fertilizantes-en-veracruz/)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -863,7 +872,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>[Tribuna](https://tribuna.com.mx/mexico/2026/06/05/sheinbaum-anuncia-inversion-de-93-mil-mdp-para-reactivar-la-industria-petroquimica-y-de-fertilizantes-en-veracruz_560837/); [Contralínea](https://contralinea.com.mx/interno/semana/presentan-plan-con-inversion-de-93-mil-mdp-para-rescatar-la-petroquimica-nacional/)</t>
+          <t>Tribuna (https://tribuna.com.mx/mexico/2026/06/05/sheinbaum-anuncia-inversion-de-93-mil-mdp-para-reactivar-la-industria-petroquimica-y-de-fertilizantes-en-veracruz_560837/); Contralínea (https://contralinea.com.mx/interno/semana/presentan-plan-con-inversion-de-93-mil-mdp-para-rescatar-la-petroquimica-nacional/)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -900,7 +909,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>[PV Magazine México](https://www.pv-magazine-mexico.com/2026/04/28/inician-en-sinaloa-la-construccion-de-la-mayor-planta-de-metanol-ultrabajo-en-carbono-a-partir-de-hidrogeno-verde/)</t>
+          <t>PV Magazine México (https://www.pv-magazine-mexico.com/2026/04/28/inician-en-sinaloa-la-construccion-de-la-mayor-planta-de-metanol-ultrabajo-en-carbono-a-partir-de-hidrogeno-verde/)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -937,7 +946,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>[H2 View](https://www.h2-view.com/story/first-ammonia-project-on-track-for-2026-fid-despite-topsoe-deal-collapse/2138792.article/)</t>
+          <t>H2 View (https://www.h2-view.com/story/first-ammonia-project-on-track-for-2026-fid-despite-topsoe-deal-collapse/2138792.article/)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -974,7 +983,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>[Debate](https://www.debate.com.mx/economia/secretaria-de-economia-complejo-de-amoniaco-en-topolobampo-prioritario-para-el-gobierno-de-mexico-20260713-0092.html)</t>
+          <t>Debate (https://www.debate.com.mx/economia/secretaria-de-economia-complejo-de-amoniaco-en-topolobampo-prioritario-para-el-gobierno-de-mexico-20260713-0092.html)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1011,7 +1020,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>[ICIS](https://www.icis.com/explore/resources/news/2025/11/13/11155109/lake-charles-methanol-ii-awards-feed-fid-expected-in-q2-2026/)</t>
+          <t>ICIS (https://www.icis.com/explore/resources/news/2025/11/13/11155109/lake-charles-methanol-ii-awards-feed-fid-expected-in-q2-2026/)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1048,7 +1057,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>[Diario del Istmo](https://diariodelistmo.com/nacional/este-es-el-avance-que-lleva-la-planta-coquizadora-en-la-refineria-de-salina-cruz/50642321)</t>
+          <t>Diario del Istmo (https://diariodelistmo.com/nacional/este-es-el-avance-que-lleva-la-planta-coquizadora-en-la-refineria-de-salina-cruz/50642321)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1085,7 +1094,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/petrochemicals/06032026/shintech-announces-us34-billion-at-louisiana-petrochemicals-complex/)</t>
+          <t>Hydrocarbon Engineering (https://www.hydrocarbonengineering.com/petrochemicals/06032026/shintech-announces-us34-billion-at-louisiana-petrochemicals-complex/)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1122,7 +1131,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>[INEOS](https://www.ineos.com/news/shared-news/ineos-acetyls-and-sandpiper-chemicals-announce-strategic-collaboration-for-the-development-of-a-low-carbon-methanol-project-in-texas-city-texas/)</t>
+          <t>INEOS (https://www.ineos.com/news/shared-news/ineos-acetyls-and-sandpiper-chemicals-announce-strategic-collaboration-for-the-development-of-a-low-carbon-methanol-project-in-texas-city-texas/)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1159,7 +1168,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/petrochemicals/13072026/oxea-confirms-fid-for-major-capacity-expansion/)</t>
+          <t>Hydrocarbon Engineering (https://www.hydrocarbonengineering.com/petrochemicals/13072026/oxea-confirms-fid-for-major-capacity-expansion/)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1196,7 +1205,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>[OGJ](https://www.ogj.com/refining-processing/gas-processing/news/55320579/targa-advances-permian-gas-pipeline-processing-expansion)</t>
+          <t>OGJ (https://www.ogj.com/refining-processing/gas-processing/news/55320579/targa-advances-permian-gas-pipeline-processing-expansion)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1233,7 +1242,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>[Business Wire](https://www.businesswire.com/news/home/20250806663187/en/Enterprise-Agrees-to-Acquire-Occidentals-Gas-Gathering-Affiliate-Enters-Into-Natural-Gas-Processing-Agreement-Announces-New-Midland-Basin-Natural-Gas-Processing-Plant)</t>
+          <t>Business Wire (https://www.businesswire.com/news/home/20250806663187/en/Enterprise-Agrees-to-Acquire-Occidentals-Gas-Gathering-Affiliate-Enters-Into-Natural-Gas-Processing-Agreement-Announces-New-Midland-Basin-Natural-Gas-Processing-Plant)</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1270,7 +1279,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>[Natural Gas Intel](https://naturalgasintel.com/news/mplx-scales-up-for-power-hungry-future-with-natural-gas-focused-growth-plan/)</t>
+          <t>Natural Gas Intel (https://naturalgasintel.com/news/mplx-scales-up-for-power-hungry-future-with-natural-gas-focused-growth-plan/)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1307,7 +1316,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>[East Daley](https://eastdaley.com/daley-note/mplx-acquires-northwind-for-2-375b-acquires-more-ngls-for-jv-project)</t>
+          <t>East Daley (https://eastdaley.com/daley-note/mplx-acquires-northwind-for-2-375b-acquires-more-ngls-for-jv-project)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1344,7 +1353,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>[Grand Forks Herald](https://www.grandforksherald.com/news/local/northern-plains-nitrogen-proposal-receiving-more-attention-amid-global-fertilizer-pressure)</t>
+          <t>Grand Forks Herald (https://www.grandforksherald.com/news/local/northern-plains-nitrogen-proposal-receiving-more-attention-amid-global-fertilizer-pressure)</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1381,7 +1390,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>[Phillips 66](https://www.phillips66.com/newsroom/iron-mesa-safely-enters-next-phase-of-construction/)</t>
+          <t>Phillips 66 (https://www.phillips66.com/newsroom/iron-mesa-safely-enters-next-phase-of-construction/)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1418,7 +1427,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>[Targa Resources](https://www.targaresources.com/news-releases/news-release-details/targa-resources-corp-announces-permian-growth-projects-and)</t>
+          <t>Targa Resources (https://www.targaresources.com/news-releases/news-release-details/targa-resources-corp-announces-permian-growth-projects-and)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1455,7 +1464,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>[Elefante Blanco](https://elefanteblanco.mx/2026/01/02/pemex-abre-30-licitaciones-para-obras-en-la-refineria-madero/)</t>
+          <t>Elefante Blanco (https://elefanteblanco.mx/2026/01/02/pemex-abre-30-licitaciones-para-obras-en-la-refineria-madero/)</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1492,7 +1501,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>[La Jornada](https://www.jornada.com.mx/noticia/2026/06/08/economia/da-inicio-ejecucion-de-planta-de-fertilizantes-en-durango-por-parte-de-fermachem)</t>
+          <t>La Jornada (https://www.jornada.com.mx/noticia/2026/06/08/economia/da-inicio-ejecucion-de-planta-de-fertilizantes-en-durango-por-parte-de-fermachem)</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1529,7 +1538,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>[Downstream Calendar](https://downstreamcalendar.com/mcdermott-secures-feed-contract-for-ascension-clean-energy-project/)</t>
+          <t>Downstream Calendar (https://downstreamcalendar.com/mcdermott-secures-feed-contract-for-ascension-clean-energy-project/)</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1566,7 +1575,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>[Business Wire](https://www.businesswire.com/news/home/20260517310811/en/Phillips-66-announces-Zeus-Gas-Plant-and-a-third-Coastal-Bend-Fractionator)</t>
+          <t>Business Wire (https://www.businesswire.com/news/home/20260517310811/en/Phillips-66-announces-Zeus-Gas-Plant-and-a-third-Coastal-Bend-Fractionator)</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1603,7 +1612,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>[USDA](https://www.usda.gov/about-usda/news/press-releases/2026/07/01/secretary-rollins-announces-500-million-fertilizer-investment-and-expansion-program-strengthen)</t>
+          <t>USDA (https://www.usda.gov/about-usda/news/press-releases/2026/07/01/secretary-rollins-announces-500-million-fertilizer-investment-and-expansion-program-strengthen)</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1640,7 +1649,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/clean-fuels/06012026/samsung-ea-announces-groundbreaking-of-low-carbon-ammonia-plant/)</t>
+          <t>Hydrocarbon Engineering (https://www.hydrocarbonengineering.com/clean-fuels/06012026/samsung-ea-announces-groundbreaking-of-low-carbon-ammonia-plant/)</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1677,7 +1686,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/refining/03062026/green-fuels-hosts-groundbreaking-ceremony-for-new-refinery/)</t>
+          <t>Hydrocarbon Engineering (https://www.hydrocarbonengineering.com/refining/03062026/green-fuels-hosts-groundbreaking-ceremony-for-new-refinery/)</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1714,7 +1723,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>[Energy Transfer](https://www.energytransfer.com/project-highlights/)</t>
+          <t>Energy Transfer (https://www.energytransfer.com/project-highlights/)</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1746,17 +1755,17 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Construcción (Bighorn US$365 millones/300 MMcf/d tratamiento alto CO2, meta mediados 2027; Cutter 60 MMcf/d en construcción, meta 4T2026; Shadowfax 150 MMcf/d reubicación completada 1T2026, en rampa)</t>
+          <t>Construcción (según reporte 2T2026 de ONEOK, ~4-8-ago-2026: Bighorn ampliada de 300 a 400 MMcf/d, tratamiento alto CO2, meta mediados 2027; Cutter 60 MMcf/d en construcción, meta 4T2026; Shadowfax 150 MMcf/d reubicada a la cuenca Midland durante el trimestre, en rampa)</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>[Inspectioneering](https://inspectioneering.com/news/2025-08-07/11702/oneok-greenlights-new-365m-delaware-basin-gas-plant)</t>
+          <t>Inspectioneering (https://inspectioneering.com/news/2025-08-07/11702/oneok-greenlights-new-365m-delaware-basin-gas-plant); BigGo Finance (https://finance.biggo.com/news/US_OKE_2026-08-04)</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -1783,17 +1792,17 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Construcción (300 MMcf/d + de-etanizadora 40 Mbpd; en servicio 3T2026)</t>
+          <t>Operando (arranque/startup completado ago-2026, según reporte 2T2026 de MPLX; eleva capacidad de procesamiento de MPLX en el noreste a 8.1 Bcf/d; planta de 300 MMcf/d + de-etanizadora 40 Mbpd)</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>[Natural Gas Intel](https://www.naturalgasintel.com/news/mplx-scales-up-for-power-hungry-future-with-natural-gas-focused-growth-plan/)</t>
+          <t>Marcellus Drilling News (https://marcellusdrilling.com/2026/08/mplx-marcellus-proc-plants-96-full-harmon-creek-iii-starts-up/); StockTitan (https://www.stocktitan.net/news/MPLX/mplx-lp-reports-second-quarter-2026-financial-9tcvq4saz6sr.html)</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -1825,7 +1834,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>[Contralínea](https://contralinea.com.mx/interno/semana/presentan-plan-con-inversion-de-93-mil-mdp-para-rescatar-la-petroquimica-nacional/); [El Diario de Juárez](https://diario.mx/nacional/2026/jan/22/adjudica-pemex-contratos-a-favoritas-1102601.html)</t>
+          <t>Contralínea (https://contralinea.com.mx/interno/semana/presentan-plan-con-inversion-de-93-mil-mdp-para-rescatar-la-petroquimica-nacional/); El Diario de Juárez (https://diario.mx/nacional/2026/jan/22/adjudica-pemex-contratos-a-favoritas-1102601.html)</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -1862,7 +1871,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>[Enterprise Reports Second Quarter 2026 Earnings](https://ir.enterpriseproducts.com/news-releases/news-release-details/enterprise-reports-second-quarter-2026-earnings)</t>
+          <t>Enterprise Reports Second Quarter 2026 Earnings (https://ir.enterpriseproducts.com/news-releases/news-release-details/enterprise-reports-second-quarter-2026-earnings)</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -1899,7 +1908,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>[Enterprise Reports Second Quarter 2026 Earnings](https://ir.enterpriseproducts.com/news-releases/news-release-details/enterprise-reports-second-quarter-2026-earnings)</t>
+          <t>Enterprise Reports Second Quarter 2026 Earnings (https://ir.enterpriseproducts.com/news-releases/news-release-details/enterprise-reports-second-quarter-2026-earnings)</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -1936,7 +1945,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>[PGJ](https://pgjonline.com/news/2026/may/targa-expands-permian-gas-processing-delaware-express-pipeline-capacity)</t>
+          <t>PGJ (https://pgjonline.com/news/2026/may/targa-expands-permian-gas-processing-delaware-express-pipeline-capacity)</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -1973,7 +1982,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>[Hydrocarbon Processing](https://www.hydrocarbonprocessing.com/news/2026/03/southern-energy-renewables-announce-14-b-methanol-and-saf-complex-in-louisiana/); [Louisiana Economic Development](https://www.opportunitylouisiana.gov/news/southern-energy-renewables-announce-1-4-billion-methanol-and-sustainable-aviation-fuel-facility-in-st-charles-parish)</t>
+          <t>Hydrocarbon Processing (https://www.hydrocarbonprocessing.com/news/2026/03/southern-energy-renewables-announce-14-b-methanol-and-saf-complex-in-louisiana/); Louisiana Economic Development (https://www.opportunitylouisiana.gov/news/southern-energy-renewables-announce-1-4-billion-methanol-and-sustainable-aviation-fuel-facility-in-st-charles-parish)</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2010,7 +2019,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>[Tri-Cities Area Journal of Business](https://www.tricitiesbusinessnews.com/articles/atlas-agro-plant-nears-decision-point); [Washington State Standard](https://washingtonstatestandard.com/2025/10/30/plan-for-1-5b-fertilizer-plant-in-central-wa-still-alive-despite-loss-of-federal-funds/)</t>
+          <t>Tri-Cities Area Journal of Business (https://www.tricitiesbusinessnews.com/articles/atlas-agro-plant-nears-decision-point); Washington State Standard (https://washingtonstatestandard.com/2025/10/30/plan-for-1-5b-fertilizer-plant-in-central-wa-still-alive-despite-loss-of-federal-funds/)</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2047,7 +2056,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>[The Engineer](https://www.theengineer.co.uk/content/news/abb-joins-team-for-22gw-hydrogen-city-project-in-texas); [Energy Capital HTX](https://energycapitalhtx.com/green-hydrogen-city-abb-mou)</t>
+          <t>The Engineer (https://www.theengineer.co.uk/content/news/abb-joins-team-for-22gw-hydrogen-city-project-in-texas); Energy Capital HTX (https://energycapitalhtx.com/green-hydrogen-city-abb-mou)</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2084,7 +2093,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>[Oil &amp; Gas Journal](https://www.ogj.com/refining-processing/gas-processing/capacities/article/55240691/targa-advances-expansion-plans-for-permian-basin-gas-processing)</t>
+          <t>Oil &amp; Gas Journal (https://www.ogj.com/refining-processing/gas-processing/capacities/article/55240691/targa-advances-expansion-plans-for-permian-basin-gas-processing)</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2108,46 +2117,46 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -2181,7 +2190,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>[Bechtel](https://www.bechtel.com/press-releases/nextdecade-executes-epc-contract-with-bechtel-for-train-4-at-the-rio-grande-lng-facility/); [Natural Gas Intel](https://naturalgasintel.com/news/nextdecade-targets-more-than-36-mty-with-rio-grande-lng-upscale-sixth-train-expansion/); [Federal Register](https://www.federalregister.gov/documents/2026/08/03/2026-15695/rio-grande-lng-train-6-llc-notice-of-intent-to-prepare-an-environmental-impact-statement-for-the); [LNG Prime](https://lngprime.com/americas/nextdecade-seeks-ferc-ok-for-sixth-rio-grande-lng-train/187820/)</t>
+          <t>Bechtel (https://www.bechtel.com/press-releases/nextdecade-executes-epc-contract-with-bechtel-for-train-4-at-the-rio-grande-lng-facility/); Natural Gas Intel (https://naturalgasintel.com/news/nextdecade-targets-more-than-36-mty-with-rio-grande-lng-upscale-sixth-train-expansion/); Federal Register (https://www.federalregister.gov/documents/2026/08/03/2026-15695/rio-grande-lng-train-6-llc-notice-of-intent-to-prepare-an-environmental-impact-statement-for-the); LNG Prime (https://lngprime.com/americas/nextdecade-seeks-ferc-ok-for-sixth-rio-grande-lng-train/187820/)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -2218,7 +2227,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>[Bechtel](https://www.bechtel.com/press-releases/sempra-infrastructure-announces-epc-contract-with-bechtel-for-port-arthur-lng-phase-2/)</t>
+          <t>Bechtel (https://www.bechtel.com/press-releases/sempra-infrastructure-announces-epc-contract-with-bechtel-for-port-arthur-lng-phase-2/)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -2255,7 +2264,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>[Woodside](https://www.woodside.com/what-we-do/growth-projects/woodside-louisiana-lng)</t>
+          <t>Woodside (https://www.woodside.com/what-we-do/growth-projects/woodside-louisiana-lng)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -2292,7 +2301,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>[GEM.wiki](https://www.gem.wiki/CP2_LNG_Terminal); [LNG Prime](https://lngprime.com/americas/top-5-news-of-the-week-july-20-26/193119/)</t>
+          <t>GEM.wiki (https://www.gem.wiki/CP2_LNG_Terminal); LNG Prime (https://lngprime.com/americas/top-5-news-of-the-week-july-20-26/193119/)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -2329,7 +2338,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>[Offshore Energy](https://www.offshore-energy.biz/kbr-zachry-to-work-on-ventures-plaquemines-lng/); [Argus Media](https://www.argusmedia.com/en/news-and-insights/latest-market-news/2755512-vg-files-expansion-plan-to-double-plaquemines-lng)</t>
+          <t>Offshore Energy (https://www.offshore-energy.biz/kbr-zachry-to-work-on-ventures-plaquemines-lng/); Argus Media (https://www.argusmedia.com/en/news-and-insights/latest-market-news/2755512-vg-files-expansion-plan-to-double-plaquemines-lng)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -2366,7 +2375,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>[Port Arthur News](https://panews.com/2026/04/24/golden-pass-lng-makes-history-with-first-export-from-sabine-pass-terminal/)</t>
+          <t>Port Arthur News (https://panews.com/2026/04/24/golden-pass-lng-makes-history-with-first-export-from-sabine-pass-terminal/)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -2403,7 +2412,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>[PGJ](https://pgjonline.com/news/2026/july/cheniere-gets-approval-to-introduce-gas-into-final-corpus-christi-lng-train); [LNG Prime](https://lngprime.com/americas/chenieres-corpus-christi-expansion-project-85-4-percent-complete/155448/); [energiesmedia](https://energiesmedia.com/ferc-approves-cheniere-train-7-energies/)</t>
+          <t>PGJ (https://pgjonline.com/news/2026/july/cheniere-gets-approval-to-introduce-gas-into-final-corpus-christi-lng-train); LNG Prime (https://lngprime.com/americas/chenieres-corpus-christi-expansion-project-85-4-percent-complete/155448/); energiesmedia (https://energiesmedia.com/ferc-approves-cheniere-train-7-energies/)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -2435,17 +2444,17 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Construcción (FID positiva jun-2026)</t>
+          <t>Construcción (FID positiva jun-2026; TDI-Brooks International adjudicado 10-ago-2026 para levantamientos geofísicos/geotécnicos submarinos del puerto de aguas profundas —inicio geofísico fin ago-2026, geotécnico fin sep-2026—, en apoyo de hasta 3 unidades FLNG, ~13.2 Mtpa)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/06/03/3306350/0/en/delfin-midstream-announces-5-billion-final-investment-decision-for-first-flng-vessel.html)</t>
+          <t>GlobeNewswire (https://www.globenewswire.com/news-release/2026/06/03/3306350/0/en/delfin-midstream-announces-5-billion-final-investment-decision-for-first-flng-vessel.html); World Oil (https://www.worldoil.com/news/2026/8/10/tdi-brooks-wins-survey-contract-for-delfin-lng-deepwater-port/)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -2477,7 +2486,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>[Dossier Político](https://dossierpolitico.com/2026/07/17/activistas-entregan-90-mil-firmas-para-frenar-proyecto-saguaro-energia-en-sonora/); [Natural Gas Intel](https://naturalgasintel.com/news/oneok-affiliate-seeks-3-year-extension-for-saguaro-connector-pipeline/)</t>
+          <t>Dossier Político (https://dossierpolitico.com/2026/07/17/activistas-entregan-90-mil-firmas-para-frenar-proyecto-saguaro-energia-en-sonora/); Natural Gas Intel (https://naturalgasintel.com/news/oneok-affiliate-seeks-3-year-extension-for-saguaro-connector-pipeline/)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -2514,7 +2523,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>[GEM Wiki](https://www.gem.wiki/New_Fortress_Altamira_FLNG_Terminal)</t>
+          <t>GEM Wiki (https://www.gem.wiki/New_Fortress_Altamira_FLNG_Terminal)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -2551,7 +2560,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>[Natural Gas Intel](https://www.naturalgasintel.com/news/glenfarne-lands-investment-for-early-work-on-texas-lng-ahead-of-fid/)</t>
+          <t>Natural Gas Intel (https://www.naturalgasintel.com/news/glenfarne-lands-investment-for-early-work-on-texas-lng-ahead-of-fid/)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -2588,7 +2597,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>[PGJ](https://pgjonline.com/news/2026/july/commonwealth-lng-awards-main-automation-contract-for-louisiana-export-terminal); [PR Newswire/Caturus](https://www.prnewswire.com/news-releases/caturus-announces-final-investment-decision-for-9-5-mtpa-commonwealth-lng-export-facility-in-cameron-la-302773264.html)</t>
+          <t>PGJ (https://pgjonline.com/news/2026/july/commonwealth-lng-awards-main-automation-contract-for-louisiana-export-terminal); PR Newswire/Caturus (https://www.prnewswire.com/news-releases/caturus-announces-final-investment-decision-for-9-5-mtpa-commonwealth-lng-export-facility-in-cameron-la-302773264.html)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -2625,7 +2634,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>[Houston Public Media](https://www.houstonpublicmedia.org/articles/galveston-county/2026/07/14/557086/galveston-pelican-island-lng/)</t>
+          <t>Houston Public Media (https://www.houstonpublicmedia.org/articles/galveston-county/2026/07/14/557086/galveston-pelican-island-lng/)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -2662,7 +2671,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>[Sempra](https://www.sempra.com/newsroom/press-releases/sempra-infrastructures-eca-lng-phase-1-exports-first-lng-cargo-mexicos); [LNG Prime](https://lngprime.com/lng-terminals/sempra-infrastructure-extends-eca-lng-commissioning-due-to-compressor-damage/193584/)</t>
+          <t>Sempra (https://www.sempra.com/newsroom/press-releases/sempra-infrastructures-eca-lng-phase-1-exports-first-lng-cargo-mexicos); LNG Prime (https://lngprime.com/lng-terminals/sempra-infrastructure-extends-eca-lng-commissioning-due-to-compressor-damage/193584/)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -2699,7 +2708,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>[LNG Prime](https://lngprime.com/americas/gato-negro-eyes-fid-on-mexico-lng-plant-in-late-2026/165906/)</t>
+          <t>LNG Prime (https://lngprime.com/americas/gato-negro-eyes-fid-on-mexico-lng-plant-in-late-2026/165906/)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -2736,7 +2745,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/amigo-lng-awards-landmark-epc-contract-to-dubai-based-drydocks-world-for-worlds-largest-flng-facility-302537739.html)</t>
+          <t>PR Newswire (https://www.prnewswire.com/news-releases/amigo-lng-awards-landmark-epc-contract-to-dubai-based-drydocks-world-for-worlds-largest-flng-facility-302537739.html)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -2773,7 +2782,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>[Rigzone](https://www.rigzone.com/news/coastal_bend_lng_enters_permitting_phase-05-aug-2026-184302-article/); [PGJ](https://pgjonline.com/news/2026/august/coastal-bend-lng-initiates-formal-permitting-and-consultation-process)</t>
+          <t>Rigzone (https://www.rigzone.com/news/coastal_bend_lng_enters_permitting_phase-05-aug-2026-184302-article/); PGJ (https://pgjonline.com/news/2026/august/coastal-bend-lng-initiates-formal-permitting-and-consultation-process)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2810,7 +2819,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>[FERC](https://www.ferc.gov/gulfstream-lng-terminal-project)</t>
+          <t>FERC (https://www.ferc.gov/gulfstream-lng-terminal-project)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2842,17 +2851,17 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Pre-FID (Cámara de Representantes de Alaska rechazó proyecto de ley de incentivos fiscales HB 381 necesario para el financiamiento de Glenfarne, 16-jul-2026; gobernador convocó sesión legislativa especial a partir del 27-jul-2026 para reintentar)</t>
+          <t>Pre-FID (Cámara de Representantes de Alaska rechazó proyecto de ley de incentivos fiscales HB 381, 16-jul-2026; gobernador Dunleavy convocó nueva sesión legislativa especial para el 20-ago-2026 con una ley de incentivos actualizada para reintentar destrabar el financiamiento)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>[Alaska Beacon](https://alaskabeacon.com/2026/07/17/hilcorp-killed-alaska-lng-bill-some-legislators-say-but-governor-calls-the-claim-bullst/)</t>
+          <t>Alaska Beacon (https://alaskabeacon.com/2026/07/17/hilcorp-killed-alaska-lng-bill-some-legislators-say-but-governor-calls-the-claim-bullst/); Your Alaska Link (https://www.youralaskalink.com/news/local/dunleavy-plans-updated-lng-bill-calls-lawmakers-back-august-20/article_4ea0fcfa-386b-45c1-815d-8fff56088739.html)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -2884,7 +2893,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>[PGJ](https://pgjonline.com/news/2026/july/311-mile-sonora-gas-pipeline-project-advances-in-mexico)</t>
+          <t>PGJ (https://pgjonline.com/news/2026/july/311-mile-sonora-gas-pipeline-project-advances-in-mexico)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2921,7 +2930,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>[OGJ](https://www.ogj.com/pipelines-transportation/pipelines/news/55322537/arm-energy-takes-fid-on-23-billion-mustang-express-pipeline)</t>
+          <t>OGJ (https://www.ogj.com/pipelines-transportation/pipelines/news/55322537/arm-energy-takes-fid-on-23-billion-mustang-express-pipeline)</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2958,7 +2967,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>[Mexico Business News](https://mexicobusiness.news/energy/news/ursus-energy-scales-investment-us21-billion)</t>
+          <t>Mexico Business News (https://mexicobusiness.news/energy/news/ursus-energy-scales-investment-us21-billion)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2995,7 +3004,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/15/3327983/0/en/Delfin-Midstream-Partners-With-EIG-s-MidOcean-Energy-to-Advance-Second-FLNG-Vessel-Issues-Limited-Notice-to-Proceed-to-Siemens-Energy.html)</t>
+          <t>GlobeNewswire (https://www.globenewswire.com/news-release/2026/07/15/3327983/0/en/Delfin-Midstream-Partners-With-EIG-s-MidOcean-Energy-to-Advance-Second-FLNG-Vessel-Issues-Limited-Notice-to-Proceed-to-Siemens-Energy.html)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -3032,7 +3041,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>[Natural Gas Intel](https://www.naturalgasintel.com/news/texas-gateway-open-season-expands-haynesville-natural-gas-links-amid-lng-growth/)</t>
+          <t>Natural Gas Intel (https://www.naturalgasintel.com/news/texas-gateway-open-season-expands-haynesville-natural-gas-links-amid-lng-growth/)</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -3069,7 +3078,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>[World Oil](https://worldoil.com/news/2026/7/24/doe-approves-20-year-export-authorization-for-argent-lng-project/); [PGJ](https://pgjonline.com/news/2026/august/argent-lng-submits-wsa-to-the-us-coast-guard-advancing-its-25-mmtpy-louisiana-lng-project)</t>
+          <t>World Oil (https://worldoil.com/news/2026/7/24/doe-approves-20-year-export-authorization-for-argent-lng-project/); PGJ (https://pgjonline.com/news/2026/august/argent-lng-submits-wsa-to-the-us-coast-guard-advancing-its-25-mmtpy-louisiana-lng-project)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -3106,7 +3115,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>[Federal Register](https://www.federalregister.gov/documents/2026/07/24/2026-14963/deepwater-port-license-application-st-lng-deepwater-port-development-project-final-environmental)</t>
+          <t>Federal Register (https://www.federalregister.gov/documents/2026/07/24/2026-14963/deepwater-port-license-application-st-lng-deepwater-port-development-project-final-environmental)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -3143,7 +3152,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>[Mississippi Today](https://mississippitoday.org/2026/08/05/ferc-new-gas-pipeline-mississippi/)</t>
+          <t>Mississippi Today (https://mississippitoday.org/2026/08/05/ferc-new-gas-pipeline-mississippi/)</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -3180,7 +3189,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>[Mississippi Today](https://mississippitoday.org/2026/08/05/ferc-new-gas-pipeline-mississippi/)</t>
+          <t>Mississippi Today (https://mississippitoday.org/2026/08/05/ferc-new-gas-pipeline-mississippi/)</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -3217,7 +3226,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>[LNG Prime](https://lngprime.com/americas/kinder-morgan-seeks-doe-extension-for-gulf-lng-export-project/184334/)</t>
+          <t>LNG Prime (https://lngprime.com/americas/kinder-morgan-seeks-doe-extension-for-gulf-lng-export-project/184334/)</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -3254,7 +3263,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>[Baker Hughes](https://investors.bakerhughes.com/news/press-releases/news-details/2026/Baker-Hughes-Secures-Substantial-Equipment-and-Services-Awards-for-Chenieres-Sabine-Pass-LNG-Facility/default.aspx)</t>
+          <t>Baker Hughes (https://investors.bakerhughes.com/news/press-releases/news-details/2026/Baker-Hughes-Secures-Substantial-Equipment-and-Services-Awards-for-Chenieres-Sabine-Pass-LNG-Facility/default.aspx)</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3291,7 +3300,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>[Federal Register](https://www.federalregister.gov/documents/2026/05/05/2026-08654/cheniere-corpus-christi-pipeline-lp-corpus-christi-liquefaction-stage-iv-llc-corpus-christi)</t>
+          <t>Federal Register (https://www.federalregister.gov/documents/2026/05/05/2026-08654/cheniere-corpus-christi-pipeline-lp-corpus-christi-liquefaction-stage-iv-llc-corpus-christi)</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -3328,7 +3337,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>[Natural Gas Intel](https://www.naturalgasintel.com/news/ferc-approves-extension-for-freeport-lngs-fourth-train-expansion-project/); [Federal Register](https://www.federalregister.gov/documents/2026/07/24/2026-15040/freeport-lng-development-lp-flng-liquefaction-llc-flng-liquefaction-2-llc-flng-liquefaction-3-llc)</t>
+          <t>Natural Gas Intel (https://www.naturalgasintel.com/news/ferc-approves-extension-for-freeport-lngs-fourth-train-expansion-project/); Federal Register (https://www.federalregister.gov/documents/2026/07/24/2026-15040/freeport-lng-development-lp-flng-liquefaction-llc-flng-liquefaction-2-llc-flng-liquefaction-3-llc)</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -3365,7 +3374,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>[Proyectos México](https://www.proyectosmexico.gob.mx/proyecto_inversion/1076-gasoducto-coatzacoalcos-ii/)</t>
+          <t>Proyectos México (https://www.proyectosmexico.gob.mx/proyecto_inversion/1076-gasoducto-coatzacoalcos-ii/)</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -3402,7 +3411,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>[LNG Industry](https://www.lngindustry.com/liquefaction/24072026/stabilis-solutions-receives-lor-from-us-coast-guard/)</t>
+          <t>LNG Industry (https://www.lngindustry.com/liquefaction/24072026/stabilis-solutions-receives-lor-from-us-coast-guard/)</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3439,7 +3448,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>[Federal Register](https://www.federalregister.gov/documents/2026/06/12/2026-11881/venture-global-cp2-lng-llc-venture-global-cp-express-llc-notice-of-application-and-establishing)</t>
+          <t>Federal Register (https://www.federalregister.gov/documents/2026/06/12/2026-11881/venture-global-cp2-lng-llc-venture-global-cp-express-llc-notice-of-application-and-establishing)</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -3476,7 +3485,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>[LNG Prime](https://lngprime.com/americas/cameron-lng-seeks-ferc-extension-for-expansion-project/167382/)</t>
+          <t>LNG Prime (https://lngprime.com/americas/cameron-lng-seeks-ferc-extension-for-expansion-project/167382/)</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -3513,7 +3522,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>[Federal Register](https://www.federalregister.gov/documents/2026/02/23/2026-03548/magnolia-lng-llc-notice-of-request-for-extension-of-time)</t>
+          <t>Federal Register (https://www.federalregister.gov/documents/2026/02/23/2026-03548/magnolia-lng-llc-notice-of-request-for-extension-of-time)</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -3550,7 +3559,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>[Storage Terminals Magazine](https://storageterminalsmag.com/kinder-morgans-trident-pipeline-project-enters-active-construction-phase-in-southeast-texas/); [Natural Gas Intel](https://www.naturalgasintel.com/news/kinder-morgan-greenlights-7b-in-natural-gas-pipeline-projects-amid-regulatory-speedup/)</t>
+          <t>Storage Terminals Magazine (https://storageterminalsmag.com/kinder-morgans-trident-pipeline-project-enters-active-construction-phase-in-southeast-texas/); Natural Gas Intel (https://www.naturalgasintel.com/news/kinder-morgan-greenlights-7b-in-natural-gas-pipeline-projects-amid-regulatory-speedup/)</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -3587,7 +3596,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>[Global Energy Monitor](https://www.gem.wiki/Centauro_del_Norte_Gas_Pipeline); [BNamericas](https://www.bnamericas.com/en/news/mexico-grants-permits-for-three-sonora-gas-projects)</t>
+          <t>Global Energy Monitor (https://www.gem.wiki/Centauro_del_Norte_Gas_Pipeline); BNamericas (https://www.bnamericas.com/en/news/mexico-grants-permits-for-three-sonora-gas-projects)</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -3624,7 +3633,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>[LNG Industry](https://www.lngindustry.com/liquid-natural-gas/07082026/enbridge-signs-option-to-acquire-ttc-connector/)</t>
+          <t>LNG Industry (https://www.lngindustry.com/liquid-natural-gas/07082026/enbridge-signs-option-to-acquire-ttc-connector/)</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -3644,50 +3653,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G77"/>
+  <dimension ref="A1:G80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -3716,17 +3725,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Ingeniería completada (PFS define mina subterránea de 20,000 t/d y planta de cátodos de 72,000 t/año) / construcción prevista H1 2026; EXIM Bank emitió carta de interés para financiamiento de hasta US$825 millones</t>
+          <t>Ingeniería completada (PFS define mina subterránea de 20,000 t/d y planta de cátodos de 72,000 t/año) / construcción prevista H1 2026; EXIM Bank gestiona ahora más de US$1,000 millones en financiamiento, como parte del paquete federal de US$3,000 millones en minerales críticos anunciado 7-8-ago-2026</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>[Mining Weekly](https://www.miningweekly.com/article/ivanhoe-electric-pencils-in-2026-construction-start-at-arizona-copper-mine-2025-06-25); [Ivanhoe Electric](https://ivanhoeelectric.com/news/ivanhoe-electric-receives-indication-for-up-to-825-million-in-financing-from-export-import-bank-of-the-united-states-for-santa/)</t>
+          <t>Mining Weekly (https://www.miningweekly.com/article/ivanhoe-electric-pencils-in-2026-construction-start-at-arizona-copper-mine-2025-06-25); MINING.COM (https://www.mining.com/web/trump-says-us-is-announcing-a-series-of-mining-projects-worth-3-billion/)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -3758,7 +3767,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>[SEC/Hudbay](https://www.sec.gov/Archives/edgar/data/1322422/000106299326001973/exhibit99-2.htm); [GlobeNewswire](https://www.globenewswire.com/news-release/2026/06/24/3317147/0/en/hudbay-completes-offering-of-us-52-million-of-4-50-municipal-bonds-for-copper-world.html)</t>
+          <t>SEC/Hudbay (https://www.sec.gov/Archives/edgar/data/1322422/000106299326001973/exhibit99-2.htm); GlobeNewswire (https://www.globenewswire.com/news-release/2026/06/24/3317147/0/en/hudbay-completes-offering-of-us-52-million-of-4-50-municipal-bonds-for-copper-world.html)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -3790,17 +3799,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Ingeniería temprana post intercambio de tierras (marzo 2026); firmó Master Supply Agreement (1-jul-2026) con Johnson Controls Inc. y United Association Local 469 (sindicato de plomeros/pipefitters) para mantenimiento de instalaciones y soporte operativo en sitio</t>
+          <t>Ingeniería temprana post intercambio de tierras (marzo 2026); firmó Master Supply Agreement (1-jul-2026) con Johnson Controls Inc. y UA Local 469; otorgó ~US$110 millones en contratos a Major Drilling America Inc. y Redpath USA Corporation (10-ago-2026) para acelerar exploración y desarrollo subterráneo, parte de programa de inversión de ~US$500 millones</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>[SEC](https://www.sec.gov/Archives/edgar/data/863064/000086306426000019/ex12d16mr_resolutionland.htm); [Resolution Copper](https://resolutioncopper.com/resolution-copper-and-united-association-local-469-enter-into-master-supply-agreement-supporting-operations-in-arizona/)</t>
+          <t>SEC (https://www.sec.gov/Archives/edgar/data/863064/000086306426000019/ex12d16mr_resolutionland.htm); International Mining (https://im-mining.com/2026/08/10/resolution-copper-accelerates-exploration-underground-development-with-major-drilling-redpath-contracts/)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -3832,7 +3841,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>[Mining Weekly](https://www.miningweekly.com/article/thacker-pass-lithium-project-us-update-2026-05-22); [Lithium Americas](https://lithiumamericas.com/news/news-details/2026/Lithium-Americas-Provides-a-Project-Update-and-2026-Capex-Guidance-for-Thacker-Pass/default.aspx)</t>
+          <t>Mining Weekly (https://www.miningweekly.com/article/thacker-pass-lithium-project-us-update-2026-05-22); Lithium Americas (https://lithiumamericas.com/news/news-details/2026/Lithium-Americas-Provides-a-Project-Update-and-2026-Capex-Guidance-for-Thacker-Pass/default.aspx)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -3869,7 +3878,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>[Mining.com](https://www.mining.com/teck-agnico-team-up-at-san-nicolas-copper-project-in-mexico/)</t>
+          <t>Mining.com (https://www.mining.com/teck-agnico-team-up-at-san-nicolas-copper-project-in-mexico/)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -3906,7 +3915,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>[Energy Magazine MX](https://energymagazine.mx/2025/10/grupo-mexico-espera-autorizacion-federal-para-continuar-proyectos-mineros-por-10-mil-200-mdd/)</t>
+          <t>Energy Magazine MX (https://energymagazine.mx/2025/10/grupo-mexico-espera-autorizacion-federal-para-continuar-proyectos-mineros-por-10-mil-200-mdd/)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -3943,7 +3952,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>[BNamericas](https://www.bnamericas.com/en/news/southern-copper-wins-permits-for-us551mn-el-pilar-in-mexico)</t>
+          <t>BNamericas (https://www.bnamericas.com/en/news/southern-copper-wins-permits-for-us551mn-el-pilar-in-mexico)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -3980,7 +3989,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>[M3 Engineering](https://m3eng.com/portfolio/buenavista-del-cobre-concentradora-no-2/)</t>
+          <t>M3 Engineering (https://m3eng.com/portfolio/buenavista-del-cobre-concentradora-no-2/)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -4017,7 +4026,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>[Minería en Línea](https://mineriaenlinea.com/2026/04/torex-gold-alcanza-velocidad-de-crucero-en-media-luna-9-meses-adelante-de-cronograma/)</t>
+          <t>Minería en Línea (https://mineriaenlinea.com/2026/04/torex-gold-alcanza-velocidad-de-crucero-en-media-luna-9-meses-adelante-de-cronograma/)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -4054,7 +4063,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>[Mining.com](https://www.mining.com/nevada-copper-unveils-restart-and-financing-plan-for-pumpkin-hollow/)</t>
+          <t>Mining.com (https://www.mining.com/nevada-copper-unveils-restart-and-financing-plan-for-pumpkin-hollow/)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -4091,7 +4100,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>[USDA](https://www.usda.gov/about-usda/news/press-releases/2026/07/07/usda-advances-trump-administration-effort-boost-us-mineral-energy-production); [Bloomberg](https://www.bloomberg.com/news/articles/2026-07-06/south32-s-arizona-zinc-and-manganese-mine-set-to-get-us-approval)</t>
+          <t>USDA (https://www.usda.gov/about-usda/news/press-releases/2026/07/07/usda-advances-trump-administration-effort-boost-us-mineral-energy-production); Bloomberg (https://www.bloomberg.com/news/articles/2026-07-06/south32-s-arizona-zinc-and-manganese-mine-set-to-get-us-approval)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -4128,7 +4137,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/perpetua-resources-advances-construction-of-the-stibnite-gold-project-302787012.html); [Departamento de Justicia de EE.UU.](https://www.justice.gov/opa/pr/justice-department-secures-motion-allow-continued-construction-idaho-gold-mine-critical)</t>
+          <t>PR Newswire (https://www.prnewswire.com/news-releases/perpetua-resources-advances-construction-of-the-stibnite-gold-project-302787012.html); Departamento de Justicia de EE.UU. (https://www.justice.gov/opa/pr/justice-department-secures-motion-allow-continued-construction-idaho-gold-mine-critical)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -4165,7 +4174,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>[Silver Tiger Metals](https://silvertigermetals.com/news/2026/silver-tiger-metals-awards-engineering-procurement-and-construction-management-contract-and-provides-construction-update)</t>
+          <t>Silver Tiger Metals (https://silvertigermetals.com/news/2026/silver-tiger-metals-awards-engineering-procurement-and-construction-management-contract-and-provides-construction-update)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -4202,7 +4211,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/vizsla-silver-awards-epcm-and-mine-design-contracts-for-the-development-of-the-panuco-silver-gold-project-302750621.html)</t>
+          <t>PR Newswire (https://www.prnewswire.com/news-releases/vizsla-silver-awards-epcm-and-mine-design-contracts-for-the-development-of-the-panuco-silver-gold-project-302750621.html)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -4239,7 +4248,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>[Orla Mining](https://orlamining.com/news/orla-announces-results-of-updated-feasibility-study-for-south-railroad-project/)</t>
+          <t>Orla Mining (https://orlamining.com/news/orla-announces-results-of-updated-feasibility-study-for-south-railroad-project/)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -4276,7 +4285,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>[Mining Weekly](https://www.miningweekly.com/article/minera-alamos-confirms-low-cost-near-term-mining-possible-at-copperstone-in-arizona-2026-05-28); [Minera Alamos](https://mineraalamos.com/news/2026/minera-alamos-announces-positive-pre-feasibility-study-for-the-copperstone-gold-project-in-arizona/)</t>
+          <t>Mining Weekly (https://www.miningweekly.com/article/minera-alamos-confirms-low-cost-near-term-mining-possible-at-copperstone-in-arizona-2026-05-28); Minera Alamos (https://mineraalamos.com/news/2026/minera-alamos-announces-positive-pre-feasibility-study-for-the-copperstone-gold-project-in-arizona/)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -4313,7 +4322,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>[Wyoming News](https://www.wyomingnews.com/rawlinstimes/plans-move-forward-for-ck-gold-project-as-developers-target-2026-construction-start/article_b2bb147e-2f92-4ca2-bf86-fcc9983917a7.html); [Discovery Alert](https://discoveryalert.com.au/ck-gold-project-permitting-construction-ready-valuation-2026/)</t>
+          <t>Wyoming News (https://www.wyomingnews.com/rawlinstimes/plans-move-forward-for-ck-gold-project-as-developers-target-2026-construction-start/article_b2bb147e-2f92-4ca2-bf86-fcc9983917a7.html); Discovery Alert (https://discoveryalert.com.au/ck-gold-project-permitting-construction-ready-valuation-2026/)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -4350,7 +4359,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>[First Majestic](https://www.juniorminingnetwork.com/junior-miner-news/press-releases/1082-tsx/ag/206222-first-majestic-receives-construction-permits-for-santo-nino-and-navidad-advances-development-across-the-santa-elena-district.html)</t>
+          <t>First Majestic (https://www.juniorminingnetwork.com/junior-miner-news/press-releases/1082-tsx/ag/206222-first-majestic-receives-construction-permits-for-santo-nino-and-navidad-advances-development-across-the-santa-elena-district.html)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -4387,7 +4396,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>[SEC/Americas Gold and Silver](https://www.sec.gov/Archives/edgar/data/0001286973/000106299326002645/exhibit99-2.htm)</t>
+          <t>SEC/Americas Gold and Silver (https://www.sec.gov/Archives/edgar/data/0001286973/000106299326002645/exhibit99-2.htm)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -4424,7 +4433,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>[Kitco](https://www.kitco.com/news/off-the-wire/2026-06-08/minera-frisco-restarts-two-mexico-mines-plans-new-silver-unit)</t>
+          <t>Kitco (https://www.kitco.com/news/off-the-wire/2026-06-08/minera-frisco-restarts-two-mexico-mines-plans-new-silver-unit)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -4461,7 +4470,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/trilogy-metals-announces-publication-of-federal-and-state-permitting-schedule-for-arctic-project-establishing-defined-timeline-toward-a-record-of-decision-by-september-2028-302827083.html)</t>
+          <t>PR Newswire (https://www.prnewswire.com/news-releases/trilogy-metals-announces-publication-of-federal-and-state-permitting-schedule-for-arctic-project-establishing-defined-timeline-toward-a-record-of-decision-by-september-2028-302827083.html)</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -4498,7 +4507,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>[Northern Miner](https://www.northernminer.com/news/gogold-approved-to-build-227m-mine-in-mexico/1003891932/); [Newsfile](https://www.newsfilecorp.com/release/300455/GoGold-Achieves-Major-Milestone-Final-Remaining-Permits-Secured-and-Construction-Approved-for-Los-Ricos-South-Underground-Mine)</t>
+          <t>Northern Miner (https://www.northernminer.com/news/gogold-approved-to-build-227m-mine-in-mexico/1003891932/); Newsfile (https://www.newsfilecorp.com/release/300455/GoGold-Achieves-Major-Milestone-Final-Remaining-Permits-Secured-and-Construction-Approved-for-Los-Ricos-South-Underground-Mine)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -4535,7 +4544,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>[BNamericas](https://www.bnamericas.com/en/news/discovery-advances-permitting-financing-at-us606mn-cordero-in-mexico)</t>
+          <t>BNamericas (https://www.bnamericas.com/en/news/discovery-advances-permitting-financing-at-us606mn-cordero-in-mexico)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -4572,7 +4581,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>[Resource World](https://resourceworld.com/tocvan-ventures-eyes-mexican-gold-pour-by-q4-2026/)</t>
+          <t>Resource World (https://resourceworld.com/tocvan-ventures-eyes-mexican-gold-pour-by-q4-2026/)</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -4609,7 +4618,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>[Fresnillo plc](https://www.fresnilloplc.com/portfolio/exploration/orisyvo/)</t>
+          <t>Fresnillo plc (https://www.fresnilloplc.com/portfolio/exploration/orisyvo/)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -4646,7 +4655,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>[Army.mil](https://www.army.mil/article/293503/army_announces_conditional_lease_awards_for_domestic_critical_mineral_processing_facilities_to_secure_defense_supply_chains)</t>
+          <t>Army.mil (https://www.army.mil/article/293503/army_announces_conditional_lease_awards_for_domestic_critical_mineral_processing_facilities_to_secure_defense_supply_chains)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -4683,7 +4692,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>[Mining.com](https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/)</t>
+          <t>Mining.com (https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/)</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -4720,7 +4729,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>[Mining.com](https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/)</t>
+          <t>Mining.com (https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/)</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -4757,7 +4766,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>[IM Mining](https://im-mining.com/2026/06/29/metso-to-supply-additional-crushing-package-for-grupo-mexico-la-caridad-copper-concentrator/)</t>
+          <t>IM Mining (https://im-mining.com/2026/06/29/metso-to-supply-additional-crushing-package-for-grupo-mexico-la-caridad-copper-concentrator/)</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -4794,7 +4803,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/05/21/3299182)</t>
+          <t>GlobeNewswire (https://www.globenewswire.com/news-release/2026/05/21/3299182)</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -4831,7 +4840,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>[Mexico Business News](https://mexicobusiness.news/mining/news/grupo-mexicos-asarco-may-reopen-united-states)</t>
+          <t>Mexico Business News (https://mexicobusiness.news/mining/news/grupo-mexicos-asarco-may-reopen-united-states)</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -4868,7 +4877,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>[Minera Alamos](https://mineraalamos.com/our-assets/cerro-de-oro-project/)</t>
+          <t>Minera Alamos (https://mineraalamos.com/our-assets/cerro-de-oro-project/)</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -4905,7 +4914,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>[Global Mining Review](https://www.globalminingreview.com/mining/11022025/antler-copper-project-achieves-critical-federal-permitting-milestone/)</t>
+          <t>Global Mining Review (https://www.globalminingreview.com/mining/11022025/antler-copper-project-achieves-critical-federal-permitting-milestone/)</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -4942,7 +4951,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>[BLM](https://www.blm.gov/press-release/blm-approves-lisbon-valley-copper-mine-expansion-utah)</t>
+          <t>BLM (https://www.blm.gov/press-release/blm-approves-lisbon-valley-copper-mine-expansion-utah)</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -4979,7 +4988,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>[InvestingNews](https://investingnews.com/smackover-lithium-announces-the-award-of-last-key-construction-contract-for-the-south-west-arkansas-project-ahead-of-final-investment-decision/); [StockTitan/SEC 6-K](https://www.stocktitan.net/sec-filings/SLI/6-k-standard-lithium-ltd-current-report-foreign-issuer-ef7db860baa3.html)</t>
+          <t>InvestingNews (https://investingnews.com/smackover-lithium-announces-the-award-of-last-key-construction-contract-for-the-south-west-arkansas-project-ahead-of-final-investment-decision/); StockTitan/SEC 6-K (https://www.stocktitan.net/sec-filings/SLI/6-k-standard-lithium-ltd-current-report-foreign-issuer-ef7db860baa3.html)</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -5016,7 +5025,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>[SEC/Freeport-McMoRan](https://www.sec.gov/Archives/edgar/data/0000831259/000083125926000033/a2q2026exhibit991.htm)</t>
+          <t>SEC/Freeport-McMoRan (https://www.sec.gov/Archives/edgar/data/0000831259/000083125926000033/a2q2026exhibit991.htm)</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -5053,7 +5062,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>[NioCorp](https://niocorp.com/niocorp-launches-construction-of-elk-creek-critical-minerals-project-mine-portal/)</t>
+          <t>NioCorp (https://niocorp.com/niocorp-launches-construction-of-elk-creek-critical-minerals-project-mine-portal/)</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -5090,7 +5099,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>[E&amp;MJ](https://www.e-mj.com/breaking-news/centerra-advances-goldfield-project-in-nevada/)</t>
+          <t>E&amp;MJ (https://www.e-mj.com/breaking-news/centerra-advances-goldfield-project-in-nevada/)</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -5127,7 +5136,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/03/02/3247157/0/en/hudbay-to-acquire-arizona-sonoran-creating-the-third-largest-copper-district-in-north-america.html); [Arizona Sonoran](https://arizonasonoran.com/news-releases/arizona-sonoran-pre-feasibility-study-delivers-exceptional-results-for-the-cactus-project-outlining-long-life-low-cost-copper-1/)</t>
+          <t>GlobeNewswire (https://www.globenewswire.com/news-release/2026/03/02/3247157/0/en/hudbay-to-acquire-arizona-sonoran-creating-the-third-largest-copper-district-in-north-america.html); Arizona Sonoran (https://arizonasonoran.com/news-releases/arizona-sonoran-pre-feasibility-study-delivers-exceptional-results-for-the-cactus-project-outlining-long-life-low-cost-copper-1/)</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -5164,7 +5173,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>[Western Exploration](https://www.westernexploration.com/news-and-updates/news/news-details/2026/Western-Exploration-Outlines-2026-Program-to-Advance-Doby-George-Permitting-and-Expand-Gravel-Creek-Resources-2026-aaotfYHcV7/default.aspx); [StreetWise Reports](https://www.streetwisereports.com/article/2026/08/03/nevada-gold-project-launches-drill-campaign-at-doby-george.html)</t>
+          <t>Western Exploration (https://www.westernexploration.com/news-and-updates/news/news-details/2026/Western-Exploration-Outlines-2026-Program-to-Advance-Doby-George-Permitting-and-Expand-Gravel-Creek-Resources-2026-aaotfYHcV7/default.aspx); StreetWise Reports (https://www.streetwisereports.com/article/2026/08/03/nevada-gold-project-launches-drill-campaign-at-doby-george.html)</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -5201,7 +5210,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>[Chesapeake Gold Corp.](https://chesapeakegold.com/metates/)</t>
+          <t>Chesapeake Gold Corp. (https://chesapeakegold.com/metates/)</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -5238,7 +5247,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>[Mining Technology](https://www.mining-technology.com/news/pathfinder-896m-loi-us-exim-copper-mine/)</t>
+          <t>Mining Technology (https://www.mining-technology.com/news/pathfinder-896m-loi-us-exim-copper-mine/)</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -5275,7 +5284,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>[Mexico Business News](https://mexicobusiness.news/mining/news/heliostar-advances-la-colorada-pit-permits-drill-data)</t>
+          <t>Mexico Business News (https://mexicobusiness.news/mining/news/heliostar-advances-la-colorada-pit-permits-drill-data)</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -5312,7 +5321,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>[The Western News](https://thewesternnews.com/news/2026/jul/24/libby-mining-project-takes-another-step-forward-with-federal-ok/)</t>
+          <t>The Western News (https://thewesternnews.com/news/2026/jul/24/libby-mining-project-takes-another-step-forward-with-federal-ok/)</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -5349,7 +5358,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>[Mining News North](https://www.miningnewsnorth.com/story/2026/07/24/news/donlin-gold-partners-form-new-novagold/9781.html)</t>
+          <t>Mining News North (https://www.miningnewsnorth.com/story/2026/07/24/news/donlin-gold-partners-form-new-novagold/9781.html)</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -5386,7 +5395,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>[IM Mining](https://im-mining.com/2026/06/23/ioneer-signals-progress-on-rhyolite-ridge-lithium-boron-project-with-kind-and-hyundai-engineering-pacts/)</t>
+          <t>IM Mining (https://im-mining.com/2026/06/23/ioneer-signals-progress-on-rhyolite-ridge-lithium-boron-project-with-kind-and-hyundai-engineering-pacts/)</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -5423,7 +5432,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>[Resource World](https://resourceworld.com/axo-metals-secures-major-environmental-permit-approval-clears-path-for-production-at-the-san-antonio-gold-project/)</t>
+          <t>Resource World (https://resourceworld.com/axo-metals-secures-major-environmental-permit-approval-clears-path-for-production-at-the-san-antonio-gold-project/)</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -5460,7 +5469,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>[Talon Metals](https://talonmetals.com/talon-metals-and-westmoreland-mining-sign-land-agreement-to-progress-north-dakota-minerals-processing-facility/)</t>
+          <t>Talon Metals (https://talonmetals.com/talon-metals-and-westmoreland-mining-sign-land-agreement-to-progress-north-dakota-minerals-processing-facility/)</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -5497,7 +5506,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/31/3337077/0/en/bunker-hill-ships-first-concentrate-to-trail-smelter-and-announces-drawdown-of-standby-facility.html)</t>
+          <t>GlobeNewswire (https://www.globenewswire.com/news-release/2026/07/31/3337077/0/en/bunker-hill-ships-first-concentrate-to-trail-smelter-and-announces-drawdown-of-standby-facility.html)</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -5534,7 +5543,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>[MPR News](https://www.mprnews.org/story/2026/07/30/newrange-copper-nickel-proposes-major-changes-to-copper-mine-plan)</t>
+          <t>MPR News (https://www.mprnews.org/story/2026/07/30/newrange-copper-nickel-proposes-major-changes-to-copper-mine-plan)</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -5571,7 +5580,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>[Energy Fuels](https://investors.energyfuels.com/2026-07-29-Commercial-Scale-Heavy-Rare-Earth-Plant-Now-Under-Construction-in-Utah); [PR Newswire](https://www.prnewswire.com/news-releases/commercial-scale-heavy-rare-earth-plant-now-under-construction-in-utah-302837314.html)</t>
+          <t>Energy Fuels (https://investors.energyfuels.com/2026-07-29-Commercial-Scale-Heavy-Rare-Earth-Plant-Now-Under-Construction-in-Utah); PR Newswire (https://www.prnewswire.com/news-releases/commercial-scale-heavy-rare-earth-plant-now-under-construction-in-utah-302837314.html)</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -5608,7 +5617,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/29/3334925/0/en/sandfire-resources-america-files-black-butte-copper-project-preliminary-feasibility-study.html)</t>
+          <t>GlobeNewswire (https://www.globenewswire.com/news-release/2026/07/29/3334925/0/en/sandfire-resources-america-files-black-butte-copper-project-preliminary-feasibility-study.html)</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -5645,7 +5654,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>[Texarkana Gazette](https://www.texarkanagazette.com/news/2026/jun/30/army-awards-lithium-company-energyx-conditional/)</t>
+          <t>Texarkana Gazette (https://www.texarkanagazette.com/news/2026/jun/30/army-awards-lithium-company-energyx-conditional/)</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -5682,7 +5691,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>[Mining.com](https://www.mining.com/orla-secures-final-permit-to-advance-underground-mining-at-camino-rojo/); [Orla Mining](https://orlamining.com/news/orla-mining-receives-permits-to-extend-operations-in-mexico-supporting-companys-long-term-commitment-to-camino-rojo/)</t>
+          <t>Mining.com (https://www.mining.com/orla-secures-final-permit-to-advance-underground-mining-at-camino-rojo/); Orla Mining (https://orlamining.com/news/orla-mining-receives-permits-to-extend-operations-in-mexico-supporting-companys-long-term-commitment-to-camino-rojo/)</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -5719,7 +5728,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>[Sonoro Gold Corp.](https://sonorogold.com/wp-content/uploads/2026/03/2026.03.01_Sonoro-Gold-Corporate-Presentation.pdf); [Mexico Mining Center](https://www.mexicominingcenter.com/sonoro-continues-discussions-with-china-based-epc-companies-and-potential-equity-investors/)</t>
+          <t>Sonoro Gold Corp. (https://sonorogold.com/wp-content/uploads/2026/03/2026.03.01_Sonoro-Gold-Corporate-Presentation.pdf); Mexico Mining Center (https://www.mexicominingcenter.com/sonoro-continues-discussions-with-china-based-epc-companies-and-potential-equity-investors/)</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -5756,7 +5765,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>[Mining Weekly](https://www.miningweekly.com/article/guardian-metals-outlines-viable-tungsten-trioxide-operation-in-nevada-2026-06-30); [StockTitan](https://www.stocktitan.net/news/GMTL/guardian-metal-resources-plc-announces-pilot-mountain-pre-tftnlr9fu3if.html)</t>
+          <t>Mining Weekly (https://www.miningweekly.com/article/guardian-metals-outlines-viable-tungsten-trioxide-operation-in-nevada-2026-06-30); StockTitan (https://www.stocktitan.net/news/GMTL/guardian-metal-resources-plc-announces-pilot-mountain-pre-tftnlr9fu3if.html)</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -5793,7 +5802,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>[Newswire](https://www.newswire.ca/news-releases/p2-gold-gabbs-project-update-feasibility-study-on-track-840759204.html)</t>
+          <t>Newswire (https://www.newswire.ca/news-releases/p2-gold-gabbs-project-update-feasibility-study-on-track-840759204.html)</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -5830,7 +5839,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/buscar-company-announces-major-advancement-in-the-permitting-process-for-the-treasure-canyon-gold-mine-project-in-california-302772744.html)</t>
+          <t>PR Newswire (https://www.prnewswire.com/news-releases/buscar-company-announces-major-advancement-in-the-permitting-process-for-the-treasure-canyon-gold-mine-project-in-california-302772744.html)</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -5867,7 +5876,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/01/29/3229150/0/en/Paramount-Gold-Receives-Federal-Approval-for-the-Grassy-Mountain-Gold-Project.html); [OPB](https://www.opb.org/article/2026/01/29/oregon-gold-mine-grassy-mountain/)</t>
+          <t>GlobeNewswire (https://www.globenewswire.com/news-release/2026/01/29/3229150/0/en/Paramount-Gold-Receives-Federal-Approval-for-the-Grassy-Mountain-Gold-Project.html); OPB (https://www.opb.org/article/2026/01/29/oregon-gold-mine-grassy-mountain/)</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -5904,7 +5913,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>[CNBC](https://www.cnbc.com/2026/02/26/mp-materials-selects-texas-for-rare-earth-magnet-manufacturing-site.html)</t>
+          <t>CNBC (https://www.cnbc.com/2026/02/26/mp-materials-selects-texas-for-rare-earth-magnet-manufacturing-site.html)</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -5941,7 +5950,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/the-united-states-is-investing-in-its-domestic-rare-earth-industry-302838375.html)</t>
+          <t>PR Newswire (https://www.prnewswire.com/news-releases/the-united-states-is-investing-in-its-domestic-rare-earth-industry-302838375.html)</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -5978,7 +5987,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>[Newsfile Corp](https://www.newsfilecorp.com/release/283399/Americas-Gold-and-Silver-Signs-Joint-Venture-Agreement-with-US-Antimony-to-Construct-Antimony-Processing-Facility-in-Idahos-Silver-Valley-Unlocking-Value-from-Its-Antimony-Production-and-Strengthening-U.S.-Critical-Mineral-Security)</t>
+          <t>Newsfile Corp (https://www.newsfilecorp.com/release/283399/Americas-Gold-and-Silver-Signs-Joint-Venture-Agreement-with-US-Antimony-to-Construct-Antimony-Processing-Facility-in-Idahos-Silver-Valley-Unlocking-Value-from-Its-Antimony-Production-and-Strengthening-U.S.-Critical-Mineral-Security)</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -6015,7 +6024,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>[DOE-LPO](https://www.energy.gov/lpo/articles/lpo-announces-conditional-commitment-michigan-potash-produce-fertilizer-us-farmers); [Northern Miner](https://www.northernminer.com/news/us-boosts-potash-projects-in-utah-michigan/1003886533/)</t>
+          <t>DOE-LPO (https://www.energy.gov/lpo/articles/lpo-announces-conditional-commitment-michigan-potash-produce-fertilizer-us-farmers); Northern Miner (https://www.northernminer.com/news/us-boosts-potash-projects-in-utah-michigan/1003886533/)</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -6052,7 +6061,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>[BLM](https://www.blm.gov/announcement/blm-approves-construction-sevier-playa-potash-mining-project)</t>
+          <t>BLM (https://www.blm.gov/announcement/blm-approves-construction-sevier-playa-potash-mining-project)</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -6089,7 +6098,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>[Ur-Energy](https://www.ur-energy.com/news-media/press-releases/detail/401/ur-energy-commences-operations-at-its-shirley-basin-isr)</t>
+          <t>Ur-Energy (https://www.ur-energy.com/news-media/press-releases/detail/401/ur-energy-commences-operations-at-its-shirley-basin-isr)</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -6126,7 +6135,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>[Mexico Business News](https://mexicobusiness.news/mining/news/silverco-targets-late-2026-restart-past-producing-cusi-mine); [Investing News Network](https://investingnews.com/silverco-mining-begins-underground-development-at-cusi-restart-remains-on-budget-and-on-schedule/)</t>
+          <t>Mexico Business News (https://mexicobusiness.news/mining/news/silverco-targets-late-2026-restart-past-producing-cusi-mine); Investing News Network (https://investingnews.com/silverco-mining-begins-underground-development-at-cusi-restart-remains-on-budget-and-on-schedule/)</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -6163,7 +6172,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>[Junior Mining Network](https://www.juniorminingnetwork.com/junior-miner-news/press-releases/2342-tsx/ti/199070-titan-mining-to-start-shipping-first-graphite-product-and-feasibility-study-underway-for-40-000-tpa-integrated-kilbourne-graphite-project.html)</t>
+          <t>Junior Mining Network (https://www.juniorminingnetwork.com/junior-miner-news/press-releases/2342-tsx/ti/199070-titan-mining-to-start-shipping-first-graphite-product-and-feasibility-study-underway-for-40-000-tpa-integrated-kilbourne-graphite-project.html)</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -6200,7 +6209,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>[Permitting Council](https://www.permitting.gov/newsroom/success-stories/project-spotlight-graphite-creek-project)</t>
+          <t>Permitting Council (https://www.permitting.gov/newsroom/success-stories/project-spotlight-graphite-creek-project)</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -6237,7 +6246,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>[Pan American Silver](https://panamericansilver.com/news/pan-american-announces-revised-pea-for-the-la-colorada-skarn-project-positions-la-colorada-as-a-future-top-tier-silver-mine/); [SEC 6-K](https://www.sec.gov/Archives/edgar/data/771992/000077199226000031/a2026_03x24lacoloradapeaup.htm)</t>
+          <t>Pan American Silver (https://panamericansilver.com/news/pan-american-announces-revised-pea-for-the-la-colorada-skarn-project-positions-la-colorada-as-a-future-top-tier-silver-mine/); SEC 6-K (https://www.sec.gov/Archives/edgar/data/771992/000077199226000031/a2026_03x24lacoloradapeaup.htm)</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -6274,7 +6283,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/i-80-gold-provides-update-on-lone-tree-plant-refurbishment-project-remains-on-schedule-and-on-budget-302836341.html)</t>
+          <t>PR Newswire (https://www.prnewswire.com/news-releases/i-80-gold-provides-update-on-lone-tree-plant-refurbishment-project-remains-on-schedule-and-on-budget-302836341.html)</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -6311,7 +6320,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/29/3335652/0/en/Kinross-reports-strong-2026-second-quarter-results.html)</t>
+          <t>GlobeNewswire (https://www.globenewswire.com/news-release/2026/07/29/3335652/0/en/Kinross-reports-strong-2026-second-quarter-results.html)</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -6348,7 +6357,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/29/3335652/0/en/Kinross-reports-strong-2026-second-quarter-results.html)</t>
+          <t>GlobeNewswire (https://www.globenewswire.com/news-release/2026/07/29/3335652/0/en/Kinross-reports-strong-2026-second-quarter-results.html)</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -6385,7 +6394,7 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>[Federal Register](https://www.federalregister.gov/documents/2026/07/29/2026-15255/black-hills-national-forest-wyoming-bear-lodge-rare-earth-project)</t>
+          <t>Federal Register (https://www.federalregister.gov/documents/2026/07/29/2026-15255/black-hills-national-forest-wyoming-bear-lodge-rare-earth-project)</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -6422,7 +6431,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>[Minería en Línea](https://mineriaenlinea.com/2026/07/southern-copper-obtiene-permisos-ambientales-para-el-pilar-produccion-a-partir-de-2029/)</t>
+          <t>Minería en Línea (https://mineriaenlinea.com/2026/07/southern-copper-obtiene-permisos-ambientales-para-el-pilar-produccion-a-partir-de-2029/)</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -6459,7 +6468,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>[Minería en Línea](https://mineriaenlinea.com/2026/07/southern-copper-obtiene-permisos-ambientales-para-el-pilar-produccion-a-partir-de-2029/)</t>
+          <t>Minería en Línea (https://mineriaenlinea.com/2026/07/southern-copper-obtiene-permisos-ambientales-para-el-pilar-produccion-a-partir-de-2029/)</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -6496,12 +6505,123 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>[Minería en Línea](https://mineriaenlinea.com/2026/07/southern-copper-obtiene-permisos-ambientales-para-el-pilar-produccion-a-partir-de-2029/)</t>
+          <t>Minería en Línea (https://mineriaenlinea.com/2026/07/southern-copper-obtiene-permisos-ambientales-para-el-pilar-produccion-a-partir-de-2029/)</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
           <t>2026-08-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Coosa Graphite Project (Kellyton Graphite Plant)</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Condado de Coosa, Alabama, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Westwater Resources Inc.</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Financiamiento/planeación (préstamo EXIM Bank de US$25 millones anunciado 7-ago-2026 para mina de grafito natural y planta de procesamiento, primera fuente de grafito natural producida en EE.UU.)</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Yellowhammer News (https://yellowhammernews.com/trump-administration-announces-25-million-exim-loan-for-westwaters-coosa-county-graphite-plant/); EXIM.GOV (https://www.exim.gov/news/trump-administration-announces-58m-major-new-critical-mineral-deals-white-house-roundtable)</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Expansión de Procesamiento de Tantalio/Niobio (Global Advanced Metals)</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Pensilvania, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Global Advanced Metals</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Financiamiento/planeación (préstamo EXIM Bank de US$25 millones anunciado 7-ago-2026 para ampliar capacidad de procesamiento)</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>EXIM.GOV (https://www.exim.gov/news/trump-administration-announces-58m-major-new-critical-mineral-deals-white-house-roundtable); SME (https://me.smenet.org/trump-administration-to-back-three-mineral-projects-with-58-million-in-financing/)</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Boron Americas Project (Fort Cady)</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>California, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>5E Advanced Materials</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Financiamiento/planeación (préstamo EXIM Bank de US$8 millones anunciado 7-ago-2026 para proyecto de boro, lixiviación/procesamiento)</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>EXIM.GOV (https://www.exim.gov/news/trump-administration-announces-58m-major-new-critical-mineral-deals-white-house-roundtable)</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -6516,50 +6636,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G81"/>
+  <dimension ref="A1:G82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -6593,7 +6713,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/vantage-breaks-ground-on-texas-gigawatt-data-center-campus-for-openai/); [Construction Owners](https://www.constructionowners.com/news/oracle-and-openai-to-power-new-texas-data-center-off-the-grid)</t>
+          <t>DCD (https://www.datacenterdynamics.com/en/news/vantage-breaks-ground-on-texas-gigawatt-data-center-campus-for-openai/); Construction Owners (https://www.constructionowners.com/news/oracle-and-openai-to-power-new-texas-data-center-off-the-grid)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -6630,7 +6750,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>[Epoch AI](https://epoch.ai/publications/openai-stargate-where-the-us-sites-stand)</t>
+          <t>Epoch AI (https://epoch.ai/publications/openai-stargate-where-the-us-sites-stand)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -6667,7 +6787,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/crusoe-tops-out-final-building-at-openai-stargate-data-center-campus-in-abilene-texas/)</t>
+          <t>DCD (https://www.datacenterdynamics.com/en/news/crusoe-tops-out-final-building-at-openai-stargate-data-center-campus-in-abilene-texas/)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -6704,7 +6824,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>[Chevron](https://www.chevron.com/newsroom/2026/q2/chevron-signs-20-year-power-agreement-with-microsoft-for-west-texas-data-center)</t>
+          <t>Chevron (https://www.chevron.com/newsroom/2026/q2/chevron-signs-20-year-power-agreement-with-microsoft-for-west-texas-data-center)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -6741,7 +6861,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>[Gobierno de México](https://www.gob.mx/presidencia/prensa/plan-mexico-avanza-se-anuncia-inversion-de-4-mil-800-mdd-de-cloudhq-para-la-construccion-de-6-centros-de-datos-en-queretaro)</t>
+          <t>Gobierno de México (https://www.gob.mx/presidencia/prensa/plan-mexico-avanza-se-anuncia-inversion-de-4-mil-800-mdd-de-cloudhq-para-la-construccion-de-6-centros-de-datos-en-queretaro)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -6778,7 +6898,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>[Global Data Center Hub](https://www.globaldatacenterhub.com/p/meta-scales-hyperion-to-5gw-and-over)</t>
+          <t>Global Data Center Hub (https://www.globaldatacenterhub.com/p/meta-scales-hyperion-to-5gw-and-over)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -6815,7 +6935,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55305086/nv1-and-the-nevada-hyperscale-boom-vantage-data-centers-bets-3b-on-the-ai-future)</t>
+          <t>Data Center Frontier (https://www.datacenterfrontier.com/site-selection/article/55305086/nv1-and-the-nevada-hyperscale-boom-vantage-data-centers-bets-3b-on-the-ai-future)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -6852,7 +6972,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/cloudburst-breaks-ground-on-gigawatt-scale-data-center-campus-in-texas/)</t>
+          <t>DCD (https://www.datacenterdynamics.com/en/news/cloudburst-breaks-ground-on-gigawatt-scale-data-center-campus-in-texas/)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -6889,7 +7009,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/prometheus-hyperscale-details-plans-for-dallas-data-center-campus/)</t>
+          <t>DCD (https://www.datacenterdynamics.com/en/news/prometheus-hyperscale-details-plans-for-dallas-data-center-campus/)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -6921,17 +7041,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Construcción de edificios de centro de datos iniciada (TCEQ ya había otorgado permiso de aire para 7.65GW de generación a gas; Amazon presentó a inicios de ago-2026 permisos de construcción para 3 edificios de centro de datos —"Pecos County Data Center", Buildings A/B/C, ~189,060 pies² c/u, ~US$300M c/u—; construcción de edificios prevista ago-dic 2026; Fase 1 de 1GW de generación prevista en operación 1S2027)</t>
+          <t>Construcción de edificios de centro de datos iniciada (TCEQ emitió permiso de aire final para la planta —35 turbinas de gas natural, hasta 33 millones de toneladas de CO2/año—; Amazon presentó a inicios de ago-2026 permisos de construcción para 3 edificios de centro de datos —"Pecos County Data Center", Buildings A/B/C, ~189,060 pies² c/u, ~US$300M c/u—; construcción de edificios prevista ago-dic 2026; primera entrega de energía prevista 1T2027, operando inicialmente fuera de la red de ERCOT)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>[Business Wire](https://www.businesswire.com/news/home/20260126236053/en/Pacifico-Energy-Secures-7.65-GW-Power-Generation-Permit-for-GW-Ranch-Project); [US Data Center Projects](https://usdatacenterprojects.com/texas/amazon-files-plans-for-new-data-center-buildings-in-texas-across-three-sites)</t>
+          <t>Business Wire (https://www.businesswire.com/news/home/20260126236053/en/Pacifico-Energy-Secures-7.65-GW-Power-Generation-Permit-for-GW-Ranch-Project); Tom's Hardware (https://www.tomshardware.com/tech-industry/data-centers/amazons-new-7-65gw-texas-ai-data-center-power-plant-could-become-the-largest-source-of-co2-pollution-in-the-us-custom-35-turbine-gas-plant-authorized-to-emit-33-million-tons-of-annual-greenhouse-gases)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -6963,7 +7083,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/amazon-looks-to-build-large-scale-data-center-campus-next-to-nuclear-plant-in-texas/)</t>
+          <t>DCD (https://www.datacenterdynamics.com/en/news/amazon-looks-to-build-large-scale-data-center-campus-next-to-nuclear-plant-in-texas/)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -7000,7 +7120,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>[Mexico News Daily](https://mexiconewsdaily.com/business/durango-data-center-fertilizer-plant-investment-fermaca/); [DCD](https://www.datacenterdynamics.com/en/news/250mw-natural-gas-powered-data-center-campus-announced-in-durango-mexico/)</t>
+          <t>Mexico News Daily (https://mexiconewsdaily.com/business/durango-data-center-fertilizer-plant-investment-fermaca/); DCD (https://www.datacenterdynamics.com/en/news/250mw-natural-gas-powered-data-center-campus-announced-in-durango-mexico/)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -7037,7 +7157,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/circe-energy-secures-2gw-of-natural-gas-capacity-for-west-texas-data-center-campus/)</t>
+          <t>DCD (https://www.datacenterdynamics.com/en/news/circe-energy-secures-2gw-of-natural-gas-capacity-for-west-texas-data-center-campus/)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -7074,7 +7194,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>[Source NM](https://sourcenm.com/2026/07/16/new-mexico-land-commissioner-blocks-project-jupiter-related-pipeline-from-building-on-state-land/)</t>
+          <t>Source NM (https://sourcenm.com/2026/07/16/new-mexico-land-commissioner-blocks-project-jupiter-related-pipeline-from-building-on-state-land/)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -7111,7 +7231,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/powerplay-ai-announces-400-mw-behind-the-meter-ai-data-center-development-in-greater-abilene-with-nasdaq-listed-neocloud-joint-venture-partner-302829610.html)</t>
+          <t>PR Newswire (https://www.prnewswire.com/news-releases/powerplay-ai-announces-400-mw-behind-the-meter-ai-data-center-development-in-greater-abilene-with-nasdaq-listed-neocloud-joint-venture-partner-302829610.html)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -7148,7 +7268,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/liberty-energy-powerbridge-form-jv-to-power-planned-2gw-data-center-in-west-texas/)</t>
+          <t>DCD (https://www.datacenterdynamics.com/en/news/liberty-energy-powerbridge-form-jv-to-power-planned-2gw-data-center-in-west-texas/)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -7185,7 +7305,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>[PowerMag](https://www.powermag.com/nuclear-natural-gas-power-generation-planned-for-massive-new-mexico-data-center-site/)</t>
+          <t>PowerMag (https://www.powermag.com/nuclear-natural-gas-power-generation-planned-for-massive-new-mexico-data-center-site/)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -7222,7 +7342,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55289667/powering-ai-in-the-permian-texas-critical-data-centers-sustainable-energy-play)</t>
+          <t>Data Center Frontier (https://www.datacenterfrontier.com/site-selection/article/55289667/powering-ai-in-the-permian-texas-critical-data-centers-sustainable-energy-play)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -7259,7 +7379,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>[OpenAI](https://openai.com/index/five-new-stargate-sites/)</t>
+          <t>OpenAI (https://openai.com/index/five-new-stargate-sites/)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -7296,7 +7416,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>[OpenAI](https://openai.com/index/five-new-stargate-sites/)</t>
+          <t>OpenAI (https://openai.com/index/five-new-stargate-sites/)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -7333,7 +7453,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>[Mexico News Daily](https://mexiconewsdaily.com/business/aws-invest-5b-mexico-data-region/)</t>
+          <t>Mexico News Daily (https://mexiconewsdaily.com/business/aws-invest-5b-mexico-data-region/)</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -7370,7 +7490,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/oracle-and-openai-start-construction-on-stargate-data-center-campus-in-saline-township-michigan/)</t>
+          <t>DCD (https://www.datacenterdynamics.com/en/news/oracle-and-openai-start-construction-on-stargate-data-center-campus-in-saline-township-michigan/)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -7407,7 +7527,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>[Valley News Live](https://www.valleynewslive.com/2026/07/13/applied-digital-expands-north-dakota-eyes-oliver-county-third-data-center/)</t>
+          <t>Valley News Live (https://www.valleynewslive.com/2026/07/13/applied-digital-expands-north-dakota-eyes-oliver-county-third-data-center/)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -7444,7 +7564,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>[Energy Magazine MX](https://energymagazine.mx/2026/01/el-data-center-verde-que-encendio-la-polemica-asi-sera-el-proyecto-de-ia-en-nuevo-leon-que-usara-tecnologia-de-nvidia/)</t>
+          <t>Energy Magazine MX (https://energymagazine.mx/2026/01/el-data-center-verde-que-encendio-la-polemica-asi-sera-el-proyecto-de-ia-en-nuevo-leon-que-usara-tecnologia-de-nvidia/)</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -7481,7 +7601,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>[Construction Dive](https://www.constructiondive.com/news/data-center-cleanarc-breaks-ground-virginia-campus/806489/)</t>
+          <t>Construction Dive (https://www.constructiondive.com/news/data-center-cleanarc-breaks-ground-virginia-campus/806489/)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -7518,7 +7638,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>[KSL](https://www.ksl.com/article/51402125/groundbreaking-for-new-millard-county-artificial-intelligence-data-center)</t>
+          <t>KSL (https://www.ksl.com/article/51402125/groundbreaking-for-new-millard-county-artificial-intelligence-data-center)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -7555,7 +7675,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>[Governor.mo.gov](https://governor.mo.gov/press-releases/archive/amazon-investing-10-billion-montgomery-county)</t>
+          <t>Governor.mo.gov (https://governor.mo.gov/press-releases/archive/amazon-investing-10-billion-montgomery-county)</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -7592,7 +7712,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>[STLPR](https://www.stlpr.org/government-politics-issues/2026-05-21/missouri-governor-google-announce-15-billion-data-center-montgomery-county)</t>
+          <t>STLPR (https://www.stlpr.org/government-politics-issues/2026-05-21/missouri-governor-google-announce-15-billion-data-center-montgomery-county)</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -7629,7 +7749,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/06/3322404/0/en/big-digital-energy-announces-partnership-with-10netzero-to-acquire-power-ready-hood-county-texas-site-for-ai-datacenter-development.html)</t>
+          <t>GlobeNewswire (https://www.globenewswire.com/news-release/2026/07/06/3322404/0/en/big-digital-energy-announces-partnership-with-10netzero-to-acquire-power-ready-hood-county-texas-site-for-ai-datacenter-development.html)</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -7666,7 +7786,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/)</t>
+          <t>DCD (https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/)</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -7703,7 +7823,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/meta-files-to-expand-campus-in-el-paso-texas-with-12-new-buildings/)</t>
+          <t>DCD (https://www.datacenterdynamics.com/en/news/meta-files-to-expand-campus-in-el-paso-texas-with-12-new-buildings/)</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -7740,7 +7860,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/softbank-eyes-10gw-data-center-at-former-doe-nuclear-enrichment-site-in-ohio/); [Bloomberg](https://www.bloomberg.com/news/articles/2026-07-26/nvidia-in-talks-on-250-billion-backing-for-openai-hub-wsj-says)</t>
+          <t>DCD (https://www.datacenterdynamics.com/en/news/softbank-eyes-10gw-data-center-at-former-doe-nuclear-enrichment-site-in-ohio/); Bloomberg (https://www.bloomberg.com/news/articles/2026-07-26/nvidia-in-talks-on-250-billion-backing-for-openai-hub-wsj-says)</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -7777,7 +7897,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/)</t>
+          <t>DCD (https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/)</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -7814,7 +7934,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>[Williams Companies](https://www.williams.com/2026/07/13/williams-announces-5-34-billion-investment-in-power-innovation-joint-venture-from-blackstone/)</t>
+          <t>Williams Companies (https://www.williams.com/2026/07/13/williams-announces-5-34-billion-investment-in-power-innovation-joint-venture-from-blackstone/)</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -7851,7 +7971,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/cleancore-solutions-zone-announces-closing-of-first-data-center-project-establishing-its-critical-infrastructure-buildout-for-the-ai-economy-302821421.html)</t>
+          <t>PR Newswire (https://www.prnewswire.com/news-releases/cleancore-solutions-zone-announces-closing-of-first-data-center-project-establishing-its-critical-infrastructure-buildout-for-the-ai-economy-302821421.html)</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -7888,7 +8008,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>[Cowboy State Daily](https://cowboystatedaily.com/2026/06/11/partner-pulling-out-doesnt-slow-huge-2-7gw-cheyenne-project-jade-data-center/)</t>
+          <t>Cowboy State Daily (https://cowboystatedaily.com/2026/06/11/partner-pulling-out-doesnt-slow-huge-2-7gw-cheyenne-project-jade-data-center/)</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -7925,7 +8045,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>[HPCwire](https://www.hpcwire.com/off-the-wire/core-scientific-plans-expansion-to-1-5gw-of-gross-power-at-pecos-texas-campus/)</t>
+          <t>HPCwire (https://www.hpcwire.com/off-the-wire/core-scientific-plans-expansion-to-1-5gw-of-gross-power-at-pecos-texas-campus/)</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -7962,7 +8082,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>[Utah News Dispatch](https://utahnewsdispatch.com/2026/05/19/renderings-show-massive-data-center-box-elder-utah-permits-could-take-years/)</t>
+          <t>Utah News Dispatch (https://utahnewsdispatch.com/2026/05/19/renderings-show-massive-data-center-box-elder-utah-permits-could-take-years/)</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -7999,7 +8119,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>[StockTitan](https://www.stocktitan.net/news/FRMI/fermi-america-tells-texas-lawmakers-project-matador-will-push-the-z7wbkjm2tsxy.html)</t>
+          <t>StockTitan (https://www.stocktitan.net/news/FRMI/fermi-america-tells-texas-lawmakers-project-matador-will-push-the-z7wbkjm2tsxy.html)</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -8036,7 +8156,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>[KLTV](https://www.kltv.com/2026/03/20/president-trump-approves-16-billion-natural-gas-generator-be-installed-anderson-county/)</t>
+          <t>KLTV (https://www.kltv.com/2026/03/20/president-trump-approves-16-billion-natural-gas-generator-be-installed-anderson-county/)</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -8073,7 +8193,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>[WV MetroNews](https://wvmetronews.com/2026/07/16/mon-power-president-says-data-centers-will-end-up-paying-for-natural-gas-powered-power-plant/)</t>
+          <t>WV MetroNews (https://wvmetronews.com/2026/07/16/mon-power-president-says-data-centers-will-end-up-paying-for-natural-gas-powered-power-plant/)</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -8110,7 +8230,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>[Utility Dive](https://www.utilitydive.com/news/iep-plans-944-mw-behind-the-meter-gas-plant-in-pennsylvania-to-power-data-c/758830/)</t>
+          <t>Utility Dive (https://www.utilitydive.com/news/iep-plans-944-mw-behind-the-meter-gas-plant-in-pennsylvania-to-power-data-c/758830/)</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -8147,7 +8267,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>[Wharton Post](https://whartonpost.com/2026/06/25/amazon-data-center-boling/)</t>
+          <t>Wharton Post (https://whartonpost.com/2026/06/25/amazon-data-center-boling/)</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -8184,7 +8304,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>[Crusoe](https://www.crusoe.ai/resources/newsroom/crusoe-and-lancium-announce-1-gigawatt-ai-data-center-campus-in-childress-texas)</t>
+          <t>Crusoe (https://www.crusoe.ai/resources/newsroom/crusoe-and-lancium-announce-1-gigawatt-ai-data-center-campus-in-childress-texas)</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -8221,7 +8341,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/)</t>
+          <t>DCD (https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/)</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -8258,7 +8378,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>[PowerMag](https://www.powermag.com/new-200-mw-gas-fired-plant-in-ohio-will-power-meta-data-center/)</t>
+          <t>PowerMag (https://www.powermag.com/new-200-mw-gas-fired-plant-in-ohio-will-power-meta-data-center/)</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -8295,7 +8415,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>[Aterio](https://www.aterio.io/blog/crusoe-launches-usd29b-goodnight-campus-in-claude-mirroring-openai-s-stargate)</t>
+          <t>Aterio (https://www.aterio.io/blog/crusoe-launches-usd29b-goodnight-campus-in-claude-mirroring-openai-s-stargate)</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -8332,7 +8452,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>[AJC](https://www.ajc.com/business/2026/07/officials-order-georgia-data-centers-pop-up-power-plant-to-halt-construction/); [Inside Climate News](https://insideclimatenews.org/news/31072026/georgia-data-center-private-power-plant/)</t>
+          <t>AJC (https://www.ajc.com/business/2026/07/officials-order-georgia-data-centers-pop-up-power-plant-to-halt-construction/); Inside Climate News (https://insideclimatenews.org/news/31072026/georgia-data-center-private-power-plant/)</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -8369,7 +8489,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/stark-power-lands-56gw-data-center-development-portfolio-in-sagebrush-acquisition/)</t>
+          <t>DCD (https://www.datacenterdynamics.com/en/news/stark-power-lands-56gw-data-center-development-portfolio-in-sagebrush-acquisition/)</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -8406,7 +8526,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55281341/pennsylvanias-homer-city-energy-campus-a-brownfield-transformed-for-data-center-innovation); [Indiana Gazette](https://www.indianagazette.com/local_news/amazon-hcr-are-conducting-commercial-discussions-on-data-center/article_733afa63-9d58-42d0-b16e-6dc61b71689b.html)</t>
+          <t>Data Center Frontier (https://www.datacenterfrontier.com/site-selection/article/55281341/pennsylvanias-homer-city-energy-campus-a-brownfield-transformed-for-data-center-innovation); Indiana Gazette (https://www.indianagazette.com/local_news/amazon-hcr-are-conducting-commercial-discussions-on-data-center/article_733afa63-9d58-42d0-b16e-6dc61b71689b.html)</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -8443,7 +8563,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>[Data Center Dynamics](https://www.datacenterdynamics.com/en/news/nebius-to-deploy-bloom-energy-fuel-cells-to-power-its-us-data-centers/)</t>
+          <t>Data Center Dynamics (https://www.datacenterdynamics.com/en/news/nebius-to-deploy-bloom-energy-fuel-cells-to-power-its-us-data-centers/)</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -8480,7 +8600,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/terravolt-inks-natural-gas-supply-deal-for-onsite-power-plant-at-planned-data-center-campus-in-idaho/)</t>
+          <t>DCD (https://www.datacenterdynamics.com/en/news/terravolt-inks-natural-gas-supply-deal-for-onsite-power-plant-at-planned-data-center-campus-in-idaho/)</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -8517,7 +8637,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/cyrusone-announces-sixth-data-center-campus-in-san-antonio-texas/)</t>
+          <t>DCD (https://www.datacenterdynamics.com/en/news/cyrusone-announces-sixth-data-center-campus-in-san-antonio-texas/)</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -8554,7 +8674,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>[Data Center Dynamics](https://www.datacenterdynamics.com/en/news/edgeconnex-plans-120mw-gas-plant-to-power-ohio-data-center/); [BeBeez](https://bebeez.eu/2026/04/14/edgeconnex-affiliate-proposes-430mw-natural-gas-plant-to-power-data-center-campus-in-new-albany-ohio/)</t>
+          <t>Data Center Dynamics (https://www.datacenterdynamics.com/en/news/edgeconnex-plans-120mw-gas-plant-to-power-ohio-data-center/); BeBeez (https://bebeez.eu/2026/04/14/edgeconnex-affiliate-proposes-430mw-natural-gas-plant-to-power-data-center-campus-in-new-albany-ohio/)</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -8591,7 +8711,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>[Technology.org](https://www.technology.org/2026/07/15/xai-59-unpermitted-gas-turbines-southaven-colossus-2/); [DCD](https://www.datacenterdynamics.com/en/news/musks-xai-gets-go-ahead-for-41-natural-gas-turbines-in-mississippi-to-power-colossus-data-centers/)</t>
+          <t>Technology.org (https://www.technology.org/2026/07/15/xai-59-unpermitted-gas-turbines-southaven-colossus-2/); DCD (https://www.datacenterdynamics.com/en/news/musks-xai-gets-go-ahead-for-41-natural-gas-turbines-in-mississippi-to-power-colossus-data-centers/)</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -8628,7 +8748,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>[Data Center Dynamics](https://www.datacenterdynamics.com/en/news/cleco-to-construct-756mw-natural-gas-plant-to-serve-applied-digitals-data-center-in-rapides-parish-louisiana-report/)</t>
+          <t>Data Center Dynamics (https://www.datacenterdynamics.com/en/news/cleco-to-construct-756mw-natural-gas-plant-to-serve-applied-digitals-data-center-in-rapides-parish-louisiana-report/)</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -8665,7 +8785,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>[Kentucky Lantern](https://kentuckylantern.com/2026/07/22/developer-proposes-hyperscale-data-center-at-the-site-at-former-eastern-kentucky-steel-mill/)</t>
+          <t>Kentucky Lantern (https://kentuckylantern.com/2026/07/22/developer-proposes-hyperscale-data-center-at-the-site-at-former-eastern-kentucky-steel-mill/)</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -8702,7 +8822,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/qts-to-build-11-data-centers-on-lancium-campus-in-hall-county-texas/)</t>
+          <t>DCD (https://www.datacenterdynamics.com/en/news/qts-to-build-11-data-centers-on-lancium-campus-in-hall-county-texas/)</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -8739,7 +8859,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/600mw-natural-gas-powered-data-center-campus-proposed-in-hubbard-texas/); [Construction Review](https://constructionreviewonline.com/5bn-anthropic-data-center-in-texas-receives-critical-financial-backing-from-google/); [CNBC](https://www.cnbc.com/2026/07/30/nexus-data-centers-in-advanced-talks-to-secure-15b-for-google-backed-anthropic-data-center.html)</t>
+          <t>DCD (https://www.datacenterdynamics.com/en/news/600mw-natural-gas-powered-data-center-campus-proposed-in-hubbard-texas/); Construction Review (https://constructionreviewonline.com/5bn-anthropic-data-center-in-texas-receives-critical-financial-backing-from-google/); CNBC (https://www.cnbc.com/2026/07/30/nexus-data-centers-in-advanced-talks-to-secure-15b-for-google-backed-anthropic-data-center.html)</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -8776,7 +8896,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/gigawatt-scale-data-center-campus-planned-outside-atlanta-georgia/)</t>
+          <t>DCD (https://www.datacenterdynamics.com/en/news/gigawatt-scale-data-center-campus-planned-outside-atlanta-georgia/)</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -8813,7 +8933,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>[Bloomberg](https://www.bloomberg.com/news/articles/2026-07-29/nextera-brookfield-to-build-100-billion-kentucky-data-campus); [Kentucky Lantern](https://kentuckylantern.com/2026/07/29/hyperscale-data-center-natural-gas-fired-project-planned-for-paducahs-former-nuclear-plant/)</t>
+          <t>Bloomberg (https://www.bloomberg.com/news/articles/2026-07-29/nextera-brookfield-to-build-100-billion-kentucky-data-campus); Kentucky Lantern (https://kentuckylantern.com/2026/07/29/hyperscale-data-center-natural-gas-fired-project-planned-for-paducahs-former-nuclear-plant/)</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -8850,7 +8970,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>[Axios](https://www.axios.com/2026/07/22/openai-savannah-georgia-data-center-project); [DCD](https://www.datacenterdynamics.com/en/news/openai-reveals-32gw-data-center-project-in-effingham-county-georgia/)</t>
+          <t>Axios (https://www.axios.com/2026/07/22/openai-savannah-georgia-data-center-project); DCD (https://www.datacenterdynamics.com/en/news/openai-reveals-32gw-data-center-project-in-effingham-county-georgia/)</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -8887,7 +9007,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/developer-proposes-867-acre-project-saltworks-data-center-in-graham-texas/); [Olney Enterprise](https://www.olneyenterprise.com/news/stream-plug-power-deal-moves-young-county-data-center-closer-reality)</t>
+          <t>DCD (https://www.datacenterdynamics.com/en/news/developer-proposes-867-acre-project-saltworks-data-center-in-graham-texas/); Olney Enterprise (https://www.olneyenterprise.com/news/stream-plug-power-deal-moves-young-county-data-center-closer-reality)</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -8924,7 +9044,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>[Illinois Times](https://www.illinoistimes.com/news/data-center-development-linked-to-power-plant-construction/)</t>
+          <t>Illinois Times (https://www.illinoistimes.com/news/data-center-development-linked-to-power-plant-construction/)</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -8961,7 +9081,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>[KSL](https://www.ksl.com/article/51355852/worlds-largest-data-center-campus-could-be-coming-to-central-utah); [Utah GOED](https://business.utah.gov/tax-credits/creekstone-energy-llc-commits-17-billion-to-millard-county-data-center-project/)</t>
+          <t>KSL (https://www.ksl.com/article/51355852/worlds-largest-data-center-campus-could-be-coming-to-central-utah); Utah GOED (https://business.utah.gov/tax-credits/creekstone-energy-llc-commits-17-billion-to-millard-county-data-center-project/)</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -8998,7 +9118,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/amazon-breaks-ground-on-10bn-data-center-complex-in-richmond-county-north-carolina/); [WFAE](https://www.wfae.org/energy-environment/2026-07-31/residents-push-back-against-large-amazon-data-center-project-during-packed-public-meeting)</t>
+          <t>DCD (https://www.datacenterdynamics.com/en/news/amazon-breaks-ground-on-10bn-data-center-complex-in-richmond-county-north-carolina/); WFAE (https://www.wfae.org/energy-environment/2026-07-31/residents-push-back-against-large-amazon-data-center-project-during-packed-public-meeting)</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -9035,7 +9155,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/160-acre-project-baccara-is-recommended-for-approval-in-maricopa-county-arizona/); [DCD](https://www.datacenterdynamics.com/en/news/two-data-center-projects-proposed-near-phoenix-arizona/)</t>
+          <t>DCD (https://www.datacenterdynamics.com/en/news/160-acre-project-baccara-is-recommended-for-approval-in-maricopa-county-arizona/); DCD (https://www.datacenterdynamics.com/en/news/two-data-center-projects-proposed-near-phoenix-arizona/)</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -9072,7 +9192,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/doe-selects-amentum-dc-blox-to-develop-behind-the-meter-ai-data-center-at-savannah-river-site-in-south-carolina/); [Energy.gov](https://www.energy.gov/nnsa/articles/nnsa-selects-amentum-ai-data-center-and-energy-project-savannah-river-site)</t>
+          <t>DCD (https://www.datacenterdynamics.com/en/news/doe-selects-amentum-dc-blox-to-develop-behind-the-meter-ai-data-center-at-savannah-river-site-in-south-carolina/); Energy.gov (https://www.energy.gov/nnsa/articles/nnsa-selects-amentum-ai-data-center-and-energy-project-savannah-river-site)</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -9109,7 +9229,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>[Community Impact](https://communityimpact.com/bastrop-cedar-creek/business/new-22b-cedar-creek-data-center-project-abatements-under-review/)</t>
+          <t>Community Impact (https://communityimpact.com/bastrop-cedar-creek/business/new-22b-cedar-creek-data-center-project-abatements-under-review/)</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -9146,7 +9266,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>[Data Centre Magazine](https://datacentremagazine.com/news/ecp-and-kkr-to-build-4bn-190mw-hyperscale-data-centre); [Connect CRE](https://www.connectcre.com/stories/energy-capital-kkr-joint-forces-on-bosque-county-data-center/)</t>
+          <t>Data Centre Magazine (https://datacentremagazine.com/news/ecp-and-kkr-to-build-4bn-190mw-hyperscale-data-centre); Connect CRE (https://www.connectcre.com/stories/energy-capital-kkr-joint-forces-on-bosque-county-data-center/)</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -9183,7 +9303,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>[WLBT](https://www.wlbt.com/2026/05/29/psc-wont-issue-opinion-hypothetical-electrical-plant-proposed-tech-site/)</t>
+          <t>WLBT (https://www.wlbt.com/2026/05/29/psc-wont-issue-opinion-hypothetical-electrical-plant-proposed-tech-site/)</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -9220,7 +9340,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/avaio-to-develop-6bn-data-center-campus-in-little-rock-arkansas/)</t>
+          <t>DCD (https://www.datacenterdynamics.com/en/news/avaio-to-develop-6bn-data-center-campus-in-little-rock-arkansas/)</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -9257,7 +9377,7 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>[Mississippi Today](https://mississippitoday.org/2026/04/22/ridgeland-data-center-entergy-mississippi-power/)</t>
+          <t>Mississippi Today (https://mississippitoday.org/2026/04/22/ridgeland-data-center-entergy-mississippi-power/)</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -9294,7 +9414,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/red-post-energy-and-wise-innovation-hub-venture-oasis-execute-letter-of-intent-to-advance-power-infrastructure-for-major-data-center-development-in-southwest-virginia-302645511.html)</t>
+          <t>PR Newswire (https://www.prnewswire.com/news-releases/red-post-energy-and-wise-innovation-hub-venture-oasis-execute-letter-of-intent-to-advance-power-infrastructure-for-major-data-center-development-in-southwest-virginia-302645511.html)</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -9331,7 +9451,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>[Virginia Mercury](https://virginiamercury.com/2026/07/20/data-centers-want-to-build-their-own-gas-turbines-would-that-skirt-state-renewable-energy-laws/)</t>
+          <t>Virginia Mercury (https://virginiamercury.com/2026/07/20/data-centers-want-to-build-their-own-gas-turbines-would-that-skirt-state-renewable-energy-laws/)</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -9368,7 +9488,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>[WBOY](https://www.wboy.com/news/tucker/state-board-approves-tucker-county-data-center-air-quality-permit/)</t>
+          <t>WBOY (https://www.wboy.com/news/tucker/state-board-approves-tucker-county-data-center-air-quality-permit/)</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -9405,7 +9525,7 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/nextera-teams-up-with-exxonmobil-to-develop-12gw-natural-gas-plant-to-power-us-data-center-sector/)</t>
+          <t>DCD (https://www.datacenterdynamics.com/en/news/nextera-teams-up-with-exxonmobil-to-develop-12gw-natural-gas-plant-to-power-us-data-center-sector/)</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -9442,7 +9562,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>[Utility Dive](https://www.utilitydive.com/news/nrg-nears-12-gw-hyperscaler-deal-amid-texas-data-center-pause/827212/)</t>
+          <t>Utility Dive (https://www.utilitydive.com/news/nrg-nears-12-gw-hyperscaler-deal-amid-texas-data-center-pause/827212/)</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -9479,7 +9599,7 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/galaxy-expands-data-center-footprint-with-acquisition-of-500-acre-campus-in-mcgregor-texas-302836014.html)</t>
+          <t>PR Newswire (https://www.prnewswire.com/news-releases/galaxy-expands-data-center-footprint-with-acquisition-of-500-acre-campus-in-mcgregor-texas-302836014.html)</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -9516,12 +9636,49 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>[The Nevada Independent](https://thenevadaindependent.com/article/nevada-data-center-rush-drives-request-for-a-novel-type-of-gas-power-plant)</t>
+          <t>The Nevada Independent (https://thenevadaindependent.com/article/nevada-data-center-rush-drives-request-for-a-novel-type-of-gas-power-plant)</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
           <t>2026-08-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Dove Creek Technology Campus</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Condado de Tom Green (cerca de San Angelo), Texas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Beacon Data Centers (vía Westline TX Holdings LLC)</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>No especificado (generación con motores reciprocantes de gas natural)</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Permitting temprano (solicitud de permiso de aire ante TCEQ presentada 10-ago-2026, hasta 2,409 MW dedicados; sitio de ~1,240 acres construibles; construcción proyectada primavera/verano 2027 si avanza)</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>San Angelo Live (https://sanangelolive.com/news/san-angelo/2026-08-10/dove-creek-data-center-has-applied-tceq-permit-heres-what-know); Concho Observer (https://conchoobserver.com/data-center-permits-detail-proposed-air-quality-footprint/)</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Agregar 5 proyectos nuevos y 4 cambios de fase (2026-08-13)
- Petroquímica: Kings Landing II, Apollo Gas Plant, IGP Gulf Coast Methanol Complex
- Mining: Niron Magnetics (imanes), Louisiana Strategic Metals Complex (Ucore)
- Actualizaciones de fase: Topolobampo/Bahía de Ohuira (pausa parcial urea/metanol),
  Salina Cruz (retraso), Plaquemines LNG Fase 2 (permitting acelerado), Alaska LNG
  (fracaso legislativo)

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J3gnJmFjYm1DLjz6SAgytM
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -20,16 +20,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -52,9 +49,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -420,50 +416,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G46"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -497,7 +493,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Fluor newsroom (https://newsroom.fluor.com/news-releases/news-details/2026/Fluor-Awarded-Contract-to-Engineer-and-Design-the-America-First-Refining-Facility-in-Brownsville-Texas/default.aspx); Tech Times (https://www.techtimes.com/articles/323235/20260805/trumps-flagship-texas-refinery-races-permit-deadline-after-326b-grid-loan.htm)</t>
+          <t>[Fluor newsroom](https://newsroom.fluor.com/news-releases/news-details/2026/Fluor-Awarded-Contract-to-Engineer-and-Design-the-America-First-Refining-Facility-in-Brownsville-Texas/default.aspx); [Tech Times](https://www.techtimes.com/articles/323235/20260805/trumps-flagship-texas-refinery-races-permit-deadline-after-326b-grid-loan.htm)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -534,7 +530,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>FuelCellsWorks (https://fuelcellsworks.com/2026/08/06/clean-energy/cf-industries-to-begin-construction-of-3-7bn-louisiana-blue-ammonia-plant); gasworld (https://www.gasworld.com/story/cf-industries-to-begin-construction-of-4bn-louisiana-blue-ammonia-project/2256572.article/)</t>
+          <t>[FuelCellsWorks](https://fuelcellsworks.com/2026/08/06/clean-energy/cf-industries-to-begin-construction-of-3-7bn-louisiana-blue-ammonia-plant); [gasworld](https://www.gasworld.com/story/cf-industries-to-begin-construction-of-4bn-louisiana-blue-ammonia-project/2256572.article/)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -571,7 +567,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>AllStream Insiders (https://allstreaminsiders.com/us-exxonmobil-may-build-cracker-pe-plant-in-texas-with-an-8-6-billion-investment/)</t>
+          <t>[AllStream Insiders](https://allstreaminsiders.com/us-exxonmobil-may-build-cracker-pe-plant-in-texas-with-an-8-6-billion-investment/)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -608,7 +604,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>BIC Magazine (https://www.bicmagazine.com/departments/operations/cpchem-golden-triangle-polymers-facility-startup-phase/)</t>
+          <t>[BIC Magazine](https://www.bicmagazine.com/departments/operations/cpchem-golden-triangle-polymers-facility-startup-phase/)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -645,7 +641,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>East Daley (https://eastdaley.com/media-and-news/the-race-is-on-to-build-permian-processing)</t>
+          <t>[East Daley](https://eastdaley.com/media-and-news/the-race-is-on-to-build-permian-processing)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -682,7 +678,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Techint (https://www.techint.com/en/our-projects/dos-bocas-refinery)</t>
+          <t>[Techint](https://www.techint.com/en/our-projects/dos-bocas-refinery)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -719,7 +715,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>OGJ (https://www.ogj.com/refining-processing/refining/optimization/article/17279334/pemex-to-proceed-with-dos-bocas-refinery-project)</t>
+          <t>[OGJ](https://www.ogj.com/refining-processing/refining/optimization/article/17279334/pemex-to-proceed-with-dos-bocas-refinery-project)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -756,7 +752,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Forbes México (https://forbes.com.mx/pemex-invertira-5300-millones-de-dolares-para-reactivar-la-industria-petroquimica/)</t>
+          <t>[Forbes México](https://forbes.com.mx/pemex-invertira-5300-millones-de-dolares-para-reactivar-la-industria-petroquimica/)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -793,7 +789,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Forbes México (https://forbes.com.mx/pemex-invertira-5300-millones-de-dolares-para-reactivar-la-industria-petroquimica/)</t>
+          <t>[Forbes México](https://forbes.com.mx/pemex-invertira-5300-millones-de-dolares-para-reactivar-la-industria-petroquimica/)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -830,7 +826,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Forbes México (https://forbes.com.mx/asi-es-la-inversion-de-1553-mdd-por-parte-de-pemex-en-una-planta-de-fertilizantes-en-veracruz/)</t>
+          <t>[Forbes México](https://forbes.com.mx/asi-es-la-inversion-de-1553-mdd-por-parte-de-pemex-en-una-planta-de-fertilizantes-en-veracruz/)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -867,7 +863,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Tribuna (https://tribuna.com.mx/mexico/2026/06/05/sheinbaum-anuncia-inversion-de-93-mil-mdp-para-reactivar-la-industria-petroquimica-y-de-fertilizantes-en-veracruz_560837/); Contralínea (https://contralinea.com.mx/interno/semana/presentan-plan-con-inversion-de-93-mil-mdp-para-rescatar-la-petroquimica-nacional/)</t>
+          <t>[Tribuna](https://tribuna.com.mx/mexico/2026/06/05/sheinbaum-anuncia-inversion-de-93-mil-mdp-para-reactivar-la-industria-petroquimica-y-de-fertilizantes-en-veracruz_560837/); [Contralínea](https://contralinea.com.mx/interno/semana/presentan-plan-con-inversion-de-93-mil-mdp-para-rescatar-la-petroquimica-nacional/)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -904,7 +900,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>PV Magazine México (https://www.pv-magazine-mexico.com/2026/04/28/inician-en-sinaloa-la-construccion-de-la-mayor-planta-de-metanol-ultrabajo-en-carbono-a-partir-de-hidrogeno-verde/)</t>
+          <t>[PV Magazine México](https://www.pv-magazine-mexico.com/2026/04/28/inician-en-sinaloa-la-construccion-de-la-mayor-planta-de-metanol-ultrabajo-en-carbono-a-partir-de-hidrogeno-verde/)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -941,7 +937,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>H2 View (https://www.h2-view.com/story/first-ammonia-project-on-track-for-2026-fid-despite-topsoe-deal-collapse/2138792.article/)</t>
+          <t>[H2 View](https://www.h2-view.com/story/first-ammonia-project-on-track-for-2026-fid-despite-topsoe-deal-collapse/2138792.article/)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -953,12 +949,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Planta de Amoniaco Topolobampo (GPO)</t>
+          <t>Planta de Amoniaco Topolobampo (GPO) — Bahía de Ohuira</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Topolobampo, Sinaloa, México</t>
+          <t>Topolobampo, Ahome, Sinaloa, México</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -973,17 +969,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Construcción (avance ~80% confirmado por Secretaría de Economía jul-2026; op. comercial H1 2027)</t>
+          <t>Construcción parcial/PAUSA parcial (unidad de amoniaco ~95% completa según Presidencia, ago-2026; unidades de urea/metanol y terminal marina PAUSADAS en espera de acuerdo ambiental; gobierno de Sinaloa presentó "Plan Integral" de conservación/desarrollo sostenible de la Bahía de Ohuira, 4-ago-2026, para destrabar continuidad del proyecto)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Debate (https://www.debate.com.mx/economia/secretaria-de-economia-complejo-de-amoniaco-en-topolobampo-prioritario-para-el-gobierno-de-mexico-20260713-0092.html)</t>
+          <t>[Ríodoce](https://riodoce.mx/2026/08/10/pausan-urea-y-metanol-pero-avanza-amoniaco-en-industria-en-la-bahia-de-ohuira/); [Gobierno de Sinaloa](https://sinaloa.gob.mx/presentan-plan-integral-para-la-conservacion-ambiental-el-bienestar-comunitario-y-el-desarrollo-sostenible-de-la-bahia-de-ohuira/)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -1015,7 +1011,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>ICIS (https://www.icis.com/explore/resources/news/2025/11/13/11155109/lake-charles-methanol-ii-awards-feed-fid-expected-in-q2-2026/)</t>
+          <t>[ICIS](https://www.icis.com/explore/resources/news/2025/11/13/11155109/lake-charles-methanol-ii-awards-feed-fid-expected-in-q2-2026/)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1047,17 +1043,17 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Construcción (~74% avance)</t>
+          <t>Construcción (~74% avance; Pemex confirmó retraso en el cronograma, finalización ahora prevista para 2S2027)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Diario del Istmo (https://diariodelistmo.com/nacional/este-es-el-avance-que-lleva-la-planta-coquizadora-en-la-refineria-de-salina-cruz/50642321)</t>
+          <t>[Diario del Istmo](https://diariodelistmo.com/nacional/este-es-el-avance-que-lleva-la-planta-coquizadora-en-la-refineria-de-salina-cruz/50642321); [Mexico Business News](https://mexicobusiness.news/oilandgas/news/salina-cruz-refinery-miss-construction-deadline-pemex)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -1089,7 +1085,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Hydrocarbon Engineering (https://www.hydrocarbonengineering.com/petrochemicals/06032026/shintech-announces-us34-billion-at-louisiana-petrochemicals-complex/)</t>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/petrochemicals/06032026/shintech-announces-us34-billion-at-louisiana-petrochemicals-complex/)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1126,7 +1122,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>INEOS (https://www.ineos.com/news/shared-news/ineos-acetyls-and-sandpiper-chemicals-announce-strategic-collaboration-for-the-development-of-a-low-carbon-methanol-project-in-texas-city-texas/)</t>
+          <t>[INEOS](https://www.ineos.com/news/shared-news/ineos-acetyls-and-sandpiper-chemicals-announce-strategic-collaboration-for-the-development-of-a-low-carbon-methanol-project-in-texas-city-texas/)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1163,7 +1159,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Hydrocarbon Engineering (https://www.hydrocarbonengineering.com/petrochemicals/13072026/oxea-confirms-fid-for-major-capacity-expansion/)</t>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/petrochemicals/13072026/oxea-confirms-fid-for-major-capacity-expansion/)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1200,7 +1196,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>OGJ (https://www.ogj.com/refining-processing/gas-processing/news/55320579/targa-advances-permian-gas-pipeline-processing-expansion)</t>
+          <t>[OGJ](https://www.ogj.com/refining-processing/gas-processing/news/55320579/targa-advances-permian-gas-pipeline-processing-expansion)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1237,7 +1233,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Business Wire (https://www.businesswire.com/news/home/20250806663187/en/Enterprise-Agrees-to-Acquire-Occidentals-Gas-Gathering-Affiliate-Enters-Into-Natural-Gas-Processing-Agreement-Announces-New-Midland-Basin-Natural-Gas-Processing-Plant)</t>
+          <t>[Business Wire](https://www.businesswire.com/news/home/20250806663187/en/Enterprise-Agrees-to-Acquire-Occidentals-Gas-Gathering-Affiliate-Enters-Into-Natural-Gas-Processing-Agreement-Announces-New-Midland-Basin-Natural-Gas-Processing-Plant)</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1274,7 +1270,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Natural Gas Intel (https://naturalgasintel.com/news/mplx-scales-up-for-power-hungry-future-with-natural-gas-focused-growth-plan/)</t>
+          <t>[Natural Gas Intel](https://naturalgasintel.com/news/mplx-scales-up-for-power-hungry-future-with-natural-gas-focused-growth-plan/)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1311,7 +1307,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>East Daley (https://eastdaley.com/daley-note/mplx-acquires-northwind-for-2-375b-acquires-more-ngls-for-jv-project)</t>
+          <t>[East Daley](https://eastdaley.com/daley-note/mplx-acquires-northwind-for-2-375b-acquires-more-ngls-for-jv-project)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1348,7 +1344,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Grand Forks Herald (https://www.grandforksherald.com/news/local/northern-plains-nitrogen-proposal-receiving-more-attention-amid-global-fertilizer-pressure)</t>
+          <t>[Grand Forks Herald](https://www.grandforksherald.com/news/local/northern-plains-nitrogen-proposal-receiving-more-attention-amid-global-fertilizer-pressure)</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1385,7 +1381,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Phillips 66 (https://www.phillips66.com/newsroom/iron-mesa-safely-enters-next-phase-of-construction/)</t>
+          <t>[Phillips 66](https://www.phillips66.com/newsroom/iron-mesa-safely-enters-next-phase-of-construction/)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1422,7 +1418,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Targa Resources (https://www.targaresources.com/news-releases/news-release-details/targa-resources-corp-announces-permian-growth-projects-and)</t>
+          <t>[Targa Resources](https://www.targaresources.com/news-releases/news-release-details/targa-resources-corp-announces-permian-growth-projects-and)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1459,7 +1455,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Elefante Blanco (https://elefanteblanco.mx/2026/01/02/pemex-abre-30-licitaciones-para-obras-en-la-refineria-madero/)</t>
+          <t>[Elefante Blanco](https://elefanteblanco.mx/2026/01/02/pemex-abre-30-licitaciones-para-obras-en-la-refineria-madero/)</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1496,7 +1492,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>La Jornada (https://www.jornada.com.mx/noticia/2026/06/08/economia/da-inicio-ejecucion-de-planta-de-fertilizantes-en-durango-por-parte-de-fermachem)</t>
+          <t>[La Jornada](https://www.jornada.com.mx/noticia/2026/06/08/economia/da-inicio-ejecucion-de-planta-de-fertilizantes-en-durango-por-parte-de-fermachem)</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1533,7 +1529,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Downstream Calendar (https://downstreamcalendar.com/mcdermott-secures-feed-contract-for-ascension-clean-energy-project/)</t>
+          <t>[Downstream Calendar](https://downstreamcalendar.com/mcdermott-secures-feed-contract-for-ascension-clean-energy-project/)</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1570,7 +1566,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Business Wire (https://www.businesswire.com/news/home/20260517310811/en/Phillips-66-announces-Zeus-Gas-Plant-and-a-third-Coastal-Bend-Fractionator)</t>
+          <t>[Business Wire](https://www.businesswire.com/news/home/20260517310811/en/Phillips-66-announces-Zeus-Gas-Plant-and-a-third-Coastal-Bend-Fractionator)</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1607,7 +1603,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>USDA (https://www.usda.gov/about-usda/news/press-releases/2026/07/01/secretary-rollins-announces-500-million-fertilizer-investment-and-expansion-program-strengthen)</t>
+          <t>[USDA](https://www.usda.gov/about-usda/news/press-releases/2026/07/01/secretary-rollins-announces-500-million-fertilizer-investment-and-expansion-program-strengthen)</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1644,7 +1640,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Hydrocarbon Engineering (https://www.hydrocarbonengineering.com/clean-fuels/06012026/samsung-ea-announces-groundbreaking-of-low-carbon-ammonia-plant/)</t>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/clean-fuels/06012026/samsung-ea-announces-groundbreaking-of-low-carbon-ammonia-plant/)</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1681,7 +1677,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Hydrocarbon Engineering (https://www.hydrocarbonengineering.com/refining/03062026/green-fuels-hosts-groundbreaking-ceremony-for-new-refinery/)</t>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/refining/03062026/green-fuels-hosts-groundbreaking-ceremony-for-new-refinery/)</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1718,7 +1714,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Energy Transfer (https://www.energytransfer.com/project-highlights/)</t>
+          <t>[Energy Transfer](https://www.energytransfer.com/project-highlights/)</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1755,7 +1751,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Inspectioneering (https://inspectioneering.com/news/2025-08-07/11702/oneok-greenlights-new-365m-delaware-basin-gas-plant); BigGo Finance (https://finance.biggo.com/news/US_OKE_2026-08-04)</t>
+          <t>[Inspectioneering](https://inspectioneering.com/news/2025-08-07/11702/oneok-greenlights-new-365m-delaware-basin-gas-plant); [BigGo Finance](https://finance.biggo.com/news/US_OKE_2026-08-04)</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1792,7 +1788,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Marcellus Drilling News (https://marcellusdrilling.com/2026/08/mplx-marcellus-proc-plants-96-full-harmon-creek-iii-starts-up/); StockTitan (https://www.stocktitan.net/news/MPLX/mplx-lp-reports-second-quarter-2026-financial-9tcvq4saz6sr.html)</t>
+          <t>[Marcellus Drilling News](https://marcellusdrilling.com/2026/08/mplx-marcellus-proc-plants-96-full-harmon-creek-iii-starts-up/); [StockTitan](https://www.stocktitan.net/news/MPLX/mplx-lp-reports-second-quarter-2026-financial-9tcvq4saz6sr.html)</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -1829,7 +1825,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Contralínea (https://contralinea.com.mx/interno/semana/presentan-plan-con-inversion-de-93-mil-mdp-para-rescatar-la-petroquimica-nacional/); El Diario de Juárez (https://diario.mx/nacional/2026/jan/22/adjudica-pemex-contratos-a-favoritas-1102601.html)</t>
+          <t>[Contralínea](https://contralinea.com.mx/interno/semana/presentan-plan-con-inversion-de-93-mil-mdp-para-rescatar-la-petroquimica-nacional/); [El Diario de Juárez](https://diario.mx/nacional/2026/jan/22/adjudica-pemex-contratos-a-favoritas-1102601.html)</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -1866,7 +1862,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Enterprise Reports Second Quarter 2026 Earnings (https://ir.enterpriseproducts.com/news-releases/news-release-details/enterprise-reports-second-quarter-2026-earnings)</t>
+          <t>[Enterprise Reports Second Quarter 2026 Earnings](https://ir.enterpriseproducts.com/news-releases/news-release-details/enterprise-reports-second-quarter-2026-earnings)</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -1903,7 +1899,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Enterprise Reports Second Quarter 2026 Earnings (https://ir.enterpriseproducts.com/news-releases/news-release-details/enterprise-reports-second-quarter-2026-earnings)</t>
+          <t>[Enterprise Reports Second Quarter 2026 Earnings](https://ir.enterpriseproducts.com/news-releases/news-release-details/enterprise-reports-second-quarter-2026-earnings)</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -1940,7 +1936,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>PGJ (https://pgjonline.com/news/2026/may/targa-expands-permian-gas-processing-delaware-express-pipeline-capacity)</t>
+          <t>[PGJ](https://pgjonline.com/news/2026/may/targa-expands-permian-gas-processing-delaware-express-pipeline-capacity)</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -1977,7 +1973,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Hydrocarbon Processing (https://www.hydrocarbonprocessing.com/news/2026/03/southern-energy-renewables-announce-14-b-methanol-and-saf-complex-in-louisiana/); Louisiana Economic Development (https://www.opportunitylouisiana.gov/news/southern-energy-renewables-announce-1-4-billion-methanol-and-sustainable-aviation-fuel-facility-in-st-charles-parish)</t>
+          <t>[Hydrocarbon Processing](https://www.hydrocarbonprocessing.com/news/2026/03/southern-energy-renewables-announce-14-b-methanol-and-saf-complex-in-louisiana/); [Louisiana Economic Development](https://www.opportunitylouisiana.gov/news/southern-energy-renewables-announce-1-4-billion-methanol-and-sustainable-aviation-fuel-facility-in-st-charles-parish)</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2014,7 +2010,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Tri-Cities Area Journal of Business (https://www.tricitiesbusinessnews.com/articles/atlas-agro-plant-nears-decision-point); Washington State Standard (https://washingtonstatestandard.com/2025/10/30/plan-for-1-5b-fertilizer-plant-in-central-wa-still-alive-despite-loss-of-federal-funds/)</t>
+          <t>[Tri-Cities Area Journal of Business](https://www.tricitiesbusinessnews.com/articles/atlas-agro-plant-nears-decision-point); [Washington State Standard](https://washingtonstatestandard.com/2025/10/30/plan-for-1-5b-fertilizer-plant-in-central-wa-still-alive-despite-loss-of-federal-funds/)</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2051,7 +2047,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>The Engineer (https://www.theengineer.co.uk/content/news/abb-joins-team-for-22gw-hydrogen-city-project-in-texas); Energy Capital HTX (https://energycapitalhtx.com/green-hydrogen-city-abb-mou)</t>
+          <t>[The Engineer](https://www.theengineer.co.uk/content/news/abb-joins-team-for-22gw-hydrogen-city-project-in-texas); [Energy Capital HTX](https://energycapitalhtx.com/green-hydrogen-city-abb-mou)</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2088,7 +2084,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Oil &amp; Gas Journal (https://www.ogj.com/refining-processing/gas-processing/capacities/article/55240691/targa-advances-expansion-plans-for-permian-basin-gas-processing)</t>
+          <t>[Oil &amp; Gas Journal](https://www.ogj.com/refining-processing/gas-processing/capacities/article/55240691/targa-advances-expansion-plans-for-permian-basin-gas-processing)</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2125,12 +2121,123 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Inspectioneering (https://inspectioneering.com/news/2026-08-11/12145/brazos-midstream-announces-new-natural-gas-processing-plant-to-support-continued); Rigzone (https://www.rigzone.com/news/brazos_to_grow_midland_gas_processing_capacity_to_11_bcfd-11-aug-2026-184346-article/)</t>
+          <t>[Inspectioneering](https://inspectioneering.com/news/2026-08-11/12145/brazos-midstream-announces-new-natural-gas-processing-plant-to-support-continued); [Rigzone](https://www.rigzone.com/news/brazos_to_grow_midland_gas_processing_capacity_to_11_bcfd-11-aug-2026-184346-article/)</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
           <t>2026-08-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Kings Landing II Gas Processing Plant</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Nuevo México, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Kinetik Holdings</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Construcción (FID alcanzada; US$260 millones; finalización prevista 2S2028)</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>[Investing.com](https://www.investing.com/news/company-news/kinetik-approves-260m-gas-processing-plant-in-new-mexico-93CH-4698224)</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Apollo Gas Plant</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Condado de Eddy, Nuevo México, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Trace Midstream Partners II</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Anuncio/planeación (planta criogénica de 250 MMcf/d)</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>[Gas Compression Magazine](https://gascompressionmagazine.com/2026/06/29/new-mexico-gains-major-gas-processing-hub/)</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>IGP Gulf Coast Methanol Complex (4 unidades)</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Plaquemine Parish (Myrtle Grove), Luisiana, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>IGP Methanol LLC</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Permiso de calidad del aire asegurado / pre-construcción (US$3,600 millones)</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>[Industrial Info Resources](https://www.industrialinfo.com/news/article.jsp?newsitemID=262022)</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -2148,47 +2255,47 @@
   <dimension ref="A1:G43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -2222,7 +2329,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Bechtel (https://www.bechtel.com/press-releases/nextdecade-executes-epc-contract-with-bechtel-for-train-4-at-the-rio-grande-lng-facility/); Natural Gas Intel (https://naturalgasintel.com/news/nextdecade-targets-more-than-36-mty-with-rio-grande-lng-upscale-sixth-train-expansion/); Federal Register (https://www.federalregister.gov/documents/2026/08/03/2026-15695/rio-grande-lng-train-6-llc-notice-of-intent-to-prepare-an-environmental-impact-statement-for-the); LNG Prime (https://lngprime.com/americas/nextdecade-seeks-ferc-ok-for-sixth-rio-grande-lng-train/187820/)</t>
+          <t>[Bechtel](https://www.bechtel.com/press-releases/nextdecade-executes-epc-contract-with-bechtel-for-train-4-at-the-rio-grande-lng-facility/); [Natural Gas Intel](https://naturalgasintel.com/news/nextdecade-targets-more-than-36-mty-with-rio-grande-lng-upscale-sixth-train-expansion/); [Federal Register](https://www.federalregister.gov/documents/2026/08/03/2026-15695/rio-grande-lng-train-6-llc-notice-of-intent-to-prepare-an-environmental-impact-statement-for-the); [LNG Prime](https://lngprime.com/americas/nextdecade-seeks-ferc-ok-for-sixth-rio-grande-lng-train/187820/)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -2259,7 +2366,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Bechtel (https://www.bechtel.com/press-releases/sempra-infrastructure-announces-epc-contract-with-bechtel-for-port-arthur-lng-phase-2/)</t>
+          <t>[Bechtel](https://www.bechtel.com/press-releases/sempra-infrastructure-announces-epc-contract-with-bechtel-for-port-arthur-lng-phase-2/)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -2296,7 +2403,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Woodside (https://www.woodside.com/what-we-do/growth-projects/woodside-louisiana-lng)</t>
+          <t>[Woodside](https://www.woodside.com/what-we-do/growth-projects/woodside-louisiana-lng)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -2333,7 +2440,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>GEM.wiki (https://www.gem.wiki/CP2_LNG_Terminal); LNG Prime (https://lngprime.com/americas/top-5-news-of-the-week-july-20-26/193119/)</t>
+          <t>[GEM.wiki](https://www.gem.wiki/CP2_LNG_Terminal); [LNG Prime](https://lngprime.com/americas/top-5-news-of-the-week-july-20-26/193119/)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -2350,7 +2457,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Plaquemines Parish, Luisiana, EE.UU.</t>
+          <t>Plaquemines Parish (Myrtle Grove/Port Sulphur), Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -2365,17 +2472,17 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Construcción (Venture Global presentó solicitud FERC para expansión adicional de 31 mtpa —24 trenes, ~USD 18,000 millones—; inicio de construcción de la expansión esperado a inicios de 2027, primera producción fin de 2028)</t>
+          <t>Construcción/Permitting acelerado (Venture Global presentó solicitud FERC para expansión adicional de 31 mtpa —24 trenes, ~USD 18,000 millones—; U.S. Army Corps of Engineers otorgó permitting expedito bajo "emergencia energética nacional" —periodo de comentario público reducido de 30 a 10 días, cerrado 2-jul-2026—, ampliaría el sitio de 590 a 1,220 acres; DOE aprobó exportaciones adicionales inmediatas desde Plaquemines; inicio de construcción de la expansión esperado a inicios de 2027, primera producción fin de 2028)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Offshore Energy (https://www.offshore-energy.biz/kbr-zachry-to-work-on-ventures-plaquemines-lng/); Argus Media (https://www.argusmedia.com/en/news-and-insights/latest-market-news/2755512-vg-files-expansion-plan-to-double-plaquemines-lng)</t>
+          <t>[Offshore Energy](https://www.offshore-energy.biz/kbr-zachry-to-work-on-ventures-plaquemines-lng/); [Verite News](https://veritenews.org/2026/08/12/lng-expansion-could-be-fast-tracked); [DOE](https://www.energy.gov/node/4856848)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -2407,7 +2514,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Port Arthur News (https://panews.com/2026/04/24/golden-pass-lng-makes-history-with-first-export-from-sabine-pass-terminal/)</t>
+          <t>[Port Arthur News](https://panews.com/2026/04/24/golden-pass-lng-makes-history-with-first-export-from-sabine-pass-terminal/)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -2444,7 +2551,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>PGJ (https://pgjonline.com/news/2026/july/cheniere-gets-approval-to-introduce-gas-into-final-corpus-christi-lng-train); LNG Prime (https://lngprime.com/americas/chenieres-corpus-christi-expansion-project-85-4-percent-complete/155448/); energiesmedia (https://energiesmedia.com/ferc-approves-cheniere-train-7-energies/)</t>
+          <t>[PGJ](https://pgjonline.com/news/2026/july/cheniere-gets-approval-to-introduce-gas-into-final-corpus-christi-lng-train); [LNG Prime](https://lngprime.com/americas/chenieres-corpus-christi-expansion-project-85-4-percent-complete/155448/); [energiesmedia](https://energiesmedia.com/ferc-approves-cheniere-train-7-energies/)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -2481,7 +2588,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>GlobeNewswire (https://www.globenewswire.com/news-release/2026/06/03/3306350/0/en/delfin-midstream-announces-5-billion-final-investment-decision-for-first-flng-vessel.html); World Oil (https://www.worldoil.com/news/2026/8/10/tdi-brooks-wins-survey-contract-for-delfin-lng-deepwater-port/)</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/06/03/3306350/0/en/delfin-midstream-announces-5-billion-final-investment-decision-for-first-flng-vessel.html); [World Oil](https://www.worldoil.com/news/2026/8/10/tdi-brooks-wins-survey-contract-for-delfin-lng-deepwater-port/)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -2518,7 +2625,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Dossier Político (https://dossierpolitico.com/2026/07/17/activistas-entregan-90-mil-firmas-para-frenar-proyecto-saguaro-energia-en-sonora/); Natural Gas Intel (https://naturalgasintel.com/news/oneok-affiliate-seeks-3-year-extension-for-saguaro-connector-pipeline/)</t>
+          <t>[Dossier Político](https://dossierpolitico.com/2026/07/17/activistas-entregan-90-mil-firmas-para-frenar-proyecto-saguaro-energia-en-sonora/); [Natural Gas Intel](https://naturalgasintel.com/news/oneok-affiliate-seeks-3-year-extension-for-saguaro-connector-pipeline/)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -2555,7 +2662,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>GEM Wiki (https://www.gem.wiki/New_Fortress_Altamira_FLNG_Terminal)</t>
+          <t>[GEM Wiki](https://www.gem.wiki/New_Fortress_Altamira_FLNG_Terminal)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -2592,7 +2699,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Natural Gas Intel (https://www.naturalgasintel.com/news/glenfarne-lands-investment-for-early-work-on-texas-lng-ahead-of-fid/)</t>
+          <t>[Natural Gas Intel](https://www.naturalgasintel.com/news/glenfarne-lands-investment-for-early-work-on-texas-lng-ahead-of-fid/)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -2629,7 +2736,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>PGJ (https://pgjonline.com/news/2026/july/commonwealth-lng-awards-main-automation-contract-for-louisiana-export-terminal); PR Newswire/Caturus (https://www.prnewswire.com/news-releases/caturus-announces-final-investment-decision-for-9-5-mtpa-commonwealth-lng-export-facility-in-cameron-la-302773264.html)</t>
+          <t>[PGJ](https://pgjonline.com/news/2026/july/commonwealth-lng-awards-main-automation-contract-for-louisiana-export-terminal); [PR Newswire/Caturus](https://www.prnewswire.com/news-releases/caturus-announces-final-investment-decision-for-9-5-mtpa-commonwealth-lng-export-facility-in-cameron-la-302773264.html)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -2666,7 +2773,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Houston Public Media (https://www.houstonpublicmedia.org/articles/galveston-county/2026/07/14/557086/galveston-pelican-island-lng/)</t>
+          <t>[Houston Public Media](https://www.houstonpublicmedia.org/articles/galveston-county/2026/07/14/557086/galveston-pelican-island-lng/)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -2703,7 +2810,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Sempra (https://www.sempra.com/newsroom/press-releases/sempra-infrastructures-eca-lng-phase-1-exports-first-lng-cargo-mexicos); LNG Prime (https://lngprime.com/lng-terminals/sempra-infrastructure-extends-eca-lng-commissioning-due-to-compressor-damage/193584/)</t>
+          <t>[Sempra](https://www.sempra.com/newsroom/press-releases/sempra-infrastructures-eca-lng-phase-1-exports-first-lng-cargo-mexicos); [LNG Prime](https://lngprime.com/lng-terminals/sempra-infrastructure-extends-eca-lng-commissioning-due-to-compressor-damage/193584/)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -2740,7 +2847,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>LNG Prime (https://lngprime.com/americas/gato-negro-eyes-fid-on-mexico-lng-plant-in-late-2026/165906/)</t>
+          <t>[LNG Prime](https://lngprime.com/americas/gato-negro-eyes-fid-on-mexico-lng-plant-in-late-2026/165906/)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -2777,7 +2884,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>PR Newswire (https://www.prnewswire.com/news-releases/amigo-lng-awards-landmark-epc-contract-to-dubai-based-drydocks-world-for-worlds-largest-flng-facility-302537739.html)</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/amigo-lng-awards-landmark-epc-contract-to-dubai-based-drydocks-world-for-worlds-largest-flng-facility-302537739.html)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -2814,7 +2921,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Rigzone (https://www.rigzone.com/news/coastal_bend_lng_enters_permitting_phase-05-aug-2026-184302-article/); PGJ (https://pgjonline.com/news/2026/august/coastal-bend-lng-initiates-formal-permitting-and-consultation-process)</t>
+          <t>[Rigzone](https://www.rigzone.com/news/coastal_bend_lng_enters_permitting_phase-05-aug-2026-184302-article/); [PGJ](https://pgjonline.com/news/2026/august/coastal-bend-lng-initiates-formal-permitting-and-consultation-process)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2851,7 +2958,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>FERC (https://www.ferc.gov/gulfstream-lng-terminal-project)</t>
+          <t>[FERC](https://www.ferc.gov/gulfstream-lng-terminal-project)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2883,17 +2990,17 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Pre-FID (Cámara de Representantes de Alaska rechazó proyecto de ley de incentivos fiscales HB 381, 16-jul-2026; gobernador Dunleavy convocó nueva sesión legislativa especial para el 20-ago-2026 con una ley de incentivos actualizada para reintentar destrabar el financiamiento)</t>
+          <t>Pre-FID/Retraso legislativo (Cámara de Representantes de Alaska rechazó proyecto de ley de incentivos fiscales HB 381, 16-jul-2026; tercera sesión legislativa especial, convocada por el gobernador Dunleavy, concluyó 13-ago-2026 SIN votación del proyecto de ley de incentivos fiscales necesario para avanzar el financiamiento; incierto si el proyecto avanza antes de que asuman nuevo gobernador/legislatura)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Alaska Beacon (https://alaskabeacon.com/2026/07/17/hilcorp-killed-alaska-lng-bill-some-legislators-say-but-governor-calls-the-claim-bullst/); Your Alaska Link (https://www.youralaskalink.com/news/local/dunleavy-plans-updated-lng-bill-calls-lawmakers-back-august-20/article_4ea0fcfa-386b-45c1-815d-8fff56088739.html)</t>
+          <t>[Alaska Beacon](https://alaskabeacon.com/2026/07/17/hilcorp-killed-alaska-lng-bill-some-legislators-say-but-governor-calls-the-claim-bullst/); [Alaska's News Source](https://www.alaskasnewssource.com/2026/08/13/alaska-lng-pipeline-bill-collapses-house-majority-says-it-lacks-votes/)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -2925,7 +3032,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>PGJ (https://pgjonline.com/news/2026/july/311-mile-sonora-gas-pipeline-project-advances-in-mexico)</t>
+          <t>[PGJ](https://pgjonline.com/news/2026/july/311-mile-sonora-gas-pipeline-project-advances-in-mexico)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2962,7 +3069,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>OGJ (https://www.ogj.com/pipelines-transportation/pipelines/news/55322537/arm-energy-takes-fid-on-23-billion-mustang-express-pipeline)</t>
+          <t>[OGJ](https://www.ogj.com/pipelines-transportation/pipelines/news/55322537/arm-energy-takes-fid-on-23-billion-mustang-express-pipeline)</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2999,7 +3106,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Mexico Business News (https://mexicobusiness.news/energy/news/ursus-energy-scales-investment-us21-billion); energynews.mx (https://energynews.mx/nace-praespero-ursus-ei-megaproyecto-de-8000-millones-de-dolares-para-veracruz/)</t>
+          <t>[Mexico Business News](https://mexicobusiness.news/energy/news/ursus-energy-scales-investment-us21-billion); [energynews.mx](https://energynews.mx/nace-praespero-ursus-ei-megaproyecto-de-8000-millones-de-dolares-para-veracruz/)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -3036,7 +3143,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>GlobeNewswire (https://www.globenewswire.com/news-release/2026/07/15/3327983/0/en/Delfin-Midstream-Partners-With-EIG-s-MidOcean-Energy-to-Advance-Second-FLNG-Vessel-Issues-Limited-Notice-to-Proceed-to-Siemens-Energy.html)</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/15/3327983/0/en/Delfin-Midstream-Partners-With-EIG-s-MidOcean-Energy-to-Advance-Second-FLNG-Vessel-Issues-Limited-Notice-to-Proceed-to-Siemens-Energy.html)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -3073,7 +3180,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Natural Gas Intel (https://www.naturalgasintel.com/news/texas-gateway-open-season-expands-haynesville-natural-gas-links-amid-lng-growth/)</t>
+          <t>[Natural Gas Intel](https://www.naturalgasintel.com/news/texas-gateway-open-season-expands-haynesville-natural-gas-links-amid-lng-growth/)</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -3110,7 +3217,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>World Oil (https://worldoil.com/news/2026/7/24/doe-approves-20-year-export-authorization-for-argent-lng-project/); PGJ (https://pgjonline.com/news/2026/august/argent-lng-submits-wsa-to-the-us-coast-guard-advancing-its-25-mmtpy-louisiana-lng-project)</t>
+          <t>[World Oil](https://worldoil.com/news/2026/7/24/doe-approves-20-year-export-authorization-for-argent-lng-project/); [PGJ](https://pgjonline.com/news/2026/august/argent-lng-submits-wsa-to-the-us-coast-guard-advancing-its-25-mmtpy-louisiana-lng-project)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -3147,7 +3254,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Federal Register (https://www.federalregister.gov/documents/2026/07/24/2026-14963/deepwater-port-license-application-st-lng-deepwater-port-development-project-final-environmental)</t>
+          <t>[Federal Register](https://www.federalregister.gov/documents/2026/07/24/2026-14963/deepwater-port-license-application-st-lng-deepwater-port-development-project-final-environmental)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -3184,7 +3291,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Mississippi Today (https://mississippitoday.org/2026/08/05/ferc-new-gas-pipeline-mississippi/)</t>
+          <t>[Mississippi Today](https://mississippitoday.org/2026/08/05/ferc-new-gas-pipeline-mississippi/)</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -3221,7 +3328,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Mississippi Today (https://mississippitoday.org/2026/08/05/ferc-new-gas-pipeline-mississippi/)</t>
+          <t>[Mississippi Today](https://mississippitoday.org/2026/08/05/ferc-new-gas-pipeline-mississippi/)</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -3258,7 +3365,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>LNG Prime (https://lngprime.com/americas/kinder-morgan-seeks-doe-extension-for-gulf-lng-export-project/184334/)</t>
+          <t>[LNG Prime](https://lngprime.com/americas/kinder-morgan-seeks-doe-extension-for-gulf-lng-export-project/184334/)</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -3295,7 +3402,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Baker Hughes (https://investors.bakerhughes.com/news/press-releases/news-details/2026/Baker-Hughes-Secures-Substantial-Equipment-and-Services-Awards-for-Chenieres-Sabine-Pass-LNG-Facility/default.aspx)</t>
+          <t>[Baker Hughes](https://investors.bakerhughes.com/news/press-releases/news-details/2026/Baker-Hughes-Secures-Substantial-Equipment-and-Services-Awards-for-Chenieres-Sabine-Pass-LNG-Facility/default.aspx)</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3332,7 +3439,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Federal Register (https://www.federalregister.gov/documents/2026/05/05/2026-08654/cheniere-corpus-christi-pipeline-lp-corpus-christi-liquefaction-stage-iv-llc-corpus-christi)</t>
+          <t>[Federal Register](https://www.federalregister.gov/documents/2026/05/05/2026-08654/cheniere-corpus-christi-pipeline-lp-corpus-christi-liquefaction-stage-iv-llc-corpus-christi)</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -3369,7 +3476,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Natural Gas Intel (https://www.naturalgasintel.com/news/ferc-approves-extension-for-freeport-lngs-fourth-train-expansion-project/); Federal Register (https://www.federalregister.gov/documents/2026/07/24/2026-15040/freeport-lng-development-lp-flng-liquefaction-llc-flng-liquefaction-2-llc-flng-liquefaction-3-llc)</t>
+          <t>[Natural Gas Intel](https://www.naturalgasintel.com/news/ferc-approves-extension-for-freeport-lngs-fourth-train-expansion-project/); [Federal Register](https://www.federalregister.gov/documents/2026/07/24/2026-15040/freeport-lng-development-lp-flng-liquefaction-llc-flng-liquefaction-2-llc-flng-liquefaction-3-llc)</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -3406,7 +3513,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Proyectos México (https://www.proyectosmexico.gob.mx/proyecto_inversion/1076-gasoducto-coatzacoalcos-ii/)</t>
+          <t>[Proyectos México](https://www.proyectosmexico.gob.mx/proyecto_inversion/1076-gasoducto-coatzacoalcos-ii/)</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -3443,7 +3550,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>LNG Industry (https://www.lngindustry.com/liquefaction/24072026/stabilis-solutions-receives-lor-from-us-coast-guard/)</t>
+          <t>[LNG Industry](https://www.lngindustry.com/liquefaction/24072026/stabilis-solutions-receives-lor-from-us-coast-guard/)</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3480,7 +3587,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Federal Register (https://www.federalregister.gov/documents/2026/06/12/2026-11881/venture-global-cp2-lng-llc-venture-global-cp-express-llc-notice-of-application-and-establishing)</t>
+          <t>[Federal Register](https://www.federalregister.gov/documents/2026/06/12/2026-11881/venture-global-cp2-lng-llc-venture-global-cp-express-llc-notice-of-application-and-establishing)</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -3517,7 +3624,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>LNG Prime (https://lngprime.com/americas/cameron-lng-seeks-ferc-extension-for-expansion-project/167382/)</t>
+          <t>[LNG Prime](https://lngprime.com/americas/cameron-lng-seeks-ferc-extension-for-expansion-project/167382/)</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -3554,7 +3661,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Federal Register (https://www.federalregister.gov/documents/2026/02/23/2026-03548/magnolia-lng-llc-notice-of-request-for-extension-of-time)</t>
+          <t>[Federal Register](https://www.federalregister.gov/documents/2026/02/23/2026-03548/magnolia-lng-llc-notice-of-request-for-extension-of-time)</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -3591,7 +3698,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Storage Terminals Magazine (https://storageterminalsmag.com/kinder-morgans-trident-pipeline-project-enters-active-construction-phase-in-southeast-texas/); Natural Gas Intel (https://www.naturalgasintel.com/news/kinder-morgan-greenlights-7b-in-natural-gas-pipeline-projects-amid-regulatory-speedup/)</t>
+          <t>[Storage Terminals Magazine](https://storageterminalsmag.com/kinder-morgans-trident-pipeline-project-enters-active-construction-phase-in-southeast-texas/); [Natural Gas Intel](https://www.naturalgasintel.com/news/kinder-morgan-greenlights-7b-in-natural-gas-pipeline-projects-amid-regulatory-speedup/)</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -3628,7 +3735,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Global Energy Monitor (https://www.gem.wiki/Centauro_del_Norte_Gas_Pipeline); BNamericas (https://www.bnamericas.com/en/news/mexico-grants-permits-for-three-sonora-gas-projects)</t>
+          <t>[Global Energy Monitor](https://www.gem.wiki/Centauro_del_Norte_Gas_Pipeline); [BNamericas](https://www.bnamericas.com/en/news/mexico-grants-permits-for-three-sonora-gas-projects)</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -3665,7 +3772,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>LNG Industry (https://www.lngindustry.com/liquid-natural-gas/07082026/enbridge-signs-option-to-acquire-ttc-connector/)</t>
+          <t>[LNG Industry](https://www.lngindustry.com/liquid-natural-gas/07082026/enbridge-signs-option-to-acquire-ttc-connector/)</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -3702,7 +3809,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Enbridge (https://www.enbridge.com/stories/2026/august/bay-runner-twin-permian-gas-pipelines-feeder-gulf-coast-lng-exports); PGJ (https://pgjonline.com/news/2026/august/enbridge-partners-announce-pipeline-s-sanctioning-blackcomb-commissioning-as-permian-gas-exports-ramp-up)</t>
+          <t>[Enbridge](https://www.enbridge.com/stories/2026/august/bay-runner-twin-permian-gas-pipelines-feeder-gulf-coast-lng-exports); [PGJ](https://pgjonline.com/news/2026/august/enbridge-partners-announce-pipeline-s-sanctioning-blackcomb-commissioning-as-permian-gas-exports-ramp-up)</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -3739,7 +3846,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>PGJ (https://pgjonline.com/news/2026/august/enbridge-partners-announce-pipeline-s-sanctioning-blackcomb-commissioning-as-permian-gas-exports-ramp-up)</t>
+          <t>[PGJ](https://pgjonline.com/news/2026/august/enbridge-partners-announce-pipeline-s-sanctioning-blackcomb-commissioning-as-permian-gas-exports-ramp-up)</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -3759,50 +3866,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G82"/>
+  <dimension ref="A1:G84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -3836,7 +3943,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Mining Weekly (https://www.miningweekly.com/article/ivanhoe-electric-pencils-in-2026-construction-start-at-arizona-copper-mine-2025-06-25); MINING.COM (https://www.mining.com/web/trump-says-us-is-announcing-a-series-of-mining-projects-worth-3-billion/)</t>
+          <t>[Mining Weekly](https://www.miningweekly.com/article/ivanhoe-electric-pencils-in-2026-construction-start-at-arizona-copper-mine-2025-06-25); [MINING.COM](https://www.mining.com/web/trump-says-us-is-announcing-a-series-of-mining-projects-worth-3-billion/)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -3873,7 +3980,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>SEC/Hudbay (https://www.sec.gov/Archives/edgar/data/1322422/000106299326001973/exhibit99-2.htm); GlobeNewswire (https://www.globenewswire.com/news-release/2026/06/24/3317147/0/en/hudbay-completes-offering-of-us-52-million-of-4-50-municipal-bonds-for-copper-world.html)</t>
+          <t>[SEC/Hudbay](https://www.sec.gov/Archives/edgar/data/1322422/000106299326001973/exhibit99-2.htm); [GlobeNewswire](https://www.globenewswire.com/news-release/2026/06/24/3317147/0/en/hudbay-completes-offering-of-us-52-million-of-4-50-municipal-bonds-for-copper-world.html)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -3910,7 +4017,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>SEC (https://www.sec.gov/Archives/edgar/data/863064/000086306426000019/ex12d16mr_resolutionland.htm); International Mining (https://im-mining.com/2026/08/10/resolution-copper-accelerates-exploration-underground-development-with-major-drilling-redpath-contracts/)</t>
+          <t>[SEC](https://www.sec.gov/Archives/edgar/data/863064/000086306426000019/ex12d16mr_resolutionland.htm); [International Mining](https://im-mining.com/2026/08/10/resolution-copper-accelerates-exploration-underground-development-with-major-drilling-redpath-contracts/)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -3947,7 +4054,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Mining Weekly (https://www.miningweekly.com/article/thacker-pass-lithium-project-us-update-2026-05-22); Lithium Americas (https://lithiumamericas.com/news/news-details/2026/Lithium-Americas-Provides-a-Project-Update-and-2026-Capex-Guidance-for-Thacker-Pass/default.aspx)</t>
+          <t>[Mining Weekly](https://www.miningweekly.com/article/thacker-pass-lithium-project-us-update-2026-05-22); [Lithium Americas](https://lithiumamericas.com/news/news-details/2026/Lithium-Americas-Provides-a-Project-Update-and-2026-Capex-Guidance-for-Thacker-Pass/default.aspx)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -3984,7 +4091,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Mining.com (https://www.mining.com/teck-agnico-team-up-at-san-nicolas-copper-project-in-mexico/)</t>
+          <t>[Mining.com](https://www.mining.com/teck-agnico-team-up-at-san-nicolas-copper-project-in-mexico/)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -4021,7 +4128,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Energy Magazine MX (https://energymagazine.mx/2025/10/grupo-mexico-espera-autorizacion-federal-para-continuar-proyectos-mineros-por-10-mil-200-mdd/)</t>
+          <t>[Energy Magazine MX](https://energymagazine.mx/2025/10/grupo-mexico-espera-autorizacion-federal-para-continuar-proyectos-mineros-por-10-mil-200-mdd/)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -4058,7 +4165,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>BNamericas (https://www.bnamericas.com/en/news/southern-copper-wins-permits-for-us551mn-el-pilar-in-mexico)</t>
+          <t>[BNamericas](https://www.bnamericas.com/en/news/southern-copper-wins-permits-for-us551mn-el-pilar-in-mexico)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -4095,7 +4202,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>M3 Engineering (https://m3eng.com/portfolio/buenavista-del-cobre-concentradora-no-2/)</t>
+          <t>[M3 Engineering](https://m3eng.com/portfolio/buenavista-del-cobre-concentradora-no-2/)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -4132,7 +4239,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Minería en Línea (https://mineriaenlinea.com/2026/04/torex-gold-alcanza-velocidad-de-crucero-en-media-luna-9-meses-adelante-de-cronograma/)</t>
+          <t>[Minería en Línea](https://mineriaenlinea.com/2026/04/torex-gold-alcanza-velocidad-de-crucero-en-media-luna-9-meses-adelante-de-cronograma/)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -4169,7 +4276,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Mining.com (https://www.mining.com/nevada-copper-unveils-restart-and-financing-plan-for-pumpkin-hollow/)</t>
+          <t>[Mining.com](https://www.mining.com/nevada-copper-unveils-restart-and-financing-plan-for-pumpkin-hollow/)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -4206,7 +4313,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>USDA (https://www.usda.gov/about-usda/news/press-releases/2026/07/07/usda-advances-trump-administration-effort-boost-us-mineral-energy-production); Bloomberg (https://www.bloomberg.com/news/articles/2026-07-06/south32-s-arizona-zinc-and-manganese-mine-set-to-get-us-approval)</t>
+          <t>[USDA](https://www.usda.gov/about-usda/news/press-releases/2026/07/07/usda-advances-trump-administration-effort-boost-us-mineral-energy-production); [Bloomberg](https://www.bloomberg.com/news/articles/2026-07-06/south32-s-arizona-zinc-and-manganese-mine-set-to-get-us-approval)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -4243,7 +4350,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>PR Newswire (https://www.prnewswire.com/news-releases/perpetua-resources-advances-construction-of-the-stibnite-gold-project-302787012.html); Departamento de Justicia de EE.UU. (https://www.justice.gov/opa/pr/justice-department-secures-motion-allow-continued-construction-idaho-gold-mine-critical)</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/perpetua-resources-advances-construction-of-the-stibnite-gold-project-302787012.html); [Departamento de Justicia de EE.UU.](https://www.justice.gov/opa/pr/justice-department-secures-motion-allow-continued-construction-idaho-gold-mine-critical)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -4280,7 +4387,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Silver Tiger Metals (https://silvertigermetals.com/news/2026/silver-tiger-metals-awards-engineering-procurement-and-construction-management-contract-and-provides-construction-update)</t>
+          <t>[Silver Tiger Metals](https://silvertigermetals.com/news/2026/silver-tiger-metals-awards-engineering-procurement-and-construction-management-contract-and-provides-construction-update)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -4317,7 +4424,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>PR Newswire (https://www.prnewswire.com/news-releases/vizsla-silver-awards-epcm-and-mine-design-contracts-for-the-development-of-the-panuco-silver-gold-project-302750621.html)</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/vizsla-silver-awards-epcm-and-mine-design-contracts-for-the-development-of-the-panuco-silver-gold-project-302750621.html)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -4354,7 +4461,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Orla Mining (https://orlamining.com/news/orla-announces-results-of-updated-feasibility-study-for-south-railroad-project/)</t>
+          <t>[Orla Mining](https://orlamining.com/news/orla-announces-results-of-updated-feasibility-study-for-south-railroad-project/)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -4391,7 +4498,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Mining Weekly (https://www.miningweekly.com/article/minera-alamos-confirms-low-cost-near-term-mining-possible-at-copperstone-in-arizona-2026-05-28); Minera Alamos (https://mineraalamos.com/news/2026/minera-alamos-announces-positive-pre-feasibility-study-for-the-copperstone-gold-project-in-arizona/)</t>
+          <t>[Mining Weekly](https://www.miningweekly.com/article/minera-alamos-confirms-low-cost-near-term-mining-possible-at-copperstone-in-arizona-2026-05-28); [Minera Alamos](https://mineraalamos.com/news/2026/minera-alamos-announces-positive-pre-feasibility-study-for-the-copperstone-gold-project-in-arizona/)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -4428,7 +4535,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Wyoming News (https://www.wyomingnews.com/rawlinstimes/plans-move-forward-for-ck-gold-project-as-developers-target-2026-construction-start/article_b2bb147e-2f92-4ca2-bf86-fcc9983917a7.html); Discovery Alert (https://discoveryalert.com.au/ck-gold-project-permitting-construction-ready-valuation-2026/)</t>
+          <t>[Wyoming News](https://www.wyomingnews.com/rawlinstimes/plans-move-forward-for-ck-gold-project-as-developers-target-2026-construction-start/article_b2bb147e-2f92-4ca2-bf86-fcc9983917a7.html); [Discovery Alert](https://discoveryalert.com.au/ck-gold-project-permitting-construction-ready-valuation-2026/)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -4465,7 +4572,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>First Majestic (https://www.juniorminingnetwork.com/junior-miner-news/press-releases/1082-tsx/ag/206222-first-majestic-receives-construction-permits-for-santo-nino-and-navidad-advances-development-across-the-santa-elena-district.html)</t>
+          <t>[First Majestic](https://www.juniorminingnetwork.com/junior-miner-news/press-releases/1082-tsx/ag/206222-first-majestic-receives-construction-permits-for-santo-nino-and-navidad-advances-development-across-the-santa-elena-district.html)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -4502,7 +4609,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>SEC/Americas Gold and Silver (https://www.sec.gov/Archives/edgar/data/0001286973/000106299326002645/exhibit99-2.htm)</t>
+          <t>[SEC/Americas Gold and Silver](https://www.sec.gov/Archives/edgar/data/0001286973/000106299326002645/exhibit99-2.htm)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -4539,7 +4646,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Kitco (https://www.kitco.com/news/off-the-wire/2026-06-08/minera-frisco-restarts-two-mexico-mines-plans-new-silver-unit)</t>
+          <t>[Kitco](https://www.kitco.com/news/off-the-wire/2026-06-08/minera-frisco-restarts-two-mexico-mines-plans-new-silver-unit)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -4576,7 +4683,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>PR Newswire (https://www.prnewswire.com/news-releases/trilogy-metals-announces-publication-of-federal-and-state-permitting-schedule-for-arctic-project-establishing-defined-timeline-toward-a-record-of-decision-by-september-2028-302827083.html)</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/trilogy-metals-announces-publication-of-federal-and-state-permitting-schedule-for-arctic-project-establishing-defined-timeline-toward-a-record-of-decision-by-september-2028-302827083.html)</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -4613,7 +4720,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Northern Miner (https://www.northernminer.com/news/gogold-approved-to-build-227m-mine-in-mexico/1003891932/); Newsfile (https://www.newsfilecorp.com/release/300455/GoGold-Achieves-Major-Milestone-Final-Remaining-Permits-Secured-and-Construction-Approved-for-Los-Ricos-South-Underground-Mine)</t>
+          <t>[Northern Miner](https://www.northernminer.com/news/gogold-approved-to-build-227m-mine-in-mexico/1003891932/); [Newsfile](https://www.newsfilecorp.com/release/300455/GoGold-Achieves-Major-Milestone-Final-Remaining-Permits-Secured-and-Construction-Approved-for-Los-Ricos-South-Underground-Mine)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -4650,7 +4757,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>BNamericas (https://www.bnamericas.com/en/news/discovery-advances-permitting-financing-at-us606mn-cordero-in-mexico)</t>
+          <t>[BNamericas](https://www.bnamericas.com/en/news/discovery-advances-permitting-financing-at-us606mn-cordero-in-mexico)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -4687,7 +4794,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Resource World (https://resourceworld.com/tocvan-ventures-eyes-mexican-gold-pour-by-q4-2026/)</t>
+          <t>[Resource World](https://resourceworld.com/tocvan-ventures-eyes-mexican-gold-pour-by-q4-2026/)</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -4724,7 +4831,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Fresnillo plc (https://www.fresnilloplc.com/portfolio/exploration/orisyvo/)</t>
+          <t>[Fresnillo plc](https://www.fresnilloplc.com/portfolio/exploration/orisyvo/)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -4761,7 +4868,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Army.mil (https://www.army.mil/article/293503/army_announces_conditional_lease_awards_for_domestic_critical_mineral_processing_facilities_to_secure_defense_supply_chains)</t>
+          <t>[Army.mil](https://www.army.mil/article/293503/army_announces_conditional_lease_awards_for_domestic_critical_mineral_processing_facilities_to_secure_defense_supply_chains)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -4798,7 +4905,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Mining.com (https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/)</t>
+          <t>[Mining.com](https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/)</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -4835,7 +4942,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Mining.com (https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/)</t>
+          <t>[Mining.com](https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/)</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -4872,7 +4979,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>IM Mining (https://im-mining.com/2026/06/29/metso-to-supply-additional-crushing-package-for-grupo-mexico-la-caridad-copper-concentrator/)</t>
+          <t>[IM Mining](https://im-mining.com/2026/06/29/metso-to-supply-additional-crushing-package-for-grupo-mexico-la-caridad-copper-concentrator/)</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -4909,7 +5016,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>GlobeNewswire (https://www.globenewswire.com/news-release/2026/05/21/3299182)</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/05/21/3299182)</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -4946,7 +5053,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Mexico Business News (https://mexicobusiness.news/mining/news/grupo-mexicos-asarco-may-reopen-united-states)</t>
+          <t>[Mexico Business News](https://mexicobusiness.news/mining/news/grupo-mexicos-asarco-may-reopen-united-states)</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -4983,7 +5090,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Minera Alamos (https://mineraalamos.com/our-assets/cerro-de-oro-project/)</t>
+          <t>[Minera Alamos](https://mineraalamos.com/our-assets/cerro-de-oro-project/)</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -5020,7 +5127,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Global Mining Review (https://www.globalminingreview.com/mining/11022025/antler-copper-project-achieves-critical-federal-permitting-milestone/)</t>
+          <t>[Global Mining Review](https://www.globalminingreview.com/mining/11022025/antler-copper-project-achieves-critical-federal-permitting-milestone/)</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -5057,7 +5164,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>BLM (https://www.blm.gov/press-release/blm-approves-lisbon-valley-copper-mine-expansion-utah)</t>
+          <t>[BLM](https://www.blm.gov/press-release/blm-approves-lisbon-valley-copper-mine-expansion-utah)</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -5094,7 +5201,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>InvestingNews (https://investingnews.com/smackover-lithium-announces-the-award-of-last-key-construction-contract-for-the-south-west-arkansas-project-ahead-of-final-investment-decision/); StockTitan/SEC 6-K (https://www.stocktitan.net/sec-filings/SLI/6-k-standard-lithium-ltd-current-report-foreign-issuer-ef7db860baa3.html)</t>
+          <t>[InvestingNews](https://investingnews.com/smackover-lithium-announces-the-award-of-last-key-construction-contract-for-the-south-west-arkansas-project-ahead-of-final-investment-decision/); [StockTitan/SEC 6-K](https://www.stocktitan.net/sec-filings/SLI/6-k-standard-lithium-ltd-current-report-foreign-issuer-ef7db860baa3.html)</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -5131,7 +5238,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>SEC/Freeport-McMoRan (https://www.sec.gov/Archives/edgar/data/0000831259/000083125926000033/a2q2026exhibit991.htm)</t>
+          <t>[SEC/Freeport-McMoRan](https://www.sec.gov/Archives/edgar/data/0000831259/000083125926000033/a2q2026exhibit991.htm)</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -5168,7 +5275,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>NioCorp (https://niocorp.com/niocorp-launches-construction-of-elk-creek-critical-minerals-project-mine-portal/); Mining.com (https://www.mining.com/updated-feasibility-study-gives-niocorps-elk-creek-critical-minerals-project-a-4b-valuation/)</t>
+          <t>[NioCorp](https://niocorp.com/niocorp-launches-construction-of-elk-creek-critical-minerals-project-mine-portal/); [Mining.com](https://www.mining.com/updated-feasibility-study-gives-niocorps-elk-creek-critical-minerals-project-a-4b-valuation/)</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -5205,7 +5312,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>E&amp;MJ (https://www.e-mj.com/breaking-news/centerra-advances-goldfield-project-in-nevada/)</t>
+          <t>[E&amp;MJ](https://www.e-mj.com/breaking-news/centerra-advances-goldfield-project-in-nevada/)</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -5242,7 +5349,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>GlobeNewswire (https://www.globenewswire.com/news-release/2026/03/02/3247157/0/en/hudbay-to-acquire-arizona-sonoran-creating-the-third-largest-copper-district-in-north-america.html); Arizona Sonoran (https://arizonasonoran.com/news-releases/arizona-sonoran-pre-feasibility-study-delivers-exceptional-results-for-the-cactus-project-outlining-long-life-low-cost-copper-1/)</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/03/02/3247157/0/en/hudbay-to-acquire-arizona-sonoran-creating-the-third-largest-copper-district-in-north-america.html); [Arizona Sonoran](https://arizonasonoran.com/news-releases/arizona-sonoran-pre-feasibility-study-delivers-exceptional-results-for-the-cactus-project-outlining-long-life-low-cost-copper-1/)</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -5279,7 +5386,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Western Exploration (https://www.westernexploration.com/news-and-updates/news/news-details/2026/Western-Exploration-Outlines-2026-Program-to-Advance-Doby-George-Permitting-and-Expand-Gravel-Creek-Resources-2026-aaotfYHcV7/default.aspx); StreetWise Reports (https://www.streetwisereports.com/article/2026/08/03/nevada-gold-project-launches-drill-campaign-at-doby-george.html)</t>
+          <t>[Western Exploration](https://www.westernexploration.com/news-and-updates/news/news-details/2026/Western-Exploration-Outlines-2026-Program-to-Advance-Doby-George-Permitting-and-Expand-Gravel-Creek-Resources-2026-aaotfYHcV7/default.aspx); [StreetWise Reports](https://www.streetwisereports.com/article/2026/08/03/nevada-gold-project-launches-drill-campaign-at-doby-george.html)</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -5316,7 +5423,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Chesapeake Gold Corp. (https://chesapeakegold.com/metates/)</t>
+          <t>[Chesapeake Gold Corp.](https://chesapeakegold.com/metates/)</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -5353,7 +5460,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Mining Technology (https://www.mining-technology.com/news/pathfinder-896m-loi-us-exim-copper-mine/)</t>
+          <t>[Mining Technology](https://www.mining-technology.com/news/pathfinder-896m-loi-us-exim-copper-mine/)</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -5390,7 +5497,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Mexico Business News (https://mexicobusiness.news/mining/news/heliostar-advances-la-colorada-pit-permits-drill-data)</t>
+          <t>[Mexico Business News](https://mexicobusiness.news/mining/news/heliostar-advances-la-colorada-pit-permits-drill-data)</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -5427,7 +5534,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>The Western News (https://thewesternnews.com/news/2026/jul/24/libby-mining-project-takes-another-step-forward-with-federal-ok/)</t>
+          <t>[The Western News](https://thewesternnews.com/news/2026/jul/24/libby-mining-project-takes-another-step-forward-with-federal-ok/)</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -5464,7 +5571,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Mining News North (https://www.miningnewsnorth.com/story/2026/07/24/news/donlin-gold-partners-form-new-novagold/9781.html)</t>
+          <t>[Mining News North](https://www.miningnewsnorth.com/story/2026/07/24/news/donlin-gold-partners-form-new-novagold/9781.html)</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -5501,7 +5608,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>IM Mining (https://im-mining.com/2026/06/23/ioneer-signals-progress-on-rhyolite-ridge-lithium-boron-project-with-kind-and-hyundai-engineering-pacts/)</t>
+          <t>[IM Mining](https://im-mining.com/2026/06/23/ioneer-signals-progress-on-rhyolite-ridge-lithium-boron-project-with-kind-and-hyundai-engineering-pacts/)</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -5538,7 +5645,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Resource World (https://resourceworld.com/axo-metals-secures-major-environmental-permit-approval-clears-path-for-production-at-the-san-antonio-gold-project/)</t>
+          <t>[Resource World](https://resourceworld.com/axo-metals-secures-major-environmental-permit-approval-clears-path-for-production-at-the-san-antonio-gold-project/)</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -5575,7 +5682,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Talon Metals (https://talonmetals.com/talon-metals-and-westmoreland-mining-sign-land-agreement-to-progress-north-dakota-minerals-processing-facility/)</t>
+          <t>[Talon Metals](https://talonmetals.com/talon-metals-and-westmoreland-mining-sign-land-agreement-to-progress-north-dakota-minerals-processing-facility/)</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -5612,7 +5719,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>GlobeNewswire (https://www.globenewswire.com/news-release/2026/07/31/3337077/0/en/bunker-hill-ships-first-concentrate-to-trail-smelter-and-announces-drawdown-of-standby-facility.html)</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/31/3337077/0/en/bunker-hill-ships-first-concentrate-to-trail-smelter-and-announces-drawdown-of-standby-facility.html)</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -5649,7 +5756,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>MPR News (https://www.mprnews.org/story/2026/07/30/newrange-copper-nickel-proposes-major-changes-to-copper-mine-plan)</t>
+          <t>[MPR News](https://www.mprnews.org/story/2026/07/30/newrange-copper-nickel-proposes-major-changes-to-copper-mine-plan)</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -5686,7 +5793,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Energy Fuels (https://investors.energyfuels.com/2026-07-29-Commercial-Scale-Heavy-Rare-Earth-Plant-Now-Under-Construction-in-Utah); PR Newswire (https://www.prnewswire.com/news-releases/commercial-scale-heavy-rare-earth-plant-now-under-construction-in-utah-302837314.html)</t>
+          <t>[Energy Fuels](https://investors.energyfuels.com/2026-07-29-Commercial-Scale-Heavy-Rare-Earth-Plant-Now-Under-Construction-in-Utah); [PR Newswire](https://www.prnewswire.com/news-releases/commercial-scale-heavy-rare-earth-plant-now-under-construction-in-utah-302837314.html)</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -5723,7 +5830,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>GlobeNewswire (https://www.globenewswire.com/news-release/2026/07/29/3334925/0/en/sandfire-resources-america-files-black-butte-copper-project-preliminary-feasibility-study.html)</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/29/3334925/0/en/sandfire-resources-america-files-black-butte-copper-project-preliminary-feasibility-study.html)</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -5760,7 +5867,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Texarkana Gazette (https://www.texarkanagazette.com/news/2026/jun/30/army-awards-lithium-company-energyx-conditional/)</t>
+          <t>[Texarkana Gazette](https://www.texarkanagazette.com/news/2026/jun/30/army-awards-lithium-company-energyx-conditional/)</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -5797,7 +5904,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Mining.com (https://www.mining.com/orla-secures-final-permit-to-advance-underground-mining-at-camino-rojo/); Orla Mining (https://orlamining.com/news/orla-mining-receives-permits-to-extend-operations-in-mexico-supporting-companys-long-term-commitment-to-camino-rojo/)</t>
+          <t>[Mining.com](https://www.mining.com/orla-secures-final-permit-to-advance-underground-mining-at-camino-rojo/); [Orla Mining](https://orlamining.com/news/orla-mining-receives-permits-to-extend-operations-in-mexico-supporting-companys-long-term-commitment-to-camino-rojo/)</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -5834,7 +5941,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Sonoro Gold Corp. (https://sonorogold.com/wp-content/uploads/2026/03/2026.03.01_Sonoro-Gold-Corporate-Presentation.pdf); Mexico Mining Center (https://www.mexicominingcenter.com/sonoro-continues-discussions-with-china-based-epc-companies-and-potential-equity-investors/)</t>
+          <t>[Sonoro Gold Corp.](https://sonorogold.com/wp-content/uploads/2026/03/2026.03.01_Sonoro-Gold-Corporate-Presentation.pdf); [Mexico Mining Center](https://www.mexicominingcenter.com/sonoro-continues-discussions-with-china-based-epc-companies-and-potential-equity-investors/)</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -5871,7 +5978,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Mining Weekly (https://www.miningweekly.com/article/guardian-metals-outlines-viable-tungsten-trioxide-operation-in-nevada-2026-06-30); StockTitan (https://www.stocktitan.net/news/GMTL/guardian-metal-resources-plc-announces-pilot-mountain-pre-tftnlr9fu3if.html)</t>
+          <t>[Mining Weekly](https://www.miningweekly.com/article/guardian-metals-outlines-viable-tungsten-trioxide-operation-in-nevada-2026-06-30); [StockTitan](https://www.stocktitan.net/news/GMTL/guardian-metal-resources-plc-announces-pilot-mountain-pre-tftnlr9fu3if.html)</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -5908,7 +6015,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Newswire (https://www.newswire.ca/news-releases/p2-gold-gabbs-project-update-feasibility-study-on-track-840759204.html)</t>
+          <t>[Newswire](https://www.newswire.ca/news-releases/p2-gold-gabbs-project-update-feasibility-study-on-track-840759204.html)</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -5945,7 +6052,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>PR Newswire (https://www.prnewswire.com/news-releases/buscar-company-announces-major-advancement-in-the-permitting-process-for-the-treasure-canyon-gold-mine-project-in-california-302772744.html)</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/buscar-company-announces-major-advancement-in-the-permitting-process-for-the-treasure-canyon-gold-mine-project-in-california-302772744.html)</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -5982,7 +6089,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>GlobeNewswire (https://www.globenewswire.com/news-release/2026/01/29/3229150/0/en/Paramount-Gold-Receives-Federal-Approval-for-the-Grassy-Mountain-Gold-Project.html); OPB (https://www.opb.org/article/2026/01/29/oregon-gold-mine-grassy-mountain/)</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/01/29/3229150/0/en/Paramount-Gold-Receives-Federal-Approval-for-the-Grassy-Mountain-Gold-Project.html); [OPB](https://www.opb.org/article/2026/01/29/oregon-gold-mine-grassy-mountain/)</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -6019,7 +6126,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>CNBC (https://www.cnbc.com/2026/02/26/mp-materials-selects-texas-for-rare-earth-magnet-manufacturing-site.html)</t>
+          <t>[CNBC](https://www.cnbc.com/2026/02/26/mp-materials-selects-texas-for-rare-earth-magnet-manufacturing-site.html)</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -6056,7 +6163,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>PR Newswire (https://www.prnewswire.com/news-releases/the-united-states-is-investing-in-its-domestic-rare-earth-industry-302838375.html)</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/the-united-states-is-investing-in-its-domestic-rare-earth-industry-302838375.html)</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -6093,7 +6200,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Newsfile Corp (https://www.newsfilecorp.com/release/283399/Americas-Gold-and-Silver-Signs-Joint-Venture-Agreement-with-US-Antimony-to-Construct-Antimony-Processing-Facility-in-Idahos-Silver-Valley-Unlocking-Value-from-Its-Antimony-Production-and-Strengthening-U.S.-Critical-Mineral-Security)</t>
+          <t>[Newsfile Corp](https://www.newsfilecorp.com/release/283399/Americas-Gold-and-Silver-Signs-Joint-Venture-Agreement-with-US-Antimony-to-Construct-Antimony-Processing-Facility-in-Idahos-Silver-Valley-Unlocking-Value-from-Its-Antimony-Production-and-Strengthening-U.S.-Critical-Mineral-Security)</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -6130,7 +6237,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>DOE-LPO (https://www.energy.gov/lpo/articles/lpo-announces-conditional-commitment-michigan-potash-produce-fertilizer-us-farmers); Northern Miner (https://www.northernminer.com/news/us-boosts-potash-projects-in-utah-michigan/1003886533/)</t>
+          <t>[DOE-LPO](https://www.energy.gov/lpo/articles/lpo-announces-conditional-commitment-michigan-potash-produce-fertilizer-us-farmers); [Northern Miner](https://www.northernminer.com/news/us-boosts-potash-projects-in-utah-michigan/1003886533/)</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -6167,7 +6274,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>BLM (https://www.blm.gov/announcement/blm-approves-construction-sevier-playa-potash-mining-project)</t>
+          <t>[BLM](https://www.blm.gov/announcement/blm-approves-construction-sevier-playa-potash-mining-project)</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -6204,7 +6311,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Ur-Energy (https://www.ur-energy.com/news-media/press-releases/detail/401/ur-energy-commences-operations-at-its-shirley-basin-isr)</t>
+          <t>[Ur-Energy](https://www.ur-energy.com/news-media/press-releases/detail/401/ur-energy-commences-operations-at-its-shirley-basin-isr)</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -6241,7 +6348,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Mexico Business News (https://mexicobusiness.news/mining/news/silverco-targets-late-2026-restart-past-producing-cusi-mine); Investing News Network (https://investingnews.com/silverco-mining-begins-underground-development-at-cusi-restart-remains-on-budget-and-on-schedule/)</t>
+          <t>[Mexico Business News](https://mexicobusiness.news/mining/news/silverco-targets-late-2026-restart-past-producing-cusi-mine); [Investing News Network](https://investingnews.com/silverco-mining-begins-underground-development-at-cusi-restart-remains-on-budget-and-on-schedule/)</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -6278,7 +6385,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Junior Mining Network (https://www.juniorminingnetwork.com/junior-miner-news/press-releases/2342-tsx/ti/199070-titan-mining-to-start-shipping-first-graphite-product-and-feasibility-study-underway-for-40-000-tpa-integrated-kilbourne-graphite-project.html)</t>
+          <t>[Junior Mining Network](https://www.juniorminingnetwork.com/junior-miner-news/press-releases/2342-tsx/ti/199070-titan-mining-to-start-shipping-first-graphite-product-and-feasibility-study-underway-for-40-000-tpa-integrated-kilbourne-graphite-project.html)</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -6315,7 +6422,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Permitting Council (https://www.permitting.gov/newsroom/success-stories/project-spotlight-graphite-creek-project)</t>
+          <t>[Permitting Council](https://www.permitting.gov/newsroom/success-stories/project-spotlight-graphite-creek-project)</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -6352,7 +6459,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Pan American Silver (https://panamericansilver.com/news/pan-american-announces-revised-pea-for-the-la-colorada-skarn-project-positions-la-colorada-as-a-future-top-tier-silver-mine/); SEC 6-K (https://www.sec.gov/Archives/edgar/data/771992/000077199226000031/a2026_03x24lacoloradapeaup.htm)</t>
+          <t>[Pan American Silver](https://panamericansilver.com/news/pan-american-announces-revised-pea-for-the-la-colorada-skarn-project-positions-la-colorada-as-a-future-top-tier-silver-mine/); [SEC 6-K](https://www.sec.gov/Archives/edgar/data/771992/000077199226000031/a2026_03x24lacoloradapeaup.htm)</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -6389,7 +6496,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>PR Newswire (https://www.prnewswire.com/news-releases/i-80-gold-provides-update-on-lone-tree-plant-refurbishment-project-remains-on-schedule-and-on-budget-302836341.html)</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/i-80-gold-provides-update-on-lone-tree-plant-refurbishment-project-remains-on-schedule-and-on-budget-302836341.html)</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -6426,7 +6533,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>GlobeNewswire (https://www.globenewswire.com/news-release/2026/07/29/3335652/0/en/Kinross-reports-strong-2026-second-quarter-results.html)</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/29/3335652/0/en/Kinross-reports-strong-2026-second-quarter-results.html)</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -6463,7 +6570,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>GlobeNewswire (https://www.globenewswire.com/news-release/2026/07/29/3335652/0/en/Kinross-reports-strong-2026-second-quarter-results.html)</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/29/3335652/0/en/Kinross-reports-strong-2026-second-quarter-results.html)</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -6500,7 +6607,7 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Federal Register (https://www.federalregister.gov/documents/2026/07/29/2026-15255/black-hills-national-forest-wyoming-bear-lodge-rare-earth-project)</t>
+          <t>[Federal Register](https://www.federalregister.gov/documents/2026/07/29/2026-15255/black-hills-national-forest-wyoming-bear-lodge-rare-earth-project)</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -6537,7 +6644,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Minería en Línea (https://mineriaenlinea.com/2026/07/southern-copper-obtiene-permisos-ambientales-para-el-pilar-produccion-a-partir-de-2029/)</t>
+          <t>[Minería en Línea](https://mineriaenlinea.com/2026/07/southern-copper-obtiene-permisos-ambientales-para-el-pilar-produccion-a-partir-de-2029/)</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -6574,7 +6681,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Minería en Línea (https://mineriaenlinea.com/2026/07/southern-copper-obtiene-permisos-ambientales-para-el-pilar-produccion-a-partir-de-2029/)</t>
+          <t>[Minería en Línea](https://mineriaenlinea.com/2026/07/southern-copper-obtiene-permisos-ambientales-para-el-pilar-produccion-a-partir-de-2029/)</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -6611,7 +6718,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Minería en Línea (https://mineriaenlinea.com/2026/07/southern-copper-obtiene-permisos-ambientales-para-el-pilar-produccion-a-partir-de-2029/)</t>
+          <t>[Minería en Línea](https://mineriaenlinea.com/2026/07/southern-copper-obtiene-permisos-ambientales-para-el-pilar-produccion-a-partir-de-2029/)</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -6648,7 +6755,7 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Yellowhammer News (https://yellowhammernews.com/trump-administration-announces-25-million-exim-loan-for-westwaters-coosa-county-graphite-plant/); EXIM.GOV (https://www.exim.gov/news/trump-administration-announces-58m-major-new-critical-mineral-deals-white-house-roundtable)</t>
+          <t>[Yellowhammer News](https://yellowhammernews.com/trump-administration-announces-25-million-exim-loan-for-westwaters-coosa-county-graphite-plant/); [EXIM.GOV](https://www.exim.gov/news/trump-administration-announces-58m-major-new-critical-mineral-deals-white-house-roundtable)</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -6685,7 +6792,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>EXIM.GOV (https://www.exim.gov/news/trump-administration-announces-58m-major-new-critical-mineral-deals-white-house-roundtable); SME (https://me.smenet.org/trump-administration-to-back-three-mineral-projects-with-58-million-in-financing/)</t>
+          <t>[EXIM.GOV](https://www.exim.gov/news/trump-administration-announces-58m-major-new-critical-mineral-deals-white-house-roundtable); [SME](https://me.smenet.org/trump-administration-to-back-three-mineral-projects-with-58-million-in-financing/)</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -6722,7 +6829,7 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>EXIM.GOV (https://www.exim.gov/news/trump-administration-announces-58m-major-new-critical-mineral-deals-white-house-roundtable)</t>
+          <t>[EXIM.GOV](https://www.exim.gov/news/trump-administration-announces-58m-major-new-critical-mineral-deals-white-house-roundtable)</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -6759,7 +6866,7 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>PR Newswire (https://www.prnewswire.com/news-releases/ramaco-resources-releases-hatch-report-and-shareholder-letter-on-exploratory-brook-mine-critical-minerals-project-302838319.html); Mining.com (https://www.mining.com/ramaco-eyes-ree-stockpile-at-wyoming-mine/)</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/ramaco-resources-releases-hatch-report-and-shareholder-letter-on-exploratory-brook-mine-critical-minerals-project-302838319.html); [Mining.com](https://www.mining.com/ramaco-eyes-ree-stockpile-at-wyoming-mine/)</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -6796,12 +6903,86 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>PR Newswire (https://www.prnewswire.com/news-releases/encore-energy-receives-bureau-of-land-management-authorization-to-begin-construction-at-dewey-burdock-uranium-project-302804230.html); Federal Register (https://www.federalregister.gov/documents/2026/08/07/2026-16132/powertech-usa-inc-dewey-burdock-uranium-in-situ-recovery-project-license-renewal)</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/encore-energy-receives-bureau-of-land-management-authorization-to-begin-construction-at-dewey-burdock-uranium-project-302804230.html); [Federal Register](https://www.federalregister.gov/documents/2026/08/07/2026-16132/powertech-usa-inc-dewey-burdock-uranium-in-situ-recovery-project-license-renewal)</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
           <t>2026-08-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Niron Magnetics — Planta de Imanes Permanentes sin Tierras Raras</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Minnesota, EE.UU. (ubicación exacta no especificada)</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Niron Magnetics</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Financiamiento asegurado (US$150 millones del Departamento de Defensa/Office of Strategic Capital, anunciado 7-8-ago-2026, parte de paquete federal de US$3,000 millones en minerales críticos)</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>[MINING.COM](https://www.mining.com/web/trump-says-us-is-announcing-a-series-of-mining-projects-worth-3-billion/); [CNBC](https://www.cnbc.com/2026/08/08/trump-admin-to-invest-3-billion-in-defense-linked-minerals-projects.html)</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Louisiana Strategic Metals Complex</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Alexandria, Luisiana, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Ucore Rare Metals Inc.</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Construcción (planta de procesamiento de tierras raras medianas/pesadas —terbio/disprosio—)</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>[Ucore Rare Metals](https://ucore.com/ucore-readies-for-louisiana-2026-heavy-rare-earth-element-processing/)</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -6819,47 +7000,47 @@
   <dimension ref="A1:G83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -6893,7 +7074,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>DCD (https://www.datacenterdynamics.com/en/news/vantage-breaks-ground-on-texas-gigawatt-data-center-campus-for-openai/); Construction Owners (https://www.constructionowners.com/news/oracle-and-openai-to-power-new-texas-data-center-off-the-grid)</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/vantage-breaks-ground-on-texas-gigawatt-data-center-campus-for-openai/); [Construction Owners](https://www.constructionowners.com/news/oracle-and-openai-to-power-new-texas-data-center-off-the-grid)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -6930,7 +7111,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Epoch AI (https://epoch.ai/publications/openai-stargate-where-the-us-sites-stand)</t>
+          <t>[Epoch AI](https://epoch.ai/publications/openai-stargate-where-the-us-sites-stand)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -6967,7 +7148,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>DCD (https://www.datacenterdynamics.com/en/news/crusoe-tops-out-final-building-at-openai-stargate-data-center-campus-in-abilene-texas/)</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/crusoe-tops-out-final-building-at-openai-stargate-data-center-campus-in-abilene-texas/)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -7004,7 +7185,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Chevron (https://www.chevron.com/newsroom/2026/q2/chevron-signs-20-year-power-agreement-with-microsoft-for-west-texas-data-center)</t>
+          <t>[Chevron](https://www.chevron.com/newsroom/2026/q2/chevron-signs-20-year-power-agreement-with-microsoft-for-west-texas-data-center)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -7041,7 +7222,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Gobierno de México (https://www.gob.mx/presidencia/prensa/plan-mexico-avanza-se-anuncia-inversion-de-4-mil-800-mdd-de-cloudhq-para-la-construccion-de-6-centros-de-datos-en-queretaro)</t>
+          <t>[Gobierno de México](https://www.gob.mx/presidencia/prensa/plan-mexico-avanza-se-anuncia-inversion-de-4-mil-800-mdd-de-cloudhq-para-la-construccion-de-6-centros-de-datos-en-queretaro)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -7078,7 +7259,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Global Data Center Hub (https://www.globaldatacenterhub.com/p/meta-scales-hyperion-to-5gw-and-over)</t>
+          <t>[Global Data Center Hub](https://www.globaldatacenterhub.com/p/meta-scales-hyperion-to-5gw-and-over)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -7115,7 +7296,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Data Center Frontier (https://www.datacenterfrontier.com/site-selection/article/55305086/nv1-and-the-nevada-hyperscale-boom-vantage-data-centers-bets-3b-on-the-ai-future)</t>
+          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55305086/nv1-and-the-nevada-hyperscale-boom-vantage-data-centers-bets-3b-on-the-ai-future)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -7152,7 +7333,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>DCD (https://www.datacenterdynamics.com/en/news/cloudburst-breaks-ground-on-gigawatt-scale-data-center-campus-in-texas/)</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/cloudburst-breaks-ground-on-gigawatt-scale-data-center-campus-in-texas/)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -7189,7 +7370,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>DCD (https://www.datacenterdynamics.com/en/news/prometheus-hyperscale-details-plans-for-dallas-data-center-campus/)</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/prometheus-hyperscale-details-plans-for-dallas-data-center-campus/)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -7226,7 +7407,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Business Wire (https://www.businesswire.com/news/home/20260126236053/en/Pacifico-Energy-Secures-7.65-GW-Power-Generation-Permit-for-GW-Ranch-Project); Tom's Hardware (https://www.tomshardware.com/tech-industry/data-centers/amazons-new-7-65gw-texas-ai-data-center-power-plant-could-become-the-largest-source-of-co2-pollution-in-the-us-custom-35-turbine-gas-plant-authorized-to-emit-33-million-tons-of-annual-greenhouse-gases)</t>
+          <t>[Business Wire](https://www.businesswire.com/news/home/20260126236053/en/Pacifico-Energy-Secures-7.65-GW-Power-Generation-Permit-for-GW-Ranch-Project); [Tom's Hardware](https://www.tomshardware.com/tech-industry/data-centers/amazons-new-7-65gw-texas-ai-data-center-power-plant-could-become-the-largest-source-of-co2-pollution-in-the-us-custom-35-turbine-gas-plant-authorized-to-emit-33-million-tons-of-annual-greenhouse-gases)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -7263,7 +7444,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>DCD (https://www.datacenterdynamics.com/en/news/amazon-looks-to-build-large-scale-data-center-campus-next-to-nuclear-plant-in-texas/)</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/amazon-looks-to-build-large-scale-data-center-campus-next-to-nuclear-plant-in-texas/)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -7300,7 +7481,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Mexico News Daily (https://mexiconewsdaily.com/business/durango-data-center-fertilizer-plant-investment-fermaca/); DCD (https://www.datacenterdynamics.com/en/news/250mw-natural-gas-powered-data-center-campus-announced-in-durango-mexico/)</t>
+          <t>[Mexico News Daily](https://mexiconewsdaily.com/business/durango-data-center-fertilizer-plant-investment-fermaca/); [DCD](https://www.datacenterdynamics.com/en/news/250mw-natural-gas-powered-data-center-campus-announced-in-durango-mexico/)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -7337,7 +7518,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>DCD (https://www.datacenterdynamics.com/en/news/circe-energy-secures-2gw-of-natural-gas-capacity-for-west-texas-data-center-campus/)</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/circe-energy-secures-2gw-of-natural-gas-capacity-for-west-texas-data-center-campus/)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -7374,7 +7555,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Source NM (https://sourcenm.com/2026/07/16/new-mexico-land-commissioner-blocks-project-jupiter-related-pipeline-from-building-on-state-land/)</t>
+          <t>[Source NM](https://sourcenm.com/2026/07/16/new-mexico-land-commissioner-blocks-project-jupiter-related-pipeline-from-building-on-state-land/)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -7411,7 +7592,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>PR Newswire (https://www.prnewswire.com/news-releases/powerplay-ai-announces-400-mw-behind-the-meter-ai-data-center-development-in-greater-abilene-with-nasdaq-listed-neocloud-joint-venture-partner-302829610.html)</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/powerplay-ai-announces-400-mw-behind-the-meter-ai-data-center-development-in-greater-abilene-with-nasdaq-listed-neocloud-joint-venture-partner-302829610.html)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -7448,7 +7629,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>DCD (https://www.datacenterdynamics.com/en/news/liberty-energy-powerbridge-form-jv-to-power-planned-2gw-data-center-in-west-texas/)</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/liberty-energy-powerbridge-form-jv-to-power-planned-2gw-data-center-in-west-texas/)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -7485,7 +7666,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>PowerMag (https://www.powermag.com/nuclear-natural-gas-power-generation-planned-for-massive-new-mexico-data-center-site/)</t>
+          <t>[PowerMag](https://www.powermag.com/nuclear-natural-gas-power-generation-planned-for-massive-new-mexico-data-center-site/)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -7522,7 +7703,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Data Center Frontier (https://www.datacenterfrontier.com/site-selection/article/55289667/powering-ai-in-the-permian-texas-critical-data-centers-sustainable-energy-play)</t>
+          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55289667/powering-ai-in-the-permian-texas-critical-data-centers-sustainable-energy-play)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -7559,7 +7740,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>OpenAI (https://openai.com/index/five-new-stargate-sites/)</t>
+          <t>[OpenAI](https://openai.com/index/five-new-stargate-sites/)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -7596,7 +7777,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>OpenAI (https://openai.com/index/five-new-stargate-sites/)</t>
+          <t>[OpenAI](https://openai.com/index/five-new-stargate-sites/)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -7633,7 +7814,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Mexico News Daily (https://mexiconewsdaily.com/business/aws-invest-5b-mexico-data-region/)</t>
+          <t>[Mexico News Daily](https://mexiconewsdaily.com/business/aws-invest-5b-mexico-data-region/)</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -7670,7 +7851,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>DCD (https://www.datacenterdynamics.com/en/news/oracle-and-openai-start-construction-on-stargate-data-center-campus-in-saline-township-michigan/)</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/oracle-and-openai-start-construction-on-stargate-data-center-campus-in-saline-township-michigan/)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -7707,7 +7888,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Valley News Live (https://www.valleynewslive.com/2026/07/13/applied-digital-expands-north-dakota-eyes-oliver-county-third-data-center/)</t>
+          <t>[Valley News Live](https://www.valleynewslive.com/2026/07/13/applied-digital-expands-north-dakota-eyes-oliver-county-third-data-center/)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -7744,7 +7925,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Energy Magazine MX (https://energymagazine.mx/2026/01/el-data-center-verde-que-encendio-la-polemica-asi-sera-el-proyecto-de-ia-en-nuevo-leon-que-usara-tecnologia-de-nvidia/)</t>
+          <t>[Energy Magazine MX](https://energymagazine.mx/2026/01/el-data-center-verde-que-encendio-la-polemica-asi-sera-el-proyecto-de-ia-en-nuevo-leon-que-usara-tecnologia-de-nvidia/)</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -7781,7 +7962,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Construction Dive (https://www.constructiondive.com/news/data-center-cleanarc-breaks-ground-virginia-campus/806489/)</t>
+          <t>[Construction Dive](https://www.constructiondive.com/news/data-center-cleanarc-breaks-ground-virginia-campus/806489/)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -7818,7 +7999,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>KSL (https://www.ksl.com/article/51402125/groundbreaking-for-new-millard-county-artificial-intelligence-data-center)</t>
+          <t>[KSL](https://www.ksl.com/article/51402125/groundbreaking-for-new-millard-county-artificial-intelligence-data-center)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -7855,7 +8036,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Governor.mo.gov (https://governor.mo.gov/press-releases/archive/amazon-investing-10-billion-montgomery-county)</t>
+          <t>[Governor.mo.gov](https://governor.mo.gov/press-releases/archive/amazon-investing-10-billion-montgomery-county)</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -7892,7 +8073,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>STLPR (https://www.stlpr.org/government-politics-issues/2026-05-21/missouri-governor-google-announce-15-billion-data-center-montgomery-county)</t>
+          <t>[STLPR](https://www.stlpr.org/government-politics-issues/2026-05-21/missouri-governor-google-announce-15-billion-data-center-montgomery-county)</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -7929,7 +8110,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>GlobeNewswire (https://www.globenewswire.com/news-release/2026/07/06/3322404/0/en/big-digital-energy-announces-partnership-with-10netzero-to-acquire-power-ready-hood-county-texas-site-for-ai-datacenter-development.html)</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/06/3322404/0/en/big-digital-energy-announces-partnership-with-10netzero-to-acquire-power-ready-hood-county-texas-site-for-ai-datacenter-development.html)</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -7966,7 +8147,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>DCD (https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/)</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/)</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -8003,7 +8184,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>DCD (https://www.datacenterdynamics.com/en/news/meta-files-to-expand-campus-in-el-paso-texas-with-12-new-buildings/)</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/meta-files-to-expand-campus-in-el-paso-texas-with-12-new-buildings/)</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -8040,7 +8221,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>DCD (https://www.datacenterdynamics.com/en/news/softbank-eyes-10gw-data-center-at-former-doe-nuclear-enrichment-site-in-ohio/); Bloomberg (https://www.bloomberg.com/news/articles/2026-07-26/nvidia-in-talks-on-250-billion-backing-for-openai-hub-wsj-says)</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/softbank-eyes-10gw-data-center-at-former-doe-nuclear-enrichment-site-in-ohio/); [Bloomberg](https://www.bloomberg.com/news/articles/2026-07-26/nvidia-in-talks-on-250-billion-backing-for-openai-hub-wsj-says)</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -8077,7 +8258,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>DCD (https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/)</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/)</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -8114,7 +8295,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Williams Companies (https://www.williams.com/2026/07/13/williams-announces-5-34-billion-investment-in-power-innovation-joint-venture-from-blackstone/)</t>
+          <t>[Williams Companies](https://www.williams.com/2026/07/13/williams-announces-5-34-billion-investment-in-power-innovation-joint-venture-from-blackstone/)</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -8151,7 +8332,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>PR Newswire (https://www.prnewswire.com/news-releases/cleancore-solutions-zone-announces-closing-of-first-data-center-project-establishing-its-critical-infrastructure-buildout-for-the-ai-economy-302821421.html)</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/cleancore-solutions-zone-announces-closing-of-first-data-center-project-establishing-its-critical-infrastructure-buildout-for-the-ai-economy-302821421.html)</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -8188,7 +8369,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Cowboy State Daily (https://cowboystatedaily.com/2026/06/11/partner-pulling-out-doesnt-slow-huge-2-7gw-cheyenne-project-jade-data-center/)</t>
+          <t>[Cowboy State Daily](https://cowboystatedaily.com/2026/06/11/partner-pulling-out-doesnt-slow-huge-2-7gw-cheyenne-project-jade-data-center/)</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -8225,7 +8406,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>HPCwire (https://www.hpcwire.com/off-the-wire/core-scientific-plans-expansion-to-1-5gw-of-gross-power-at-pecos-texas-campus/)</t>
+          <t>[HPCwire](https://www.hpcwire.com/off-the-wire/core-scientific-plans-expansion-to-1-5gw-of-gross-power-at-pecos-texas-campus/)</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -8262,7 +8443,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Utah News Dispatch (https://utahnewsdispatch.com/2026/05/19/renderings-show-massive-data-center-box-elder-utah-permits-could-take-years/)</t>
+          <t>[Utah News Dispatch](https://utahnewsdispatch.com/2026/05/19/renderings-show-massive-data-center-box-elder-utah-permits-could-take-years/)</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -8299,7 +8480,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>StockTitan (https://www.stocktitan.net/news/FRMI/fermi-america-tells-texas-lawmakers-project-matador-will-push-the-z7wbkjm2tsxy.html)</t>
+          <t>[StockTitan](https://www.stocktitan.net/news/FRMI/fermi-america-tells-texas-lawmakers-project-matador-will-push-the-z7wbkjm2tsxy.html)</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -8336,7 +8517,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>KLTV (https://www.kltv.com/2026/03/20/president-trump-approves-16-billion-natural-gas-generator-be-installed-anderson-county/)</t>
+          <t>[KLTV](https://www.kltv.com/2026/03/20/president-trump-approves-16-billion-natural-gas-generator-be-installed-anderson-county/)</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -8373,7 +8554,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>WV MetroNews (https://wvmetronews.com/2026/07/16/mon-power-president-says-data-centers-will-end-up-paying-for-natural-gas-powered-power-plant/)</t>
+          <t>[WV MetroNews](https://wvmetronews.com/2026/07/16/mon-power-president-says-data-centers-will-end-up-paying-for-natural-gas-powered-power-plant/)</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -8410,7 +8591,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Utility Dive (https://www.utilitydive.com/news/iep-plans-944-mw-behind-the-meter-gas-plant-in-pennsylvania-to-power-data-c/758830/)</t>
+          <t>[Utility Dive](https://www.utilitydive.com/news/iep-plans-944-mw-behind-the-meter-gas-plant-in-pennsylvania-to-power-data-c/758830/)</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -8447,7 +8628,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Wharton Post (https://whartonpost.com/2026/06/25/amazon-data-center-boling/)</t>
+          <t>[Wharton Post](https://whartonpost.com/2026/06/25/amazon-data-center-boling/)</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -8484,7 +8665,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Crusoe (https://www.crusoe.ai/resources/newsroom/crusoe-and-lancium-announce-1-gigawatt-ai-data-center-campus-in-childress-texas)</t>
+          <t>[Crusoe](https://www.crusoe.ai/resources/newsroom/crusoe-and-lancium-announce-1-gigawatt-ai-data-center-campus-in-childress-texas)</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -8521,7 +8702,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>DCD (https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/)</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/blackstone-invests-534bn-in-williams-behind-the-meter-natural-gas-power-projects-for-the-data-center-sector/)</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -8558,7 +8739,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>PowerMag (https://www.powermag.com/new-200-mw-gas-fired-plant-in-ohio-will-power-meta-data-center/)</t>
+          <t>[PowerMag](https://www.powermag.com/new-200-mw-gas-fired-plant-in-ohio-will-power-meta-data-center/)</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -8595,7 +8776,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Aterio (https://www.aterio.io/blog/crusoe-launches-usd29b-goodnight-campus-in-claude-mirroring-openai-s-stargate)</t>
+          <t>[Aterio](https://www.aterio.io/blog/crusoe-launches-usd29b-goodnight-campus-in-claude-mirroring-openai-s-stargate)</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -8632,7 +8813,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>AJC (https://www.ajc.com/business/2026/07/officials-order-georgia-data-centers-pop-up-power-plant-to-halt-construction/); Inside Climate News (https://insideclimatenews.org/news/31072026/georgia-data-center-private-power-plant/)</t>
+          <t>[AJC](https://www.ajc.com/business/2026/07/officials-order-georgia-data-centers-pop-up-power-plant-to-halt-construction/); [Inside Climate News](https://insideclimatenews.org/news/31072026/georgia-data-center-private-power-plant/)</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -8669,7 +8850,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>DCD (https://www.datacenterdynamics.com/en/news/stark-power-lands-56gw-data-center-development-portfolio-in-sagebrush-acquisition/)</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/stark-power-lands-56gw-data-center-development-portfolio-in-sagebrush-acquisition/)</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -8706,7 +8887,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Data Center Frontier (https://www.datacenterfrontier.com/site-selection/article/55281341/pennsylvanias-homer-city-energy-campus-a-brownfield-transformed-for-data-center-innovation); Indiana Gazette (https://www.indianagazette.com/local_news/amazon-hcr-are-conducting-commercial-discussions-on-data-center/article_733afa63-9d58-42d0-b16e-6dc61b71689b.html)</t>
+          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55281341/pennsylvanias-homer-city-energy-campus-a-brownfield-transformed-for-data-center-innovation); [Indiana Gazette](https://www.indianagazette.com/local_news/amazon-hcr-are-conducting-commercial-discussions-on-data-center/article_733afa63-9d58-42d0-b16e-6dc61b71689b.html)</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -8743,7 +8924,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Data Center Dynamics (https://www.datacenterdynamics.com/en/news/nebius-to-deploy-bloom-energy-fuel-cells-to-power-its-us-data-centers/)</t>
+          <t>[Data Center Dynamics](https://www.datacenterdynamics.com/en/news/nebius-to-deploy-bloom-energy-fuel-cells-to-power-its-us-data-centers/)</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -8780,7 +8961,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>DCD (https://www.datacenterdynamics.com/en/news/terravolt-inks-natural-gas-supply-deal-for-onsite-power-plant-at-planned-data-center-campus-in-idaho/)</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/terravolt-inks-natural-gas-supply-deal-for-onsite-power-plant-at-planned-data-center-campus-in-idaho/)</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -8817,7 +8998,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>DCD (https://www.datacenterdynamics.com/en/news/cyrusone-announces-sixth-data-center-campus-in-san-antonio-texas/)</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/cyrusone-announces-sixth-data-center-campus-in-san-antonio-texas/)</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -8854,7 +9035,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Data Center Dynamics (https://www.datacenterdynamics.com/en/news/edgeconnex-plans-120mw-gas-plant-to-power-ohio-data-center/); BeBeez (https://bebeez.eu/2026/04/14/edgeconnex-affiliate-proposes-430mw-natural-gas-plant-to-power-data-center-campus-in-new-albany-ohio/)</t>
+          <t>[Data Center Dynamics](https://www.datacenterdynamics.com/en/news/edgeconnex-plans-120mw-gas-plant-to-power-ohio-data-center/); [BeBeez](https://bebeez.eu/2026/04/14/edgeconnex-affiliate-proposes-430mw-natural-gas-plant-to-power-data-center-campus-in-new-albany-ohio/)</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -8891,7 +9072,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Technology.org (https://www.technology.org/2026/07/15/xai-59-unpermitted-gas-turbines-southaven-colossus-2/); DCD (https://www.datacenterdynamics.com/en/news/musks-xai-gets-go-ahead-for-41-natural-gas-turbines-in-mississippi-to-power-colossus-data-centers/)</t>
+          <t>[Technology.org](https://www.technology.org/2026/07/15/xai-59-unpermitted-gas-turbines-southaven-colossus-2/); [DCD](https://www.datacenterdynamics.com/en/news/musks-xai-gets-go-ahead-for-41-natural-gas-turbines-in-mississippi-to-power-colossus-data-centers/)</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -8928,7 +9109,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Data Center Dynamics (https://www.datacenterdynamics.com/en/news/cleco-to-construct-756mw-natural-gas-plant-to-serve-applied-digitals-data-center-in-rapides-parish-louisiana-report/)</t>
+          <t>[Data Center Dynamics](https://www.datacenterdynamics.com/en/news/cleco-to-construct-756mw-natural-gas-plant-to-serve-applied-digitals-data-center-in-rapides-parish-louisiana-report/)</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -8965,7 +9146,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Kentucky Lantern (https://kentuckylantern.com/2026/07/22/developer-proposes-hyperscale-data-center-at-the-site-at-former-eastern-kentucky-steel-mill/)</t>
+          <t>[Kentucky Lantern](https://kentuckylantern.com/2026/07/22/developer-proposes-hyperscale-data-center-at-the-site-at-former-eastern-kentucky-steel-mill/)</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -9002,7 +9183,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>DCD (https://www.datacenterdynamics.com/en/news/qts-to-build-11-data-centers-on-lancium-campus-in-hall-county-texas/)</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/qts-to-build-11-data-centers-on-lancium-campus-in-hall-county-texas/)</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -9039,7 +9220,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>DCD (https://www.datacenterdynamics.com/en/news/600mw-natural-gas-powered-data-center-campus-proposed-in-hubbard-texas/); Construction Review (https://constructionreviewonline.com/5bn-anthropic-data-center-in-texas-receives-critical-financial-backing-from-google/); CNBC (https://www.cnbc.com/2026/07/30/nexus-data-centers-in-advanced-talks-to-secure-15b-for-google-backed-anthropic-data-center.html)</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/600mw-natural-gas-powered-data-center-campus-proposed-in-hubbard-texas/); [Construction Review](https://constructionreviewonline.com/5bn-anthropic-data-center-in-texas-receives-critical-financial-backing-from-google/); [CNBC](https://www.cnbc.com/2026/07/30/nexus-data-centers-in-advanced-talks-to-secure-15b-for-google-backed-anthropic-data-center.html)</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -9076,7 +9257,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>DCD (https://www.datacenterdynamics.com/en/news/gigawatt-scale-data-center-campus-planned-outside-atlanta-georgia/)</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/gigawatt-scale-data-center-campus-planned-outside-atlanta-georgia/)</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -9113,7 +9294,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Bloomberg (https://www.bloomberg.com/news/articles/2026-07-29/nextera-brookfield-to-build-100-billion-kentucky-data-campus); Kentucky Lantern (https://kentuckylantern.com/2026/07/29/hyperscale-data-center-natural-gas-fired-project-planned-for-paducahs-former-nuclear-plant/)</t>
+          <t>[Bloomberg](https://www.bloomberg.com/news/articles/2026-07-29/nextera-brookfield-to-build-100-billion-kentucky-data-campus); [Kentucky Lantern](https://kentuckylantern.com/2026/07/29/hyperscale-data-center-natural-gas-fired-project-planned-for-paducahs-former-nuclear-plant/)</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -9150,7 +9331,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Axios (https://www.axios.com/2026/07/22/openai-savannah-georgia-data-center-project); DCD (https://www.datacenterdynamics.com/en/news/openai-reveals-32gw-data-center-project-in-effingham-county-georgia/)</t>
+          <t>[Axios](https://www.axios.com/2026/07/22/openai-savannah-georgia-data-center-project); [DCD](https://www.datacenterdynamics.com/en/news/openai-reveals-32gw-data-center-project-in-effingham-county-georgia/)</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -9187,7 +9368,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>DCD (https://www.datacenterdynamics.com/en/news/developer-proposes-867-acre-project-saltworks-data-center-in-graham-texas/); Olney Enterprise (https://www.olneyenterprise.com/news/stream-plug-power-deal-moves-young-county-data-center-closer-reality)</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/developer-proposes-867-acre-project-saltworks-data-center-in-graham-texas/); [Olney Enterprise](https://www.olneyenterprise.com/news/stream-plug-power-deal-moves-young-county-data-center-closer-reality)</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -9224,7 +9405,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Illinois Times (https://www.illinoistimes.com/news/data-center-development-linked-to-power-plant-construction/)</t>
+          <t>[Illinois Times](https://www.illinoistimes.com/news/data-center-development-linked-to-power-plant-construction/)</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -9261,7 +9442,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>KSL (https://www.ksl.com/article/51355852/worlds-largest-data-center-campus-could-be-coming-to-central-utah); Utah GOED (https://business.utah.gov/tax-credits/creekstone-energy-llc-commits-17-billion-to-millard-county-data-center-project/)</t>
+          <t>[KSL](https://www.ksl.com/article/51355852/worlds-largest-data-center-campus-could-be-coming-to-central-utah); [Utah GOED](https://business.utah.gov/tax-credits/creekstone-energy-llc-commits-17-billion-to-millard-county-data-center-project/)</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -9298,7 +9479,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>DCD (https://www.datacenterdynamics.com/en/news/amazon-breaks-ground-on-10bn-data-center-complex-in-richmond-county-north-carolina/); DCD - Clean Air Act (https://www.datacenterdynamics.com/en/news/amazon-duke-energy-accused-of-evading-clean-air-act-at-under-development-data-center-in-hamlet-north-carolina/); NCSU (https://cnr.ncsu.edu/news/2026/08/richmond-county-data-center-air-pollution/)</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/amazon-breaks-ground-on-10bn-data-center-complex-in-richmond-county-north-carolina/); [DCD - Clean Air Act](https://www.datacenterdynamics.com/en/news/amazon-duke-energy-accused-of-evading-clean-air-act-at-under-development-data-center-in-hamlet-north-carolina/); [NCSU](https://cnr.ncsu.edu/news/2026/08/richmond-county-data-center-air-pollution/)</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -9335,7 +9516,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>DCD (https://www.datacenterdynamics.com/en/news/160-acre-project-baccara-is-recommended-for-approval-in-maricopa-county-arizona/); DCD (https://www.datacenterdynamics.com/en/news/two-data-center-projects-proposed-near-phoenix-arizona/)</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/160-acre-project-baccara-is-recommended-for-approval-in-maricopa-county-arizona/); [DCD](https://www.datacenterdynamics.com/en/news/two-data-center-projects-proposed-near-phoenix-arizona/)</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -9372,7 +9553,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>DCD (https://www.datacenterdynamics.com/en/news/doe-selects-amentum-dc-blox-to-develop-behind-the-meter-ai-data-center-at-savannah-river-site-in-south-carolina/); Energy.gov (https://www.energy.gov/nnsa/articles/nnsa-selects-amentum-ai-data-center-and-energy-project-savannah-river-site)</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/doe-selects-amentum-dc-blox-to-develop-behind-the-meter-ai-data-center-at-savannah-river-site-in-south-carolina/); [Energy.gov](https://www.energy.gov/nnsa/articles/nnsa-selects-amentum-ai-data-center-and-energy-project-savannah-river-site)</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -9409,7 +9590,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Community Impact (https://communityimpact.com/bastrop-cedar-creek/business/new-22b-cedar-creek-data-center-project-abatements-under-review/)</t>
+          <t>[Community Impact](https://communityimpact.com/bastrop-cedar-creek/business/new-22b-cedar-creek-data-center-project-abatements-under-review/)</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -9446,7 +9627,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Data Centre Magazine (https://datacentremagazine.com/news/ecp-and-kkr-to-build-4bn-190mw-hyperscale-data-centre); Connect CRE (https://www.connectcre.com/stories/energy-capital-kkr-joint-forces-on-bosque-county-data-center/)</t>
+          <t>[Data Centre Magazine](https://datacentremagazine.com/news/ecp-and-kkr-to-build-4bn-190mw-hyperscale-data-centre); [Connect CRE](https://www.connectcre.com/stories/energy-capital-kkr-joint-forces-on-bosque-county-data-center/)</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -9483,7 +9664,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>WLBT (https://www.wlbt.com/2026/05/29/psc-wont-issue-opinion-hypothetical-electrical-plant-proposed-tech-site/)</t>
+          <t>[WLBT](https://www.wlbt.com/2026/05/29/psc-wont-issue-opinion-hypothetical-electrical-plant-proposed-tech-site/)</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -9520,7 +9701,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>DCD (https://www.datacenterdynamics.com/en/news/avaio-to-develop-6bn-data-center-campus-in-little-rock-arkansas/)</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/avaio-to-develop-6bn-data-center-campus-in-little-rock-arkansas/)</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -9557,7 +9738,7 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Mississippi Today (https://mississippitoday.org/2026/04/22/ridgeland-data-center-entergy-mississippi-power/)</t>
+          <t>[Mississippi Today](https://mississippitoday.org/2026/04/22/ridgeland-data-center-entergy-mississippi-power/)</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -9594,7 +9775,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>PR Newswire (https://www.prnewswire.com/news-releases/red-post-energy-and-wise-innovation-hub-venture-oasis-execute-letter-of-intent-to-advance-power-infrastructure-for-major-data-center-development-in-southwest-virginia-302645511.html)</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/red-post-energy-and-wise-innovation-hub-venture-oasis-execute-letter-of-intent-to-advance-power-infrastructure-for-major-data-center-development-in-southwest-virginia-302645511.html)</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -9631,7 +9812,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Virginia Mercury (https://virginiamercury.com/2026/07/20/data-centers-want-to-build-their-own-gas-turbines-would-that-skirt-state-renewable-energy-laws/)</t>
+          <t>[Virginia Mercury](https://virginiamercury.com/2026/07/20/data-centers-want-to-build-their-own-gas-turbines-would-that-skirt-state-renewable-energy-laws/)</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -9668,7 +9849,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>WBOY (https://www.wboy.com/news/tucker/state-board-approves-tucker-county-data-center-air-quality-permit/)</t>
+          <t>[WBOY](https://www.wboy.com/news/tucker/state-board-approves-tucker-county-data-center-air-quality-permit/)</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -9705,7 +9886,7 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>DCD (https://www.datacenterdynamics.com/en/news/nextera-teams-up-with-exxonmobil-to-develop-12gw-natural-gas-plant-to-power-us-data-center-sector/)</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/nextera-teams-up-with-exxonmobil-to-develop-12gw-natural-gas-plant-to-power-us-data-center-sector/)</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -9742,7 +9923,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Utility Dive (https://www.utilitydive.com/news/nrg-nears-12-gw-hyperscaler-deal-amid-texas-data-center-pause/827212/)</t>
+          <t>[Utility Dive](https://www.utilitydive.com/news/nrg-nears-12-gw-hyperscaler-deal-amid-texas-data-center-pause/827212/)</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -9779,7 +9960,7 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>PR Newswire (https://www.prnewswire.com/news-releases/galaxy-expands-data-center-footprint-with-acquisition-of-500-acre-campus-in-mcgregor-texas-302836014.html)</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/galaxy-expands-data-center-footprint-with-acquisition-of-500-acre-campus-in-mcgregor-texas-302836014.html)</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -9816,7 +9997,7 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>The Nevada Independent (https://thenevadaindependent.com/article/nevada-data-center-rush-drives-request-for-a-novel-type-of-gas-power-plant)</t>
+          <t>[The Nevada Independent](https://thenevadaindependent.com/article/nevada-data-center-rush-drives-request-for-a-novel-type-of-gas-power-plant)</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -9853,7 +10034,7 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>San Angelo Live (https://sanangelolive.com/news/san-angelo/2026-08-10/dove-creek-data-center-has-applied-tceq-permit-heres-what-know); Concho Valley Homepage (https://www.conchovalleyhomepage.com/news/local-news/concho-valley-data-centers/darby-calls-for-clarity-from-beacon-data-centers-requests-public-tceq-meeting/)</t>
+          <t>[San Angelo Live](https://sanangelolive.com/news/san-angelo/2026-08-10/dove-creek-data-center-has-applied-tceq-permit-heres-what-know); [Concho Valley Homepage](https://www.conchovalleyhomepage.com/news/local-news/concho-valley-data-centers/darby-calls-for-clarity-from-beacon-data-centers-requests-public-tceq-meeting/)</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -9890,7 +10071,7 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Utility Dive (https://www.utilitydive.com/news/ppl-blackstone-joint-venture-secures-5-gw-of-gas-turbines-for-data-centers/827408/); DCD (https://www.datacenterdynamics.com/en/news/pennsylvania-utility-ppl-sees-advanced-stage-data-center-pipeline-grow-to-318gw/)</t>
+          <t>[Utility Dive](https://www.utilitydive.com/news/ppl-blackstone-joint-venture-secures-5-gw-of-gas-turbines-for-data-centers/827408/); [DCD](https://www.datacenterdynamics.com/en/news/pennsylvania-utility-ppl-sees-advanced-stage-data-center-pipeline-grow-to-318gw/)</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">

</xml_diff>

<commit_message>
Monitoreo diario 2026-08-14: 1 proyecto nuevo, 6 actualizaciones
- Nuevo: Eastern Montana Fertilizer Project (Cyan H2/KBR, Montana)
- Actualizado: Galveston LNG (Pelican Island), Gran Pilar Gold-Silver,
  Stibnite Gold Project, Bagdad Mine Concentrator Expansion,
  Shirley Basin Uranium Project, Fermi America Project Matador

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YCHAiymatbsHmDfNdxP5ku
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2238,6 +2238,43 @@
       <c r="G49" t="inlineStr">
         <is>
           <t>2026-08-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Eastern Montana Fertilizer Project (planta de urea)</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Culbertson, Montana, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Cyan H2</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>KBR (MoU: tecnología, ingeniería, procura y gestión de construcción)</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Desarrollo/financiamiento (busca cierre de subvención USDA de US$150 millones —vence 17-ago-2026— y préstamo DOE de US$1,000 millones; groundbreaking previsto fin de 2026)</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>[Northern Plains Independent](https://www.northernplainsindependent.com/2026/08/13/proposed-fertilizer-plant-making-strides/); [World Fertilizer](https://www.worldfertilizer.com/project-news/26112025/cyan-h2-signs-mou-for-montana-fertilizer-project/)</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2795,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Power LNG Ventures, LLC</t>
+          <t>Power LNG Ventures, LLC / Énestas (socio estratégico de capital, ago-2026)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -2768,17 +2805,17 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Permitting temprano (arrendamiento preliminar de 30 acres con Galveston Wharves; solicitud federal de exportación presentada; producción prevista dic-2028)</t>
+          <t>Permitting/pre-FID (Power LNG y Énestas firmaron asociación estratégica 12-ago-2026 —Énestas aporta capital, equipos de transporte/almacenamiento de GNL y arranque de distribución por camión mientras avanza la terminal "Harborside"/Project Seawolf—; terminal valuada en ~US$250 millones; arrendamiento preliminar de 30 acres con Galveston Wharves; solicitud federal de exportación presentada; producción prevista dic-2028)</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>[Houston Public Media](https://www.houstonpublicmedia.org/articles/galveston-county/2026/07/14/557086/galveston-pelican-island-lng/)</t>
+          <t>[Houston Public Media](https://www.houstonpublicmedia.org/articles/galveston-county/2026/07/14/557086/galveston-pelican-island-lng/); [LNG Industry](https://www.lngindustry.com/small-scale-lng/13082026/nestas-and-power-lng-establish-strategic-partnership-for-port-of-galveston/)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -4345,17 +4382,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Construcción (corte federal de Idaho negó en jun-2026 moción para detener obras; Export-Import Bank de EE.UU. aprobó en may-2026 préstamo garantizado de USD 2,900 millones, desembolso esperado 2S2026)</t>
+          <t>Construcción (corte federal de Idaho negó en jun-2026 moción para detener obras; Export-Import Bank de EE.UU. aprobó en may-2026 préstamo garantizado de USD 2,900 millones, desembolso esperado 2S2026; nuevos objetivos de exploración de oro/antimonio de alta ley identificados y posible nueva fuente de tungsteno reportados 7-ago-2026)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/perpetua-resources-advances-construction-of-the-stibnite-gold-project-302787012.html); [Departamento de Justicia de EE.UU.](https://www.justice.gov/opa/pr/justice-department-secures-motion-allow-continued-construction-idaho-gold-mine-critical)</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/perpetua-resources-advances-construction-of-the-stibnite-gold-project-302787012.html); [Departamento de Justicia de EE.UU.](https://www.justice.gov/opa/pr/justice-department-secures-motion-allow-continued-construction-idaho-gold-mine-critical); [StreetWise Reports](https://www.streetwisereports.com/article/2026/08/10/idaho-gold-antimony-project-hits-high-grade-intercepts-at-stibnite.html)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -4789,17 +4826,17 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Construcción (piloto; primer doré previsto Q4 2026)</t>
+          <t>Construcción (piloto; primer doré previsto Q4 2026; nuevo hallazgo de mineralización aurífera de alta ley reportado 10/12-ago-2026 —215m, incluyendo intervalo de 16.0 g/t Au—)</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>[Resource World](https://resourceworld.com/tocvan-ventures-eyes-mexican-gold-pour-by-q4-2026/)</t>
+          <t>[Resource World](https://resourceworld.com/tocvan-ventures-eyes-mexican-gold-pour-by-q4-2026/); [Minería en Línea](https://mineriaenlinea.com/2026/08/tocvan-descubre-215-metros-de-mineralizacion-aurifera-de-alta-ley-en-gran-pilar-sonora/)</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -5233,17 +5270,17 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Pre-FID/ingeniería avanzada (estudio para más que duplicar capacidad del concentrador, +200-250 Mlb/año cobre; capex incremental estimado ~US$3,500 millones bajo revisión; US$150M asignados en 2026 para ingeniería y obras tempranas; decisión de inversión esperada 2S-2026)</t>
+          <t>Pre-FID/ingeniería avanzada (estudio para más que duplicar capacidad del concentrador, +200-250 Mlb/año cobre; capex incremental revisado al alza ~30% a ~US$4,500 millones —antes ~US$3,500 millones—, reportado 7/8-ago-2026; US$150M asignados en 2026 para ingeniería y obras tempranas; decisión de inversión esperada 2S-2026)</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>[SEC/Freeport-McMoRan](https://www.sec.gov/Archives/edgar/data/0000831259/000083125926000033/a2q2026exhibit991.htm)</t>
+          <t>[SEC/Freeport-McMoRan](https://www.sec.gov/Archives/edgar/data/0000831259/000083125926000033/a2q2026exhibit991.htm); [ABC15](https://www.abc15.com/news/business/freeport-mcmoran-eyes-4-5b-expansion-of-arizona-mine-as-investment-decision-looms)</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -6306,17 +6343,17 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Construcción/Inicio de operación (planta satélite ISR integrada con Lost Creek; inicio de minado abr-2026; envío de resina cargada a Lost Creek previsto verano 2026)</t>
+          <t>Producción (autorización final del estado de Wyoming para operar a plena producción, reportada 10-ago-2026; planta satélite ISR integrada con Lost Creek; infraestructura de planta y transporte ya en sitio)</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>[Ur-Energy](https://www.ur-energy.com/news-media/press-releases/detail/401/ur-energy-commences-operations-at-its-shirley-basin-isr)</t>
+          <t>[Ur-Energy](https://www.ur-energy.com/news-media/press-releases/detail/401/ur-energy-commences-operations-at-its-shirley-basin-isr); [Junior Mining Network](https://www.juniorminingnetwork.com/junior-miner-news/press-releases/557-tsx/ure/208831-ur-energy-reports-second-quarter-2026-results.html)</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -8470,22 +8507,22 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Primoris Services Corporation (balance of plant, turbinas de gas); Siemens Energy (suministro de turbinas); Energy Transfer (interconexión de gasoducto)</t>
+          <t>Primoris Services Corporation (balance of plant, turbinas de gas); Siemens Energy (suministro de turbinas); Energy Transfer (interconexión de gasoducto); Hillcore Energy Capital (nuevo esquema BOOT "Hillcore Power Center", acuerdo anunciado 11-ago-2026)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Construcción (movimiento de tierra del campus inicial completo; 4.6 millas de gasoducto de 450 MMcf/d instaladas y conectadas al sistema interestatal de Energy Transfer, suficiente para los primeros 2GW; tubería de agua de 20"/7.2 millas completa; turbinas en sitio/tránsito: 3x GE Frame 6B, 3x Siemens SGT6-5000F, 6x Siemens SGT-800; Fermi planea solicitar permiso TCEQ adicional por 5GW más, meta total 17GW)</t>
+          <t>Construcción (movimiento de tierra del campus inicial completo; 4.6 millas de gasoducto de 450 MMcf/d instaladas y conectadas al sistema interestatal de Energy Transfer, suficiente para los primeros 2GW; tubería de agua de 20"/7.2 millas completa; turbinas en sitio/tránsito: 3x GE Frame 6B, 3x Siemens SGT6-5000F, 6x Siemens SGT-800; nuevo acuerdo con Hillcore Energy Capital para "Hillcore Power Center" de ~2.6GW —2.5GW gas natural + 100MW solar/batería—, primer bloque de ~350MW inicia construcción al firmarse acuerdos definitivos, duplicando la generación en sitio a 4.8GW en ~30 meses; Fermi planea solicitar permiso TCEQ adicional por 5GW más, meta total 17GW)</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>[StockTitan](https://www.stocktitan.net/news/FRMI/fermi-america-tells-texas-lawmakers-project-matador-will-push-the-z7wbkjm2tsxy.html)</t>
+          <t>[StockTitan](https://www.stocktitan.net/news/FRMI/fermi-america-tells-texas-lawmakers-project-matador-will-push-the-z7wbkjm2tsxy.html); [DCD](https://www.datacenterdynamics.com/en/news/fermi-taps-hillcore-to-construct-26gw-gas-plant-for-up-to-11gw-project-matador-in-amarillo-texas/)</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitoreo diario 2026-08-14: 1 proyecto nuevo, 6 actualizaciones (#23)
- Nuevo: Eastern Montana Fertilizer Project (Cyan H2/KBR, Montana)
- Actualizado: Galveston LNG (Pelican Island), Gran Pilar Gold-Silver,
  Stibnite Gold Project, Bagdad Mine Concentrator Expansion,
  Shirley Basin Uranium Project, Fermi America Project Matador


Claude-Session: https://claude.ai/code/session_01YCHAiymatbsHmDfNdxP5ku

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2238,6 +2238,43 @@
       <c r="G49" t="inlineStr">
         <is>
           <t>2026-08-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Eastern Montana Fertilizer Project (planta de urea)</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Culbertson, Montana, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Cyan H2</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>KBR (MoU: tecnología, ingeniería, procura y gestión de construcción)</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Desarrollo/financiamiento (busca cierre de subvención USDA de US$150 millones —vence 17-ago-2026— y préstamo DOE de US$1,000 millones; groundbreaking previsto fin de 2026)</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>[Northern Plains Independent](https://www.northernplainsindependent.com/2026/08/13/proposed-fertilizer-plant-making-strides/); [World Fertilizer](https://www.worldfertilizer.com/project-news/26112025/cyan-h2-signs-mou-for-montana-fertilizer-project/)</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2795,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Power LNG Ventures, LLC</t>
+          <t>Power LNG Ventures, LLC / Énestas (socio estratégico de capital, ago-2026)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -2768,17 +2805,17 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Permitting temprano (arrendamiento preliminar de 30 acres con Galveston Wharves; solicitud federal de exportación presentada; producción prevista dic-2028)</t>
+          <t>Permitting/pre-FID (Power LNG y Énestas firmaron asociación estratégica 12-ago-2026 —Énestas aporta capital, equipos de transporte/almacenamiento de GNL y arranque de distribución por camión mientras avanza la terminal "Harborside"/Project Seawolf—; terminal valuada en ~US$250 millones; arrendamiento preliminar de 30 acres con Galveston Wharves; solicitud federal de exportación presentada; producción prevista dic-2028)</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>[Houston Public Media](https://www.houstonpublicmedia.org/articles/galveston-county/2026/07/14/557086/galveston-pelican-island-lng/)</t>
+          <t>[Houston Public Media](https://www.houstonpublicmedia.org/articles/galveston-county/2026/07/14/557086/galveston-pelican-island-lng/); [LNG Industry](https://www.lngindustry.com/small-scale-lng/13082026/nestas-and-power-lng-establish-strategic-partnership-for-port-of-galveston/)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -4345,17 +4382,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Construcción (corte federal de Idaho negó en jun-2026 moción para detener obras; Export-Import Bank de EE.UU. aprobó en may-2026 préstamo garantizado de USD 2,900 millones, desembolso esperado 2S2026)</t>
+          <t>Construcción (corte federal de Idaho negó en jun-2026 moción para detener obras; Export-Import Bank de EE.UU. aprobó en may-2026 préstamo garantizado de USD 2,900 millones, desembolso esperado 2S2026; nuevos objetivos de exploración de oro/antimonio de alta ley identificados y posible nueva fuente de tungsteno reportados 7-ago-2026)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/perpetua-resources-advances-construction-of-the-stibnite-gold-project-302787012.html); [Departamento de Justicia de EE.UU.](https://www.justice.gov/opa/pr/justice-department-secures-motion-allow-continued-construction-idaho-gold-mine-critical)</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/perpetua-resources-advances-construction-of-the-stibnite-gold-project-302787012.html); [Departamento de Justicia de EE.UU.](https://www.justice.gov/opa/pr/justice-department-secures-motion-allow-continued-construction-idaho-gold-mine-critical); [StreetWise Reports](https://www.streetwisereports.com/article/2026/08/10/idaho-gold-antimony-project-hits-high-grade-intercepts-at-stibnite.html)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -4789,17 +4826,17 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Construcción (piloto; primer doré previsto Q4 2026)</t>
+          <t>Construcción (piloto; primer doré previsto Q4 2026; nuevo hallazgo de mineralización aurífera de alta ley reportado 10/12-ago-2026 —215m, incluyendo intervalo de 16.0 g/t Au—)</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>[Resource World](https://resourceworld.com/tocvan-ventures-eyes-mexican-gold-pour-by-q4-2026/)</t>
+          <t>[Resource World](https://resourceworld.com/tocvan-ventures-eyes-mexican-gold-pour-by-q4-2026/); [Minería en Línea](https://mineriaenlinea.com/2026/08/tocvan-descubre-215-metros-de-mineralizacion-aurifera-de-alta-ley-en-gran-pilar-sonora/)</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -5233,17 +5270,17 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Pre-FID/ingeniería avanzada (estudio para más que duplicar capacidad del concentrador, +200-250 Mlb/año cobre; capex incremental estimado ~US$3,500 millones bajo revisión; US$150M asignados en 2026 para ingeniería y obras tempranas; decisión de inversión esperada 2S-2026)</t>
+          <t>Pre-FID/ingeniería avanzada (estudio para más que duplicar capacidad del concentrador, +200-250 Mlb/año cobre; capex incremental revisado al alza ~30% a ~US$4,500 millones —antes ~US$3,500 millones—, reportado 7/8-ago-2026; US$150M asignados en 2026 para ingeniería y obras tempranas; decisión de inversión esperada 2S-2026)</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>[SEC/Freeport-McMoRan](https://www.sec.gov/Archives/edgar/data/0000831259/000083125926000033/a2q2026exhibit991.htm)</t>
+          <t>[SEC/Freeport-McMoRan](https://www.sec.gov/Archives/edgar/data/0000831259/000083125926000033/a2q2026exhibit991.htm); [ABC15](https://www.abc15.com/news/business/freeport-mcmoran-eyes-4-5b-expansion-of-arizona-mine-as-investment-decision-looms)</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -6306,17 +6343,17 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Construcción/Inicio de operación (planta satélite ISR integrada con Lost Creek; inicio de minado abr-2026; envío de resina cargada a Lost Creek previsto verano 2026)</t>
+          <t>Producción (autorización final del estado de Wyoming para operar a plena producción, reportada 10-ago-2026; planta satélite ISR integrada con Lost Creek; infraestructura de planta y transporte ya en sitio)</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>[Ur-Energy](https://www.ur-energy.com/news-media/press-releases/detail/401/ur-energy-commences-operations-at-its-shirley-basin-isr)</t>
+          <t>[Ur-Energy](https://www.ur-energy.com/news-media/press-releases/detail/401/ur-energy-commences-operations-at-its-shirley-basin-isr); [Junior Mining Network](https://www.juniorminingnetwork.com/junior-miner-news/press-releases/557-tsx/ure/208831-ur-energy-reports-second-quarter-2026-results.html)</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -8470,22 +8507,22 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Primoris Services Corporation (balance of plant, turbinas de gas); Siemens Energy (suministro de turbinas); Energy Transfer (interconexión de gasoducto)</t>
+          <t>Primoris Services Corporation (balance of plant, turbinas de gas); Siemens Energy (suministro de turbinas); Energy Transfer (interconexión de gasoducto); Hillcore Energy Capital (nuevo esquema BOOT "Hillcore Power Center", acuerdo anunciado 11-ago-2026)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Construcción (movimiento de tierra del campus inicial completo; 4.6 millas de gasoducto de 450 MMcf/d instaladas y conectadas al sistema interestatal de Energy Transfer, suficiente para los primeros 2GW; tubería de agua de 20"/7.2 millas completa; turbinas en sitio/tránsito: 3x GE Frame 6B, 3x Siemens SGT6-5000F, 6x Siemens SGT-800; Fermi planea solicitar permiso TCEQ adicional por 5GW más, meta total 17GW)</t>
+          <t>Construcción (movimiento de tierra del campus inicial completo; 4.6 millas de gasoducto de 450 MMcf/d instaladas y conectadas al sistema interestatal de Energy Transfer, suficiente para los primeros 2GW; tubería de agua de 20"/7.2 millas completa; turbinas en sitio/tránsito: 3x GE Frame 6B, 3x Siemens SGT6-5000F, 6x Siemens SGT-800; nuevo acuerdo con Hillcore Energy Capital para "Hillcore Power Center" de ~2.6GW —2.5GW gas natural + 100MW solar/batería—, primer bloque de ~350MW inicia construcción al firmarse acuerdos definitivos, duplicando la generación en sitio a 4.8GW en ~30 meses; Fermi planea solicitar permiso TCEQ adicional por 5GW más, meta total 17GW)</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>[StockTitan](https://www.stocktitan.net/news/FRMI/fermi-america-tells-texas-lawmakers-project-matador-will-push-the-z7wbkjm2tsxy.html)</t>
+          <t>[StockTitan](https://www.stocktitan.net/news/FRMI/fermi-america-tells-texas-lawmakers-project-matador-will-push-the-z7wbkjm2tsxy.html); [DCD](https://www.datacenterdynamics.com/en/news/fermi-taps-hillcore-to-construct-26gw-gas-plant-for-up-to-11gw-project-matador-in-amarillo-texas/)</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitoreo 2026-08-17: nuevo data center PA + 4 actualizaciones de fase
- Nuevo: Alpha Compute Corp — Campus de Data Center a Gas Natural (norte de
  Pensilvania, Formación Marcellus)
- Actualizado: CP2 LNG Fase 3 (FERC abrió periodo de scoping NEPA 17-ago-2026),
  South Railroad Project (BLM emitió ROD positivo, ahora bajo Equinox Gold tras
  fusión con Orla Mining), Project Jupiter (gasoducto Green Chile retrasado a
  1-feb-2027), Texas Critical Data Centers Campus (permisos de construcción
  obtenidos)

proyectos.xlsx regenerado con el acumulado completo (49 Petroquímica, 42 LNG,
83 Mining, 83 Data Centers).
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -419,13 +419,13 @@
   <dimension ref="A1:G50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2292,13 +2292,13 @@
   <dimension ref="A1:G43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3619,17 +3619,17 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Permitting (FERC exoneró proceso de pre-filing 16-abr-2026; solicitud formal presentada 26-may-2026; Notice of Application publicado 12-jun-2026; 6 bloques de licuefacción adicionales/12 trenes, planta de energía de 720MW, tercer atracadero marino; eleva capacidad pico del complejo de 28 a 35 mtpa)</t>
+          <t>Permitting (FERC exoneró proceso de pre-filing 16-abr-2026; solicitud formal presentada 26-may-2026; Notice of Application publicado 12-jun-2026; FERC abrió formalmente el periodo de scoping NEPA el 17-ago-2026 —Docket CP26-530/533—, con comentario público hasta 11-sep-2026 y sesiones de scoping presenciales en Cameron Parish, LA y Jasper County, TX; 6 bloques de licuefacción adicionales/12 trenes, planta de energía de 720MW, tercer atracadero marino, más ~1,900 MMpc/d de capacidad incremental en el gasoducto CP Express; eleva capacidad pico del complejo de 28 a 35 mtpa)</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>[Federal Register](https://www.federalregister.gov/documents/2026/06/12/2026-11881/venture-global-cp2-lng-llc-venture-global-cp-express-llc-notice-of-application-and-establishing)</t>
+          <t>[Federal Register - Notice of Application](https://www.federalregister.gov/documents/2026/06/12/2026-11881/venture-global-cp2-lng-llc-venture-global-cp-express-llc-notice-of-application-and-establishing); [Federal Register - Notice of Scoping Period](https://www.federalregister.gov/documents/2026/08/17/2026-16739/venture-global-cp2-lng-llc-venture-global-cp-express-llc-notice-of-scoping-period-requesting)</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -3906,13 +3906,13 @@
   <dimension ref="A1:G84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4483,7 +4483,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Orla Mining Ltd.</t>
+          <t>Equinox Gold Corp. (tras fusión con Orla Mining Ltd.)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -4493,17 +4493,17 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Construcción (inicio previsto mediados 2026, pendiente ROD final de BLM)</t>
+          <t>Construcción (BLM emitió Record of Decision positivo el 17-ago-2026, completando el permiso federal NEPA bajo el proceso acelerado FAST-41 —primera mina a cielo abierto procesada bajo este esquema—, habilitando el inicio de construcción; mina de oro/plata a cielo abierto con lixiviación en pilas, ~130,000 oz Au/año promedio en los primeros 5 años; capex inicial ~US$395 millones; ~600 empleos en construcción)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>[Orla Mining](https://orlamining.com/news/orla-announces-results-of-updated-feasibility-study-for-south-railroad-project/)</t>
+          <t>[StockTitan/Equinox Gold](https://www.stocktitan.net/news/EQX/equinox-gold-receives-positive-record-of-decision-for-south-railroad-ds4bk9llu3hv.html); [BLM.gov](https://www.blm.gov/announcement/blm-approves-nevada-gold-and-silver-mine-support-american-mineral-production)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -7034,16 +7034,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G83"/>
+  <dimension ref="A1:G84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7587,17 +7587,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Construcción activa con riesgo regulatorio (Comisionada de Tierras de NM rechazó por segunda vez el derecho de vía en terrenos estatales para el gasoducto "Green Chile" de Energy Transfer, 14-jul-2026; NMED pospuso la decisión final sobre permisos de calidad de aire de las dos plantas de gas gemelas y programó audiencia pública para 19-oct-2026; meta de entrada en servicio ago-2026 en riesgo)</t>
+          <t>Construcción activa con retraso regulatorio confirmado (Comisionada de Tierras de NM rechazó por segunda vez el derecho de vía en terrenos estatales para el gasoducto "Green Chile" de Energy Transfer/Transwestern Pipeline, 14-jul-2026; filing regulatorio reportado 14-ago-2026 confirma que la fecha de entrada en servicio del gasoducto —que alimentará hasta 2.5GW de celdas de combustible Bloom Energy— se retrasó de 15-ago-2026 a 1-feb-2027; NMED pospuso decisión final sobre permisos de calidad de aire de las dos plantas de gas gemelas, audiencia pública programada 19-oct-2026; analistas citados advierten riesgo de nuevo retraso a 2S2027)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>[Source NM](https://sourcenm.com/2026/07/16/new-mexico-land-commissioner-blocks-project-jupiter-related-pipeline-from-building-on-state-land/)</t>
+          <t>[Source NM](https://sourcenm.com/2026/07/16/new-mexico-land-commissioner-blocks-project-jupiter-related-pipeline-from-building-on-state-land/); [Bloomberg](https://www.bloomberg.com/news/articles/2026-08-14/new-mexico-gas-pipeline-for-oracle-data-center-delayed-to-2027)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -7730,22 +7730,22 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Stream Data Centers (JV vía LOI); Thunderhead Energy Solutions (carta de acuerdo no vinculante para ~250MW de gen. de gas behind-the-meter)</t>
+          <t>Stream Data Centers (JV vía LOI); Thunderhead Energy Solutions (~250MW de gen. de gas behind-the-meter)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Ingeniería Fase Two (438 acres totales; permiso de aire en trámite; construcción total prevista en 2026, primeros 100MW dic-2026)</t>
+          <t>Permisos de construcción obtenidos (New Era Energy &amp; Digital anunció 14-ago-2026, junto con su reporte 10-Q 2T2026, que ya cuenta con los permisos de construcción para TCDC; sitio escalable hacia 1.4GW; construcción total prevista en 2026, primeros 100MW dic-2026)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55289667/powering-ai-in-the-permian-texas-critical-data-centers-sustainable-energy-play)</t>
+          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55289667/powering-ai-in-the-permian-texas-critical-data-centers-sustainable-energy-play); [GlobeNewswire](https://www.globenewswire.com/news-release/2026/08/14/3345632/0/en/new-era-energy-digital-files-q2-2026-form-10-q-and-announces-tcdc-construction-permits.html)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -10114,6 +10114,43 @@
       <c r="G83" t="inlineStr">
         <is>
           <t>2026-08-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Alpha Compute Corp — Campus de Data Center a Gas Natural</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Norte de Pensilvania, EE.UU. (región de gas Marcellus)</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Alpha Compute Corp</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Pre-construcción (term sheet vinculante firmado 11-ago-2026 para adquirir ~1,800 acres de derechos minerales de petróleo/gas —Formación Marcellus— más activos de superficie/espacio de poro, para desarrollar campus de data center a gas natural behind-the-meter; fase inicial 200MW, expansión potencial a 1GW; precio base de compra US$55 millones; pendiente permisos de PA DEP/Susquehanna River Basin Commission, financiamiento y acuerdos definitivos)</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/08/11/3343083/0/en/alpha-compute-signs-binding-term-sheet-for-planned-200-mw-natural-gas-powered-data-center-campus-in-pennsylvania-with-potential-expansion-to-1-gw.html)</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitoreo 2026-08-17: nuevo data center en PA + 4 actualizaciones de fase
- Nuevo: Alpha Compute Corp — Campus de Data Center a Gas Natural (norte de
  Pensilvania, Formación Marcellus)
- Actualizado: CP2 LNG Fase 3 (FERC abrió periodo de scoping NEPA 17-ago-2026),
  South Railroad Project (BLM emitió ROD positivo, ahora bajo Equinox Gold tras
  fusión con Orla Mining), Project Jupiter (gasoducto Green Chile retrasado a
  1-feb-2027), Texas Critical Data Centers Campus (permisos de construcción
  obtenidos)

proyectos.xlsx regenerado con el acumulado completo (49 Petroquímica, 42 LNG,
83 Mining, 83 Data Centers).

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -419,13 +419,13 @@
   <dimension ref="A1:G50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2292,13 +2292,13 @@
   <dimension ref="A1:G43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3619,17 +3619,17 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Permitting (FERC exoneró proceso de pre-filing 16-abr-2026; solicitud formal presentada 26-may-2026; Notice of Application publicado 12-jun-2026; 6 bloques de licuefacción adicionales/12 trenes, planta de energía de 720MW, tercer atracadero marino; eleva capacidad pico del complejo de 28 a 35 mtpa)</t>
+          <t>Permitting (FERC exoneró proceso de pre-filing 16-abr-2026; solicitud formal presentada 26-may-2026; Notice of Application publicado 12-jun-2026; FERC abrió formalmente el periodo de scoping NEPA el 17-ago-2026 —Docket CP26-530/533—, con comentario público hasta 11-sep-2026 y sesiones de scoping presenciales en Cameron Parish, LA y Jasper County, TX; 6 bloques de licuefacción adicionales/12 trenes, planta de energía de 720MW, tercer atracadero marino, más ~1,900 MMpc/d de capacidad incremental en el gasoducto CP Express; eleva capacidad pico del complejo de 28 a 35 mtpa)</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>[Federal Register](https://www.federalregister.gov/documents/2026/06/12/2026-11881/venture-global-cp2-lng-llc-venture-global-cp-express-llc-notice-of-application-and-establishing)</t>
+          <t>[Federal Register - Notice of Application](https://www.federalregister.gov/documents/2026/06/12/2026-11881/venture-global-cp2-lng-llc-venture-global-cp-express-llc-notice-of-application-and-establishing); [Federal Register - Notice of Scoping Period](https://www.federalregister.gov/documents/2026/08/17/2026-16739/venture-global-cp2-lng-llc-venture-global-cp-express-llc-notice-of-scoping-period-requesting)</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -3906,13 +3906,13 @@
   <dimension ref="A1:G84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4483,7 +4483,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Orla Mining Ltd.</t>
+          <t>Equinox Gold Corp. (tras fusión con Orla Mining Ltd.)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -4493,17 +4493,17 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Construcción (inicio previsto mediados 2026, pendiente ROD final de BLM)</t>
+          <t>Construcción (BLM emitió Record of Decision positivo el 17-ago-2026, completando el permiso federal NEPA bajo el proceso acelerado FAST-41 —primera mina a cielo abierto procesada bajo este esquema—, habilitando el inicio de construcción; mina de oro/plata a cielo abierto con lixiviación en pilas, ~130,000 oz Au/año promedio en los primeros 5 años; capex inicial ~US$395 millones; ~600 empleos en construcción)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>[Orla Mining](https://orlamining.com/news/orla-announces-results-of-updated-feasibility-study-for-south-railroad-project/)</t>
+          <t>[StockTitan/Equinox Gold](https://www.stocktitan.net/news/EQX/equinox-gold-receives-positive-record-of-decision-for-south-railroad-ds4bk9llu3hv.html); [BLM.gov](https://www.blm.gov/announcement/blm-approves-nevada-gold-and-silver-mine-support-american-mineral-production)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -7034,16 +7034,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G83"/>
+  <dimension ref="A1:G84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7587,17 +7587,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Construcción activa con riesgo regulatorio (Comisionada de Tierras de NM rechazó por segunda vez el derecho de vía en terrenos estatales para el gasoducto "Green Chile" de Energy Transfer, 14-jul-2026; NMED pospuso la decisión final sobre permisos de calidad de aire de las dos plantas de gas gemelas y programó audiencia pública para 19-oct-2026; meta de entrada en servicio ago-2026 en riesgo)</t>
+          <t>Construcción activa con retraso regulatorio confirmado (Comisionada de Tierras de NM rechazó por segunda vez el derecho de vía en terrenos estatales para el gasoducto "Green Chile" de Energy Transfer/Transwestern Pipeline, 14-jul-2026; filing regulatorio reportado 14-ago-2026 confirma que la fecha de entrada en servicio del gasoducto —que alimentará hasta 2.5GW de celdas de combustible Bloom Energy— se retrasó de 15-ago-2026 a 1-feb-2027; NMED pospuso decisión final sobre permisos de calidad de aire de las dos plantas de gas gemelas, audiencia pública programada 19-oct-2026; analistas citados advierten riesgo de nuevo retraso a 2S2027)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>[Source NM](https://sourcenm.com/2026/07/16/new-mexico-land-commissioner-blocks-project-jupiter-related-pipeline-from-building-on-state-land/)</t>
+          <t>[Source NM](https://sourcenm.com/2026/07/16/new-mexico-land-commissioner-blocks-project-jupiter-related-pipeline-from-building-on-state-land/); [Bloomberg](https://www.bloomberg.com/news/articles/2026-08-14/new-mexico-gas-pipeline-for-oracle-data-center-delayed-to-2027)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -7730,22 +7730,22 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Stream Data Centers (JV vía LOI); Thunderhead Energy Solutions (carta de acuerdo no vinculante para ~250MW de gen. de gas behind-the-meter)</t>
+          <t>Stream Data Centers (JV vía LOI); Thunderhead Energy Solutions (~250MW de gen. de gas behind-the-meter)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Ingeniería Fase Two (438 acres totales; permiso de aire en trámite; construcción total prevista en 2026, primeros 100MW dic-2026)</t>
+          <t>Permisos de construcción obtenidos (New Era Energy &amp; Digital anunció 14-ago-2026, junto con su reporte 10-Q 2T2026, que ya cuenta con los permisos de construcción para TCDC; sitio escalable hacia 1.4GW; construcción total prevista en 2026, primeros 100MW dic-2026)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55289667/powering-ai-in-the-permian-texas-critical-data-centers-sustainable-energy-play)</t>
+          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55289667/powering-ai-in-the-permian-texas-critical-data-centers-sustainable-energy-play); [GlobeNewswire](https://www.globenewswire.com/news-release/2026/08/14/3345632/0/en/new-era-energy-digital-files-q2-2026-form-10-q-and-announces-tcdc-construction-permits.html)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -10114,6 +10114,43 @@
       <c r="G83" t="inlineStr">
         <is>
           <t>2026-08-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Alpha Compute Corp — Campus de Data Center a Gas Natural</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Norte de Pensilvania, EE.UU. (región de gas Marcellus)</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Alpha Compute Corp</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Pre-construcción (term sheet vinculante firmado 11-ago-2026 para adquirir ~1,800 acres de derechos minerales de petróleo/gas —Formación Marcellus— más activos de superficie/espacio de poro, para desarrollar campus de data center a gas natural behind-the-meter; fase inicial 200MW, expansión potencial a 1GW; precio base de compra US$55 millones; pendiente permisos de PA DEP/Susquehanna River Basin Commission, financiamiento y acuerdos definitivos)</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/08/11/3343083/0/en/alpha-compute-signs-binding-term-sheet-for-planned-200-mw-natural-gas-powered-data-center-campus-in-pennsylvania-with-potential-expansion-to-1-gw.html)</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitoreo 2026-08-19: 6 proyectos nuevos + 4 actualizaciones de fase
- Nuevos: Distrito Copper Creek/San Manuel (AZ), IMA Mine (ID), Railroad
  Valley Minerals/Super-Brine Complex (NV), New Amalga Gold Project (AK),
  ElementUSA Gramercy (LA) en Mining; Crusoe/Blue Energy Port of Victoria
  (TX) en Data Centers.
- Actualizaciones: Planta de Amoniaco Topolobampo GPO, Santa Cruz Copper
  Project, Elk Creek Critical Minerals Project, Fermi America Project
  Matador.
- proyectos.xlsx regenerado con las 4 hojas por industria.
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -431,9 +431,9 @@
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -978,17 +978,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Construcción parcial/PAUSA parcial (unidad de amoniaco ~95% completa según Presidencia, ago-2026; unidades de urea/metanol y terminal marina PAUSADAS en espera de acuerdo ambiental; gobierno de Sinaloa presentó "Plan Integral" de conservación/desarrollo sostenible de la Bahía de Ohuira, 4-ago-2026, para destrabar continuidad del proyecto)</t>
+          <t>Construcción parcial/PAUSA parcial (unidad de amoniaco ~95% completa según Presidencia, ago-2026, aunque reportes locales citan avance de solo ~60% con obra detenida por bloqueo; movimiento indígena yoreme-mayo "¡Aquí No!" mantiene plantón bloqueando el acceso de personal a la obra desde el 7-jun-2026; GPO ofreció (8/10-ago-2026) pausar formalmente las fases de urea, metanol y terminal marina como condición para levantar el bloqueo; Secretaría de Economía sostuvo reuniones con comunidades de Ohuira, Paredones, Lázaro Cárdenas y Topolobampo presentando el "Plan Integral", pero las comunidades respondieron con desconfianza y mantienen el plantón indefinido)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>[Ríodoce](https://riodoce.mx/2026/08/10/pausan-urea-y-metanol-pero-avanza-amoniaco-en-industria-en-la-bahia-de-ohuira/); [Gobierno de Sinaloa](https://sinaloa.gob.mx/presentan-plan-integral-para-la-conservacion-ambiental-el-bienestar-comunitario-y-el-desarrollo-sostenible-de-la-bahia-de-ohuira/)</t>
+          <t>[Ríodoce](https://riodoce.mx/2026/08/10/pausan-urea-y-metanol-pero-avanza-amoniaco-en-industria-en-la-bahia-de-ohuira/); [La Silla Rota](https://lasillarota.com/estados/2026/8/8/planta-de-amoniaco-en-sinaloa-gobierno-busca-luz-verde-al-proyecto-en-ohuira-523789.html); [Gobierno de Sinaloa](https://sinaloa.gob.mx/presentan-plan-integral-para-la-conservacion-ambiental-el-bienestar-comunitario-y-el-desarrollo-sostenible-de-la-bahia-de-ohuira/)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-19</t>
         </is>
       </c>
     </row>
@@ -2378,9 +2378,9 @@
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -3986,15 +3986,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G84"/>
+  <dimension ref="A1:G89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -4058,17 +4058,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Ingeniería completada (PFS define mina subterránea de 20,000 t/d y planta de cátodos de 72,000 t/año) / construcción prevista H1 2026; EXIM Bank gestiona ahora más de US$1,000 millones en financiamiento, como parte del paquete federal de US$3,000 millones en minerales críticos anunciado 7-8-ago-2026</t>
+          <t>Construcción (PFS define mina subterránea de 20,000 t/d y planta de cátodos de 72,000 t/año; EXIM Bank gestiona más de US$1,000 millones en financiamiento, como parte del paquete federal de US$3,000 millones en minerales críticos anunciado 7-8-ago-2026; Ivanhoe completó el pago final de adquisición de terreno —US$39.3 millones— satisfaciendo el acuerdo de compraventa, y cerró una línea de crédito bancario de US$200 millones para financiar el inicio de actividades mayores de construcción en 2026; primera producción de cobre prevista 2028)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>[Mining Weekly](https://www.miningweekly.com/article/ivanhoe-electric-pencils-in-2026-construction-start-at-arizona-copper-mine-2025-06-25); [MINING.COM](https://www.mining.com/web/trump-says-us-is-announcing-a-series-of-mining-projects-worth-3-billion/)</t>
+          <t>[Mining Weekly](https://www.miningweekly.com/article/ivanhoe-electric-pencils-in-2026-construction-start-at-arizona-copper-mine-2025-06-25); [Ivanhoe Electric](https://ivanhoeelectric.com/news/ivanhoe-electric-makes-final-land-acquisition-payment-at-the-santa-cruz-copper-project-in-arizona/)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-19</t>
         </is>
       </c>
     </row>
@@ -5390,17 +5390,17 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Construcción (portal de mina de doble rampa, ~US$44.6 millones, iniciado feb/mar-2026; nuevo Feasibility Study NI 43-101 —publicado 11/15-ago-2026— amplía el proyecto a 8 productos, incluyendo óxidos de disprosio y terbio, VPN8% antes de impuestos US$4,100 millones, vida de mina de 40 años, capex inicial US$1,850 millones a 35 meses; MOU firmado con Lockheed Martin para venta de ~16.5 ton/año de escandio; avanzando a ingeniería detallada, procura y contratación EPC; proyecto de niobio/escandio/titanio/tierras raras con planta de superficie que requerirá tubería de proceso)</t>
+          <t>Construcción (portal de mina de doble rampa, ~US$44.6 millones, iniciado feb/mar-2026; nuevo Feasibility Study NI 43-101 —publicado 11/15-ago-2026— amplía el proyecto a 8 productos, incluyendo óxidos de disprosio y terbio, VPN8% antes de impuestos US$4,100 millones, vida de mina de 40 años, capex inicial US$1,850 millones a 35 meses; MOU firmado con Lockheed Martin para venta de ~16.5 ton/año de escandio; Departamento de Defensa (programa DPA Title III) otorgó hasta US$10 millones a la subsidiaria Elk Creek Resources Corp. para desarrollo de producción de escandio, ago-2026; avanzando a ingeniería detallada, procura y contratación EPC; proyecto de niobio/escandio/titanio/tierras raras con planta de superficie que requerirá tubería de proceso)</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>[NioCorp](https://niocorp.com/niocorp-launches-construction-of-elk-creek-critical-minerals-project-mine-portal/); [Mining.com](https://www.mining.com/updated-feasibility-study-gives-niocorps-elk-creek-critical-minerals-project-a-4b-valuation/); [Daily Political](https://www.dailypolitical.com/2026/08/15/niocorps-elk-creek-study-sees-4-1b-npv-40-year-critical-minerals-mine.html)</t>
+          <t>[NioCorp](https://niocorp.com/niocorp-launches-construction-of-elk-creek-critical-minerals-project-mine-portal/); [Mining.com](https://www.mining.com/updated-feasibility-study-gives-niocorps-elk-creek-critical-minerals-project-a-4b-valuation/); [NioCorp DoD](https://www.niocorp.com/u-s-department-of-defense-awards-up-to-10-million-to-niocorps-subsidiary-elk-creek-resources-corp/)</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
     </row>
@@ -7103,6 +7103,191 @@
       <c r="G84" t="inlineStr">
         <is>
           <t>2026-08-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Distrito Copper Creek / San Manuel</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Condado de Pinal, Arizona, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Faraday Copper Corp. (adquiriendo la propiedad San Manuel de BHP; BHP recibirá ~30% de acciones de Faraday)</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Exploración/definición de recursos (Faraday firmó acuerdo definitivo para comprar la antigua mina San Manuel de BHP —subterránea y de tajo/ISL, operada 1955-1999— y combinarla con su proyecto adyacente Copper Creek, creando un distrito de &gt;18,000 millones de libras de cobre; asamblea de accionistas 25-ago-2026 para aprobar la transacción, cierre esperado 3T2026; plan de 23,000+ metros de perforación de confirmación desde 4T2026, recurso combinado a mediados de 2027)</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>[MINING.COM](https://www.mining.com/faraday-targets-18b-lb-arizona-copper-district/)</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>IMA Mine</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Condado de Lemhi, Idaho, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>American Tungsten Corp.</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>No especificado (geotécnica de presas de jales: NewFields MTDs)</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Reactivación/pruebas metalúrgicas (mina histórica de tungsteno, produjo WO3 1945-1957; Fase I: reprocesamiento de jales superficiales; Fase II: rehabilitación de mina subterránea; pruebas metalúrgicas iniciadas jul-2026; definición de recursos, permisos y pruebas previstas concluir 4T2026, construcción fin de 2026/1T2027, primera venta de concentrado prevista inicios de 2027)</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>[MINING.COM](https://www.mining.com/american-tungsten-kinks-off-construction-at-ima-project-in-idaho/)</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Railroad Valley Minerals / Super-Brine Complex</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Railroad Valley, Nevada, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>3 Proton Lithium (3PL Operating Inc.)</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Exploración avanzada (depósito multi-mineral confirmado: litio, potasa, boro y lo que la empresa describe como el mayor depósito de tungsteno de EE.UU. —~1.78 millones de toneladas, valorado en ~US$152,000 millones in-situ—; ~17 millas cuadradas del área están retiradas de minería desde 2023 por solicitud de la NASA para calibración de satélites, lo que representa un obstáculo regulatorio; sin decisión de construcción)</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>[MINING.COM](https://www.mining.com/largest-us-tungsten-discovery-hits-nasa-roadblock/)</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>New Amalga Gold Project</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>~25 km al norte de Juneau, Alaska, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Grande Portage Resources Ltd.</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Permitting temprano (recurso Indicado de 1.44 millones oz Au a 9.47 g/t e Inferido de 515,700 oz Au; obtuvo estatus de "Covered Project" bajo FAST-41 el 30-jul-2026, acelerando la revisión federal coordinada; quinta mina en Alaska con cobertura FAST-41, junto con Arctic, Johnson Tract, Donlin Gold y Graphite Creek)</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>[Mining News North](https://www.miningnewsnorth.com/story/2026/08/07/news/new-amalga-gold-project-enters-fast-41/9803.html)</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>ElementUSA Gramercy — Planta de Tierras Raras/Minerales Críticos</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Gramercy, St. John the Baptist Parish, Luisiana, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>ElementUSA Inc. (en colaboración con Colorado School of Mines)</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Ingeniería/financiamiento asegurado (proyecto de US$850 millones para procesar "lodo rojo"/bauxite residue del antiguo refinerio de alúmina Atalco —~34 millones de toneladas almacenadas— y extraer galio, escandio, disprosio, gadolinio, iterbio, germanio e itrio; recibió US$67 millones del DOE y US$29.9 millones del DoD; construcción de planta de demostración prevista a iniciar mediados de 2027, producción inicial 3T2028)</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>[Biz New Orleans](https://bizneworleans.com/elementusa-plans-850m-critical-minerals-refining-facility/); [Colorado School of Mines](https://www.minesnewsroom.com/news/colorado-school-mines-and-elementusa-awarded-67m-doe-construction-rare-earth-processing-plant)</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
         </is>
       </c>
     </row>
@@ -7117,15 +7302,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G84"/>
+  <dimension ref="A1:G85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -8595,17 +8780,17 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Construcción (movimiento de tierra del campus inicial completo; 4.6 millas de gasoducto de 450 MMcf/d instaladas y conectadas al sistema interestatal de Energy Transfer, suficiente para los primeros 2GW; tubería de agua de 20"/7.2 millas completa; turbinas en sitio/tránsito: 3x GE Frame 6B, 3x Siemens SGT6-5000F, 6x Siemens SGT-800; nuevo acuerdo con Hillcore Energy Capital para "Hillcore Power Center" de ~2.6GW —2.5GW gas natural + 100MW solar/batería—, primer bloque de ~350MW inicia construcción al firmarse acuerdos definitivos, duplicando la generación en sitio a 4.8GW en ~30 meses; Fermi planea solicitar permiso TCEQ adicional por 5GW más, meta total 17GW)</t>
+          <t>Construcción (movimiento de tierra del campus inicial completo; 4.6 millas de gasoducto de 450 MMcf/d instaladas y conectadas al sistema interestatal de Energy Transfer, suficiente para los primeros 2GW; tubería de agua de 20"/7.2 millas completa; turbinas en sitio/tránsito: 3x GE Frame 6B, 3x Siemens SGT6-5000F, 6x Siemens SGT-800; nuevo acuerdo con Hillcore Energy Capital para "Hillcore Power Center" de ~2.6GW —2.5GW gas natural + 100MW solar/batería—, primer bloque de ~350MW inicia construcción al firmarse acuerdos definitivos, duplicando la generación en sitio a 4.8GW en ~30 meses; Fermi planea solicitar permiso TCEQ adicional por 5GW más, meta total 17GW; primer contrato de arrendamiento vinculante anunciado 10-ago-2026 con TensorWave —~US$6,500 millones a 15 años, instalación de 222MW con derechos de expansión hasta &gt;650MW combinados—; nombramiento 13-ago-2026 de Lee McIntire —ex-Bechtel/TerraPower— como nuevo CEO para liderar transición de desarrollo a construcción, meta de ~200MW de primera energía comercial en 6 meses; ~6GW de los 17GW planeados ya permitidos, &gt;US$1,500 millones invertidos a la fecha)</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>[StockTitan](https://www.stocktitan.net/news/FRMI/fermi-america-tells-texas-lawmakers-project-matador-will-push-the-z7wbkjm2tsxy.html); [DCD](https://www.datacenterdynamics.com/en/news/fermi-taps-hillcore-to-construct-26gw-gas-plant-for-up-to-11gw-project-matador-in-amarillo-texas/)</t>
+          <t>[StockTitan](https://www.stocktitan.net/news/FRMI/fermi-america-tells-texas-lawmakers-project-matador-will-push-the-z7wbkjm2tsxy.html); [DCD](https://www.datacenterdynamics.com/en/news/fermi-taps-hillcore-to-construct-26gw-gas-plant-for-up-to-11gw-project-matador-in-amarillo-texas/); [NewsChannel 10](https://www.newschannel10.com/2026/08/10/fermi-america-announces-65-billion-contract-with-tensorwave/); [247wallst](https://247wallst.com/investing/2026/08/13/fermi-lands-its-first-anchor-customer-and-names-a-ceo-as-project-matador-moves-to-construction/)</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-19</t>
         </is>
       </c>
     </row>
@@ -10234,6 +10419,43 @@
       <c r="G84" t="inlineStr">
         <is>
           <t>2026-08-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Crusoe / Blue Energy — Port of Victoria Campus</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Victoria, Texas, EE.UU. (Puerto de Victoria, campus de ~1,600 acres)</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Crusoe (desarrollador/operador del centro de datos de IA); suministro de energía: Blue Energy</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>GE Vernova Hitachi Nuclear Energy (GVH, reactores modulares SMR BWRX-300); GE Vernova (turbinas de gas 7HA.02)</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Ingeniería/licenciamiento (Blue Energy y GE Vernova Hitachi firmaron acuerdo 13-ago-2026 para lanzar la siguiente fase —ingeniería de diseño, licenciamiento y análisis de seguridad— de una planta híbrida gas+nuclear de 2.5GW; dos turbinas de gas GE Vernova 7HA.02 suministrarían ~1GW como "puente de gas" desde 2030, seguido de hasta 1.5GW adicionales de hasta cinco SMR BWRX-300 desde 2032, para alimentar un campus de centro de datos de Crusoe de hasta 1.5GW; FID prevista 2027)</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>[GE Vernova](https://www.gevernova.com/news/press-releases/blue-energy-ge-vernova-hitachi-launch-next-phase-gas-plus-nuclear-project); [DCD](https://www.datacenterdynamics.com/en/news/blue-energy-ge-vernova-hitachi-advance-25gw-gas-plus-nuclear-plant-in-texas-to-power-up-to-15gw-data-center/)</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitoreo 2026-08-21: 0 proyectos nuevos + 1 actualización
- LNG: Alaska LNG — la tercera sesión especial de la Legislatura de
  Alaska terminó sin votar el proyecto de ley de exenciones fiscales
  (HB 4001); el gobernador Dunleavy dio por concluido el esfuerzo
  legislativo de este año y Glenfarne declaró que evalúa "rutas
  alternativas" mientras continúa el trabajo comercial, de ingeniería
  y financiero del proyecto completo.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011YRaNrF2K1CETN3GYxW1Cf
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -67,7 +67,7 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -442,10 +442,10 @@
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -2389,10 +2389,10 @@
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -3122,17 +3122,17 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Pre-FID/Retraso legislativo persistente (tras el fracaso del HB 381, la coalición mayoritaria de la Cámara de Alaska anunció 13/14-ago-2026 que el nuevo proyecto de ley HB 4001 —exenciones fiscales necesarias para el gasoducto de 20 Mtpa— tampoco tiene los votos para pasar, por diferencias sobre alivio de impuesto predial; gobernador Dunleavy llamó a reconvocar sesión el 20-ago-2026; pese al estancamiento legislativo, avances comerciales recientes incluyen acuerdo de suministro de acero con POSCO vía Glenfarne y acuerdos preliminares de compra con JERA y Tokyo Gas por 2 Mtpa; Glenfarne aún no alcanza el umbral de contratos vinculantes por el 80% de la capacidad)</t>
+          <t>Pre-FID/Sesión especial legislativa terminó SIN acción (tras el fracaso del HB 381 y luego del HB 4001, el liderazgo del Senado de Alaska decidió no reconvocar la cámara para votar el proyecto de ley de exenciones fiscales de Dunleavy; el propio gobernador señaló 18/19-ago-2026 que ya no hay razón para continuar la tercera sesión especial y que la Legislatura no retomará la legislación fiscal este año, dando por terminado el esfuerzo; Glenfarne declaró que el fracaso del recorte fiscal causará retraso de cronograma y aumento de costos, y que evalúa "rutas alternativas" mientras continúa el trabajo comercial, de ingeniería y financiero para el proyecto completo —incluida la terminal de exportación de LNG—, valuado en hasta US$55,000 millones, con Glenfarne dueño de 75% y Alaska Gasline Development Corp del 25% restante; avances comerciales previos incluyen acuerdo de suministro de acero con POSCO y acuerdos preliminares de compra con JERA y Tokyo Gas por 2 Mtpa)</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>[Alaska Beacon](https://alaskabeacon.com/2026/07/17/hilcorp-killed-alaska-lng-bill-some-legislators-say-but-governor-calls-the-claim-bullst/); [Alaska's News Source](https://www.alaskasnewssource.com/2026/08/13/alaska-lng-pipeline-bill-collapses-house-majority-says-it-lacks-votes/)</t>
+          <t>[Alaska Beacon](https://alaskabeacon.com/2026/07/17/hilcorp-killed-alaska-lng-bill-some-legislators-say-but-governor-calls-the-claim-bullst/); [Anchorage Daily News](https://www.adn.com/business-economy/energy/2026/08/19/alaska-lng-developer-looks-for-alternative-paths-after-effort-to-secure-multibillion-dollar-tax-cut-fails/)</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -4040,10 +4040,10 @@
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -7393,10 +7393,10 @@
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>

</xml_diff>

<commit_message>
Monitoreo 2026-08-21: 0 proyectos nuevos + 1 actualización (#28)
- LNG: Alaska LNG — la tercera sesión especial de la Legislatura de
  Alaska terminó sin votar el proyecto de ley de exenciones fiscales
  (HB 4001); el gobernador Dunleavy dio por concluido el esfuerzo
  legislativo de este año y Glenfarne declaró que evalúa "rutas
  alternativas" mientras continúa el trabajo comercial, de ingeniería
  y financiero del proyecto completo.


Claude-Session: https://claude.ai/code/session_011YRaNrF2K1CETN3GYxW1Cf

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -67,7 +67,7 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -442,10 +442,10 @@
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -2389,10 +2389,10 @@
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -3122,17 +3122,17 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Pre-FID/Retraso legislativo persistente (tras el fracaso del HB 381, la coalición mayoritaria de la Cámara de Alaska anunció 13/14-ago-2026 que el nuevo proyecto de ley HB 4001 —exenciones fiscales necesarias para el gasoducto de 20 Mtpa— tampoco tiene los votos para pasar, por diferencias sobre alivio de impuesto predial; gobernador Dunleavy llamó a reconvocar sesión el 20-ago-2026; pese al estancamiento legislativo, avances comerciales recientes incluyen acuerdo de suministro de acero con POSCO vía Glenfarne y acuerdos preliminares de compra con JERA y Tokyo Gas por 2 Mtpa; Glenfarne aún no alcanza el umbral de contratos vinculantes por el 80% de la capacidad)</t>
+          <t>Pre-FID/Sesión especial legislativa terminó SIN acción (tras el fracaso del HB 381 y luego del HB 4001, el liderazgo del Senado de Alaska decidió no reconvocar la cámara para votar el proyecto de ley de exenciones fiscales de Dunleavy; el propio gobernador señaló 18/19-ago-2026 que ya no hay razón para continuar la tercera sesión especial y que la Legislatura no retomará la legislación fiscal este año, dando por terminado el esfuerzo; Glenfarne declaró que el fracaso del recorte fiscal causará retraso de cronograma y aumento de costos, y que evalúa "rutas alternativas" mientras continúa el trabajo comercial, de ingeniería y financiero para el proyecto completo —incluida la terminal de exportación de LNG—, valuado en hasta US$55,000 millones, con Glenfarne dueño de 75% y Alaska Gasline Development Corp del 25% restante; avances comerciales previos incluyen acuerdo de suministro de acero con POSCO y acuerdos preliminares de compra con JERA y Tokyo Gas por 2 Mtpa)</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>[Alaska Beacon](https://alaskabeacon.com/2026/07/17/hilcorp-killed-alaska-lng-bill-some-legislators-say-but-governor-calls-the-claim-bullst/); [Alaska's News Source](https://www.alaskasnewssource.com/2026/08/13/alaska-lng-pipeline-bill-collapses-house-majority-says-it-lacks-votes/)</t>
+          <t>[Alaska Beacon](https://alaskabeacon.com/2026/07/17/hilcorp-killed-alaska-lng-bill-some-legislators-say-but-governor-calls-the-claim-bullst/); [Anchorage Daily News](https://www.adn.com/business-economy/energy/2026/08/19/alaska-lng-developer-looks-for-alternative-paths-after-effort-to-secure-multibillion-dollar-tax-cut-fails/)</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -4040,10 +4040,10 @@
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -7393,10 +7393,10 @@
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>

</xml_diff>

<commit_message>
Monitoreo 2026-08-24: 4 proyectos nuevos + 15 actualizaciones de fase
Nuevos: La Preciosa Project (Mining); KIO Data Centers QRO3, Prometheus
Hyperscale Pecos/Istmo, Riot Platforms Rockdale/Anthropic (Data Centers).

Actualizaciones: Topolobampo GPO, Targa Wrangler/Ranger/Ranger II
(Petroquímica); Rio Grande LNG, Corpus Christi Stage 3 (LNG); Thacker
Pass, Media Luna, Stibnite, CK Gold, Galena Complex, Los Ricos South,
Hermosa, Shirley Basin (Mining); TCDC, Anthropic/Nexus Hubbard (Data
Centers). Se agregó nota sobre pausa regulatoria ERCOT/PUCT en Texas.

proyectos.xlsx regenerado con el acumulado completo (272 proyectos).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VX2fVsTxp6qwkT81FGhrJW
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -31,25 +31,19 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
-        <bgColor rgb="001F4E78"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -66,8 +60,8 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -440,16 +434,16 @@
   <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proyecto</t>
@@ -990,7 +984,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Construcción parcial/PAUSA parcial (unidad de amoniaco ~95% completa según Presidencia, ago-2026, aunque reportes locales citan avance de solo ~60% con obra detenida por bloqueo; movimiento indígena yoreme-mayo "¡Aquí No!" mantiene plantón bloqueando el acceso de personal a la obra desde el 7-jun-2026; GPO ofreció (8/10-ago-2026) pausar formalmente las fases de urea, metanol y terminal marina como condición para levantar el bloqueo; Secretaría de Economía sostuvo reuniones con comunidades de Ohuira, Paredones, Lázaro Cárdenas y Topolobampo presentando el "Plan Integral", pero las comunidades respondieron con desconfianza y mantienen el plantón indefinido)</t>
+          <t>Construcción parcial/PAUSA parcial (unidad de amoniaco ~95% completa según Presidencia, ago-2026 —prensa local cita 88% de avance—, aunque reportes locales previos citaban solo ~60% con obra detenida por bloqueo; movimiento indígena yoreme-mayo "¡Aquí No!" mantiene plantón bloqueando el acceso de personal a la obra desde el 7-jun-2026; GPO ofreció (8/10-ago-2026) pausar formalmente las fases de urea, metanol y terminal marina como condición para levantar el bloqueo; Secretaría de Economía sostuvo reuniones con comunidades de Ohuira, Paredones, Lázaro Cárdenas y Topolobampo presentando el "Plan Integral", pero las comunidades respondieron con desconfianza y mantienen el plantón indefinido)</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -1000,7 +994,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -2322,17 +2316,17 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Anuncio/Planeación (anunciado 17-ago-2026; tres nuevas plantas criogénicas con capacidad combinada ~825 MMcf/d, más nuevo gasoducto de ~70 millas "Bull Run II" hacia el hub de Waha; entrada en servicio prevista 1S2028)</t>
+          <t>Anuncio/Planeación (anunciado 17-ago-2026; tres nuevas plantas criogénicas con capacidad combinada ~825 MMcf/d, más nuevo gasoducto de ~70 millas "Bull Run II" hacia el hub de Waha; entrada en servicio prevista 1S2028; Targa evalúa además hasta 5 plantas adicionales en Permian Delaware a más largo plazo)</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>[EnergyNow](https://energynow.com/2026/08/targa-to-build-three-permian-gas-processing-plants-new-pipeline/)</t>
+          <t>[EnergyNow](https://energynow.com/2026/08/targa-to-build-three-permian-gas-processing-plants-new-pipeline/); [Targa Resources](https://www.targaresources.com/news-releases/news-release-details/targa-resources-corp-announces-20-year-agreements-exxonmobil-and)</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -2387,16 +2381,16 @@
   <dimension ref="A1:G44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proyecto</t>
@@ -2456,17 +2450,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Construcción (FERC aprobó inicio de construcción de Trenes 4 y 5 en mar-2026; gasoducto de alimentación Rio Bravo Pipeline —138 millas, JV Whitewater/MPLX/Enbridge— en camino a entrar en servicio 2S2026); Train 6 avanza a permitting formal (FERC inició scoping del EIS, solicitud presentada 26-may-2026, sesión de scoping virtual 19-ago-2026, FID prevista 2027; ~6.03 mtpa adicionales, llevando el sitio a 48 mtpa con Trenes 7-8)</t>
+          <t>Construcción (FERC aprobó inicio de construcción de Trenes 4 y 5 en mar-2026; gasoducto de alimentación Rio Bravo Pipeline —138 millas, JV Whitewater/MPLX/Enbridge— en camino a entrar en servicio 2S2026); Train 6 avanza a permitting formal (FERC inició scoping del EIS, solicitud presentada 26-may-2026, sesión de scoping virtual 19-ago-2026, FID prevista 2027; ~6.03 mtpa adicionales, llevando el sitio a 48 mtpa con Trenes 7-8); adicionalmente FERC publicó 19-ago-2026 el calendario de preparación de una Environmental Assessment para la "Rio Grande LNG Capacity Amendment", que alinearía la capacidad aprobada de Trenes 4-5 de 5.4 a ~6.03 mtpa por tren (27.0→~30.15 mtpa); EA programada 25-ago-2026, decisión final 23-nov-2026</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>[Bechtel](https://www.bechtel.com/press-releases/nextdecade-executes-epc-contract-with-bechtel-for-train-4-at-the-rio-grande-lng-facility/); [Natural Gas Intel](https://naturalgasintel.com/news/nextdecade-targets-more-than-36-mty-with-rio-grande-lng-upscale-sixth-train-expansion/); [Federal Register](https://www.federalregister.gov/documents/2026/08/03/2026-15695/rio-grande-lng-train-6-llc-notice-of-intent-to-prepare-an-environmental-impact-statement-for-the); [LNG Prime](https://lngprime.com/americas/nextdecade-seeks-ferc-ok-for-sixth-rio-grande-lng-train/187820/)</t>
+          <t>[Bechtel](https://www.bechtel.com/press-releases/nextdecade-executes-epc-contract-with-bechtel-for-train-4-at-the-rio-grande-lng-facility/); [Natural Gas Intel](https://naturalgasintel.com/news/nextdecade-targets-more-than-36-mty-with-rio-grande-lng-upscale-sixth-train-expansion/); [Federal Register - Capacity Amendment](https://www.federalregister.gov/documents/2026/08/19/2026-16922); [LNG Prime](https://lngprime.com/americas/nextdecade-seeks-ferc-ok-for-sixth-rio-grande-lng-train/187820/)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -2678,17 +2672,17 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Construcción (FERC autorizó introducción de gas combustible en Train 7, 17-jul-2026, y autorizó introducción de gas natural al Train 7, 28-jul-2026; FERC aprobó formalmente la introducción de gas natural al Train 7 —séptimo y último tren de la expansión midscale— el 4-ago-2026; primera producción de LNG esperada ago-2026, servicio comercial sep-2026; Trenes 5 y 6 completados mar/jun-2026; expansión completa de 7 trenes 85.4% de avance, prevista para fin de 2026)</t>
+          <t>Construcción (FERC autorizó introducción de gas combustible en Train 7, 17-jul-2026, y autorizó introducción de gas natural al Train 7, 28-jul-2026; FERC aprobó formalmente la introducción de gas natural al Train 7 —séptimo y último tren de la expansión midscale— el 4-ago-2026; Cheniere completó dos trenes adicionales de licuefacción en Stage 3 a mediados de ago-2026, elevando el avance del proyecto a ~98% completo; Train 7 en fase final de comisionamiento; finalización del build-out de 7 trenes prevista para fin de 2026)</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>[PGJ](https://pgjonline.com/news/2026/july/cheniere-gets-approval-to-introduce-gas-into-final-corpus-christi-lng-train); [LNG Prime](https://lngprime.com/americas/chenieres-corpus-christi-expansion-project-85-4-percent-complete/155448/); [energiesmedia](https://energiesmedia.com/ferc-approves-cheniere-train-7-energies/)</t>
+          <t>[PGJ](https://pgjonline.com/news/2026/july/cheniere-gets-approval-to-introduce-gas-into-final-corpus-christi-lng-train); [OGJ](https://www.ogj.com/pipelines-transportation/lng/news/55340460/cheniere-completes-two-more-corpus-christi-stage-3-trains); [LNG Prime](https://lngprime.com/americas/chenieres-corpus-christi-stage-3-project-98-percent-complete/190871/)</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -4035,19 +4029,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G90"/>
+  <dimension ref="A1:G91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proyecto</t>
@@ -4218,7 +4212,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Construcción (ingeniería de detalle &gt;95% completa, procura &gt;70% completa a may-2026; capex guía 2026 de US$1,300-1,600 millones; terminación mecánica prevista fines de 2027)</t>
+          <t>Construcción (reporte 2T2026: ingeniería de detalle &gt;95% completa, procura &gt;80% completa; US$1,800 millones de un capex total de US$2,930 millones ya incurridos; +1,600 trabajadores en sitio; comisionamiento anticipado de servicios previsto fines de 2026, terminación mecánica prevista fines de 2027)</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -4228,7 +4222,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -4403,17 +4397,17 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Construcción (tubería de pasta pendiente)</t>
+          <t>Construcción de la mina principal CONCLUIDA (alcanzó tasa de diseño de 7,500 tpd, 9 meses antes de lo previsto); Media Luna North en desarrollo (avance completado del "North Adit", iniciando instalación de ventilación e infraestructura; primera producción esperada fines de 2026)</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>[Minería en Línea](https://mineriaenlinea.com/2026/04/torex-gold-alcanza-velocidad-de-crucero-en-media-luna-9-meses-adelante-de-cronograma/)</t>
+          <t>[Minería en Línea](https://mineriaenlinea.com/2026/04/torex-gold-alcanza-velocidad-de-crucero-en-media-luna-9-meses-adelante-de-cronograma/); [Minería PA](https://mineria-pa.com/2026/08/11/mexico-media-luna-norte-proyecta-su-primera-produccion-para-fines-de-2026/)</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -4477,17 +4471,17 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Construcción (Record of Decision final emitido por USFS 7-jul-2026 para infraestructura en Coronado National Forest; ~50% avance en porción privada) / Permitting adicional para desarrollo completo (USFS publicó 15-ago-2026 el Draft EIS y Draft Record of Decision para el desarrollo completo de Hermosa, abriendo periodo de objeción de 45 días seguido de 45 días de resolución; decisión final esperada verano 2026; primer proyecto minero aceptado en programa federal FAST-41; primer concentrado proyectado H1-2028)</t>
+          <t>Construcción (Record of Decision final emitido por USFS 7-jul-2026 para infraestructura en Coronado National Forest; ~50% avance en porción privada) / Permitting adicional para desarrollo completo (USFS publicó 15-ago-2026 el Draft EIS y Draft Record of Decision para el desarrollo completo de Hermosa, abriendo periodo de objeción de 45 días seguido de 45 días de resolución; decisión final esperada verano 2026; primer proyecto minero aceptado en programa federal FAST-41; primer concentrado proyectado H1-2028); South32 aumentó el capex de Taylor en ~US$1,100 millones (total ~US$3,300 millones) y retrasó la primera producción de mediados de 2027 a mediados de 2028 (capacidad plena ahora en FY2031), aunque Ore Reserves aumentaron +52% y la vida de mina se extendió a ~33 años</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>[USDA](https://www.usda.gov/about-usda/news/press-releases/2026/07/07/usda-advances-trump-administration-effort-boost-us-mineral-energy-production); [Tucson Sentinel](https://www.tucsonsentinel.com/local/report/030626_hermosa_mine_review/hermosa-mine-hits-milestone-after-forest-service-releases-enviro-review/)</t>
+          <t>[USDA](https://www.usda.gov/about-usda/news/press-releases/2026/07/07/usda-advances-trump-administration-effort-boost-us-mineral-energy-production); [Tucson Sentinel](https://www.tucsonsentinel.com/local/report/030626_hermosa_mine_review/hermosa-mine-hits-milestone-after-forest-service-releases-enviro-review/); [TipRanks](https://www.tipranks.com/news/company-announcements/south32-lifts-hermosa-taylor-mine-life-capex-and-delays-ramp-up-to-fy31)</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -4514,17 +4508,17 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Construcción (corte federal de Idaho negó en jun-2026 moción para detener obras; Export-Import Bank de EE.UU. aprobó en may-2026 préstamo garantizado de USD 2,900 millones, desembolso esperado 2S2026; nuevos objetivos de exploración de oro/antimonio de alta ley identificados y posible nueva fuente de tungsteno reportados 7-ago-2026)</t>
+          <t>Construcción (corte federal de Idaho negó en jun-2026 moción para detener obras; Directorio del Export-Import Bank de EE.UU. aprobó por unanimidad, 20-ago-2026, el préstamo garantizado senior de USD 2,900 millones para financiar el desarrollo; nuevos objetivos de exploración de oro/antimonio de alta ley identificados y posible nueva fuente de tungsteno reportados 7-ago-2026)</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/perpetua-resources-advances-construction-of-the-stibnite-gold-project-302787012.html); [Departamento de Justicia de EE.UU.](https://www.justice.gov/opa/pr/justice-department-secures-motion-allow-continued-construction-idaho-gold-mine-critical); [StreetWise Reports](https://www.streetwisereports.com/article/2026/08/10/idaho-gold-antimony-project-hits-high-grade-intercepts-at-stibnite.html)</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/perpetua-resources-advances-construction-of-the-stibnite-gold-project-302787012.html); [Departamento de Justicia de EE.UU.](https://www.justice.gov/opa/pr/justice-department-secures-motion-allow-continued-construction-idaho-gold-mine-critical); [StreetWise Reports](https://www.streetwisereports.com/article/2026/08/20/idaho-gold-antimony-developer-wins-2-9b-exim-loan-approval.html)</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -4699,17 +4693,17 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Permiso de Emplazamiento Industrial (Industrial Siting Permit) otorgado por Wyoming DEQ el 20-jun-2026, habilitando construcción y operación sin requerir NEPA (no involucra tierra federal); construcción pesada prevista hasta 2027, producción 2028</t>
+          <t>Permiso de Emplazamiento Industrial (Industrial Siting Permit) otorgado por Wyoming DEQ el 20-jun-2026, habilitando construcción y operación sin requerir NEPA (no involucra tierra federal); U.S. Gold Corp completó el permitting estatal —proyecto "totalmente permisado"—, lo que disparó interés estratégico de proveedores de capital y posible M&amp;A, reportado 20-ago-2026; construcción pesada prevista hasta 2027, producción 2028</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>[Wyoming News](https://www.wyomingnews.com/rawlinstimes/plans-move-forward-for-ck-gold-project-as-developers-target-2026-construction-start/article_b2bb147e-2f92-4ca2-bf86-fcc9983917a7.html); [Discovery Alert](https://discoveryalert.com.au/ck-gold-project-permitting-construction-ready-valuation-2026/)</t>
+          <t>[Wyoming News](https://www.wyomingnews.com/rawlinstimes/plans-move-forward-for-ck-gold-project-as-developers-target-2026-construction-start/article_b2bb147e-2f92-4ca2-bf86-fcc9983917a7.html); [Crux Investor](https://www.cruxinvestor.com/posts/us-gold-corp-evaluates-m-a-interest-as-ck-gold-project-advances)</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -4773,17 +4767,17 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Construcción (comisionamiento previsto Q4 2026)</t>
+          <t>Construcción SUSTANCIALMENTE COMPLETA en sitio Wardner; comisionamiento esperado dentro de las semanas siguientes al 31-jul-2026 (antes Q4 2026)</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>[SEC/Americas Gold and Silver](https://www.sec.gov/Archives/edgar/data/0001286973/000106299326002645/exhibit99-2.htm)</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/31/3337077/0/en/bunker-hill-ships-first-concentrate-to-trail-smelter-and-announces-drawdown-of-standby-facility.html)</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -4879,12 +4873,12 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Cominvi (contratista minero mexicano seleccionado); M3 Mexicana (diseño de planta, 55% completo)</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Construcción aprobada por el consejo (permisos SEMARNAT completos jun-2026; presupuesto ~US$227 millones; ventana de construcción de ~24 meses; primer vertido de metal previsto mediados de 2028)</t>
+          <t>Construcción aprobada por el consejo (permisos SEMARNAT completos jun-2026; presupuesto ~US$227 millones; ventana de construcción de ~24 meses; planta SART 70% completa; primer vertido de metal previsto mediados de 2028)</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -4894,7 +4888,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -6475,17 +6469,17 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Producción (autorización final del estado de Wyoming para operar a plena producción, reportada 10-ago-2026; planta satélite ISR integrada con Lost Creek; infraestructura de planta y transporte ya en sitio)</t>
+          <t>Producción (autorización final del estado de Wyoming para operar a plena producción, reportada 10-ago-2026; Ur-Energy realizó su PRIMER EMBARQUE de uranio desde la mina hacia la planta de procesamiento Lost Creek, 19-ago-2026 —transición de construcción a producción en 2.5 años—; planta satélite ISR integrada con Lost Creek)</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>[Ur-Energy](https://www.ur-energy.com/news-media/press-releases/detail/401/ur-energy-commences-operations-at-its-shirley-basin-isr); [Junior Mining Network](https://www.juniorminingnetwork.com/junior-miner-news/press-releases/557-tsx/ure/208831-ur-energy-reports-second-quarter-2026-results.html)</t>
+          <t>[Ur-Energy](https://www.ur-energy.com/news-media/press-releases/detail/410/ur-energy-announces-first-shipment-of-uranium-from-shirley); [Junior Mining Network](https://www.juniorminingnetwork.com/junior-miner-news/press-releases/557-tsx/ure/208831-ur-energy-reports-second-quarter-2026-results.html)</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -7374,6 +7368,43 @@
       <c r="G90" s="2" t="inlineStr">
         <is>
           <t>2026-08-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>La Preciosa Project</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>Durango, México</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>Avino Silver &amp; Gold Mines Ltd.</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>Construcción (desarrollo subterráneo en curso —rampa/decline de 360m—; permisos mineros ya obtenidos; producción objetivo 4T2026)</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>[AccessWire](https://www.accessnewswire.com/newsroom/en/metals-and-mining/avino-provides-update-on-its-100-owned-la-preciosa-property-preparing-for-producti-837173); [MarketScreener](https://www.marketscreener.com/quote/stock/AVINO-SILVER-GOLD-MINES-L-1409069/news/Avino-Silver-Gold-Mines-Ltd-Commences-Underground-Development-At-La-Preciosa-48766238/)</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -7388,19 +7419,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G86"/>
+  <dimension ref="A1:G89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proyecto</t>
@@ -8084,22 +8115,22 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Stream Data Centers (JV vía LOI); Thunderhead Energy Solutions (~250MW de gen. de gas behind-the-meter)</t>
+          <t>Stream Data Centers (JV vía LOI); Thunderhead Energy Solutions (gen. de gas behind-the-meter)</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Permisos de construcción obtenidos (New Era Energy &amp; Digital anunció 14-ago-2026, junto con su reporte 10-Q 2T2026, que ya cuenta con los permisos de construcción para TCDC; sitio escalable hacia 1.4GW; construcción total prevista en 2026, primeros 100MW dic-2026)</t>
+          <t>Permisos de construcción obtenidos (New Era Energy &amp; Digital anunció 14-ago-2026, junto con su reporte 10-Q 2T2026, que ya cuenta con los permisos de construcción para TCDC; sitio escalable hacia 1.4GW; New Era aseguró permisos clave adicionales —Development Structure Permit, Drive Approach Permit— y presentó Notice of Intent ante TCEQ para nivelación de terreno, 17-ago-2026; capacidad combinada Fase 1+2 aumentó de ~650MW a 757MW vía nuevo permiso de aire TCEQ de Thunderhead (Fase 2: 450→550MW); construcción total prevista en 2026, primeros 100MW dic-2026)</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55289667/powering-ai-in-the-permian-texas-critical-data-centers-sustainable-energy-play); [GlobeNewswire](https://www.globenewswire.com/news-release/2026/08/14/3345632/0/en/new-era-energy-digital-files-q2-2026-form-10-q-and-announces-tcdc-construction-permits.html)</t>
+          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55289667/powering-ai-in-the-permian-texas-critical-data-centers-sustainable-energy-play); [GlobeNewswire](https://www.globenewswire.com/news-release/2026/08/14/3345632/0/en/new-era-energy-digital-files-q2-2026-form-10-q-and-announces-tcdc-construction-permits.html); [Minichart](https://www.minichart.com.sg/2026/08/17/new-era-energy-secures-construction-permits-for-texas-data-center-campus/)</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -9596,7 +9627,7 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Anthropic (operado por Nexus Data Centers; respaldo financiero de Google)</t>
+          <t>Anthropic (confirmado como tenant ancla tras proceso de licitación competitivo; operado por Nexus Data Centers; respaldo financiero de Google)</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
@@ -9606,17 +9637,17 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Construcción iniciada (primera fase 500-612MW prevista 2026, ampliable a ~7.2-7.7GW; planta de gas natural behind-the-meter cerca de gasoducto principal; financiamiento avanzado: banca liderada por Morgan Stanley en negociaciones finales para prestar USD 15 mil millones a Nexus Data Centers —incluye préstamo puente de USD 14 mil millones más línea de crédito revolvente—; Google otorgaría garantías sobre obligaciones de arrendamiento y pago de energía de Anthropic a cambio de ~20% de participación accionaria en el proyecto combinado)</t>
+          <t>Construcción iniciada (primera fase 500-612MW prevista 2026, ampliable a ~7.2-7.7GW; planta de gas natural behind-the-meter cerca de gasoducto principal; permisos de primera fase cubren ~491,000 pies² de cómputo de alta densidad; Eagle Point Credit Management lidera un préstamo de crédito privado mezzanine de USD 1,300 millones, parte de un paquete de financiamiento de ~USD 16,000 millones, 19-ago-2026; Google garantiza la deuda senior)</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/600mw-natural-gas-powered-data-center-campus-proposed-in-hubbard-texas/); [Construction Review](https://constructionreviewonline.com/5bn-anthropic-data-center-in-texas-receives-critical-financial-backing-from-google/); [CNBC](https://www.cnbc.com/2026/07/30/nexus-data-centers-in-advanced-talks-to-secure-15b-for-google-backed-anthropic-data-center.html)</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/600mw-natural-gas-powered-data-center-campus-proposed-in-hubbard-texas/); [Construction Review](https://constructionreviewonline.com/5bn-anthropic-data-center-in-texas-receives-critical-financial-backing-from-google/); [Private Equity Wire](https://www.privateequitywire.co.uk/eagle-point-leads-1-3bn-private-credit-loan-for-anthropic-linked-texas-data-centre/)</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -10579,6 +10610,117 @@
       <c r="G86" s="2" t="inlineStr">
         <is>
           <t>2026-08-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>KIO Data Centers — Expansión QRO3</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>El Marqués, Querétaro, México</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>KIO Data Centers</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>Anuncio de inversión (~US$1,300 millones, ~100MW adicionales, ~8,100 empleos proyectados)</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>[CódigoQro](https://codigoqro.mx/nota/local/2026/08/13/invertira-empresa-mexicana-mil-300-mdd-ampliacion-tercer-centro-datos-queretaro)</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>Prometheus Hyperscale "Pecos Project" (con Istmo Energy)</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>Reeves County, Texas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>Prometheus Hyperscale / Istmo Energy (JV)</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>Anuncio de desarrollo (hasta 2.5GW, dual-fuel —gas natural + metano de planta de fraccionamiento de Istmo Midstream—; primera energía prevista 2027)</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>[Data Center Dynamics](https://www.datacenterdynamics.com/en/news/prometheus-hyperscale-partners-with-istmo-to-develop-up-to-25gw-gas-powered-data-center-in-reeves-county-texas/)</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>Riot Platforms — Campus Rockdale (Anthropic)</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>Rockdale, Texas, EE.UU. (antigua planta de Alcoa)</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>Anthropic (tenant ancla) / Riot Platforms (desarrollador-operador)</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>Contrato de arrendamiento firmado (20 años, 191MW, ~US$9,100 millones; financiamiento interino de construcción de US$573 millones vía Morgan Stanley; primera fase de 96MW prevista dic-2027)</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>[Austin American-Statesman](https://www.statesman.com/business/technology/article/anthropic-riot-platforms-rockdale-texas-22383624.php); [Bloomberg](https://www.bloomberg.com/news/articles/2026-08-11/anthropic-strikes-9-billion-deal-with-cloud-computing-firm-riot)</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitoreo 2026-08-24: 4 proyectos nuevos + 15 actualizaciones de fase (#29)
Nuevos: La Preciosa Project (Mining); KIO Data Centers QRO3, Prometheus
Hyperscale Pecos/Istmo, Riot Platforms Rockdale/Anthropic (Data Centers).

Actualizaciones: Topolobampo GPO, Targa Wrangler/Ranger/Ranger II
(Petroquímica); Rio Grande LNG, Corpus Christi Stage 3 (LNG); Thacker
Pass, Media Luna, Stibnite, CK Gold, Galena Complex, Los Ricos South,
Hermosa, Shirley Basin (Mining); TCDC, Anthropic/Nexus Hubbard (Data
Centers). Se agregó nota sobre pausa regulatoria ERCOT/PUCT en Texas.

proyectos.xlsx regenerado con el acumulado completo (272 proyectos).


Claude-Session: https://claude.ai/code/session_01VX2fVsTxp6qwkT81FGhrJW

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -31,25 +31,19 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
-        <bgColor rgb="001F4E78"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -66,8 +60,8 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -440,16 +434,16 @@
   <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proyecto</t>
@@ -990,7 +984,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Construcción parcial/PAUSA parcial (unidad de amoniaco ~95% completa según Presidencia, ago-2026, aunque reportes locales citan avance de solo ~60% con obra detenida por bloqueo; movimiento indígena yoreme-mayo "¡Aquí No!" mantiene plantón bloqueando el acceso de personal a la obra desde el 7-jun-2026; GPO ofreció (8/10-ago-2026) pausar formalmente las fases de urea, metanol y terminal marina como condición para levantar el bloqueo; Secretaría de Economía sostuvo reuniones con comunidades de Ohuira, Paredones, Lázaro Cárdenas y Topolobampo presentando el "Plan Integral", pero las comunidades respondieron con desconfianza y mantienen el plantón indefinido)</t>
+          <t>Construcción parcial/PAUSA parcial (unidad de amoniaco ~95% completa según Presidencia, ago-2026 —prensa local cita 88% de avance—, aunque reportes locales previos citaban solo ~60% con obra detenida por bloqueo; movimiento indígena yoreme-mayo "¡Aquí No!" mantiene plantón bloqueando el acceso de personal a la obra desde el 7-jun-2026; GPO ofreció (8/10-ago-2026) pausar formalmente las fases de urea, metanol y terminal marina como condición para levantar el bloqueo; Secretaría de Economía sostuvo reuniones con comunidades de Ohuira, Paredones, Lázaro Cárdenas y Topolobampo presentando el "Plan Integral", pero las comunidades respondieron con desconfianza y mantienen el plantón indefinido)</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -1000,7 +994,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -2322,17 +2316,17 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Anuncio/Planeación (anunciado 17-ago-2026; tres nuevas plantas criogénicas con capacidad combinada ~825 MMcf/d, más nuevo gasoducto de ~70 millas "Bull Run II" hacia el hub de Waha; entrada en servicio prevista 1S2028)</t>
+          <t>Anuncio/Planeación (anunciado 17-ago-2026; tres nuevas plantas criogénicas con capacidad combinada ~825 MMcf/d, más nuevo gasoducto de ~70 millas "Bull Run II" hacia el hub de Waha; entrada en servicio prevista 1S2028; Targa evalúa además hasta 5 plantas adicionales en Permian Delaware a más largo plazo)</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>[EnergyNow](https://energynow.com/2026/08/targa-to-build-three-permian-gas-processing-plants-new-pipeline/)</t>
+          <t>[EnergyNow](https://energynow.com/2026/08/targa-to-build-three-permian-gas-processing-plants-new-pipeline/); [Targa Resources](https://www.targaresources.com/news-releases/news-release-details/targa-resources-corp-announces-20-year-agreements-exxonmobil-and)</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -2387,16 +2381,16 @@
   <dimension ref="A1:G44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proyecto</t>
@@ -2456,17 +2450,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Construcción (FERC aprobó inicio de construcción de Trenes 4 y 5 en mar-2026; gasoducto de alimentación Rio Bravo Pipeline —138 millas, JV Whitewater/MPLX/Enbridge— en camino a entrar en servicio 2S2026); Train 6 avanza a permitting formal (FERC inició scoping del EIS, solicitud presentada 26-may-2026, sesión de scoping virtual 19-ago-2026, FID prevista 2027; ~6.03 mtpa adicionales, llevando el sitio a 48 mtpa con Trenes 7-8)</t>
+          <t>Construcción (FERC aprobó inicio de construcción de Trenes 4 y 5 en mar-2026; gasoducto de alimentación Rio Bravo Pipeline —138 millas, JV Whitewater/MPLX/Enbridge— en camino a entrar en servicio 2S2026); Train 6 avanza a permitting formal (FERC inició scoping del EIS, solicitud presentada 26-may-2026, sesión de scoping virtual 19-ago-2026, FID prevista 2027; ~6.03 mtpa adicionales, llevando el sitio a 48 mtpa con Trenes 7-8); adicionalmente FERC publicó 19-ago-2026 el calendario de preparación de una Environmental Assessment para la "Rio Grande LNG Capacity Amendment", que alinearía la capacidad aprobada de Trenes 4-5 de 5.4 a ~6.03 mtpa por tren (27.0→~30.15 mtpa); EA programada 25-ago-2026, decisión final 23-nov-2026</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>[Bechtel](https://www.bechtel.com/press-releases/nextdecade-executes-epc-contract-with-bechtel-for-train-4-at-the-rio-grande-lng-facility/); [Natural Gas Intel](https://naturalgasintel.com/news/nextdecade-targets-more-than-36-mty-with-rio-grande-lng-upscale-sixth-train-expansion/); [Federal Register](https://www.federalregister.gov/documents/2026/08/03/2026-15695/rio-grande-lng-train-6-llc-notice-of-intent-to-prepare-an-environmental-impact-statement-for-the); [LNG Prime](https://lngprime.com/americas/nextdecade-seeks-ferc-ok-for-sixth-rio-grande-lng-train/187820/)</t>
+          <t>[Bechtel](https://www.bechtel.com/press-releases/nextdecade-executes-epc-contract-with-bechtel-for-train-4-at-the-rio-grande-lng-facility/); [Natural Gas Intel](https://naturalgasintel.com/news/nextdecade-targets-more-than-36-mty-with-rio-grande-lng-upscale-sixth-train-expansion/); [Federal Register - Capacity Amendment](https://www.federalregister.gov/documents/2026/08/19/2026-16922); [LNG Prime](https://lngprime.com/americas/nextdecade-seeks-ferc-ok-for-sixth-rio-grande-lng-train/187820/)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -2678,17 +2672,17 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Construcción (FERC autorizó introducción de gas combustible en Train 7, 17-jul-2026, y autorizó introducción de gas natural al Train 7, 28-jul-2026; FERC aprobó formalmente la introducción de gas natural al Train 7 —séptimo y último tren de la expansión midscale— el 4-ago-2026; primera producción de LNG esperada ago-2026, servicio comercial sep-2026; Trenes 5 y 6 completados mar/jun-2026; expansión completa de 7 trenes 85.4% de avance, prevista para fin de 2026)</t>
+          <t>Construcción (FERC autorizó introducción de gas combustible en Train 7, 17-jul-2026, y autorizó introducción de gas natural al Train 7, 28-jul-2026; FERC aprobó formalmente la introducción de gas natural al Train 7 —séptimo y último tren de la expansión midscale— el 4-ago-2026; Cheniere completó dos trenes adicionales de licuefacción en Stage 3 a mediados de ago-2026, elevando el avance del proyecto a ~98% completo; Train 7 en fase final de comisionamiento; finalización del build-out de 7 trenes prevista para fin de 2026)</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>[PGJ](https://pgjonline.com/news/2026/july/cheniere-gets-approval-to-introduce-gas-into-final-corpus-christi-lng-train); [LNG Prime](https://lngprime.com/americas/chenieres-corpus-christi-expansion-project-85-4-percent-complete/155448/); [energiesmedia](https://energiesmedia.com/ferc-approves-cheniere-train-7-energies/)</t>
+          <t>[PGJ](https://pgjonline.com/news/2026/july/cheniere-gets-approval-to-introduce-gas-into-final-corpus-christi-lng-train); [OGJ](https://www.ogj.com/pipelines-transportation/lng/news/55340460/cheniere-completes-two-more-corpus-christi-stage-3-trains); [LNG Prime](https://lngprime.com/americas/chenieres-corpus-christi-stage-3-project-98-percent-complete/190871/)</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -4035,19 +4029,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G90"/>
+  <dimension ref="A1:G91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proyecto</t>
@@ -4218,7 +4212,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Construcción (ingeniería de detalle &gt;95% completa, procura &gt;70% completa a may-2026; capex guía 2026 de US$1,300-1,600 millones; terminación mecánica prevista fines de 2027)</t>
+          <t>Construcción (reporte 2T2026: ingeniería de detalle &gt;95% completa, procura &gt;80% completa; US$1,800 millones de un capex total de US$2,930 millones ya incurridos; +1,600 trabajadores en sitio; comisionamiento anticipado de servicios previsto fines de 2026, terminación mecánica prevista fines de 2027)</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -4228,7 +4222,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -4403,17 +4397,17 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Construcción (tubería de pasta pendiente)</t>
+          <t>Construcción de la mina principal CONCLUIDA (alcanzó tasa de diseño de 7,500 tpd, 9 meses antes de lo previsto); Media Luna North en desarrollo (avance completado del "North Adit", iniciando instalación de ventilación e infraestructura; primera producción esperada fines de 2026)</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>[Minería en Línea](https://mineriaenlinea.com/2026/04/torex-gold-alcanza-velocidad-de-crucero-en-media-luna-9-meses-adelante-de-cronograma/)</t>
+          <t>[Minería en Línea](https://mineriaenlinea.com/2026/04/torex-gold-alcanza-velocidad-de-crucero-en-media-luna-9-meses-adelante-de-cronograma/); [Minería PA](https://mineria-pa.com/2026/08/11/mexico-media-luna-norte-proyecta-su-primera-produccion-para-fines-de-2026/)</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -4477,17 +4471,17 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Construcción (Record of Decision final emitido por USFS 7-jul-2026 para infraestructura en Coronado National Forest; ~50% avance en porción privada) / Permitting adicional para desarrollo completo (USFS publicó 15-ago-2026 el Draft EIS y Draft Record of Decision para el desarrollo completo de Hermosa, abriendo periodo de objeción de 45 días seguido de 45 días de resolución; decisión final esperada verano 2026; primer proyecto minero aceptado en programa federal FAST-41; primer concentrado proyectado H1-2028)</t>
+          <t>Construcción (Record of Decision final emitido por USFS 7-jul-2026 para infraestructura en Coronado National Forest; ~50% avance en porción privada) / Permitting adicional para desarrollo completo (USFS publicó 15-ago-2026 el Draft EIS y Draft Record of Decision para el desarrollo completo de Hermosa, abriendo periodo de objeción de 45 días seguido de 45 días de resolución; decisión final esperada verano 2026; primer proyecto minero aceptado en programa federal FAST-41; primer concentrado proyectado H1-2028); South32 aumentó el capex de Taylor en ~US$1,100 millones (total ~US$3,300 millones) y retrasó la primera producción de mediados de 2027 a mediados de 2028 (capacidad plena ahora en FY2031), aunque Ore Reserves aumentaron +52% y la vida de mina se extendió a ~33 años</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>[USDA](https://www.usda.gov/about-usda/news/press-releases/2026/07/07/usda-advances-trump-administration-effort-boost-us-mineral-energy-production); [Tucson Sentinel](https://www.tucsonsentinel.com/local/report/030626_hermosa_mine_review/hermosa-mine-hits-milestone-after-forest-service-releases-enviro-review/)</t>
+          <t>[USDA](https://www.usda.gov/about-usda/news/press-releases/2026/07/07/usda-advances-trump-administration-effort-boost-us-mineral-energy-production); [Tucson Sentinel](https://www.tucsonsentinel.com/local/report/030626_hermosa_mine_review/hermosa-mine-hits-milestone-after-forest-service-releases-enviro-review/); [TipRanks](https://www.tipranks.com/news/company-announcements/south32-lifts-hermosa-taylor-mine-life-capex-and-delays-ramp-up-to-fy31)</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -4514,17 +4508,17 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Construcción (corte federal de Idaho negó en jun-2026 moción para detener obras; Export-Import Bank de EE.UU. aprobó en may-2026 préstamo garantizado de USD 2,900 millones, desembolso esperado 2S2026; nuevos objetivos de exploración de oro/antimonio de alta ley identificados y posible nueva fuente de tungsteno reportados 7-ago-2026)</t>
+          <t>Construcción (corte federal de Idaho negó en jun-2026 moción para detener obras; Directorio del Export-Import Bank de EE.UU. aprobó por unanimidad, 20-ago-2026, el préstamo garantizado senior de USD 2,900 millones para financiar el desarrollo; nuevos objetivos de exploración de oro/antimonio de alta ley identificados y posible nueva fuente de tungsteno reportados 7-ago-2026)</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/perpetua-resources-advances-construction-of-the-stibnite-gold-project-302787012.html); [Departamento de Justicia de EE.UU.](https://www.justice.gov/opa/pr/justice-department-secures-motion-allow-continued-construction-idaho-gold-mine-critical); [StreetWise Reports](https://www.streetwisereports.com/article/2026/08/10/idaho-gold-antimony-project-hits-high-grade-intercepts-at-stibnite.html)</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/perpetua-resources-advances-construction-of-the-stibnite-gold-project-302787012.html); [Departamento de Justicia de EE.UU.](https://www.justice.gov/opa/pr/justice-department-secures-motion-allow-continued-construction-idaho-gold-mine-critical); [StreetWise Reports](https://www.streetwisereports.com/article/2026/08/20/idaho-gold-antimony-developer-wins-2-9b-exim-loan-approval.html)</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -4699,17 +4693,17 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Permiso de Emplazamiento Industrial (Industrial Siting Permit) otorgado por Wyoming DEQ el 20-jun-2026, habilitando construcción y operación sin requerir NEPA (no involucra tierra federal); construcción pesada prevista hasta 2027, producción 2028</t>
+          <t>Permiso de Emplazamiento Industrial (Industrial Siting Permit) otorgado por Wyoming DEQ el 20-jun-2026, habilitando construcción y operación sin requerir NEPA (no involucra tierra federal); U.S. Gold Corp completó el permitting estatal —proyecto "totalmente permisado"—, lo que disparó interés estratégico de proveedores de capital y posible M&amp;A, reportado 20-ago-2026; construcción pesada prevista hasta 2027, producción 2028</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>[Wyoming News](https://www.wyomingnews.com/rawlinstimes/plans-move-forward-for-ck-gold-project-as-developers-target-2026-construction-start/article_b2bb147e-2f92-4ca2-bf86-fcc9983917a7.html); [Discovery Alert](https://discoveryalert.com.au/ck-gold-project-permitting-construction-ready-valuation-2026/)</t>
+          <t>[Wyoming News](https://www.wyomingnews.com/rawlinstimes/plans-move-forward-for-ck-gold-project-as-developers-target-2026-construction-start/article_b2bb147e-2f92-4ca2-bf86-fcc9983917a7.html); [Crux Investor](https://www.cruxinvestor.com/posts/us-gold-corp-evaluates-m-a-interest-as-ck-gold-project-advances)</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -4773,17 +4767,17 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Construcción (comisionamiento previsto Q4 2026)</t>
+          <t>Construcción SUSTANCIALMENTE COMPLETA en sitio Wardner; comisionamiento esperado dentro de las semanas siguientes al 31-jul-2026 (antes Q4 2026)</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>[SEC/Americas Gold and Silver](https://www.sec.gov/Archives/edgar/data/0001286973/000106299326002645/exhibit99-2.htm)</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/31/3337077/0/en/bunker-hill-ships-first-concentrate-to-trail-smelter-and-announces-drawdown-of-standby-facility.html)</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -4879,12 +4873,12 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Cominvi (contratista minero mexicano seleccionado); M3 Mexicana (diseño de planta, 55% completo)</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Construcción aprobada por el consejo (permisos SEMARNAT completos jun-2026; presupuesto ~US$227 millones; ventana de construcción de ~24 meses; primer vertido de metal previsto mediados de 2028)</t>
+          <t>Construcción aprobada por el consejo (permisos SEMARNAT completos jun-2026; presupuesto ~US$227 millones; ventana de construcción de ~24 meses; planta SART 70% completa; primer vertido de metal previsto mediados de 2028)</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -4894,7 +4888,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -6475,17 +6469,17 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Producción (autorización final del estado de Wyoming para operar a plena producción, reportada 10-ago-2026; planta satélite ISR integrada con Lost Creek; infraestructura de planta y transporte ya en sitio)</t>
+          <t>Producción (autorización final del estado de Wyoming para operar a plena producción, reportada 10-ago-2026; Ur-Energy realizó su PRIMER EMBARQUE de uranio desde la mina hacia la planta de procesamiento Lost Creek, 19-ago-2026 —transición de construcción a producción en 2.5 años—; planta satélite ISR integrada con Lost Creek)</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>[Ur-Energy](https://www.ur-energy.com/news-media/press-releases/detail/401/ur-energy-commences-operations-at-its-shirley-basin-isr); [Junior Mining Network](https://www.juniorminingnetwork.com/junior-miner-news/press-releases/557-tsx/ure/208831-ur-energy-reports-second-quarter-2026-results.html)</t>
+          <t>[Ur-Energy](https://www.ur-energy.com/news-media/press-releases/detail/410/ur-energy-announces-first-shipment-of-uranium-from-shirley); [Junior Mining Network](https://www.juniorminingnetwork.com/junior-miner-news/press-releases/557-tsx/ure/208831-ur-energy-reports-second-quarter-2026-results.html)</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -7374,6 +7368,43 @@
       <c r="G90" s="2" t="inlineStr">
         <is>
           <t>2026-08-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>La Preciosa Project</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>Durango, México</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>Avino Silver &amp; Gold Mines Ltd.</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>Construcción (desarrollo subterráneo en curso —rampa/decline de 360m—; permisos mineros ya obtenidos; producción objetivo 4T2026)</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>[AccessWire](https://www.accessnewswire.com/newsroom/en/metals-and-mining/avino-provides-update-on-its-100-owned-la-preciosa-property-preparing-for-producti-837173); [MarketScreener](https://www.marketscreener.com/quote/stock/AVINO-SILVER-GOLD-MINES-L-1409069/news/Avino-Silver-Gold-Mines-Ltd-Commences-Underground-Development-At-La-Preciosa-48766238/)</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -7388,19 +7419,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G86"/>
+  <dimension ref="A1:G89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proyecto</t>
@@ -8084,22 +8115,22 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Stream Data Centers (JV vía LOI); Thunderhead Energy Solutions (~250MW de gen. de gas behind-the-meter)</t>
+          <t>Stream Data Centers (JV vía LOI); Thunderhead Energy Solutions (gen. de gas behind-the-meter)</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Permisos de construcción obtenidos (New Era Energy &amp; Digital anunció 14-ago-2026, junto con su reporte 10-Q 2T2026, que ya cuenta con los permisos de construcción para TCDC; sitio escalable hacia 1.4GW; construcción total prevista en 2026, primeros 100MW dic-2026)</t>
+          <t>Permisos de construcción obtenidos (New Era Energy &amp; Digital anunció 14-ago-2026, junto con su reporte 10-Q 2T2026, que ya cuenta con los permisos de construcción para TCDC; sitio escalable hacia 1.4GW; New Era aseguró permisos clave adicionales —Development Structure Permit, Drive Approach Permit— y presentó Notice of Intent ante TCEQ para nivelación de terreno, 17-ago-2026; capacidad combinada Fase 1+2 aumentó de ~650MW a 757MW vía nuevo permiso de aire TCEQ de Thunderhead (Fase 2: 450→550MW); construcción total prevista en 2026, primeros 100MW dic-2026)</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55289667/powering-ai-in-the-permian-texas-critical-data-centers-sustainable-energy-play); [GlobeNewswire](https://www.globenewswire.com/news-release/2026/08/14/3345632/0/en/new-era-energy-digital-files-q2-2026-form-10-q-and-announces-tcdc-construction-permits.html)</t>
+          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55289667/powering-ai-in-the-permian-texas-critical-data-centers-sustainable-energy-play); [GlobeNewswire](https://www.globenewswire.com/news-release/2026/08/14/3345632/0/en/new-era-energy-digital-files-q2-2026-form-10-q-and-announces-tcdc-construction-permits.html); [Minichart](https://www.minichart.com.sg/2026/08/17/new-era-energy-secures-construction-permits-for-texas-data-center-campus/)</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -9596,7 +9627,7 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Anthropic (operado por Nexus Data Centers; respaldo financiero de Google)</t>
+          <t>Anthropic (confirmado como tenant ancla tras proceso de licitación competitivo; operado por Nexus Data Centers; respaldo financiero de Google)</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
@@ -9606,17 +9637,17 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Construcción iniciada (primera fase 500-612MW prevista 2026, ampliable a ~7.2-7.7GW; planta de gas natural behind-the-meter cerca de gasoducto principal; financiamiento avanzado: banca liderada por Morgan Stanley en negociaciones finales para prestar USD 15 mil millones a Nexus Data Centers —incluye préstamo puente de USD 14 mil millones más línea de crédito revolvente—; Google otorgaría garantías sobre obligaciones de arrendamiento y pago de energía de Anthropic a cambio de ~20% de participación accionaria en el proyecto combinado)</t>
+          <t>Construcción iniciada (primera fase 500-612MW prevista 2026, ampliable a ~7.2-7.7GW; planta de gas natural behind-the-meter cerca de gasoducto principal; permisos de primera fase cubren ~491,000 pies² de cómputo de alta densidad; Eagle Point Credit Management lidera un préstamo de crédito privado mezzanine de USD 1,300 millones, parte de un paquete de financiamiento de ~USD 16,000 millones, 19-ago-2026; Google garantiza la deuda senior)</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/600mw-natural-gas-powered-data-center-campus-proposed-in-hubbard-texas/); [Construction Review](https://constructionreviewonline.com/5bn-anthropic-data-center-in-texas-receives-critical-financial-backing-from-google/); [CNBC](https://www.cnbc.com/2026/07/30/nexus-data-centers-in-advanced-talks-to-secure-15b-for-google-backed-anthropic-data-center.html)</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/600mw-natural-gas-powered-data-center-campus-proposed-in-hubbard-texas/); [Construction Review](https://constructionreviewonline.com/5bn-anthropic-data-center-in-texas-receives-critical-financial-backing-from-google/); [Private Equity Wire](https://www.privateequitywire.co.uk/eagle-point-leads-1-3bn-private-credit-loan-for-anthropic-linked-texas-data-centre/)</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
@@ -10579,6 +10610,117 @@
       <c r="G86" s="2" t="inlineStr">
         <is>
           <t>2026-08-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>KIO Data Centers — Expansión QRO3</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>El Marqués, Querétaro, México</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>KIO Data Centers</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>Anuncio de inversión (~US$1,300 millones, ~100MW adicionales, ~8,100 empleos proyectados)</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>[CódigoQro](https://codigoqro.mx/nota/local/2026/08/13/invertira-empresa-mexicana-mil-300-mdd-ampliacion-tercer-centro-datos-queretaro)</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>Prometheus Hyperscale "Pecos Project" (con Istmo Energy)</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>Reeves County, Texas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>Prometheus Hyperscale / Istmo Energy (JV)</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>Anuncio de desarrollo (hasta 2.5GW, dual-fuel —gas natural + metano de planta de fraccionamiento de Istmo Midstream—; primera energía prevista 2027)</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>[Data Center Dynamics](https://www.datacenterdynamics.com/en/news/prometheus-hyperscale-partners-with-istmo-to-develop-up-to-25gw-gas-powered-data-center-in-reeves-county-texas/)</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>Riot Platforms — Campus Rockdale (Anthropic)</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>Rockdale, Texas, EE.UU. (antigua planta de Alcoa)</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>Anthropic (tenant ancla) / Riot Platforms (desarrollador-operador)</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>Contrato de arrendamiento firmado (20 años, 191MW, ~US$9,100 millones; financiamiento interino de construcción de US$573 millones vía Morgan Stanley; primera fase de 96MW prevista dic-2027)</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>[Austin American-Statesman](https://www.statesman.com/business/technology/article/anthropic-riot-platforms-rockdale-texas-22383624.php); [Bloomberg](https://www.bloomberg.com/news/articles/2026-08-11/anthropic-strikes-9-billion-deal-with-cloud-computing-firm-riot)</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitoreo 2026-08-25: 5 proyectos nuevos + 1 actualización de fase
Nuevos: Great Salt Lake Lithium Facility, Project SHIELD (Nth Cycle),
Refinería de Sulfato de Cobalto (Formation Holdings/Jervois), Schlachter
Realty Data Center Power Station, Meitner Energy Center.
Actualización: Woodside Louisiana LNG (28% de avance de construcción).
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,21 +29,22 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Arial"/>
       <b val="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="10"/>
+      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F2937"/>
+        <bgColor rgb="001F2937"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -60,10 +61,10 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -434,13 +435,13 @@
   <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2381,13 +2382,13 @@
   <dimension ref="A1:G44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2524,17 +2525,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Construcción</t>
+          <t>Construcción (28% de avance global reportado ago-2026: Tren 1 35%, Tren 2 25%, Tren 3 18%; acero estructural erigido en Trenes 1 y 2, avance de pilotes de concreto en Tren 3; proyecto de US$17,500 millones dentro de presupuesto; primer cargamento previsto 2029)</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>[Woodside](https://www.woodside.com/what-we-do/growth-projects/woodside-louisiana-lng)</t>
+          <t>[Ocean News](https://oceannews.com/news/energy/drone-footage-captures-louisiana-lng-construction-progress-at-28-percent/); [Natural Gas Intel](https://naturalgasintel.com/news/woodside-reports-strong-construction-progress-at-165-mty-louisiana-lng-terminal/)</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-08-25</t>
         </is>
       </c>
     </row>
@@ -4029,16 +4030,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G91"/>
+  <dimension ref="A1:G94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7405,6 +7406,117 @@
       <c r="G91" s="2" t="inlineStr">
         <is>
           <t>2026-08-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>Great Salt Lake Lithium Facility</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>Condado de Box Elder, Utah, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>Lilac Solutions (subsidiaria Waterleaf P1 HoldCo)</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>Hatch (EPCM, seleccionado jun-2026)</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>Desarrollo/Ingeniería (DOE anunció 20/21-ago-2026 subvención de hasta US$100 millones para construir planta comercial de extracción/refinación de litio por intercambio iónico directo desde salmuera del Great Salt Lake, 5,000 t/año; primera producción prevista 2028)</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>[KSL](https://www.ksl.com/article/51614351/california-company-awarded-100m-to-develop-critical-mineral-facility-on-great-salt-lake-shore); [Hatch](https://www.hatch.com/About-Us/News-And-Media/2026/06/Lilac-Solutions-Selects-Hatch-as-EPCM-Partner-for-Great-Salt-Lake-Lithium-Facility)</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>Project SHIELD (refinería de "black mass" de baterías)</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>Carolina del Sur, EE.UU. (sitio exacto por definir)</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>Nth Cycle, Inc.</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>Negociación de subvención/preconstrucción (DOE seleccionó a Nth Cycle 20/21-ago-2026 para negociar premio de hasta US$100 millones; planta de refinación de "black mass" de baterías de litio, producirá MHP de níquel y carbonato de litio grado batería, 24,000 t/año; operación proyectada 2028)</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>[Nth Cycle](https://nthcycle.com/newsroom/u.s.-department-of-energy-selects-nth-cycle-to-enter-award-negotiations-for-up-to-100-million-to-build-new-critical-mineral-refining-facility)</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>Refinería de Sulfato de Cobalto — Formation Holdings/Jervois</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>Sitio por definir, EE.UU. (empresa con sede en Salmon, Idaho)</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>Formation Holdings US, Inc. (dba Jervois)</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>Desarrollo/financiamiento (DOE otorgó 21-ago-2026 subvención de US$100 millones para construir refinería comercial de sulfato de cobalto grado batería; ubicación específica de la planta aún no anunciada)</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>[Local News 8](https://localnews8.com/news/business-watch/2026/08/21/salmon-company-wins-100-million-grant-to-build-cobalt-refinery/); [Local News 8 (seguimiento)](https://localnews8.com/news/local-news/2026/08/24/100m-grant-to-salmon-based-jervois-could-jumpstart-idahos-cobalt-industry/)</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
         </is>
       </c>
     </row>
@@ -7419,16 +7531,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G89"/>
+  <dimension ref="A1:G91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -10724,6 +10836,80 @@
         </is>
       </c>
     </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>Schlachter Realty Data Center Power Station</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>Al sur de Dallas, Texas, EE.UU. (condado exacto no confirmado)</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>Schlachter Realty (solicitante del permiso; operador final del data center no identificado)</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>Permitting (solicitud de permiso de aire ante TCEQ para instalar 891 generadores reciprocantes Caterpillar 3516E a gas, complejo de generación dedicado a data center; uno de 74+ proyectos de plantas de gas ≥100MW para data centers identificados a nivel nacional, 32 en Texas)</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>[Inside Climate News](https://insideclimatenews.org/news/25082026/texas-data-center-gas-projects/)</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>Meitner Energy Center</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>Condados de Gray y Roberts, Texas Panhandle, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>Google (en sociedad con Intersect Power)</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>Intersect Power (desarrollador/operador de generación)</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>Construcción (groundbreaking; complejo &gt;1GW combinando eólica, solar, almacenamiento en batería y generación a gas natural on-site para respaldo/firming; inversión reportada ~US$14,000 millones; ~840 MW de capacidad de data center)</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>[Intersect Power](https://www.intersect.com/news/google-and-intersect-deepen-texas-roots-with-new-data-center-and-energy-investments-in-gray-and-roberts-counties)</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Monitoreo 2026-08-25: 5 proyectos nuevos + 1 actualización de fase (#30)
Nuevos: Great Salt Lake Lithium Facility, Project SHIELD (Nth Cycle),
Refinería de Sulfato de Cobalto (Formation Holdings/Jervois), Schlachter
Realty Data Center Power Station, Meitner Energy Center.
Actualización: Woodside Louisiana LNG (28% de avance de construcción).

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,21 +29,22 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Arial"/>
       <b val="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="10"/>
+      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F2937"/>
+        <bgColor rgb="001F2937"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -60,10 +61,10 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -434,13 +435,13 @@
   <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2381,13 +2382,13 @@
   <dimension ref="A1:G44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2524,17 +2525,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Construcción</t>
+          <t>Construcción (28% de avance global reportado ago-2026: Tren 1 35%, Tren 2 25%, Tren 3 18%; acero estructural erigido en Trenes 1 y 2, avance de pilotes de concreto en Tren 3; proyecto de US$17,500 millones dentro de presupuesto; primer cargamento previsto 2029)</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>[Woodside](https://www.woodside.com/what-we-do/growth-projects/woodside-louisiana-lng)</t>
+          <t>[Ocean News](https://oceannews.com/news/energy/drone-footage-captures-louisiana-lng-construction-progress-at-28-percent/); [Natural Gas Intel](https://naturalgasintel.com/news/woodside-reports-strong-construction-progress-at-165-mty-louisiana-lng-terminal/)</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-08-25</t>
         </is>
       </c>
     </row>
@@ -4029,16 +4030,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G91"/>
+  <dimension ref="A1:G94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7405,6 +7406,117 @@
       <c r="G91" s="2" t="inlineStr">
         <is>
           <t>2026-08-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>Great Salt Lake Lithium Facility</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>Condado de Box Elder, Utah, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>Lilac Solutions (subsidiaria Waterleaf P1 HoldCo)</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>Hatch (EPCM, seleccionado jun-2026)</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>Desarrollo/Ingeniería (DOE anunció 20/21-ago-2026 subvención de hasta US$100 millones para construir planta comercial de extracción/refinación de litio por intercambio iónico directo desde salmuera del Great Salt Lake, 5,000 t/año; primera producción prevista 2028)</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>[KSL](https://www.ksl.com/article/51614351/california-company-awarded-100m-to-develop-critical-mineral-facility-on-great-salt-lake-shore); [Hatch](https://www.hatch.com/About-Us/News-And-Media/2026/06/Lilac-Solutions-Selects-Hatch-as-EPCM-Partner-for-Great-Salt-Lake-Lithium-Facility)</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>Project SHIELD (refinería de "black mass" de baterías)</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>Carolina del Sur, EE.UU. (sitio exacto por definir)</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>Nth Cycle, Inc.</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>Negociación de subvención/preconstrucción (DOE seleccionó a Nth Cycle 20/21-ago-2026 para negociar premio de hasta US$100 millones; planta de refinación de "black mass" de baterías de litio, producirá MHP de níquel y carbonato de litio grado batería, 24,000 t/año; operación proyectada 2028)</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>[Nth Cycle](https://nthcycle.com/newsroom/u.s.-department-of-energy-selects-nth-cycle-to-enter-award-negotiations-for-up-to-100-million-to-build-new-critical-mineral-refining-facility)</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>Refinería de Sulfato de Cobalto — Formation Holdings/Jervois</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>Sitio por definir, EE.UU. (empresa con sede en Salmon, Idaho)</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>Formation Holdings US, Inc. (dba Jervois)</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>Desarrollo/financiamiento (DOE otorgó 21-ago-2026 subvención de US$100 millones para construir refinería comercial de sulfato de cobalto grado batería; ubicación específica de la planta aún no anunciada)</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>[Local News 8](https://localnews8.com/news/business-watch/2026/08/21/salmon-company-wins-100-million-grant-to-build-cobalt-refinery/); [Local News 8 (seguimiento)](https://localnews8.com/news/local-news/2026/08/24/100m-grant-to-salmon-based-jervois-could-jumpstart-idahos-cobalt-industry/)</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
         </is>
       </c>
     </row>
@@ -7419,16 +7531,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G89"/>
+  <dimension ref="A1:G91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -10724,6 +10836,80 @@
         </is>
       </c>
     </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>Schlachter Realty Data Center Power Station</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>Al sur de Dallas, Texas, EE.UU. (condado exacto no confirmado)</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>Schlachter Realty (solicitante del permiso; operador final del data center no identificado)</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>Permitting (solicitud de permiso de aire ante TCEQ para instalar 891 generadores reciprocantes Caterpillar 3516E a gas, complejo de generación dedicado a data center; uno de 74+ proyectos de plantas de gas ≥100MW para data centers identificados a nivel nacional, 32 en Texas)</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>[Inside Climate News](https://insideclimatenews.org/news/25082026/texas-data-center-gas-projects/)</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>Meitner Energy Center</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>Condados de Gray y Roberts, Texas Panhandle, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>Google (en sociedad con Intersect Power)</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>Intersect Power (desarrollador/operador de generación)</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>Construcción (groundbreaking; complejo &gt;1GW combinando eólica, solar, almacenamiento en batería y generación a gas natural on-site para respaldo/firming; inversión reportada ~US$14,000 millones; ~840 MW de capacidad de data center)</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>[Intersect Power](https://www.intersect.com/news/google-and-intersect-deepen-texas-roots-with-new-data-center-and-energy-investments-in-gray-and-roberts-counties)</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Monitoreo 2026-08-27: 9 proyectos nuevos + 33 actualizaciones de fase
Petroquímica: LSB Industries El Dorado, Yara/Enbridge Ingleside.
Mining: Korea Zinc/Nyrstar smelter, Aclara heavy rare earths, Archimedes
(i-80 Gold), Sweetwater Uranium ISR, Velvet-Wood uranium-vanadium.
Data Centers: Nscale Monarch Compute Campus, Dominion Chesterfield ERC.

Actualizaciones de fase en proyectos ya rastreados de petroquímica (2),
mining (14) y data centers (15): FIDs, permisos, contratos EPC y avances
de construcción confirmados 23-27 ago 2026.
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Petroquímica" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Petroquimica" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="LNG" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Mining" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Data Centers" sheetId="4" state="visible" r:id="rId4"/>
@@ -20,10 +20,18 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
@@ -49,8 +57,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -416,50 +425,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G53"/>
+  <dimension ref="A1:G55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -525,17 +534,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Construcción (Luisiana y el U.S. Army Corps of Engineers emitieron en jul-2026 los permisos de construcción civil necesarios; CF Industries confirmó en su reporte 2T2026 —8-K, 5-ago-2026— el inicio de construcción en ago-2026 de la planta de amoniaco bajo carbono, ~708,000-1.4 MTPA, ~US$3.7-4,000 millones; producción prevista 2029)</t>
+          <t>Construcción (Luisiana y el U.S. Army Corps of Engineers emitieron en jul-2026 los permisos de construcción civil necesarios; CF Industries confirmó en su reporte 2T2026 —8-K, 5-ago-2026— el inicio de construcción en ago-2026 de la planta de amoniaco bajo carbono, ~708,000-1.4 MTPA, ~US$3.7-4,000 millones; producción prevista 2029) ; groundbreaking formal el 26-ago-2026 con la Secretaria de Agricultura de EE.UU., Brooke Rollins, confirmando el inicio físico de construcción</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>[FuelCellsWorks](https://fuelcellsworks.com/2026/08/06/clean-energy/cf-industries-to-begin-construction-of-3-7bn-louisiana-blue-ammonia-plant); [gasworld](https://www.gasworld.com/story/cf-industries-to-begin-construction-of-4bn-louisiana-blue-ammonia-project/2256572.article/)</t>
+          <t>[FuelCellsWorks](https://fuelcellsworks.com/2026/08/06/clean-energy/cf-industries-to-begin-construction-of-3-7bn-louisiana-blue-ammonia-plant); [gasworld](https://www.gasworld.com/story/cf-industries-to-begin-construction-of-4bn-louisiana-blue-ammonia-project/2256572.article/) ; [Brownfield Ag News](https://www.brownfieldagnews.com/news/blue-point-ammonia-plant-groundbreaking-marks-step-toward-more-u-s-fertilizer-supply/)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -599,17 +608,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Construcción (comisionamiento)</t>
+          <t>Construcción (comisionamiento) ; arranque ahora esperado en 2027 (retrasado al menos 6 meses respecto a 2026), según East Daley Analytics, por menor demanda de etano proyectada</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>[BIC Magazine](https://www.bicmagazine.com/departments/operations/cpchem-golden-triangle-polymers-facility-startup-phase/)</t>
+          <t>[BIC Magazine](https://www.bicmagazine.com/departments/operations/cpchem-golden-triangle-polymers-facility-startup-phase/) ; [East Daley](https://eastdaley.com/daley-note/back-a-frac-supply-growth-creates-next-ngl-bottleneck-2)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -2386,6 +2395,80 @@
       <c r="G53" t="inlineStr">
         <is>
           <t>2026-08-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>LSB Industries — Expansión de Amoniaco El Dorado</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>El Dorado, Arkansas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>LSB Industries</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Pre-FID (decisión final de inversión proyectada para 2T2027; expansión de 100,000 toneladas/año incrementales de amoniaco, costo neto US$105-120 millones, bruto US$135-150 millones incluyendo infraestructura)</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>[The Motley Fool](https://www.fool.com/earnings/call-transcripts/2026/08/07/lsb-industries-lxu-q2-2026-earnings-call-transcript/)</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Yara/Enbridge — Amoniaco Azul Ingleside</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Enbridge Ingleside Energy Center, cerca de Corpus Christi, Texas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Yara Clean Ammonia / Enbridge (JV 50/50)</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Ingeniería (FEED en curso, pendiente FID; capacidad 1.2-1.4 MMTPA, inversión estimada US$2,600-2,900 millones; reforming autotérmico con captura de CO2 ~95%; enfrenta oposición comunitaria activa)</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>[QC Intel](https://www.qcintel.com/ammonia/article/yara-enbridge-continue-ingleside-blue-ammonia-plans-despite-pushback-28727.html)</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -2403,47 +2486,47 @@
   <dimension ref="A1:G46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -4125,50 +4208,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G102"/>
+  <dimension ref="A1:G107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -4197,17 +4280,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Construcción (PFS define mina subterránea de 20,000 t/d y planta de cátodos de 72,000 t/año; EXIM Bank gestiona más de US$1,000 millones en financiamiento, como parte del paquete federal de US$3,000 millones en minerales críticos anunciado 7-8-ago-2026; Ivanhoe completó el pago final de adquisición de terreno —US$39.3 millones— satisfaciendo el acuerdo de compraventa, y cerró una línea de crédito bancario de US$200 millones para financiar el inicio de actividades mayores de construcción en 2026; primera producción de cobre prevista 2028)</t>
+          <t>Construcción (PFS define mina subterránea de 20,000 t/d y planta de cátodos de 72,000 t/año; EXIM Bank gestiona más de US$1,000 millones en financiamiento, como parte del paquete federal de US$3,000 millones en minerales críticos anunciado 7-8-ago-2026; Ivanhoe completó el pago final de adquisición de terreno —US$39.3 millones— satisfaciendo el acuerdo de compraventa, y cerró una línea de crédito bancario de US$200 millones para financiar el inicio de actividades mayores de construcción en 2026; primera producción de cobre prevista 2028) ; ciudad de Casa Grande aprobó el Site Development Plan (mar-2026); Ivanhoe Electric adquirió tuneladora (TBM) Robbins; excavación del box-cut programada para 3T2026</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>[Mining Weekly](https://www.miningweekly.com/article/ivanhoe-electric-pencils-in-2026-construction-start-at-arizona-copper-mine-2025-06-25); [Ivanhoe Electric](https://ivanhoeelectric.com/news/ivanhoe-electric-makes-final-land-acquisition-payment-at-the-santa-cruz-copper-project-in-arizona/)</t>
+          <t>[Mining Weekly](https://www.miningweekly.com/article/ivanhoe-electric-pencils-in-2026-construction-start-at-arizona-copper-mine-2025-06-25); [Ivanhoe Electric](https://ivanhoeelectric.com/news/ivanhoe-electric-makes-final-land-acquisition-payment-at-the-santa-cruz-copper-project-in-arizona/) ; [Mining Technology](https://www.mining-technology.com/news/ivanhoe-electric-to-buy-tbm-arizona-project/)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -4234,7 +4317,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Ingeniería/Feasibility (DFS &gt;85% completo; colocación de bonos municipales por US$52 millones completada 24-jun-2026 para financiar el proyecto, ya totalmente permisado para iniciar construcción)</t>
+          <t>Ingeniería/Feasibility (DFS &gt;85% completo; colocación de bonos municipales por US$52 millones completada 24-jun-2026 para financiar el proyecto, ya totalmente permisado para iniciar construcción) ; bajo Hudbay Minerals (tras adquisición de Arizona Sonoran Copper, jun-2026), definitive feasibility study previsto para mediados de 2026, con FID esperada después en 2026</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -4244,7 +4327,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -4271,17 +4354,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Ingeniería temprana post intercambio de tierras (marzo 2026); firmó Master Supply Agreement (1-jul-2026) con Johnson Controls Inc. y UA Local 469; otorgó ~US$110 millones en contratos a Major Drilling America Inc. y Redpath USA Corporation (10-ago-2026) para acelerar exploración y desarrollo subterráneo, parte de programa de inversión de ~US$500 millones</t>
+          <t>Ingeniería temprana post intercambio de tierras (marzo 2026); firmó Master Supply Agreement (1-jul-2026) con Johnson Controls Inc. y UA Local 469; otorgó ~US$110 millones en contratos a Major Drilling America Inc. y Redpath USA Corporation (10-ago-2026) para acelerar exploración y desarrollo subterráneo, parte de programa de inversión de ~US$500 millones ; otorgó contratos por ~US$110 millones a Major Drilling America y Redpath USA Corporation para avanzar exploración y desarrollo subterráneo</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>[SEC](https://www.sec.gov/Archives/edgar/data/863064/000086306426000019/ex12d16mr_resolutionland.htm); [International Mining](https://im-mining.com/2026/08/10/resolution-copper-accelerates-exploration-underground-development-with-major-drilling-redpath-contracts/)</t>
+          <t>[SEC](https://www.sec.gov/Archives/edgar/data/863064/000086306426000019/ex12d16mr_resolutionland.htm); [International Mining](https://im-mining.com/2026/08/10/resolution-copper-accelerates-exploration-underground-development-with-major-drilling-redpath-contracts/) ; [Mining Technology](https://www.mining-technology.com/news/resolution-copper-110m-contracts-arizona-mine-2/)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -4308,17 +4391,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Construcción (reporte 2T2026: ingeniería de detalle &gt;95% completa, procura &gt;80% completa; US$1,800 millones de un capex total de US$2,930 millones ya incurridos; +1,600 trabajadores en sitio; comisionamiento anticipado de servicios previsto fines de 2026, terminación mecánica prevista fines de 2027)</t>
+          <t>Construcción (reporte 2T2026: ingeniería de detalle &gt;95% completa, procura &gt;80% completa; US$1,800 millones de un capex total de US$2,930 millones ya incurridos; +1,600 trabajadores en sitio; comisionamiento anticipado de servicios previsto fines de 2026, terminación mecánica prevista fines de 2027) ; DOE aprobó préstamo de US$2,260 millones; ingeniería detallada 93% completa y procura 60% completa (fin de 2025); concreto principal del sitio se completaría en 3T2026, con comisionamiento inicial de plantas individuales desde 4T2026</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>[Mining Weekly](https://www.miningweekly.com/article/thacker-pass-lithium-project-us-update-2026-05-22); [Lithium Americas](https://lithiumamericas.com/news/news-details/2026/Lithium-Americas-Provides-a-Project-Update-and-2026-Capex-Guidance-for-Thacker-Pass/default.aspx)</t>
+          <t>[Mining Weekly](https://www.miningweekly.com/article/thacker-pass-lithium-project-us-update-2026-05-22); [Lithium Americas](https://lithiumamericas.com/news/news-details/2026/Lithium-Americas-Provides-a-Project-Update-and-2026-Capex-Guidance-for-Thacker-Pass/default.aspx) ; [Carbon Credits](https://carboncredits.com/u-s-doe-approves-2-26-billion-for-nevada-lithium-mine/)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -4345,17 +4428,17 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Construcción, producción esperada 2026</t>
+          <t>Construcción, producción esperada 2026 ; backlog de permisos en Zacatecas bajó de 25 a 5 según CAMIMEX; de continuar el ritmo de destrabe regulatorio, el proyecto podría iniciar construcción antes de finalizar 2026</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>[Mining.com](https://www.mining.com/teck-agnico-team-up-at-san-nicolas-copper-project-in-mexico/)</t>
+          <t>[Mining.com](https://www.mining.com/teck-agnico-team-up-at-san-nicolas-copper-project-in-mexico/) ; [Minería en Línea](https://mineriaenlinea.com/2026/08/inversion-minera-en-mexico-creceria-30-en-2026-segun-camimex/)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4502,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Permisos ambientales asegurados (MIA aprobada ~28-jul-2026, destrabando obras preliminares de sitio —líneas de transmisión, acueducto, caminos de acceso, campamento— programadas sep-dic 2026; construcción completa desde 1T2027; primera producción de cátodos de cobre en 2S2029; inversión US$551 millones; capacidad 36,000 t/año de cátodos; reservas probadas/probables de 317 Mt a 0.249% Cu)</t>
+          <t>Permisos ambientales asegurados (MIA aprobada ~28-jul-2026, destrabando obras preliminares de sitio —líneas de transmisión, acueducto, caminos de acceso, campamento— programadas sep-dic 2026; construcción completa desde 1T2027; primera producción de cátodos de cobre en 2S2029; inversión US$551 millones; capacidad 36,000 t/año de cátodos; reservas probadas/probables de 317 Mt a 0.249% Cu) ; Southern Copper obtuvo los permisos ambientales necesarios; trabajos preliminares de sitio inician sep-2026, con construcción del proyecto arrancando en 1T2027</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -4429,7 +4512,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -4641,17 +4724,17 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Construcción (166 personas en sitio, 100,000 horas-hombre; primer vaciado previsto dic-2027)</t>
+          <t>Construcción (166 personas en sitio, 100,000 horas-hombre; primer vaciado previsto dic-2027) ; en construcción con presupuesto de US$180 millones; inicio de operaciones proyectado en 2026</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>[Silver Tiger Metals](https://silvertigermetals.com/news/2026/silver-tiger-metals-awards-engineering-procurement-and-construction-management-contract-and-provides-construction-update)</t>
+          <t>[Silver Tiger Metals](https://silvertigermetals.com/news/2026/silver-tiger-metals-awards-engineering-procurement-and-construction-management-contract-and-provides-construction-update) ; [Minería en Línea](https://mineriaenlinea.com/2026/08/inversion-minera-en-mexico-creceria-30-en-2026-segun-camimex/)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -4715,17 +4798,17 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Construcción (BLM emitió Record of Decision positivo el 17-ago-2026, completando el permiso federal NEPA bajo el proceso acelerado FAST-41 —primera mina a cielo abierto procesada bajo este esquema—, habilitando el inicio de construcción; mina de oro/plata a cielo abierto con lixiviación en pilas, ~130,000 oz Au/año promedio en los primeros 5 años; capex inicial ~US$395 millones; ~600 empleos en construcción)</t>
+          <t>Construcción (BLM emitió Record of Decision positivo el 17-ago-2026, completando el permiso federal NEPA bajo el proceso acelerado FAST-41 —primera mina a cielo abierto procesada bajo este esquema—, habilitando el inicio de construcción; mina de oro/plata a cielo abierto con lixiviación en pilas, ~130,000 oz Au/año promedio en los primeros 5 años; capex inicial ~US$395 millones; ~600 empleos en construcción) ; BLM aprobó el proyecto el 14-ago-2026, habilitando a Gold Standard Ventures (US) Inc. a iniciar la mina; construcción emplearía hasta 600 personas</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>[StockTitan/Equinox Gold](https://www.stocktitan.net/news/EQX/equinox-gold-receives-positive-record-of-decision-for-south-railroad-ds4bk9llu3hv.html); [BLM.gov](https://www.blm.gov/announcement/blm-approves-nevada-gold-and-silver-mine-support-american-mineral-production)</t>
+          <t>[StockTitan/Equinox Gold](https://www.stocktitan.net/news/EQX/equinox-gold-receives-positive-record-of-decision-for-south-railroad-ds4bk9llu3hv.html); [BLM.gov](https://www.blm.gov/announcement/blm-approves-nevada-gold-and-silver-mine-support-american-mineral-production) ; [BLM](https://www.blm.gov/announcement/blm-approves-nevada-gold-and-silver-mine-support-american-mineral-production)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -4863,17 +4946,17 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Construcción SUSTANCIALMENTE COMPLETA en sitio Wardner; comisionamiento esperado dentro de las semanas siguientes al 31-jul-2026 (antes Q4 2026)</t>
+          <t>Construcción SUSTANCIALMENTE COMPLETA en sitio Wardner; comisionamiento esperado dentro de las semanas siguientes al 31-jul-2026 (antes Q4 2026) ; equipos mayores (espesador, filtro prensa, planta de mezcla) en fabricación con entregas desde jun-2026; construcción civil en marcha desde may-2026; puesta en marcha prevista 4T2026; capex total US$11.9 millones</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/31/3337077/0/en/bunker-hill-ships-first-concentrate-to-trail-smelter-and-announces-drawdown-of-standby-facility.html)</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/31/3337077/0/en/bunker-hill-ships-first-concentrate-to-trail-smelter-and-announces-drawdown-of-standby-facility.html) ; [SEC 6-K Americas Gold &amp; Silver](https://www.sec.gov/Archives/edgar/data/0001286973/000106299326002149/exhibit99-1.htm)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -5455,7 +5538,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Ingeniería de detalle/procura temprana (contrato EPCC otorgado, NTP limitado activo; FID esperada en 2026; planta diseñada para 22,500 tpa de carbonato de litio grado batería; DOE emitió FONSI —Finding of No Significant Impact—, paso clave hacia la FID; producción comercial estimada 2029)</t>
+          <t>Ingeniería de detalle/procura temprana (contrato EPCC otorgado, NTP limitado activo; FID esperada en 2026; planta diseñada para 22,500 tpa de carbonato de litio grado batería; DOE emitió FONSI —Finding of No Significant Impact—, paso clave hacia la FID; producción comercial estimada 2029) ; Standard Lithium completó el definitive feasibility study (DFS) tras finalizar el FEED; se espera FID y arranque de construcción en 2026, con 2-3 años de construcción/comisionamiento</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -5465,7 +5548,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -5566,17 +5649,17 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Ingeniería/Construcción temprana (ingeniería de detalle y procura de largo plazo en 2026; construcción mayor de pila de lixiviación y circuitos de trituración/procesamiento en 2027; primera producción fin de 2028)</t>
+          <t>Ingeniería/Construcción temprana (ingeniería de detalle y procura de largo plazo en 2026; construcción mayor de pila de lixiviación y circuitos de trituración/procesamiento en 2027; primera producción fin de 2028) ; Centerra Gold finalizará estudios de ingeniería, lanzará adquisiciones de largo plazo e iniciará trabajos de establecimiento de sitio durante 2026</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>[E&amp;MJ](https://www.e-mj.com/breaking-news/centerra-advances-goldfield-project-in-nevada/)</t>
+          <t>[E&amp;MJ](https://www.e-mj.com/breaking-news/centerra-advances-goldfield-project-in-nevada/) ; [E&amp;MJ](https://www.e-mj.com/breaking-news/centerra-advances-goldfield-project-in-nevada/)</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -5603,17 +5686,17 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Desarrollo/Feasibility (planta SX-EW de cátodos de cobre, ~103,000 t Cu/año proyectadas; Hudbay busca fusionarlo con el distrito Copper World adyacente ya rastreado; DFS en curso con FID apuntada para 4T2026 y construcción prevista en 2027)</t>
+          <t>Desarrollo/Feasibility (planta SX-EW de cátodos de cobre, ~103,000 t Cu/año proyectadas; Hudbay busca fusionarlo con el distrito Copper World adyacente ya rastreado; DFS en curso con FID apuntada para 4T2026 y construcción prevista en 2027) ; Hudbay Minerals completó la adquisición de Arizona Sonoran Copper el 24-jun-2026, creando el tercer distrito cuprífero más grande de Norteamérica; feasibility study esperado 2S2026, FID posible 4T2026</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/03/02/3247157/0/en/hudbay-to-acquire-arizona-sonoran-creating-the-third-largest-copper-district-in-north-america.html); [Arizona Sonoran](https://arizonasonoran.com/news-releases/arizona-sonoran-pre-feasibility-study-delivers-exceptional-results-for-the-cactus-project-outlining-long-life-low-cost-copper-1/)</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/03/02/3247157/0/en/hudbay-to-acquire-arizona-sonoran-creating-the-third-largest-copper-district-in-north-america.html); [Arizona Sonoran](https://arizonasonoran.com/news-releases/arizona-sonoran-pre-feasibility-study-delivers-exceptional-results-for-the-cactus-project-outlining-long-life-low-cost-copper-1/) ; [Hudbay Minerals](https://hudbayminerals.com/investors/press-releases/press-release-details/2026/Hudbay-Completes-Acquisition-of-Arizona-Sonoran-to-Create-the-Third-Largest-Copper-District-in-North-America/default.aspx)</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -5751,17 +5834,17 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Permisos completos obtenidos (2026); waste stripping programado 3T2026; producción de zona expandida esperada 1S2027</t>
+          <t>Permisos completos obtenidos (2026); waste stripping programado 3T2026; producción de zona expandida esperada 1S2027 ; RMS preparó estimación de capital para planta de relleno en pasta: US$99 millones en construcción inicial más US$20 millones en capital sostenido para expansión del sistema de distribución subterránea</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>[Mexico Business News](https://mexicobusiness.news/mining/news/heliostar-advances-la-colorada-pit-permits-drill-data)</t>
+          <t>[Mexico Business News](https://mexicobusiness.news/mining/news/heliostar-advances-la-colorada-pit-permits-drill-data) ; [SEC 6-K Pan American Silver](https://www.sec.gov/Archives/edgar/data/0000771992/000077199226000047/a20260428pasni43-101xworki.htm)</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -6639,17 +6722,17 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Ingeniería/Feasibility (planta demostrativa ya en producción/calificación de clientes 2026; decisión de construcción esperada fines de 2026/2027; proyecto integrado de 40,000 tpa)</t>
+          <t>Ingeniería/Feasibility (planta demostrativa ya en producción/calificación de clientes 2026; decisión de construcción esperada fines de 2026/2027; proyecto integrado de 40,000 tpa) ; subsidiaria Empire State Mines recibió Conditional Selection Notice del US Army para diseñar, financiar, construir y operar la planta de purificación de grafito; decisión de construcción esperada a fines de 2026 o inicios de 2027</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>[Junior Mining Network](https://www.juniorminingnetwork.com/junior-miner-news/press-releases/2342-tsx/ti/199070-titan-mining-to-start-shipping-first-graphite-product-and-feasibility-study-underway-for-40-000-tpa-integrated-kilbourne-graphite-project.html)</t>
+          <t>[Junior Mining Network](https://www.juniorminingnetwork.com/junior-miner-news/press-releases/2342-tsx/ti/199070-titan-mining-to-start-shipping-first-graphite-product-and-feasibility-study-underway-for-40-000-tpa-integrated-kilbourne-graphite-project.html) ; [Titan Mining Corp](https://www.titanminingcorp.com/news/news-releases/titan-mining-selected-by-the-us-army-to-establish-first-ever-public-private-partnership-for-domestic-critical-minerals-processing-on-strategic-defense-installations)</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -7527,17 +7610,17 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Desarrollo/Ingeniería (DOE anunció 20/21-ago-2026 subvención de hasta US$100 millones para construir planta comercial de extracción/refinación de litio por intercambio iónico directo desde salmuera del Great Salt Lake, 5,000 t/año; primera producción prevista 2028)</t>
+          <t>Desarrollo/Ingeniería (DOE anunció 20/21-ago-2026 subvención de hasta US$100 millones para construir planta comercial de extracción/refinación de litio por intercambio iónico directo desde salmuera del Great Salt Lake, 5,000 t/año; primera producción prevista 2028) ; DOE otorgó US$100 millones (anuncio 20-ago-2026) para la instalación comercial de extracción/refinación de litio mediante DLE de Lilac Solutions; capacidad de primera fase 5,000 ton/año, producción objetivo 2028</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>[KSL](https://www.ksl.com/article/51614351/california-company-awarded-100m-to-develop-critical-mineral-facility-on-great-salt-lake-shore); [Hatch](https://www.hatch.com/About-Us/News-And-Media/2026/06/Lilac-Solutions-Selects-Hatch-as-EPCM-Partner-for-Great-Salt-Lake-Lithium-Facility)</t>
+          <t>[KSL](https://www.ksl.com/article/51614351/california-company-awarded-100m-to-develop-critical-mineral-facility-on-great-salt-lake-shore); [Hatch](https://www.hatch.com/About-Us/News-And-Media/2026/06/Lilac-Solutions-Selects-Hatch-as-EPCM-Partner-for-Great-Salt-Lake-Lithium-Facility) ; [DOE](https://www.energy.gov/articles/energy-department-announces-500-million-secure-americas-critical-mineral-and-battery)</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -7601,17 +7684,17 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Desarrollo/financiamiento (DOE otorgó 21-ago-2026 subvención de US$100 millones para construir refinería comercial de sulfato de cobalto grado batería; ubicación específica de la planta aún no anunciada)</t>
+          <t>Desarrollo/financiamiento (DOE otorgó 21-ago-2026 subvención de US$100 millones para construir refinería comercial de sulfato de cobalto grado batería; ubicación específica de la planta aún no anunciada) ; DOE seleccionó el proyecto para un aporte federal de US$100 millones (anuncio 20-ago-2026) hacia una refinería comercial de cobalto; sitio industrial aún por determinar</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>[Local News 8](https://localnews8.com/news/business-watch/2026/08/21/salmon-company-wins-100-million-grant-to-build-cobalt-refinery/); [Local News 8 (seguimiento)](https://localnews8.com/news/local-news/2026/08/24/100m-grant-to-salmon-based-jervois-could-jumpstart-idahos-cobalt-industry/)</t>
+          <t>[Local News 8](https://localnews8.com/news/business-watch/2026/08/21/salmon-company-wins-100-million-grant-to-build-cobalt-refinery/); [Local News 8 (seguimiento)](https://localnews8.com/news/local-news/2026/08/24/100m-grant-to-salmon-based-jervois-could-jumpstart-idahos-cobalt-industry/) ; [DOE](https://www.energy.gov/articles/energy-department-announces-500-million-secure-americas-critical-mineral-and-battery)</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -7908,6 +7991,191 @@
       <c r="G102" t="inlineStr">
         <is>
           <t>2026-08-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Korea Zinc / Nyrstar Critical Minerals Smelter</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Clarksville, Tennessee, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Korea Zinc / U.S. Department of War / U.S. Department of Commerce (participación ~10%)</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Preparación de sitio en 2026, construcción completa en 2027 (inversión US$7,400 millones, capex US$6,600 millones; producirá zinc, plomo, cobre, oro, plata, antimonio, indio, bismuto, telurio, cadmio, galio, germanio, paladio y ácido sulfúrico; planta altamente intensiva en tubería/piping)</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>[Korea Zinc](https://www.koreazinc.co.kr/en/korea-zinc-partners-with-the-u-s-department-of-war-and-u-s-department-of-commerce-to-build-a-state-of-the-art-critical-minerals-smelter-in-the-united-states-with-6-6-billion-of-capital-expenditures/); [Carbon Credits](https://carboncredits.com/big-bet-bigger-stakes-korea-zincs-7-4-billion-smelter-reshapes-u-s-critical-minerals-supply/)</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Aclara Heavy Rare Earth Separation Facility</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Port of Vinton, Calcasieu Parish, Luisiana, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Aclara Resources Inc.</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Planeación (inversión US$277 millones; groundbreaking previsto 4T2026, construcción hasta 2027; procesará mineral de depósitos propios en Brasil/Chile)</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>[Louisiana Economic Development](https://www.opportunitylouisiana.gov/news/aclara-invests-277-million-to-build-nations-first-heavy-rare-earth-separation-facility-in-southwest-louisiana)</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Archimedes Project (i-80 Gold)</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Ruby Hill, Eureka County, Nevada, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>i-80 Gold Corp</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Construcción (permisos de Nevada DEP y BLM obtenidos; desarrollo subterráneo en curso; producción esperada 4T2026, objetivo 150,000-200,000 oz Au/año hacia 2028)</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>[Resource World](https://resourceworld.com/i-80-gold-obtains-construction-permits-and-begins-underground-development-at-archimedes-project-nevada/)</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Sweetwater Uranium In-Situ Recovery (ISR) Project</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Sweetwater County, Wyoming, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Sweetwater Uranium, Inc.</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Permitting (Plan de Operaciones sometido al BLM nov-2025, periodo de comentarios públicos mar-abr 2026, proyecto designado FAST-41; sería la mayor instalación de producción de uranio de EE.UU. combinando procesamiento convencional e ISR)</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>[BLM](https://www.blm.gov/announcement/sweetwater-uranium-situ-recovery-irs-project-mine-plan-operations)</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Velvet-Wood Uranium-Vanadium Project</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>San Juan County, Utah, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Anfield Energy Inc.</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Construcción (Fase 1 de construcción superficial completada jun-2026; desarrollo subterráneo Fase 2 en curso; regreso a producción previsto fines de 2026)</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/06/01/3304179/0/en/Anfield-Energy-Inc-Completes-Phase-One-Surface-Construction-at-Velvet-Wood-Project.html)</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -7922,50 +8190,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G94"/>
+  <dimension ref="A1:G96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -7994,17 +8262,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Construcción (rompimiento de tierra formal completado; 1,200 acres/10 edificios/1.4GW; VoltaGrid aprobado para operar 210 generadores de gas industrial, 700MW combinados, permitiendo operación fuera de la red pública; primera instalación en servicio 2S2026)</t>
+          <t>Construcción (rompimiento de tierra formal completado; 1,200 acres/10 edificios/1.4GW; VoltaGrid aprobado para operar 210 generadores de gas industrial, 700MW combinados, permitiendo operación fuera de la red pública; primera instalación en servicio 2S2026) ; VoltaGrid fue aprobado por TCEQ para operar 210 generadores industriales a gas (700 MW: 197 generación primaria + 13 respaldo) con motores Jenbacher; Vantage Data Centers confirmado como socio desarrollador; primer edificio previsto para fines de 2026</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/vantage-breaks-ground-on-texas-gigawatt-data-center-campus-for-openai/); [Construction Owners](https://www.constructionowners.com/news/oracle-and-openai-to-power-new-texas-data-center-off-the-grid)</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/vantage-breaks-ground-on-texas-gigawatt-data-center-campus-for-openai/); [Construction Owners](https://www.constructionowners.com/news/oracle-and-openai-to-power-new-texas-data-center-off-the-grid) ; [Construction Owners Association](https://www.constructionowners.com/news/oracle-and-openai-to-power-new-texas-data-center-off-the-grid)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -8068,17 +8336,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Construcción</t>
+          <t>Construcción ; planta simple-cycle de 1,015 MW cerca de completarse para los primeros 10 edificios; ya construidas 10 turbinas de gas más 62 generadores diésel de respaldo; se solicitan 41 turbinas y 18 generadores adicionales</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/crusoe-tops-out-final-building-at-openai-stargate-data-center-campus-in-abilene-texas/)</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/crusoe-tops-out-final-building-at-openai-stargate-data-center-campus-in-abilene-texas/) ; [Texas Observer](https://www.texasobserver.org/abilene-texas-stargate-natural-gas-plant-harms/)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -8105,17 +8373,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Construcción temprana/Ingeniería (capacidad rampa a 2.67GW; flujo de energía previsto fines de 2028; FID de la planta esperada fines de 2026)</t>
+          <t>Construcción temprana/Ingeniería (capacidad rampa a 2.67GW; flujo de energía previsto fines de 2028; FID de la planta esperada fines de 2026) ; Chevron (vía subsidiaria Energy Forge One LLC) firmó PPA a 20 años con Microsoft; 2.67 GW de capacidad, turbinas principalmente GE Vernova más Solar Turbines (Caterpillar); ubicación precisada en Condado de Reeves (2,000+ acres); FID esperada fin de 2026, arranque 2028</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>[Chevron](https://www.chevron.com/newsroom/2026/q2/chevron-signs-20-year-power-agreement-with-microsoft-for-west-texas-data-center)</t>
+          <t>[Chevron](https://www.chevron.com/newsroom/2026/q2/chevron-signs-20-year-power-agreement-with-microsoft-for-west-texas-data-center) ; [Chevron](https://www.chevron.com/newsroom/2026/q2/chevron-signs-20-year-power-agreement-with-microsoft-for-west-texas-data-center)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -8327,17 +8595,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Construcción de edificios de centro de datos iniciada (TCEQ emitió permiso de aire final para la planta —35 turbinas de gas natural, hasta 33 millones de toneladas de CO2/año—; Amazon presentó a inicios de ago-2026 permisos de construcción para 3 edificios de centro de datos —"Pecos County Data Center", Buildings A/B/C, ~189,060 pies² c/u, ~US$300M c/u—; construcción de edificios prevista ago-dic 2026; primera entrega de energía prevista 1T2027, operando inicialmente fuera de la red de ERCOT)</t>
+          <t>Construcción de edificios de centro de datos iniciada (TCEQ emitió permiso de aire final para la planta —35 turbinas de gas natural, hasta 33 millones de toneladas de CO2/año—; Amazon presentó a inicios de ago-2026 permisos de construcción para 3 edificios de centro de datos —"Pecos County Data Center", Buildings A/B/C, ~189,060 pies² c/u, ~US$300M c/u—; construcción de edificios prevista ago-dic 2026; primera entrega de energía prevista 1T2027, operando inicialmente fuera de la red de ERCOT) ; Amazon confirmó públicamente su propiedad del proyecto; permiso otorgado para 35 turbinas de gas natural (hasta 7.65 GW), el permiso de emisiones más grande otorgado este año en el país (~33 millones de toneladas de CO2/año); incluye hasta 750 MW solar y 1.8 GW de almacenamiento en baterías; primera energía prevista 1T2027, 1 GW en servicio en 2028</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>[Business Wire](https://www.businesswire.com/news/home/20260126236053/en/Pacifico-Energy-Secures-7.65-GW-Power-Generation-Permit-for-GW-Ranch-Project); [Tom's Hardware](https://www.tomshardware.com/tech-industry/data-centers/amazons-new-7-65gw-texas-ai-data-center-power-plant-could-become-the-largest-source-of-co2-pollution-in-the-us-custom-35-turbine-gas-plant-authorized-to-emit-33-million-tons-of-annual-greenhouse-gases)</t>
+          <t>[Business Wire](https://www.businesswire.com/news/home/20260126236053/en/Pacifico-Energy-Secures-7.65-GW-Power-Generation-Permit-for-GW-Ranch-Project); [Tom's Hardware](https://www.tomshardware.com/tech-industry/data-centers/amazons-new-7-65gw-texas-ai-data-center-power-plant-could-become-the-largest-source-of-co2-pollution-in-the-us-custom-35-turbine-gas-plant-authorized-to-emit-33-million-tons-of-annual-greenhouse-gases) ; [ENR](https://www.enr.com/articles/63464-amazon-discloses-ownership-of-gw-ranch-giant-texas-data-center-gas-power-complex)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -8475,17 +8743,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Construcción activa con retraso regulatorio confirmado (Comisionada de Tierras de NM rechazó por segunda vez el derecho de vía en terrenos estatales para el gasoducto "Green Chile" de Energy Transfer/Transwestern Pipeline, 14-jul-2026; filing regulatorio reportado 14-ago-2026 confirma que la fecha de entrada en servicio del gasoducto —que alimentará hasta 2.5GW de celdas de combustible Bloom Energy— se retrasó de 15-ago-2026 a 1-feb-2027; NMED pospuso decisión final sobre permisos de calidad de aire de las dos plantas de gas gemelas, audiencia pública programada 19-oct-2026; analistas citados advierten riesgo de nuevo retraso a 2S2027)</t>
+          <t>Construcción activa con retraso regulatorio confirmado (Comisionada de Tierras de NM rechazó por segunda vez el derecho de vía en terrenos estatales para el gasoducto "Green Chile" de Energy Transfer/Transwestern Pipeline, 14-jul-2026; filing regulatorio reportado 14-ago-2026 confirma que la fecha de entrada en servicio del gasoducto —que alimentará hasta 2.5GW de celdas de combustible Bloom Energy— se retrasó de 15-ago-2026 a 1-feb-2027; NMED pospuso decisión final sobre permisos de calidad de aire de las dos plantas de gas gemelas, audiencia pública programada 19-oct-2026; analistas citados advierten riesgo de nuevo retraso a 2S2027) ; Oracle/BorderPlex Digital Assets cambiaron el plan de generación de turbinas de gas/generadores diésel a un microgrid de celdas de combustible para reducir uso de agua e impacto en calidad del aire; gasoducto asociado 'Green Chile Project' (~US$60 millones, 17.7 millas) bajo revisión FERC enfrenta protesta de personal regulador federal, entrada en servicio prevista ago-2026</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>[Source NM](https://sourcenm.com/2026/07/16/new-mexico-land-commissioner-blocks-project-jupiter-related-pipeline-from-building-on-state-land/); [Bloomberg](https://www.bloomberg.com/news/articles/2026-08-14/new-mexico-gas-pipeline-for-oracle-data-center-delayed-to-2027)</t>
+          <t>[Source NM](https://sourcenm.com/2026/07/16/new-mexico-land-commissioner-blocks-project-jupiter-related-pipeline-from-building-on-state-land/); [Bloomberg](https://www.bloomberg.com/news/articles/2026-08-14/new-mexico-gas-pipeline-for-oracle-data-center-delayed-to-2027) ; [Source NM](https://sourcenm.com/2026/04/27/nm-project-jupiter-data-center-developers-announce-new-plans-for-generating-power/)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -8586,17 +8854,17 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Planeación temprana (opción de terreno)</t>
+          <t>Planeación temprana (opción de terreno) ; se formalizó opción de compra de ~3,500 acres en Condado de Lea, Nuevo México, para hub de IA de 7 GW; marca el primer desarrollo enteramente propio, separado del joint venture TCDC; planea &gt;2 GW de gas natural más 5+ GW de generación nuclear</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>[PowerMag](https://www.powermag.com/nuclear-natural-gas-power-generation-planned-for-massive-new-mexico-data-center-site/)</t>
+          <t>[PowerMag](https://www.powermag.com/nuclear-natural-gas-power-generation-planned-for-massive-new-mexico-data-center-site/) ; [Barchart](https://www.barchart.com/story/news/35949566/new-era-energy-digital-enters-into-land-option-purchase-agreement-for-3-500-acres-in-new-mexico-for-7gw-ai-data-center-hub-marks-first-wholly-owned-development-separate-from-tcdc-joint-venture)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -9141,17 +9409,17 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Planeación avanzada/contratos firmados (17/18-ago-2026: OpenAI firmó arrendamiento a 20 años por ~8GW-IT en el sitio; NVIDIA garantiza financiamiento de hasta US$105 mil millones más US$1,500 millones de inversión directa en SB Energy, a cambio de derechos exclusivos para suministrar el cómputo IA del sitio; SB Energy construirá 9.2GW de generación a gas natural, financiamiento de US$33.3 mil millones por SoftBank, más US$4.2 mil millones en transmisión; primeros 800MW previstos 2028, construcción de 6 años generaría 35,000 empleos)</t>
+          <t>Planeación avanzada/contratos firmados (17/18-ago-2026: OpenAI firmó arrendamiento a 20 años por ~8GW-IT en el sitio; NVIDIA garantiza financiamiento de hasta US$105 mil millones más US$1,500 millones de inversión directa en SB Energy, a cambio de derechos exclusivos para suministrar el cómputo IA del sitio; SB Energy construirá 9.2GW de generación a gas natural, financiamiento de US$33.3 mil millones por SoftBank, más US$4.2 mil millones en transmisión; primeros 800MW previstos 2028, construcción de 6 años generaría 35,000 empleos) ; OpenAI se unió como inversionista/arrendatario; Nvidia garantiza hasta US$105,000 millones en obligaciones de arrendamiento y pago de energía; escala confirmada en 8 IT-GW de cómputo/10 GW de generación nueva (9.2 GW de gas natural); costo total potencial hasta US$500,000 millones; primera fase de 800 MW en operación en 2028</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/softbank-eyes-10gw-data-center-at-former-doe-nuclear-enrichment-site-in-ohio/); [NVIDIA Newsroom](https://nvidianews.nvidia.com/news/nvidia-guarantees-sb-energy-s-ports-pike-technology-campus-in-ohio-to-exclusively-host-nvidia-ai-compute); [CNBC](https://www.cnbc.com/2026/08/17/nvidia-financing-open-ai-data-center-ohio.html)</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/softbank-eyes-10gw-data-center-at-former-doe-nuclear-enrichment-site-in-ohio/); [NVIDIA Newsroom](https://nvidianews.nvidia.com/news/nvidia-guarantees-sb-energy-s-ports-pike-technology-campus-in-ohio-to-exclusively-host-nvidia-ai-compute); [CNBC](https://www.cnbc.com/2026/08/17/nvidia-financing-open-ai-data-center-ohio.html) ; [CNBC](https://www.cnbc.com/2026/08/17/nvidia-financing-open-ai-data-center-ohio.html)</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -9289,17 +9557,17 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Desarrollo CONTINÚA con nuevo desarrollador (Crusoe salió del proyecto pero Black Hills Corp. avanza directamente con el cliente; permisos locales de Wyoming vigentes; 1.8GW inicial escalable a 10GW)</t>
+          <t>Desarrollo CONTINÚA con nuevo desarrollador (Crusoe salió del proyecto pero Black Hills Corp. avanza directamente con el cliente; permisos locales de Wyoming vigentes; 1.8GW inicial escalable a 10GW) ; Comisionados del Condado de Laramie, Wyoming, aprobaron por unanimidad la construcción; campus escalable de 1.8 GW hasta 10 GW; planta de generación asociada 'BFC Power and Cheyenne Power Hub' (Tallgrass Energy) con 2.7 GW de generación a gas natural, vinculada a hub de captura/secuestro de CO2 existente</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>[Cowboy State Daily](https://cowboystatedaily.com/2026/06/11/partner-pulling-out-doesnt-slow-huge-2-7gw-cheyenne-project-jade-data-center/)</t>
+          <t>[Cowboy State Daily](https://cowboystatedaily.com/2026/06/11/partner-pulling-out-doesnt-slow-huge-2-7gw-cheyenne-project-jade-data-center/) ; [Inside Climate News](https://insideclimatenews.org/news/14012026/wyoming-county-approves-ai-data-center/)</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -9400,17 +9668,17 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Construcción (movimiento de tierra del campus inicial completo; 4.6 millas de gasoducto de 450 MMcf/d instaladas y conectadas al sistema interestatal de Energy Transfer, suficiente para los primeros 2GW; tubería de agua de 20"/7.2 millas completa; turbinas en sitio/tránsito: 3x GE Frame 6B, 3x Siemens SGT6-5000F, 6x Siemens SGT-800; nuevo acuerdo con Hillcore Energy Capital para "Hillcore Power Center" de ~2.6GW —2.5GW gas natural + 100MW solar/batería—, primer bloque de ~350MW inicia construcción al firmarse acuerdos definitivos, duplicando la generación en sitio a 4.8GW en ~30 meses; Fermi planea solicitar permiso TCEQ adicional por 5GW más, meta total 17GW; primer contrato de arrendamiento vinculante anunciado 10-ago-2026 con TensorWave —~US$6,500 millones a 15 años, instalación de 222MW con derechos de expansión hasta &gt;650MW combinados—; nombramiento 13-ago-2026 de Lee McIntire —ex-Bechtel/TerraPower— como nuevo CEO para liderar transición de desarrollo a construcción, meta de ~200MW de primera energía comercial en 6 meses; ~6GW de los 17GW planeados ya permitidos, &gt;US$1,500 millones invertidos a la fecha)</t>
+          <t>Construcción (movimiento de tierra del campus inicial completo; 4.6 millas de gasoducto de 450 MMcf/d instaladas y conectadas al sistema interestatal de Energy Transfer, suficiente para los primeros 2GW; tubería de agua de 20"/7.2 millas completa; turbinas en sitio/tránsito: 3x GE Frame 6B, 3x Siemens SGT6-5000F, 6x Siemens SGT-800; nuevo acuerdo con Hillcore Energy Capital para "Hillcore Power Center" de ~2.6GW —2.5GW gas natural + 100MW solar/batería—, primer bloque de ~350MW inicia construcción al firmarse acuerdos definitivos, duplicando la generación en sitio a 4.8GW en ~30 meses; Fermi planea solicitar permiso TCEQ adicional por 5GW más, meta total 17GW; primer contrato de arrendamiento vinculante anunciado 10-ago-2026 con TensorWave —~US$6,500 millones a 15 años, instalación de 222MW con derechos de expansión hasta &gt;650MW combinados—; nombramiento 13-ago-2026 de Lee McIntire —ex-Bechtel/TerraPower— como nuevo CEO para liderar transición de desarrollo a construcción, meta de ~200MW de primera energía comercial en 6 meses; ~6GW de los 17GW planeados ya permitidos, &gt;US$1,500 millones invertidos a la fecha) ; detalles del permiso: 90 turbinas de gas de ciclo combinado, 16 torres de enfriamiento, 6 motores generadores de emergencia; ~24 millones de toneladas de GEI/año</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>[StockTitan](https://www.stocktitan.net/news/FRMI/fermi-america-tells-texas-lawmakers-project-matador-will-push-the-z7wbkjm2tsxy.html); [DCD](https://www.datacenterdynamics.com/en/news/fermi-taps-hillcore-to-construct-26gw-gas-plant-for-up-to-11gw-project-matador-in-amarillo-texas/); [NewsChannel 10](https://www.newschannel10.com/2026/08/10/fermi-america-announces-65-billion-contract-with-tensorwave/); [247wallst](https://247wallst.com/investing/2026/08/13/fermi-lands-its-first-anchor-customer-and-names-a-ceo-as-project-matador-moves-to-construction/)</t>
+          <t>[StockTitan](https://www.stocktitan.net/news/FRMI/fermi-america-tells-texas-lawmakers-project-matador-will-push-the-z7wbkjm2tsxy.html); [DCD](https://www.datacenterdynamics.com/en/news/fermi-taps-hillcore-to-construct-26gw-gas-plant-for-up-to-11gw-project-matador-in-amarillo-texas/); [NewsChannel 10](https://www.newschannel10.com/2026/08/10/fermi-america-announces-65-billion-contract-with-tensorwave/); [247wallst](https://247wallst.com/investing/2026/08/13/fermi-lands-its-first-anchor-customer-and-names-a-ceo-as-project-matador-moves-to-construction/) ; [Inside Climate News](https://insideclimatenews.org/news/25082026/texas-data-center-gas-projects/)</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -9807,17 +10075,17 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Construcción (cimentación subterránea concluida y primeras vigas de acero verticales en erección a mediados de ago-2026; planta de gas de 4.5GW, la más grande planeada en EE.UU.; primeras entregas de turbinas 2026, operación comercial 2027; Amazon confirmó —7-ago-2026, tras solicitudes FOI— estar en pláticas para posible datacenter junto a la planta, sin acuerdo definitivo, como parte de su compromiso de invertir US$20,000 millones en Pensilvania)</t>
+          <t>Construcción (cimentación subterránea concluida y primeras vigas de acero verticales en erección a mediados de ago-2026; planta de gas de 4.5GW, la más grande planeada en EE.UU.; primeras entregas de turbinas 2026, operación comercial 2027; Amazon confirmó —7-ago-2026, tras solicitudes FOI— estar en pláticas para posible datacenter junto a la planta, sin acuerdo definitivo, como parte de su compromiso de invertir US$20,000 millones en Pensilvania) ; Kiewit confirmado como EPC; turbinas GE Vernova habilitadas para hidrógeno con primeras entregas iniciando en 2026; planta de 4.5 GW, la más grande de Norteamérica</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55281341/pennsylvanias-homer-city-energy-campus-a-brownfield-transformed-for-data-center-innovation); [Indiana Gazette](https://www.indianagazette.com/local_news/amazon-hcr-are-conducting-commercial-discussions-on-data-center/article_733afa63-9d58-42d0-b16e-6dc61b71689b.html); [Pittsburgh Post-Gazette](https://www.post-gazette.com/business/powersource/2026/08/07/amazon-homer-city-data-center/stories/202608070053)</t>
+          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55281341/pennsylvanias-homer-city-energy-campus-a-brownfield-transformed-for-data-center-innovation); [Indiana Gazette](https://www.indianagazette.com/local_news/amazon-hcr-are-conducting-commercial-discussions-on-data-center/article_733afa63-9d58-42d0-b16e-6dc61b71689b.html); [Pittsburgh Post-Gazette](https://www.post-gazette.com/business/powersource/2026/08/07/amazon-homer-city-data-center/stories/202608070053) ; [ENR](https://www.enr.com/articles/60531-kiewit-to-build-record-45-gw-gas-power-plant-for-pa-data-center-complex)</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -9992,17 +10260,17 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Operando parcialmente/en expansión con crisis regulatoria activa (59 turbinas de gas natural operando en Southaven, la mayoría sin permisos federales de Clean Air Act; demanda de NAACP/Southern Environmental Law Center/Earthjustice desde abr-2026; xAI recibió aprobación para 41 turbinas de gas adicionales, ~1.2GW, en el sitio de Southaven para alimentar Colossus 2 y el próximo Colossus 3; DOJ intervino en litigio citando uso de Grok por el Departamento de Defensa; capacidad total del sitio creciendo hacia 2GW+ en tres edificios)</t>
+          <t>Operando parcialmente/en expansión con crisis regulatoria activa (59 turbinas de gas natural operando en Southaven, la mayoría sin permisos federales de Clean Air Act; demanda de NAACP/Southern Environmental Law Center/Earthjustice desde abr-2026; xAI recibió aprobación para 41 turbinas de gas adicionales, ~1.2GW, en el sitio de Southaven para alimentar Colossus 2 y el próximo Colossus 3; DOJ intervino en litigio citando uso de Grok por el Departamento de Defensa; capacidad total del sitio creciendo hacia 2GW+ en tres edificios) ; Mississippi Department of Environmental Quality otorgó permiso para 41 turbinas de gas permanentes en la planta de Southaven (~1.2 GW) que alimentará Colossus 2 (Memphis) y el próximo Colossus 3 en Mississippi; investigaciones revelaron que xAI operó 59 turbinas sin permiso (el doble de lo declarado), generando demanda legal de Earthjustice/SELC</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>[Technology.org](https://www.technology.org/2026/07/15/xai-59-unpermitted-gas-turbines-southaven-colossus-2/); [DCD](https://www.datacenterdynamics.com/en/news/musks-xai-gets-go-ahead-for-41-natural-gas-turbines-in-mississippi-to-power-colossus-data-centers/)</t>
+          <t>[Technology.org](https://www.technology.org/2026/07/15/xai-59-unpermitted-gas-turbines-southaven-colossus-2/); [DCD](https://www.datacenterdynamics.com/en/news/musks-xai-gets-go-ahead-for-41-natural-gas-turbines-in-mississippi-to-power-colossus-data-centers/) ; [DCD](https://www.datacenterdynamics.com/en/news/musks-xai-gets-go-ahead-for-41-natural-gas-turbines-in-mississippi-to-power-colossus-data-centers/)</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -10029,17 +10297,17 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Construcción (campus de USD 3.6 mil millones/430MW, la mayor carga individual jamás atendida por Cleco; rompimiento de tierra ene-2026; operaciones iniciales objetivo mediados de 2027)</t>
+          <t>Construcción (campus de USD 3.6 mil millones/430MW, la mayor carga individual jamás atendida por Cleco; rompimiento de tierra ene-2026; operaciones iniciales objetivo mediados de 2027) ; Babcock &amp; Wilcox firmó Limited Notice to Proceed (LNTP) por un proyecto valuado en &gt;US$1,500 millones para diseñar e instalar 1 GW de generación adicional (cuatro plantas de 300 MW a gas natural con calderas y turbinas de vapor); contrato completo esperado 1T2026; arranque operativo 2028</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>[Data Center Dynamics](https://www.datacenterdynamics.com/en/news/cleco-to-construct-756mw-natural-gas-plant-to-serve-applied-digitals-data-center-in-rapides-parish-louisiana-report/)</t>
+          <t>[Data Center Dynamics](https://www.datacenterdynamics.com/en/news/cleco-to-construct-756mw-natural-gas-plant-to-serve-applied-digitals-data-center-in-rapides-parish-louisiana-report/) ; [Babcock &amp; Wilcox](https://www.babcock.com/home/about/corporate/news/babcock-and-wilcox-announces-ai-data-center-power-generation-solution-and-signs-lntp-with-applied-digital-to-design-and-install-one-gigawatt-of-electric-power)</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -10214,17 +10482,17 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Anuncio/desarrollo temprano (hasta 1.8GW; incluye nueva planta de gas natural de ~2GW y hasta 2.6GW de almacenamiento en baterías; ~US$100 mil millones de inversión privada total, el mayor proyecto de desarrollo económico en la historia de Kentucky)</t>
+          <t>Anuncio/desarrollo temprano (hasta 1.8GW; incluye nueva planta de gas natural de ~2GW y hasta 2.6GW de almacenamiento en baterías; ~US$100 mil millones de inversión privada total, el mayor proyecto de desarrollo económico en la historia de Kentucky) ; Brookfield y NextEra Energy lanzaron formalmente el campus en el sitio DOE de Paducah; &gt;US$100,000 millones de inversión privada; campus de IA de 1.8 GW respaldado por 2 GW de generación a gas natural nueva más hasta 2.6 GW de almacenamiento en baterías; ~8,000 empleos de construcción</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>[Bloomberg](https://www.bloomberg.com/news/articles/2026-07-29/nextera-brookfield-to-build-100-billion-kentucky-data-campus); [Kentucky Lantern](https://kentuckylantern.com/2026/07/29/hyperscale-data-center-natural-gas-fired-project-planned-for-paducahs-former-nuclear-plant/)</t>
+          <t>[Bloomberg](https://www.bloomberg.com/news/articles/2026-07-29/nextera-brookfield-to-build-100-billion-kentucky-data-campus); [Kentucky Lantern](https://kentuckylantern.com/2026/07/29/hyperscale-data-center-natural-gas-fired-project-planned-for-paducahs-former-nuclear-plant/) ; [Data Center Knowledge](https://www.datacenterknowledge.com/data-center-construction/brookfield-nextera-launch-100b-ai-campus-at-doe-s-paducah-site)</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -10547,17 +10815,17 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Construcción (primera inversión de la asociación estratégica ECP-KKR; campus de ~700,000 pies², inversión total cercana a US$4,000 millones, capacidad inicial de TI de 144MW sobre 190MW total; operación prevista 4T2026)</t>
+          <t>Construcción (primera inversión de la asociación estratégica ECP-KKR; campus de ~700,000 pies², inversión total cercana a US$4,000 millones, capacidad inicial de TI de 144MW sobre 190MW total; operación prevista 4T2026) ; Calpine/CyrusOne anunciaron Fase 2 del acuerdo de tierra energizada en el Thad Hill Energy Center, añadiendo 210 MW (total 400 MW); campus en construcción, operación prevista 4T2026</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>[Data Centre Magazine](https://datacentremagazine.com/news/ecp-and-kkr-to-build-4bn-190mw-hyperscale-data-centre); [Connect CRE](https://www.connectcre.com/stories/energy-capital-kkr-joint-forces-on-bosque-county-data-center/)</t>
+          <t>[Data Centre Magazine](https://datacentremagazine.com/news/ecp-and-kkr-to-build-4bn-190mw-hyperscale-data-centre); [Connect CRE](https://www.connectcre.com/stories/energy-capital-kkr-joint-forces-on-bosque-county-data-center/) ; [CyrusOne](https://www.cyrusone.com/resources/press-releases/calpine-and-cyrusone-announce-phase-2-of-powered-land-agreement-to-support-hyperscale-data-center-at-thad-hill-energy-center-in-texas)</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -10954,17 +11222,17 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Permitting temprano (solicitud de permiso de aire ante TCEQ presentada 10-ago-2026, hasta 2,409 MW dedicados; sitio de ~1,240 acres construibles; construcción proyectada primavera/verano 2027 si avanza; diputado estatal Drew Darby solicitó formalmente audiencia pública de TCEQ ante oposición vecinal)</t>
+          <t>Permitting temprano (solicitud de permiso de aire ante TCEQ presentada 10-ago-2026, hasta 2,409 MW dedicados; sitio de ~1,240 acres construibles; construcción proyectada primavera/verano 2027 si avanza; diputado estatal Drew Darby solicitó formalmente audiencia pública de TCEQ ante oposición vecinal) ; planta de energía asociada identificada como 'Westline 2335' (desarrollador Westline TX Holdings LLC, vinculado a Beacon Data Centers); solicitud de permiso TCEQ para 2,409 MW mediante 240 motores reciprocantes a gas en 20 'engine halls', cerca de San Angelo</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>[San Angelo Live](https://sanangelolive.com/news/san-angelo/2026-08-10/dove-creek-data-center-has-applied-tceq-permit-heres-what-know); [Concho Valley Homepage](https://www.conchovalleyhomepage.com/news/local-news/concho-valley-data-centers/darby-calls-for-clarity-from-beacon-data-centers-requests-public-tceq-meeting/)</t>
+          <t>[San Angelo Live](https://sanangelolive.com/news/san-angelo/2026-08-10/dove-creek-data-center-has-applied-tceq-permit-heres-what-know); [Concho Valley Homepage](https://www.conchovalleyhomepage.com/news/local-news/concho-valley-data-centers/darby-calls-for-clarity-from-beacon-data-centers-requests-public-tceq-meeting/) ; [San Angelo LIVE!](https://sanangelolive.com/news/san-angelo/2026-08-10/dove-creek-data-center-has-applied-tceq-permit-heres-what-know)</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -11409,6 +11677,80 @@
       <c r="G94" t="inlineStr">
         <is>
           <t>2026-08-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Nscale "Monarch Compute Campus"</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Point Pleasant, Condado de Mason, West Virginia, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Nscale (respaldada por Nvidia); Microsoft (arrendatario de 1.35 GW de cómputo)</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Caterpillar (motores de combustión interna a gas, ~2 GW)</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Planeación/desarrollo (campus de 2,250 acres planeado a 8 GW total; Fase 1 de 1.35 GW con entrega objetivo a inicios de 2028; microgrid fuera de red alimentado por gasoducto dedicado de gas Marcellus Shale)</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/nscale-acquires-8gw-monarch-compute-campus-microsoft-signs-on-for-135gw-of-compute/); [Latitude Media](https://www.latitudemedia.com/news/microsoft-is-embracing-off-grid-gas-for-west-virginia-data-centers/)</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Dominion Energy — Chesterfield Energy Reliability Center (CERC)</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Chesterfield, Virginia, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Dominion Energy (utility; impulsada por demanda de data centers regionales)</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Aprobado/planeación (State Corporation Commission de Virginia aprobó el proyecto; 944 MW —cuatro turbinas de gas de 250 MW—, costo ~US$1,470 millones, operación comercial prevista 2029; primera de seis plantas de gas planeadas por Dominion para atender demanda de data centers)</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>[POWER Magazine](https://www.powermag.com/dominion-seeks-virginia-approval-for-1-gw-gas-fired-power-plant/); [Virginia Mercury](https://virginiamercury.com/2025/11/25/scc-approves-chesterfield-gas-plant-and-dominion-rate-hike-creates-new-rate-class-for-data-centers/)</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitoreo 2026-08-27: 9 proyectos nuevos + 33 actualizaciones de fase (#32)
Petroquímica: LSB Industries El Dorado, Yara/Enbridge Ingleside.
Mining: Korea Zinc/Nyrstar smelter, Aclara heavy rare earths, Archimedes
(i-80 Gold), Sweetwater Uranium ISR, Velvet-Wood uranium-vanadium.
Data Centers: Nscale Monarch Compute Campus, Dominion Chesterfield ERC.

Actualizaciones de fase en proyectos ya rastreados de petroquímica (2),
mining (14) y data centers (15): FIDs, permisos, contratos EPC y avances
de construcción confirmados 23-27 ago 2026.

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Petroquímica" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Petroquimica" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="LNG" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Mining" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Data Centers" sheetId="4" state="visible" r:id="rId4"/>
@@ -20,10 +20,18 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
@@ -49,8 +57,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -416,50 +425,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G53"/>
+  <dimension ref="A1:G55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -525,17 +534,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Construcción (Luisiana y el U.S. Army Corps of Engineers emitieron en jul-2026 los permisos de construcción civil necesarios; CF Industries confirmó en su reporte 2T2026 —8-K, 5-ago-2026— el inicio de construcción en ago-2026 de la planta de amoniaco bajo carbono, ~708,000-1.4 MTPA, ~US$3.7-4,000 millones; producción prevista 2029)</t>
+          <t>Construcción (Luisiana y el U.S. Army Corps of Engineers emitieron en jul-2026 los permisos de construcción civil necesarios; CF Industries confirmó en su reporte 2T2026 —8-K, 5-ago-2026— el inicio de construcción en ago-2026 de la planta de amoniaco bajo carbono, ~708,000-1.4 MTPA, ~US$3.7-4,000 millones; producción prevista 2029) ; groundbreaking formal el 26-ago-2026 con la Secretaria de Agricultura de EE.UU., Brooke Rollins, confirmando el inicio físico de construcción</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>[FuelCellsWorks](https://fuelcellsworks.com/2026/08/06/clean-energy/cf-industries-to-begin-construction-of-3-7bn-louisiana-blue-ammonia-plant); [gasworld](https://www.gasworld.com/story/cf-industries-to-begin-construction-of-4bn-louisiana-blue-ammonia-project/2256572.article/)</t>
+          <t>[FuelCellsWorks](https://fuelcellsworks.com/2026/08/06/clean-energy/cf-industries-to-begin-construction-of-3-7bn-louisiana-blue-ammonia-plant); [gasworld](https://www.gasworld.com/story/cf-industries-to-begin-construction-of-4bn-louisiana-blue-ammonia-project/2256572.article/) ; [Brownfield Ag News](https://www.brownfieldagnews.com/news/blue-point-ammonia-plant-groundbreaking-marks-step-toward-more-u-s-fertilizer-supply/)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -599,17 +608,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Construcción (comisionamiento)</t>
+          <t>Construcción (comisionamiento) ; arranque ahora esperado en 2027 (retrasado al menos 6 meses respecto a 2026), según East Daley Analytics, por menor demanda de etano proyectada</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>[BIC Magazine](https://www.bicmagazine.com/departments/operations/cpchem-golden-triangle-polymers-facility-startup-phase/)</t>
+          <t>[BIC Magazine](https://www.bicmagazine.com/departments/operations/cpchem-golden-triangle-polymers-facility-startup-phase/) ; [East Daley](https://eastdaley.com/daley-note/back-a-frac-supply-growth-creates-next-ngl-bottleneck-2)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -2386,6 +2395,80 @@
       <c r="G53" t="inlineStr">
         <is>
           <t>2026-08-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>LSB Industries — Expansión de Amoniaco El Dorado</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>El Dorado, Arkansas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>LSB Industries</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Pre-FID (decisión final de inversión proyectada para 2T2027; expansión de 100,000 toneladas/año incrementales de amoniaco, costo neto US$105-120 millones, bruto US$135-150 millones incluyendo infraestructura)</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>[The Motley Fool](https://www.fool.com/earnings/call-transcripts/2026/08/07/lsb-industries-lxu-q2-2026-earnings-call-transcript/)</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Yara/Enbridge — Amoniaco Azul Ingleside</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Enbridge Ingleside Energy Center, cerca de Corpus Christi, Texas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Yara Clean Ammonia / Enbridge (JV 50/50)</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Ingeniería (FEED en curso, pendiente FID; capacidad 1.2-1.4 MMTPA, inversión estimada US$2,600-2,900 millones; reforming autotérmico con captura de CO2 ~95%; enfrenta oposición comunitaria activa)</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>[QC Intel](https://www.qcintel.com/ammonia/article/yara-enbridge-continue-ingleside-blue-ammonia-plans-despite-pushback-28727.html)</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -2403,47 +2486,47 @@
   <dimension ref="A1:G46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -4125,50 +4208,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G102"/>
+  <dimension ref="A1:G107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -4197,17 +4280,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Construcción (PFS define mina subterránea de 20,000 t/d y planta de cátodos de 72,000 t/año; EXIM Bank gestiona más de US$1,000 millones en financiamiento, como parte del paquete federal de US$3,000 millones en minerales críticos anunciado 7-8-ago-2026; Ivanhoe completó el pago final de adquisición de terreno —US$39.3 millones— satisfaciendo el acuerdo de compraventa, y cerró una línea de crédito bancario de US$200 millones para financiar el inicio de actividades mayores de construcción en 2026; primera producción de cobre prevista 2028)</t>
+          <t>Construcción (PFS define mina subterránea de 20,000 t/d y planta de cátodos de 72,000 t/año; EXIM Bank gestiona más de US$1,000 millones en financiamiento, como parte del paquete federal de US$3,000 millones en minerales críticos anunciado 7-8-ago-2026; Ivanhoe completó el pago final de adquisición de terreno —US$39.3 millones— satisfaciendo el acuerdo de compraventa, y cerró una línea de crédito bancario de US$200 millones para financiar el inicio de actividades mayores de construcción en 2026; primera producción de cobre prevista 2028) ; ciudad de Casa Grande aprobó el Site Development Plan (mar-2026); Ivanhoe Electric adquirió tuneladora (TBM) Robbins; excavación del box-cut programada para 3T2026</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>[Mining Weekly](https://www.miningweekly.com/article/ivanhoe-electric-pencils-in-2026-construction-start-at-arizona-copper-mine-2025-06-25); [Ivanhoe Electric](https://ivanhoeelectric.com/news/ivanhoe-electric-makes-final-land-acquisition-payment-at-the-santa-cruz-copper-project-in-arizona/)</t>
+          <t>[Mining Weekly](https://www.miningweekly.com/article/ivanhoe-electric-pencils-in-2026-construction-start-at-arizona-copper-mine-2025-06-25); [Ivanhoe Electric](https://ivanhoeelectric.com/news/ivanhoe-electric-makes-final-land-acquisition-payment-at-the-santa-cruz-copper-project-in-arizona/) ; [Mining Technology](https://www.mining-technology.com/news/ivanhoe-electric-to-buy-tbm-arizona-project/)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -4234,7 +4317,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Ingeniería/Feasibility (DFS &gt;85% completo; colocación de bonos municipales por US$52 millones completada 24-jun-2026 para financiar el proyecto, ya totalmente permisado para iniciar construcción)</t>
+          <t>Ingeniería/Feasibility (DFS &gt;85% completo; colocación de bonos municipales por US$52 millones completada 24-jun-2026 para financiar el proyecto, ya totalmente permisado para iniciar construcción) ; bajo Hudbay Minerals (tras adquisición de Arizona Sonoran Copper, jun-2026), definitive feasibility study previsto para mediados de 2026, con FID esperada después en 2026</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -4244,7 +4327,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -4271,17 +4354,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Ingeniería temprana post intercambio de tierras (marzo 2026); firmó Master Supply Agreement (1-jul-2026) con Johnson Controls Inc. y UA Local 469; otorgó ~US$110 millones en contratos a Major Drilling America Inc. y Redpath USA Corporation (10-ago-2026) para acelerar exploración y desarrollo subterráneo, parte de programa de inversión de ~US$500 millones</t>
+          <t>Ingeniería temprana post intercambio de tierras (marzo 2026); firmó Master Supply Agreement (1-jul-2026) con Johnson Controls Inc. y UA Local 469; otorgó ~US$110 millones en contratos a Major Drilling America Inc. y Redpath USA Corporation (10-ago-2026) para acelerar exploración y desarrollo subterráneo, parte de programa de inversión de ~US$500 millones ; otorgó contratos por ~US$110 millones a Major Drilling America y Redpath USA Corporation para avanzar exploración y desarrollo subterráneo</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>[SEC](https://www.sec.gov/Archives/edgar/data/863064/000086306426000019/ex12d16mr_resolutionland.htm); [International Mining](https://im-mining.com/2026/08/10/resolution-copper-accelerates-exploration-underground-development-with-major-drilling-redpath-contracts/)</t>
+          <t>[SEC](https://www.sec.gov/Archives/edgar/data/863064/000086306426000019/ex12d16mr_resolutionland.htm); [International Mining](https://im-mining.com/2026/08/10/resolution-copper-accelerates-exploration-underground-development-with-major-drilling-redpath-contracts/) ; [Mining Technology](https://www.mining-technology.com/news/resolution-copper-110m-contracts-arizona-mine-2/)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -4308,17 +4391,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Construcción (reporte 2T2026: ingeniería de detalle &gt;95% completa, procura &gt;80% completa; US$1,800 millones de un capex total de US$2,930 millones ya incurridos; +1,600 trabajadores en sitio; comisionamiento anticipado de servicios previsto fines de 2026, terminación mecánica prevista fines de 2027)</t>
+          <t>Construcción (reporte 2T2026: ingeniería de detalle &gt;95% completa, procura &gt;80% completa; US$1,800 millones de un capex total de US$2,930 millones ya incurridos; +1,600 trabajadores en sitio; comisionamiento anticipado de servicios previsto fines de 2026, terminación mecánica prevista fines de 2027) ; DOE aprobó préstamo de US$2,260 millones; ingeniería detallada 93% completa y procura 60% completa (fin de 2025); concreto principal del sitio se completaría en 3T2026, con comisionamiento inicial de plantas individuales desde 4T2026</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>[Mining Weekly](https://www.miningweekly.com/article/thacker-pass-lithium-project-us-update-2026-05-22); [Lithium Americas](https://lithiumamericas.com/news/news-details/2026/Lithium-Americas-Provides-a-Project-Update-and-2026-Capex-Guidance-for-Thacker-Pass/default.aspx)</t>
+          <t>[Mining Weekly](https://www.miningweekly.com/article/thacker-pass-lithium-project-us-update-2026-05-22); [Lithium Americas](https://lithiumamericas.com/news/news-details/2026/Lithium-Americas-Provides-a-Project-Update-and-2026-Capex-Guidance-for-Thacker-Pass/default.aspx) ; [Carbon Credits](https://carboncredits.com/u-s-doe-approves-2-26-billion-for-nevada-lithium-mine/)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -4345,17 +4428,17 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Construcción, producción esperada 2026</t>
+          <t>Construcción, producción esperada 2026 ; backlog de permisos en Zacatecas bajó de 25 a 5 según CAMIMEX; de continuar el ritmo de destrabe regulatorio, el proyecto podría iniciar construcción antes de finalizar 2026</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>[Mining.com](https://www.mining.com/teck-agnico-team-up-at-san-nicolas-copper-project-in-mexico/)</t>
+          <t>[Mining.com](https://www.mining.com/teck-agnico-team-up-at-san-nicolas-copper-project-in-mexico/) ; [Minería en Línea](https://mineriaenlinea.com/2026/08/inversion-minera-en-mexico-creceria-30-en-2026-segun-camimex/)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4502,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Permisos ambientales asegurados (MIA aprobada ~28-jul-2026, destrabando obras preliminares de sitio —líneas de transmisión, acueducto, caminos de acceso, campamento— programadas sep-dic 2026; construcción completa desde 1T2027; primera producción de cátodos de cobre en 2S2029; inversión US$551 millones; capacidad 36,000 t/año de cátodos; reservas probadas/probables de 317 Mt a 0.249% Cu)</t>
+          <t>Permisos ambientales asegurados (MIA aprobada ~28-jul-2026, destrabando obras preliminares de sitio —líneas de transmisión, acueducto, caminos de acceso, campamento— programadas sep-dic 2026; construcción completa desde 1T2027; primera producción de cátodos de cobre en 2S2029; inversión US$551 millones; capacidad 36,000 t/año de cátodos; reservas probadas/probables de 317 Mt a 0.249% Cu) ; Southern Copper obtuvo los permisos ambientales necesarios; trabajos preliminares de sitio inician sep-2026, con construcción del proyecto arrancando en 1T2027</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -4429,7 +4512,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -4641,17 +4724,17 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Construcción (166 personas en sitio, 100,000 horas-hombre; primer vaciado previsto dic-2027)</t>
+          <t>Construcción (166 personas en sitio, 100,000 horas-hombre; primer vaciado previsto dic-2027) ; en construcción con presupuesto de US$180 millones; inicio de operaciones proyectado en 2026</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>[Silver Tiger Metals](https://silvertigermetals.com/news/2026/silver-tiger-metals-awards-engineering-procurement-and-construction-management-contract-and-provides-construction-update)</t>
+          <t>[Silver Tiger Metals](https://silvertigermetals.com/news/2026/silver-tiger-metals-awards-engineering-procurement-and-construction-management-contract-and-provides-construction-update) ; [Minería en Línea](https://mineriaenlinea.com/2026/08/inversion-minera-en-mexico-creceria-30-en-2026-segun-camimex/)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -4715,17 +4798,17 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Construcción (BLM emitió Record of Decision positivo el 17-ago-2026, completando el permiso federal NEPA bajo el proceso acelerado FAST-41 —primera mina a cielo abierto procesada bajo este esquema—, habilitando el inicio de construcción; mina de oro/plata a cielo abierto con lixiviación en pilas, ~130,000 oz Au/año promedio en los primeros 5 años; capex inicial ~US$395 millones; ~600 empleos en construcción)</t>
+          <t>Construcción (BLM emitió Record of Decision positivo el 17-ago-2026, completando el permiso federal NEPA bajo el proceso acelerado FAST-41 —primera mina a cielo abierto procesada bajo este esquema—, habilitando el inicio de construcción; mina de oro/plata a cielo abierto con lixiviación en pilas, ~130,000 oz Au/año promedio en los primeros 5 años; capex inicial ~US$395 millones; ~600 empleos en construcción) ; BLM aprobó el proyecto el 14-ago-2026, habilitando a Gold Standard Ventures (US) Inc. a iniciar la mina; construcción emplearía hasta 600 personas</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>[StockTitan/Equinox Gold](https://www.stocktitan.net/news/EQX/equinox-gold-receives-positive-record-of-decision-for-south-railroad-ds4bk9llu3hv.html); [BLM.gov](https://www.blm.gov/announcement/blm-approves-nevada-gold-and-silver-mine-support-american-mineral-production)</t>
+          <t>[StockTitan/Equinox Gold](https://www.stocktitan.net/news/EQX/equinox-gold-receives-positive-record-of-decision-for-south-railroad-ds4bk9llu3hv.html); [BLM.gov](https://www.blm.gov/announcement/blm-approves-nevada-gold-and-silver-mine-support-american-mineral-production) ; [BLM](https://www.blm.gov/announcement/blm-approves-nevada-gold-and-silver-mine-support-american-mineral-production)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -4863,17 +4946,17 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Construcción SUSTANCIALMENTE COMPLETA en sitio Wardner; comisionamiento esperado dentro de las semanas siguientes al 31-jul-2026 (antes Q4 2026)</t>
+          <t>Construcción SUSTANCIALMENTE COMPLETA en sitio Wardner; comisionamiento esperado dentro de las semanas siguientes al 31-jul-2026 (antes Q4 2026) ; equipos mayores (espesador, filtro prensa, planta de mezcla) en fabricación con entregas desde jun-2026; construcción civil en marcha desde may-2026; puesta en marcha prevista 4T2026; capex total US$11.9 millones</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/31/3337077/0/en/bunker-hill-ships-first-concentrate-to-trail-smelter-and-announces-drawdown-of-standby-facility.html)</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/31/3337077/0/en/bunker-hill-ships-first-concentrate-to-trail-smelter-and-announces-drawdown-of-standby-facility.html) ; [SEC 6-K Americas Gold &amp; Silver](https://www.sec.gov/Archives/edgar/data/0001286973/000106299326002149/exhibit99-1.htm)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -5455,7 +5538,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Ingeniería de detalle/procura temprana (contrato EPCC otorgado, NTP limitado activo; FID esperada en 2026; planta diseñada para 22,500 tpa de carbonato de litio grado batería; DOE emitió FONSI —Finding of No Significant Impact—, paso clave hacia la FID; producción comercial estimada 2029)</t>
+          <t>Ingeniería de detalle/procura temprana (contrato EPCC otorgado, NTP limitado activo; FID esperada en 2026; planta diseñada para 22,500 tpa de carbonato de litio grado batería; DOE emitió FONSI —Finding of No Significant Impact—, paso clave hacia la FID; producción comercial estimada 2029) ; Standard Lithium completó el definitive feasibility study (DFS) tras finalizar el FEED; se espera FID y arranque de construcción en 2026, con 2-3 años de construcción/comisionamiento</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -5465,7 +5548,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -5566,17 +5649,17 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Ingeniería/Construcción temprana (ingeniería de detalle y procura de largo plazo en 2026; construcción mayor de pila de lixiviación y circuitos de trituración/procesamiento en 2027; primera producción fin de 2028)</t>
+          <t>Ingeniería/Construcción temprana (ingeniería de detalle y procura de largo plazo en 2026; construcción mayor de pila de lixiviación y circuitos de trituración/procesamiento en 2027; primera producción fin de 2028) ; Centerra Gold finalizará estudios de ingeniería, lanzará adquisiciones de largo plazo e iniciará trabajos de establecimiento de sitio durante 2026</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>[E&amp;MJ](https://www.e-mj.com/breaking-news/centerra-advances-goldfield-project-in-nevada/)</t>
+          <t>[E&amp;MJ](https://www.e-mj.com/breaking-news/centerra-advances-goldfield-project-in-nevada/) ; [E&amp;MJ](https://www.e-mj.com/breaking-news/centerra-advances-goldfield-project-in-nevada/)</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -5603,17 +5686,17 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Desarrollo/Feasibility (planta SX-EW de cátodos de cobre, ~103,000 t Cu/año proyectadas; Hudbay busca fusionarlo con el distrito Copper World adyacente ya rastreado; DFS en curso con FID apuntada para 4T2026 y construcción prevista en 2027)</t>
+          <t>Desarrollo/Feasibility (planta SX-EW de cátodos de cobre, ~103,000 t Cu/año proyectadas; Hudbay busca fusionarlo con el distrito Copper World adyacente ya rastreado; DFS en curso con FID apuntada para 4T2026 y construcción prevista en 2027) ; Hudbay Minerals completó la adquisición de Arizona Sonoran Copper el 24-jun-2026, creando el tercer distrito cuprífero más grande de Norteamérica; feasibility study esperado 2S2026, FID posible 4T2026</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/03/02/3247157/0/en/hudbay-to-acquire-arizona-sonoran-creating-the-third-largest-copper-district-in-north-america.html); [Arizona Sonoran](https://arizonasonoran.com/news-releases/arizona-sonoran-pre-feasibility-study-delivers-exceptional-results-for-the-cactus-project-outlining-long-life-low-cost-copper-1/)</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/03/02/3247157/0/en/hudbay-to-acquire-arizona-sonoran-creating-the-third-largest-copper-district-in-north-america.html); [Arizona Sonoran](https://arizonasonoran.com/news-releases/arizona-sonoran-pre-feasibility-study-delivers-exceptional-results-for-the-cactus-project-outlining-long-life-low-cost-copper-1/) ; [Hudbay Minerals](https://hudbayminerals.com/investors/press-releases/press-release-details/2026/Hudbay-Completes-Acquisition-of-Arizona-Sonoran-to-Create-the-Third-Largest-Copper-District-in-North-America/default.aspx)</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -5751,17 +5834,17 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Permisos completos obtenidos (2026); waste stripping programado 3T2026; producción de zona expandida esperada 1S2027</t>
+          <t>Permisos completos obtenidos (2026); waste stripping programado 3T2026; producción de zona expandida esperada 1S2027 ; RMS preparó estimación de capital para planta de relleno en pasta: US$99 millones en construcción inicial más US$20 millones en capital sostenido para expansión del sistema de distribución subterránea</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>[Mexico Business News](https://mexicobusiness.news/mining/news/heliostar-advances-la-colorada-pit-permits-drill-data)</t>
+          <t>[Mexico Business News](https://mexicobusiness.news/mining/news/heliostar-advances-la-colorada-pit-permits-drill-data) ; [SEC 6-K Pan American Silver](https://www.sec.gov/Archives/edgar/data/0000771992/000077199226000047/a20260428pasni43-101xworki.htm)</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -6639,17 +6722,17 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Ingeniería/Feasibility (planta demostrativa ya en producción/calificación de clientes 2026; decisión de construcción esperada fines de 2026/2027; proyecto integrado de 40,000 tpa)</t>
+          <t>Ingeniería/Feasibility (planta demostrativa ya en producción/calificación de clientes 2026; decisión de construcción esperada fines de 2026/2027; proyecto integrado de 40,000 tpa) ; subsidiaria Empire State Mines recibió Conditional Selection Notice del US Army para diseñar, financiar, construir y operar la planta de purificación de grafito; decisión de construcción esperada a fines de 2026 o inicios de 2027</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>[Junior Mining Network](https://www.juniorminingnetwork.com/junior-miner-news/press-releases/2342-tsx/ti/199070-titan-mining-to-start-shipping-first-graphite-product-and-feasibility-study-underway-for-40-000-tpa-integrated-kilbourne-graphite-project.html)</t>
+          <t>[Junior Mining Network](https://www.juniorminingnetwork.com/junior-miner-news/press-releases/2342-tsx/ti/199070-titan-mining-to-start-shipping-first-graphite-product-and-feasibility-study-underway-for-40-000-tpa-integrated-kilbourne-graphite-project.html) ; [Titan Mining Corp](https://www.titanminingcorp.com/news/news-releases/titan-mining-selected-by-the-us-army-to-establish-first-ever-public-private-partnership-for-domestic-critical-minerals-processing-on-strategic-defense-installations)</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -7527,17 +7610,17 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Desarrollo/Ingeniería (DOE anunció 20/21-ago-2026 subvención de hasta US$100 millones para construir planta comercial de extracción/refinación de litio por intercambio iónico directo desde salmuera del Great Salt Lake, 5,000 t/año; primera producción prevista 2028)</t>
+          <t>Desarrollo/Ingeniería (DOE anunció 20/21-ago-2026 subvención de hasta US$100 millones para construir planta comercial de extracción/refinación de litio por intercambio iónico directo desde salmuera del Great Salt Lake, 5,000 t/año; primera producción prevista 2028) ; DOE otorgó US$100 millones (anuncio 20-ago-2026) para la instalación comercial de extracción/refinación de litio mediante DLE de Lilac Solutions; capacidad de primera fase 5,000 ton/año, producción objetivo 2028</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>[KSL](https://www.ksl.com/article/51614351/california-company-awarded-100m-to-develop-critical-mineral-facility-on-great-salt-lake-shore); [Hatch](https://www.hatch.com/About-Us/News-And-Media/2026/06/Lilac-Solutions-Selects-Hatch-as-EPCM-Partner-for-Great-Salt-Lake-Lithium-Facility)</t>
+          <t>[KSL](https://www.ksl.com/article/51614351/california-company-awarded-100m-to-develop-critical-mineral-facility-on-great-salt-lake-shore); [Hatch](https://www.hatch.com/About-Us/News-And-Media/2026/06/Lilac-Solutions-Selects-Hatch-as-EPCM-Partner-for-Great-Salt-Lake-Lithium-Facility) ; [DOE](https://www.energy.gov/articles/energy-department-announces-500-million-secure-americas-critical-mineral-and-battery)</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -7601,17 +7684,17 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Desarrollo/financiamiento (DOE otorgó 21-ago-2026 subvención de US$100 millones para construir refinería comercial de sulfato de cobalto grado batería; ubicación específica de la planta aún no anunciada)</t>
+          <t>Desarrollo/financiamiento (DOE otorgó 21-ago-2026 subvención de US$100 millones para construir refinería comercial de sulfato de cobalto grado batería; ubicación específica de la planta aún no anunciada) ; DOE seleccionó el proyecto para un aporte federal de US$100 millones (anuncio 20-ago-2026) hacia una refinería comercial de cobalto; sitio industrial aún por determinar</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>[Local News 8](https://localnews8.com/news/business-watch/2026/08/21/salmon-company-wins-100-million-grant-to-build-cobalt-refinery/); [Local News 8 (seguimiento)](https://localnews8.com/news/local-news/2026/08/24/100m-grant-to-salmon-based-jervois-could-jumpstart-idahos-cobalt-industry/)</t>
+          <t>[Local News 8](https://localnews8.com/news/business-watch/2026/08/21/salmon-company-wins-100-million-grant-to-build-cobalt-refinery/); [Local News 8 (seguimiento)](https://localnews8.com/news/local-news/2026/08/24/100m-grant-to-salmon-based-jervois-could-jumpstart-idahos-cobalt-industry/) ; [DOE](https://www.energy.gov/articles/energy-department-announces-500-million-secure-americas-critical-mineral-and-battery)</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -7908,6 +7991,191 @@
       <c r="G102" t="inlineStr">
         <is>
           <t>2026-08-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Korea Zinc / Nyrstar Critical Minerals Smelter</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Clarksville, Tennessee, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Korea Zinc / U.S. Department of War / U.S. Department of Commerce (participación ~10%)</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Preparación de sitio en 2026, construcción completa en 2027 (inversión US$7,400 millones, capex US$6,600 millones; producirá zinc, plomo, cobre, oro, plata, antimonio, indio, bismuto, telurio, cadmio, galio, germanio, paladio y ácido sulfúrico; planta altamente intensiva en tubería/piping)</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>[Korea Zinc](https://www.koreazinc.co.kr/en/korea-zinc-partners-with-the-u-s-department-of-war-and-u-s-department-of-commerce-to-build-a-state-of-the-art-critical-minerals-smelter-in-the-united-states-with-6-6-billion-of-capital-expenditures/); [Carbon Credits](https://carboncredits.com/big-bet-bigger-stakes-korea-zincs-7-4-billion-smelter-reshapes-u-s-critical-minerals-supply/)</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Aclara Heavy Rare Earth Separation Facility</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Port of Vinton, Calcasieu Parish, Luisiana, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Aclara Resources Inc.</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Planeación (inversión US$277 millones; groundbreaking previsto 4T2026, construcción hasta 2027; procesará mineral de depósitos propios en Brasil/Chile)</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>[Louisiana Economic Development](https://www.opportunitylouisiana.gov/news/aclara-invests-277-million-to-build-nations-first-heavy-rare-earth-separation-facility-in-southwest-louisiana)</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Archimedes Project (i-80 Gold)</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Ruby Hill, Eureka County, Nevada, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>i-80 Gold Corp</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Construcción (permisos de Nevada DEP y BLM obtenidos; desarrollo subterráneo en curso; producción esperada 4T2026, objetivo 150,000-200,000 oz Au/año hacia 2028)</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>[Resource World](https://resourceworld.com/i-80-gold-obtains-construction-permits-and-begins-underground-development-at-archimedes-project-nevada/)</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Sweetwater Uranium In-Situ Recovery (ISR) Project</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Sweetwater County, Wyoming, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Sweetwater Uranium, Inc.</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Permitting (Plan de Operaciones sometido al BLM nov-2025, periodo de comentarios públicos mar-abr 2026, proyecto designado FAST-41; sería la mayor instalación de producción de uranio de EE.UU. combinando procesamiento convencional e ISR)</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>[BLM](https://www.blm.gov/announcement/sweetwater-uranium-situ-recovery-irs-project-mine-plan-operations)</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Velvet-Wood Uranium-Vanadium Project</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>San Juan County, Utah, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Anfield Energy Inc.</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Construcción (Fase 1 de construcción superficial completada jun-2026; desarrollo subterráneo Fase 2 en curso; regreso a producción previsto fines de 2026)</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/06/01/3304179/0/en/Anfield-Energy-Inc-Completes-Phase-One-Surface-Construction-at-Velvet-Wood-Project.html)</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -7922,50 +8190,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G94"/>
+  <dimension ref="A1:G96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -7994,17 +8262,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Construcción (rompimiento de tierra formal completado; 1,200 acres/10 edificios/1.4GW; VoltaGrid aprobado para operar 210 generadores de gas industrial, 700MW combinados, permitiendo operación fuera de la red pública; primera instalación en servicio 2S2026)</t>
+          <t>Construcción (rompimiento de tierra formal completado; 1,200 acres/10 edificios/1.4GW; VoltaGrid aprobado para operar 210 generadores de gas industrial, 700MW combinados, permitiendo operación fuera de la red pública; primera instalación en servicio 2S2026) ; VoltaGrid fue aprobado por TCEQ para operar 210 generadores industriales a gas (700 MW: 197 generación primaria + 13 respaldo) con motores Jenbacher; Vantage Data Centers confirmado como socio desarrollador; primer edificio previsto para fines de 2026</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/vantage-breaks-ground-on-texas-gigawatt-data-center-campus-for-openai/); [Construction Owners](https://www.constructionowners.com/news/oracle-and-openai-to-power-new-texas-data-center-off-the-grid)</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/vantage-breaks-ground-on-texas-gigawatt-data-center-campus-for-openai/); [Construction Owners](https://www.constructionowners.com/news/oracle-and-openai-to-power-new-texas-data-center-off-the-grid) ; [Construction Owners Association](https://www.constructionowners.com/news/oracle-and-openai-to-power-new-texas-data-center-off-the-grid)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -8068,17 +8336,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Construcción</t>
+          <t>Construcción ; planta simple-cycle de 1,015 MW cerca de completarse para los primeros 10 edificios; ya construidas 10 turbinas de gas más 62 generadores diésel de respaldo; se solicitan 41 turbinas y 18 generadores adicionales</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/crusoe-tops-out-final-building-at-openai-stargate-data-center-campus-in-abilene-texas/)</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/crusoe-tops-out-final-building-at-openai-stargate-data-center-campus-in-abilene-texas/) ; [Texas Observer](https://www.texasobserver.org/abilene-texas-stargate-natural-gas-plant-harms/)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -8105,17 +8373,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Construcción temprana/Ingeniería (capacidad rampa a 2.67GW; flujo de energía previsto fines de 2028; FID de la planta esperada fines de 2026)</t>
+          <t>Construcción temprana/Ingeniería (capacidad rampa a 2.67GW; flujo de energía previsto fines de 2028; FID de la planta esperada fines de 2026) ; Chevron (vía subsidiaria Energy Forge One LLC) firmó PPA a 20 años con Microsoft; 2.67 GW de capacidad, turbinas principalmente GE Vernova más Solar Turbines (Caterpillar); ubicación precisada en Condado de Reeves (2,000+ acres); FID esperada fin de 2026, arranque 2028</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>[Chevron](https://www.chevron.com/newsroom/2026/q2/chevron-signs-20-year-power-agreement-with-microsoft-for-west-texas-data-center)</t>
+          <t>[Chevron](https://www.chevron.com/newsroom/2026/q2/chevron-signs-20-year-power-agreement-with-microsoft-for-west-texas-data-center) ; [Chevron](https://www.chevron.com/newsroom/2026/q2/chevron-signs-20-year-power-agreement-with-microsoft-for-west-texas-data-center)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -8327,17 +8595,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Construcción de edificios de centro de datos iniciada (TCEQ emitió permiso de aire final para la planta —35 turbinas de gas natural, hasta 33 millones de toneladas de CO2/año—; Amazon presentó a inicios de ago-2026 permisos de construcción para 3 edificios de centro de datos —"Pecos County Data Center", Buildings A/B/C, ~189,060 pies² c/u, ~US$300M c/u—; construcción de edificios prevista ago-dic 2026; primera entrega de energía prevista 1T2027, operando inicialmente fuera de la red de ERCOT)</t>
+          <t>Construcción de edificios de centro de datos iniciada (TCEQ emitió permiso de aire final para la planta —35 turbinas de gas natural, hasta 33 millones de toneladas de CO2/año—; Amazon presentó a inicios de ago-2026 permisos de construcción para 3 edificios de centro de datos —"Pecos County Data Center", Buildings A/B/C, ~189,060 pies² c/u, ~US$300M c/u—; construcción de edificios prevista ago-dic 2026; primera entrega de energía prevista 1T2027, operando inicialmente fuera de la red de ERCOT) ; Amazon confirmó públicamente su propiedad del proyecto; permiso otorgado para 35 turbinas de gas natural (hasta 7.65 GW), el permiso de emisiones más grande otorgado este año en el país (~33 millones de toneladas de CO2/año); incluye hasta 750 MW solar y 1.8 GW de almacenamiento en baterías; primera energía prevista 1T2027, 1 GW en servicio en 2028</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>[Business Wire](https://www.businesswire.com/news/home/20260126236053/en/Pacifico-Energy-Secures-7.65-GW-Power-Generation-Permit-for-GW-Ranch-Project); [Tom's Hardware](https://www.tomshardware.com/tech-industry/data-centers/amazons-new-7-65gw-texas-ai-data-center-power-plant-could-become-the-largest-source-of-co2-pollution-in-the-us-custom-35-turbine-gas-plant-authorized-to-emit-33-million-tons-of-annual-greenhouse-gases)</t>
+          <t>[Business Wire](https://www.businesswire.com/news/home/20260126236053/en/Pacifico-Energy-Secures-7.65-GW-Power-Generation-Permit-for-GW-Ranch-Project); [Tom's Hardware](https://www.tomshardware.com/tech-industry/data-centers/amazons-new-7-65gw-texas-ai-data-center-power-plant-could-become-the-largest-source-of-co2-pollution-in-the-us-custom-35-turbine-gas-plant-authorized-to-emit-33-million-tons-of-annual-greenhouse-gases) ; [ENR](https://www.enr.com/articles/63464-amazon-discloses-ownership-of-gw-ranch-giant-texas-data-center-gas-power-complex)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -8475,17 +8743,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Construcción activa con retraso regulatorio confirmado (Comisionada de Tierras de NM rechazó por segunda vez el derecho de vía en terrenos estatales para el gasoducto "Green Chile" de Energy Transfer/Transwestern Pipeline, 14-jul-2026; filing regulatorio reportado 14-ago-2026 confirma que la fecha de entrada en servicio del gasoducto —que alimentará hasta 2.5GW de celdas de combustible Bloom Energy— se retrasó de 15-ago-2026 a 1-feb-2027; NMED pospuso decisión final sobre permisos de calidad de aire de las dos plantas de gas gemelas, audiencia pública programada 19-oct-2026; analistas citados advierten riesgo de nuevo retraso a 2S2027)</t>
+          <t>Construcción activa con retraso regulatorio confirmado (Comisionada de Tierras de NM rechazó por segunda vez el derecho de vía en terrenos estatales para el gasoducto "Green Chile" de Energy Transfer/Transwestern Pipeline, 14-jul-2026; filing regulatorio reportado 14-ago-2026 confirma que la fecha de entrada en servicio del gasoducto —que alimentará hasta 2.5GW de celdas de combustible Bloom Energy— se retrasó de 15-ago-2026 a 1-feb-2027; NMED pospuso decisión final sobre permisos de calidad de aire de las dos plantas de gas gemelas, audiencia pública programada 19-oct-2026; analistas citados advierten riesgo de nuevo retraso a 2S2027) ; Oracle/BorderPlex Digital Assets cambiaron el plan de generación de turbinas de gas/generadores diésel a un microgrid de celdas de combustible para reducir uso de agua e impacto en calidad del aire; gasoducto asociado 'Green Chile Project' (~US$60 millones, 17.7 millas) bajo revisión FERC enfrenta protesta de personal regulador federal, entrada en servicio prevista ago-2026</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>[Source NM](https://sourcenm.com/2026/07/16/new-mexico-land-commissioner-blocks-project-jupiter-related-pipeline-from-building-on-state-land/); [Bloomberg](https://www.bloomberg.com/news/articles/2026-08-14/new-mexico-gas-pipeline-for-oracle-data-center-delayed-to-2027)</t>
+          <t>[Source NM](https://sourcenm.com/2026/07/16/new-mexico-land-commissioner-blocks-project-jupiter-related-pipeline-from-building-on-state-land/); [Bloomberg](https://www.bloomberg.com/news/articles/2026-08-14/new-mexico-gas-pipeline-for-oracle-data-center-delayed-to-2027) ; [Source NM](https://sourcenm.com/2026/04/27/nm-project-jupiter-data-center-developers-announce-new-plans-for-generating-power/)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -8586,17 +8854,17 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Planeación temprana (opción de terreno)</t>
+          <t>Planeación temprana (opción de terreno) ; se formalizó opción de compra de ~3,500 acres en Condado de Lea, Nuevo México, para hub de IA de 7 GW; marca el primer desarrollo enteramente propio, separado del joint venture TCDC; planea &gt;2 GW de gas natural más 5+ GW de generación nuclear</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>[PowerMag](https://www.powermag.com/nuclear-natural-gas-power-generation-planned-for-massive-new-mexico-data-center-site/)</t>
+          <t>[PowerMag](https://www.powermag.com/nuclear-natural-gas-power-generation-planned-for-massive-new-mexico-data-center-site/) ; [Barchart](https://www.barchart.com/story/news/35949566/new-era-energy-digital-enters-into-land-option-purchase-agreement-for-3-500-acres-in-new-mexico-for-7gw-ai-data-center-hub-marks-first-wholly-owned-development-separate-from-tcdc-joint-venture)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -9141,17 +9409,17 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Planeación avanzada/contratos firmados (17/18-ago-2026: OpenAI firmó arrendamiento a 20 años por ~8GW-IT en el sitio; NVIDIA garantiza financiamiento de hasta US$105 mil millones más US$1,500 millones de inversión directa en SB Energy, a cambio de derechos exclusivos para suministrar el cómputo IA del sitio; SB Energy construirá 9.2GW de generación a gas natural, financiamiento de US$33.3 mil millones por SoftBank, más US$4.2 mil millones en transmisión; primeros 800MW previstos 2028, construcción de 6 años generaría 35,000 empleos)</t>
+          <t>Planeación avanzada/contratos firmados (17/18-ago-2026: OpenAI firmó arrendamiento a 20 años por ~8GW-IT en el sitio; NVIDIA garantiza financiamiento de hasta US$105 mil millones más US$1,500 millones de inversión directa en SB Energy, a cambio de derechos exclusivos para suministrar el cómputo IA del sitio; SB Energy construirá 9.2GW de generación a gas natural, financiamiento de US$33.3 mil millones por SoftBank, más US$4.2 mil millones en transmisión; primeros 800MW previstos 2028, construcción de 6 años generaría 35,000 empleos) ; OpenAI se unió como inversionista/arrendatario; Nvidia garantiza hasta US$105,000 millones en obligaciones de arrendamiento y pago de energía; escala confirmada en 8 IT-GW de cómputo/10 GW de generación nueva (9.2 GW de gas natural); costo total potencial hasta US$500,000 millones; primera fase de 800 MW en operación en 2028</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>[DCD](https://www.datacenterdynamics.com/en/news/softbank-eyes-10gw-data-center-at-former-doe-nuclear-enrichment-site-in-ohio/); [NVIDIA Newsroom](https://nvidianews.nvidia.com/news/nvidia-guarantees-sb-energy-s-ports-pike-technology-campus-in-ohio-to-exclusively-host-nvidia-ai-compute); [CNBC](https://www.cnbc.com/2026/08/17/nvidia-financing-open-ai-data-center-ohio.html)</t>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/softbank-eyes-10gw-data-center-at-former-doe-nuclear-enrichment-site-in-ohio/); [NVIDIA Newsroom](https://nvidianews.nvidia.com/news/nvidia-guarantees-sb-energy-s-ports-pike-technology-campus-in-ohio-to-exclusively-host-nvidia-ai-compute); [CNBC](https://www.cnbc.com/2026/08/17/nvidia-financing-open-ai-data-center-ohio.html) ; [CNBC](https://www.cnbc.com/2026/08/17/nvidia-financing-open-ai-data-center-ohio.html)</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -9289,17 +9557,17 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Desarrollo CONTINÚA con nuevo desarrollador (Crusoe salió del proyecto pero Black Hills Corp. avanza directamente con el cliente; permisos locales de Wyoming vigentes; 1.8GW inicial escalable a 10GW)</t>
+          <t>Desarrollo CONTINÚA con nuevo desarrollador (Crusoe salió del proyecto pero Black Hills Corp. avanza directamente con el cliente; permisos locales de Wyoming vigentes; 1.8GW inicial escalable a 10GW) ; Comisionados del Condado de Laramie, Wyoming, aprobaron por unanimidad la construcción; campus escalable de 1.8 GW hasta 10 GW; planta de generación asociada 'BFC Power and Cheyenne Power Hub' (Tallgrass Energy) con 2.7 GW de generación a gas natural, vinculada a hub de captura/secuestro de CO2 existente</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>[Cowboy State Daily](https://cowboystatedaily.com/2026/06/11/partner-pulling-out-doesnt-slow-huge-2-7gw-cheyenne-project-jade-data-center/)</t>
+          <t>[Cowboy State Daily](https://cowboystatedaily.com/2026/06/11/partner-pulling-out-doesnt-slow-huge-2-7gw-cheyenne-project-jade-data-center/) ; [Inside Climate News](https://insideclimatenews.org/news/14012026/wyoming-county-approves-ai-data-center/)</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -9400,17 +9668,17 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Construcción (movimiento de tierra del campus inicial completo; 4.6 millas de gasoducto de 450 MMcf/d instaladas y conectadas al sistema interestatal de Energy Transfer, suficiente para los primeros 2GW; tubería de agua de 20"/7.2 millas completa; turbinas en sitio/tránsito: 3x GE Frame 6B, 3x Siemens SGT6-5000F, 6x Siemens SGT-800; nuevo acuerdo con Hillcore Energy Capital para "Hillcore Power Center" de ~2.6GW —2.5GW gas natural + 100MW solar/batería—, primer bloque de ~350MW inicia construcción al firmarse acuerdos definitivos, duplicando la generación en sitio a 4.8GW en ~30 meses; Fermi planea solicitar permiso TCEQ adicional por 5GW más, meta total 17GW; primer contrato de arrendamiento vinculante anunciado 10-ago-2026 con TensorWave —~US$6,500 millones a 15 años, instalación de 222MW con derechos de expansión hasta &gt;650MW combinados—; nombramiento 13-ago-2026 de Lee McIntire —ex-Bechtel/TerraPower— como nuevo CEO para liderar transición de desarrollo a construcción, meta de ~200MW de primera energía comercial en 6 meses; ~6GW de los 17GW planeados ya permitidos, &gt;US$1,500 millones invertidos a la fecha)</t>
+          <t>Construcción (movimiento de tierra del campus inicial completo; 4.6 millas de gasoducto de 450 MMcf/d instaladas y conectadas al sistema interestatal de Energy Transfer, suficiente para los primeros 2GW; tubería de agua de 20"/7.2 millas completa; turbinas en sitio/tránsito: 3x GE Frame 6B, 3x Siemens SGT6-5000F, 6x Siemens SGT-800; nuevo acuerdo con Hillcore Energy Capital para "Hillcore Power Center" de ~2.6GW —2.5GW gas natural + 100MW solar/batería—, primer bloque de ~350MW inicia construcción al firmarse acuerdos definitivos, duplicando la generación en sitio a 4.8GW en ~30 meses; Fermi planea solicitar permiso TCEQ adicional por 5GW más, meta total 17GW; primer contrato de arrendamiento vinculante anunciado 10-ago-2026 con TensorWave —~US$6,500 millones a 15 años, instalación de 222MW con derechos de expansión hasta &gt;650MW combinados—; nombramiento 13-ago-2026 de Lee McIntire —ex-Bechtel/TerraPower— como nuevo CEO para liderar transición de desarrollo a construcción, meta de ~200MW de primera energía comercial en 6 meses; ~6GW de los 17GW planeados ya permitidos, &gt;US$1,500 millones invertidos a la fecha) ; detalles del permiso: 90 turbinas de gas de ciclo combinado, 16 torres de enfriamiento, 6 motores generadores de emergencia; ~24 millones de toneladas de GEI/año</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>[StockTitan](https://www.stocktitan.net/news/FRMI/fermi-america-tells-texas-lawmakers-project-matador-will-push-the-z7wbkjm2tsxy.html); [DCD](https://www.datacenterdynamics.com/en/news/fermi-taps-hillcore-to-construct-26gw-gas-plant-for-up-to-11gw-project-matador-in-amarillo-texas/); [NewsChannel 10](https://www.newschannel10.com/2026/08/10/fermi-america-announces-65-billion-contract-with-tensorwave/); [247wallst](https://247wallst.com/investing/2026/08/13/fermi-lands-its-first-anchor-customer-and-names-a-ceo-as-project-matador-moves-to-construction/)</t>
+          <t>[StockTitan](https://www.stocktitan.net/news/FRMI/fermi-america-tells-texas-lawmakers-project-matador-will-push-the-z7wbkjm2tsxy.html); [DCD](https://www.datacenterdynamics.com/en/news/fermi-taps-hillcore-to-construct-26gw-gas-plant-for-up-to-11gw-project-matador-in-amarillo-texas/); [NewsChannel 10](https://www.newschannel10.com/2026/08/10/fermi-america-announces-65-billion-contract-with-tensorwave/); [247wallst](https://247wallst.com/investing/2026/08/13/fermi-lands-its-first-anchor-customer-and-names-a-ceo-as-project-matador-moves-to-construction/) ; [Inside Climate News](https://insideclimatenews.org/news/25082026/texas-data-center-gas-projects/)</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -9807,17 +10075,17 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Construcción (cimentación subterránea concluida y primeras vigas de acero verticales en erección a mediados de ago-2026; planta de gas de 4.5GW, la más grande planeada en EE.UU.; primeras entregas de turbinas 2026, operación comercial 2027; Amazon confirmó —7-ago-2026, tras solicitudes FOI— estar en pláticas para posible datacenter junto a la planta, sin acuerdo definitivo, como parte de su compromiso de invertir US$20,000 millones en Pensilvania)</t>
+          <t>Construcción (cimentación subterránea concluida y primeras vigas de acero verticales en erección a mediados de ago-2026; planta de gas de 4.5GW, la más grande planeada en EE.UU.; primeras entregas de turbinas 2026, operación comercial 2027; Amazon confirmó —7-ago-2026, tras solicitudes FOI— estar en pláticas para posible datacenter junto a la planta, sin acuerdo definitivo, como parte de su compromiso de invertir US$20,000 millones en Pensilvania) ; Kiewit confirmado como EPC; turbinas GE Vernova habilitadas para hidrógeno con primeras entregas iniciando en 2026; planta de 4.5 GW, la más grande de Norteamérica</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55281341/pennsylvanias-homer-city-energy-campus-a-brownfield-transformed-for-data-center-innovation); [Indiana Gazette](https://www.indianagazette.com/local_news/amazon-hcr-are-conducting-commercial-discussions-on-data-center/article_733afa63-9d58-42d0-b16e-6dc61b71689b.html); [Pittsburgh Post-Gazette](https://www.post-gazette.com/business/powersource/2026/08/07/amazon-homer-city-data-center/stories/202608070053)</t>
+          <t>[Data Center Frontier](https://www.datacenterfrontier.com/site-selection/article/55281341/pennsylvanias-homer-city-energy-campus-a-brownfield-transformed-for-data-center-innovation); [Indiana Gazette](https://www.indianagazette.com/local_news/amazon-hcr-are-conducting-commercial-discussions-on-data-center/article_733afa63-9d58-42d0-b16e-6dc61b71689b.html); [Pittsburgh Post-Gazette](https://www.post-gazette.com/business/powersource/2026/08/07/amazon-homer-city-data-center/stories/202608070053) ; [ENR](https://www.enr.com/articles/60531-kiewit-to-build-record-45-gw-gas-power-plant-for-pa-data-center-complex)</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -9992,17 +10260,17 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Operando parcialmente/en expansión con crisis regulatoria activa (59 turbinas de gas natural operando en Southaven, la mayoría sin permisos federales de Clean Air Act; demanda de NAACP/Southern Environmental Law Center/Earthjustice desde abr-2026; xAI recibió aprobación para 41 turbinas de gas adicionales, ~1.2GW, en el sitio de Southaven para alimentar Colossus 2 y el próximo Colossus 3; DOJ intervino en litigio citando uso de Grok por el Departamento de Defensa; capacidad total del sitio creciendo hacia 2GW+ en tres edificios)</t>
+          <t>Operando parcialmente/en expansión con crisis regulatoria activa (59 turbinas de gas natural operando en Southaven, la mayoría sin permisos federales de Clean Air Act; demanda de NAACP/Southern Environmental Law Center/Earthjustice desde abr-2026; xAI recibió aprobación para 41 turbinas de gas adicionales, ~1.2GW, en el sitio de Southaven para alimentar Colossus 2 y el próximo Colossus 3; DOJ intervino en litigio citando uso de Grok por el Departamento de Defensa; capacidad total del sitio creciendo hacia 2GW+ en tres edificios) ; Mississippi Department of Environmental Quality otorgó permiso para 41 turbinas de gas permanentes en la planta de Southaven (~1.2 GW) que alimentará Colossus 2 (Memphis) y el próximo Colossus 3 en Mississippi; investigaciones revelaron que xAI operó 59 turbinas sin permiso (el doble de lo declarado), generando demanda legal de Earthjustice/SELC</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>[Technology.org](https://www.technology.org/2026/07/15/xai-59-unpermitted-gas-turbines-southaven-colossus-2/); [DCD](https://www.datacenterdynamics.com/en/news/musks-xai-gets-go-ahead-for-41-natural-gas-turbines-in-mississippi-to-power-colossus-data-centers/)</t>
+          <t>[Technology.org](https://www.technology.org/2026/07/15/xai-59-unpermitted-gas-turbines-southaven-colossus-2/); [DCD](https://www.datacenterdynamics.com/en/news/musks-xai-gets-go-ahead-for-41-natural-gas-turbines-in-mississippi-to-power-colossus-data-centers/) ; [DCD](https://www.datacenterdynamics.com/en/news/musks-xai-gets-go-ahead-for-41-natural-gas-turbines-in-mississippi-to-power-colossus-data-centers/)</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -10029,17 +10297,17 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Construcción (campus de USD 3.6 mil millones/430MW, la mayor carga individual jamás atendida por Cleco; rompimiento de tierra ene-2026; operaciones iniciales objetivo mediados de 2027)</t>
+          <t>Construcción (campus de USD 3.6 mil millones/430MW, la mayor carga individual jamás atendida por Cleco; rompimiento de tierra ene-2026; operaciones iniciales objetivo mediados de 2027) ; Babcock &amp; Wilcox firmó Limited Notice to Proceed (LNTP) por un proyecto valuado en &gt;US$1,500 millones para diseñar e instalar 1 GW de generación adicional (cuatro plantas de 300 MW a gas natural con calderas y turbinas de vapor); contrato completo esperado 1T2026; arranque operativo 2028</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>[Data Center Dynamics](https://www.datacenterdynamics.com/en/news/cleco-to-construct-756mw-natural-gas-plant-to-serve-applied-digitals-data-center-in-rapides-parish-louisiana-report/)</t>
+          <t>[Data Center Dynamics](https://www.datacenterdynamics.com/en/news/cleco-to-construct-756mw-natural-gas-plant-to-serve-applied-digitals-data-center-in-rapides-parish-louisiana-report/) ; [Babcock &amp; Wilcox](https://www.babcock.com/home/about/corporate/news/babcock-and-wilcox-announces-ai-data-center-power-generation-solution-and-signs-lntp-with-applied-digital-to-design-and-install-one-gigawatt-of-electric-power)</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -10214,17 +10482,17 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Anuncio/desarrollo temprano (hasta 1.8GW; incluye nueva planta de gas natural de ~2GW y hasta 2.6GW de almacenamiento en baterías; ~US$100 mil millones de inversión privada total, el mayor proyecto de desarrollo económico en la historia de Kentucky)</t>
+          <t>Anuncio/desarrollo temprano (hasta 1.8GW; incluye nueva planta de gas natural de ~2GW y hasta 2.6GW de almacenamiento en baterías; ~US$100 mil millones de inversión privada total, el mayor proyecto de desarrollo económico en la historia de Kentucky) ; Brookfield y NextEra Energy lanzaron formalmente el campus en el sitio DOE de Paducah; &gt;US$100,000 millones de inversión privada; campus de IA de 1.8 GW respaldado por 2 GW de generación a gas natural nueva más hasta 2.6 GW de almacenamiento en baterías; ~8,000 empleos de construcción</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>[Bloomberg](https://www.bloomberg.com/news/articles/2026-07-29/nextera-brookfield-to-build-100-billion-kentucky-data-campus); [Kentucky Lantern](https://kentuckylantern.com/2026/07/29/hyperscale-data-center-natural-gas-fired-project-planned-for-paducahs-former-nuclear-plant/)</t>
+          <t>[Bloomberg](https://www.bloomberg.com/news/articles/2026-07-29/nextera-brookfield-to-build-100-billion-kentucky-data-campus); [Kentucky Lantern](https://kentuckylantern.com/2026/07/29/hyperscale-data-center-natural-gas-fired-project-planned-for-paducahs-former-nuclear-plant/) ; [Data Center Knowledge](https://www.datacenterknowledge.com/data-center-construction/brookfield-nextera-launch-100b-ai-campus-at-doe-s-paducah-site)</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -10547,17 +10815,17 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Construcción (primera inversión de la asociación estratégica ECP-KKR; campus de ~700,000 pies², inversión total cercana a US$4,000 millones, capacidad inicial de TI de 144MW sobre 190MW total; operación prevista 4T2026)</t>
+          <t>Construcción (primera inversión de la asociación estratégica ECP-KKR; campus de ~700,000 pies², inversión total cercana a US$4,000 millones, capacidad inicial de TI de 144MW sobre 190MW total; operación prevista 4T2026) ; Calpine/CyrusOne anunciaron Fase 2 del acuerdo de tierra energizada en el Thad Hill Energy Center, añadiendo 210 MW (total 400 MW); campus en construcción, operación prevista 4T2026</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>[Data Centre Magazine](https://datacentremagazine.com/news/ecp-and-kkr-to-build-4bn-190mw-hyperscale-data-centre); [Connect CRE](https://www.connectcre.com/stories/energy-capital-kkr-joint-forces-on-bosque-county-data-center/)</t>
+          <t>[Data Centre Magazine](https://datacentremagazine.com/news/ecp-and-kkr-to-build-4bn-190mw-hyperscale-data-centre); [Connect CRE](https://www.connectcre.com/stories/energy-capital-kkr-joint-forces-on-bosque-county-data-center/) ; [CyrusOne](https://www.cyrusone.com/resources/press-releases/calpine-and-cyrusone-announce-phase-2-of-powered-land-agreement-to-support-hyperscale-data-center-at-thad-hill-energy-center-in-texas)</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -10954,17 +11222,17 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Permitting temprano (solicitud de permiso de aire ante TCEQ presentada 10-ago-2026, hasta 2,409 MW dedicados; sitio de ~1,240 acres construibles; construcción proyectada primavera/verano 2027 si avanza; diputado estatal Drew Darby solicitó formalmente audiencia pública de TCEQ ante oposición vecinal)</t>
+          <t>Permitting temprano (solicitud de permiso de aire ante TCEQ presentada 10-ago-2026, hasta 2,409 MW dedicados; sitio de ~1,240 acres construibles; construcción proyectada primavera/verano 2027 si avanza; diputado estatal Drew Darby solicitó formalmente audiencia pública de TCEQ ante oposición vecinal) ; planta de energía asociada identificada como 'Westline 2335' (desarrollador Westline TX Holdings LLC, vinculado a Beacon Data Centers); solicitud de permiso TCEQ para 2,409 MW mediante 240 motores reciprocantes a gas en 20 'engine halls', cerca de San Angelo</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>[San Angelo Live](https://sanangelolive.com/news/san-angelo/2026-08-10/dove-creek-data-center-has-applied-tceq-permit-heres-what-know); [Concho Valley Homepage](https://www.conchovalleyhomepage.com/news/local-news/concho-valley-data-centers/darby-calls-for-clarity-from-beacon-data-centers-requests-public-tceq-meeting/)</t>
+          <t>[San Angelo Live](https://sanangelolive.com/news/san-angelo/2026-08-10/dove-creek-data-center-has-applied-tceq-permit-heres-what-know); [Concho Valley Homepage](https://www.conchovalleyhomepage.com/news/local-news/concho-valley-data-centers/darby-calls-for-clarity-from-beacon-data-centers-requests-public-tceq-meeting/) ; [San Angelo LIVE!](https://sanangelolive.com/news/san-angelo/2026-08-10/dove-creek-data-center-has-applied-tceq-permit-heres-what-know)</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
@@ -11409,6 +11677,80 @@
       <c r="G94" t="inlineStr">
         <is>
           <t>2026-08-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Nscale "Monarch Compute Campus"</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Point Pleasant, Condado de Mason, West Virginia, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Nscale (respaldada por Nvidia); Microsoft (arrendatario de 1.35 GW de cómputo)</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Caterpillar (motores de combustión interna a gas, ~2 GW)</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Planeación/desarrollo (campus de 2,250 acres planeado a 8 GW total; Fase 1 de 1.35 GW con entrega objetivo a inicios de 2028; microgrid fuera de red alimentado por gasoducto dedicado de gas Marcellus Shale)</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>[DCD](https://www.datacenterdynamics.com/en/news/nscale-acquires-8gw-monarch-compute-campus-microsoft-signs-on-for-135gw-of-compute/); [Latitude Media](https://www.latitudemedia.com/news/microsoft-is-embracing-off-grid-gas-for-west-virginia-data-centers/)</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Dominion Energy — Chesterfield Energy Reliability Center (CERC)</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Chesterfield, Virginia, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Dominion Energy (utility; impulsada por demanda de data centers regionales)</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Aprobado/planeación (State Corporation Commission de Virginia aprobó el proyecto; 944 MW —cuatro turbinas de gas de 250 MW—, costo ~US$1,470 millones, operación comercial prevista 2029; primera de seis plantas de gas planeadas por Dominion para atender demanda de data centers)</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>[POWER Magazine](https://www.powermag.com/dominion-seeks-virginia-approval-for-1-gw-gas-fired-power-plant/); [Virginia Mercury](https://virginiamercury.com/2025/11/25/scc-approves-chesterfield-gas-plant-and-dominion-rate-hike-creates-new-rate-class-for-data-centers/)</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitoreo 2026-08-28: 1 proyecto nuevo + 4 actualizaciones de fase
- Data Centers (1 nuevo): PORTS-Pike Technology Campus (Pike County, Ohio) — SB Energy/SoftBank con OpenAI de arrendatario ancla y NVIDIA, US$33,000 millones para 9.2 GW de generación a gas.
- LNG: CP2 LNG Fase 2 — Corte de Apelaciones del Circuito de D.C. confirmó por unanimidad las aprobaciones de FERC (25-ago-2026).
- Mining: Elk Creek Critical Minerals Project — incorporación de tecnología de acarreo Railveyor al plan de mina.
- Mining: Thacker Pass Lithium Mine (Fase I) — transición a oficios de tubería (piping) y eléctricos en la planta de proceso.
- Petroquímica: Planta de Amoniaco Topolobampo (GPO) — nueva gobernadora interina de Sinaloa se suma al diálogo con la comunidad mayo-yoreme.

Se regeneró proyectos.xlsx completo (54 Petroquímica, 45 LNG, 106 Mining, 96 Data Centers).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CPYpj9HhxRRYNQedZx6RMe
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Petroquimica" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Petroquímica" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="LNG" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Mining" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Data Centers" sheetId="4" state="visible" r:id="rId4"/>
@@ -20,18 +20,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <b val="1"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
@@ -57,9 +49,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -427,48 +418,39 @@
   </sheetPr>
   <dimension ref="A1:G55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -978,17 +960,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Construcción parcial/PAUSA parcial (unidad de amoniaco ~95% completa según Presidencia, ago-2026 —prensa local cita 88% de avance—, aunque reportes locales previos citaban solo ~60% con obra detenida por bloqueo; movimiento indígena yoreme-mayo "¡Aquí No!" mantiene plantón bloqueando el acceso de personal a la obra desde el 7-jun-2026; GPO ofreció (8/10-ago-2026) pausar formalmente las fases de urea, metanol y terminal marina como condición para levantar el bloqueo; Secretaría de Economía sostuvo reuniones con comunidades de Ohuira, Paredones, Lázaro Cárdenas y Topolobampo presentando el "Plan Integral", pero las comunidades respondieron con desconfianza y mantienen el plantón indefinido)</t>
+          <t>Construcción parcial/PAUSA parcial (unidad de amoniaco ~95% completa según Presidencia, ago-2026 —prensa local cita 88% de avance—, aunque reportes locales previos citaban solo ~60% con obra detenida por bloqueo; movimiento indígena yoreme-mayo "¡Aquí No!" mantiene plantón bloqueando el acceso de personal a la obra desde el 7-jun-2026; GPO ofreció (8/10-ago-2026) pausar formalmente las fases de urea, metanol y terminal marina como condición para levantar el bloqueo; Secretaría de Economía sostuvo reuniones con comunidades de Ohuira, Paredones, Lázaro Cárdenas y Topolobampo presentando el "Plan Integral", pero las comunidades respondieron con desconfianza y mantienen el plantón indefinido; nueva gobernadora interina de Sinaloa, Graciela Domínguez Nava, anunció el 26-ago-2026 que el gobierno estatal se sumará a la ruta federal de diálogo con la comunidad mayo-yoreme y GPO para destrabar el conflicto)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>[Ríodoce](https://riodoce.mx/2026/08/10/pausan-urea-y-metanol-pero-avanza-amoniaco-en-industria-en-la-bahia-de-ohuira/); [La Silla Rota](https://lasillarota.com/estados/2026/8/8/planta-de-amoniaco-en-sinaloa-gobierno-busca-luz-verde-al-proyecto-en-ohuira-523789.html); [Gobierno de Sinaloa](https://sinaloa.gob.mx/presentan-plan-integral-para-la-conservacion-ambiental-el-bienestar-comunitario-y-el-desarrollo-sostenible-de-la-bahia-de-ohuira/)</t>
+          <t>[Ríodoce](https://riodoce.mx/2026/08/10/pausan-urea-y-metanol-pero-avanza-amoniaco-en-industria-en-la-bahia-de-ohuira/); [La Silla Rota](https://lasillarota.com/estados/2026/8/8/planta-de-amoniaco-en-sinaloa-gobierno-busca-luz-verde-al-proyecto-en-ohuira-523789.html); [Infobae](https://www.infobae.com/mexico/2026/08/26/topolobampo-entre-las-prioridades-de-graciela-dominguez-promete-atender-a-comunidad-mayo-yoreme-y-a-empresarios/)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -2485,48 +2467,39 @@
   </sheetPr>
   <dimension ref="A1:G46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -2666,17 +2639,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Construcción (FID alcanzada mar-2026, NTP completo a Worley; Baker Hughes recibió pedido para suministrar 12 módulos de licuefacción, reportado semana del 20-26 jul-2026)</t>
+          <t>Construcción (FID alcanzada mar-2026, NTP completo a Worley; Baker Hughes recibió pedido para suministrar 12 módulos de licuefacción, reportado semana del 20-26 jul-2026; Corte de Apelaciones del Circuito de D.C. confirmó por unanimidad, 25-ago-2026, la aprobación de FERC para la terminal y el gasoducto asociado CP Express —91 millas—, rechazando 11 impugnaciones ambientalistas/pesqueras; construcción del proyecto de US$28,000 millones continúa sin interrupción; Venture Global solicita además ampliar capacidad en 11.7 MTPA adicionales)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>[GEM.wiki](https://www.gem.wiki/CP2_LNG_Terminal); [LNG Prime](https://lngprime.com/americas/top-5-news-of-the-week-july-20-26/193119/)</t>
+          <t>[GEM.wiki](https://www.gem.wiki/CP2_LNG_Terminal); [LNG Prime](https://lngprime.com/americas/top-5-news-of-the-week-july-20-26/193119/); [ENR](https://www.enr.com/articles/63562-appeals-court-upholds-federal-approvals-for-28b-cp2-lng-project)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -4210,48 +4183,39 @@
   </sheetPr>
   <dimension ref="A1:G107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -4391,7 +4355,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Construcción (reporte 2T2026: ingeniería de detalle &gt;95% completa, procura &gt;80% completa; US$1,800 millones de un capex total de US$2,930 millones ya incurridos; +1,600 trabajadores en sitio; comisionamiento anticipado de servicios previsto fines de 2026, terminación mecánica prevista fines de 2027) ; DOE aprobó préstamo de US$2,260 millones; ingeniería detallada 93% completa y procura 60% completa (fin de 2025); concreto principal del sitio se completaría en 3T2026, con comisionamiento inicial de plantas individuales desde 4T2026</t>
+          <t>Construcción (reporte 2T2026: ingeniería de detalle &gt;95% completa, procura &gt;80% completa; US$1,800 millones de un capex total de US$2,930 millones ya incurridos; +1,600 trabajadores en sitio; obra estructural/concreto de la planta de proceso avanzando con transición a oficios de tubería (piping) y eléctricos; comisionamiento anticipado de servicios previsto fines de 2026, terminación mecánica prevista fines de 2027; energización prevista 4T2026) ; DOE aprobó préstamo de US$2,260 millones; ingeniería detallada 93% completa y procura 60% completa (fin de 2025); concreto principal del sitio se completaría en 3T2026, con comisionamiento inicial de plantas individuales desde 4T2026</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -4401,7 +4365,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -5612,17 +5576,17 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Construcción (portal de mina de doble rampa, ~US$44.6 millones, iniciado feb/mar-2026; nuevo Feasibility Study NI 43-101 —publicado 11/15-ago-2026— amplía el proyecto a 8 productos, incluyendo óxidos de disprosio y terbio, VPN8% antes de impuestos US$4,100 millones, vida de mina de 40 años, capex inicial US$1,850 millones a 35 meses; MOU firmado con Lockheed Martin para venta de ~16.5 ton/año de escandio; Departamento de Defensa (programa DPA Title III) otorgó hasta US$10 millones a la subsidiaria Elk Creek Resources Corp. para desarrollo de producción de escandio, ago-2026; avanzando a ingeniería detallada, procura y contratación EPC; proyecto de niobio/escandio/titanio/tierras raras con planta de superficie que requerirá tubería de proceso)</t>
+          <t>Construcción (portal de mina de doble rampa, ~US$44.6 millones, iniciado feb/mar-2026; nuevo Feasibility Study NI 43-101 —publicado 11/15-ago-2026— amplía el proyecto a 8 productos, incluyendo óxidos de disprosio y terbio, VPN8% antes de impuestos US$4,100 millones, vida de mina de 40 años, capex inicial US$1,850 millones a 35 meses; MOU firmado con Lockheed Martin para venta de ~16.5 ton/año de escandio; Departamento de Defensa (programa DPA Title III) otorgó hasta US$10 millones a la subsidiaria Elk Creek Resources Corp. para desarrollo de producción de escandio, ago-2026; avanzando a ingeniería detallada, procura y contratación EPC; proyecto de niobio/escandio/titanio/tierras raras con planta de superficie que requerirá tubería de proceso; NioCorp incorporó tecnología de acarreo eléctrico Railveyor al plan de mina, confirmado 27-ago-2026)</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>[NioCorp](https://niocorp.com/niocorp-launches-construction-of-elk-creek-critical-minerals-project-mine-portal/); [Mining.com](https://www.mining.com/updated-feasibility-study-gives-niocorps-elk-creek-critical-minerals-project-a-4b-valuation/); [NioCorp DoD](https://www.niocorp.com/u-s-department-of-defense-awards-up-to-10-million-to-niocorps-subsidiary-elk-creek-resources-corp/)</t>
+          <t>[NioCorp](https://niocorp.com/niocorp-launches-construction-of-elk-creek-critical-minerals-project-mine-portal/); [Mining.com](https://www.mining.com/updated-feasibility-study-gives-niocorps-elk-creek-critical-minerals-project-a-4b-valuation/); [NioCorp DoD](https://www.niocorp.com/u-s-department-of-defense-awards-up-to-10-million-to-niocorps-subsidiary-elk-creek-resources-corp/); [Global Mining Review](https://www.globalminingreview.com/mining/27082026/niocorp-incorporates-railveyors-electric-haulage-technology-into-elk-creek-critical-minerals-project-plan/)</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
@@ -8190,50 +8154,41 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G96"/>
+  <dimension ref="A1:G97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -11751,6 +11706,43 @@
       <c r="G96" t="inlineStr">
         <is>
           <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>PORTS-Pike Technology Campus</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Pike County (sitio del antiguo Portsmouth/Piketon uranium enrichment), Ohio, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>SB Energy (subsidiaria de SoftBank); OpenAI (arrendatario ancla); NVIDIA (exclusividad de cómputo)</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>No especificado (participación del Dept. of Energy de EE.UU. en el sitio)</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Acuerdo firmado/pre-construcción (anunciado 17-ago-2026; inversión de US$33,000 millones para más de 9.2 GW de generación a gas natural, campus total de 10 GW/8 GW-IT, más US$4,000 millones en líneas de transmisión; primeros 800 MW esperados en 2028, buildout completo a 2032)</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>[OpenAI](https://openai.com/index/openai-joins-ports-pike-project/)</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Agrega 4 proyectos nuevos y actualiza 2 fases (1-sep-2026)
Nuevos: Port Arthur LNG North (Sempra, TX), Twin Metals Minnesota,
Falcon Copper fundición/refinería (Glencore MOU), NorthMark/Valara
Spartanburg Data Center (SC). Actualiza fase de Corpus Christi Stage 3
(terminación sustancial) y Stibnite Gold Project (confirmación judicial
y avance de construcción). Regenera proyectos.xlsx desde tracker.md.
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -20,10 +20,18 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
@@ -49,8 +57,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -418,39 +427,48 @@
   </sheetPr>
   <dimension ref="A1:G55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -2465,41 +2483,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G46"/>
+  <dimension ref="A1:G47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -2750,17 +2777,17 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Construcción (FERC autorizó introducción de gas combustible en Train 7, 17-jul-2026, y autorizó introducción de gas natural al Train 7, 28-jul-2026; FERC aprobó formalmente la introducción de gas natural al Train 7 —séptimo y último tren de la expansión midscale— el 4-ago-2026; Cheniere completó dos trenes adicionales de licuefacción en Stage 3 a mediados de ago-2026, elevando el avance del proyecto a ~98% completo; Train 7 en fase final de comisionamiento; finalización del build-out de 7 trenes prevista para fin de 2026)</t>
+          <t>Construcción/Terminación sustancial (FERC autorizó introducción de gas combustible en Train 7, 17-jul-2026, y autorizó introducción de gas natural al Train 7, 28-jul-2026; FERC aprobó formalmente la introducción de gas natural al Train 7 —séptimo y último tren de la expansión midscale— el 4-ago-2026; Cheniere completó dos trenes adicionales de licuefacción en Stage 3 a mediados de ago-2026, elevando el avance del proyecto a ~98% completo; Bechtel entregó formalmente el séptimo y último tren de licuefacción, terminación sustancial alcanzada 28-ago-2026, elevando la capacidad total de Cheniere a ~56 MTPA)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>[PGJ](https://pgjonline.com/news/2026/july/cheniere-gets-approval-to-introduce-gas-into-final-corpus-christi-lng-train); [OGJ](https://www.ogj.com/pipelines-transportation/lng/news/55340460/cheniere-completes-two-more-corpus-christi-stage-3-trains); [LNG Prime](https://lngprime.com/americas/chenieres-corpus-christi-stage-3-project-98-percent-complete/190871/)</t>
+          <t>[PGJ](https://pgjonline.com/news/2026/july/cheniere-gets-approval-to-introduce-gas-into-final-corpus-christi-lng-train); [OGJ](https://www.ogj.com/pipelines-transportation/lng/news/55340460/cheniere-completes-two-more-corpus-christi-stage-3-trains); [LNG Prime](https://lngprime.com/americas/chenieres-corpus-christi-stage-3-project-98-percent-complete/190871/); [Upstream](https://www.upstreamonline.com/lng/us-lng-exporter-crosses-finish-line-for-texas-expansion-project/2-1-2036962)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
@@ -4167,6 +4194,43 @@
       <c r="G46" t="inlineStr">
         <is>
           <t>2026-08-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Port Arthur LNG North (expansión brownfield, Trenes 5-8)</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Port Arthur, Texas, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Sempra Infrastructure (Sempra PALNG)</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>No adjudicado (fase temprana)</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Permitting (pre-filing FERC iniciado 31-ago-2026; ~27 MTPA adicionales vía 4 nuevos trenes, 3 tanques y 2 muelles marinos nuevos, usará el gasoducto Texas Connector Pipeline existente sin nueva alimentación; solicitud formal ante FERC esperada jul-2027, decisión FERC ~jul-2028, inicio de construcción estimado 2S-2029)</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>[LNG Industry](https://www.lngindustry.com/liquefaction/31082026/sempra-submits-ferc-pre-filing-for-port-arthur-lng-north/); [LNG Prime](https://lngprime.com/americas/sempra-infrastructure-plans-27-mtpa-port-arthur-lng-expansion/195837/); [BIC Magazine](https://www.bicmagazine.com/projects-expansions/midstream/sempra-begins-permitting-for-port-arthur-lng/)</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
@@ -4181,41 +4245,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G107"/>
+  <dimension ref="A1:G109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -4651,17 +4724,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Construcción (corte federal de Idaho negó en jun-2026 moción para detener obras; Directorio del Export-Import Bank de EE.UU. aprobó por unanimidad, 20-ago-2026, el préstamo garantizado senior de USD 2,900 millones para financiar el desarrollo; nuevos objetivos de exploración de oro/antimonio de alta ley identificados y posible nueva fuente de tungsteno reportados 7-ago-2026)</t>
+          <t>Construcción (corte federal de Idaho negó en jun-2026 moción para detener obras; Directorio del Export-Import Bank de EE.UU. aprobó por unanimidad, 20-ago-2026, el préstamo garantizado senior de USD 2,900 millones para financiar el desarrollo; nuevos objetivos de exploración de oro/antimonio de alta ley identificados y posible nueva fuente de tungsteno reportados 7-ago-2026; Corte Federal de Distrito de Idaho confirmó 18-ago-2026 las aprobaciones federales del USFS ante impugnación ambiental —apelación pendiente no detiene la obra—; Perpetua confirmó mediante actualización de construcción, 31-ago-2026, que el trabajo temprano continúa avanzando hacia FID, con primer oro previsto 2029)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/perpetua-resources-advances-construction-of-the-stibnite-gold-project-302787012.html); [Departamento de Justicia de EE.UU.](https://www.justice.gov/opa/pr/justice-department-secures-motion-allow-continued-construction-idaho-gold-mine-critical); [StreetWise Reports](https://www.streetwisereports.com/article/2026/08/20/idaho-gold-antimony-developer-wins-2-9b-exim-loan-approval.html)</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/perpetua-resources-advances-construction-of-the-stibnite-gold-project-302787012.html); [Departamento de Justicia de EE.UU.](https://www.justice.gov/opa/pr/justice-department-secures-motion-allow-continued-construction-idaho-gold-mine-critical); [StreetWise Reports](https://www.streetwisereports.com/article/2026/08/20/idaho-gold-antimony-developer-wins-2-9b-exim-loan-approval.html); [Northern Miner](https://www.northernminer.com/news/court-ruling-backs-perpetuas-1-3b-stibnite-build/1003894465/); [PRNewswire](https://www.prnewswire.com/news-releases/perpetua-resources-provides-construction-update-on-the-stibnite-gold-project-and-exploration-activities-302864546.html)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
@@ -8140,6 +8213,80 @@
       <c r="G107" t="inlineStr">
         <is>
           <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Twin Metals Minnesota</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Ely, Minnesota, EE.UU. (cerca de Boundary Waters)</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Antofagasta plc (Twin Metals Minnesota LLC)</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>No definido</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Permitting/Pre-EIS (plan de mina formal —concentradora de flotación de 20,000 tpd, cobre-níquel-EGP— presentado ante BLM y Minnesota DNR; el gobernador Walz frenó el trámite estatal en ago-2026, pero el proceso federal continúa activo; construcción aún a años de distancia)</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>[MinnPost](http://www.minnpost.com/state-government/2026/08/walz-halts-state-action-on-mine-near-boundary-waters-but-federal-process-stays-on-track/); [Star Tribune](https://www.startribune.com/twin-metals-submits-formal-mine-plan-to-minnesota-federal-officials/566311242)</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Falcon Copper — Fundición y Refinería de Cobre (greenfield)</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Arizona (fundición) / Costa del Golfo (refinería), EE.UU. (sitios por definir)</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Falcon Copper Corp. (MOU con Glencore)</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>No definido</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Evaluación/pre-FEED (proyecto greenfield de ~US$2,000 millones para fundición primaria de cobre más refinería electrolítica; sin sitio definitivo ni FID)</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>[Fastmarkets](https://www.fastmarkets.com/insights/us-copper-smelting-equation-gap-or-glut-hotter-commodities-articles/); [Falcon Copper](https://www.falconcopper.com/projects/works)</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
@@ -8154,41 +8301,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G97"/>
+  <dimension ref="A1:G98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Cliente/Dueño</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>EPC/Contratista</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Última actualización</t>
         </is>
@@ -11743,6 +11899,43 @@
       <c r="G97" t="inlineStr">
         <is>
           <t>2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>NorthMark/Valara Spartanburg Data Center Campus</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Spartanburg County, Carolina del Sur, EE.UU. (antigua planta Kohler)</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>NorthMark Strategies / Valara Holdings</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Permitting favorable/desarrollo temprano (Comisión de Servicios Públicos de Carolina del Sur dictaminó 27-ago-2026 que el proyecto no está sujeto a regulación de utility pública, despejando el camino para autogeneración behind-the-meter de 450+ MW en turbinas de gas, ampliando el permiso inicial de 48 MW; complejo de cómputo de US$2,800 millones; primera etapa operativa prevista 3T2026, construcción hasta 2028)</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>[SC Daily Gazette](https://scdailygazette.com/2026/08/27/spartanburg-data-center-not-subject-to-public-power-plant-rules-sc-regulators-rule/); [Post and Courier](https://www.postandcourier.com/spartanburg/news/spartanburg-data-center-northmark-water-power/article_07cc2de8-9eb6-4711-ad7f-90ef8230b158.html)</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitoreo 2026-09-03: 2 proyectos nuevos + 2 actualizaciones de fase
- Nuevos: Spring Valley Gold Mine (NV), Pitarrilla Project (Durango)
- Actualizaciones: Plaquemines LNG Fase 2 (gasoducto Delta Access de
  Williams), Planta de Purificación de Grafito US Army (sitio primario
  confirmado en Pine Bluff Arsenal)
- proyectos.xlsx regenerado con el acumulado completo (309 proyectos)

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013AGyaisBCeoWfGs74eCHnn
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -54,9 +54,7 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -425,16 +423,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G56"/>
+  <dimension ref="A1:G55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -810,276 +808,276 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Proyecto Escolín (amoniaco/urea)</t>
+          <t>Rehab. Fertinal-ProAgro (urea y fosfatos)</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Poza Rica, Veracruz, México</t>
+          <t>Lázaro Cárdenas, Michoacán, México</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Pemex Transformación Industrial</t>
+          <t>Pemex</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Mota-Engil México (EPC confirmado, US$1,200 millones, 47 meses); Duro Felguera (España) se integró formalmente 17-ago-2026 al contrato para gestión de proyecto y coordinación técnica de la ingeniería (supervisión de ingeniería externa, coordinación de suministros del tecnólogo, gestión de sistemas auxiliares); Casale (proveedor de tecnología)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/inicio de construcción (inversión confirmada US$1,553 millones; capacidad objetivo &gt;700,000 ton/año de amoniaco, urea y AdBlue; citado explícitamente por la Presidenta Sheinbaum en su Segundo Informe de Gobierno —1-sep-2026— como parte del "rescate de la petroquímica" junto con Cosoleacaque, Morelos y Cangrejera)</t>
+          <t>Ingeniería/rehabilitación (incorporado al plan de reactivación petroquímica de Pemex, jun-2026; 13,700 millones de pesos asignados para los complejos Lázaro Cárdenas y ProAgro; meta de 2.4 millones ton/año de urea y fertilizantes fosfatados)</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>[Forbes México](https://forbes.com.mx/asi-es-la-inversion-de-1553-mdd-por-parte-de-pemex-en-una-planta-de-fertilizantes-en-veracruz/); [El Español](https://www.elespanol.com/invertia/empresas/energia/20260817/duro-felguera-convoca-junta-extraordinaria-septiembre-aprobar-proyecto-clave-mota-engil-mexico/1003744355543_0.html); [La Política en Rosa](https://www.lapoliticaenrosa.com/2026/09/01/desde-veracruz-inicia-rescate-de-petroquimica-del-pais-destaca-claudia-sheinbaum-en-segundo-informe-de-gobierno/)</t>
+          <t>[Tribuna](https://tribuna.com.mx/mexico/2026/06/05/sheinbaum-anuncia-inversion-de-93-mil-mdp-para-reactivar-la-industria-petroquimica-y-de-fertilizantes-en-veracruz_560837/); [Contralínea](https://contralinea.com.mx/interno/semana/presentan-plan-con-inversion-de-93-mil-mdp-para-rescatar-la-petroquimica-nacional/)</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Rehab. Fertinal-ProAgro (urea y fosfatos)</t>
+          <t>Pacífico Mexinol (metanol ultra bajo carbono)</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Lázaro Cárdenas, Michoacán, México</t>
+          <t>Topolobampo, Sinaloa, México</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Pemex</t>
+          <t>Transition Industries</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Siemens Energy / Techint E&amp;C (FEED electrolizador)</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/rehabilitación (incorporado al plan de reactivación petroquímica de Pemex, jun-2026; 13,700 millones de pesos asignados para los complejos Lázaro Cárdenas y ProAgro; meta de 2.4 millones ton/año de urea y fertilizantes fosfatados)</t>
+          <t>Construcción (iniciada abr-2026)</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>[Tribuna](https://tribuna.com.mx/mexico/2026/06/05/sheinbaum-anuncia-inversion-de-93-mil-mdp-para-reactivar-la-industria-petroquimica-y-de-fertilizantes-en-veracruz_560837/); [Contralínea](https://contralinea.com.mx/interno/semana/presentan-plan-con-inversion-de-93-mil-mdp-para-rescatar-la-petroquimica-nacional/)</t>
+          <t>[PV Magazine México](https://www.pv-magazine-mexico.com/2026/04/28/inician-en-sinaloa-la-construccion-de-la-mayor-planta-de-metanol-ultrabajo-en-carbono-a-partir-de-hidrogeno-verde/)</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-10</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Pacífico Mexinol (metanol ultra bajo carbono)</t>
+          <t>First Ammonia (amoniaco verde)</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Topolobampo, Sinaloa, México</t>
+          <t>Victoria, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Transition Industries</t>
+          <t>First Ammonia / Cox Group USA</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Siemens Energy / Techint E&amp;C (FEED electrolizador)</t>
+          <t>Worley (FEED); Topsoe (tecnología de síntesis de amoniaco, seleccionada 12-ago-2026)</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Construcción (iniciada abr-2026)</t>
+          <t>Ingeniería (FEED completo; Topsoe suministrará su tecnología dinámica de síntesis de amoniaco) / cierre financiero esperado en 2026, FID prevista 2026, operación comercial estimada 2029</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>[PV Magazine México](https://www.pv-magazine-mexico.com/2026/04/28/inician-en-sinaloa-la-construccion-de-la-mayor-planta-de-metanol-ultrabajo-en-carbono-a-partir-de-hidrogeno-verde/)</t>
+          <t>[H2 View](https://www.h2-view.com/story/first-ammonia-project-on-track-for-2026-fid-despite-topsoe-deal-collapse/2138792.article/); [World Fertilizer](https://www.worldfertilizer.com/project-news/12082026/topsoe-to-provide-technology-for-first-ammonia/); [Topsoe](https://www.topsoe.com/news/topsoe-to-provide-ammonia-technology-for-first-ammonias-green-ammonia-project-in-texas)</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-08-20</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>First Ammonia (amoniaco verde)</t>
+          <t>Planta de Amoniaco Topolobampo (GPO) — Bahía de Ohuira</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Victoria, Texas, EE.UU.</t>
+          <t>Topolobampo, Ahome, Sinaloa, México</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>First Ammonia / Cox Group USA</t>
+          <t>Gas y Petroquímica de Occidente (GPO) / Proman AG</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Worley (FEED); Topsoe (tecnología de síntesis de amoniaco, seleccionada 12-ago-2026)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería (FEED completo; Topsoe suministrará su tecnología dinámica de síntesis de amoniaco) / cierre financiero esperado en 2026, FID prevista 2026, operación comercial estimada 2029</t>
+          <t>Construcción parcial/PAUSA parcial (unidad de amoniaco ~95% completa según Presidencia, ago-2026 —prensa local cita 88% de avance—, aunque reportes locales previos citaban solo ~60% con obra detenida por bloqueo; movimiento indígena yoreme-mayo "¡Aquí No!" mantiene plantón bloqueando el acceso de personal a la obra desde el 7-jun-2026; GPO ofreció (8/10-ago-2026) pausar formalmente las fases de urea, metanol y terminal marina como condición para levantar el bloqueo; Secretaría de Economía sostuvo reuniones con comunidades de Ohuira, Paredones, Lázaro Cárdenas y Topolobampo presentando el "Plan Integral", pero las comunidades respondieron con desconfianza y mantienen el plantón indefinido; nueva gobernadora interina de Sinaloa, Graciela Domínguez Nava, anunció el 26-ago-2026 que el gobierno estatal se sumará a la ruta federal de diálogo con la comunidad mayo-yoreme y GPO para destrabar el conflicto)</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>[H2 View](https://www.h2-view.com/story/first-ammonia-project-on-track-for-2026-fid-despite-topsoe-deal-collapse/2138792.article/); [World Fertilizer](https://www.worldfertilizer.com/project-news/12082026/topsoe-to-provide-technology-for-first-ammonia/); [Topsoe](https://www.topsoe.com/news/topsoe-to-provide-ammonia-technology-for-first-ammonias-green-ammonia-project-in-texas)</t>
+          <t>[Ríodoce](https://riodoce.mx/2026/08/10/pausan-urea-y-metanol-pero-avanza-amoniaco-en-industria-en-la-bahia-de-ohuira/); [La Silla Rota](https://lasillarota.com/estados/2026/8/8/planta-de-amoniaco-en-sinaloa-gobierno-busca-luz-verde-al-proyecto-en-ohuira-523789.html); [Infobae](https://www.infobae.com/mexico/2026/08/26/topolobampo-entre-las-prioridades-de-graciela-dominguez-promete-atender-a-comunidad-mayo-yoreme-y-a-empresarios/)</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Planta de Amoniaco Topolobampo (GPO) — Bahía de Ohuira</t>
+          <t>Lake Charles Methanol II</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Topolobampo, Ahome, Sinaloa, México</t>
+          <t>Lake Charles, Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Gas y Petroquímica de Occidente (GPO) / Proman AG</t>
+          <t>Lake Charles Methanol II LLC</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Zachry Group (FEED)</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Construcción parcial/PAUSA parcial (unidad de amoniaco ~95% completa según Presidencia, ago-2026 —prensa local cita 88% de avance—, aunque reportes locales previos citaban solo ~60% con obra detenida por bloqueo; movimiento indígena yoreme-mayo "¡Aquí No!" mantiene plantón bloqueando el acceso de personal a la obra desde el 7-jun-2026; GPO ofreció (8/10-ago-2026) pausar formalmente las fases de urea, metanol y terminal marina como condición para levantar el bloqueo; Secretaría de Economía sostuvo reuniones con comunidades de Ohuira, Paredones, Lázaro Cárdenas y Topolobampo presentando el "Plan Integral", pero las comunidades respondieron con desconfianza y mantienen el plantón indefinido; nueva gobernadora interina de Sinaloa, Graciela Domínguez Nava, anunció el 26-ago-2026 que el gobierno estatal se sumará a la ruta federal de diálogo con la comunidad mayo-yoreme y GPO para destrabar el conflicto)</t>
+          <t>Ingeniería (FEED) / FID prevista</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>[Ríodoce](https://riodoce.mx/2026/08/10/pausan-urea-y-metanol-pero-avanza-amoniaco-en-industria-en-la-bahia-de-ohuira/); [La Silla Rota](https://lasillarota.com/estados/2026/8/8/planta-de-amoniaco-en-sinaloa-gobierno-busca-luz-verde-al-proyecto-en-ohuira-523789.html); [Infobae](https://www.infobae.com/mexico/2026/08/26/topolobampo-entre-las-prioridades-de-graciela-dominguez-promete-atender-a-comunidad-mayo-yoreme-y-a-empresarios/)</t>
+          <t>[ICIS](https://www.icis.com/explore/resources/news/2025/11/13/11155109/lake-charles-methanol-ii-awards-feed-fid-expected-in-q2-2026/)</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Lake Charles Methanol II</t>
+          <t>Planta Coquizadora Salina Cruz</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Lake Charles, Luisiana, EE.UU.</t>
+          <t>Salina Cruz, Oaxaca, México</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Lake Charles Methanol II LLC</t>
+          <t>Pemex</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Zachry Group (FEED)</t>
+          <t>ICA Fluor</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería (FEED) / FID prevista</t>
+          <t>Construcción (~74% avance; Pemex confirmó retraso en el cronograma, finalización ahora prevista para 2S2027; avance reafirmado por la Presidenta Sheinbaum en su Segundo Informe de Gobierno, 1-sep-2026, como parte del programa de rehabilitación del Sistema Nacional de Refinación)</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>[ICIS](https://www.icis.com/explore/resources/news/2025/11/13/11155109/lake-charles-methanol-ii-awards-feed-fid-expected-in-q2-2026/)</t>
+          <t>[Diario del Istmo](https://diariodelistmo.com/nacional/este-es-el-avance-que-lleva-la-planta-coquizadora-en-la-refineria-de-salina-cruz/50642321); [Mexico Business News](https://mexicobusiness.news/oilandgas/news/salina-cruz-refinery-miss-construction-deadline-pemex); [La Razón](https://www.razon.com.mx/negocios/2026/09/01/sheinbaum-destaca-reduccion-de-deuda-de-pemex-y-avances-en-soberania-energetica/)</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-09-02</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Planta Coquizadora Salina Cruz</t>
+          <t>Shintech Louisiana — Expansión Plaquemine (2do craqueador de etileno + 4ta unidad cloro-álcali/VCM)</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Salina Cruz, Oaxaca, México</t>
+          <t>Plaquemine, Iberville Parish, Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Pemex</t>
+          <t>Shintech Louisiana, LLC</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>ICA Fluor</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Construcción (~74% avance; Pemex confirmó retraso en el cronograma, finalización ahora prevista para 2S2027; avance reafirmado por la Presidenta Sheinbaum en su Segundo Informe de Gobierno, 1-sep-2026, como parte del programa de rehabilitación del Sistema Nacional de Refinación)</t>
+          <t>Ingeniería/planeación (construcción por fases, 1a fase prevista 2030)</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>[Diario del Istmo](https://diariodelistmo.com/nacional/este-es-el-avance-que-lleva-la-planta-coquizadora-en-la-refineria-de-salina-cruz/50642321); [Mexico Business News](https://mexicobusiness.news/oilandgas/news/salina-cruz-refinery-miss-construction-deadline-pemex); [La Razón](https://www.razon.com.mx/negocios/2026/09/01/sheinbaum-destaca-reduccion-de-deuda-de-pemex-y-avances-en-soberania-energetica/)</t>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/petrochemicals/06032026/shintech-announces-us34-billion-at-louisiana-petrochemicals-complex/)</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-07-14</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Shintech Louisiana — Expansión Plaquemine (2do craqueador de etileno + 4ta unidad cloro-álcali/VCM)</t>
+          <t>Sandpiper Chemicals (metanol bajo carbono)</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Plaquemine, Iberville Parish, Luisiana, EE.UU.</t>
+          <t>Texas City, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Shintech Louisiana, LLC</t>
+          <t>Sandpiper Chemicals, LLC / INEOS Acetyls (colaboración estratégica, abr-2026)</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -1089,86 +1087,86 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/planeación (construcción por fases, 1a fase prevista 2030)</t>
+          <t>Ingeniería (FEED en curso desde 2T2026; US$1,700 millones, 1.1 MMtpa; INEOS Acetyls tomará 300,000 ton/año para su unidad de ácido acético) / FID prevista 2027, primera producción ~2030</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/petrochemicals/06032026/shintech-announces-us34-billion-at-louisiana-petrochemicals-complex/)</t>
+          <t>[INEOS](https://www.ineos.com/news/shared-news/ineos-acetyls-and-sandpiper-chemicals-announce-strategic-collaboration-for-the-development-of-a-low-carbon-methanol-project-in-texas-city-texas/)</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-29</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Sandpiper Chemicals (metanol bajo carbono)</t>
+          <t>OXEA Bay City Capacity Expansion + Air Liquide POX Syngas Unit</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Texas City, Texas, EE.UU.</t>
+          <t>Bay City, Matagorda County, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Sandpiper Chemicals, LLC / INEOS Acetyls (colaboración estratégica, abr-2026)</t>
+          <t>OXEA (oxo chemicals) / Air Liquide (unidad de syngas)</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Air Liquide (unidad propia); OXEA no especificado</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería (FEED en curso desde 2T2026; US$1,700 millones, 1.1 MMtpa; INEOS Acetyls tomará 300,000 ton/año para su unidad de ácido acético) / FID prevista 2027, primera producción ~2030</t>
+          <t>Construcción (FID confirmado 13-jul-2026; preparación de sitio 3T2026; finalización fines de 2028)</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>[INEOS](https://www.ineos.com/news/shared-news/ineos-acetyls-and-sandpiper-chemicals-announce-strategic-collaboration-for-the-development-of-a-low-carbon-methanol-project-in-texas-city-texas/)</t>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/petrochemicals/13072026/oxea-confirms-fid-for-major-capacity-expansion/)</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>OXEA Bay City Capacity Expansion + Air Liquide POX Syngas Unit</t>
+          <t>Targa Resources East Driver Gas Processing Plant</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Bay City, Matagorda County, Texas, EE.UU.</t>
+          <t>Condado de Midland, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>OXEA (oxo chemicals) / Air Liquide (unidad de syngas)</t>
+          <t>Targa Resources Corp.</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Air Liquide (unidad propia); OXEA no especificado</t>
+          <t>Targa Resources (propietario-constructor)</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Construcción (FID confirmado 13-jul-2026; preparación de sitio 3T2026; finalización fines de 2028)</t>
+          <t>Construcción (planta criogénica 275 MMcf/d; arranque previsto 3T2026)</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/petrochemicals/13072026/oxea-confirms-fid-for-major-capacity-expansion/)</t>
+          <t>[OGJ](https://www.ogj.com/refining-processing/gas-processing/news/55320579/targa-advances-permian-gas-pipeline-processing-expansion)</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -1180,32 +1178,32 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Targa Resources East Driver Gas Processing Plant</t>
+          <t>Enterprise Products "Athena" Natural Gas Processing Plant</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Condado de Midland, Texas, EE.UU.</t>
+          <t>Cuenca Midland (cuatro condados), Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Targa Resources Corp.</t>
+          <t>Enterprise Products Partners L.P.</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Targa Resources (propietario-constructor)</t>
+          <t>Enterprise Products (propietario-constructor)</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Construcción (planta criogénica 275 MMcf/d; arranque previsto 3T2026)</t>
+          <t>Construcción (300 MMcf/d + hasta 40,000 bpd de NGLs; en servicio 4T2026)</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>[OGJ](https://www.ogj.com/refining-processing/gas-processing/news/55320579/targa-advances-permian-gas-pipeline-processing-expansion)</t>
+          <t>[Business Wire](https://www.businesswire.com/news/home/20250806663187/en/Enterprise-Agrees-to-Acquire-Occidentals-Gas-Gathering-Affiliate-Enters-Into-Natural-Gas-Processing-Agreement-Announces-New-Midland-Basin-Natural-Gas-Processing-Plant)</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -1217,32 +1215,32 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Enterprise Products "Athena" Natural Gas Processing Plant</t>
+          <t>MPLX Secretariat II Gas Processing Plant</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Cuenca Midland (cuatro condados), Texas, EE.UU.</t>
+          <t>Cuenca Pérmica (subcuenca Delaware), Texas/Nuevo México, EE.UU.</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Enterprise Products Partners L.P.</t>
+          <t>MPLX LP</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Enterprise Products (propietario-constructor)</t>
+          <t>MPLX (propietario-constructor)</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Construcción (300 MMcf/d + hasta 40,000 bpd de NGLs; en servicio 4T2026)</t>
+          <t>Planeada/desarrollo (300 MMcf/d; en servicio 2S2028)</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>[Business Wire](https://www.businesswire.com/news/home/20250806663187/en/Enterprise-Agrees-to-Acquire-Occidentals-Gas-Gathering-Affiliate-Enters-Into-Natural-Gas-Processing-Agreement-Announces-New-Midland-Basin-Natural-Gas-Processing-Plant)</t>
+          <t>[Natural Gas Intel](https://naturalgasintel.com/news/mplx-scales-up-for-power-hungry-future-with-natural-gas-focused-growth-plan/)</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -1254,12 +1252,12 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>MPLX Secretariat II Gas Processing Plant</t>
+          <t>MPLX Titan Complex (Northwind) — Expansión de Tratamiento de Gas Amargo</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Cuenca Pérmica (subcuenca Delaware), Texas/Nuevo México, EE.UU.</t>
+          <t>Condado de Lea, Nuevo México / frontera TX-NM, EE.UU.</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -1274,12 +1272,12 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Planeada/desarrollo (300 MMcf/d; en servicio 2S2028)</t>
+          <t>Construcción (expansión de capacidad &gt;400 MMcf/d; plenamente operativo 4T2026)</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>[Natural Gas Intel](https://naturalgasintel.com/news/mplx-scales-up-for-power-hungry-future-with-natural-gas-focused-growth-plan/)</t>
+          <t>[East Daley](https://eastdaley.com/daley-note/mplx-acquires-northwind-for-2-375b-acquires-more-ngls-for-jv-project)</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -1291,32 +1289,32 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>MPLX Titan Complex (Northwind) — Expansión de Tratamiento de Gas Amargo</t>
+          <t>Northern Plains Nitrogen (urea/amoniaco)</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Condado de Lea, Nuevo México / frontera TX-NM, EE.UU.</t>
+          <t>Grand Forks, Dakota del Norte, EE.UU.</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>MPLX LP</t>
+          <t>Northern Plains Nitrogen LLC</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>MPLX (propietario-constructor)</t>
+          <t>EPC no designado</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Construcción (expansión de capacidad &gt;400 MMcf/d; plenamente operativo 4T2026)</t>
+          <t>Pre-FEED completo / FID buscada 4T2026</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>[East Daley](https://eastdaley.com/daley-note/mplx-acquires-northwind-for-2-375b-acquires-more-ngls-for-jv-project)</t>
+          <t>[Grand Forks Herald](https://www.grandforksherald.com/news/local/northern-plains-nitrogen-proposal-receiving-more-attention-amid-global-fertilizer-pressure)</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -1328,54 +1326,54 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Northern Plains Nitrogen (urea/amoniaco)</t>
+          <t>Iron Mesa (planta de gas)</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Grand Forks, Dakota del Norte, EE.UU.</t>
+          <t>Goldsmith, Ector County, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Northern Plains Nitrogen LLC</t>
+          <t>Phillips 66</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>EPC no designado</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Pre-FEED completo / FID buscada 4T2026</t>
+          <t>Construcción (arranque previsto Q1 2027)</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>[Grand Forks Herald](https://www.grandforksherald.com/news/local/northern-plains-nitrogen-proposal-receiving-more-attention-amid-global-fertilizer-pressure)</t>
+          <t>[Phillips 66](https://www.phillips66.com/newsroom/iron-mesa-safely-enters-next-phase-of-construction/)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-15</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Iron Mesa (planta de gas)</t>
+          <t>Yeti II (planta de gas)</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Goldsmith, Ector County, Texas, EE.UU.</t>
+          <t>Cuenca Delaware (Permian), Texas/Nuevo México, EE.UU.</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Phillips 66</t>
+          <t>Targa Resources</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1385,12 +1383,12 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Construcción (arranque previsto Q1 2027)</t>
+          <t>Ingeniería/planeación (en línea previsto Q4 2027)</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>[Phillips 66](https://www.phillips66.com/newsroom/iron-mesa-safely-enters-next-phase-of-construction/)</t>
+          <t>[Targa Resources](https://www.targaresources.com/news-releases/news-release-details/targa-resources-corp-announces-permian-growth-projects-and)</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -1402,32 +1400,32 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Yeti II (planta de gas)</t>
+          <t>Refinería Francisco I. Madero (rehabilitación)</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Cuenca Delaware (Permian), Texas/Nuevo México, EE.UU.</t>
+          <t>Ciudad Madero, Tamaulipas, México</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Targa Resources</t>
+          <t>Pemex</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Múltiples contratistas por licitar (30+ licitaciones)</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/planeación (en línea previsto Q4 2027)</t>
+          <t>Licitación/bidding</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>[Targa Resources](https://www.targaresources.com/news-releases/news-release-details/targa-resources-corp-announces-permian-growth-projects-and)</t>
+          <t>[Elefante Blanco](https://elefanteblanco.mx/2026/01/02/pemex-abre-30-licitaciones-para-obras-en-la-refineria-madero/)</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -1439,106 +1437,106 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Refinería Francisco I. Madero (rehabilitación)</t>
+          <t>Fermachem Planta de Urea/Amoniaco</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Ciudad Madero, Tamaulipas, México</t>
+          <t>Ejido Sapioris, Lerdo, Durango, México</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Pemex</t>
+          <t>Fermaca Dreams (Fermachem)</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Múltiples contratistas por licitar (30+ licitaciones)</t>
+          <t>Técnicas Reunidas (licencia/tecnología KBR-Stamicarbon)</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Licitación/bidding</t>
+          <t>Construcción con retraso administrativo (obra pausada ~mes y medio por revisión legal/administrativa; Secretario de Desarrollo Económico de Durango confirmó 13-ago-2026 que Semarnat y Profepa no encontraron impedimento, reanudación de obra esperada en 1-2 semanas)</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>[Elefante Blanco](https://elefanteblanco.mx/2026/01/02/pemex-abre-30-licitaciones-para-obras-en-la-refineria-madero/)</t>
+          <t>[La Jornada](https://www.jornada.com.mx/noticia/2026/06/08/economia/da-inicio-ejecucion-de-planta-de-fertilizantes-en-durango-por-parte-de-fermachem); [Grem Noticieros](https://www.noticierosgrem.com.mx/costruccion-de-fermachem-podria-arrancar-en-dos-semanas-desarrollo-economico-de-durango/)</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-08-18</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Fermachem Planta de Urea/Amoniaco</t>
+          <t>Ascension Clean Energy (ACE) — amoniaco azul</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Ejido Sapioris, Lerdo, Durango, México</t>
+          <t>Donaldsonville, Ascension Parish, Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Fermaca Dreams (Fermachem)</t>
+          <t>Clean Hydrogen Works</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Técnicas Reunidas (licencia/tecnología KBR-Stamicarbon)</t>
+          <t>McDermott (FEED)</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Construcción con retraso administrativo (obra pausada ~mes y medio por revisión legal/administrativa; Secretario de Desarrollo Económico de Durango confirmó 13-ago-2026 que Semarnat y Profepa no encontraron impedimento, reanudación de obra esperada en 1-2 semanas)</t>
+          <t>Ingeniería (FEED) / Pre-FID</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>[La Jornada](https://www.jornada.com.mx/noticia/2026/06/08/economia/da-inicio-ejecucion-de-planta-de-fertilizantes-en-durango-por-parte-de-fermachem); [Grem Noticieros](https://www.noticierosgrem.com.mx/costruccion-de-fermachem-podria-arrancar-en-dos-semanas-desarrollo-economico-de-durango/)</t>
+          <t>[Downstream Calendar](https://downstreamcalendar.com/mcdermott-secures-feed-contract-for-ascension-clean-energy-project/)</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-07-17</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Ascension Clean Energy (ACE) — amoniaco azul</t>
+          <t>Zeus Gas Plant + 3ra Fraccionadora Coastal Bend</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Donaldsonville, Ascension Parish, Luisiana, EE.UU.</t>
+          <t>Cuenca Pérmica, Texas / Robstown, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Clean Hydrogen Works</t>
+          <t>Phillips 66</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>McDermott (FEED)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería (FEED) / Pre-FID</t>
+          <t>Ingeniería (sancionado; en línea 2028)</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>[Downstream Calendar](https://downstreamcalendar.com/mcdermott-secures-feed-contract-for-ascension-clean-energy-project/)</t>
+          <t>[Business Wire](https://www.businesswire.com/news/home/20260517310811/en/Phillips-66-announces-Zeus-Gas-Plant-and-a-third-Coastal-Bend-Fractionator)</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -1550,128 +1548,128 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Zeus Gas Plant + 3ra Fraccionadora Coastal Bend</t>
+          <t>Project Meadowlark (complejo de amoniaco azul/UAN/ATS/DEF)</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Cuenca Pérmica, Texas / Robstown, Texas, EE.UU.</t>
+          <t>Gothenburg, Nebraska, EE.UU.</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Phillips 66</t>
+          <t>J. Westling &amp; Co. (JWC Gburg, LLC)</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>No especificado (tecnología licenciada Topsoe SynCOR Ammonia); contrato EPC/fabricación asegurado</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería (sancionado; en línea 2028)</t>
+          <t>Ingeniería/Permisos (permiso de aire emitido, sitio zonificado; obras civiles previstas 2027, operación comercial 2029)</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>[Business Wire](https://www.businesswire.com/news/home/20260517310811/en/Phillips-66-announces-Zeus-Gas-Plant-and-a-third-Coastal-Bend-Fractionator)</t>
+          <t>[USDA](https://www.usda.gov/about-usda/news/press-releases/2026/07/01/secretary-rollins-announces-500-million-fertilizer-investment-and-expansion-program-strengthen)</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Project Meadowlark (complejo de amoniaco azul/UAN/ATS/DEF)</t>
+          <t>Wabash Low-Carbon Ammonia Project</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Gothenburg, Nebraska, EE.UU.</t>
+          <t>West Terre Haute, Indiana, EE.UU.</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>J. Westling &amp; Co. (JWC Gburg, LLC)</t>
+          <t>Wabash Valley Resources</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>No especificado (tecnología licenciada Topsoe SynCOR Ammonia); contrato EPC/fabricación asegurado</t>
+          <t>Samsung E&amp;C (contrato EPF ~US$475 millones)</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/Permisos (permiso de aire emitido, sitio zonificado; obras civiles previstas 2027, operación comercial 2029)</t>
+          <t>Construcción (groundbreaking 5-ene-2026; amoniaco bajo en carbono 500,000 ton/año con captura de 1.67 millones ton CO2/año; meta de finalización 2029)</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>[USDA](https://www.usda.gov/about-usda/news/press-releases/2026/07/01/secretary-rollins-announces-500-million-fertilizer-investment-and-expansion-program-strengthen)</t>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/clean-fuels/06012026/samsung-ea-announces-groundbreaking-of-low-carbon-ammonia-plant/)</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-24</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Wabash Low-Carbon Ammonia Project</t>
+          <t>Green Fuels Operating — Refinería Duncan</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>West Terre Haute, Indiana, EE.UU.</t>
+          <t>Duncan, Stephens County, Oklahoma, EE.UU.</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Wabash Valley Resources</t>
+          <t>Green Fuels Operating</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Samsung E&amp;C (contrato EPF ~US$475 millones)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Construcción (groundbreaking 5-ene-2026; amoniaco bajo en carbono 500,000 ton/año con captura de 1.67 millones ton CO2/año; meta de finalización 2029)</t>
+          <t>Construcción (groundbreaking 29-may-2026; inversión US$400 millones; capacidad inicial 30,000 bbl/d, expandible a 50,000 bbl/d, sobre sitio de refinería histórica de los años 1920)</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/clean-fuels/06012026/samsung-ea-announces-groundbreaking-of-low-carbon-ammonia-plant/)</t>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/refining/03062026/green-fuels-hosts-groundbreaking-ceremony-for-new-refinery/)</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Green Fuels Operating — Refinería Duncan</t>
+          <t>Energy Transfer Mustang Draw I &amp; II (plantas de gas)</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Duncan, Stephens County, Oklahoma, EE.UU.</t>
+          <t>Cuenca Midland, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Green Fuels Operating</t>
+          <t>Energy Transfer LP</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -1681,34 +1679,34 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Construcción (groundbreaking 29-may-2026; inversión US$400 millones; capacidad inicial 30,000 bbl/d, expandible a 50,000 bbl/d, sobre sitio de refinería histórica de los años 1920)</t>
+          <t>Construcción (Mustang Draw I en comisionamiento, servicio pleno ~jun-2026; Mustang Draw II en construcción, en servicio 4T2026; 275 MMcf/d cada una)</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/refining/03062026/green-fuels-hosts-groundbreaking-ceremony-for-new-refinery/)</t>
+          <t>[Energy Transfer](https://www.energytransfer.com/project-highlights/)</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Energy Transfer Mustang Draw I &amp; II (plantas de gas)</t>
+          <t>ONEOK Bighorn / Cutter / Shadowfax (plantas de gas)</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Cuenca Midland, Texas, EE.UU.</t>
+          <t>Cuenca Delaware (Bighorn), Texas / Cuenca Powder River (Cutter), Wyoming / Cuenca Midland (Shadowfax reubicada), Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Energy Transfer LP</t>
+          <t>ONEOK Inc.</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -1718,49 +1716,49 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Construcción (Mustang Draw I en comisionamiento, servicio pleno ~jun-2026; Mustang Draw II en construcción, en servicio 4T2026; 275 MMcf/d cada una)</t>
+          <t>Construcción (según reporte 2T2026 de ONEOK, ~4-8-ago-2026: Bighorn ampliada de 300 a 400 MMcf/d, tratamiento alto CO2, meta mediados 2027; Cutter 60 MMcf/d en construcción, meta 4T2026; Shadowfax 150 MMcf/d reubicada a la cuenca Midland durante el trimestre, en rampa)</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>[Energy Transfer](https://www.energytransfer.com/project-highlights/)</t>
+          <t>[Inspectioneering](https://inspectioneering.com/news/2025-08-07/11702/oneok-greenlights-new-365m-delaware-basin-gas-plant); [BigGo Finance](https://finance.biggo.com/news/US_OKE_2026-08-04)</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>ONEOK Bighorn / Cutter / Shadowfax (plantas de gas)</t>
+          <t>MPLX Harmon Creek III (planta de gas + de-etanizadora)</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Cuenca Delaware (Bighorn), Texas / Cuenca Powder River (Cutter), Wyoming / Cuenca Midland (Shadowfax reubicada), Texas, EE.UU.</t>
+          <t>Región Marcellus/Utica, noreste de EE.UU. (ubicación exacta no especificada)</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>ONEOK Inc.</t>
+          <t>MPLX LP</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>MPLX (propietario-constructor)</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Construcción (según reporte 2T2026 de ONEOK, ~4-8-ago-2026: Bighorn ampliada de 300 a 400 MMcf/d, tratamiento alto CO2, meta mediados 2027; Cutter 60 MMcf/d en construcción, meta 4T2026; Shadowfax 150 MMcf/d reubicada a la cuenca Midland durante el trimestre, en rampa)</t>
+          <t>Operando (arranque/startup completado ago-2026, según reporte 2T2026 de MPLX; eleva capacidad de procesamiento de MPLX en el noreste a 8.1 Bcf/d; planta de 300 MMcf/d + de-etanizadora 40 Mbpd)</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>[Inspectioneering](https://inspectioneering.com/news/2025-08-07/11702/oneok-greenlights-new-365m-delaware-basin-gas-plant); [BigGo Finance](https://finance.biggo.com/news/US_OKE_2026-08-04)</t>
+          <t>[Marcellus Drilling News](https://marcellusdrilling.com/2026/08/mplx-marcellus-proc-plants-96-full-harmon-creek-iii-starts-up/); [StockTitan](https://www.stocktitan.net/news/MPLX/mplx-lp-reports-second-quarter-2026-financial-9tcvq4saz6sr.html)</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -1772,86 +1770,86 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>MPLX Harmon Creek III (planta de gas + de-etanizadora)</t>
+          <t>Rehab. Complejo Cosoleacaque (amoniaco) + Complejo Morelos (etano-etileno)</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Región Marcellus/Utica, noreste de EE.UU. (ubicación exacta no especificada)</t>
+          <t>Cosoleacaque y Complejo Morelos, Veracruz, México</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>MPLX LP</t>
+          <t>Pemex Transformación Industrial</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>MPLX (propietario-constructor)</t>
+          <t>Mota-Engil México (plantas VI/VII y TASP Pajaritos); ICA (paquete relacionado)</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Operando (arranque/startup completado ago-2026, según reporte 2T2026 de MPLX; eleva capacidad de procesamiento de MPLX en el noreste a 8.1 Bcf/d; planta de 300 MMcf/d + de-etanizadora 40 Mbpd)</t>
+          <t>Ingeniería/planeación (parte del plan de reactivación petroquímica de Pemex de 93,000 mdp anunciado jun-2026; 13,000 mdp para 2 plantas de amoniaco en Cosoleacaque, meta 957,000 ton/año; Complejo Morelos incluido en programa de rehabilitación etano-etileno de 30,000 mdp/5 plantas, meta 520,000 ton/año de polietilenos/óxido de etileno/glicoles; contratos de rehabilitación y confiabilidad adjudicados dic-2025, confirmados ene-2026)</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>[Marcellus Drilling News](https://marcellusdrilling.com/2026/08/mplx-marcellus-proc-plants-96-full-harmon-creek-iii-starts-up/); [StockTitan](https://www.stocktitan.net/news/MPLX/mplx-lp-reports-second-quarter-2026-financial-9tcvq4saz6sr.html)</t>
+          <t>[Contralínea](https://contralinea.com.mx/interno/semana/presentan-plan-con-inversion-de-93-mil-mdp-para-rescatar-la-petroquimica-nacional/); [El Diario de Juárez](https://diario.mx/nacional/2026/jan/22/adjudica-pemex-contratos-a-favoritas-1102601.html)</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-06</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Rehab. Complejo Cosoleacaque (amoniaco) + Complejo Morelos (etano-etileno)</t>
+          <t>Enterprise Products — Nuevas Plantas de Gas Permian (Plant 11 Midland / Plant 13 Delaware) + NGL Frac 15 Mont Belvieu</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Cosoleacaque y Complejo Morelos, Veracruz, México</t>
+          <t>Cuenca Midland y Cuenca Delaware, Texas, EE.UU. / Mont Belvieu, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Pemex Transformación Industrial</t>
+          <t>Enterprise Products Partners L.P.</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Mota-Engil México (plantas VI/VII y TASP Pajaritos); ICA (paquete relacionado)</t>
+          <t>Enterprise Products (propietario-constructor)</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/planeación (parte del plan de reactivación petroquímica de Pemex de 93,000 mdp anunciado jun-2026; 13,000 mdp para 2 plantas de amoniaco en Cosoleacaque, meta 957,000 ton/año; Complejo Morelos incluido en programa de rehabilitación etano-etileno de 30,000 mdp/5 plantas, meta 520,000 ton/año de polietilenos/óxido de etileno/glicoles; contratos de rehabilitación y confiabilidad adjudicados dic-2025, confirmados ene-2026)</t>
+          <t>Construcción (sancionadas/aprobadas en resultados 2T2026: Plant 11 Midland Basin 300 MMcf/d en servicio 1T2029; Plant 13 Delaware Basin 300 MMcf/d en servicio 3T2028; NGL Frac 15 en Mont Belvieu 150 MBPD en servicio 1T2028; gasto de capital de crecimiento 2026 aumentado en más de US$700 millones por estas sanciones)</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>[Contralínea](https://contralinea.com.mx/interno/semana/presentan-plan-con-inversion-de-93-mil-mdp-para-rescatar-la-petroquimica-nacional/); [El Diario de Juárez](https://diario.mx/nacional/2026/jan/22/adjudica-pemex-contratos-a-favoritas-1102601.html)</t>
+          <t>[Enterprise Reports Second Quarter 2026 Earnings](https://ir.enterpriseproducts.com/news-releases/news-release-details/enterprise-reports-second-quarter-2026-earnings)</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-07-31</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Enterprise Products — Nuevas Plantas de Gas Permian (Plant 11 Midland / Plant 13 Delaware) + NGL Frac 15 Mont Belvieu</t>
+          <t>Enterprise Products — Plant 12 (Delaware Basin) y Athena 2 (Midland Basin)</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Cuenca Midland y Cuenca Delaware, Texas, EE.UU. / Mont Belvieu, Texas, EE.UU.</t>
+          <t>Cuenca Delaware y Cuenca Midland, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -1866,7 +1864,7 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Construcción (sancionadas/aprobadas en resultados 2T2026: Plant 11 Midland Basin 300 MMcf/d en servicio 1T2029; Plant 13 Delaware Basin 300 MMcf/d en servicio 3T2028; NGL Frac 15 en Mont Belvieu 150 MBPD en servicio 1T2028; gasto de capital de crecimiento 2026 aumentado en más de US$700 millones por estas sanciones)</t>
+          <t>Construcción (sancionadas, divulgadas en resultados 2T2026 el 30-jul-2026; Plant 12 Delaware Basin ~300 MMcf/d en servicio 4T2027; Athena 2 Midland Basin en servicio 3T2027)</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -1876,39 +1874,39 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Enterprise Products — Plant 12 (Delaware Basin) y Athena 2 (Midland Basin)</t>
+          <t>Targa Resources Roadrunner III / Copperhead II (plantas de gas)</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Cuenca Delaware y Cuenca Midland, Texas, EE.UU.</t>
+          <t>Cuenca Delaware (Permian), Texas/Nuevo México, EE.UU.</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Enterprise Products Partners L.P.</t>
+          <t>Targa Resources Corp.</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Enterprise Products (propietario-constructor)</t>
+          <t>Targa Resources (propietario-constructor)</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Construcción (sancionadas, divulgadas en resultados 2T2026 el 30-jul-2026; Plant 12 Delaware Basin ~300 MMcf/d en servicio 4T2027; Athena 2 Midland Basin en servicio 3T2027)</t>
+          <t>Construcción (aprobadas may-2026; Roadrunner III 265 MMcf/d, Copperhead II 275 MMcf/d; en servicio previsto 1T2028)</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>[Enterprise Reports Second Quarter 2026 Earnings](https://ir.enterpriseproducts.com/news-releases/news-release-details/enterprise-reports-second-quarter-2026-earnings)</t>
+          <t>[PGJ](https://pgjonline.com/news/2026/may/targa-expands-permian-gas-processing-delaware-express-pipeline-capacity)</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -1920,54 +1918,54 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Targa Resources Roadrunner III / Copperhead II (plantas de gas)</t>
+          <t>Southern Energy Renewables — Complejo de Metanol y SAF</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Cuenca Delaware (Permian), Texas/Nuevo México, EE.UU.</t>
+          <t>St. Charles Parish (Killona), Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Targa Resources Corp.</t>
+          <t>Southern Energy Renewables</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Targa Resources (propietario-constructor)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Construcción (aprobadas may-2026; Roadrunner III 265 MMcf/d, Copperhead II 275 MMcf/d; en servicio previsto 1T2028)</t>
+          <t>Planeación/pre-construcción (inversión US$1,400 millones; convierte biomasa de desecho de madera en metanol verde y combustible de aviación sostenible; construcción prevista a iniciar fines de 2027, producción prevista fines de 2029)</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>[PGJ](https://pgjonline.com/news/2026/may/targa-expands-permian-gas-processing-delaware-express-pipeline-capacity)</t>
+          <t>[Hydrocarbon Processing](https://www.hydrocarbonprocessing.com/news/2026/03/southern-energy-renewables-announce-14-b-methanol-and-saf-complex-in-louisiana/); [Louisiana Economic Development](https://www.opportunitylouisiana.gov/news/southern-energy-renewables-announce-1-4-billion-methanol-and-sustainable-aviation-fuel-facility-in-st-charles-parish)</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Southern Energy Renewables — Complejo de Metanol y SAF</t>
+          <t>Atlas Agro — Pacific Green Fertilizer Plant</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>St. Charles Parish (Killona), Luisiana, EE.UU.</t>
+          <t>Richland, Washington, EE.UU.</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Southern Energy Renewables</t>
+          <t>Atlas Agro</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -1977,49 +1975,49 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Planeación/pre-construcción (inversión US$1,400 millones; convierte biomasa de desecho de madera en metanol verde y combustible de aviación sostenible; construcción prevista a iniciar fines de 2027, producción prevista fines de 2029)</t>
+          <t>Ingeniería/FEED (diseño ~70% completo, USD 315 millones de capital levantado, permisos en proceso; planta de fertilizante nitrato ~0.7 Mt/año, inversión USD 1,100-1,500 millones; debe iniciar construcción antes de fines de 2027 para calificar a créditos fiscales federales; construcción estimada en 36 meses)</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>[Hydrocarbon Processing](https://www.hydrocarbonprocessing.com/news/2026/03/southern-energy-renewables-announce-14-b-methanol-and-saf-complex-in-louisiana/); [Louisiana Economic Development](https://www.opportunitylouisiana.gov/news/southern-energy-renewables-announce-1-4-billion-methanol-and-sustainable-aviation-fuel-facility-in-st-charles-parish)</t>
+          <t>[Tri-Cities Area Journal of Business](https://www.tricitiesbusinessnews.com/articles/atlas-agro-plant-nears-decision-point); [Washington State Standard](https://washingtonstatestandard.com/2025/10/30/plan-for-1-5b-fertilizer-plant-in-central-wa-still-alive-despite-loss-of-federal-funds/)</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-06</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Atlas Agro — Pacific Green Fertilizer Plant</t>
+          <t>Hydrogen City (complejo Power-to-X / e-metanol)</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Richland, Washington, EE.UU.</t>
+          <t>Piedras Pintas Salt Dome, Condado de Duval, sur de Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Atlas Agro</t>
+          <t>Green Hydrogen International (GHI)</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>ABB (automatización/control, vía MOU)</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/FEED (diseño ~70% completo, USD 315 millones de capital levantado, permisos en proceso; planta de fertilizante nitrato ~0.7 Mt/año, inversión USD 1,100-1,500 millones; debe iniciar construcción antes de fines de 2027 para calificar a créditos fiscales federales; construcción estimada en 36 meses)</t>
+          <t>Ingeniería/FEED (inversión USD 6,000-10,000 millones; electrolizador de 2.2 GW; producirá 1.4 Mt/año de e-metanol y capturará ~2 Mt/año de CO2; construcción planeada desde 2026, primera producción estimada 2030)</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>[Tri-Cities Area Journal of Business](https://www.tricitiesbusinessnews.com/articles/atlas-agro-plant-nears-decision-point); [Washington State Standard](https://washingtonstatestandard.com/2025/10/30/plan-for-1-5b-fertilizer-plant-in-central-wa-still-alive-despite-loss-of-federal-funds/)</t>
+          <t>[The Engineer](https://www.theengineer.co.uk/content/news/abb-joins-team-for-22gw-hydrogen-city-project-in-texas); [Energy Capital HTX](https://energycapitalhtx.com/green-hydrogen-city-abb-mou)</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -2031,91 +2029,91 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Hydrogen City (complejo Power-to-X / e-metanol)</t>
+          <t>Targa Resources Falcon II Gas Processing Plant</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Piedras Pintas Salt Dome, Condado de Duval, sur de Texas, EE.UU.</t>
+          <t>Cuenca Delaware, Permian Basin, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Green Hydrogen International (GHI)</t>
+          <t>Targa Resources Corp.</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>ABB (automatización/control, vía MOU)</t>
+          <t>Targa Resources (propietario-constructor)</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/FEED (inversión USD 6,000-10,000 millones; electrolizador de 2.2 GW; producirá 1.4 Mt/año de e-metanol y capturará ~2 Mt/año de CO2; construcción planeada desde 2026, primera producción estimada 2030)</t>
+          <t>Construcción/Comisionamiento (planta criogénica; arranque adelantado a 1T2026, dos trimestres antes de lo previsto; según reporte 2T2026 de Targa —6-ago-2026—, el segundo tren quedó completo y en preparación para producción plena, llevando la capacidad total a ~685 MMcf/d)</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>[The Engineer](https://www.theengineer.co.uk/content/news/abb-joins-team-for-22gw-hydrogen-city-project-in-texas); [Energy Capital HTX](https://energycapitalhtx.com/green-hydrogen-city-abb-mou)</t>
+          <t>[Oil &amp; Gas Journal](https://www.ogj.com/refining-processing/gas-processing/capacities/article/55240691/targa-advances-expansion-plans-for-permian-basin-gas-processing); [Targa Resources Q2 2026 Results](https://www.globenewswire.com/news-release/2026/08/06/3340017/14074/en/Targa-Resources-Corp-Reports-Record-Second-Quarter-2026-Financial-Results.html)</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-20</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Targa Resources Falcon II Gas Processing Plant</t>
+          <t>Cassidy II Gas Processing Plant</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Cuenca Delaware, Permian Basin, Texas, EE.UU.</t>
+          <t>Condado de Glasscock, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Targa Resources Corp.</t>
+          <t>Brazos Midstream</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Targa Resources (propietario-constructor)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Construcción/Comisionamiento (planta criogénica; arranque adelantado a 1T2026, dos trimestres antes de lo previsto; según reporte 2T2026 de Targa —6-ago-2026—, el segundo tren quedó completo y en preparación para producción plena, llevando la capacidad total a ~685 MMcf/d)</t>
+          <t>Anuncio/Construcción (planta criogénica de 300 MMcf/d adicional a Cassidy I —300 MMcf/d, en servicio antes de fin de 2026—; eleva capacidad total de Brazos en Midland Basin a ~1.1 Bcf/d; respaldada por ~575,000 acres bajo dedicación; entrada en operación prevista verano 2027; anunciado 11-ago-2026)</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>[Oil &amp; Gas Journal](https://www.ogj.com/refining-processing/gas-processing/capacities/article/55240691/targa-advances-expansion-plans-for-permian-basin-gas-processing); [Targa Resources Q2 2026 Results](https://www.globenewswire.com/news-release/2026/08/06/3340017/14074/en/Targa-Resources-Corp-Reports-Record-Second-Quarter-2026-Financial-Results.html)</t>
+          <t>[Inspectioneering](https://inspectioneering.com/news/2026-08-11/12145/brazos-midstream-announces-new-natural-gas-processing-plant-to-support-continued); [Rigzone](https://www.rigzone.com/news/brazos_to_grow_midland_gas_processing_capacity_to_11_bcfd-11-aug-2026-184346-article/)</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Cassidy II Gas Processing Plant</t>
+          <t>Kings Landing II Gas Processing Plant</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Condado de Glasscock, Texas, EE.UU.</t>
+          <t>Nuevo México, EE.UU.</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Brazos Midstream</t>
+          <t>Kinetik Holdings</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -2125,34 +2123,34 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Anuncio/Construcción (planta criogénica de 300 MMcf/d adicional a Cassidy I —300 MMcf/d, en servicio antes de fin de 2026—; eleva capacidad total de Brazos en Midland Basin a ~1.1 Bcf/d; respaldada por ~575,000 acres bajo dedicación; entrada en operación prevista verano 2027; anunciado 11-ago-2026)</t>
+          <t>Construcción (FID alcanzada; US$260 millones; finalización prevista 2S2028)</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>[Inspectioneering](https://inspectioneering.com/news/2026-08-11/12145/brazos-midstream-announces-new-natural-gas-processing-plant-to-support-continued); [Rigzone](https://www.rigzone.com/news/brazos_to_grow_midland_gas_processing_capacity_to_11_bcfd-11-aug-2026-184346-article/)</t>
+          <t>[Investing.com](https://www.investing.com/news/company-news/kinetik-approves-260m-gas-processing-plant-in-new-mexico-93CH-4698224)</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Kings Landing II Gas Processing Plant</t>
+          <t>Apollo Gas Plant</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Nuevo México, EE.UU.</t>
+          <t>Condado de Eddy, Nuevo México, EE.UU.</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Kinetik Holdings</t>
+          <t>Trace Midstream Partners II</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -2162,12 +2160,12 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Construcción (FID alcanzada; US$260 millones; finalización prevista 2S2028)</t>
+          <t>Anuncio/planeación (planta criogénica de 250 MMcf/d)</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>[Investing.com](https://www.investing.com/news/company-news/kinetik-approves-260m-gas-processing-plant-in-new-mexico-93CH-4698224)</t>
+          <t>[Gas Compression Magazine](https://gascompressionmagazine.com/2026/06/29/new-mexico-gains-major-gas-processing-hub/)</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -2179,17 +2177,17 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Apollo Gas Plant</t>
+          <t>IGP Gulf Coast Methanol Complex (4 unidades)</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Condado de Eddy, Nuevo México, EE.UU.</t>
+          <t>Plaquemine Parish (Myrtle Grove), Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Trace Midstream Partners II</t>
+          <t>IGP Methanol LLC</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -2199,12 +2197,12 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Anuncio/planeación (planta criogénica de 250 MMcf/d)</t>
+          <t>Permiso de calidad del aire asegurado / pre-construcción (US$3,600 millones)</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>[Gas Compression Magazine](https://gascompressionmagazine.com/2026/06/29/new-mexico-gains-major-gas-processing-hub/)</t>
+          <t>[Industrial Info Resources](https://www.industrialinfo.com/news/article.jsp?newsitemID=262022)</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -2216,91 +2214,91 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>IGP Gulf Coast Methanol Complex (4 unidades)</t>
+          <t>Eastern Montana Fertilizer Project (planta de urea)</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Plaquemine Parish (Myrtle Grove), Luisiana, EE.UU.</t>
+          <t>Culbertson, Montana, EE.UU.</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>IGP Methanol LLC</t>
+          <t>Cyan H2</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>KBR (MoU: tecnología, ingeniería, procura y gestión de construcción)</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Permiso de calidad del aire asegurado / pre-construcción (US$3,600 millones)</t>
+          <t>Desarrollo/financiamiento (busca cierre de subvención USDA de US$150 millones —vence 17-ago-2026— y préstamo DOE de US$1,000 millones; groundbreaking previsto fin de 2026)</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>[Industrial Info Resources](https://www.industrialinfo.com/news/article.jsp?newsitemID=262022)</t>
+          <t>[Northern Plains Independent](https://www.northernplainsindependent.com/2026/08/13/proposed-fertilizer-plant-making-strides/); [World Fertilizer](https://www.worldfertilizer.com/project-news/26112025/cyan-h2-signs-mou-for-montana-fertilizer-project/)</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Eastern Montana Fertilizer Project (planta de urea)</t>
+          <t>Targa Resources — Plantas Wrangler, Ranger y Ranger II (procesamiento de gas)</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Culbertson, Montana, EE.UU.</t>
+          <t>Cuenca Delaware (Permian), Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Cyan H2</t>
+          <t>Targa Resources Corp. (acuerdo de 20 años con subsidiarias de ExxonMobil)</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>KBR (MoU: tecnología, ingeniería, procura y gestión de construcción)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Desarrollo/financiamiento (busca cierre de subvención USDA de US$150 millones —vence 17-ago-2026— y préstamo DOE de US$1,000 millones; groundbreaking previsto fin de 2026)</t>
+          <t>Anuncio/Planeación (anunciado 17-ago-2026; tres nuevas plantas criogénicas con capacidad combinada ~825 MMcf/d, más nuevo gasoducto de ~70 millas "Bull Run II" hacia el hub de Waha; entrada en servicio prevista 1S2028; Targa evalúa además hasta 5 plantas adicionales en Permian Delaware a más largo plazo)</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>[Northern Plains Independent](https://www.northernplainsindependent.com/2026/08/13/proposed-fertilizer-plant-making-strides/); [World Fertilizer](https://www.worldfertilizer.com/project-news/26112025/cyan-h2-signs-mou-for-montana-fertilizer-project/)</t>
+          <t>[EnergyNow](https://energynow.com/2026/08/targa-to-build-three-permian-gas-processing-plants-new-pipeline/); [Targa Resources](https://www.targaresources.com/news-releases/news-release-details/targa-resources-corp-announces-20-year-agreements-exxonmobil-and)</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Targa Resources — Plantas Wrangler, Ranger y Ranger II (procesamiento de gas)</t>
+          <t>México Amoníaco y Urea (MAYU)</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Cuenca Delaware (Permian), Texas, EE.UU.</t>
+          <t>Costa del Pacífico, Sonora, México (ciudad exacta no especificada)</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Targa Resources Corp. (acuerdo de 20 años con subsidiarias de ExxonMobil)</t>
+          <t>México Amoníaco y Urea (desarrollador privado)</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -2310,34 +2308,34 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Anuncio/Planeación (anunciado 17-ago-2026; tres nuevas plantas criogénicas con capacidad combinada ~825 MMcf/d, más nuevo gasoducto de ~70 millas "Bull Run II" hacia el hub de Waha; entrada en servicio prevista 1S2028; Targa evalúa además hasta 5 plantas adicionales en Permian Delaware a más largo plazo)</t>
+          <t>Desarrollo muy temprano (planta de amoniaco azul y urea bajo en carbono, capacidad &gt;900,000 ton/año, usando gas natural de la Cuenca Pérmica vía costa del Pacífico; sin autorización de impacto ambiental ni contrato EPC confirmado públicamente a la fecha)</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>[EnergyNow](https://energynow.com/2026/08/targa-to-build-three-permian-gas-processing-plants-new-pipeline/); [Targa Resources](https://www.targaresources.com/news-releases/news-release-details/targa-resources-corp-announces-20-year-agreements-exxonmobil-and)</t>
+          <t>[MAYU](https://mayu.com.mx/en/)</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-18</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>México Amoníaco y Urea (MAYU)</t>
+          <t>Ampliación Terminal de Exportación NGL Nederland</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Costa del Pacífico, Sonora, México (ciudad exacta no especificada)</t>
+          <t>Nederland/Port Neches, Jefferson County, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>México Amoníaco y Urea (desarrollador privado)</t>
+          <t>Energy Transfer LP</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -2347,34 +2345,34 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Desarrollo muy temprano (planta de amoniaco azul y urea bajo en carbono, capacidad &gt;900,000 ton/año, usando gas natural de la Cuenca Pérmica vía costa del Pacífico; sin autorización de impacto ambiental ni contrato EPC confirmado públicamente a la fecha)</t>
+          <t>Totalmente comprometida (fully subscribed; contratos de largo plazo hasta la década de 2040; incluye ampliación del ducto de NGL Mont Belvieu-Nederland y construcción de dos muelles adicionales; anunciado 18-jun-2026; entrada en servicio por etapas desde 2028)</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>[MAYU](https://mayu.com.mx/en/)</t>
+          <t>[Rigzone](https://www.rigzone.com/news/energy_transfer_to_expand_texas_ngl_export_terminal-19-jun-2026-183955-article/); [Energy Transfer IR](https://ir.energytransfer.com/news-releases/news-release-details/energy-transfer-announces-fully-subscribed-export-expansion)</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-26</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Ampliación Terminal de Exportación NGL Nederland</t>
+          <t>LSB Industries — Expansión de Amoniaco El Dorado</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Nederland/Port Neches, Jefferson County, Texas, EE.UU.</t>
+          <t>El Dorado, Arkansas, EE.UU.</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Energy Transfer LP</t>
+          <t>LSB Industries</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
@@ -2384,34 +2382,34 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>Totalmente comprometida (fully subscribed; contratos de largo plazo hasta la década de 2040; incluye ampliación del ducto de NGL Mont Belvieu-Nederland y construcción de dos muelles adicionales; anunciado 18-jun-2026; entrada en servicio por etapas desde 2028)</t>
+          <t>Pre-FID (decisión final de inversión proyectada para 2T2027; expansión de 100,000 toneladas/año incrementales de amoniaco, costo neto US$105-120 millones, bruto US$135-150 millones incluyendo infraestructura)</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>[Rigzone](https://www.rigzone.com/news/energy_transfer_to_expand_texas_ngl_export_terminal-19-jun-2026-183955-article/); [Energy Transfer IR](https://ir.energytransfer.com/news-releases/news-release-details/energy-transfer-announces-fully-subscribed-export-expansion)</t>
+          <t>[The Motley Fool](https://www.fool.com/earnings/call-transcripts/2026/08/07/lsb-industries-lxu-q2-2026-earnings-call-transcript/)</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>LSB Industries — Expansión de Amoniaco El Dorado</t>
+          <t>Yara/Enbridge — Amoniaco Azul Ingleside</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>El Dorado, Arkansas, EE.UU.</t>
+          <t>Enbridge Ingleside Energy Center, cerca de Corpus Christi, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>LSB Industries</t>
+          <t>Yara Clean Ammonia / Enbridge (JV 50/50)</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
@@ -2421,12 +2419,12 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Pre-FID (decisión final de inversión proyectada para 2T2027; expansión de 100,000 toneladas/año incrementales de amoniaco, costo neto US$105-120 millones, bruto US$135-150 millones incluyendo infraestructura)</t>
+          <t>Ingeniería (FEED en curso, pendiente FID; capacidad 1.2-1.4 MMTPA, inversión estimada US$2,600-2,900 millones; reforming autotérmico con captura de CO2 ~95%; enfrenta oposición comunitaria activa)</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>[The Motley Fool](https://www.fool.com/earnings/call-transcripts/2026/08/07/lsb-industries-lxu-q2-2026-earnings-call-transcript/)</t>
+          <t>[QC Intel](https://www.qcintel.com/ammonia/article/yara-enbridge-continue-ingleside-blue-ammonia-plans-despite-pushback-28727.html)</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -2438,72 +2436,35 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Yara/Enbridge — Amoniaco Azul Ingleside</t>
+          <t>Cronus Chemicals — Planta de Amoniaco/Fertilizantes Tuscola</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Enbridge Ingleside Energy Center, cerca de Corpus Christi, Texas, EE.UU.</t>
+          <t>Tuscola, Illinois, EE.UU.</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Yara Clean Ammonia / Enbridge (JV 50/50)</t>
+          <t>Cronus Chemicals LLC</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>thyssenkrupp Industrial Solutions (EPC llave en mano, lump-sum)</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería (FEED en curso, pendiente FID; capacidad 1.2-1.4 MMTPA, inversión estimada US$2,600-2,900 millones; reforming autotérmico con captura de CO2 ~95%; enfrenta oposición comunitaria activa)</t>
+          <t>Construcción (proyecto de ~US$2,000-2,300 millones, hasta ~2,300 t/día / ~950,000 ton/año de amoniaco; obtuvo el permiso final de construcción/aire de la EPA tras más de una década en planeación desde 2012; construcción de ~40 meses, hasta 2,000-2,500 empleos pico)</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>[QC Intel](https://www.qcintel.com/ammonia/article/yara-enbridge-continue-ingleside-blue-ammonia-plans-despite-pushback-28727.html)</t>
+          <t>[News-Gazette](https://www.news-gazette.com/business/employment/after-almost-13-years-2-3-billion-tuscola-fertilizer-plant-clears-final-regulatory-hurdle-for/); [FarmWeek Now](https://www.farmweeknow.com/policy/state/construction-to-begin-on-tuscola-ammonia-plant/)</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="2" t="inlineStr">
-        <is>
-          <t>Cronus Chemicals — Planta de Amoniaco/Fertilizantes Tuscola</t>
-        </is>
-      </c>
-      <c r="B56" s="2" t="inlineStr">
-        <is>
-          <t>Tuscola, Illinois, EE.UU.</t>
-        </is>
-      </c>
-      <c r="C56" s="2" t="inlineStr">
-        <is>
-          <t>Cronus Chemicals LLC</t>
-        </is>
-      </c>
-      <c r="D56" s="2" t="inlineStr">
-        <is>
-          <t>thyssenkrupp Industrial Solutions (EPC llave en mano, lump-sum)</t>
-        </is>
-      </c>
-      <c r="E56" s="2" t="inlineStr">
-        <is>
-          <t>Construcción (proyecto de ~US$2,000-2,300 millones, hasta ~2,300 t/día / ~950,000 ton/año de amoniaco; obtuvo el permiso final de construcción/aire de la EPA tras más de una década en planeación desde 2012; construcción de ~40 meses, hasta 2,000-2,500 empleos pico)</t>
-        </is>
-      </c>
-      <c r="F56" s="2" t="inlineStr">
-        <is>
-          <t>[News-Gazette](https://www.news-gazette.com/business/employment/after-almost-13-years-2-3-billion-tuscola-fertilizer-plant-clears-final-regulatory-hurdle-for/); [FarmWeek Now](https://www.farmweeknow.com/policy/state/construction-to-begin-on-tuscola-ammonia-plant/)</t>
-        </is>
-      </c>
-      <c r="G56" s="2" t="inlineStr">
         <is>
           <t>2026-09-02</t>
         </is>
@@ -2523,13 +2484,13 @@
   <dimension ref="A1:G47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2740,17 +2701,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Construcción/Permitting acelerado (Venture Global presentó solicitud FERC para expansión adicional de 31 mtpa —24 trenes, ~USD 18,000 millones—; U.S. Army Corps of Engineers otorgó permitting expedito bajo "emergencia energética nacional" —periodo de comentario público reducido de 30 a 10 días, cerrado 2-jul-2026—, ampliaría el sitio de 590 a 1,220 acres; DOE aprobó exportaciones adicionales inmediatas desde Plaquemines; inicio de construcción de la expansión esperado a inicios de 2027, primera producción fin de 2028)</t>
+          <t>Construcción/Permitting acelerado (Venture Global presentó solicitud FERC para expansión adicional de 31 mtpa —24 trenes, ~USD 18,000 millones—; U.S. Army Corps of Engineers otorgó permitting expedito bajo "emergencia energética nacional" —periodo de comentario público reducido de 30 a 10 días, cerrado 2-jul-2026—, ampliaría el sitio de 590 a 1,220 acres; DOE aprobó exportaciones adicionales inmediatas desde Plaquemines; inicio de construcción de la expansión esperado a inicios de 2027, primera producción fin de 2028) ; Williams Companies sancionó (FID) el gasoducto "Delta Access" (US$1,500 millones, 2.25 Bcf/d iniciales ampliable a 3.5 Bcf/d, de Gillis LA hacia el corredor Transco, en servicio 1T2029) diseñado para alimentar esta expansión vía interconexión con el gasoducto intraestatal Cloud Connector de Venture Global, confirmado en su reporte 2T2026 (4-ago-2026)</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>[Offshore Energy](https://www.offshore-energy.biz/kbr-zachry-to-work-on-ventures-plaquemines-lng/); [Verite News](https://veritenews.org/2026/08/12/lng-expansion-could-be-fast-tracked); [DOE](https://www.energy.gov/node/4856848)</t>
+          <t>[Offshore Energy](https://www.offshore-energy.biz/kbr-zachry-to-work-on-ventures-plaquemines-lng/); [Verite News](https://veritenews.org/2026/08/12/lng-expansion-could-be-fast-tracked); [DOE](https://www.energy.gov/node/4856848); [Natural Gas Intel](https://www.naturalgasintel.com/news/plaquemines-expansion-to-anchor-east-end-of-williams-delta-access/)</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-09-03</t>
         </is>
       </c>
     </row>
@@ -4285,13 +4246,13 @@
   <dimension ref="A1:G110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5301,7 +5262,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Pine Bluff Arsenal, Arkansas o Anniston Army Depot, Alabama (sin confirmar), EE.UU.</t>
+          <t>Pine Bluff Arsenal, Arkansas (sitio primario, ~245 acres) y Anniston Army Depot, Alabama (~97 acres), EE.UU.</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -5311,22 +5272,22 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Titan Mining Corp.</t>
+          <t>Titan Mining Corp. (vía subsidiaria Empire State Mines)</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Acuerdo firmado/planeación (construcción prevista desde 2027)</t>
+          <t>Acuerdo firmado/planeación (Notificaciones de Selección Condicional del Ejército confirmadas para ambos sitios bajo arrendamientos de uso mejorado —EUL— de hasta 50 años; construcción prevista para 2S-2027)</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>[Mining.com](https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/)</t>
+          <t>[Mining.com](https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/); [NNY360](https://www.nny360.com/news/statenews/empire-state-mines-moves-forward-with-first-u-s-graphite-mine-in-generations/article_6cac15a0-daf9-57bb-be6a-0e41c5c9231d.html)</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-09-03</t>
         </is>
       </c>
     </row>
@@ -7035,12 +6996,12 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>Proyecto de Cobre Angangueo</t>
+          <t>Modernización Complejo Metalúrgico Empalme</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>Angangueo, Michoacán, México</t>
+          <t>Empalme, Sonora, México</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
@@ -7055,7 +7016,7 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Pre-desarrollo (en negociación de permisos con gobierno federal)</t>
+          <t>Pre-desarrollo (en negociación de permisos; fundición existente a modernizar)</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
@@ -7072,17 +7033,17 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Proyecto de Cobre Chalchihuites</t>
+          <t>Coosa Graphite Project (Kellyton Graphite Plant)</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>Chalchihuites, Zacatecas, México</t>
+          <t>Condado de Coosa, Alabama, EE.UU.</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Southern Copper Corporation (Grupo México)</t>
+          <t>Westwater Resources Inc.</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
@@ -7092,34 +7053,34 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Pre-desarrollo (en negociación de permisos)</t>
+          <t>Financiamiento/planeación (préstamo EXIM Bank de US$25 millones anunciado 7-ago-2026 para mina de grafito natural y planta de procesamiento, primera fuente de grafito natural producida en EE.UU.)</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>[Minería en Línea](https://mineriaenlinea.com/2026/07/southern-copper-obtiene-permisos-ambientales-para-el-pilar-produccion-a-partir-de-2029/)</t>
+          <t>[Yellowhammer News](https://yellowhammernews.com/trump-administration-announces-25-million-exim-loan-for-westwaters-coosa-county-graphite-plant/); [EXIM.GOV](https://www.exim.gov/news/trump-administration-announces-58m-major-new-critical-mineral-deals-white-house-roundtable)</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>Modernización Complejo Metalúrgico Empalme</t>
+          <t>Expansión de Procesamiento de Tantalio/Niobio (Global Advanced Metals)</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>Empalme, Sonora, México</t>
+          <t>Pensilvania, EE.UU.</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>Southern Copper Corporation (Grupo México)</t>
+          <t>Global Advanced Metals</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
@@ -7129,34 +7090,34 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Pre-desarrollo (en negociación de permisos; fundición existente a modernizar)</t>
+          <t>Financiamiento/planeación (préstamo EXIM Bank de US$25 millones anunciado 7-ago-2026 para ampliar capacidad de procesamiento)</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>[Minería en Línea](https://mineriaenlinea.com/2026/07/southern-copper-obtiene-permisos-ambientales-para-el-pilar-produccion-a-partir-de-2029/)</t>
+          <t>[EXIM.GOV](https://www.exim.gov/news/trump-administration-announces-58m-major-new-critical-mineral-deals-white-house-roundtable); [SME](https://me.smenet.org/trump-administration-to-back-three-mineral-projects-with-58-million-in-financing/)</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>Coosa Graphite Project (Kellyton Graphite Plant)</t>
+          <t>Boron Americas Project (Fort Cady)</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>Condado de Coosa, Alabama, EE.UU.</t>
+          <t>California, EE.UU.</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Westwater Resources Inc.</t>
+          <t>5E Advanced Materials</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
@@ -7166,12 +7127,12 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Financiamiento/planeación (préstamo EXIM Bank de US$25 millones anunciado 7-ago-2026 para mina de grafito natural y planta de procesamiento, primera fuente de grafito natural producida en EE.UU.)</t>
+          <t>Financiamiento/planeación (préstamo EXIM Bank de US$8 millones anunciado 7-ago-2026 para proyecto de boro, lixiviación/procesamiento)</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>[Yellowhammer News](https://yellowhammernews.com/trump-administration-announces-25-million-exim-loan-for-westwaters-coosa-county-graphite-plant/); [EXIM.GOV](https://www.exim.gov/news/trump-administration-announces-58m-major-new-critical-mineral-deals-white-house-roundtable)</t>
+          <t>[EXIM.GOV](https://www.exim.gov/news/trump-administration-announces-58m-major-new-critical-mineral-deals-white-house-roundtable)</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -7183,54 +7144,54 @@
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>Expansión de Procesamiento de Tantalio/Niobio (Global Advanced Metals)</t>
+          <t>Brook Mine (tierras raras/minerales críticos de carbón)</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>Pensilvania, EE.UU.</t>
+          <t>Ranchester/Sheridan, Wyoming, EE.UU.</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>Global Advanced Metals</t>
+          <t>Ramaco Resources</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Hatch Associates Consultants (ingeniería/estudio)</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>Financiamiento/planeación (préstamo EXIM Bank de US$25 millones anunciado 7-ago-2026 para ampliar capacidad de procesamiento)</t>
+          <t>Ingeniería/Construcción de planta piloto (Hatch publicó Initial Assessment Report jul-2026 con capex preliminar ~US$3,200 millones + US$800 millones de contingencia, VPN interno ~US$8,000 millones; planta piloto en construcción desde oct-2025; primer procesamiento de concentrados de óxido de tierras raras para la Defense Logistics Agency, ago-2026; construcción de planta comercial podría iniciar fines de 2026, producción comercial 2028)</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>[EXIM.GOV](https://www.exim.gov/news/trump-administration-announces-58m-major-new-critical-mineral-deals-white-house-roundtable); [SME](https://me.smenet.org/trump-administration-to-back-three-mineral-projects-with-58-million-in-financing/)</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/ramaco-resources-releases-hatch-report-and-shareholder-letter-on-exploratory-brook-mine-critical-minerals-project-302838319.html); [Mining.com](https://www.mining.com/ramaco-eyes-ree-stockpile-at-wyoming-mine/)</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>Boron Americas Project (Fort Cady)</t>
+          <t>Dewey-Burdock Uranium ISR Project</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>California, EE.UU.</t>
+          <t>Fall River/Custer Counties, Dakota del Sur, EE.UU.</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>5E Advanced Materials</t>
+          <t>enCore Energy (Powertech USA)</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
@@ -7240,71 +7201,71 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Financiamiento/planeación (préstamo EXIM Bank de US$8 millones anunciado 7-ago-2026 para proyecto de boro, lixiviación/procesamiento)</t>
+          <t>Construcción autorizada/permitting (BLM autorizó inicio de construcción de infraestructura —caminos, pozos de monitoreo, líneas eléctricas— jun-2026; NRC renovó la licencia, publicado en Federal Register 7-ago-2026; pendiente permiso estatal de Dakota del Sur, proceso reiniciado tras 13 años de pausa)</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>[EXIM.GOV](https://www.exim.gov/news/trump-administration-announces-58m-major-new-critical-mineral-deals-white-house-roundtable)</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/encore-energy-receives-bureau-of-land-management-authorization-to-begin-construction-at-dewey-burdock-uranium-project-302804230.html); [Federal Register](https://www.federalregister.gov/documents/2026/08/07/2026-16132/powertech-usa-inc-dewey-burdock-uranium-in-situ-recovery-project-license-renewal)</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>Brook Mine (tierras raras/minerales críticos de carbón)</t>
+          <t>Niron Magnetics — Planta de Imanes Permanentes sin Tierras Raras</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>Ranchester/Sheridan, Wyoming, EE.UU.</t>
+          <t>Minnesota, EE.UU. (ubicación exacta no especificada)</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>Ramaco Resources</t>
+          <t>Niron Magnetics</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>Hatch Associates Consultants (ingeniería/estudio)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/Construcción de planta piloto (Hatch publicó Initial Assessment Report jul-2026 con capex preliminar ~US$3,200 millones + US$800 millones de contingencia, VPN interno ~US$8,000 millones; planta piloto en construcción desde oct-2025; primer procesamiento de concentrados de óxido de tierras raras para la Defense Logistics Agency, ago-2026; construcción de planta comercial podría iniciar fines de 2026, producción comercial 2028)</t>
+          <t>Financiamiento asegurado (US$150 millones del Departamento de Defensa/Office of Strategic Capital, anunciado 7-8-ago-2026, parte de paquete federal de US$3,000 millones en minerales críticos)</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/ramaco-resources-releases-hatch-report-and-shareholder-letter-on-exploratory-brook-mine-critical-minerals-project-302838319.html); [Mining.com](https://www.mining.com/ramaco-eyes-ree-stockpile-at-wyoming-mine/)</t>
+          <t>[MINING.COM](https://www.mining.com/web/trump-says-us-is-announcing-a-series-of-mining-projects-worth-3-billion/); [CNBC](https://www.cnbc.com/2026/08/08/trump-admin-to-invest-3-billion-in-defense-linked-minerals-projects.html)</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Dewey-Burdock Uranium ISR Project</t>
+          <t>Louisiana Strategic Metals Complex</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>Fall River/Custer Counties, Dakota del Sur, EE.UU.</t>
+          <t>Alexandria, Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>enCore Energy (Powertech USA)</t>
+          <t>Ucore Rare Metals Inc.</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
@@ -7314,34 +7275,34 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Construcción autorizada/permitting (BLM autorizó inicio de construcción de infraestructura —caminos, pozos de monitoreo, líneas eléctricas— jun-2026; NRC renovó la licencia, publicado en Federal Register 7-ago-2026; pendiente permiso estatal de Dakota del Sur, proceso reiniciado tras 13 años de pausa)</t>
+          <t>Construcción (planta de procesamiento de tierras raras medianas/pesadas —terbio/disprosio—)</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/encore-energy-receives-bureau-of-land-management-authorization-to-begin-construction-at-dewey-burdock-uranium-project-302804230.html); [Federal Register](https://www.federalregister.gov/documents/2026/08/07/2026-16132/powertech-usa-inc-dewey-burdock-uranium-in-situ-recovery-project-license-renewal)</t>
+          <t>[Ucore Rare Metals](https://ucore.com/ucore-readies-for-louisiana-2026-heavy-rare-earth-element-processing/)</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>Niron Magnetics — Planta de Imanes Permanentes sin Tierras Raras</t>
+          <t>Distrito Copper Creek / San Manuel</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>Minnesota, EE.UU. (ubicación exacta no especificada)</t>
+          <t>Condado de Pinal, Arizona, EE.UU.</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>Niron Magnetics</t>
+          <t>Faraday Copper Corp. (adquiriendo la propiedad San Manuel de BHP; BHP recibirá ~30% de acciones de Faraday)</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
@@ -7351,71 +7312,71 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Financiamiento asegurado (US$150 millones del Departamento de Defensa/Office of Strategic Capital, anunciado 7-8-ago-2026, parte de paquete federal de US$3,000 millones en minerales críticos)</t>
+          <t>Exploración/definición de recursos (Faraday firmó acuerdo definitivo para comprar la antigua mina San Manuel de BHP —subterránea y de tajo/ISL, operada 1955-1999— y combinarla con su proyecto adyacente Copper Creek, creando un distrito de &gt;18,000 millones de libras de cobre; asamblea de accionistas 25-ago-2026 para aprobar la transacción, cierre esperado 3T2026; plan de 23,000+ metros de perforación de confirmación desde 4T2026, recurso combinado a mediados de 2027)</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>[MINING.COM](https://www.mining.com/web/trump-says-us-is-announcing-a-series-of-mining-projects-worth-3-billion/); [CNBC](https://www.cnbc.com/2026/08/08/trump-admin-to-invest-3-billion-in-defense-linked-minerals-projects.html)</t>
+          <t>[MINING.COM](https://www.mining.com/faraday-targets-18b-lb-arizona-copper-district/)</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-19</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>Louisiana Strategic Metals Complex</t>
+          <t>IMA Mine</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>Alexandria, Luisiana, EE.UU.</t>
+          <t>Condado de Lemhi, Idaho, EE.UU.</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>Ucore Rare Metals Inc.</t>
+          <t>American Tungsten Corp.</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>No especificado (geotécnica de presas de jales: NewFields MTDs)</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Construcción (planta de procesamiento de tierras raras medianas/pesadas —terbio/disprosio—)</t>
+          <t>Reactivación/pruebas metalúrgicas (mina histórica de tungsteno, produjo WO3 1945-1957; Fase I: reprocesamiento de jales superficiales; Fase II: rehabilitación de mina subterránea; pruebas metalúrgicas iniciadas jul-2026; definición de recursos, permisos y pruebas previstas concluir 4T2026, construcción fin de 2026/1T2027, primera venta de concentrado prevista inicios de 2027)</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>[Ucore Rare Metals](https://ucore.com/ucore-readies-for-louisiana-2026-heavy-rare-earth-element-processing/)</t>
+          <t>[MINING.COM](https://www.mining.com/american-tungsten-kinks-off-construction-at-ima-project-in-idaho/)</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-19</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>Distrito Copper Creek / San Manuel</t>
+          <t>Railroad Valley Minerals / Super-Brine Complex</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>Condado de Pinal, Arizona, EE.UU.</t>
+          <t>Railroad Valley, Nevada, EE.UU.</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>Faraday Copper Corp. (adquiriendo la propiedad San Manuel de BHP; BHP recibirá ~30% de acciones de Faraday)</t>
+          <t>3 Proton Lithium (3PL Operating Inc.)</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
@@ -7425,12 +7386,12 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Exploración/definición de recursos (Faraday firmó acuerdo definitivo para comprar la antigua mina San Manuel de BHP —subterránea y de tajo/ISL, operada 1955-1999— y combinarla con su proyecto adyacente Copper Creek, creando un distrito de &gt;18,000 millones de libras de cobre; asamblea de accionistas 25-ago-2026 para aprobar la transacción, cierre esperado 3T2026; plan de 23,000+ metros de perforación de confirmación desde 4T2026, recurso combinado a mediados de 2027)</t>
+          <t>Exploración avanzada (depósito multi-mineral confirmado: litio, potasa, boro y lo que la empresa describe como el mayor depósito de tungsteno de EE.UU. —~1.78 millones de toneladas, valorado en ~US$152,000 millones in-situ—; ~17 millas cuadradas del área están retiradas de minería desde 2023 por solicitud de la NASA para calibración de satélites, lo que representa un obstáculo regulatorio; sin decisión de construcción)</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>[MINING.COM](https://www.mining.com/faraday-targets-18b-lb-arizona-copper-district/)</t>
+          <t>[MINING.COM](https://www.mining.com/largest-us-tungsten-discovery-hits-nasa-roadblock/)</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -7442,32 +7403,32 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>IMA Mine</t>
+          <t>New Amalga Gold Project</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>Condado de Lemhi, Idaho, EE.UU.</t>
+          <t>~25 km al norte de Juneau, Alaska, EE.UU.</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>American Tungsten Corp.</t>
+          <t>Grande Portage Resources Ltd.</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>No especificado (geotécnica de presas de jales: NewFields MTDs)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Reactivación/pruebas metalúrgicas (mina histórica de tungsteno, produjo WO3 1945-1957; Fase I: reprocesamiento de jales superficiales; Fase II: rehabilitación de mina subterránea; pruebas metalúrgicas iniciadas jul-2026; definición de recursos, permisos y pruebas previstas concluir 4T2026, construcción fin de 2026/1T2027, primera venta de concentrado prevista inicios de 2027)</t>
+          <t>Permitting temprano (recurso Indicado de 1.44 millones oz Au a 9.47 g/t e Inferido de 515,700 oz Au; obtuvo estatus de "Covered Project" bajo FAST-41 el 30-jul-2026, acelerando la revisión federal coordinada; quinta mina en Alaska con cobertura FAST-41, junto con Arctic, Johnson Tract, Donlin Gold y Graphite Creek)</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>[MINING.COM](https://www.mining.com/american-tungsten-kinks-off-construction-at-ima-project-in-idaho/)</t>
+          <t>[Mining News North](https://www.miningnewsnorth.com/story/2026/08/07/news/new-amalga-gold-project-enters-fast-41/9803.html)</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -7479,17 +7440,17 @@
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>Railroad Valley Minerals / Super-Brine Complex</t>
+          <t>ElementUSA Gramercy — Planta de Tierras Raras/Minerales Críticos</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>Railroad Valley, Nevada, EE.UU.</t>
+          <t>Gramercy, St. John the Baptist Parish, Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>3 Proton Lithium (3PL Operating Inc.)</t>
+          <t>ElementUSA Inc. (en colaboración con Colorado School of Mines)</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
@@ -7499,71 +7460,71 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Exploración avanzada (depósito multi-mineral confirmado: litio, potasa, boro y lo que la empresa describe como el mayor depósito de tungsteno de EE.UU. —~1.78 millones de toneladas, valorado en ~US$152,000 millones in-situ—; ~17 millas cuadradas del área están retiradas de minería desde 2023 por solicitud de la NASA para calibración de satélites, lo que representa un obstáculo regulatorio; sin decisión de construcción)</t>
+          <t>Ingeniería/financiamiento asegurado (proyecto de US$850 millones para procesar "lodo rojo"/bauxite residue del antiguo refinerio de alúmina Atalco —~34 millones de toneladas almacenadas— y extraer galio, escandio, disprosio, gadolinio, iterbio, germanio e itrio; recibió US$67 millones del DOE y US$29.9 millones del DoD; construcción de planta de demostración prevista a iniciar mediados de 2027, producción inicial 3T2028); Atalco (refinería de alúmina que aloja el sitio, entidad distinta co-ubicada) recibió 28-ago-2026 una inversión de capital adicional de US$100 millones del Departamento de Guerra de EE.UU. —participación total del DoW ahora US$400M, US$800M contando coinversión privada desde ene-2026— para restaurar la refinería, única refinería de alúmina activa en EE.UU., a su capacidad nominal de 1.2 millones ton/año, lo que apoya indirectamente la operación de ElementUSA en el mismo sitio</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>[MINING.COM](https://www.mining.com/largest-us-tungsten-discovery-hits-nasa-roadblock/)</t>
+          <t>[Biz New Orleans](https://bizneworleans.com/elementusa-plans-850m-critical-minerals-refining-facility/); [Colorado School of Mines](https://www.minesnewsroom.com/news/colorado-school-mines-and-elementusa-awarded-67m-doe-construction-rare-earth-processing-plant); [Departamento de Guerra de EE.UU.](https://www.war.gov/News/Releases/Release/Article/4585310/department-of-war-announces-a-100-million-follow-on-equity-investment-in-atalco/)</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-09-02</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>New Amalga Gold Project</t>
+          <t>Planta de Refinación de Tierras Raras y Minerales Críticos Marion (ReElement Technologies)</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>~25 km al norte de Juneau, Alaska, EE.UU.</t>
+          <t>Marion, Indiana, EE.UU.</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>Grande Portage Resources Ltd.</t>
+          <t>American Resources Corporation (NASDAQ: AREC) vía subsidiaria ReElement Technologies</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>No especificado (acondicionamiento interno de la ex planta RCA Thomson, 425,000 pies² en campus de 42 acres)</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>Permitting temprano (recurso Indicado de 1.44 millones oz Au a 9.47 g/t e Inferido de 515,700 oz Au; obtuvo estatus de "Covered Project" bajo FAST-41 el 30-jul-2026, acelerando la revisión federal coordinada; quinta mina en Alaska con cobertura FAST-41, junto con Arctic, Johnson Tract, Donlin Gold y Graphite Creek)</t>
+          <t>Permiso de aire obtenido/comisionamiento (IDEM —Indiana— otorgó el permiso "Minor Source" para 4 líneas de producción de Fase 1, &gt;16,000 t/año de óxidos separados de alta pureza —Nd, Pr, Dy, Tb, Gd, Sm, Y, galio, germanio—; arranque de producción inicial previsto 3T2026)</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>[Mining News North](https://www.miningnewsnorth.com/story/2026/08/07/news/new-amalga-gold-project-enters-fast-41/9803.html)</t>
+          <t>[Mining Technology](https://www.mining-technology.com/news/air-permits-reelements-marion-refinery-indiana/); [Investing News Network](https://investingnews.com/reelement-technologies-receives-air-permits-for-marion-indiana-rare-earth-and-critical-mineral-refinery/)</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>ElementUSA Gramercy — Planta de Tierras Raras/Minerales Críticos</t>
+          <t>La Preciosa Project</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>Gramercy, St. John the Baptist Parish, Luisiana, EE.UU.</t>
+          <t>Durango, México</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>ElementUSA Inc. (en colaboración con Colorado School of Mines)</t>
+          <t>Avino Silver &amp; Gold Mines Ltd.</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
@@ -7573,71 +7534,71 @@
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/financiamiento asegurado (proyecto de US$850 millones para procesar "lodo rojo"/bauxite residue del antiguo refinerio de alúmina Atalco —~34 millones de toneladas almacenadas— y extraer galio, escandio, disprosio, gadolinio, iterbio, germanio e itrio; recibió US$67 millones del DOE y US$29.9 millones del DoD; construcción de planta de demostración prevista a iniciar mediados de 2027, producción inicial 3T2028); Atalco (refinería de alúmina que aloja el sitio, entidad distinta co-ubicada) recibió 28-ago-2026 una inversión de capital adicional de US$100 millones del Departamento de Guerra de EE.UU. —participación total del DoW ahora US$400M, US$800M contando coinversión privada desde ene-2026— para restaurar la refinería, única refinería de alúmina activa en EE.UU., a su capacidad nominal de 1.2 millones ton/año, lo que apoya indirectamente la operación de ElementUSA en el mismo sitio</t>
+          <t>Construcción (desarrollo subterráneo en curso —rampa/decline de 360m—; permisos mineros ya obtenidos; producción objetivo 4T2026)</t>
         </is>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>[Biz New Orleans](https://bizneworleans.com/elementusa-plans-850m-critical-minerals-refining-facility/); [Colorado School of Mines](https://www.minesnewsroom.com/news/colorado-school-mines-and-elementusa-awarded-67m-doe-construction-rare-earth-processing-plant); [Departamento de Guerra de EE.UU.](https://www.war.gov/News/Releases/Release/Article/4585310/department-of-war-announces-a-100-million-follow-on-equity-investment-in-atalco/)</t>
+          <t>[AccessWire](https://www.accessnewswire.com/newsroom/en/metals-and-mining/avino-provides-update-on-its-100-owned-la-preciosa-property-preparing-for-producti-837173); [MarketScreener](https://www.marketscreener.com/quote/stock/AVINO-SILVER-GOLD-MINES-L-1409069/news/Avino-Silver-Gold-Mines-Ltd-Commences-Underground-Development-At-La-Preciosa-48766238/)</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>Planta de Refinación de Tierras Raras y Minerales Críticos Marion (ReElement Technologies)</t>
+          <t>Great Salt Lake Lithium Facility</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>Marion, Indiana, EE.UU.</t>
+          <t>Condado de Box Elder, Utah, EE.UU.</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>American Resources Corporation (NASDAQ: AREC) vía subsidiaria ReElement Technologies</t>
+          <t>Lilac Solutions (subsidiaria Waterleaf P1 HoldCo)</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>No especificado (acondicionamiento interno de la ex planta RCA Thomson, 425,000 pies² en campus de 42 acres)</t>
+          <t>Hatch (EPCM, seleccionado jun-2026)</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>Permiso de aire obtenido/comisionamiento (IDEM —Indiana— otorgó el permiso "Minor Source" para 4 líneas de producción de Fase 1, &gt;16,000 t/año de óxidos separados de alta pureza —Nd, Pr, Dy, Tb, Gd, Sm, Y, galio, germanio—; arranque de producción inicial previsto 3T2026)</t>
+          <t>Desarrollo/Ingeniería (DOE anunció 20/21-ago-2026 subvención de hasta US$100 millones para construir planta comercial de extracción/refinación de litio por intercambio iónico directo desde salmuera del Great Salt Lake, 5,000 t/año; primera producción prevista 2028) ; DOE otorgó US$100 millones (anuncio 20-ago-2026) para la instalación comercial de extracción/refinación de litio mediante DLE de Lilac Solutions; capacidad de primera fase 5,000 ton/año, producción objetivo 2028</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>[Mining Technology](https://www.mining-technology.com/news/air-permits-reelements-marion-refinery-indiana/); [Investing News Network](https://investingnews.com/reelement-technologies-receives-air-permits-for-marion-indiana-rare-earth-and-critical-mineral-refinery/)</t>
+          <t>[KSL](https://www.ksl.com/article/51614351/california-company-awarded-100m-to-develop-critical-mineral-facility-on-great-salt-lake-shore); [Hatch](https://www.hatch.com/About-Us/News-And-Media/2026/06/Lilac-Solutions-Selects-Hatch-as-EPCM-Partner-for-Great-Salt-Lake-Lithium-Facility) ; [DOE](https://www.energy.gov/articles/energy-department-announces-500-million-secure-americas-critical-mineral-and-battery)</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>La Preciosa Project</t>
+          <t>Project SHIELD (refinería de "black mass" de baterías)</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>Durango, México</t>
+          <t>Carolina del Sur, EE.UU. (sitio exacto por definir)</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>Avino Silver &amp; Gold Mines Ltd.</t>
+          <t>Nth Cycle, Inc.</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
@@ -7647,49 +7608,49 @@
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>Construcción (desarrollo subterráneo en curso —rampa/decline de 360m—; permisos mineros ya obtenidos; producción objetivo 4T2026)</t>
+          <t>Negociación de subvención/preconstrucción (DOE seleccionó a Nth Cycle 20/21-ago-2026 para negociar premio de hasta US$100 millones; planta de refinación de "black mass" de baterías de litio, producirá MHP de níquel y carbonato de litio grado batería, 24,000 t/año; operación proyectada 2028)</t>
         </is>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>[AccessWire](https://www.accessnewswire.com/newsroom/en/metals-and-mining/avino-provides-update-on-its-100-owned-la-preciosa-property-preparing-for-producti-837173); [MarketScreener](https://www.marketscreener.com/quote/stock/AVINO-SILVER-GOLD-MINES-L-1409069/news/Avino-Silver-Gold-Mines-Ltd-Commences-Underground-Development-At-La-Preciosa-48766238/)</t>
+          <t>[Nth Cycle](https://nthcycle.com/newsroom/u.s.-department-of-energy-selects-nth-cycle-to-enter-award-negotiations-for-up-to-100-million-to-build-new-critical-mineral-refining-facility)</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>Great Salt Lake Lithium Facility</t>
+          <t>Refinería de Sulfato de Cobalto — Formation Holdings/Jervois</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>Condado de Box Elder, Utah, EE.UU.</t>
+          <t>Sitio por definir, EE.UU. (empresa con sede en Salmon, Idaho)</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>Lilac Solutions (subsidiaria Waterleaf P1 HoldCo)</t>
+          <t>Formation Holdings US, Inc. (dba Jervois)</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>Hatch (EPCM, seleccionado jun-2026)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>Desarrollo/Ingeniería (DOE anunció 20/21-ago-2026 subvención de hasta US$100 millones para construir planta comercial de extracción/refinación de litio por intercambio iónico directo desde salmuera del Great Salt Lake, 5,000 t/año; primera producción prevista 2028) ; DOE otorgó US$100 millones (anuncio 20-ago-2026) para la instalación comercial de extracción/refinación de litio mediante DLE de Lilac Solutions; capacidad de primera fase 5,000 ton/año, producción objetivo 2028</t>
+          <t>Desarrollo/financiamiento (DOE otorgó 21-ago-2026 subvención de US$100 millones para construir refinería comercial de sulfato de cobalto grado batería; ubicación específica de la planta aún no anunciada) ; DOE seleccionó el proyecto para un aporte federal de US$100 millones (anuncio 20-ago-2026) hacia una refinería comercial de cobalto; sitio industrial aún por determinar</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>[KSL](https://www.ksl.com/article/51614351/california-company-awarded-100m-to-develop-critical-mineral-facility-on-great-salt-lake-shore); [Hatch](https://www.hatch.com/About-Us/News-And-Media/2026/06/Lilac-Solutions-Selects-Hatch-as-EPCM-Partner-for-Great-Salt-Lake-Lithium-Facility) ; [DOE](https://www.energy.gov/articles/energy-department-announces-500-million-secure-americas-critical-mineral-and-battery)</t>
+          <t>[Local News 8](https://localnews8.com/news/business-watch/2026/08/21/salmon-company-wins-100-million-grant-to-build-cobalt-refinery/); [Local News 8 (seguimiento)](https://localnews8.com/news/local-news/2026/08/24/100m-grant-to-salmon-based-jervois-could-jumpstart-idahos-cobalt-industry/) ; [DOE](https://www.energy.gov/articles/energy-department-announces-500-million-secure-americas-critical-mineral-and-battery)</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
@@ -7701,106 +7662,106 @@
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>Project SHIELD (refinería de "black mass" de baterías)</t>
+          <t>Copperwood Project</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>Carolina del Sur, EE.UU. (sitio exacto por definir)</t>
+          <t>Península Superior Occidental, cerca de Wakefield, Michigan, EE.UU.</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>Nth Cycle, Inc.</t>
+          <t>Highland Copper Company</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>DRA Americas Inc. (FEED)</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>Negociación de subvención/preconstrucción (DOE seleccionó a Nth Cycle 20/21-ago-2026 para negociar premio de hasta US$100 millones; planta de refinación de "black mass" de baterías de litio, producirá MHP de níquel y carbonato de litio grado batería, 24,000 t/año; operación proyectada 2028)</t>
+          <t>Ingeniería/FEED (~40% completo para 4T2026; decisión de construcción esperada en 2S2026; producción de cobre proyectada 2029; capex ~US$425 millones)</t>
         </is>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>[Nth Cycle](https://nthcycle.com/newsroom/u.s.-department-of-energy-selects-nth-cycle-to-enter-award-negotiations-for-up-to-100-million-to-build-new-critical-mineral-refining-facility)</t>
+          <t>[Highland Copper](https://www.highlandcopper.com/news/highland-copper-recaps-2025-execution-and-announces-2026-work-plan-to-advance-copperwood-toward-construction-decision/)</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>Refinería de Sulfato de Cobalto — Formation Holdings/Jervois</t>
+          <t>Modernización Refinería de Cobre El Paso</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>Sitio por definir, EE.UU. (empresa con sede en Salmon, Idaho)</t>
+          <t>El Paso, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>Formation Holdings US, Inc. (dba Jervois)</t>
+          <t>Freeport-McMoRan</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>EPCM Group (tecnología de cátodos permanentes); Metso (equipo de tankhouse)</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>Desarrollo/financiamiento (DOE otorgó 21-ago-2026 subvención de US$100 millones para construir refinería comercial de sulfato de cobalto grado batería; ubicación específica de la planta aún no anunciada) ; DOE seleccionó el proyecto para un aporte federal de US$100 millones (anuncio 20-ago-2026) hacia una refinería comercial de cobalto; sitio industrial aún por determinar</t>
+          <t>Contrato adjudicado 2026 (modernización de refinería electrolítica, 46,650 cátodos permanentes, sustituye tecnología de láminas de arranque tradicional)</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>[Local News 8](https://localnews8.com/news/business-watch/2026/08/21/salmon-company-wins-100-million-grant-to-build-cobalt-refinery/); [Local News 8 (seguimiento)](https://localnews8.com/news/local-news/2026/08/24/100m-grant-to-salmon-based-jervois-could-jumpstart-idahos-cobalt-industry/) ; [DOE](https://www.energy.gov/articles/energy-department-announces-500-million-secure-americas-critical-mineral-and-battery)</t>
+          <t>[EPCM Group](https://www.epcm.com/epcm-secures-prestigious-contract-with-freeport-mcmoran-to-advance-el-paso-copper-refinery-modernization/)</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-26</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>Copperwood Project</t>
+          <t>Round Top Rare Earth Project</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>Península Superior Occidental, cerca de Wakefield, Michigan, EE.UU.</t>
+          <t>Sierra Blanca, Condado de Hudspeth, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>Highland Copper Company</t>
+          <t>USA Rare Earth Inc.</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>DRA Americas Inc. (FEED)</t>
+          <t>Fluor Corporation / WSP Global Inc. (EPCM para estudio de factibilidad definitivo)</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/FEED (~40% completo para 4T2026; decisión de construcción esperada en 2S2026; producción de cobre proyectada 2029; capex ~US$425 millones)</t>
+          <t>Ingeniería/DFS (en curso; subvención estatal de Texas de US$14.2 millones, may-2026; inversión estimada &gt;US$1,400 millones; producción adelantada a fines de 2028; tierras raras pesadas)</t>
         </is>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>[Highland Copper](https://www.highlandcopper.com/news/highland-copper-recaps-2025-execution-and-announces-2026-work-plan-to-advance-copperwood-toward-construction-decision/)</t>
+          <t>[IM Mining](https://im-mining.com/2026/01/23/fluor-and-wsp-on-board-usa-rare-earth-incs-round-top-rare-earth-project/)</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
@@ -7812,32 +7773,32 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>Modernización Refinería de Cobre El Paso</t>
+          <t>Expansión Fundición de Antimonio Thompson Falls</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>El Paso, Texas, EE.UU.</t>
+          <t>Thompson Falls, Montana, EE.UU.</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>Freeport-McMoRan</t>
+          <t>United States Antimony Corporation (USAC)</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>EPCM Group (tecnología de cátodos permanentes); Metso (equipo de tankhouse)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>Contrato adjudicado 2026 (modernización de refinería electrolítica, 46,650 cátodos permanentes, sustituye tecnología de láminas de arranque tradicional)</t>
+          <t>Comisionamiento (nueva fundición construida; comisionamiento de 9 hornos a gas iniciado may-2026; financiada con US$27 millones del Departamento de Guerra, mar-2026)</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>[EPCM Group](https://www.epcm.com/epcm-secures-prestigious-contract-with-freeport-mcmoran-to-advance-el-paso-copper-refinery-modernization/)</t>
+          <t>[Montana Public Radio](https://www.mtpr.org/montana-news/2026-04-06/montana-antimony-facility-expands-amid-federal-push-for-domestic-sources)</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
@@ -7849,32 +7810,32 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>Round Top Rare Earth Project</t>
+          <t>Expansión Planta de Lixiviación de Concentrados (CLP) Morenci</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>Sierra Blanca, Condado de Hudspeth, Texas, EE.UU.</t>
+          <t>Morenci, Arizona, EE.UU.</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>USA Rare Earth Inc.</t>
+          <t>Freeport-McMoRan</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>Fluor Corporation / WSP Global Inc. (EPCM para estudio de factibilidad definitivo)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/DFS (en curso; subvención estatal de Texas de US$14.2 millones, may-2026; inversión estimada &gt;US$1,400 millones; producción adelantada a fines de 2028; tierras raras pesadas)</t>
+          <t>Comisionamiento (segundo y último vaso de la expansión en comisionamiento/ajuste durante 2026; objetivo casi duplicar throughput de 24 a 40 ton/hora)</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>[IM Mining](https://im-mining.com/2026/01/23/fluor-and-wsp-on-board-usa-rare-earth-incs-round-top-rare-earth-project/)</t>
+          <t>[Freeport-McMoRan](https://www.fcx.com/freeport-features/112125)</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
@@ -7886,17 +7847,17 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>Expansión Fundición de Antimonio Thompson Falls</t>
+          <t>Reconstrucción Fundición y Refinería Kennecott</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>Thompson Falls, Montana, EE.UU.</t>
+          <t>Bingham Canyon/Kennecott, Utah, EE.UU.</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>United States Antimony Corporation (USAC)</t>
+          <t>Rio Tinto (Kennecott Utah Copper)</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
@@ -7906,12 +7867,12 @@
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>Comisionamiento (nueva fundición construida; comisionamiento de 9 hornos a gas iniciado may-2026; financiada con US$27 millones del Departamento de Guerra, mar-2026)</t>
+          <t>Construcción (reconstrucción de fundición US$300 millones y actualización de refinería/tankhouse y circuito de flotación de molibdeno US$120 millones en curso durante 2026; reparación adicional tras falla de horno flash en jun-2026, ~75 días)</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>[Montana Public Radio](https://www.mtpr.org/montana-news/2026-04-06/montana-antimony-facility-expands-amid-federal-push-for-domestic-sources)</t>
+          <t>[Mining.com](https://www.mining.com/web/rio-tinto-to-invest-almost-1-billion-in-kennecott-copper-mine/)</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
@@ -7923,32 +7884,32 @@
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>Expansión Planta de Lixiviación de Concentrados (CLP) Morenci</t>
+          <t>Fourmile (decline Bullion Hill)</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>Morenci, Arizona, EE.UU.</t>
+          <t>Carlin Trend, condados de Elko/Eureka, Nevada, EE.UU.</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>Freeport-McMoRan</t>
+          <t>Barrick Mining Corporation (JV Nevada Gold Mines, desde ago-2026)</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Barminco (Perenti) — contrato A$275 millones/45 meses</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>Comisionamiento (segundo y último vaso de la expansión en comisionamiento/ajuste durante 2026; objetivo casi duplicar throughput de 24 a 40 ton/hora)</t>
+          <t>Construcción (inicio de desarrollo subterráneo/portales programado jul/3T2026; ~16 km de desarrollo lateral subterráneo planeados; adyacente al complejo Goldrush)</t>
         </is>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>[Freeport-McMoRan](https://www.fcx.com/freeport-features/112125)</t>
+          <t>[Northern Miner](https://www.northernminer.com/news/mining-forum-americas-fourmile-anchors-barricks-nevada-plan/1003882789/)</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -7960,17 +7921,17 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>Reconstrucción Fundición y Refinería Kennecott</t>
+          <t>Puerto del Aire (distrito Mulatos)</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>Bingham Canyon/Kennecott, Utah, EE.UU.</t>
+          <t>Sonora, México</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>Rio Tinto (Kennecott Utah Copper)</t>
+          <t>Alamos Gold Inc.</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
@@ -7980,12 +7941,12 @@
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>Construcción (reconstrucción de fundición US$300 millones y actualización de refinería/tankhouse y circuito de flotación de molibdeno US$120 millones en curso durante 2026; reparación adicional tras falla de horno flash en jun-2026, ~75 días)</t>
+          <t>Construcción (en curso desde 2025-2026 tras permiso ambiental ene-2025; procura de equipos de molienda de largo plazo de entrega; capex total US$165 millones; primera producción prevista mediados 2027)</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>[Mining.com](https://www.mining.com/web/rio-tinto-to-invest-almost-1-billion-in-kennecott-copper-mine/)</t>
+          <t>[Alamos Gold](https://www.alamosgold.com/news-and-events/news/news-details/2025/Alamos-Gold-Announces-Receipt-of-Environmental-Permit-Amendment-Allowing-for-the-Start-of-Construction-on-the-Puerto-Del-Aire-Project-in-Mexico/default.aspx)</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -7997,54 +7958,54 @@
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>Fourmile (decline Bullion Hill)</t>
+          <t>Korea Zinc / Nyrstar Critical Minerals Smelter</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>Carlin Trend, condados de Elko/Eureka, Nevada, EE.UU.</t>
+          <t>Clarksville, Tennessee, EE.UU.</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>Barrick Mining Corporation (JV Nevada Gold Mines, desde ago-2026)</t>
+          <t>Korea Zinc / U.S. Department of War / U.S. Department of Commerce (participación ~10%)</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>Barminco (Perenti) — contrato A$275 millones/45 meses</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>Construcción (inicio de desarrollo subterráneo/portales programado jul/3T2026; ~16 km de desarrollo lateral subterráneo planeados; adyacente al complejo Goldrush)</t>
+          <t>Preparación de sitio en 2026, construcción completa en 2027 (inversión US$7,400 millones, capex US$6,600 millones; producirá zinc, plomo, cobre, oro, plata, antimonio, indio, bismuto, telurio, cadmio, galio, germanio, paladio y ácido sulfúrico; planta altamente intensiva en tubería/piping)</t>
         </is>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>[Northern Miner](https://www.northernminer.com/news/mining-forum-americas-fourmile-anchors-barricks-nevada-plan/1003882789/)</t>
+          <t>[Korea Zinc](https://www.koreazinc.co.kr/en/korea-zinc-partners-with-the-u-s-department-of-war-and-u-s-department-of-commerce-to-build-a-state-of-the-art-critical-minerals-smelter-in-the-united-states-with-6-6-billion-of-capital-expenditures/); [Carbon Credits](https://carboncredits.com/big-bet-bigger-stakes-korea-zincs-7-4-billion-smelter-reshapes-u-s-critical-minerals-supply/)</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>Puerto del Aire (distrito Mulatos)</t>
+          <t>Aclara Heavy Rare Earth Separation Facility</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>Sonora, México</t>
+          <t>Port of Vinton, Calcasieu Parish, Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>Alamos Gold Inc.</t>
+          <t>Aclara Resources Inc.</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
@@ -8054,34 +8015,34 @@
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>Construcción (en curso desde 2025-2026 tras permiso ambiental ene-2025; procura de equipos de molienda de largo plazo de entrega; capex total US$165 millones; primera producción prevista mediados 2027)</t>
+          <t>Planeación (inversión US$277 millones; groundbreaking previsto 4T2026, construcción hasta 2027; procesará mineral de depósitos propios en Brasil/Chile)</t>
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>[Alamos Gold](https://www.alamosgold.com/news-and-events/news/news-details/2025/Alamos-Gold-Announces-Receipt-of-Environmental-Permit-Amendment-Allowing-for-the-Start-of-Construction-on-the-Puerto-Del-Aire-Project-in-Mexico/default.aspx)</t>
+          <t>[Louisiana Economic Development](https://www.opportunitylouisiana.gov/news/aclara-invests-277-million-to-build-nations-first-heavy-rare-earth-separation-facility-in-southwest-louisiana)</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>Korea Zinc / Nyrstar Critical Minerals Smelter</t>
+          <t>Archimedes Project (i-80 Gold)</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>Clarksville, Tennessee, EE.UU.</t>
+          <t>Ruby Hill, Eureka County, Nevada, EE.UU.</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>Korea Zinc / U.S. Department of War / U.S. Department of Commerce (participación ~10%)</t>
+          <t>i-80 Gold Corp</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
@@ -8091,12 +8052,12 @@
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>Preparación de sitio en 2026, construcción completa en 2027 (inversión US$7,400 millones, capex US$6,600 millones; producirá zinc, plomo, cobre, oro, plata, antimonio, indio, bismuto, telurio, cadmio, galio, germanio, paladio y ácido sulfúrico; planta altamente intensiva en tubería/piping)</t>
+          <t>Construcción (permisos de Nevada DEP y BLM obtenidos; desarrollo subterráneo en curso; producción esperada 4T2026, objetivo 150,000-200,000 oz Au/año hacia 2028)</t>
         </is>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>[Korea Zinc](https://www.koreazinc.co.kr/en/korea-zinc-partners-with-the-u-s-department-of-war-and-u-s-department-of-commerce-to-build-a-state-of-the-art-critical-minerals-smelter-in-the-united-states-with-6-6-billion-of-capital-expenditures/); [Carbon Credits](https://carboncredits.com/big-bet-bigger-stakes-korea-zincs-7-4-billion-smelter-reshapes-u-s-critical-minerals-supply/)</t>
+          <t>[Resource World](https://resourceworld.com/i-80-gold-obtains-construction-permits-and-begins-underground-development-at-archimedes-project-nevada/)</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -8108,17 +8069,17 @@
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>Aclara Heavy Rare Earth Separation Facility</t>
+          <t>Sweetwater Uranium In-Situ Recovery (ISR) Project</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>Port of Vinton, Calcasieu Parish, Luisiana, EE.UU.</t>
+          <t>Sweetwater County, Wyoming, EE.UU.</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>Aclara Resources Inc.</t>
+          <t>Sweetwater Uranium, Inc.</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
@@ -8128,12 +8089,12 @@
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>Planeación (inversión US$277 millones; groundbreaking previsto 4T2026, construcción hasta 2027; procesará mineral de depósitos propios en Brasil/Chile)</t>
+          <t>Permitting (Plan de Operaciones sometido al BLM nov-2025, periodo de comentarios públicos mar-abr 2026, proyecto designado FAST-41; sería la mayor instalación de producción de uranio de EE.UU. combinando procesamiento convencional e ISR)</t>
         </is>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>[Louisiana Economic Development](https://www.opportunitylouisiana.gov/news/aclara-invests-277-million-to-build-nations-first-heavy-rare-earth-separation-facility-in-southwest-louisiana)</t>
+          <t>[BLM](https://www.blm.gov/announcement/sweetwater-uranium-situ-recovery-irs-project-mine-plan-operations)</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -8145,17 +8106,17 @@
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>Archimedes Project (i-80 Gold)</t>
+          <t>Velvet-Wood Uranium-Vanadium Project</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>Ruby Hill, Eureka County, Nevada, EE.UU.</t>
+          <t>San Juan County, Utah, EE.UU.</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>i-80 Gold Corp</t>
+          <t>Anfield Energy Inc.</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
@@ -8165,12 +8126,12 @@
       </c>
       <c r="E105" s="2" t="inlineStr">
         <is>
-          <t>Construcción (permisos de Nevada DEP y BLM obtenidos; desarrollo subterráneo en curso; producción esperada 4T2026, objetivo 150,000-200,000 oz Au/año hacia 2028)</t>
+          <t>Construcción (Fase 1 de construcción superficial completada jun-2026; desarrollo subterráneo Fase 2 en curso; regreso a producción previsto fines de 2026)</t>
         </is>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>[Resource World](https://resourceworld.com/i-80-gold-obtains-construction-permits-and-begins-underground-development-at-archimedes-project-nevada/)</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/06/01/3304179/0/en/Anfield-Energy-Inc-Completes-Phase-One-Surface-Construction-at-Velvet-Wood-Project.html)</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -8182,185 +8143,185 @@
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>Sweetwater Uranium In-Situ Recovery (ISR) Project</t>
+          <t>Twin Metals Minnesota</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>Sweetwater County, Wyoming, EE.UU.</t>
+          <t>Ely, Minnesota, EE.UU. (cerca de Boundary Waters)</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>Sweetwater Uranium, Inc.</t>
+          <t>Antofagasta plc (Twin Metals Minnesota LLC)</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>No definido</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
         <is>
-          <t>Permitting (Plan de Operaciones sometido al BLM nov-2025, periodo de comentarios públicos mar-abr 2026, proyecto designado FAST-41; sería la mayor instalación de producción de uranio de EE.UU. combinando procesamiento convencional e ISR)</t>
+          <t>Permitting/Pre-EIS (plan de mina formal —concentradora de flotación de 20,000 tpd, cobre-níquel-EGP— presentado ante BLM y Minnesota DNR; el gobernador Walz frenó el trámite estatal en ago-2026, pero el proceso federal continúa activo; construcción aún a años de distancia)</t>
         </is>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>[BLM](https://www.blm.gov/announcement/sweetwater-uranium-situ-recovery-irs-project-mine-plan-operations)</t>
+          <t>[MinnPost](http://www.minnpost.com/state-government/2026/08/walz-halts-state-action-on-mine-near-boundary-waters-but-federal-process-stays-on-track/); [Star Tribune](https://www.startribune.com/twin-metals-submits-formal-mine-plan-to-minnesota-federal-officials/566311242)</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>Velvet-Wood Uranium-Vanadium Project</t>
+          <t>Falcon Copper — Fundición y Refinería de Cobre (greenfield)</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>San Juan County, Utah, EE.UU.</t>
+          <t>Arizona (fundición) / Costa del Golfo (refinería), EE.UU. (sitios por definir)</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>Anfield Energy Inc.</t>
+          <t>Falcon Copper Corp. (MOU con Glencore)</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>No definido</t>
         </is>
       </c>
       <c r="E107" s="2" t="inlineStr">
         <is>
-          <t>Construcción (Fase 1 de construcción superficial completada jun-2026; desarrollo subterráneo Fase 2 en curso; regreso a producción previsto fines de 2026)</t>
+          <t>Evaluación/pre-FEED (proyecto greenfield de ~US$2,000 millones para fundición primaria de cobre más refinería electrolítica; sin sitio definitivo ni FID)</t>
         </is>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/06/01/3304179/0/en/Anfield-Energy-Inc-Completes-Phase-One-Surface-Construction-at-Velvet-Wood-Project.html)</t>
+          <t>[Fastmarkets](https://www.fastmarkets.com/insights/us-copper-smelting-equation-gap-or-glut-hotter-commodities-articles/); [Falcon Copper](https://www.falconcopper.com/projects/works)</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>Twin Metals Minnesota</t>
+          <t>Del Sol Refinery (antimonio/tungsteno) + White Spar Antimony Mine</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>Ely, Minnesota, EE.UU. (cerca de Boundary Waters)</t>
+          <t>Amargosa Valley, Nevada (refinería) / Arizona (mina), EE.UU.</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>Antofagasta plc (Twin Metals Minnesota LLC)</t>
+          <t>American Tungsten &amp; Antimony Corp (ATALF)</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>No definido</t>
+          <t>Metso Finland Oy (estudio de alcance)</t>
         </is>
       </c>
       <c r="E108" s="2" t="inlineStr">
         <is>
-          <t>Permitting/Pre-EIS (plan de mina formal —concentradora de flotación de 20,000 tpd, cobre-níquel-EGP— presentado ante BLM y Minnesota DNR; el gobernador Walz frenó el trámite estatal en ago-2026, pero el proceso federal continúa activo; construcción aún a años de distancia)</t>
+          <t>Ingeniería/estudio (adquirió el 28-jul-2026 la refinería hidrometalúrgica permisada de antimonio Del Sol —18,500 t/año de capacidad de alimentación— y la mina White Spar (AZ) como fuente de mineral; 1-sep-2026 contrató a Metso para estudio de alcance de un circuito de producción de paratungstato de amonio —APT—, Fase 1: 2,500 t/año, posible Fase 2 a 5,000 t/año; la refinería también recibirá mineral del proyecto Antimony Canyon, Utah)</t>
         </is>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>[MinnPost](http://www.minnpost.com/state-government/2026/08/walz-halts-state-action-on-mine-near-boundary-waters-but-federal-process-stays-on-track/); [Star Tribune](https://www.startribune.com/twin-metals-submits-formal-mine-plan-to-minnesota-federal-officials/566311242)</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/american-tungsten-and-antimony-announces-study-for-tungsten-production-at-del-sol-refinery-in-nevada-302866335.html); [PR Newswire](https://www.prnewswire.com/news-releases/american-tungsten-and-antimony-to-acquire-permitted-critical-metals-refinery-in-nevada-and-white-spar-antimony-mine-in-arizona-302836579.html)</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-02</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>Falcon Copper — Fundición y Refinería de Cobre (greenfield)</t>
+          <t>Spring Valley Gold Mine</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>Arizona (fundición) / Costa del Golfo (refinería), EE.UU. (sitios por definir)</t>
+          <t>Condado de Pershing, Nevada, EE.UU.</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>Falcon Copper Corp. (MOU con Glencore)</t>
+          <t>Solidus Resources LLC (subsidiaria de Waterton Gold)</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
-          <t>No definido</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E109" s="2" t="inlineStr">
         <is>
-          <t>Evaluación/pre-FEED (proyecto greenfield de ~US$2,000 millones para fundición primaria de cobre más refinería electrolítica; sin sitio definitivo ni FID)</t>
+          <t>Construcción (todos los permisos federales en mano —BLM aprobó el plan de operaciones—; proyecto totalmente financiado, ~US$1,300 millones de capital comprometido incl. stream de oro de US$670M de Wheaton Precious Metals; trabajos de sitio tempranos en curso, construcción completa inicia en 2026; primera producción de oro proyectada 1S2028; reservas probadas/probables de 3.8 Moz Au)</t>
         </is>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>[Fastmarkets](https://www.fastmarkets.com/insights/us-copper-smelting-equation-gap-or-glut-hotter-commodities-articles/); [Falcon Copper](https://www.falconcopper.com/projects/works)</t>
+          <t>[BLM](https://www.blm.gov/announcement/blm-approves-spring-valley-gold-mine-pershing-county); [Wheaton Precious Metals](https://www.wheatonpm.com/portfolio/development-projects/spring-valley/default.aspx); [The Pershing Post](https://www.thepershingpost.com/article/496,spring-valley-mine-project-moves-into-construction-phase-hiring-to-begin-in-2026)</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-03</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>Del Sol Refinery (antimonio/tungsteno) + White Spar Antimony Mine</t>
+          <t>Pitarrilla Project (plata-plomo-zinc)</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>Amargosa Valley, Nevada (refinería) / Arizona (mina), EE.UU.</t>
+          <t>160 km al norte de la ciudad de Durango, Durango, México</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>American Tungsten &amp; Antimony Corp (ATALF)</t>
+          <t>Endeavour Silver Corp.</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>Metso Finland Oy (estudio de alcance)</t>
+          <t>SGS Canada / SGS Bateman / JDS Energy &amp; Mining / T Engineering / Stantec / SRK Consulting (estudio de factibilidad)</t>
         </is>
       </c>
       <c r="E110" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/estudio (adquirió el 28-jul-2026 la refinería hidrometalúrgica permisada de antimonio Del Sol —18,500 t/año de capacidad de alimentación— y la mina White Spar (AZ) como fuente de mineral; 1-sep-2026 contrató a Metso para estudio de alcance de un circuito de producción de paratungstato de amonio —APT—, Fase 1: 2,500 t/año, posible Fase 2 a 5,000 t/año; la refinería también recibirá mineral del proyecto Antimony Canyon, Utah)</t>
+          <t>Ingeniería/estudio de factibilidad (inversión 2026 de US$65.8 millones: US$15M para estudio de factibilidad, US$48M en capex de preparación minera y 1,300 m de desarrollo subterráneo; aún sin decisión de construcción)</t>
         </is>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/american-tungsten-and-antimony-announces-study-for-tungsten-production-at-del-sol-refinery-in-nevada-302866335.html); [PR Newswire](https://www.prnewswire.com/news-releases/american-tungsten-and-antimony-to-acquire-permitted-critical-metals-refinery-in-nevada-and-white-spar-antimony-mine-in-arizona-302836579.html)</t>
+          <t>[Mexico Business News](https://mexicobusiness.news/mining/news/endeavour-silver-forecasts-89moz-silver-2026); [Endeavour Silver](https://edrsilver.com/portfolio/development/pitarrilla/)</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
     </row>
@@ -8378,13 +8339,13 @@
   <dimension ref="A1:G101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Monitoreo 2026-09-03: 2 proyectos nuevos + 2 actualizaciones de fase (#36)
- Nuevos: Spring Valley Gold Mine (NV), Pitarrilla Project (Durango)
- Actualizaciones: Plaquemines LNG Fase 2 (gasoducto Delta Access de
  Williams), Planta de Purificación de Grafito US Army (sitio primario
  confirmado en Pine Bluff Arsenal)
- proyectos.xlsx regenerado con el acumulado completo (309 proyectos)


Claude-Session: https://claude.ai/code/session_013AGyaisBCeoWfGs74eCHnn

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -54,9 +54,7 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -425,16 +423,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G56"/>
+  <dimension ref="A1:G55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -810,276 +808,276 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Proyecto Escolín (amoniaco/urea)</t>
+          <t>Rehab. Fertinal-ProAgro (urea y fosfatos)</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Poza Rica, Veracruz, México</t>
+          <t>Lázaro Cárdenas, Michoacán, México</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Pemex Transformación Industrial</t>
+          <t>Pemex</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Mota-Engil México (EPC confirmado, US$1,200 millones, 47 meses); Duro Felguera (España) se integró formalmente 17-ago-2026 al contrato para gestión de proyecto y coordinación técnica de la ingeniería (supervisión de ingeniería externa, coordinación de suministros del tecnólogo, gestión de sistemas auxiliares); Casale (proveedor de tecnología)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/inicio de construcción (inversión confirmada US$1,553 millones; capacidad objetivo &gt;700,000 ton/año de amoniaco, urea y AdBlue; citado explícitamente por la Presidenta Sheinbaum en su Segundo Informe de Gobierno —1-sep-2026— como parte del "rescate de la petroquímica" junto con Cosoleacaque, Morelos y Cangrejera)</t>
+          <t>Ingeniería/rehabilitación (incorporado al plan de reactivación petroquímica de Pemex, jun-2026; 13,700 millones de pesos asignados para los complejos Lázaro Cárdenas y ProAgro; meta de 2.4 millones ton/año de urea y fertilizantes fosfatados)</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>[Forbes México](https://forbes.com.mx/asi-es-la-inversion-de-1553-mdd-por-parte-de-pemex-en-una-planta-de-fertilizantes-en-veracruz/); [El Español](https://www.elespanol.com/invertia/empresas/energia/20260817/duro-felguera-convoca-junta-extraordinaria-septiembre-aprobar-proyecto-clave-mota-engil-mexico/1003744355543_0.html); [La Política en Rosa](https://www.lapoliticaenrosa.com/2026/09/01/desde-veracruz-inicia-rescate-de-petroquimica-del-pais-destaca-claudia-sheinbaum-en-segundo-informe-de-gobierno/)</t>
+          <t>[Tribuna](https://tribuna.com.mx/mexico/2026/06/05/sheinbaum-anuncia-inversion-de-93-mil-mdp-para-reactivar-la-industria-petroquimica-y-de-fertilizantes-en-veracruz_560837/); [Contralínea](https://contralinea.com.mx/interno/semana/presentan-plan-con-inversion-de-93-mil-mdp-para-rescatar-la-petroquimica-nacional/)</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Rehab. Fertinal-ProAgro (urea y fosfatos)</t>
+          <t>Pacífico Mexinol (metanol ultra bajo carbono)</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Lázaro Cárdenas, Michoacán, México</t>
+          <t>Topolobampo, Sinaloa, México</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Pemex</t>
+          <t>Transition Industries</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Siemens Energy / Techint E&amp;C (FEED electrolizador)</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/rehabilitación (incorporado al plan de reactivación petroquímica de Pemex, jun-2026; 13,700 millones de pesos asignados para los complejos Lázaro Cárdenas y ProAgro; meta de 2.4 millones ton/año de urea y fertilizantes fosfatados)</t>
+          <t>Construcción (iniciada abr-2026)</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>[Tribuna](https://tribuna.com.mx/mexico/2026/06/05/sheinbaum-anuncia-inversion-de-93-mil-mdp-para-reactivar-la-industria-petroquimica-y-de-fertilizantes-en-veracruz_560837/); [Contralínea](https://contralinea.com.mx/interno/semana/presentan-plan-con-inversion-de-93-mil-mdp-para-rescatar-la-petroquimica-nacional/)</t>
+          <t>[PV Magazine México](https://www.pv-magazine-mexico.com/2026/04/28/inician-en-sinaloa-la-construccion-de-la-mayor-planta-de-metanol-ultrabajo-en-carbono-a-partir-de-hidrogeno-verde/)</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-10</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Pacífico Mexinol (metanol ultra bajo carbono)</t>
+          <t>First Ammonia (amoniaco verde)</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Topolobampo, Sinaloa, México</t>
+          <t>Victoria, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Transition Industries</t>
+          <t>First Ammonia / Cox Group USA</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Siemens Energy / Techint E&amp;C (FEED electrolizador)</t>
+          <t>Worley (FEED); Topsoe (tecnología de síntesis de amoniaco, seleccionada 12-ago-2026)</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Construcción (iniciada abr-2026)</t>
+          <t>Ingeniería (FEED completo; Topsoe suministrará su tecnología dinámica de síntesis de amoniaco) / cierre financiero esperado en 2026, FID prevista 2026, operación comercial estimada 2029</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>[PV Magazine México](https://www.pv-magazine-mexico.com/2026/04/28/inician-en-sinaloa-la-construccion-de-la-mayor-planta-de-metanol-ultrabajo-en-carbono-a-partir-de-hidrogeno-verde/)</t>
+          <t>[H2 View](https://www.h2-view.com/story/first-ammonia-project-on-track-for-2026-fid-despite-topsoe-deal-collapse/2138792.article/); [World Fertilizer](https://www.worldfertilizer.com/project-news/12082026/topsoe-to-provide-technology-for-first-ammonia/); [Topsoe](https://www.topsoe.com/news/topsoe-to-provide-ammonia-technology-for-first-ammonias-green-ammonia-project-in-texas)</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-08-20</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>First Ammonia (amoniaco verde)</t>
+          <t>Planta de Amoniaco Topolobampo (GPO) — Bahía de Ohuira</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Victoria, Texas, EE.UU.</t>
+          <t>Topolobampo, Ahome, Sinaloa, México</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>First Ammonia / Cox Group USA</t>
+          <t>Gas y Petroquímica de Occidente (GPO) / Proman AG</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Worley (FEED); Topsoe (tecnología de síntesis de amoniaco, seleccionada 12-ago-2026)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería (FEED completo; Topsoe suministrará su tecnología dinámica de síntesis de amoniaco) / cierre financiero esperado en 2026, FID prevista 2026, operación comercial estimada 2029</t>
+          <t>Construcción parcial/PAUSA parcial (unidad de amoniaco ~95% completa según Presidencia, ago-2026 —prensa local cita 88% de avance—, aunque reportes locales previos citaban solo ~60% con obra detenida por bloqueo; movimiento indígena yoreme-mayo "¡Aquí No!" mantiene plantón bloqueando el acceso de personal a la obra desde el 7-jun-2026; GPO ofreció (8/10-ago-2026) pausar formalmente las fases de urea, metanol y terminal marina como condición para levantar el bloqueo; Secretaría de Economía sostuvo reuniones con comunidades de Ohuira, Paredones, Lázaro Cárdenas y Topolobampo presentando el "Plan Integral", pero las comunidades respondieron con desconfianza y mantienen el plantón indefinido; nueva gobernadora interina de Sinaloa, Graciela Domínguez Nava, anunció el 26-ago-2026 que el gobierno estatal se sumará a la ruta federal de diálogo con la comunidad mayo-yoreme y GPO para destrabar el conflicto)</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>[H2 View](https://www.h2-view.com/story/first-ammonia-project-on-track-for-2026-fid-despite-topsoe-deal-collapse/2138792.article/); [World Fertilizer](https://www.worldfertilizer.com/project-news/12082026/topsoe-to-provide-technology-for-first-ammonia/); [Topsoe](https://www.topsoe.com/news/topsoe-to-provide-ammonia-technology-for-first-ammonias-green-ammonia-project-in-texas)</t>
+          <t>[Ríodoce](https://riodoce.mx/2026/08/10/pausan-urea-y-metanol-pero-avanza-amoniaco-en-industria-en-la-bahia-de-ohuira/); [La Silla Rota](https://lasillarota.com/estados/2026/8/8/planta-de-amoniaco-en-sinaloa-gobierno-busca-luz-verde-al-proyecto-en-ohuira-523789.html); [Infobae](https://www.infobae.com/mexico/2026/08/26/topolobampo-entre-las-prioridades-de-graciela-dominguez-promete-atender-a-comunidad-mayo-yoreme-y-a-empresarios/)</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Planta de Amoniaco Topolobampo (GPO) — Bahía de Ohuira</t>
+          <t>Lake Charles Methanol II</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Topolobampo, Ahome, Sinaloa, México</t>
+          <t>Lake Charles, Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Gas y Petroquímica de Occidente (GPO) / Proman AG</t>
+          <t>Lake Charles Methanol II LLC</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Zachry Group (FEED)</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Construcción parcial/PAUSA parcial (unidad de amoniaco ~95% completa según Presidencia, ago-2026 —prensa local cita 88% de avance—, aunque reportes locales previos citaban solo ~60% con obra detenida por bloqueo; movimiento indígena yoreme-mayo "¡Aquí No!" mantiene plantón bloqueando el acceso de personal a la obra desde el 7-jun-2026; GPO ofreció (8/10-ago-2026) pausar formalmente las fases de urea, metanol y terminal marina como condición para levantar el bloqueo; Secretaría de Economía sostuvo reuniones con comunidades de Ohuira, Paredones, Lázaro Cárdenas y Topolobampo presentando el "Plan Integral", pero las comunidades respondieron con desconfianza y mantienen el plantón indefinido; nueva gobernadora interina de Sinaloa, Graciela Domínguez Nava, anunció el 26-ago-2026 que el gobierno estatal se sumará a la ruta federal de diálogo con la comunidad mayo-yoreme y GPO para destrabar el conflicto)</t>
+          <t>Ingeniería (FEED) / FID prevista</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>[Ríodoce](https://riodoce.mx/2026/08/10/pausan-urea-y-metanol-pero-avanza-amoniaco-en-industria-en-la-bahia-de-ohuira/); [La Silla Rota](https://lasillarota.com/estados/2026/8/8/planta-de-amoniaco-en-sinaloa-gobierno-busca-luz-verde-al-proyecto-en-ohuira-523789.html); [Infobae](https://www.infobae.com/mexico/2026/08/26/topolobampo-entre-las-prioridades-de-graciela-dominguez-promete-atender-a-comunidad-mayo-yoreme-y-a-empresarios/)</t>
+          <t>[ICIS](https://www.icis.com/explore/resources/news/2025/11/13/11155109/lake-charles-methanol-ii-awards-feed-fid-expected-in-q2-2026/)</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Lake Charles Methanol II</t>
+          <t>Planta Coquizadora Salina Cruz</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Lake Charles, Luisiana, EE.UU.</t>
+          <t>Salina Cruz, Oaxaca, México</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Lake Charles Methanol II LLC</t>
+          <t>Pemex</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Zachry Group (FEED)</t>
+          <t>ICA Fluor</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería (FEED) / FID prevista</t>
+          <t>Construcción (~74% avance; Pemex confirmó retraso en el cronograma, finalización ahora prevista para 2S2027; avance reafirmado por la Presidenta Sheinbaum en su Segundo Informe de Gobierno, 1-sep-2026, como parte del programa de rehabilitación del Sistema Nacional de Refinación)</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>[ICIS](https://www.icis.com/explore/resources/news/2025/11/13/11155109/lake-charles-methanol-ii-awards-feed-fid-expected-in-q2-2026/)</t>
+          <t>[Diario del Istmo](https://diariodelistmo.com/nacional/este-es-el-avance-que-lleva-la-planta-coquizadora-en-la-refineria-de-salina-cruz/50642321); [Mexico Business News](https://mexicobusiness.news/oilandgas/news/salina-cruz-refinery-miss-construction-deadline-pemex); [La Razón](https://www.razon.com.mx/negocios/2026/09/01/sheinbaum-destaca-reduccion-de-deuda-de-pemex-y-avances-en-soberania-energetica/)</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-09-02</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Planta Coquizadora Salina Cruz</t>
+          <t>Shintech Louisiana — Expansión Plaquemine (2do craqueador de etileno + 4ta unidad cloro-álcali/VCM)</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Salina Cruz, Oaxaca, México</t>
+          <t>Plaquemine, Iberville Parish, Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Pemex</t>
+          <t>Shintech Louisiana, LLC</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>ICA Fluor</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Construcción (~74% avance; Pemex confirmó retraso en el cronograma, finalización ahora prevista para 2S2027; avance reafirmado por la Presidenta Sheinbaum en su Segundo Informe de Gobierno, 1-sep-2026, como parte del programa de rehabilitación del Sistema Nacional de Refinación)</t>
+          <t>Ingeniería/planeación (construcción por fases, 1a fase prevista 2030)</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>[Diario del Istmo](https://diariodelistmo.com/nacional/este-es-el-avance-que-lleva-la-planta-coquizadora-en-la-refineria-de-salina-cruz/50642321); [Mexico Business News](https://mexicobusiness.news/oilandgas/news/salina-cruz-refinery-miss-construction-deadline-pemex); [La Razón](https://www.razon.com.mx/negocios/2026/09/01/sheinbaum-destaca-reduccion-de-deuda-de-pemex-y-avances-en-soberania-energetica/)</t>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/petrochemicals/06032026/shintech-announces-us34-billion-at-louisiana-petrochemicals-complex/)</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-07-14</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Shintech Louisiana — Expansión Plaquemine (2do craqueador de etileno + 4ta unidad cloro-álcali/VCM)</t>
+          <t>Sandpiper Chemicals (metanol bajo carbono)</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Plaquemine, Iberville Parish, Luisiana, EE.UU.</t>
+          <t>Texas City, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Shintech Louisiana, LLC</t>
+          <t>Sandpiper Chemicals, LLC / INEOS Acetyls (colaboración estratégica, abr-2026)</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -1089,86 +1087,86 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/planeación (construcción por fases, 1a fase prevista 2030)</t>
+          <t>Ingeniería (FEED en curso desde 2T2026; US$1,700 millones, 1.1 MMtpa; INEOS Acetyls tomará 300,000 ton/año para su unidad de ácido acético) / FID prevista 2027, primera producción ~2030</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/petrochemicals/06032026/shintech-announces-us34-billion-at-louisiana-petrochemicals-complex/)</t>
+          <t>[INEOS](https://www.ineos.com/news/shared-news/ineos-acetyls-and-sandpiper-chemicals-announce-strategic-collaboration-for-the-development-of-a-low-carbon-methanol-project-in-texas-city-texas/)</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-29</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Sandpiper Chemicals (metanol bajo carbono)</t>
+          <t>OXEA Bay City Capacity Expansion + Air Liquide POX Syngas Unit</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Texas City, Texas, EE.UU.</t>
+          <t>Bay City, Matagorda County, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Sandpiper Chemicals, LLC / INEOS Acetyls (colaboración estratégica, abr-2026)</t>
+          <t>OXEA (oxo chemicals) / Air Liquide (unidad de syngas)</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Air Liquide (unidad propia); OXEA no especificado</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería (FEED en curso desde 2T2026; US$1,700 millones, 1.1 MMtpa; INEOS Acetyls tomará 300,000 ton/año para su unidad de ácido acético) / FID prevista 2027, primera producción ~2030</t>
+          <t>Construcción (FID confirmado 13-jul-2026; preparación de sitio 3T2026; finalización fines de 2028)</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>[INEOS](https://www.ineos.com/news/shared-news/ineos-acetyls-and-sandpiper-chemicals-announce-strategic-collaboration-for-the-development-of-a-low-carbon-methanol-project-in-texas-city-texas/)</t>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/petrochemicals/13072026/oxea-confirms-fid-for-major-capacity-expansion/)</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>OXEA Bay City Capacity Expansion + Air Liquide POX Syngas Unit</t>
+          <t>Targa Resources East Driver Gas Processing Plant</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Bay City, Matagorda County, Texas, EE.UU.</t>
+          <t>Condado de Midland, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>OXEA (oxo chemicals) / Air Liquide (unidad de syngas)</t>
+          <t>Targa Resources Corp.</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Air Liquide (unidad propia); OXEA no especificado</t>
+          <t>Targa Resources (propietario-constructor)</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Construcción (FID confirmado 13-jul-2026; preparación de sitio 3T2026; finalización fines de 2028)</t>
+          <t>Construcción (planta criogénica 275 MMcf/d; arranque previsto 3T2026)</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/petrochemicals/13072026/oxea-confirms-fid-for-major-capacity-expansion/)</t>
+          <t>[OGJ](https://www.ogj.com/refining-processing/gas-processing/news/55320579/targa-advances-permian-gas-pipeline-processing-expansion)</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -1180,32 +1178,32 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Targa Resources East Driver Gas Processing Plant</t>
+          <t>Enterprise Products "Athena" Natural Gas Processing Plant</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Condado de Midland, Texas, EE.UU.</t>
+          <t>Cuenca Midland (cuatro condados), Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Targa Resources Corp.</t>
+          <t>Enterprise Products Partners L.P.</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Targa Resources (propietario-constructor)</t>
+          <t>Enterprise Products (propietario-constructor)</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Construcción (planta criogénica 275 MMcf/d; arranque previsto 3T2026)</t>
+          <t>Construcción (300 MMcf/d + hasta 40,000 bpd de NGLs; en servicio 4T2026)</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>[OGJ](https://www.ogj.com/refining-processing/gas-processing/news/55320579/targa-advances-permian-gas-pipeline-processing-expansion)</t>
+          <t>[Business Wire](https://www.businesswire.com/news/home/20250806663187/en/Enterprise-Agrees-to-Acquire-Occidentals-Gas-Gathering-Affiliate-Enters-Into-Natural-Gas-Processing-Agreement-Announces-New-Midland-Basin-Natural-Gas-Processing-Plant)</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -1217,32 +1215,32 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Enterprise Products "Athena" Natural Gas Processing Plant</t>
+          <t>MPLX Secretariat II Gas Processing Plant</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Cuenca Midland (cuatro condados), Texas, EE.UU.</t>
+          <t>Cuenca Pérmica (subcuenca Delaware), Texas/Nuevo México, EE.UU.</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Enterprise Products Partners L.P.</t>
+          <t>MPLX LP</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Enterprise Products (propietario-constructor)</t>
+          <t>MPLX (propietario-constructor)</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Construcción (300 MMcf/d + hasta 40,000 bpd de NGLs; en servicio 4T2026)</t>
+          <t>Planeada/desarrollo (300 MMcf/d; en servicio 2S2028)</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>[Business Wire](https://www.businesswire.com/news/home/20250806663187/en/Enterprise-Agrees-to-Acquire-Occidentals-Gas-Gathering-Affiliate-Enters-Into-Natural-Gas-Processing-Agreement-Announces-New-Midland-Basin-Natural-Gas-Processing-Plant)</t>
+          <t>[Natural Gas Intel](https://naturalgasintel.com/news/mplx-scales-up-for-power-hungry-future-with-natural-gas-focused-growth-plan/)</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -1254,12 +1252,12 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>MPLX Secretariat II Gas Processing Plant</t>
+          <t>MPLX Titan Complex (Northwind) — Expansión de Tratamiento de Gas Amargo</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Cuenca Pérmica (subcuenca Delaware), Texas/Nuevo México, EE.UU.</t>
+          <t>Condado de Lea, Nuevo México / frontera TX-NM, EE.UU.</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -1274,12 +1272,12 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Planeada/desarrollo (300 MMcf/d; en servicio 2S2028)</t>
+          <t>Construcción (expansión de capacidad &gt;400 MMcf/d; plenamente operativo 4T2026)</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>[Natural Gas Intel](https://naturalgasintel.com/news/mplx-scales-up-for-power-hungry-future-with-natural-gas-focused-growth-plan/)</t>
+          <t>[East Daley](https://eastdaley.com/daley-note/mplx-acquires-northwind-for-2-375b-acquires-more-ngls-for-jv-project)</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -1291,32 +1289,32 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>MPLX Titan Complex (Northwind) — Expansión de Tratamiento de Gas Amargo</t>
+          <t>Northern Plains Nitrogen (urea/amoniaco)</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Condado de Lea, Nuevo México / frontera TX-NM, EE.UU.</t>
+          <t>Grand Forks, Dakota del Norte, EE.UU.</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>MPLX LP</t>
+          <t>Northern Plains Nitrogen LLC</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>MPLX (propietario-constructor)</t>
+          <t>EPC no designado</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Construcción (expansión de capacidad &gt;400 MMcf/d; plenamente operativo 4T2026)</t>
+          <t>Pre-FEED completo / FID buscada 4T2026</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>[East Daley](https://eastdaley.com/daley-note/mplx-acquires-northwind-for-2-375b-acquires-more-ngls-for-jv-project)</t>
+          <t>[Grand Forks Herald](https://www.grandforksherald.com/news/local/northern-plains-nitrogen-proposal-receiving-more-attention-amid-global-fertilizer-pressure)</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -1328,54 +1326,54 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Northern Plains Nitrogen (urea/amoniaco)</t>
+          <t>Iron Mesa (planta de gas)</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Grand Forks, Dakota del Norte, EE.UU.</t>
+          <t>Goldsmith, Ector County, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Northern Plains Nitrogen LLC</t>
+          <t>Phillips 66</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>EPC no designado</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Pre-FEED completo / FID buscada 4T2026</t>
+          <t>Construcción (arranque previsto Q1 2027)</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>[Grand Forks Herald](https://www.grandforksherald.com/news/local/northern-plains-nitrogen-proposal-receiving-more-attention-amid-global-fertilizer-pressure)</t>
+          <t>[Phillips 66](https://www.phillips66.com/newsroom/iron-mesa-safely-enters-next-phase-of-construction/)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-15</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Iron Mesa (planta de gas)</t>
+          <t>Yeti II (planta de gas)</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Goldsmith, Ector County, Texas, EE.UU.</t>
+          <t>Cuenca Delaware (Permian), Texas/Nuevo México, EE.UU.</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Phillips 66</t>
+          <t>Targa Resources</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1385,12 +1383,12 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Construcción (arranque previsto Q1 2027)</t>
+          <t>Ingeniería/planeación (en línea previsto Q4 2027)</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>[Phillips 66](https://www.phillips66.com/newsroom/iron-mesa-safely-enters-next-phase-of-construction/)</t>
+          <t>[Targa Resources](https://www.targaresources.com/news-releases/news-release-details/targa-resources-corp-announces-permian-growth-projects-and)</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -1402,32 +1400,32 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Yeti II (planta de gas)</t>
+          <t>Refinería Francisco I. Madero (rehabilitación)</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Cuenca Delaware (Permian), Texas/Nuevo México, EE.UU.</t>
+          <t>Ciudad Madero, Tamaulipas, México</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Targa Resources</t>
+          <t>Pemex</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Múltiples contratistas por licitar (30+ licitaciones)</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/planeación (en línea previsto Q4 2027)</t>
+          <t>Licitación/bidding</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>[Targa Resources](https://www.targaresources.com/news-releases/news-release-details/targa-resources-corp-announces-permian-growth-projects-and)</t>
+          <t>[Elefante Blanco](https://elefanteblanco.mx/2026/01/02/pemex-abre-30-licitaciones-para-obras-en-la-refineria-madero/)</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -1439,106 +1437,106 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Refinería Francisco I. Madero (rehabilitación)</t>
+          <t>Fermachem Planta de Urea/Amoniaco</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Ciudad Madero, Tamaulipas, México</t>
+          <t>Ejido Sapioris, Lerdo, Durango, México</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Pemex</t>
+          <t>Fermaca Dreams (Fermachem)</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Múltiples contratistas por licitar (30+ licitaciones)</t>
+          <t>Técnicas Reunidas (licencia/tecnología KBR-Stamicarbon)</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Licitación/bidding</t>
+          <t>Construcción con retraso administrativo (obra pausada ~mes y medio por revisión legal/administrativa; Secretario de Desarrollo Económico de Durango confirmó 13-ago-2026 que Semarnat y Profepa no encontraron impedimento, reanudación de obra esperada en 1-2 semanas)</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>[Elefante Blanco](https://elefanteblanco.mx/2026/01/02/pemex-abre-30-licitaciones-para-obras-en-la-refineria-madero/)</t>
+          <t>[La Jornada](https://www.jornada.com.mx/noticia/2026/06/08/economia/da-inicio-ejecucion-de-planta-de-fertilizantes-en-durango-por-parte-de-fermachem); [Grem Noticieros](https://www.noticierosgrem.com.mx/costruccion-de-fermachem-podria-arrancar-en-dos-semanas-desarrollo-economico-de-durango/)</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-08-18</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Fermachem Planta de Urea/Amoniaco</t>
+          <t>Ascension Clean Energy (ACE) — amoniaco azul</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Ejido Sapioris, Lerdo, Durango, México</t>
+          <t>Donaldsonville, Ascension Parish, Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Fermaca Dreams (Fermachem)</t>
+          <t>Clean Hydrogen Works</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Técnicas Reunidas (licencia/tecnología KBR-Stamicarbon)</t>
+          <t>McDermott (FEED)</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Construcción con retraso administrativo (obra pausada ~mes y medio por revisión legal/administrativa; Secretario de Desarrollo Económico de Durango confirmó 13-ago-2026 que Semarnat y Profepa no encontraron impedimento, reanudación de obra esperada en 1-2 semanas)</t>
+          <t>Ingeniería (FEED) / Pre-FID</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>[La Jornada](https://www.jornada.com.mx/noticia/2026/06/08/economia/da-inicio-ejecucion-de-planta-de-fertilizantes-en-durango-por-parte-de-fermachem); [Grem Noticieros](https://www.noticierosgrem.com.mx/costruccion-de-fermachem-podria-arrancar-en-dos-semanas-desarrollo-economico-de-durango/)</t>
+          <t>[Downstream Calendar](https://downstreamcalendar.com/mcdermott-secures-feed-contract-for-ascension-clean-energy-project/)</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-07-17</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Ascension Clean Energy (ACE) — amoniaco azul</t>
+          <t>Zeus Gas Plant + 3ra Fraccionadora Coastal Bend</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Donaldsonville, Ascension Parish, Luisiana, EE.UU.</t>
+          <t>Cuenca Pérmica, Texas / Robstown, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Clean Hydrogen Works</t>
+          <t>Phillips 66</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>McDermott (FEED)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería (FEED) / Pre-FID</t>
+          <t>Ingeniería (sancionado; en línea 2028)</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>[Downstream Calendar](https://downstreamcalendar.com/mcdermott-secures-feed-contract-for-ascension-clean-energy-project/)</t>
+          <t>[Business Wire](https://www.businesswire.com/news/home/20260517310811/en/Phillips-66-announces-Zeus-Gas-Plant-and-a-third-Coastal-Bend-Fractionator)</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -1550,128 +1548,128 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Zeus Gas Plant + 3ra Fraccionadora Coastal Bend</t>
+          <t>Project Meadowlark (complejo de amoniaco azul/UAN/ATS/DEF)</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Cuenca Pérmica, Texas / Robstown, Texas, EE.UU.</t>
+          <t>Gothenburg, Nebraska, EE.UU.</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Phillips 66</t>
+          <t>J. Westling &amp; Co. (JWC Gburg, LLC)</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>No especificado (tecnología licenciada Topsoe SynCOR Ammonia); contrato EPC/fabricación asegurado</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería (sancionado; en línea 2028)</t>
+          <t>Ingeniería/Permisos (permiso de aire emitido, sitio zonificado; obras civiles previstas 2027, operación comercial 2029)</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>[Business Wire](https://www.businesswire.com/news/home/20260517310811/en/Phillips-66-announces-Zeus-Gas-Plant-and-a-third-Coastal-Bend-Fractionator)</t>
+          <t>[USDA](https://www.usda.gov/about-usda/news/press-releases/2026/07/01/secretary-rollins-announces-500-million-fertilizer-investment-and-expansion-program-strengthen)</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Project Meadowlark (complejo de amoniaco azul/UAN/ATS/DEF)</t>
+          <t>Wabash Low-Carbon Ammonia Project</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Gothenburg, Nebraska, EE.UU.</t>
+          <t>West Terre Haute, Indiana, EE.UU.</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>J. Westling &amp; Co. (JWC Gburg, LLC)</t>
+          <t>Wabash Valley Resources</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>No especificado (tecnología licenciada Topsoe SynCOR Ammonia); contrato EPC/fabricación asegurado</t>
+          <t>Samsung E&amp;C (contrato EPF ~US$475 millones)</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/Permisos (permiso de aire emitido, sitio zonificado; obras civiles previstas 2027, operación comercial 2029)</t>
+          <t>Construcción (groundbreaking 5-ene-2026; amoniaco bajo en carbono 500,000 ton/año con captura de 1.67 millones ton CO2/año; meta de finalización 2029)</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>[USDA](https://www.usda.gov/about-usda/news/press-releases/2026/07/01/secretary-rollins-announces-500-million-fertilizer-investment-and-expansion-program-strengthen)</t>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/clean-fuels/06012026/samsung-ea-announces-groundbreaking-of-low-carbon-ammonia-plant/)</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-24</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Wabash Low-Carbon Ammonia Project</t>
+          <t>Green Fuels Operating — Refinería Duncan</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>West Terre Haute, Indiana, EE.UU.</t>
+          <t>Duncan, Stephens County, Oklahoma, EE.UU.</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Wabash Valley Resources</t>
+          <t>Green Fuels Operating</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Samsung E&amp;C (contrato EPF ~US$475 millones)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Construcción (groundbreaking 5-ene-2026; amoniaco bajo en carbono 500,000 ton/año con captura de 1.67 millones ton CO2/año; meta de finalización 2029)</t>
+          <t>Construcción (groundbreaking 29-may-2026; inversión US$400 millones; capacidad inicial 30,000 bbl/d, expandible a 50,000 bbl/d, sobre sitio de refinería histórica de los años 1920)</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/clean-fuels/06012026/samsung-ea-announces-groundbreaking-of-low-carbon-ammonia-plant/)</t>
+          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/refining/03062026/green-fuels-hosts-groundbreaking-ceremony-for-new-refinery/)</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Green Fuels Operating — Refinería Duncan</t>
+          <t>Energy Transfer Mustang Draw I &amp; II (plantas de gas)</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Duncan, Stephens County, Oklahoma, EE.UU.</t>
+          <t>Cuenca Midland, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Green Fuels Operating</t>
+          <t>Energy Transfer LP</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -1681,34 +1679,34 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Construcción (groundbreaking 29-may-2026; inversión US$400 millones; capacidad inicial 30,000 bbl/d, expandible a 50,000 bbl/d, sobre sitio de refinería histórica de los años 1920)</t>
+          <t>Construcción (Mustang Draw I en comisionamiento, servicio pleno ~jun-2026; Mustang Draw II en construcción, en servicio 4T2026; 275 MMcf/d cada una)</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>[Hydrocarbon Engineering](https://www.hydrocarbonengineering.com/refining/03062026/green-fuels-hosts-groundbreaking-ceremony-for-new-refinery/)</t>
+          <t>[Energy Transfer](https://www.energytransfer.com/project-highlights/)</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Energy Transfer Mustang Draw I &amp; II (plantas de gas)</t>
+          <t>ONEOK Bighorn / Cutter / Shadowfax (plantas de gas)</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Cuenca Midland, Texas, EE.UU.</t>
+          <t>Cuenca Delaware (Bighorn), Texas / Cuenca Powder River (Cutter), Wyoming / Cuenca Midland (Shadowfax reubicada), Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Energy Transfer LP</t>
+          <t>ONEOK Inc.</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -1718,49 +1716,49 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Construcción (Mustang Draw I en comisionamiento, servicio pleno ~jun-2026; Mustang Draw II en construcción, en servicio 4T2026; 275 MMcf/d cada una)</t>
+          <t>Construcción (según reporte 2T2026 de ONEOK, ~4-8-ago-2026: Bighorn ampliada de 300 a 400 MMcf/d, tratamiento alto CO2, meta mediados 2027; Cutter 60 MMcf/d en construcción, meta 4T2026; Shadowfax 150 MMcf/d reubicada a la cuenca Midland durante el trimestre, en rampa)</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>[Energy Transfer](https://www.energytransfer.com/project-highlights/)</t>
+          <t>[Inspectioneering](https://inspectioneering.com/news/2025-08-07/11702/oneok-greenlights-new-365m-delaware-basin-gas-plant); [BigGo Finance](https://finance.biggo.com/news/US_OKE_2026-08-04)</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>ONEOK Bighorn / Cutter / Shadowfax (plantas de gas)</t>
+          <t>MPLX Harmon Creek III (planta de gas + de-etanizadora)</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Cuenca Delaware (Bighorn), Texas / Cuenca Powder River (Cutter), Wyoming / Cuenca Midland (Shadowfax reubicada), Texas, EE.UU.</t>
+          <t>Región Marcellus/Utica, noreste de EE.UU. (ubicación exacta no especificada)</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>ONEOK Inc.</t>
+          <t>MPLX LP</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>MPLX (propietario-constructor)</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Construcción (según reporte 2T2026 de ONEOK, ~4-8-ago-2026: Bighorn ampliada de 300 a 400 MMcf/d, tratamiento alto CO2, meta mediados 2027; Cutter 60 MMcf/d en construcción, meta 4T2026; Shadowfax 150 MMcf/d reubicada a la cuenca Midland durante el trimestre, en rampa)</t>
+          <t>Operando (arranque/startup completado ago-2026, según reporte 2T2026 de MPLX; eleva capacidad de procesamiento de MPLX en el noreste a 8.1 Bcf/d; planta de 300 MMcf/d + de-etanizadora 40 Mbpd)</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>[Inspectioneering](https://inspectioneering.com/news/2025-08-07/11702/oneok-greenlights-new-365m-delaware-basin-gas-plant); [BigGo Finance](https://finance.biggo.com/news/US_OKE_2026-08-04)</t>
+          <t>[Marcellus Drilling News](https://marcellusdrilling.com/2026/08/mplx-marcellus-proc-plants-96-full-harmon-creek-iii-starts-up/); [StockTitan](https://www.stocktitan.net/news/MPLX/mplx-lp-reports-second-quarter-2026-financial-9tcvq4saz6sr.html)</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -1772,86 +1770,86 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>MPLX Harmon Creek III (planta de gas + de-etanizadora)</t>
+          <t>Rehab. Complejo Cosoleacaque (amoniaco) + Complejo Morelos (etano-etileno)</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Región Marcellus/Utica, noreste de EE.UU. (ubicación exacta no especificada)</t>
+          <t>Cosoleacaque y Complejo Morelos, Veracruz, México</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>MPLX LP</t>
+          <t>Pemex Transformación Industrial</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>MPLX (propietario-constructor)</t>
+          <t>Mota-Engil México (plantas VI/VII y TASP Pajaritos); ICA (paquete relacionado)</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Operando (arranque/startup completado ago-2026, según reporte 2T2026 de MPLX; eleva capacidad de procesamiento de MPLX en el noreste a 8.1 Bcf/d; planta de 300 MMcf/d + de-etanizadora 40 Mbpd)</t>
+          <t>Ingeniería/planeación (parte del plan de reactivación petroquímica de Pemex de 93,000 mdp anunciado jun-2026; 13,000 mdp para 2 plantas de amoniaco en Cosoleacaque, meta 957,000 ton/año; Complejo Morelos incluido en programa de rehabilitación etano-etileno de 30,000 mdp/5 plantas, meta 520,000 ton/año de polietilenos/óxido de etileno/glicoles; contratos de rehabilitación y confiabilidad adjudicados dic-2025, confirmados ene-2026)</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>[Marcellus Drilling News](https://marcellusdrilling.com/2026/08/mplx-marcellus-proc-plants-96-full-harmon-creek-iii-starts-up/); [StockTitan](https://www.stocktitan.net/news/MPLX/mplx-lp-reports-second-quarter-2026-financial-9tcvq4saz6sr.html)</t>
+          <t>[Contralínea](https://contralinea.com.mx/interno/semana/presentan-plan-con-inversion-de-93-mil-mdp-para-rescatar-la-petroquimica-nacional/); [El Diario de Juárez](https://diario.mx/nacional/2026/jan/22/adjudica-pemex-contratos-a-favoritas-1102601.html)</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-06</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Rehab. Complejo Cosoleacaque (amoniaco) + Complejo Morelos (etano-etileno)</t>
+          <t>Enterprise Products — Nuevas Plantas de Gas Permian (Plant 11 Midland / Plant 13 Delaware) + NGL Frac 15 Mont Belvieu</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Cosoleacaque y Complejo Morelos, Veracruz, México</t>
+          <t>Cuenca Midland y Cuenca Delaware, Texas, EE.UU. / Mont Belvieu, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Pemex Transformación Industrial</t>
+          <t>Enterprise Products Partners L.P.</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Mota-Engil México (plantas VI/VII y TASP Pajaritos); ICA (paquete relacionado)</t>
+          <t>Enterprise Products (propietario-constructor)</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/planeación (parte del plan de reactivación petroquímica de Pemex de 93,000 mdp anunciado jun-2026; 13,000 mdp para 2 plantas de amoniaco en Cosoleacaque, meta 957,000 ton/año; Complejo Morelos incluido en programa de rehabilitación etano-etileno de 30,000 mdp/5 plantas, meta 520,000 ton/año de polietilenos/óxido de etileno/glicoles; contratos de rehabilitación y confiabilidad adjudicados dic-2025, confirmados ene-2026)</t>
+          <t>Construcción (sancionadas/aprobadas en resultados 2T2026: Plant 11 Midland Basin 300 MMcf/d en servicio 1T2029; Plant 13 Delaware Basin 300 MMcf/d en servicio 3T2028; NGL Frac 15 en Mont Belvieu 150 MBPD en servicio 1T2028; gasto de capital de crecimiento 2026 aumentado en más de US$700 millones por estas sanciones)</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>[Contralínea](https://contralinea.com.mx/interno/semana/presentan-plan-con-inversion-de-93-mil-mdp-para-rescatar-la-petroquimica-nacional/); [El Diario de Juárez](https://diario.mx/nacional/2026/jan/22/adjudica-pemex-contratos-a-favoritas-1102601.html)</t>
+          <t>[Enterprise Reports Second Quarter 2026 Earnings](https://ir.enterpriseproducts.com/news-releases/news-release-details/enterprise-reports-second-quarter-2026-earnings)</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-07-31</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Enterprise Products — Nuevas Plantas de Gas Permian (Plant 11 Midland / Plant 13 Delaware) + NGL Frac 15 Mont Belvieu</t>
+          <t>Enterprise Products — Plant 12 (Delaware Basin) y Athena 2 (Midland Basin)</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Cuenca Midland y Cuenca Delaware, Texas, EE.UU. / Mont Belvieu, Texas, EE.UU.</t>
+          <t>Cuenca Delaware y Cuenca Midland, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -1866,7 +1864,7 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Construcción (sancionadas/aprobadas en resultados 2T2026: Plant 11 Midland Basin 300 MMcf/d en servicio 1T2029; Plant 13 Delaware Basin 300 MMcf/d en servicio 3T2028; NGL Frac 15 en Mont Belvieu 150 MBPD en servicio 1T2028; gasto de capital de crecimiento 2026 aumentado en más de US$700 millones por estas sanciones)</t>
+          <t>Construcción (sancionadas, divulgadas en resultados 2T2026 el 30-jul-2026; Plant 12 Delaware Basin ~300 MMcf/d en servicio 4T2027; Athena 2 Midland Basin en servicio 3T2027)</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -1876,39 +1874,39 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Enterprise Products — Plant 12 (Delaware Basin) y Athena 2 (Midland Basin)</t>
+          <t>Targa Resources Roadrunner III / Copperhead II (plantas de gas)</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Cuenca Delaware y Cuenca Midland, Texas, EE.UU.</t>
+          <t>Cuenca Delaware (Permian), Texas/Nuevo México, EE.UU.</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Enterprise Products Partners L.P.</t>
+          <t>Targa Resources Corp.</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Enterprise Products (propietario-constructor)</t>
+          <t>Targa Resources (propietario-constructor)</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Construcción (sancionadas, divulgadas en resultados 2T2026 el 30-jul-2026; Plant 12 Delaware Basin ~300 MMcf/d en servicio 4T2027; Athena 2 Midland Basin en servicio 3T2027)</t>
+          <t>Construcción (aprobadas may-2026; Roadrunner III 265 MMcf/d, Copperhead II 275 MMcf/d; en servicio previsto 1T2028)</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>[Enterprise Reports Second Quarter 2026 Earnings](https://ir.enterpriseproducts.com/news-releases/news-release-details/enterprise-reports-second-quarter-2026-earnings)</t>
+          <t>[PGJ](https://pgjonline.com/news/2026/may/targa-expands-permian-gas-processing-delaware-express-pipeline-capacity)</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -1920,54 +1918,54 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Targa Resources Roadrunner III / Copperhead II (plantas de gas)</t>
+          <t>Southern Energy Renewables — Complejo de Metanol y SAF</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Cuenca Delaware (Permian), Texas/Nuevo México, EE.UU.</t>
+          <t>St. Charles Parish (Killona), Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Targa Resources Corp.</t>
+          <t>Southern Energy Renewables</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Targa Resources (propietario-constructor)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Construcción (aprobadas may-2026; Roadrunner III 265 MMcf/d, Copperhead II 275 MMcf/d; en servicio previsto 1T2028)</t>
+          <t>Planeación/pre-construcción (inversión US$1,400 millones; convierte biomasa de desecho de madera en metanol verde y combustible de aviación sostenible; construcción prevista a iniciar fines de 2027, producción prevista fines de 2029)</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>[PGJ](https://pgjonline.com/news/2026/may/targa-expands-permian-gas-processing-delaware-express-pipeline-capacity)</t>
+          <t>[Hydrocarbon Processing](https://www.hydrocarbonprocessing.com/news/2026/03/southern-energy-renewables-announce-14-b-methanol-and-saf-complex-in-louisiana/); [Louisiana Economic Development](https://www.opportunitylouisiana.gov/news/southern-energy-renewables-announce-1-4-billion-methanol-and-sustainable-aviation-fuel-facility-in-st-charles-parish)</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Southern Energy Renewables — Complejo de Metanol y SAF</t>
+          <t>Atlas Agro — Pacific Green Fertilizer Plant</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>St. Charles Parish (Killona), Luisiana, EE.UU.</t>
+          <t>Richland, Washington, EE.UU.</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Southern Energy Renewables</t>
+          <t>Atlas Agro</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -1977,49 +1975,49 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Planeación/pre-construcción (inversión US$1,400 millones; convierte biomasa de desecho de madera en metanol verde y combustible de aviación sostenible; construcción prevista a iniciar fines de 2027, producción prevista fines de 2029)</t>
+          <t>Ingeniería/FEED (diseño ~70% completo, USD 315 millones de capital levantado, permisos en proceso; planta de fertilizante nitrato ~0.7 Mt/año, inversión USD 1,100-1,500 millones; debe iniciar construcción antes de fines de 2027 para calificar a créditos fiscales federales; construcción estimada en 36 meses)</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>[Hydrocarbon Processing](https://www.hydrocarbonprocessing.com/news/2026/03/southern-energy-renewables-announce-14-b-methanol-and-saf-complex-in-louisiana/); [Louisiana Economic Development](https://www.opportunitylouisiana.gov/news/southern-energy-renewables-announce-1-4-billion-methanol-and-sustainable-aviation-fuel-facility-in-st-charles-parish)</t>
+          <t>[Tri-Cities Area Journal of Business](https://www.tricitiesbusinessnews.com/articles/atlas-agro-plant-nears-decision-point); [Washington State Standard](https://washingtonstatestandard.com/2025/10/30/plan-for-1-5b-fertilizer-plant-in-central-wa-still-alive-despite-loss-of-federal-funds/)</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-06</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Atlas Agro — Pacific Green Fertilizer Plant</t>
+          <t>Hydrogen City (complejo Power-to-X / e-metanol)</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Richland, Washington, EE.UU.</t>
+          <t>Piedras Pintas Salt Dome, Condado de Duval, sur de Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Atlas Agro</t>
+          <t>Green Hydrogen International (GHI)</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>ABB (automatización/control, vía MOU)</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/FEED (diseño ~70% completo, USD 315 millones de capital levantado, permisos en proceso; planta de fertilizante nitrato ~0.7 Mt/año, inversión USD 1,100-1,500 millones; debe iniciar construcción antes de fines de 2027 para calificar a créditos fiscales federales; construcción estimada en 36 meses)</t>
+          <t>Ingeniería/FEED (inversión USD 6,000-10,000 millones; electrolizador de 2.2 GW; producirá 1.4 Mt/año de e-metanol y capturará ~2 Mt/año de CO2; construcción planeada desde 2026, primera producción estimada 2030)</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>[Tri-Cities Area Journal of Business](https://www.tricitiesbusinessnews.com/articles/atlas-agro-plant-nears-decision-point); [Washington State Standard](https://washingtonstatestandard.com/2025/10/30/plan-for-1-5b-fertilizer-plant-in-central-wa-still-alive-despite-loss-of-federal-funds/)</t>
+          <t>[The Engineer](https://www.theengineer.co.uk/content/news/abb-joins-team-for-22gw-hydrogen-city-project-in-texas); [Energy Capital HTX](https://energycapitalhtx.com/green-hydrogen-city-abb-mou)</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -2031,91 +2029,91 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Hydrogen City (complejo Power-to-X / e-metanol)</t>
+          <t>Targa Resources Falcon II Gas Processing Plant</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Piedras Pintas Salt Dome, Condado de Duval, sur de Texas, EE.UU.</t>
+          <t>Cuenca Delaware, Permian Basin, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Green Hydrogen International (GHI)</t>
+          <t>Targa Resources Corp.</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>ABB (automatización/control, vía MOU)</t>
+          <t>Targa Resources (propietario-constructor)</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/FEED (inversión USD 6,000-10,000 millones; electrolizador de 2.2 GW; producirá 1.4 Mt/año de e-metanol y capturará ~2 Mt/año de CO2; construcción planeada desde 2026, primera producción estimada 2030)</t>
+          <t>Construcción/Comisionamiento (planta criogénica; arranque adelantado a 1T2026, dos trimestres antes de lo previsto; según reporte 2T2026 de Targa —6-ago-2026—, el segundo tren quedó completo y en preparación para producción plena, llevando la capacidad total a ~685 MMcf/d)</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>[The Engineer](https://www.theengineer.co.uk/content/news/abb-joins-team-for-22gw-hydrogen-city-project-in-texas); [Energy Capital HTX](https://energycapitalhtx.com/green-hydrogen-city-abb-mou)</t>
+          <t>[Oil &amp; Gas Journal](https://www.ogj.com/refining-processing/gas-processing/capacities/article/55240691/targa-advances-expansion-plans-for-permian-basin-gas-processing); [Targa Resources Q2 2026 Results](https://www.globenewswire.com/news-release/2026/08/06/3340017/14074/en/Targa-Resources-Corp-Reports-Record-Second-Quarter-2026-Financial-Results.html)</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-20</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Targa Resources Falcon II Gas Processing Plant</t>
+          <t>Cassidy II Gas Processing Plant</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Cuenca Delaware, Permian Basin, Texas, EE.UU.</t>
+          <t>Condado de Glasscock, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Targa Resources Corp.</t>
+          <t>Brazos Midstream</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Targa Resources (propietario-constructor)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Construcción/Comisionamiento (planta criogénica; arranque adelantado a 1T2026, dos trimestres antes de lo previsto; según reporte 2T2026 de Targa —6-ago-2026—, el segundo tren quedó completo y en preparación para producción plena, llevando la capacidad total a ~685 MMcf/d)</t>
+          <t>Anuncio/Construcción (planta criogénica de 300 MMcf/d adicional a Cassidy I —300 MMcf/d, en servicio antes de fin de 2026—; eleva capacidad total de Brazos en Midland Basin a ~1.1 Bcf/d; respaldada por ~575,000 acres bajo dedicación; entrada en operación prevista verano 2027; anunciado 11-ago-2026)</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>[Oil &amp; Gas Journal](https://www.ogj.com/refining-processing/gas-processing/capacities/article/55240691/targa-advances-expansion-plans-for-permian-basin-gas-processing); [Targa Resources Q2 2026 Results](https://www.globenewswire.com/news-release/2026/08/06/3340017/14074/en/Targa-Resources-Corp-Reports-Record-Second-Quarter-2026-Financial-Results.html)</t>
+          <t>[Inspectioneering](https://inspectioneering.com/news/2026-08-11/12145/brazos-midstream-announces-new-natural-gas-processing-plant-to-support-continued); [Rigzone](https://www.rigzone.com/news/brazos_to_grow_midland_gas_processing_capacity_to_11_bcfd-11-aug-2026-184346-article/)</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Cassidy II Gas Processing Plant</t>
+          <t>Kings Landing II Gas Processing Plant</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Condado de Glasscock, Texas, EE.UU.</t>
+          <t>Nuevo México, EE.UU.</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Brazos Midstream</t>
+          <t>Kinetik Holdings</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -2125,34 +2123,34 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Anuncio/Construcción (planta criogénica de 300 MMcf/d adicional a Cassidy I —300 MMcf/d, en servicio antes de fin de 2026—; eleva capacidad total de Brazos en Midland Basin a ~1.1 Bcf/d; respaldada por ~575,000 acres bajo dedicación; entrada en operación prevista verano 2027; anunciado 11-ago-2026)</t>
+          <t>Construcción (FID alcanzada; US$260 millones; finalización prevista 2S2028)</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>[Inspectioneering](https://inspectioneering.com/news/2026-08-11/12145/brazos-midstream-announces-new-natural-gas-processing-plant-to-support-continued); [Rigzone](https://www.rigzone.com/news/brazos_to_grow_midland_gas_processing_capacity_to_11_bcfd-11-aug-2026-184346-article/)</t>
+          <t>[Investing.com](https://www.investing.com/news/company-news/kinetik-approves-260m-gas-processing-plant-in-new-mexico-93CH-4698224)</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Kings Landing II Gas Processing Plant</t>
+          <t>Apollo Gas Plant</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Nuevo México, EE.UU.</t>
+          <t>Condado de Eddy, Nuevo México, EE.UU.</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Kinetik Holdings</t>
+          <t>Trace Midstream Partners II</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -2162,12 +2160,12 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Construcción (FID alcanzada; US$260 millones; finalización prevista 2S2028)</t>
+          <t>Anuncio/planeación (planta criogénica de 250 MMcf/d)</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>[Investing.com](https://www.investing.com/news/company-news/kinetik-approves-260m-gas-processing-plant-in-new-mexico-93CH-4698224)</t>
+          <t>[Gas Compression Magazine](https://gascompressionmagazine.com/2026/06/29/new-mexico-gains-major-gas-processing-hub/)</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -2179,17 +2177,17 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Apollo Gas Plant</t>
+          <t>IGP Gulf Coast Methanol Complex (4 unidades)</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Condado de Eddy, Nuevo México, EE.UU.</t>
+          <t>Plaquemine Parish (Myrtle Grove), Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Trace Midstream Partners II</t>
+          <t>IGP Methanol LLC</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -2199,12 +2197,12 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Anuncio/planeación (planta criogénica de 250 MMcf/d)</t>
+          <t>Permiso de calidad del aire asegurado / pre-construcción (US$3,600 millones)</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>[Gas Compression Magazine](https://gascompressionmagazine.com/2026/06/29/new-mexico-gains-major-gas-processing-hub/)</t>
+          <t>[Industrial Info Resources](https://www.industrialinfo.com/news/article.jsp?newsitemID=262022)</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -2216,91 +2214,91 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>IGP Gulf Coast Methanol Complex (4 unidades)</t>
+          <t>Eastern Montana Fertilizer Project (planta de urea)</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Plaquemine Parish (Myrtle Grove), Luisiana, EE.UU.</t>
+          <t>Culbertson, Montana, EE.UU.</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>IGP Methanol LLC</t>
+          <t>Cyan H2</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>KBR (MoU: tecnología, ingeniería, procura y gestión de construcción)</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Permiso de calidad del aire asegurado / pre-construcción (US$3,600 millones)</t>
+          <t>Desarrollo/financiamiento (busca cierre de subvención USDA de US$150 millones —vence 17-ago-2026— y préstamo DOE de US$1,000 millones; groundbreaking previsto fin de 2026)</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>[Industrial Info Resources](https://www.industrialinfo.com/news/article.jsp?newsitemID=262022)</t>
+          <t>[Northern Plains Independent](https://www.northernplainsindependent.com/2026/08/13/proposed-fertilizer-plant-making-strides/); [World Fertilizer](https://www.worldfertilizer.com/project-news/26112025/cyan-h2-signs-mou-for-montana-fertilizer-project/)</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Eastern Montana Fertilizer Project (planta de urea)</t>
+          <t>Targa Resources — Plantas Wrangler, Ranger y Ranger II (procesamiento de gas)</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Culbertson, Montana, EE.UU.</t>
+          <t>Cuenca Delaware (Permian), Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Cyan H2</t>
+          <t>Targa Resources Corp. (acuerdo de 20 años con subsidiarias de ExxonMobil)</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>KBR (MoU: tecnología, ingeniería, procura y gestión de construcción)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Desarrollo/financiamiento (busca cierre de subvención USDA de US$150 millones —vence 17-ago-2026— y préstamo DOE de US$1,000 millones; groundbreaking previsto fin de 2026)</t>
+          <t>Anuncio/Planeación (anunciado 17-ago-2026; tres nuevas plantas criogénicas con capacidad combinada ~825 MMcf/d, más nuevo gasoducto de ~70 millas "Bull Run II" hacia el hub de Waha; entrada en servicio prevista 1S2028; Targa evalúa además hasta 5 plantas adicionales en Permian Delaware a más largo plazo)</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>[Northern Plains Independent](https://www.northernplainsindependent.com/2026/08/13/proposed-fertilizer-plant-making-strides/); [World Fertilizer](https://www.worldfertilizer.com/project-news/26112025/cyan-h2-signs-mou-for-montana-fertilizer-project/)</t>
+          <t>[EnergyNow](https://energynow.com/2026/08/targa-to-build-three-permian-gas-processing-plants-new-pipeline/); [Targa Resources](https://www.targaresources.com/news-releases/news-release-details/targa-resources-corp-announces-20-year-agreements-exxonmobil-and)</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Targa Resources — Plantas Wrangler, Ranger y Ranger II (procesamiento de gas)</t>
+          <t>México Amoníaco y Urea (MAYU)</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Cuenca Delaware (Permian), Texas, EE.UU.</t>
+          <t>Costa del Pacífico, Sonora, México (ciudad exacta no especificada)</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Targa Resources Corp. (acuerdo de 20 años con subsidiarias de ExxonMobil)</t>
+          <t>México Amoníaco y Urea (desarrollador privado)</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -2310,34 +2308,34 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Anuncio/Planeación (anunciado 17-ago-2026; tres nuevas plantas criogénicas con capacidad combinada ~825 MMcf/d, más nuevo gasoducto de ~70 millas "Bull Run II" hacia el hub de Waha; entrada en servicio prevista 1S2028; Targa evalúa además hasta 5 plantas adicionales en Permian Delaware a más largo plazo)</t>
+          <t>Desarrollo muy temprano (planta de amoniaco azul y urea bajo en carbono, capacidad &gt;900,000 ton/año, usando gas natural de la Cuenca Pérmica vía costa del Pacífico; sin autorización de impacto ambiental ni contrato EPC confirmado públicamente a la fecha)</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>[EnergyNow](https://energynow.com/2026/08/targa-to-build-three-permian-gas-processing-plants-new-pipeline/); [Targa Resources](https://www.targaresources.com/news-releases/news-release-details/targa-resources-corp-announces-20-year-agreements-exxonmobil-and)</t>
+          <t>[MAYU](https://mayu.com.mx/en/)</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-18</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>México Amoníaco y Urea (MAYU)</t>
+          <t>Ampliación Terminal de Exportación NGL Nederland</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Costa del Pacífico, Sonora, México (ciudad exacta no especificada)</t>
+          <t>Nederland/Port Neches, Jefferson County, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>México Amoníaco y Urea (desarrollador privado)</t>
+          <t>Energy Transfer LP</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -2347,34 +2345,34 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Desarrollo muy temprano (planta de amoniaco azul y urea bajo en carbono, capacidad &gt;900,000 ton/año, usando gas natural de la Cuenca Pérmica vía costa del Pacífico; sin autorización de impacto ambiental ni contrato EPC confirmado públicamente a la fecha)</t>
+          <t>Totalmente comprometida (fully subscribed; contratos de largo plazo hasta la década de 2040; incluye ampliación del ducto de NGL Mont Belvieu-Nederland y construcción de dos muelles adicionales; anunciado 18-jun-2026; entrada en servicio por etapas desde 2028)</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>[MAYU](https://mayu.com.mx/en/)</t>
+          <t>[Rigzone](https://www.rigzone.com/news/energy_transfer_to_expand_texas_ngl_export_terminal-19-jun-2026-183955-article/); [Energy Transfer IR](https://ir.energytransfer.com/news-releases/news-release-details/energy-transfer-announces-fully-subscribed-export-expansion)</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-26</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Ampliación Terminal de Exportación NGL Nederland</t>
+          <t>LSB Industries — Expansión de Amoniaco El Dorado</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Nederland/Port Neches, Jefferson County, Texas, EE.UU.</t>
+          <t>El Dorado, Arkansas, EE.UU.</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Energy Transfer LP</t>
+          <t>LSB Industries</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
@@ -2384,34 +2382,34 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>Totalmente comprometida (fully subscribed; contratos de largo plazo hasta la década de 2040; incluye ampliación del ducto de NGL Mont Belvieu-Nederland y construcción de dos muelles adicionales; anunciado 18-jun-2026; entrada en servicio por etapas desde 2028)</t>
+          <t>Pre-FID (decisión final de inversión proyectada para 2T2027; expansión de 100,000 toneladas/año incrementales de amoniaco, costo neto US$105-120 millones, bruto US$135-150 millones incluyendo infraestructura)</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>[Rigzone](https://www.rigzone.com/news/energy_transfer_to_expand_texas_ngl_export_terminal-19-jun-2026-183955-article/); [Energy Transfer IR](https://ir.energytransfer.com/news-releases/news-release-details/energy-transfer-announces-fully-subscribed-export-expansion)</t>
+          <t>[The Motley Fool](https://www.fool.com/earnings/call-transcripts/2026/08/07/lsb-industries-lxu-q2-2026-earnings-call-transcript/)</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>LSB Industries — Expansión de Amoniaco El Dorado</t>
+          <t>Yara/Enbridge — Amoniaco Azul Ingleside</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>El Dorado, Arkansas, EE.UU.</t>
+          <t>Enbridge Ingleside Energy Center, cerca de Corpus Christi, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>LSB Industries</t>
+          <t>Yara Clean Ammonia / Enbridge (JV 50/50)</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
@@ -2421,12 +2419,12 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Pre-FID (decisión final de inversión proyectada para 2T2027; expansión de 100,000 toneladas/año incrementales de amoniaco, costo neto US$105-120 millones, bruto US$135-150 millones incluyendo infraestructura)</t>
+          <t>Ingeniería (FEED en curso, pendiente FID; capacidad 1.2-1.4 MMTPA, inversión estimada US$2,600-2,900 millones; reforming autotérmico con captura de CO2 ~95%; enfrenta oposición comunitaria activa)</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>[The Motley Fool](https://www.fool.com/earnings/call-transcripts/2026/08/07/lsb-industries-lxu-q2-2026-earnings-call-transcript/)</t>
+          <t>[QC Intel](https://www.qcintel.com/ammonia/article/yara-enbridge-continue-ingleside-blue-ammonia-plans-despite-pushback-28727.html)</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -2438,72 +2436,35 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Yara/Enbridge — Amoniaco Azul Ingleside</t>
+          <t>Cronus Chemicals — Planta de Amoniaco/Fertilizantes Tuscola</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Enbridge Ingleside Energy Center, cerca de Corpus Christi, Texas, EE.UU.</t>
+          <t>Tuscola, Illinois, EE.UU.</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Yara Clean Ammonia / Enbridge (JV 50/50)</t>
+          <t>Cronus Chemicals LLC</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>thyssenkrupp Industrial Solutions (EPC llave en mano, lump-sum)</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería (FEED en curso, pendiente FID; capacidad 1.2-1.4 MMTPA, inversión estimada US$2,600-2,900 millones; reforming autotérmico con captura de CO2 ~95%; enfrenta oposición comunitaria activa)</t>
+          <t>Construcción (proyecto de ~US$2,000-2,300 millones, hasta ~2,300 t/día / ~950,000 ton/año de amoniaco; obtuvo el permiso final de construcción/aire de la EPA tras más de una década en planeación desde 2012; construcción de ~40 meses, hasta 2,000-2,500 empleos pico)</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>[QC Intel](https://www.qcintel.com/ammonia/article/yara-enbridge-continue-ingleside-blue-ammonia-plans-despite-pushback-28727.html)</t>
+          <t>[News-Gazette](https://www.news-gazette.com/business/employment/after-almost-13-years-2-3-billion-tuscola-fertilizer-plant-clears-final-regulatory-hurdle-for/); [FarmWeek Now](https://www.farmweeknow.com/policy/state/construction-to-begin-on-tuscola-ammonia-plant/)</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="2" t="inlineStr">
-        <is>
-          <t>Cronus Chemicals — Planta de Amoniaco/Fertilizantes Tuscola</t>
-        </is>
-      </c>
-      <c r="B56" s="2" t="inlineStr">
-        <is>
-          <t>Tuscola, Illinois, EE.UU.</t>
-        </is>
-      </c>
-      <c r="C56" s="2" t="inlineStr">
-        <is>
-          <t>Cronus Chemicals LLC</t>
-        </is>
-      </c>
-      <c r="D56" s="2" t="inlineStr">
-        <is>
-          <t>thyssenkrupp Industrial Solutions (EPC llave en mano, lump-sum)</t>
-        </is>
-      </c>
-      <c r="E56" s="2" t="inlineStr">
-        <is>
-          <t>Construcción (proyecto de ~US$2,000-2,300 millones, hasta ~2,300 t/día / ~950,000 ton/año de amoniaco; obtuvo el permiso final de construcción/aire de la EPA tras más de una década en planeación desde 2012; construcción de ~40 meses, hasta 2,000-2,500 empleos pico)</t>
-        </is>
-      </c>
-      <c r="F56" s="2" t="inlineStr">
-        <is>
-          <t>[News-Gazette](https://www.news-gazette.com/business/employment/after-almost-13-years-2-3-billion-tuscola-fertilizer-plant-clears-final-regulatory-hurdle-for/); [FarmWeek Now](https://www.farmweeknow.com/policy/state/construction-to-begin-on-tuscola-ammonia-plant/)</t>
-        </is>
-      </c>
-      <c r="G56" s="2" t="inlineStr">
         <is>
           <t>2026-09-02</t>
         </is>
@@ -2523,13 +2484,13 @@
   <dimension ref="A1:G47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2740,17 +2701,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Construcción/Permitting acelerado (Venture Global presentó solicitud FERC para expansión adicional de 31 mtpa —24 trenes, ~USD 18,000 millones—; U.S. Army Corps of Engineers otorgó permitting expedito bajo "emergencia energética nacional" —periodo de comentario público reducido de 30 a 10 días, cerrado 2-jul-2026—, ampliaría el sitio de 590 a 1,220 acres; DOE aprobó exportaciones adicionales inmediatas desde Plaquemines; inicio de construcción de la expansión esperado a inicios de 2027, primera producción fin de 2028)</t>
+          <t>Construcción/Permitting acelerado (Venture Global presentó solicitud FERC para expansión adicional de 31 mtpa —24 trenes, ~USD 18,000 millones—; U.S. Army Corps of Engineers otorgó permitting expedito bajo "emergencia energética nacional" —periodo de comentario público reducido de 30 a 10 días, cerrado 2-jul-2026—, ampliaría el sitio de 590 a 1,220 acres; DOE aprobó exportaciones adicionales inmediatas desde Plaquemines; inicio de construcción de la expansión esperado a inicios de 2027, primera producción fin de 2028) ; Williams Companies sancionó (FID) el gasoducto "Delta Access" (US$1,500 millones, 2.25 Bcf/d iniciales ampliable a 3.5 Bcf/d, de Gillis LA hacia el corredor Transco, en servicio 1T2029) diseñado para alimentar esta expansión vía interconexión con el gasoducto intraestatal Cloud Connector de Venture Global, confirmado en su reporte 2T2026 (4-ago-2026)</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>[Offshore Energy](https://www.offshore-energy.biz/kbr-zachry-to-work-on-ventures-plaquemines-lng/); [Verite News](https://veritenews.org/2026/08/12/lng-expansion-could-be-fast-tracked); [DOE](https://www.energy.gov/node/4856848)</t>
+          <t>[Offshore Energy](https://www.offshore-energy.biz/kbr-zachry-to-work-on-ventures-plaquemines-lng/); [Verite News](https://veritenews.org/2026/08/12/lng-expansion-could-be-fast-tracked); [DOE](https://www.energy.gov/node/4856848); [Natural Gas Intel](https://www.naturalgasintel.com/news/plaquemines-expansion-to-anchor-east-end-of-williams-delta-access/)</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-09-03</t>
         </is>
       </c>
     </row>
@@ -4285,13 +4246,13 @@
   <dimension ref="A1:G110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5301,7 +5262,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Pine Bluff Arsenal, Arkansas o Anniston Army Depot, Alabama (sin confirmar), EE.UU.</t>
+          <t>Pine Bluff Arsenal, Arkansas (sitio primario, ~245 acres) y Anniston Army Depot, Alabama (~97 acres), EE.UU.</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -5311,22 +5272,22 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Titan Mining Corp.</t>
+          <t>Titan Mining Corp. (vía subsidiaria Empire State Mines)</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Acuerdo firmado/planeación (construcción prevista desde 2027)</t>
+          <t>Acuerdo firmado/planeación (Notificaciones de Selección Condicional del Ejército confirmadas para ambos sitios bajo arrendamientos de uso mejorado —EUL— de hasta 50 años; construcción prevista para 2S-2027)</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>[Mining.com](https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/)</t>
+          <t>[Mining.com](https://www.mining.com/web/us-army-bases-to-host-critical-minerals-plants-in-onshoring-push/); [NNY360](https://www.nny360.com/news/statenews/empire-state-mines-moves-forward-with-first-u-s-graphite-mine-in-generations/article_6cac15a0-daf9-57bb-be6a-0e41c5c9231d.html)</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-09-03</t>
         </is>
       </c>
     </row>
@@ -7035,12 +6996,12 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>Proyecto de Cobre Angangueo</t>
+          <t>Modernización Complejo Metalúrgico Empalme</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>Angangueo, Michoacán, México</t>
+          <t>Empalme, Sonora, México</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
@@ -7055,7 +7016,7 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Pre-desarrollo (en negociación de permisos con gobierno federal)</t>
+          <t>Pre-desarrollo (en negociación de permisos; fundición existente a modernizar)</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
@@ -7072,17 +7033,17 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Proyecto de Cobre Chalchihuites</t>
+          <t>Coosa Graphite Project (Kellyton Graphite Plant)</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>Chalchihuites, Zacatecas, México</t>
+          <t>Condado de Coosa, Alabama, EE.UU.</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Southern Copper Corporation (Grupo México)</t>
+          <t>Westwater Resources Inc.</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
@@ -7092,34 +7053,34 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Pre-desarrollo (en negociación de permisos)</t>
+          <t>Financiamiento/planeación (préstamo EXIM Bank de US$25 millones anunciado 7-ago-2026 para mina de grafito natural y planta de procesamiento, primera fuente de grafito natural producida en EE.UU.)</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>[Minería en Línea](https://mineriaenlinea.com/2026/07/southern-copper-obtiene-permisos-ambientales-para-el-pilar-produccion-a-partir-de-2029/)</t>
+          <t>[Yellowhammer News](https://yellowhammernews.com/trump-administration-announces-25-million-exim-loan-for-westwaters-coosa-county-graphite-plant/); [EXIM.GOV](https://www.exim.gov/news/trump-administration-announces-58m-major-new-critical-mineral-deals-white-house-roundtable)</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>Modernización Complejo Metalúrgico Empalme</t>
+          <t>Expansión de Procesamiento de Tantalio/Niobio (Global Advanced Metals)</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>Empalme, Sonora, México</t>
+          <t>Pensilvania, EE.UU.</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>Southern Copper Corporation (Grupo México)</t>
+          <t>Global Advanced Metals</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
@@ -7129,34 +7090,34 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Pre-desarrollo (en negociación de permisos; fundición existente a modernizar)</t>
+          <t>Financiamiento/planeación (préstamo EXIM Bank de US$25 millones anunciado 7-ago-2026 para ampliar capacidad de procesamiento)</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>[Minería en Línea](https://mineriaenlinea.com/2026/07/southern-copper-obtiene-permisos-ambientales-para-el-pilar-produccion-a-partir-de-2029/)</t>
+          <t>[EXIM.GOV](https://www.exim.gov/news/trump-administration-announces-58m-major-new-critical-mineral-deals-white-house-roundtable); [SME](https://me.smenet.org/trump-administration-to-back-three-mineral-projects-with-58-million-in-financing/)</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>Coosa Graphite Project (Kellyton Graphite Plant)</t>
+          <t>Boron Americas Project (Fort Cady)</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>Condado de Coosa, Alabama, EE.UU.</t>
+          <t>California, EE.UU.</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Westwater Resources Inc.</t>
+          <t>5E Advanced Materials</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
@@ -7166,12 +7127,12 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Financiamiento/planeación (préstamo EXIM Bank de US$25 millones anunciado 7-ago-2026 para mina de grafito natural y planta de procesamiento, primera fuente de grafito natural producida en EE.UU.)</t>
+          <t>Financiamiento/planeación (préstamo EXIM Bank de US$8 millones anunciado 7-ago-2026 para proyecto de boro, lixiviación/procesamiento)</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>[Yellowhammer News](https://yellowhammernews.com/trump-administration-announces-25-million-exim-loan-for-westwaters-coosa-county-graphite-plant/); [EXIM.GOV](https://www.exim.gov/news/trump-administration-announces-58m-major-new-critical-mineral-deals-white-house-roundtable)</t>
+          <t>[EXIM.GOV](https://www.exim.gov/news/trump-administration-announces-58m-major-new-critical-mineral-deals-white-house-roundtable)</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -7183,54 +7144,54 @@
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>Expansión de Procesamiento de Tantalio/Niobio (Global Advanced Metals)</t>
+          <t>Brook Mine (tierras raras/minerales críticos de carbón)</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>Pensilvania, EE.UU.</t>
+          <t>Ranchester/Sheridan, Wyoming, EE.UU.</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>Global Advanced Metals</t>
+          <t>Ramaco Resources</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Hatch Associates Consultants (ingeniería/estudio)</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>Financiamiento/planeación (préstamo EXIM Bank de US$25 millones anunciado 7-ago-2026 para ampliar capacidad de procesamiento)</t>
+          <t>Ingeniería/Construcción de planta piloto (Hatch publicó Initial Assessment Report jul-2026 con capex preliminar ~US$3,200 millones + US$800 millones de contingencia, VPN interno ~US$8,000 millones; planta piloto en construcción desde oct-2025; primer procesamiento de concentrados de óxido de tierras raras para la Defense Logistics Agency, ago-2026; construcción de planta comercial podría iniciar fines de 2026, producción comercial 2028)</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>[EXIM.GOV](https://www.exim.gov/news/trump-administration-announces-58m-major-new-critical-mineral-deals-white-house-roundtable); [SME](https://me.smenet.org/trump-administration-to-back-three-mineral-projects-with-58-million-in-financing/)</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/ramaco-resources-releases-hatch-report-and-shareholder-letter-on-exploratory-brook-mine-critical-minerals-project-302838319.html); [Mining.com](https://www.mining.com/ramaco-eyes-ree-stockpile-at-wyoming-mine/)</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>Boron Americas Project (Fort Cady)</t>
+          <t>Dewey-Burdock Uranium ISR Project</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>California, EE.UU.</t>
+          <t>Fall River/Custer Counties, Dakota del Sur, EE.UU.</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>5E Advanced Materials</t>
+          <t>enCore Energy (Powertech USA)</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
@@ -7240,71 +7201,71 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Financiamiento/planeación (préstamo EXIM Bank de US$8 millones anunciado 7-ago-2026 para proyecto de boro, lixiviación/procesamiento)</t>
+          <t>Construcción autorizada/permitting (BLM autorizó inicio de construcción de infraestructura —caminos, pozos de monitoreo, líneas eléctricas— jun-2026; NRC renovó la licencia, publicado en Federal Register 7-ago-2026; pendiente permiso estatal de Dakota del Sur, proceso reiniciado tras 13 años de pausa)</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>[EXIM.GOV](https://www.exim.gov/news/trump-administration-announces-58m-major-new-critical-mineral-deals-white-house-roundtable)</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/encore-energy-receives-bureau-of-land-management-authorization-to-begin-construction-at-dewey-burdock-uranium-project-302804230.html); [Federal Register](https://www.federalregister.gov/documents/2026/08/07/2026-16132/powertech-usa-inc-dewey-burdock-uranium-in-situ-recovery-project-license-renewal)</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>Brook Mine (tierras raras/minerales críticos de carbón)</t>
+          <t>Niron Magnetics — Planta de Imanes Permanentes sin Tierras Raras</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>Ranchester/Sheridan, Wyoming, EE.UU.</t>
+          <t>Minnesota, EE.UU. (ubicación exacta no especificada)</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>Ramaco Resources</t>
+          <t>Niron Magnetics</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>Hatch Associates Consultants (ingeniería/estudio)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/Construcción de planta piloto (Hatch publicó Initial Assessment Report jul-2026 con capex preliminar ~US$3,200 millones + US$800 millones de contingencia, VPN interno ~US$8,000 millones; planta piloto en construcción desde oct-2025; primer procesamiento de concentrados de óxido de tierras raras para la Defense Logistics Agency, ago-2026; construcción de planta comercial podría iniciar fines de 2026, producción comercial 2028)</t>
+          <t>Financiamiento asegurado (US$150 millones del Departamento de Defensa/Office of Strategic Capital, anunciado 7-8-ago-2026, parte de paquete federal de US$3,000 millones en minerales críticos)</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/ramaco-resources-releases-hatch-report-and-shareholder-letter-on-exploratory-brook-mine-critical-minerals-project-302838319.html); [Mining.com](https://www.mining.com/ramaco-eyes-ree-stockpile-at-wyoming-mine/)</t>
+          <t>[MINING.COM](https://www.mining.com/web/trump-says-us-is-announcing-a-series-of-mining-projects-worth-3-billion/); [CNBC](https://www.cnbc.com/2026/08/08/trump-admin-to-invest-3-billion-in-defense-linked-minerals-projects.html)</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Dewey-Burdock Uranium ISR Project</t>
+          <t>Louisiana Strategic Metals Complex</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>Fall River/Custer Counties, Dakota del Sur, EE.UU.</t>
+          <t>Alexandria, Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>enCore Energy (Powertech USA)</t>
+          <t>Ucore Rare Metals Inc.</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
@@ -7314,34 +7275,34 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Construcción autorizada/permitting (BLM autorizó inicio de construcción de infraestructura —caminos, pozos de monitoreo, líneas eléctricas— jun-2026; NRC renovó la licencia, publicado en Federal Register 7-ago-2026; pendiente permiso estatal de Dakota del Sur, proceso reiniciado tras 13 años de pausa)</t>
+          <t>Construcción (planta de procesamiento de tierras raras medianas/pesadas —terbio/disprosio—)</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/encore-energy-receives-bureau-of-land-management-authorization-to-begin-construction-at-dewey-burdock-uranium-project-302804230.html); [Federal Register](https://www.federalregister.gov/documents/2026/08/07/2026-16132/powertech-usa-inc-dewey-burdock-uranium-in-situ-recovery-project-license-renewal)</t>
+          <t>[Ucore Rare Metals](https://ucore.com/ucore-readies-for-louisiana-2026-heavy-rare-earth-element-processing/)</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>Niron Magnetics — Planta de Imanes Permanentes sin Tierras Raras</t>
+          <t>Distrito Copper Creek / San Manuel</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>Minnesota, EE.UU. (ubicación exacta no especificada)</t>
+          <t>Condado de Pinal, Arizona, EE.UU.</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>Niron Magnetics</t>
+          <t>Faraday Copper Corp. (adquiriendo la propiedad San Manuel de BHP; BHP recibirá ~30% de acciones de Faraday)</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
@@ -7351,71 +7312,71 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Financiamiento asegurado (US$150 millones del Departamento de Defensa/Office of Strategic Capital, anunciado 7-8-ago-2026, parte de paquete federal de US$3,000 millones en minerales críticos)</t>
+          <t>Exploración/definición de recursos (Faraday firmó acuerdo definitivo para comprar la antigua mina San Manuel de BHP —subterránea y de tajo/ISL, operada 1955-1999— y combinarla con su proyecto adyacente Copper Creek, creando un distrito de &gt;18,000 millones de libras de cobre; asamblea de accionistas 25-ago-2026 para aprobar la transacción, cierre esperado 3T2026; plan de 23,000+ metros de perforación de confirmación desde 4T2026, recurso combinado a mediados de 2027)</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>[MINING.COM](https://www.mining.com/web/trump-says-us-is-announcing-a-series-of-mining-projects-worth-3-billion/); [CNBC](https://www.cnbc.com/2026/08/08/trump-admin-to-invest-3-billion-in-defense-linked-minerals-projects.html)</t>
+          <t>[MINING.COM](https://www.mining.com/faraday-targets-18b-lb-arizona-copper-district/)</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-19</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>Louisiana Strategic Metals Complex</t>
+          <t>IMA Mine</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>Alexandria, Luisiana, EE.UU.</t>
+          <t>Condado de Lemhi, Idaho, EE.UU.</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>Ucore Rare Metals Inc.</t>
+          <t>American Tungsten Corp.</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>No especificado (geotécnica de presas de jales: NewFields MTDs)</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Construcción (planta de procesamiento de tierras raras medianas/pesadas —terbio/disprosio—)</t>
+          <t>Reactivación/pruebas metalúrgicas (mina histórica de tungsteno, produjo WO3 1945-1957; Fase I: reprocesamiento de jales superficiales; Fase II: rehabilitación de mina subterránea; pruebas metalúrgicas iniciadas jul-2026; definición de recursos, permisos y pruebas previstas concluir 4T2026, construcción fin de 2026/1T2027, primera venta de concentrado prevista inicios de 2027)</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>[Ucore Rare Metals](https://ucore.com/ucore-readies-for-louisiana-2026-heavy-rare-earth-element-processing/)</t>
+          <t>[MINING.COM](https://www.mining.com/american-tungsten-kinks-off-construction-at-ima-project-in-idaho/)</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-19</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>Distrito Copper Creek / San Manuel</t>
+          <t>Railroad Valley Minerals / Super-Brine Complex</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>Condado de Pinal, Arizona, EE.UU.</t>
+          <t>Railroad Valley, Nevada, EE.UU.</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>Faraday Copper Corp. (adquiriendo la propiedad San Manuel de BHP; BHP recibirá ~30% de acciones de Faraday)</t>
+          <t>3 Proton Lithium (3PL Operating Inc.)</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
@@ -7425,12 +7386,12 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Exploración/definición de recursos (Faraday firmó acuerdo definitivo para comprar la antigua mina San Manuel de BHP —subterránea y de tajo/ISL, operada 1955-1999— y combinarla con su proyecto adyacente Copper Creek, creando un distrito de &gt;18,000 millones de libras de cobre; asamblea de accionistas 25-ago-2026 para aprobar la transacción, cierre esperado 3T2026; plan de 23,000+ metros de perforación de confirmación desde 4T2026, recurso combinado a mediados de 2027)</t>
+          <t>Exploración avanzada (depósito multi-mineral confirmado: litio, potasa, boro y lo que la empresa describe como el mayor depósito de tungsteno de EE.UU. —~1.78 millones de toneladas, valorado en ~US$152,000 millones in-situ—; ~17 millas cuadradas del área están retiradas de minería desde 2023 por solicitud de la NASA para calibración de satélites, lo que representa un obstáculo regulatorio; sin decisión de construcción)</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>[MINING.COM](https://www.mining.com/faraday-targets-18b-lb-arizona-copper-district/)</t>
+          <t>[MINING.COM](https://www.mining.com/largest-us-tungsten-discovery-hits-nasa-roadblock/)</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -7442,32 +7403,32 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>IMA Mine</t>
+          <t>New Amalga Gold Project</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>Condado de Lemhi, Idaho, EE.UU.</t>
+          <t>~25 km al norte de Juneau, Alaska, EE.UU.</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>American Tungsten Corp.</t>
+          <t>Grande Portage Resources Ltd.</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>No especificado (geotécnica de presas de jales: NewFields MTDs)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Reactivación/pruebas metalúrgicas (mina histórica de tungsteno, produjo WO3 1945-1957; Fase I: reprocesamiento de jales superficiales; Fase II: rehabilitación de mina subterránea; pruebas metalúrgicas iniciadas jul-2026; definición de recursos, permisos y pruebas previstas concluir 4T2026, construcción fin de 2026/1T2027, primera venta de concentrado prevista inicios de 2027)</t>
+          <t>Permitting temprano (recurso Indicado de 1.44 millones oz Au a 9.47 g/t e Inferido de 515,700 oz Au; obtuvo estatus de "Covered Project" bajo FAST-41 el 30-jul-2026, acelerando la revisión federal coordinada; quinta mina en Alaska con cobertura FAST-41, junto con Arctic, Johnson Tract, Donlin Gold y Graphite Creek)</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>[MINING.COM](https://www.mining.com/american-tungsten-kinks-off-construction-at-ima-project-in-idaho/)</t>
+          <t>[Mining News North](https://www.miningnewsnorth.com/story/2026/08/07/news/new-amalga-gold-project-enters-fast-41/9803.html)</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -7479,17 +7440,17 @@
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>Railroad Valley Minerals / Super-Brine Complex</t>
+          <t>ElementUSA Gramercy — Planta de Tierras Raras/Minerales Críticos</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>Railroad Valley, Nevada, EE.UU.</t>
+          <t>Gramercy, St. John the Baptist Parish, Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>3 Proton Lithium (3PL Operating Inc.)</t>
+          <t>ElementUSA Inc. (en colaboración con Colorado School of Mines)</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
@@ -7499,71 +7460,71 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Exploración avanzada (depósito multi-mineral confirmado: litio, potasa, boro y lo que la empresa describe como el mayor depósito de tungsteno de EE.UU. —~1.78 millones de toneladas, valorado en ~US$152,000 millones in-situ—; ~17 millas cuadradas del área están retiradas de minería desde 2023 por solicitud de la NASA para calibración de satélites, lo que representa un obstáculo regulatorio; sin decisión de construcción)</t>
+          <t>Ingeniería/financiamiento asegurado (proyecto de US$850 millones para procesar "lodo rojo"/bauxite residue del antiguo refinerio de alúmina Atalco —~34 millones de toneladas almacenadas— y extraer galio, escandio, disprosio, gadolinio, iterbio, germanio e itrio; recibió US$67 millones del DOE y US$29.9 millones del DoD; construcción de planta de demostración prevista a iniciar mediados de 2027, producción inicial 3T2028); Atalco (refinería de alúmina que aloja el sitio, entidad distinta co-ubicada) recibió 28-ago-2026 una inversión de capital adicional de US$100 millones del Departamento de Guerra de EE.UU. —participación total del DoW ahora US$400M, US$800M contando coinversión privada desde ene-2026— para restaurar la refinería, única refinería de alúmina activa en EE.UU., a su capacidad nominal de 1.2 millones ton/año, lo que apoya indirectamente la operación de ElementUSA en el mismo sitio</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>[MINING.COM](https://www.mining.com/largest-us-tungsten-discovery-hits-nasa-roadblock/)</t>
+          <t>[Biz New Orleans](https://bizneworleans.com/elementusa-plans-850m-critical-minerals-refining-facility/); [Colorado School of Mines](https://www.minesnewsroom.com/news/colorado-school-mines-and-elementusa-awarded-67m-doe-construction-rare-earth-processing-plant); [Departamento de Guerra de EE.UU.](https://www.war.gov/News/Releases/Release/Article/4585310/department-of-war-announces-a-100-million-follow-on-equity-investment-in-atalco/)</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-09-02</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>New Amalga Gold Project</t>
+          <t>Planta de Refinación de Tierras Raras y Minerales Críticos Marion (ReElement Technologies)</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>~25 km al norte de Juneau, Alaska, EE.UU.</t>
+          <t>Marion, Indiana, EE.UU.</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>Grande Portage Resources Ltd.</t>
+          <t>American Resources Corporation (NASDAQ: AREC) vía subsidiaria ReElement Technologies</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>No especificado (acondicionamiento interno de la ex planta RCA Thomson, 425,000 pies² en campus de 42 acres)</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>Permitting temprano (recurso Indicado de 1.44 millones oz Au a 9.47 g/t e Inferido de 515,700 oz Au; obtuvo estatus de "Covered Project" bajo FAST-41 el 30-jul-2026, acelerando la revisión federal coordinada; quinta mina en Alaska con cobertura FAST-41, junto con Arctic, Johnson Tract, Donlin Gold y Graphite Creek)</t>
+          <t>Permiso de aire obtenido/comisionamiento (IDEM —Indiana— otorgó el permiso "Minor Source" para 4 líneas de producción de Fase 1, &gt;16,000 t/año de óxidos separados de alta pureza —Nd, Pr, Dy, Tb, Gd, Sm, Y, galio, germanio—; arranque de producción inicial previsto 3T2026)</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>[Mining News North](https://www.miningnewsnorth.com/story/2026/08/07/news/new-amalga-gold-project-enters-fast-41/9803.html)</t>
+          <t>[Mining Technology](https://www.mining-technology.com/news/air-permits-reelements-marion-refinery-indiana/); [Investing News Network](https://investingnews.com/reelement-technologies-receives-air-permits-for-marion-indiana-rare-earth-and-critical-mineral-refinery/)</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>ElementUSA Gramercy — Planta de Tierras Raras/Minerales Críticos</t>
+          <t>La Preciosa Project</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>Gramercy, St. John the Baptist Parish, Luisiana, EE.UU.</t>
+          <t>Durango, México</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>ElementUSA Inc. (en colaboración con Colorado School of Mines)</t>
+          <t>Avino Silver &amp; Gold Mines Ltd.</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
@@ -7573,71 +7534,71 @@
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/financiamiento asegurado (proyecto de US$850 millones para procesar "lodo rojo"/bauxite residue del antiguo refinerio de alúmina Atalco —~34 millones de toneladas almacenadas— y extraer galio, escandio, disprosio, gadolinio, iterbio, germanio e itrio; recibió US$67 millones del DOE y US$29.9 millones del DoD; construcción de planta de demostración prevista a iniciar mediados de 2027, producción inicial 3T2028); Atalco (refinería de alúmina que aloja el sitio, entidad distinta co-ubicada) recibió 28-ago-2026 una inversión de capital adicional de US$100 millones del Departamento de Guerra de EE.UU. —participación total del DoW ahora US$400M, US$800M contando coinversión privada desde ene-2026— para restaurar la refinería, única refinería de alúmina activa en EE.UU., a su capacidad nominal de 1.2 millones ton/año, lo que apoya indirectamente la operación de ElementUSA en el mismo sitio</t>
+          <t>Construcción (desarrollo subterráneo en curso —rampa/decline de 360m—; permisos mineros ya obtenidos; producción objetivo 4T2026)</t>
         </is>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>[Biz New Orleans](https://bizneworleans.com/elementusa-plans-850m-critical-minerals-refining-facility/); [Colorado School of Mines](https://www.minesnewsroom.com/news/colorado-school-mines-and-elementusa-awarded-67m-doe-construction-rare-earth-processing-plant); [Departamento de Guerra de EE.UU.](https://www.war.gov/News/Releases/Release/Article/4585310/department-of-war-announces-a-100-million-follow-on-equity-investment-in-atalco/)</t>
+          <t>[AccessWire](https://www.accessnewswire.com/newsroom/en/metals-and-mining/avino-provides-update-on-its-100-owned-la-preciosa-property-preparing-for-producti-837173); [MarketScreener](https://www.marketscreener.com/quote/stock/AVINO-SILVER-GOLD-MINES-L-1409069/news/Avino-Silver-Gold-Mines-Ltd-Commences-Underground-Development-At-La-Preciosa-48766238/)</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>Planta de Refinación de Tierras Raras y Minerales Críticos Marion (ReElement Technologies)</t>
+          <t>Great Salt Lake Lithium Facility</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>Marion, Indiana, EE.UU.</t>
+          <t>Condado de Box Elder, Utah, EE.UU.</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>American Resources Corporation (NASDAQ: AREC) vía subsidiaria ReElement Technologies</t>
+          <t>Lilac Solutions (subsidiaria Waterleaf P1 HoldCo)</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>No especificado (acondicionamiento interno de la ex planta RCA Thomson, 425,000 pies² en campus de 42 acres)</t>
+          <t>Hatch (EPCM, seleccionado jun-2026)</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>Permiso de aire obtenido/comisionamiento (IDEM —Indiana— otorgó el permiso "Minor Source" para 4 líneas de producción de Fase 1, &gt;16,000 t/año de óxidos separados de alta pureza —Nd, Pr, Dy, Tb, Gd, Sm, Y, galio, germanio—; arranque de producción inicial previsto 3T2026)</t>
+          <t>Desarrollo/Ingeniería (DOE anunció 20/21-ago-2026 subvención de hasta US$100 millones para construir planta comercial de extracción/refinación de litio por intercambio iónico directo desde salmuera del Great Salt Lake, 5,000 t/año; primera producción prevista 2028) ; DOE otorgó US$100 millones (anuncio 20-ago-2026) para la instalación comercial de extracción/refinación de litio mediante DLE de Lilac Solutions; capacidad de primera fase 5,000 ton/año, producción objetivo 2028</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>[Mining Technology](https://www.mining-technology.com/news/air-permits-reelements-marion-refinery-indiana/); [Investing News Network](https://investingnews.com/reelement-technologies-receives-air-permits-for-marion-indiana-rare-earth-and-critical-mineral-refinery/)</t>
+          <t>[KSL](https://www.ksl.com/article/51614351/california-company-awarded-100m-to-develop-critical-mineral-facility-on-great-salt-lake-shore); [Hatch](https://www.hatch.com/About-Us/News-And-Media/2026/06/Lilac-Solutions-Selects-Hatch-as-EPCM-Partner-for-Great-Salt-Lake-Lithium-Facility) ; [DOE](https://www.energy.gov/articles/energy-department-announces-500-million-secure-americas-critical-mineral-and-battery)</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>La Preciosa Project</t>
+          <t>Project SHIELD (refinería de "black mass" de baterías)</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>Durango, México</t>
+          <t>Carolina del Sur, EE.UU. (sitio exacto por definir)</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>Avino Silver &amp; Gold Mines Ltd.</t>
+          <t>Nth Cycle, Inc.</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
@@ -7647,49 +7608,49 @@
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>Construcción (desarrollo subterráneo en curso —rampa/decline de 360m—; permisos mineros ya obtenidos; producción objetivo 4T2026)</t>
+          <t>Negociación de subvención/preconstrucción (DOE seleccionó a Nth Cycle 20/21-ago-2026 para negociar premio de hasta US$100 millones; planta de refinación de "black mass" de baterías de litio, producirá MHP de níquel y carbonato de litio grado batería, 24,000 t/año; operación proyectada 2028)</t>
         </is>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>[AccessWire](https://www.accessnewswire.com/newsroom/en/metals-and-mining/avino-provides-update-on-its-100-owned-la-preciosa-property-preparing-for-producti-837173); [MarketScreener](https://www.marketscreener.com/quote/stock/AVINO-SILVER-GOLD-MINES-L-1409069/news/Avino-Silver-Gold-Mines-Ltd-Commences-Underground-Development-At-La-Preciosa-48766238/)</t>
+          <t>[Nth Cycle](https://nthcycle.com/newsroom/u.s.-department-of-energy-selects-nth-cycle-to-enter-award-negotiations-for-up-to-100-million-to-build-new-critical-mineral-refining-facility)</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>Great Salt Lake Lithium Facility</t>
+          <t>Refinería de Sulfato de Cobalto — Formation Holdings/Jervois</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>Condado de Box Elder, Utah, EE.UU.</t>
+          <t>Sitio por definir, EE.UU. (empresa con sede en Salmon, Idaho)</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>Lilac Solutions (subsidiaria Waterleaf P1 HoldCo)</t>
+          <t>Formation Holdings US, Inc. (dba Jervois)</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>Hatch (EPCM, seleccionado jun-2026)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>Desarrollo/Ingeniería (DOE anunció 20/21-ago-2026 subvención de hasta US$100 millones para construir planta comercial de extracción/refinación de litio por intercambio iónico directo desde salmuera del Great Salt Lake, 5,000 t/año; primera producción prevista 2028) ; DOE otorgó US$100 millones (anuncio 20-ago-2026) para la instalación comercial de extracción/refinación de litio mediante DLE de Lilac Solutions; capacidad de primera fase 5,000 ton/año, producción objetivo 2028</t>
+          <t>Desarrollo/financiamiento (DOE otorgó 21-ago-2026 subvención de US$100 millones para construir refinería comercial de sulfato de cobalto grado batería; ubicación específica de la planta aún no anunciada) ; DOE seleccionó el proyecto para un aporte federal de US$100 millones (anuncio 20-ago-2026) hacia una refinería comercial de cobalto; sitio industrial aún por determinar</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>[KSL](https://www.ksl.com/article/51614351/california-company-awarded-100m-to-develop-critical-mineral-facility-on-great-salt-lake-shore); [Hatch](https://www.hatch.com/About-Us/News-And-Media/2026/06/Lilac-Solutions-Selects-Hatch-as-EPCM-Partner-for-Great-Salt-Lake-Lithium-Facility) ; [DOE](https://www.energy.gov/articles/energy-department-announces-500-million-secure-americas-critical-mineral-and-battery)</t>
+          <t>[Local News 8](https://localnews8.com/news/business-watch/2026/08/21/salmon-company-wins-100-million-grant-to-build-cobalt-refinery/); [Local News 8 (seguimiento)](https://localnews8.com/news/local-news/2026/08/24/100m-grant-to-salmon-based-jervois-could-jumpstart-idahos-cobalt-industry/) ; [DOE](https://www.energy.gov/articles/energy-department-announces-500-million-secure-americas-critical-mineral-and-battery)</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
@@ -7701,106 +7662,106 @@
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>Project SHIELD (refinería de "black mass" de baterías)</t>
+          <t>Copperwood Project</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>Carolina del Sur, EE.UU. (sitio exacto por definir)</t>
+          <t>Península Superior Occidental, cerca de Wakefield, Michigan, EE.UU.</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>Nth Cycle, Inc.</t>
+          <t>Highland Copper Company</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>DRA Americas Inc. (FEED)</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>Negociación de subvención/preconstrucción (DOE seleccionó a Nth Cycle 20/21-ago-2026 para negociar premio de hasta US$100 millones; planta de refinación de "black mass" de baterías de litio, producirá MHP de níquel y carbonato de litio grado batería, 24,000 t/año; operación proyectada 2028)</t>
+          <t>Ingeniería/FEED (~40% completo para 4T2026; decisión de construcción esperada en 2S2026; producción de cobre proyectada 2029; capex ~US$425 millones)</t>
         </is>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>[Nth Cycle](https://nthcycle.com/newsroom/u.s.-department-of-energy-selects-nth-cycle-to-enter-award-negotiations-for-up-to-100-million-to-build-new-critical-mineral-refining-facility)</t>
+          <t>[Highland Copper](https://www.highlandcopper.com/news/highland-copper-recaps-2025-execution-and-announces-2026-work-plan-to-advance-copperwood-toward-construction-decision/)</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>Refinería de Sulfato de Cobalto — Formation Holdings/Jervois</t>
+          <t>Modernización Refinería de Cobre El Paso</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>Sitio por definir, EE.UU. (empresa con sede en Salmon, Idaho)</t>
+          <t>El Paso, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>Formation Holdings US, Inc. (dba Jervois)</t>
+          <t>Freeport-McMoRan</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>EPCM Group (tecnología de cátodos permanentes); Metso (equipo de tankhouse)</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>Desarrollo/financiamiento (DOE otorgó 21-ago-2026 subvención de US$100 millones para construir refinería comercial de sulfato de cobalto grado batería; ubicación específica de la planta aún no anunciada) ; DOE seleccionó el proyecto para un aporte federal de US$100 millones (anuncio 20-ago-2026) hacia una refinería comercial de cobalto; sitio industrial aún por determinar</t>
+          <t>Contrato adjudicado 2026 (modernización de refinería electrolítica, 46,650 cátodos permanentes, sustituye tecnología de láminas de arranque tradicional)</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>[Local News 8](https://localnews8.com/news/business-watch/2026/08/21/salmon-company-wins-100-million-grant-to-build-cobalt-refinery/); [Local News 8 (seguimiento)](https://localnews8.com/news/local-news/2026/08/24/100m-grant-to-salmon-based-jervois-could-jumpstart-idahos-cobalt-industry/) ; [DOE](https://www.energy.gov/articles/energy-department-announces-500-million-secure-americas-critical-mineral-and-battery)</t>
+          <t>[EPCM Group](https://www.epcm.com/epcm-secures-prestigious-contract-with-freeport-mcmoran-to-advance-el-paso-copper-refinery-modernization/)</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-26</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>Copperwood Project</t>
+          <t>Round Top Rare Earth Project</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>Península Superior Occidental, cerca de Wakefield, Michigan, EE.UU.</t>
+          <t>Sierra Blanca, Condado de Hudspeth, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>Highland Copper Company</t>
+          <t>USA Rare Earth Inc.</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>DRA Americas Inc. (FEED)</t>
+          <t>Fluor Corporation / WSP Global Inc. (EPCM para estudio de factibilidad definitivo)</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/FEED (~40% completo para 4T2026; decisión de construcción esperada en 2S2026; producción de cobre proyectada 2029; capex ~US$425 millones)</t>
+          <t>Ingeniería/DFS (en curso; subvención estatal de Texas de US$14.2 millones, may-2026; inversión estimada &gt;US$1,400 millones; producción adelantada a fines de 2028; tierras raras pesadas)</t>
         </is>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>[Highland Copper](https://www.highlandcopper.com/news/highland-copper-recaps-2025-execution-and-announces-2026-work-plan-to-advance-copperwood-toward-construction-decision/)</t>
+          <t>[IM Mining](https://im-mining.com/2026/01/23/fluor-and-wsp-on-board-usa-rare-earth-incs-round-top-rare-earth-project/)</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
@@ -7812,32 +7773,32 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>Modernización Refinería de Cobre El Paso</t>
+          <t>Expansión Fundición de Antimonio Thompson Falls</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>El Paso, Texas, EE.UU.</t>
+          <t>Thompson Falls, Montana, EE.UU.</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>Freeport-McMoRan</t>
+          <t>United States Antimony Corporation (USAC)</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>EPCM Group (tecnología de cátodos permanentes); Metso (equipo de tankhouse)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>Contrato adjudicado 2026 (modernización de refinería electrolítica, 46,650 cátodos permanentes, sustituye tecnología de láminas de arranque tradicional)</t>
+          <t>Comisionamiento (nueva fundición construida; comisionamiento de 9 hornos a gas iniciado may-2026; financiada con US$27 millones del Departamento de Guerra, mar-2026)</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>[EPCM Group](https://www.epcm.com/epcm-secures-prestigious-contract-with-freeport-mcmoran-to-advance-el-paso-copper-refinery-modernization/)</t>
+          <t>[Montana Public Radio](https://www.mtpr.org/montana-news/2026-04-06/montana-antimony-facility-expands-amid-federal-push-for-domestic-sources)</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
@@ -7849,32 +7810,32 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>Round Top Rare Earth Project</t>
+          <t>Expansión Planta de Lixiviación de Concentrados (CLP) Morenci</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>Sierra Blanca, Condado de Hudspeth, Texas, EE.UU.</t>
+          <t>Morenci, Arizona, EE.UU.</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>USA Rare Earth Inc.</t>
+          <t>Freeport-McMoRan</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>Fluor Corporation / WSP Global Inc. (EPCM para estudio de factibilidad definitivo)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/DFS (en curso; subvención estatal de Texas de US$14.2 millones, may-2026; inversión estimada &gt;US$1,400 millones; producción adelantada a fines de 2028; tierras raras pesadas)</t>
+          <t>Comisionamiento (segundo y último vaso de la expansión en comisionamiento/ajuste durante 2026; objetivo casi duplicar throughput de 24 a 40 ton/hora)</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>[IM Mining](https://im-mining.com/2026/01/23/fluor-and-wsp-on-board-usa-rare-earth-incs-round-top-rare-earth-project/)</t>
+          <t>[Freeport-McMoRan](https://www.fcx.com/freeport-features/112125)</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
@@ -7886,17 +7847,17 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>Expansión Fundición de Antimonio Thompson Falls</t>
+          <t>Reconstrucción Fundición y Refinería Kennecott</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>Thompson Falls, Montana, EE.UU.</t>
+          <t>Bingham Canyon/Kennecott, Utah, EE.UU.</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>United States Antimony Corporation (USAC)</t>
+          <t>Rio Tinto (Kennecott Utah Copper)</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
@@ -7906,12 +7867,12 @@
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>Comisionamiento (nueva fundición construida; comisionamiento de 9 hornos a gas iniciado may-2026; financiada con US$27 millones del Departamento de Guerra, mar-2026)</t>
+          <t>Construcción (reconstrucción de fundición US$300 millones y actualización de refinería/tankhouse y circuito de flotación de molibdeno US$120 millones en curso durante 2026; reparación adicional tras falla de horno flash en jun-2026, ~75 días)</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>[Montana Public Radio](https://www.mtpr.org/montana-news/2026-04-06/montana-antimony-facility-expands-amid-federal-push-for-domestic-sources)</t>
+          <t>[Mining.com](https://www.mining.com/web/rio-tinto-to-invest-almost-1-billion-in-kennecott-copper-mine/)</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
@@ -7923,32 +7884,32 @@
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>Expansión Planta de Lixiviación de Concentrados (CLP) Morenci</t>
+          <t>Fourmile (decline Bullion Hill)</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>Morenci, Arizona, EE.UU.</t>
+          <t>Carlin Trend, condados de Elko/Eureka, Nevada, EE.UU.</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>Freeport-McMoRan</t>
+          <t>Barrick Mining Corporation (JV Nevada Gold Mines, desde ago-2026)</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Barminco (Perenti) — contrato A$275 millones/45 meses</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>Comisionamiento (segundo y último vaso de la expansión en comisionamiento/ajuste durante 2026; objetivo casi duplicar throughput de 24 a 40 ton/hora)</t>
+          <t>Construcción (inicio de desarrollo subterráneo/portales programado jul/3T2026; ~16 km de desarrollo lateral subterráneo planeados; adyacente al complejo Goldrush)</t>
         </is>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>[Freeport-McMoRan](https://www.fcx.com/freeport-features/112125)</t>
+          <t>[Northern Miner](https://www.northernminer.com/news/mining-forum-americas-fourmile-anchors-barricks-nevada-plan/1003882789/)</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -7960,17 +7921,17 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>Reconstrucción Fundición y Refinería Kennecott</t>
+          <t>Puerto del Aire (distrito Mulatos)</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>Bingham Canyon/Kennecott, Utah, EE.UU.</t>
+          <t>Sonora, México</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>Rio Tinto (Kennecott Utah Copper)</t>
+          <t>Alamos Gold Inc.</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
@@ -7980,12 +7941,12 @@
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>Construcción (reconstrucción de fundición US$300 millones y actualización de refinería/tankhouse y circuito de flotación de molibdeno US$120 millones en curso durante 2026; reparación adicional tras falla de horno flash en jun-2026, ~75 días)</t>
+          <t>Construcción (en curso desde 2025-2026 tras permiso ambiental ene-2025; procura de equipos de molienda de largo plazo de entrega; capex total US$165 millones; primera producción prevista mediados 2027)</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>[Mining.com](https://www.mining.com/web/rio-tinto-to-invest-almost-1-billion-in-kennecott-copper-mine/)</t>
+          <t>[Alamos Gold](https://www.alamosgold.com/news-and-events/news/news-details/2025/Alamos-Gold-Announces-Receipt-of-Environmental-Permit-Amendment-Allowing-for-the-Start-of-Construction-on-the-Puerto-Del-Aire-Project-in-Mexico/default.aspx)</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -7997,54 +7958,54 @@
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>Fourmile (decline Bullion Hill)</t>
+          <t>Korea Zinc / Nyrstar Critical Minerals Smelter</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>Carlin Trend, condados de Elko/Eureka, Nevada, EE.UU.</t>
+          <t>Clarksville, Tennessee, EE.UU.</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>Barrick Mining Corporation (JV Nevada Gold Mines, desde ago-2026)</t>
+          <t>Korea Zinc / U.S. Department of War / U.S. Department of Commerce (participación ~10%)</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>Barminco (Perenti) — contrato A$275 millones/45 meses</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>Construcción (inicio de desarrollo subterráneo/portales programado jul/3T2026; ~16 km de desarrollo lateral subterráneo planeados; adyacente al complejo Goldrush)</t>
+          <t>Preparación de sitio en 2026, construcción completa en 2027 (inversión US$7,400 millones, capex US$6,600 millones; producirá zinc, plomo, cobre, oro, plata, antimonio, indio, bismuto, telurio, cadmio, galio, germanio, paladio y ácido sulfúrico; planta altamente intensiva en tubería/piping)</t>
         </is>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>[Northern Miner](https://www.northernminer.com/news/mining-forum-americas-fourmile-anchors-barricks-nevada-plan/1003882789/)</t>
+          <t>[Korea Zinc](https://www.koreazinc.co.kr/en/korea-zinc-partners-with-the-u-s-department-of-war-and-u-s-department-of-commerce-to-build-a-state-of-the-art-critical-minerals-smelter-in-the-united-states-with-6-6-billion-of-capital-expenditures/); [Carbon Credits](https://carboncredits.com/big-bet-bigger-stakes-korea-zincs-7-4-billion-smelter-reshapes-u-s-critical-minerals-supply/)</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>Puerto del Aire (distrito Mulatos)</t>
+          <t>Aclara Heavy Rare Earth Separation Facility</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>Sonora, México</t>
+          <t>Port of Vinton, Calcasieu Parish, Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>Alamos Gold Inc.</t>
+          <t>Aclara Resources Inc.</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
@@ -8054,34 +8015,34 @@
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>Construcción (en curso desde 2025-2026 tras permiso ambiental ene-2025; procura de equipos de molienda de largo plazo de entrega; capex total US$165 millones; primera producción prevista mediados 2027)</t>
+          <t>Planeación (inversión US$277 millones; groundbreaking previsto 4T2026, construcción hasta 2027; procesará mineral de depósitos propios en Brasil/Chile)</t>
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>[Alamos Gold](https://www.alamosgold.com/news-and-events/news/news-details/2025/Alamos-Gold-Announces-Receipt-of-Environmental-Permit-Amendment-Allowing-for-the-Start-of-Construction-on-the-Puerto-Del-Aire-Project-in-Mexico/default.aspx)</t>
+          <t>[Louisiana Economic Development](https://www.opportunitylouisiana.gov/news/aclara-invests-277-million-to-build-nations-first-heavy-rare-earth-separation-facility-in-southwest-louisiana)</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>Korea Zinc / Nyrstar Critical Minerals Smelter</t>
+          <t>Archimedes Project (i-80 Gold)</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>Clarksville, Tennessee, EE.UU.</t>
+          <t>Ruby Hill, Eureka County, Nevada, EE.UU.</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>Korea Zinc / U.S. Department of War / U.S. Department of Commerce (participación ~10%)</t>
+          <t>i-80 Gold Corp</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
@@ -8091,12 +8052,12 @@
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>Preparación de sitio en 2026, construcción completa en 2027 (inversión US$7,400 millones, capex US$6,600 millones; producirá zinc, plomo, cobre, oro, plata, antimonio, indio, bismuto, telurio, cadmio, galio, germanio, paladio y ácido sulfúrico; planta altamente intensiva en tubería/piping)</t>
+          <t>Construcción (permisos de Nevada DEP y BLM obtenidos; desarrollo subterráneo en curso; producción esperada 4T2026, objetivo 150,000-200,000 oz Au/año hacia 2028)</t>
         </is>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>[Korea Zinc](https://www.koreazinc.co.kr/en/korea-zinc-partners-with-the-u-s-department-of-war-and-u-s-department-of-commerce-to-build-a-state-of-the-art-critical-minerals-smelter-in-the-united-states-with-6-6-billion-of-capital-expenditures/); [Carbon Credits](https://carboncredits.com/big-bet-bigger-stakes-korea-zincs-7-4-billion-smelter-reshapes-u-s-critical-minerals-supply/)</t>
+          <t>[Resource World](https://resourceworld.com/i-80-gold-obtains-construction-permits-and-begins-underground-development-at-archimedes-project-nevada/)</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -8108,17 +8069,17 @@
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>Aclara Heavy Rare Earth Separation Facility</t>
+          <t>Sweetwater Uranium In-Situ Recovery (ISR) Project</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>Port of Vinton, Calcasieu Parish, Luisiana, EE.UU.</t>
+          <t>Sweetwater County, Wyoming, EE.UU.</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>Aclara Resources Inc.</t>
+          <t>Sweetwater Uranium, Inc.</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
@@ -8128,12 +8089,12 @@
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>Planeación (inversión US$277 millones; groundbreaking previsto 4T2026, construcción hasta 2027; procesará mineral de depósitos propios en Brasil/Chile)</t>
+          <t>Permitting (Plan de Operaciones sometido al BLM nov-2025, periodo de comentarios públicos mar-abr 2026, proyecto designado FAST-41; sería la mayor instalación de producción de uranio de EE.UU. combinando procesamiento convencional e ISR)</t>
         </is>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>[Louisiana Economic Development](https://www.opportunitylouisiana.gov/news/aclara-invests-277-million-to-build-nations-first-heavy-rare-earth-separation-facility-in-southwest-louisiana)</t>
+          <t>[BLM](https://www.blm.gov/announcement/sweetwater-uranium-situ-recovery-irs-project-mine-plan-operations)</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -8145,17 +8106,17 @@
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>Archimedes Project (i-80 Gold)</t>
+          <t>Velvet-Wood Uranium-Vanadium Project</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>Ruby Hill, Eureka County, Nevada, EE.UU.</t>
+          <t>San Juan County, Utah, EE.UU.</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>i-80 Gold Corp</t>
+          <t>Anfield Energy Inc.</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
@@ -8165,12 +8126,12 @@
       </c>
       <c r="E105" s="2" t="inlineStr">
         <is>
-          <t>Construcción (permisos de Nevada DEP y BLM obtenidos; desarrollo subterráneo en curso; producción esperada 4T2026, objetivo 150,000-200,000 oz Au/año hacia 2028)</t>
+          <t>Construcción (Fase 1 de construcción superficial completada jun-2026; desarrollo subterráneo Fase 2 en curso; regreso a producción previsto fines de 2026)</t>
         </is>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>[Resource World](https://resourceworld.com/i-80-gold-obtains-construction-permits-and-begins-underground-development-at-archimedes-project-nevada/)</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/06/01/3304179/0/en/Anfield-Energy-Inc-Completes-Phase-One-Surface-Construction-at-Velvet-Wood-Project.html)</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -8182,185 +8143,185 @@
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>Sweetwater Uranium In-Situ Recovery (ISR) Project</t>
+          <t>Twin Metals Minnesota</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>Sweetwater County, Wyoming, EE.UU.</t>
+          <t>Ely, Minnesota, EE.UU. (cerca de Boundary Waters)</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>Sweetwater Uranium, Inc.</t>
+          <t>Antofagasta plc (Twin Metals Minnesota LLC)</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>No definido</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
         <is>
-          <t>Permitting (Plan de Operaciones sometido al BLM nov-2025, periodo de comentarios públicos mar-abr 2026, proyecto designado FAST-41; sería la mayor instalación de producción de uranio de EE.UU. combinando procesamiento convencional e ISR)</t>
+          <t>Permitting/Pre-EIS (plan de mina formal —concentradora de flotación de 20,000 tpd, cobre-níquel-EGP— presentado ante BLM y Minnesota DNR; el gobernador Walz frenó el trámite estatal en ago-2026, pero el proceso federal continúa activo; construcción aún a años de distancia)</t>
         </is>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>[BLM](https://www.blm.gov/announcement/sweetwater-uranium-situ-recovery-irs-project-mine-plan-operations)</t>
+          <t>[MinnPost](http://www.minnpost.com/state-government/2026/08/walz-halts-state-action-on-mine-near-boundary-waters-but-federal-process-stays-on-track/); [Star Tribune](https://www.startribune.com/twin-metals-submits-formal-mine-plan-to-minnesota-federal-officials/566311242)</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>Velvet-Wood Uranium-Vanadium Project</t>
+          <t>Falcon Copper — Fundición y Refinería de Cobre (greenfield)</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>San Juan County, Utah, EE.UU.</t>
+          <t>Arizona (fundición) / Costa del Golfo (refinería), EE.UU. (sitios por definir)</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>Anfield Energy Inc.</t>
+          <t>Falcon Copper Corp. (MOU con Glencore)</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>No definido</t>
         </is>
       </c>
       <c r="E107" s="2" t="inlineStr">
         <is>
-          <t>Construcción (Fase 1 de construcción superficial completada jun-2026; desarrollo subterráneo Fase 2 en curso; regreso a producción previsto fines de 2026)</t>
+          <t>Evaluación/pre-FEED (proyecto greenfield de ~US$2,000 millones para fundición primaria de cobre más refinería electrolítica; sin sitio definitivo ni FID)</t>
         </is>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/06/01/3304179/0/en/Anfield-Energy-Inc-Completes-Phase-One-Surface-Construction-at-Velvet-Wood-Project.html)</t>
+          <t>[Fastmarkets](https://www.fastmarkets.com/insights/us-copper-smelting-equation-gap-or-glut-hotter-commodities-articles/); [Falcon Copper](https://www.falconcopper.com/projects/works)</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>Twin Metals Minnesota</t>
+          <t>Del Sol Refinery (antimonio/tungsteno) + White Spar Antimony Mine</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>Ely, Minnesota, EE.UU. (cerca de Boundary Waters)</t>
+          <t>Amargosa Valley, Nevada (refinería) / Arizona (mina), EE.UU.</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>Antofagasta plc (Twin Metals Minnesota LLC)</t>
+          <t>American Tungsten &amp; Antimony Corp (ATALF)</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>No definido</t>
+          <t>Metso Finland Oy (estudio de alcance)</t>
         </is>
       </c>
       <c r="E108" s="2" t="inlineStr">
         <is>
-          <t>Permitting/Pre-EIS (plan de mina formal —concentradora de flotación de 20,000 tpd, cobre-níquel-EGP— presentado ante BLM y Minnesota DNR; el gobernador Walz frenó el trámite estatal en ago-2026, pero el proceso federal continúa activo; construcción aún a años de distancia)</t>
+          <t>Ingeniería/estudio (adquirió el 28-jul-2026 la refinería hidrometalúrgica permisada de antimonio Del Sol —18,500 t/año de capacidad de alimentación— y la mina White Spar (AZ) como fuente de mineral; 1-sep-2026 contrató a Metso para estudio de alcance de un circuito de producción de paratungstato de amonio —APT—, Fase 1: 2,500 t/año, posible Fase 2 a 5,000 t/año; la refinería también recibirá mineral del proyecto Antimony Canyon, Utah)</t>
         </is>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>[MinnPost](http://www.minnpost.com/state-government/2026/08/walz-halts-state-action-on-mine-near-boundary-waters-but-federal-process-stays-on-track/); [Star Tribune](https://www.startribune.com/twin-metals-submits-formal-mine-plan-to-minnesota-federal-officials/566311242)</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/american-tungsten-and-antimony-announces-study-for-tungsten-production-at-del-sol-refinery-in-nevada-302866335.html); [PR Newswire](https://www.prnewswire.com/news-releases/american-tungsten-and-antimony-to-acquire-permitted-critical-metals-refinery-in-nevada-and-white-spar-antimony-mine-in-arizona-302836579.html)</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-02</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>Falcon Copper — Fundición y Refinería de Cobre (greenfield)</t>
+          <t>Spring Valley Gold Mine</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>Arizona (fundición) / Costa del Golfo (refinería), EE.UU. (sitios por definir)</t>
+          <t>Condado de Pershing, Nevada, EE.UU.</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>Falcon Copper Corp. (MOU con Glencore)</t>
+          <t>Solidus Resources LLC (subsidiaria de Waterton Gold)</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
-          <t>No definido</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E109" s="2" t="inlineStr">
         <is>
-          <t>Evaluación/pre-FEED (proyecto greenfield de ~US$2,000 millones para fundición primaria de cobre más refinería electrolítica; sin sitio definitivo ni FID)</t>
+          <t>Construcción (todos los permisos federales en mano —BLM aprobó el plan de operaciones—; proyecto totalmente financiado, ~US$1,300 millones de capital comprometido incl. stream de oro de US$670M de Wheaton Precious Metals; trabajos de sitio tempranos en curso, construcción completa inicia en 2026; primera producción de oro proyectada 1S2028; reservas probadas/probables de 3.8 Moz Au)</t>
         </is>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>[Fastmarkets](https://www.fastmarkets.com/insights/us-copper-smelting-equation-gap-or-glut-hotter-commodities-articles/); [Falcon Copper](https://www.falconcopper.com/projects/works)</t>
+          <t>[BLM](https://www.blm.gov/announcement/blm-approves-spring-valley-gold-mine-pershing-county); [Wheaton Precious Metals](https://www.wheatonpm.com/portfolio/development-projects/spring-valley/default.aspx); [The Pershing Post](https://www.thepershingpost.com/article/496,spring-valley-mine-project-moves-into-construction-phase-hiring-to-begin-in-2026)</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-03</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>Del Sol Refinery (antimonio/tungsteno) + White Spar Antimony Mine</t>
+          <t>Pitarrilla Project (plata-plomo-zinc)</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>Amargosa Valley, Nevada (refinería) / Arizona (mina), EE.UU.</t>
+          <t>160 km al norte de la ciudad de Durango, Durango, México</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>American Tungsten &amp; Antimony Corp (ATALF)</t>
+          <t>Endeavour Silver Corp.</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>Metso Finland Oy (estudio de alcance)</t>
+          <t>SGS Canada / SGS Bateman / JDS Energy &amp; Mining / T Engineering / Stantec / SRK Consulting (estudio de factibilidad)</t>
         </is>
       </c>
       <c r="E110" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/estudio (adquirió el 28-jul-2026 la refinería hidrometalúrgica permisada de antimonio Del Sol —18,500 t/año de capacidad de alimentación— y la mina White Spar (AZ) como fuente de mineral; 1-sep-2026 contrató a Metso para estudio de alcance de un circuito de producción de paratungstato de amonio —APT—, Fase 1: 2,500 t/año, posible Fase 2 a 5,000 t/año; la refinería también recibirá mineral del proyecto Antimony Canyon, Utah)</t>
+          <t>Ingeniería/estudio de factibilidad (inversión 2026 de US$65.8 millones: US$15M para estudio de factibilidad, US$48M en capex de preparación minera y 1,300 m de desarrollo subterráneo; aún sin decisión de construcción)</t>
         </is>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/american-tungsten-and-antimony-announces-study-for-tungsten-production-at-del-sol-refinery-in-nevada-302866335.html); [PR Newswire](https://www.prnewswire.com/news-releases/american-tungsten-and-antimony-to-acquire-permitted-critical-metals-refinery-in-nevada-and-white-spar-antimony-mine-in-arizona-302836579.html)</t>
+          <t>[Mexico Business News](https://mexicobusiness.news/mining/news/endeavour-silver-forecasts-89moz-silver-2026); [Endeavour Silver](https://edrsilver.com/portfolio/development/pitarrilla/)</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
     </row>
@@ -8378,13 +8339,13 @@
   <dimension ref="A1:G101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Monitoreo 2026-09-04: 3 proyectos nuevos + 1 actualización de fase
- Nuevos: Red Dog Mine Life Extension Project (Alaska, Mining), Fleet
  Data Centers Peru Ridge & South Valley Self-Generation Projects
  (Nevada, Data Centers), Cuasar Data Center Campus (Durango, México,
  Data Centers).
- Actualización de fase: Saguaro Energía LNG (más de nueve amparos
  judiciales activos y suspensión de ingreso de buques metaneros al
  Golfo de California).
- proyectos.xlsx regenerado con el acumulado completo en 4 hojas.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014D76wwULT3tWpnkg8hSics
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,15 +29,27 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Arial"/>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+        <bgColor rgb="001F4E78"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -54,8 +66,10 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -426,13 +440,13 @@
   <dimension ref="A1:G55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2484,13 +2498,13 @@
   <dimension ref="A1:G47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2849,17 +2863,17 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Pre-FID PAUSADO (suspensión judicial desde abr-2026 por demanda ambiental sobre ballenas en el Mar de Cortés; presión de activistas contra financiadores JPMorgan/Santander, 17-jul-2026; afiliada de ONEOK solicitó extensión de 3 años del plazo de construcción del Saguaro Connector Pipeline, de feb-2027 a feb-2030, confirmando que la construcción del gasoducto aún no inicia; definición de autorización pendiente para 2026)</t>
+          <t>Pre-FID PAUSADO (suspensión judicial desde abr-2026 por demanda ambiental sobre ballenas en el Mar de Cortés; presión de activistas contra financiadores JPMorgan/Santander, 17-jul-2026; afiliada de ONEOK solicitó extensión de 3 años del plazo de construcción del Saguaro Connector Pipeline, de feb-2027 a feb-2030, confirmando que la construcción del gasoducto aún no inicia; reporte del 1-sep-2026 confirma que más de nueve amparos/suspensiones judiciales distintos mantienen frenado el proyecto, incluyendo una suspensión que impide el ingreso de buques metaneros vinculados al proyecto al Golfo de California; la autorización ambiental original de 2018 —modificada de planta de regasificación a terminal de exportación— sigue sin resolverse en definitiva; litigante activo: Nuestro Futuro A.C.)</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>[Dossier Político](https://dossierpolitico.com/2026/07/17/activistas-entregan-90-mil-firmas-para-frenar-proyecto-saguaro-energia-en-sonora/); [Natural Gas Intel](https://naturalgasintel.com/news/oneok-affiliate-seeks-3-year-extension-for-saguaro-connector-pipeline/)</t>
+          <t>[Dossier Político](https://dossierpolitico.com/2026/07/17/activistas-entregan-90-mil-firmas-para-frenar-proyecto-saguaro-energia-en-sonora/); [Natural Gas Intel](https://naturalgasintel.com/news/oneok-affiliate-seeks-3-year-extension-for-saguaro-connector-pipeline/); [Dossier Político](https://dossierpolitico.com/2026/09/01/suspensiones-judiciales-mantienen-frenados-los-megaproyectos-de-gnl-en-sonora-nuestro-futuro/)</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-09-04</t>
         </is>
       </c>
     </row>
@@ -4243,16 +4257,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G110"/>
+  <dimension ref="A1:G109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6108,17 +6122,17 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>NewRange Copper Nickel (Proyecto NorthMet) — Rediseño Mayor</t>
+          <t>White Mesa Mill — Expansión de Tierras Raras Pesadas</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Babbitt/Hoyt Lakes, Minnesota, EE.UU. (Iron Range)</t>
+          <t>Blanding, Utah, EE.UU.</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>NewRange Copper Nickel (JV PolyMet/Glencore + Teck)</t>
+          <t>Energy Fuels Inc.</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -6128,86 +6142,86 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Permitting (rediseño mayor elimina la represa de jales propuesta —roca estéril se almacenaría en tajos de mineral de hierro existentes—; solicitud de permiso de humedales Sección 404/Clean Water Act presentada ante USACE; revisión ambiental suplementaria (SEIS) solicitada a Minnesota DNR)</t>
+          <t>Construcción (planta comercial de tierras raras pesadas —disprosio/terbio— iniciada 29-jul-2026; capex ~US$104 millones, para uso en imanes/defensa/vehículos eléctricos)</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>[MPR News](https://www.mprnews.org/story/2026/07/30/newrange-copper-nickel-proposes-major-changes-to-copper-mine-plan)</t>
+          <t>[Energy Fuels](https://investors.energyfuels.com/2026-07-29-Commercial-Scale-Heavy-Rare-Earth-Plant-Now-Under-Construction-in-Utah); [PR Newswire](https://www.prnewswire.com/news-releases/commercial-scale-heavy-rare-earth-plant-now-under-construction-in-utah-302837314.html)</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-07-30</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>White Mesa Mill — Expansión de Tierras Raras Pesadas</t>
+          <t>Black Butte Copper Project</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Blanding, Utah, EE.UU.</t>
+          <t>Meagher County, Montana, EE.UU.</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Energy Fuels Inc.</t>
+          <t>Sandfire Resources America Inc. (Sandfire Resources)</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Por definir (PFS elaborado por DM Consulting)</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Construcción (planta comercial de tierras raras pesadas —disprosio/terbio— iniciada 29-jul-2026; capex ~US$104 millones, para uso en imanes/defensa/vehículos eléctricos)</t>
+          <t>Feasibility (PFS actualizado presentado 28-jul-2026 con nuevas reservas Lowry, vida de mina de 12 años; mina subterránea de cobre de alta ley)</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>[Energy Fuels](https://investors.energyfuels.com/2026-07-29-Commercial-Scale-Heavy-Rare-Earth-Plant-Now-Under-Construction-in-Utah); [PR Newswire](https://www.prnewswire.com/news-releases/commercial-scale-heavy-rare-earth-plant-now-under-construction-in-utah-302837314.html)</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/29/3334925/0/en/sandfire-resources-america-files-black-butte-copper-project-preliminary-feasibility-study.html)</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-03</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Black Butte Copper Project</t>
+          <t>Planta de Procesamiento de Litio Red River (US Army)</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Meagher County, Montana, EE.UU.</t>
+          <t>Bowie County, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Sandfire Resources America Inc. (Sandfire Resources)</t>
+          <t>Pentágono / Departamento del Ejército de EE.UU.</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Por definir (PFS elaborado por DM Consulting)</t>
+          <t>EnergyX (desarrollador-operador)</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>Feasibility (PFS actualizado presentado 28-jul-2026 con nuevas reservas Lowry, vida de mina de 12 años; mina subterránea de cobre de alta ley)</t>
+          <t>Acuerdo de arrendamiento condicional otorgado (confirmado 25-jun-2026; 5to sitio del programa de minerales críticos en bases del Ejército, junto con Tooele, Pine Bluff/Anniston; construcción prevista desde 2027)</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/29/3334925/0/en/sandfire-resources-america-files-black-butte-copper-project-preliminary-feasibility-study.html)</t>
+          <t>[Texarkana Gazette](https://www.texarkanagazette.com/news/2026/jun/30/army-awards-lithium-company-energyx-conditional/)</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -6219,54 +6233,54 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Planta de Procesamiento de Litio Red River (US Army)</t>
+          <t>Cerro Caliche Gold Project</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Bowie County, Texas, EE.UU.</t>
+          <t>Sonora, México</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Pentágono / Departamento del Ejército de EE.UU.</t>
+          <t>Sonoro Gold Corp.</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>EnergyX (desarrollador-operador)</t>
+          <t>EPC por definir (en negociación con múltiples empresas EPC de China)</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Acuerdo de arrendamiento condicional otorgado (confirmado 25-jun-2026; 5to sitio del programa de minerales críticos en bases del Ejército, junto con Tooele, Pine Bluff/Anniston; construcción prevista desde 2027)</t>
+          <t>Permisos/estructuración de financiamiento EPC (plataforma consolidada de 3,924 hectáreas en 25 concesiones; finalización de permisos esperada 1T2026; 4 empresas EPC chinas evaluando financiamiento de deuda y desarrollo)</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>[Texarkana Gazette](https://www.texarkanagazette.com/news/2026/jun/30/army-awards-lithium-company-energyx-conditional/)</t>
+          <t>[Sonoro Gold Corp.](https://sonorogold.com/wp-content/uploads/2026/03/2026.03.01_Sonoro-Gold-Corporate-Presentation.pdf); [Mexico Mining Center](https://www.mexicominingcenter.com/sonoro-continues-discussions-with-china-based-epc-companies-and-potential-equity-investors/)</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Camino Rojo — Proyecto Subterráneo (extensión)</t>
+          <t>Pilot Mountain Tungsten Project</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Zacatecas, México</t>
+          <t>Mineral County, Nevada, EE.UU.</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Orla Mining Ltd.</t>
+          <t>Guardian Metal Resources PLC (vía Golden Metal Resources USA LLC)</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
@@ -6276,71 +6290,71 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Permisos completos/inicio de desarrollo subterráneo (SEMARNAT aprobó MIA 18-mar-2026, habilitando minado del resto del tajo de óxidos y construcción de rampa de exploración subterránea; inicio de obras de acceso subterráneo previsto 2S2026; PEA de proyecto subterráneo indica VPN de US$1,300 millones)</t>
+          <t>Ingeniería/Feasibility (PFS positivo completado jun-2026, respaldado por USD 6.2 millones del Departamento de Guerra/DPA Title III; presentación del Mine Plan of Operations federal prevista ago-2026; producción 4T2028)</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>[Mining.com](https://www.mining.com/orla-secures-final-permit-to-advance-underground-mining-at-camino-rojo/); [Orla Mining](https://orlamining.com/news/orla-mining-receives-permits-to-extend-operations-in-mexico-supporting-companys-long-term-commitment-to-camino-rojo/)</t>
+          <t>[Mining Weekly](https://www.miningweekly.com/article/guardian-metals-outlines-viable-tungsten-trioxide-operation-in-nevada-2026-06-30); [StockTitan](https://www.stocktitan.net/news/GMTL/guardian-metal-resources-plc-announces-pilot-mountain-pre-tftnlr9fu3if.html)</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-06</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Cerro Caliche Gold Project</t>
+          <t>Gabbs Project</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Sonora, México</t>
+          <t>Walker-Lane Trend, Nevada, EE.UU.</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Sonoro Gold Corp.</t>
+          <t>P2 Gold Inc.</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>EPC por definir (en negociación con múltiples empresas EPC de China)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Permisos/estructuración de financiamiento EPC (plataforma consolidada de 3,924 hectáreas en 25 concesiones; finalización de permisos esperada 1T2026; 4 empresas EPC chinas evaluando financiamiento de deuda y desarrollo)</t>
+          <t>Ingeniería/Feasibility (proyecto oro-cobre; feasibility study en curso, meta 4T2026)</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>[Sonoro Gold Corp.](https://sonorogold.com/wp-content/uploads/2026/03/2026.03.01_Sonoro-Gold-Corporate-Presentation.pdf); [Mexico Mining Center](https://www.mexicominingcenter.com/sonoro-continues-discussions-with-china-based-epc-companies-and-potential-equity-investors/)</t>
+          <t>[Newswire](https://www.newswire.ca/news-releases/p2-gold-gabbs-project-update-feasibility-study-on-track-840759204.html)</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-06</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Pilot Mountain Tungsten Project</t>
+          <t>Treasure Canyon Gold Mine</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Mineral County, Nevada, EE.UU.</t>
+          <t>Plumas National Forest, cerca de Taylorsville, California, EE.UU.</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Guardian Metal Resources PLC (vía Golden Metal Resources USA LLC)</t>
+          <t>Buscar Company (CGLD)</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
@@ -6350,12 +6364,12 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/Feasibility (PFS positivo completado jun-2026, respaldado por USD 6.2 millones del Departamento de Guerra/DPA Title III; presentación del Mine Plan of Operations federal prevista ago-2026; producción 4T2028)</t>
+          <t>Permitting (Plan de Operaciones sometido a US Forest Service feb-2026; en revisión por agencias federales/estatales)</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>[Mining Weekly](https://www.miningweekly.com/article/guardian-metals-outlines-viable-tungsten-trioxide-operation-in-nevada-2026-06-30); [StockTitan](https://www.stocktitan.net/news/GMTL/guardian-metal-resources-plc-announces-pilot-mountain-pre-tftnlr9fu3if.html)</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/buscar-company-announces-major-advancement-in-the-permitting-process-for-the-treasure-canyon-gold-mine-project-in-california-302772744.html)</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -6367,17 +6381,17 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Gabbs Project</t>
+          <t>Grassy Mountain Gold Project</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Walker-Lane Trend, Nevada, EE.UU.</t>
+          <t>Malheur County, Oregon, EE.UU.</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>P2 Gold Inc.</t>
+          <t>Paramount Gold Nevada Corp. (vía Calico Resources)</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
@@ -6387,12 +6401,12 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/Feasibility (proyecto oro-cobre; feasibility study en curso, meta 4T2026)</t>
+          <t>Permitting (Record of Decision federal firmado 29-ene-2026 bajo NEPA; permisos estatales pendientes, esperados 2S2026; Feasibility Study ya completo con VPN de USD 375 millones)</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>[Newswire](https://www.newswire.ca/news-releases/p2-gold-gabbs-project-update-feasibility-study-on-track-840759204.html)</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/01/29/3229150/0/en/Paramount-Gold-Receives-Federal-Approval-for-the-Grassy-Mountain-Gold-Project.html); [OPB](https://www.opb.org/article/2026/01/29/oregon-gold-mine-grassy-mountain/)</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -6404,17 +6418,17 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Treasure Canyon Gold Mine</t>
+          <t>MP Materials 10X Magnet Manufacturing Facility</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Plumas National Forest, cerca de Taylorsville, California, EE.UU.</t>
+          <t>Northlake, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Buscar Company (CGLD)</t>
+          <t>MP Materials</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -6424,12 +6438,12 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Permitting (Plan de Operaciones sometido a US Forest Service feb-2026; en revisión por agencias federales/estatales)</t>
+          <t>Construcción (rompimiento de tierra 1T2026; planta de imanes de tierras raras de USD 1,250 millones; ~7,000 t/año de capacidad adicional)</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/buscar-company-announces-major-advancement-in-the-permitting-process-for-the-treasure-canyon-gold-mine-project-in-california-302772744.html)</t>
+          <t>[CNBC](https://www.cnbc.com/2026/02/26/mp-materials-selects-texas-for-rare-earth-magnet-manufacturing-site.html)</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -6441,17 +6455,17 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Grassy Mountain Gold Project</t>
+          <t>Expansión de Separación de Tierras Raras Pesadas — Mountain Pass</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Malheur County, Oregon, EE.UU.</t>
+          <t>Mountain Pass, California, EE.UU.</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Paramount Gold Nevada Corp. (vía Calico Resources)</t>
+          <t>MP Materials</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
@@ -6461,12 +6475,12 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Permitting (Record of Decision federal firmado 29-ene-2026 bajo NEPA; permisos estatales pendientes, esperados 2S2026; Feasibility Study ya completo con VPN de USD 375 millones)</t>
+          <t>Ingeniería/Construcción temprana (financiamiento de USD 550 millones del Departamento de Defensa, feb-2026, para agregar capacidad de separación de tierras raras pesadas en la mina/planta existente)</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/01/29/3229150/0/en/Paramount-Gold-Receives-Federal-Approval-for-the-Grassy-Mountain-Gold-Project.html); [OPB](https://www.opb.org/article/2026/01/29/oregon-gold-mine-grassy-mountain/)</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/the-united-states-is-investing-in-its-domestic-rare-earth-industry-302838375.html)</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -6478,17 +6492,17 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>MP Materials 10X Magnet Manufacturing Facility</t>
+          <t>Planta de Procesamiento de Antimonio (JV Galena Complex)</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Northlake, Texas, EE.UU.</t>
+          <t>Silver Valley, Wallace, Idaho, EE.UU.</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>MP Materials</t>
+          <t>JV Americas Gold and Silver Corporation (51%) / United States Antimony Corp (49%)</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
@@ -6498,12 +6512,12 @@
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>Construcción (rompimiento de tierra 1T2026; planta de imanes de tierras raras de USD 1,250 millones; ~7,000 t/año de capacidad adicional)</t>
+          <t>Ingeniería/Construcción (JV firmado feb-2026 para construir y operar planta de procesamiento de antimonio dentro de los permisos existentes del Galena Complex)</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>[CNBC](https://www.cnbc.com/2026/02/26/mp-materials-selects-texas-for-rare-earth-magnet-manufacturing-site.html)</t>
+          <t>[Newsfile Corp](https://www.newsfilecorp.com/release/283399/Americas-Gold-and-Silver-Signs-Joint-Venture-Agreement-with-US-Antimony-to-Construct-Antimony-Processing-Facility-in-Idahos-Silver-Valley-Unlocking-Value-from-Its-Antimony-Production-and-Strengthening-U.S.-Critical-Mineral-Security)</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -6515,17 +6529,17 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Expansión de Separación de Tierras Raras Pesadas — Mountain Pass</t>
+          <t>Michigan Potash Project</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Mountain Pass, California, EE.UU.</t>
+          <t>Osceola County, Michigan, EE.UU.</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>MP Materials</t>
+          <t>Michigan Potash &amp; Salt Co.</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -6535,12 +6549,12 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/Construcción temprana (financiamiento de USD 550 millones del Departamento de Defensa, feb-2026, para agregar capacidad de separación de tierras raras pesadas en la mina/planta existente)</t>
+          <t>Financiamiento/pre-construcción (mina de solución de potasa + planta de proceso; garantía de préstamo condicional DOE de USD 1,260 millones; posible aprobación FAST-41 en 2026; ~726,000 t/año)</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/the-united-states-is-investing-in-its-domestic-rare-earth-industry-302838375.html)</t>
+          <t>[DOE-LPO](https://www.energy.gov/lpo/articles/lpo-announces-conditional-commitment-michigan-potash-produce-fertilizer-us-farmers); [Northern Miner](https://www.northernminer.com/news/us-boosts-potash-projects-in-utah-michigan/1003886533/)</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -6552,17 +6566,17 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>Planta de Procesamiento de Antimonio (JV Galena Complex)</t>
+          <t>Sevier Playa Potash Project</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Silver Valley, Wallace, Idaho, EE.UU.</t>
+          <t>Millard County, Utah, EE.UU.</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>JV Americas Gold and Silver Corporation (51%) / United States Antimony Corp (49%)</t>
+          <t>Peak Minerals (respaldado por EMR Capital)</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
@@ -6572,12 +6586,12 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/Construcción (JV firmado feb-2026 para construir y operar planta de procesamiento de antimonio dentro de los permisos existentes del Galena Complex)</t>
+          <t>Construcción (BLM aprobó construcción de la etapa inicial de 195,000 t en jun-2026; capex total USD 435 millones; subvención USDA de USD 80 millones)</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>[Newsfile Corp](https://www.newsfilecorp.com/release/283399/Americas-Gold-and-Silver-Signs-Joint-Venture-Agreement-with-US-Antimony-to-Construct-Antimony-Processing-Facility-in-Idahos-Silver-Valley-Unlocking-Value-from-Its-Antimony-Production-and-Strengthening-U.S.-Critical-Mineral-Security)</t>
+          <t>[BLM](https://www.blm.gov/announcement/blm-approves-construction-sevier-playa-potash-mining-project)</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -6589,17 +6603,17 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Michigan Potash Project</t>
+          <t>Shirley Basin Uranium Project</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Osceola County, Michigan, EE.UU.</t>
+          <t>Wyoming, EE.UU.</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Michigan Potash &amp; Salt Co.</t>
+          <t>Ur-Energy Inc.</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
@@ -6609,34 +6623,34 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Financiamiento/pre-construcción (mina de solución de potasa + planta de proceso; garantía de préstamo condicional DOE de USD 1,260 millones; posible aprobación FAST-41 en 2026; ~726,000 t/año)</t>
+          <t>Producción (autorización final del estado de Wyoming para operar a plena producción, reportada 10-ago-2026; Ur-Energy realizó su PRIMER EMBARQUE de uranio desde la mina hacia la planta de procesamiento Lost Creek, 19-ago-2026 —transición de construcción a producción en 2.5 años—; planta satélite ISR integrada con Lost Creek)</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>[DOE-LPO](https://www.energy.gov/lpo/articles/lpo-announces-conditional-commitment-michigan-potash-produce-fertilizer-us-farmers); [Northern Miner](https://www.northernminer.com/news/us-boosts-potash-projects-in-utah-michigan/1003886533/)</t>
+          <t>[Ur-Energy](https://www.ur-energy.com/news-media/press-releases/detail/410/ur-energy-announces-first-shipment-of-uranium-from-shirley); [Junior Mining Network](https://www.juniorminingnetwork.com/junior-miner-news/press-releases/557-tsx/ure/208831-ur-energy-reports-second-quarter-2026-results.html)</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>Sevier Playa Potash Project</t>
+          <t>Cusi Mine (Reinicio)</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Millard County, Utah, EE.UU.</t>
+          <t>Chihuahua, México</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Peak Minerals (respaldado por EMR Capital)</t>
+          <t>Silverco Mining Ltd.</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
@@ -6646,12 +6660,12 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>Construcción (BLM aprobó construcción de la etapa inicial de 195,000 t en jun-2026; capex total USD 435 millones; subvención USDA de USD 80 millones)</t>
+          <t>Construcción (reinicio 68% completo; rehabilitación de la planta Mal Paso; primer concentrado previsto 4T2026)</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>[BLM](https://www.blm.gov/announcement/blm-approves-construction-sevier-playa-potash-mining-project)</t>
+          <t>[Mexico Business News](https://mexicobusiness.news/mining/news/silverco-targets-late-2026-restart-past-producing-cusi-mine); [Investing News Network](https://investingnews.com/silverco-mining-begins-underground-development-at-cusi-restart-remains-on-budget-and-on-schedule/)</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -6663,17 +6677,17 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Shirley Basin Uranium Project</t>
+          <t>Kilbourne Graphite Project</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Wyoming, EE.UU.</t>
+          <t>Nueva York, EE.UU.</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Ur-Energy Inc.</t>
+          <t>Titan Mining Corporation</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -6683,34 +6697,34 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Producción (autorización final del estado de Wyoming para operar a plena producción, reportada 10-ago-2026; Ur-Energy realizó su PRIMER EMBARQUE de uranio desde la mina hacia la planta de procesamiento Lost Creek, 19-ago-2026 —transición de construcción a producción en 2.5 años—; planta satélite ISR integrada con Lost Creek)</t>
+          <t>Ingeniería/Feasibility (planta demostrativa ya en producción/calificación de clientes 2026; decisión de construcción esperada fines de 2026/2027; proyecto integrado de 40,000 tpa) ; subsidiaria Empire State Mines recibió Conditional Selection Notice del US Army para diseñar, financiar, construir y operar la planta de purificación de grafito; decisión de construcción esperada a fines de 2026 o inicios de 2027</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>[Ur-Energy](https://www.ur-energy.com/news-media/press-releases/detail/410/ur-energy-announces-first-shipment-of-uranium-from-shirley); [Junior Mining Network](https://www.juniorminingnetwork.com/junior-miner-news/press-releases/557-tsx/ure/208831-ur-energy-reports-second-quarter-2026-results.html)</t>
+          <t>[Junior Mining Network](https://www.juniorminingnetwork.com/junior-miner-news/press-releases/2342-tsx/ti/199070-titan-mining-to-start-shipping-first-graphite-product-and-feasibility-study-underway-for-40-000-tpa-integrated-kilbourne-graphite-project.html) ; [Titan Mining Corp](https://www.titanminingcorp.com/news/news-releases/titan-mining-selected-by-the-us-army-to-establish-first-ever-public-private-partnership-for-domestic-critical-minerals-processing-on-strategic-defense-installations)</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>Cusi Mine (Reinicio)</t>
+          <t>Graphite Creek Project</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>Chihuahua, México</t>
+          <t>Alaska, EE.UU.</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>Silverco Mining Ltd.</t>
+          <t>Graphite One Inc.</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
@@ -6720,12 +6734,12 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Construcción (reinicio 68% completo; rehabilitación de la planta Mal Paso; primer concentrado previsto 4T2026)</t>
+          <t>Permitting (permitting federal en curso bajo programa FAST-41, finalización prevista 29-sep-2026)</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>[Mexico Business News](https://mexicobusiness.news/mining/news/silverco-targets-late-2026-restart-past-producing-cusi-mine); [Investing News Network](https://investingnews.com/silverco-mining-begins-underground-development-at-cusi-restart-remains-on-budget-and-on-schedule/)</t>
+          <t>[Permitting Council](https://www.permitting.gov/newsroom/success-stories/project-spotlight-graphite-creek-project)</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -6737,17 +6751,17 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Kilbourne Graphite Project</t>
+          <t>La Colorada Skarn Project</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Nueva York, EE.UU.</t>
+          <t>Zacatecas, México</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Titan Mining Corporation</t>
+          <t>Pan American Silver Corp.</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
@@ -6757,123 +6771,123 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/Feasibility (planta demostrativa ya en producción/calificación de clientes 2026; decisión de construcción esperada fines de 2026/2027; proyecto integrado de 40,000 tpa) ; subsidiaria Empire State Mines recibió Conditional Selection Notice del US Army para diseñar, financiar, construir y operar la planta de purificación de grafito; decisión de construcción esperada a fines de 2026 o inicios de 2027</t>
+          <t>Ingeniería/Feasibility (PEA revisada publicada mar-2026 para nueva planta de flotación selectiva de 15,000 t/d en área Candelaria oriente; gasto de capital 2026 estimado USD 92-95 millones, incluye "588 Decline Project" de 12.4 km de rampa; producción media proyectada de 19.1 Moz Ag/año en años pico)</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>[Junior Mining Network](https://www.juniorminingnetwork.com/junior-miner-news/press-releases/2342-tsx/ti/199070-titan-mining-to-start-shipping-first-graphite-product-and-feasibility-study-underway-for-40-000-tpa-integrated-kilbourne-graphite-project.html) ; [Titan Mining Corp](https://www.titanminingcorp.com/news/news-releases/titan-mining-selected-by-the-us-army-to-establish-first-ever-public-private-partnership-for-domestic-critical-minerals-processing-on-strategic-defense-installations)</t>
+          <t>[Pan American Silver](https://panamericansilver.com/news/pan-american-announces-revised-pea-for-the-la-colorada-skarn-project-positions-la-colorada-as-a-future-top-tier-silver-mine/); [SEC 6-K](https://www.sec.gov/Archives/edgar/data/771992/000077199226000031/a2026_03x24lacoloradapeaup.htm)</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-06</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>Graphite Creek Project</t>
+          <t>Lone Tree Plant (Refurbishment Autoclave/CIL)</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>Alaska, EE.UU.</t>
+          <t>Lovelock, Nevada, EE.UU.</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Graphite One Inc.</t>
+          <t>i-80 Gold Corp</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Hatch (EPCM)</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Permitting (permitting federal en curso bajo programa FAST-41, finalización prevista 29-sep-2026)</t>
+          <t>Construcción (obras tempranas y movilización de contratistas en curso; construcción mayor prevista 4T2026)</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>[Permitting Council](https://www.permitting.gov/newsroom/success-stories/project-spotlight-graphite-creek-project)</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/i-80-gold-provides-update-on-lone-tree-plant-refurbishment-project-remains-on-schedule-and-on-budget-302836341.html)</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>La Colorada Skarn Project</t>
+          <t>Round Mountain Phase X — Planta de Paste Backfill</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Zacatecas, México</t>
+          <t>Nye County, Nevada, EE.UU.</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Pan American Silver Corp.</t>
+          <t>Kinross Gold Corporation</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>No especificado (paquetes de equipo móvil, ventiladores y planta CRF ya adjudicados)</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/Feasibility (PEA revisada publicada mar-2026 para nueva planta de flotación selectiva de 15,000 t/d en área Candelaria oriente; gasto de capital 2026 estimado USD 92-95 millones, incluye "588 Decline Project" de 12.4 km de rampa; producción media proyectada de 19.1 Moz Ag/año en años pico)</t>
+          <t>Construcción/Ingeniería detallada</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>[Pan American Silver](https://panamericansilver.com/news/pan-american-announces-revised-pea-for-the-la-colorada-skarn-project-positions-la-colorada-as-a-future-top-tier-silver-mine/); [SEC 6-K](https://www.sec.gov/Archives/edgar/data/771992/000077199226000031/a2026_03x24lacoloradapeaup.htm)</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/29/3335652/0/en/Kinross-reports-strong-2026-second-quarter-results.html)</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>Lone Tree Plant (Refurbishment Autoclave/CIL)</t>
+          <t>Bald Mountain Redbird 2 — Planta SART (ácido/lixiviación)</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>Lovelock, Nevada, EE.UU.</t>
+          <t>White Pine County, Nevada, EE.UU.</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>i-80 Gold Corp</t>
+          <t>Kinross Gold Corporation</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Hatch (EPCM)</t>
+          <t>Contratista de ingeniería detallada ya seleccionado, no revelado en la fuente</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>Construcción (obras tempranas y movilización de contratistas en curso; construcción mayor prevista 4T2026)</t>
+          <t>Ingeniería (básica ~50% completa)</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/i-80-gold-provides-update-on-lone-tree-plant-refurbishment-project-remains-on-schedule-and-on-budget-302836341.html)</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/29/3335652/0/en/Kinross-reports-strong-2026-second-quarter-results.html)</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -6885,32 +6899,32 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Round Mountain Phase X — Planta de Paste Backfill</t>
+          <t>Bear Lodge Rare Earth Project</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Nye County, Nevada, EE.UU.</t>
+          <t>Crook County, Wyoming, EE.UU.</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Kinross Gold Corporation</t>
+          <t>Rare Element Resources Ltd. (afiliada de General Atomics/Synchron)</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>No especificado (paquetes de equipo móvil, ventiladores y planta CRF ya adjudicados)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Construcción/Ingeniería detallada</t>
+          <t>Permitting (designación FAST-41; aviso NEPA publicado en Federal Register 29-jul-2026)</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/29/3335652/0/en/Kinross-reports-strong-2026-second-quarter-results.html)</t>
+          <t>[Federal Register](https://www.federalregister.gov/documents/2026/07/29/2026-15255/black-hills-national-forest-wyoming-bear-lodge-rare-earth-project)</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -6922,32 +6936,32 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>Bald Mountain Redbird 2 — Planta SART (ácido/lixiviación)</t>
+          <t>Modernización Complejo Metalúrgico Empalme</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>White Pine County, Nevada, EE.UU.</t>
+          <t>Empalme, Sonora, México</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>Kinross Gold Corporation</t>
+          <t>Southern Copper Corporation (Grupo México)</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>Contratista de ingeniería detallada ya seleccionado, no revelado en la fuente</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería (básica ~50% completa)</t>
+          <t>Pre-desarrollo (en negociación de permisos; fundición existente a modernizar)</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/29/3335652/0/en/Kinross-reports-strong-2026-second-quarter-results.html)</t>
+          <t>[Minería en Línea](https://mineriaenlinea.com/2026/07/southern-copper-obtiene-permisos-ambientales-para-el-pilar-produccion-a-partir-de-2029/)</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -6959,17 +6973,17 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>Bear Lodge Rare Earth Project</t>
+          <t>Coosa Graphite Project (Kellyton Graphite Plant)</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>Crook County, Wyoming, EE.UU.</t>
+          <t>Condado de Coosa, Alabama, EE.UU.</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>Rare Element Resources Ltd. (afiliada de General Atomics/Synchron)</t>
+          <t>Westwater Resources Inc.</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
@@ -6979,34 +6993,34 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Permitting (designación FAST-41; aviso NEPA publicado en Federal Register 29-jul-2026)</t>
+          <t>Financiamiento/planeación (préstamo EXIM Bank de US$25 millones anunciado 7-ago-2026 para mina de grafito natural y planta de procesamiento, primera fuente de grafito natural producida en EE.UU.)</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>[Federal Register](https://www.federalregister.gov/documents/2026/07/29/2026-15255/black-hills-national-forest-wyoming-bear-lodge-rare-earth-project)</t>
+          <t>[Yellowhammer News](https://yellowhammernews.com/trump-administration-announces-25-million-exim-loan-for-westwaters-coosa-county-graphite-plant/); [EXIM.GOV](https://www.exim.gov/news/trump-administration-announces-58m-major-new-critical-mineral-deals-white-house-roundtable)</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>Modernización Complejo Metalúrgico Empalme</t>
+          <t>Expansión de Procesamiento de Tantalio/Niobio (Global Advanced Metals)</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>Empalme, Sonora, México</t>
+          <t>Pensilvania, EE.UU.</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>Southern Copper Corporation (Grupo México)</t>
+          <t>Global Advanced Metals</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
@@ -7016,34 +7030,34 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Pre-desarrollo (en negociación de permisos; fundición existente a modernizar)</t>
+          <t>Financiamiento/planeación (préstamo EXIM Bank de US$25 millones anunciado 7-ago-2026 para ampliar capacidad de procesamiento)</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>[Minería en Línea](https://mineriaenlinea.com/2026/07/southern-copper-obtiene-permisos-ambientales-para-el-pilar-produccion-a-partir-de-2029/)</t>
+          <t>[EXIM.GOV](https://www.exim.gov/news/trump-administration-announces-58m-major-new-critical-mineral-deals-white-house-roundtable); [SME](https://me.smenet.org/trump-administration-to-back-three-mineral-projects-with-58-million-in-financing/)</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Coosa Graphite Project (Kellyton Graphite Plant)</t>
+          <t>Boron Americas Project (Fort Cady)</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>Condado de Coosa, Alabama, EE.UU.</t>
+          <t>California, EE.UU.</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Westwater Resources Inc.</t>
+          <t>5E Advanced Materials</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
@@ -7053,12 +7067,12 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Financiamiento/planeación (préstamo EXIM Bank de US$25 millones anunciado 7-ago-2026 para mina de grafito natural y planta de procesamiento, primera fuente de grafito natural producida en EE.UU.)</t>
+          <t>Financiamiento/planeación (préstamo EXIM Bank de US$8 millones anunciado 7-ago-2026 para proyecto de boro, lixiviación/procesamiento)</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>[Yellowhammer News](https://yellowhammernews.com/trump-administration-announces-25-million-exim-loan-for-westwaters-coosa-county-graphite-plant/); [EXIM.GOV](https://www.exim.gov/news/trump-administration-announces-58m-major-new-critical-mineral-deals-white-house-roundtable)</t>
+          <t>[EXIM.GOV](https://www.exim.gov/news/trump-administration-announces-58m-major-new-critical-mineral-deals-white-house-roundtable)</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -7070,54 +7084,54 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>Expansión de Procesamiento de Tantalio/Niobio (Global Advanced Metals)</t>
+          <t>Brook Mine (tierras raras/minerales críticos de carbón)</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>Pensilvania, EE.UU.</t>
+          <t>Ranchester/Sheridan, Wyoming, EE.UU.</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>Global Advanced Metals</t>
+          <t>Ramaco Resources</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Hatch Associates Consultants (ingeniería/estudio)</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Financiamiento/planeación (préstamo EXIM Bank de US$25 millones anunciado 7-ago-2026 para ampliar capacidad de procesamiento)</t>
+          <t>Ingeniería/Construcción de planta piloto (Hatch publicó Initial Assessment Report jul-2026 con capex preliminar ~US$3,200 millones + US$800 millones de contingencia, VPN interno ~US$8,000 millones; planta piloto en construcción desde oct-2025; primer procesamiento de concentrados de óxido de tierras raras para la Defense Logistics Agency, ago-2026; construcción de planta comercial podría iniciar fines de 2026, producción comercial 2028)</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>[EXIM.GOV](https://www.exim.gov/news/trump-administration-announces-58m-major-new-critical-mineral-deals-white-house-roundtable); [SME](https://me.smenet.org/trump-administration-to-back-three-mineral-projects-with-58-million-in-financing/)</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/ramaco-resources-releases-hatch-report-and-shareholder-letter-on-exploratory-brook-mine-critical-minerals-project-302838319.html); [Mining.com](https://www.mining.com/ramaco-eyes-ree-stockpile-at-wyoming-mine/)</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>Boron Americas Project (Fort Cady)</t>
+          <t>Dewey-Burdock Uranium ISR Project</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>California, EE.UU.</t>
+          <t>Fall River/Custer Counties, Dakota del Sur, EE.UU.</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>5E Advanced Materials</t>
+          <t>enCore Energy (Powertech USA)</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
@@ -7127,71 +7141,71 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Financiamiento/planeación (préstamo EXIM Bank de US$8 millones anunciado 7-ago-2026 para proyecto de boro, lixiviación/procesamiento)</t>
+          <t>Construcción autorizada/permitting (BLM autorizó inicio de construcción de infraestructura —caminos, pozos de monitoreo, líneas eléctricas— jun-2026; NRC renovó la licencia, publicado en Federal Register 7-ago-2026; pendiente permiso estatal de Dakota del Sur, proceso reiniciado tras 13 años de pausa)</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>[EXIM.GOV](https://www.exim.gov/news/trump-administration-announces-58m-major-new-critical-mineral-deals-white-house-roundtable)</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/encore-energy-receives-bureau-of-land-management-authorization-to-begin-construction-at-dewey-burdock-uranium-project-302804230.html); [Federal Register](https://www.federalregister.gov/documents/2026/08/07/2026-16132/powertech-usa-inc-dewey-burdock-uranium-in-situ-recovery-project-license-renewal)</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>Brook Mine (tierras raras/minerales críticos de carbón)</t>
+          <t>Niron Magnetics — Planta de Imanes Permanentes sin Tierras Raras</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>Ranchester/Sheridan, Wyoming, EE.UU.</t>
+          <t>Minnesota, EE.UU. (ubicación exacta no especificada)</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>Ramaco Resources</t>
+          <t>Niron Magnetics</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>Hatch Associates Consultants (ingeniería/estudio)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/Construcción de planta piloto (Hatch publicó Initial Assessment Report jul-2026 con capex preliminar ~US$3,200 millones + US$800 millones de contingencia, VPN interno ~US$8,000 millones; planta piloto en construcción desde oct-2025; primer procesamiento de concentrados de óxido de tierras raras para la Defense Logistics Agency, ago-2026; construcción de planta comercial podría iniciar fines de 2026, producción comercial 2028)</t>
+          <t>Financiamiento asegurado (US$150 millones del Departamento de Defensa/Office of Strategic Capital, anunciado 7-8-ago-2026, parte de paquete federal de US$3,000 millones en minerales críticos)</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/ramaco-resources-releases-hatch-report-and-shareholder-letter-on-exploratory-brook-mine-critical-minerals-project-302838319.html); [Mining.com](https://www.mining.com/ramaco-eyes-ree-stockpile-at-wyoming-mine/)</t>
+          <t>[MINING.COM](https://www.mining.com/web/trump-says-us-is-announcing-a-series-of-mining-projects-worth-3-billion/); [CNBC](https://www.cnbc.com/2026/08/08/trump-admin-to-invest-3-billion-in-defense-linked-minerals-projects.html)</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>Dewey-Burdock Uranium ISR Project</t>
+          <t>Louisiana Strategic Metals Complex</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>Fall River/Custer Counties, Dakota del Sur, EE.UU.</t>
+          <t>Alexandria, Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>enCore Energy (Powertech USA)</t>
+          <t>Ucore Rare Metals Inc.</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
@@ -7201,34 +7215,34 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Construcción autorizada/permitting (BLM autorizó inicio de construcción de infraestructura —caminos, pozos de monitoreo, líneas eléctricas— jun-2026; NRC renovó la licencia, publicado en Federal Register 7-ago-2026; pendiente permiso estatal de Dakota del Sur, proceso reiniciado tras 13 años de pausa)</t>
+          <t>Construcción (planta de procesamiento de tierras raras medianas/pesadas —terbio/disprosio—)</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/encore-energy-receives-bureau-of-land-management-authorization-to-begin-construction-at-dewey-burdock-uranium-project-302804230.html); [Federal Register](https://www.federalregister.gov/documents/2026/08/07/2026-16132/powertech-usa-inc-dewey-burdock-uranium-in-situ-recovery-project-license-renewal)</t>
+          <t>[Ucore Rare Metals](https://ucore.com/ucore-readies-for-louisiana-2026-heavy-rare-earth-element-processing/)</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>Niron Magnetics — Planta de Imanes Permanentes sin Tierras Raras</t>
+          <t>Distrito Copper Creek / San Manuel</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>Minnesota, EE.UU. (ubicación exacta no especificada)</t>
+          <t>Condado de Pinal, Arizona, EE.UU.</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>Niron Magnetics</t>
+          <t>Faraday Copper Corp. (adquiriendo la propiedad San Manuel de BHP; BHP recibirá ~30% de acciones de Faraday)</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
@@ -7238,71 +7252,71 @@
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>Financiamiento asegurado (US$150 millones del Departamento de Defensa/Office of Strategic Capital, anunciado 7-8-ago-2026, parte de paquete federal de US$3,000 millones en minerales críticos)</t>
+          <t>Exploración/definición de recursos (Faraday firmó acuerdo definitivo para comprar la antigua mina San Manuel de BHP —subterránea y de tajo/ISL, operada 1955-1999— y combinarla con su proyecto adyacente Copper Creek, creando un distrito de &gt;18,000 millones de libras de cobre; asamblea de accionistas 25-ago-2026 para aprobar la transacción, cierre esperado 3T2026; plan de 23,000+ metros de perforación de confirmación desde 4T2026, recurso combinado a mediados de 2027)</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>[MINING.COM](https://www.mining.com/web/trump-says-us-is-announcing-a-series-of-mining-projects-worth-3-billion/); [CNBC](https://www.cnbc.com/2026/08/08/trump-admin-to-invest-3-billion-in-defense-linked-minerals-projects.html)</t>
+          <t>[MINING.COM](https://www.mining.com/faraday-targets-18b-lb-arizona-copper-district/)</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-19</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Louisiana Strategic Metals Complex</t>
+          <t>IMA Mine</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>Alexandria, Luisiana, EE.UU.</t>
+          <t>Condado de Lemhi, Idaho, EE.UU.</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>Ucore Rare Metals Inc.</t>
+          <t>American Tungsten Corp.</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>No especificado (geotécnica de presas de jales: NewFields MTDs)</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Construcción (planta de procesamiento de tierras raras medianas/pesadas —terbio/disprosio—)</t>
+          <t>Reactivación/pruebas metalúrgicas (mina histórica de tungsteno, produjo WO3 1945-1957; Fase I: reprocesamiento de jales superficiales; Fase II: rehabilitación de mina subterránea; pruebas metalúrgicas iniciadas jul-2026; definición de recursos, permisos y pruebas previstas concluir 4T2026, construcción fin de 2026/1T2027, primera venta de concentrado prevista inicios de 2027)</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>[Ucore Rare Metals](https://ucore.com/ucore-readies-for-louisiana-2026-heavy-rare-earth-element-processing/)</t>
+          <t>[MINING.COM](https://www.mining.com/american-tungsten-kinks-off-construction-at-ima-project-in-idaho/)</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-19</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>Distrito Copper Creek / San Manuel</t>
+          <t>Railroad Valley Minerals / Super-Brine Complex</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>Condado de Pinal, Arizona, EE.UU.</t>
+          <t>Railroad Valley, Nevada, EE.UU.</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>Faraday Copper Corp. (adquiriendo la propiedad San Manuel de BHP; BHP recibirá ~30% de acciones de Faraday)</t>
+          <t>3 Proton Lithium (3PL Operating Inc.)</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
@@ -7312,12 +7326,12 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Exploración/definición de recursos (Faraday firmó acuerdo definitivo para comprar la antigua mina San Manuel de BHP —subterránea y de tajo/ISL, operada 1955-1999— y combinarla con su proyecto adyacente Copper Creek, creando un distrito de &gt;18,000 millones de libras de cobre; asamblea de accionistas 25-ago-2026 para aprobar la transacción, cierre esperado 3T2026; plan de 23,000+ metros de perforación de confirmación desde 4T2026, recurso combinado a mediados de 2027)</t>
+          <t>Exploración avanzada (depósito multi-mineral confirmado: litio, potasa, boro y lo que la empresa describe como el mayor depósito de tungsteno de EE.UU. —~1.78 millones de toneladas, valorado en ~US$152,000 millones in-situ—; ~17 millas cuadradas del área están retiradas de minería desde 2023 por solicitud de la NASA para calibración de satélites, lo que representa un obstáculo regulatorio; sin decisión de construcción)</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>[MINING.COM](https://www.mining.com/faraday-targets-18b-lb-arizona-copper-district/)</t>
+          <t>[MINING.COM](https://www.mining.com/largest-us-tungsten-discovery-hits-nasa-roadblock/)</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -7329,32 +7343,32 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>IMA Mine</t>
+          <t>New Amalga Gold Project</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>Condado de Lemhi, Idaho, EE.UU.</t>
+          <t>~25 km al norte de Juneau, Alaska, EE.UU.</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>American Tungsten Corp.</t>
+          <t>Grande Portage Resources Ltd.</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>No especificado (geotécnica de presas de jales: NewFields MTDs)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Reactivación/pruebas metalúrgicas (mina histórica de tungsteno, produjo WO3 1945-1957; Fase I: reprocesamiento de jales superficiales; Fase II: rehabilitación de mina subterránea; pruebas metalúrgicas iniciadas jul-2026; definición de recursos, permisos y pruebas previstas concluir 4T2026, construcción fin de 2026/1T2027, primera venta de concentrado prevista inicios de 2027)</t>
+          <t>Permitting temprano (recurso Indicado de 1.44 millones oz Au a 9.47 g/t e Inferido de 515,700 oz Au; obtuvo estatus de "Covered Project" bajo FAST-41 el 30-jul-2026, acelerando la revisión federal coordinada; quinta mina en Alaska con cobertura FAST-41, junto con Arctic, Johnson Tract, Donlin Gold y Graphite Creek)</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>[MINING.COM](https://www.mining.com/american-tungsten-kinks-off-construction-at-ima-project-in-idaho/)</t>
+          <t>[Mining News North](https://www.miningnewsnorth.com/story/2026/08/07/news/new-amalga-gold-project-enters-fast-41/9803.html)</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -7366,17 +7380,17 @@
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>Railroad Valley Minerals / Super-Brine Complex</t>
+          <t>ElementUSA Gramercy — Planta de Tierras Raras/Minerales Críticos</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>Railroad Valley, Nevada, EE.UU.</t>
+          <t>Gramercy, St. John the Baptist Parish, Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>3 Proton Lithium (3PL Operating Inc.)</t>
+          <t>ElementUSA Inc. (en colaboración con Colorado School of Mines)</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
@@ -7386,71 +7400,71 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Exploración avanzada (depósito multi-mineral confirmado: litio, potasa, boro y lo que la empresa describe como el mayor depósito de tungsteno de EE.UU. —~1.78 millones de toneladas, valorado en ~US$152,000 millones in-situ—; ~17 millas cuadradas del área están retiradas de minería desde 2023 por solicitud de la NASA para calibración de satélites, lo que representa un obstáculo regulatorio; sin decisión de construcción)</t>
+          <t>Ingeniería/financiamiento asegurado (proyecto de US$850 millones para procesar "lodo rojo"/bauxite residue del antiguo refinerio de alúmina Atalco —~34 millones de toneladas almacenadas— y extraer galio, escandio, disprosio, gadolinio, iterbio, germanio e itrio; recibió US$67 millones del DOE y US$29.9 millones del DoD; construcción de planta de demostración prevista a iniciar mediados de 2027, producción inicial 3T2028); Atalco (refinería de alúmina que aloja el sitio, entidad distinta co-ubicada) recibió 28-ago-2026 una inversión de capital adicional de US$100 millones del Departamento de Guerra de EE.UU. —participación total del DoW ahora US$400M, US$800M contando coinversión privada desde ene-2026— para restaurar la refinería, única refinería de alúmina activa en EE.UU., a su capacidad nominal de 1.2 millones ton/año, lo que apoya indirectamente la operación de ElementUSA en el mismo sitio</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>[MINING.COM](https://www.mining.com/largest-us-tungsten-discovery-hits-nasa-roadblock/)</t>
+          <t>[Biz New Orleans](https://bizneworleans.com/elementusa-plans-850m-critical-minerals-refining-facility/); [Colorado School of Mines](https://www.minesnewsroom.com/news/colorado-school-mines-and-elementusa-awarded-67m-doe-construction-rare-earth-processing-plant); [Departamento de Guerra de EE.UU.](https://www.war.gov/News/Releases/Release/Article/4585310/department-of-war-announces-a-100-million-follow-on-equity-investment-in-atalco/)</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-09-02</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>New Amalga Gold Project</t>
+          <t>Planta de Refinación de Tierras Raras y Minerales Críticos Marion (ReElement Technologies)</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>~25 km al norte de Juneau, Alaska, EE.UU.</t>
+          <t>Marion, Indiana, EE.UU.</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>Grande Portage Resources Ltd.</t>
+          <t>American Resources Corporation (NASDAQ: AREC) vía subsidiaria ReElement Technologies</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>No especificado (acondicionamiento interno de la ex planta RCA Thomson, 425,000 pies² en campus de 42 acres)</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Permitting temprano (recurso Indicado de 1.44 millones oz Au a 9.47 g/t e Inferido de 515,700 oz Au; obtuvo estatus de "Covered Project" bajo FAST-41 el 30-jul-2026, acelerando la revisión federal coordinada; quinta mina en Alaska con cobertura FAST-41, junto con Arctic, Johnson Tract, Donlin Gold y Graphite Creek)</t>
+          <t>Permiso de aire obtenido/comisionamiento (IDEM —Indiana— otorgó el permiso "Minor Source" para 4 líneas de producción de Fase 1, &gt;16,000 t/año de óxidos separados de alta pureza —Nd, Pr, Dy, Tb, Gd, Sm, Y, galio, germanio—; arranque de producción inicial previsto 3T2026)</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>[Mining News North](https://www.miningnewsnorth.com/story/2026/08/07/news/new-amalga-gold-project-enters-fast-41/9803.html)</t>
+          <t>[Mining Technology](https://www.mining-technology.com/news/air-permits-reelements-marion-refinery-indiana/); [Investing News Network](https://investingnews.com/reelement-technologies-receives-air-permits-for-marion-indiana-rare-earth-and-critical-mineral-refinery/)</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>ElementUSA Gramercy — Planta de Tierras Raras/Minerales Críticos</t>
+          <t>La Preciosa Project</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>Gramercy, St. John the Baptist Parish, Luisiana, EE.UU.</t>
+          <t>Durango, México</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>ElementUSA Inc. (en colaboración con Colorado School of Mines)</t>
+          <t>Avino Silver &amp; Gold Mines Ltd.</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
@@ -7460,71 +7474,71 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/financiamiento asegurado (proyecto de US$850 millones para procesar "lodo rojo"/bauxite residue del antiguo refinerio de alúmina Atalco —~34 millones de toneladas almacenadas— y extraer galio, escandio, disprosio, gadolinio, iterbio, germanio e itrio; recibió US$67 millones del DOE y US$29.9 millones del DoD; construcción de planta de demostración prevista a iniciar mediados de 2027, producción inicial 3T2028); Atalco (refinería de alúmina que aloja el sitio, entidad distinta co-ubicada) recibió 28-ago-2026 una inversión de capital adicional de US$100 millones del Departamento de Guerra de EE.UU. —participación total del DoW ahora US$400M, US$800M contando coinversión privada desde ene-2026— para restaurar la refinería, única refinería de alúmina activa en EE.UU., a su capacidad nominal de 1.2 millones ton/año, lo que apoya indirectamente la operación de ElementUSA en el mismo sitio</t>
+          <t>Construcción (desarrollo subterráneo en curso —rampa/decline de 360m—; permisos mineros ya obtenidos; producción objetivo 4T2026)</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>[Biz New Orleans](https://bizneworleans.com/elementusa-plans-850m-critical-minerals-refining-facility/); [Colorado School of Mines](https://www.minesnewsroom.com/news/colorado-school-mines-and-elementusa-awarded-67m-doe-construction-rare-earth-processing-plant); [Departamento de Guerra de EE.UU.](https://www.war.gov/News/Releases/Release/Article/4585310/department-of-war-announces-a-100-million-follow-on-equity-investment-in-atalco/)</t>
+          <t>[AccessWire](https://www.accessnewswire.com/newsroom/en/metals-and-mining/avino-provides-update-on-its-100-owned-la-preciosa-property-preparing-for-producti-837173); [MarketScreener](https://www.marketscreener.com/quote/stock/AVINO-SILVER-GOLD-MINES-L-1409069/news/Avino-Silver-Gold-Mines-Ltd-Commences-Underground-Development-At-La-Preciosa-48766238/)</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>Planta de Refinación de Tierras Raras y Minerales Críticos Marion (ReElement Technologies)</t>
+          <t>Great Salt Lake Lithium Facility</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>Marion, Indiana, EE.UU.</t>
+          <t>Condado de Box Elder, Utah, EE.UU.</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>American Resources Corporation (NASDAQ: AREC) vía subsidiaria ReElement Technologies</t>
+          <t>Lilac Solutions (subsidiaria Waterleaf P1 HoldCo)</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>No especificado (acondicionamiento interno de la ex planta RCA Thomson, 425,000 pies² en campus de 42 acres)</t>
+          <t>Hatch (EPCM, seleccionado jun-2026)</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>Permiso de aire obtenido/comisionamiento (IDEM —Indiana— otorgó el permiso "Minor Source" para 4 líneas de producción de Fase 1, &gt;16,000 t/año de óxidos separados de alta pureza —Nd, Pr, Dy, Tb, Gd, Sm, Y, galio, germanio—; arranque de producción inicial previsto 3T2026)</t>
+          <t>Desarrollo/Ingeniería (DOE anunció 20/21-ago-2026 subvención de hasta US$100 millones para construir planta comercial de extracción/refinación de litio por intercambio iónico directo desde salmuera del Great Salt Lake, 5,000 t/año; primera producción prevista 2028) ; DOE otorgó US$100 millones (anuncio 20-ago-2026) para la instalación comercial de extracción/refinación de litio mediante DLE de Lilac Solutions; capacidad de primera fase 5,000 ton/año, producción objetivo 2028</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>[Mining Technology](https://www.mining-technology.com/news/air-permits-reelements-marion-refinery-indiana/); [Investing News Network](https://investingnews.com/reelement-technologies-receives-air-permits-for-marion-indiana-rare-earth-and-critical-mineral-refinery/)</t>
+          <t>[KSL](https://www.ksl.com/article/51614351/california-company-awarded-100m-to-develop-critical-mineral-facility-on-great-salt-lake-shore); [Hatch](https://www.hatch.com/About-Us/News-And-Media/2026/06/Lilac-Solutions-Selects-Hatch-as-EPCM-Partner-for-Great-Salt-Lake-Lithium-Facility) ; [DOE](https://www.energy.gov/articles/energy-department-announces-500-million-secure-americas-critical-mineral-and-battery)</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>La Preciosa Project</t>
+          <t>Project SHIELD (refinería de "black mass" de baterías)</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>Durango, México</t>
+          <t>Carolina del Sur, EE.UU. (sitio exacto por definir)</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>Avino Silver &amp; Gold Mines Ltd.</t>
+          <t>Nth Cycle, Inc.</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
@@ -7534,49 +7548,49 @@
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>Construcción (desarrollo subterráneo en curso —rampa/decline de 360m—; permisos mineros ya obtenidos; producción objetivo 4T2026)</t>
+          <t>Negociación de subvención/preconstrucción (DOE seleccionó a Nth Cycle 20/21-ago-2026 para negociar premio de hasta US$100 millones; planta de refinación de "black mass" de baterías de litio, producirá MHP de níquel y carbonato de litio grado batería, 24,000 t/año; operación proyectada 2028)</t>
         </is>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>[AccessWire](https://www.accessnewswire.com/newsroom/en/metals-and-mining/avino-provides-update-on-its-100-owned-la-preciosa-property-preparing-for-producti-837173); [MarketScreener](https://www.marketscreener.com/quote/stock/AVINO-SILVER-GOLD-MINES-L-1409069/news/Avino-Silver-Gold-Mines-Ltd-Commences-Underground-Development-At-La-Preciosa-48766238/)</t>
+          <t>[Nth Cycle](https://nthcycle.com/newsroom/u.s.-department-of-energy-selects-nth-cycle-to-enter-award-negotiations-for-up-to-100-million-to-build-new-critical-mineral-refining-facility)</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>Great Salt Lake Lithium Facility</t>
+          <t>Refinería de Sulfato de Cobalto — Formation Holdings/Jervois</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>Condado de Box Elder, Utah, EE.UU.</t>
+          <t>Sitio por definir, EE.UU. (empresa con sede en Salmon, Idaho)</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>Lilac Solutions (subsidiaria Waterleaf P1 HoldCo)</t>
+          <t>Formation Holdings US, Inc. (dba Jervois)</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>Hatch (EPCM, seleccionado jun-2026)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>Desarrollo/Ingeniería (DOE anunció 20/21-ago-2026 subvención de hasta US$100 millones para construir planta comercial de extracción/refinación de litio por intercambio iónico directo desde salmuera del Great Salt Lake, 5,000 t/año; primera producción prevista 2028) ; DOE otorgó US$100 millones (anuncio 20-ago-2026) para la instalación comercial de extracción/refinación de litio mediante DLE de Lilac Solutions; capacidad de primera fase 5,000 ton/año, producción objetivo 2028</t>
+          <t>Desarrollo/financiamiento (DOE otorgó 21-ago-2026 subvención de US$100 millones para construir refinería comercial de sulfato de cobalto grado batería; ubicación específica de la planta aún no anunciada) ; DOE seleccionó el proyecto para un aporte federal de US$100 millones (anuncio 20-ago-2026) hacia una refinería comercial de cobalto; sitio industrial aún por determinar</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>[KSL](https://www.ksl.com/article/51614351/california-company-awarded-100m-to-develop-critical-mineral-facility-on-great-salt-lake-shore); [Hatch](https://www.hatch.com/About-Us/News-And-Media/2026/06/Lilac-Solutions-Selects-Hatch-as-EPCM-Partner-for-Great-Salt-Lake-Lithium-Facility) ; [DOE](https://www.energy.gov/articles/energy-department-announces-500-million-secure-americas-critical-mineral-and-battery)</t>
+          <t>[Local News 8](https://localnews8.com/news/business-watch/2026/08/21/salmon-company-wins-100-million-grant-to-build-cobalt-refinery/); [Local News 8 (seguimiento)](https://localnews8.com/news/local-news/2026/08/24/100m-grant-to-salmon-based-jervois-could-jumpstart-idahos-cobalt-industry/) ; [DOE](https://www.energy.gov/articles/energy-department-announces-500-million-secure-americas-critical-mineral-and-battery)</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
@@ -7588,106 +7602,106 @@
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>Project SHIELD (refinería de "black mass" de baterías)</t>
+          <t>Copperwood Project</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>Carolina del Sur, EE.UU. (sitio exacto por definir)</t>
+          <t>Península Superior Occidental, cerca de Wakefield, Michigan, EE.UU.</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>Nth Cycle, Inc.</t>
+          <t>Highland Copper Company</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>DRA Americas Inc. (FEED)</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>Negociación de subvención/preconstrucción (DOE seleccionó a Nth Cycle 20/21-ago-2026 para negociar premio de hasta US$100 millones; planta de refinación de "black mass" de baterías de litio, producirá MHP de níquel y carbonato de litio grado batería, 24,000 t/año; operación proyectada 2028)</t>
+          <t>Ingeniería/FEED (~40% completo para 4T2026; decisión de construcción esperada en 2S2026; producción de cobre proyectada 2029; capex ~US$425 millones)</t>
         </is>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>[Nth Cycle](https://nthcycle.com/newsroom/u.s.-department-of-energy-selects-nth-cycle-to-enter-award-negotiations-for-up-to-100-million-to-build-new-critical-mineral-refining-facility)</t>
+          <t>[Highland Copper](https://www.highlandcopper.com/news/highland-copper-recaps-2025-execution-and-announces-2026-work-plan-to-advance-copperwood-toward-construction-decision/)</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>Refinería de Sulfato de Cobalto — Formation Holdings/Jervois</t>
+          <t>Modernización Refinería de Cobre El Paso</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>Sitio por definir, EE.UU. (empresa con sede en Salmon, Idaho)</t>
+          <t>El Paso, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>Formation Holdings US, Inc. (dba Jervois)</t>
+          <t>Freeport-McMoRan</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>EPCM Group (tecnología de cátodos permanentes); Metso (equipo de tankhouse)</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>Desarrollo/financiamiento (DOE otorgó 21-ago-2026 subvención de US$100 millones para construir refinería comercial de sulfato de cobalto grado batería; ubicación específica de la planta aún no anunciada) ; DOE seleccionó el proyecto para un aporte federal de US$100 millones (anuncio 20-ago-2026) hacia una refinería comercial de cobalto; sitio industrial aún por determinar</t>
+          <t>Contrato adjudicado 2026 (modernización de refinería electrolítica, 46,650 cátodos permanentes, sustituye tecnología de láminas de arranque tradicional)</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>[Local News 8](https://localnews8.com/news/business-watch/2026/08/21/salmon-company-wins-100-million-grant-to-build-cobalt-refinery/); [Local News 8 (seguimiento)](https://localnews8.com/news/local-news/2026/08/24/100m-grant-to-salmon-based-jervois-could-jumpstart-idahos-cobalt-industry/) ; [DOE](https://www.energy.gov/articles/energy-department-announces-500-million-secure-americas-critical-mineral-and-battery)</t>
+          <t>[EPCM Group](https://www.epcm.com/epcm-secures-prestigious-contract-with-freeport-mcmoran-to-advance-el-paso-copper-refinery-modernization/)</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-26</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>Copperwood Project</t>
+          <t>Round Top Rare Earth Project</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>Península Superior Occidental, cerca de Wakefield, Michigan, EE.UU.</t>
+          <t>Sierra Blanca, Condado de Hudspeth, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>Highland Copper Company</t>
+          <t>USA Rare Earth Inc.</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>DRA Americas Inc. (FEED)</t>
+          <t>Fluor Corporation / WSP Global Inc. (EPCM para estudio de factibilidad definitivo)</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/FEED (~40% completo para 4T2026; decisión de construcción esperada en 2S2026; producción de cobre proyectada 2029; capex ~US$425 millones)</t>
+          <t>Ingeniería/DFS (en curso; subvención estatal de Texas de US$14.2 millones, may-2026; inversión estimada &gt;US$1,400 millones; producción adelantada a fines de 2028; tierras raras pesadas)</t>
         </is>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>[Highland Copper](https://www.highlandcopper.com/news/highland-copper-recaps-2025-execution-and-announces-2026-work-plan-to-advance-copperwood-toward-construction-decision/)</t>
+          <t>[IM Mining](https://im-mining.com/2026/01/23/fluor-and-wsp-on-board-usa-rare-earth-incs-round-top-rare-earth-project/)</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
@@ -7699,32 +7713,32 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>Modernización Refinería de Cobre El Paso</t>
+          <t>Expansión Fundición de Antimonio Thompson Falls</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>El Paso, Texas, EE.UU.</t>
+          <t>Thompson Falls, Montana, EE.UU.</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>Freeport-McMoRan</t>
+          <t>United States Antimony Corporation (USAC)</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>EPCM Group (tecnología de cátodos permanentes); Metso (equipo de tankhouse)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>Contrato adjudicado 2026 (modernización de refinería electrolítica, 46,650 cátodos permanentes, sustituye tecnología de láminas de arranque tradicional)</t>
+          <t>Comisionamiento (nueva fundición construida; comisionamiento de 9 hornos a gas iniciado may-2026; financiada con US$27 millones del Departamento de Guerra, mar-2026)</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>[EPCM Group](https://www.epcm.com/epcm-secures-prestigious-contract-with-freeport-mcmoran-to-advance-el-paso-copper-refinery-modernization/)</t>
+          <t>[Montana Public Radio](https://www.mtpr.org/montana-news/2026-04-06/montana-antimony-facility-expands-amid-federal-push-for-domestic-sources)</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
@@ -7736,32 +7750,32 @@
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>Round Top Rare Earth Project</t>
+          <t>Expansión Planta de Lixiviación de Concentrados (CLP) Morenci</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>Sierra Blanca, Condado de Hudspeth, Texas, EE.UU.</t>
+          <t>Morenci, Arizona, EE.UU.</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>USA Rare Earth Inc.</t>
+          <t>Freeport-McMoRan</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>Fluor Corporation / WSP Global Inc. (EPCM para estudio de factibilidad definitivo)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/DFS (en curso; subvención estatal de Texas de US$14.2 millones, may-2026; inversión estimada &gt;US$1,400 millones; producción adelantada a fines de 2028; tierras raras pesadas)</t>
+          <t>Comisionamiento (segundo y último vaso de la expansión en comisionamiento/ajuste durante 2026; objetivo casi duplicar throughput de 24 a 40 ton/hora)</t>
         </is>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>[IM Mining](https://im-mining.com/2026/01/23/fluor-and-wsp-on-board-usa-rare-earth-incs-round-top-rare-earth-project/)</t>
+          <t>[Freeport-McMoRan](https://www.fcx.com/freeport-features/112125)</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
@@ -7773,17 +7787,17 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>Expansión Fundición de Antimonio Thompson Falls</t>
+          <t>Reconstrucción Fundición y Refinería Kennecott</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>Thompson Falls, Montana, EE.UU.</t>
+          <t>Bingham Canyon/Kennecott, Utah, EE.UU.</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>United States Antimony Corporation (USAC)</t>
+          <t>Rio Tinto (Kennecott Utah Copper)</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
@@ -7793,12 +7807,12 @@
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>Comisionamiento (nueva fundición construida; comisionamiento de 9 hornos a gas iniciado may-2026; financiada con US$27 millones del Departamento de Guerra, mar-2026)</t>
+          <t>Construcción (reconstrucción de fundición US$300 millones y actualización de refinería/tankhouse y circuito de flotación de molibdeno US$120 millones en curso durante 2026; reparación adicional tras falla de horno flash en jun-2026, ~75 días)</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>[Montana Public Radio](https://www.mtpr.org/montana-news/2026-04-06/montana-antimony-facility-expands-amid-federal-push-for-domestic-sources)</t>
+          <t>[Mining.com](https://www.mining.com/web/rio-tinto-to-invest-almost-1-billion-in-kennecott-copper-mine/)</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
@@ -7810,32 +7824,32 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>Expansión Planta de Lixiviación de Concentrados (CLP) Morenci</t>
+          <t>Fourmile (decline Bullion Hill)</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>Morenci, Arizona, EE.UU.</t>
+          <t>Carlin Trend, condados de Elko/Eureka, Nevada, EE.UU.</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>Freeport-McMoRan</t>
+          <t>Barrick Mining Corporation (JV Nevada Gold Mines, desde ago-2026)</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Barminco (Perenti) — contrato A$275 millones/45 meses</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>Comisionamiento (segundo y último vaso de la expansión en comisionamiento/ajuste durante 2026; objetivo casi duplicar throughput de 24 a 40 ton/hora)</t>
+          <t>Construcción (inicio de desarrollo subterráneo/portales programado jul/3T2026; ~16 km de desarrollo lateral subterráneo planeados; adyacente al complejo Goldrush)</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>[Freeport-McMoRan](https://www.fcx.com/freeport-features/112125)</t>
+          <t>[Northern Miner](https://www.northernminer.com/news/mining-forum-americas-fourmile-anchors-barricks-nevada-plan/1003882789/)</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
@@ -7847,17 +7861,17 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>Reconstrucción Fundición y Refinería Kennecott</t>
+          <t>Puerto del Aire (distrito Mulatos)</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>Bingham Canyon/Kennecott, Utah, EE.UU.</t>
+          <t>Sonora, México</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>Rio Tinto (Kennecott Utah Copper)</t>
+          <t>Alamos Gold Inc.</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
@@ -7867,12 +7881,12 @@
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>Construcción (reconstrucción de fundición US$300 millones y actualización de refinería/tankhouse y circuito de flotación de molibdeno US$120 millones en curso durante 2026; reparación adicional tras falla de horno flash en jun-2026, ~75 días)</t>
+          <t>Construcción (en curso desde 2025-2026 tras permiso ambiental ene-2025; procura de equipos de molienda de largo plazo de entrega; capex total US$165 millones; primera producción prevista mediados 2027)</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>[Mining.com](https://www.mining.com/web/rio-tinto-to-invest-almost-1-billion-in-kennecott-copper-mine/)</t>
+          <t>[Alamos Gold](https://www.alamosgold.com/news-and-events/news/news-details/2025/Alamos-Gold-Announces-Receipt-of-Environmental-Permit-Amendment-Allowing-for-the-Start-of-Construction-on-the-Puerto-Del-Aire-Project-in-Mexico/default.aspx)</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
@@ -7884,54 +7898,54 @@
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>Fourmile (decline Bullion Hill)</t>
+          <t>Korea Zinc / Nyrstar Critical Minerals Smelter</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>Carlin Trend, condados de Elko/Eureka, Nevada, EE.UU.</t>
+          <t>Clarksville, Tennessee, EE.UU.</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>Barrick Mining Corporation (JV Nevada Gold Mines, desde ago-2026)</t>
+          <t>Korea Zinc / U.S. Department of War / U.S. Department of Commerce (participación ~10%)</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>Barminco (Perenti) — contrato A$275 millones/45 meses</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>Construcción (inicio de desarrollo subterráneo/portales programado jul/3T2026; ~16 km de desarrollo lateral subterráneo planeados; adyacente al complejo Goldrush)</t>
+          <t>Preparación de sitio en 2026, construcción completa en 2027 (inversión US$7,400 millones, capex US$6,600 millones; producirá zinc, plomo, cobre, oro, plata, antimonio, indio, bismuto, telurio, cadmio, galio, germanio, paladio y ácido sulfúrico; planta altamente intensiva en tubería/piping)</t>
         </is>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>[Northern Miner](https://www.northernminer.com/news/mining-forum-americas-fourmile-anchors-barricks-nevada-plan/1003882789/)</t>
+          <t>[Korea Zinc](https://www.koreazinc.co.kr/en/korea-zinc-partners-with-the-u-s-department-of-war-and-u-s-department-of-commerce-to-build-a-state-of-the-art-critical-minerals-smelter-in-the-united-states-with-6-6-billion-of-capital-expenditures/); [Carbon Credits](https://carboncredits.com/big-bet-bigger-stakes-korea-zincs-7-4-billion-smelter-reshapes-u-s-critical-minerals-supply/)</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>Puerto del Aire (distrito Mulatos)</t>
+          <t>Aclara Heavy Rare Earth Separation Facility</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>Sonora, México</t>
+          <t>Port of Vinton, Calcasieu Parish, Luisiana, EE.UU.</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>Alamos Gold Inc.</t>
+          <t>Aclara Resources Inc.</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
@@ -7941,34 +7955,34 @@
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>Construcción (en curso desde 2025-2026 tras permiso ambiental ene-2025; procura de equipos de molienda de largo plazo de entrega; capex total US$165 millones; primera producción prevista mediados 2027)</t>
+          <t>Planeación (inversión US$277 millones; groundbreaking previsto 4T2026, construcción hasta 2027; procesará mineral de depósitos propios en Brasil/Chile)</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>[Alamos Gold](https://www.alamosgold.com/news-and-events/news/news-details/2025/Alamos-Gold-Announces-Receipt-of-Environmental-Permit-Amendment-Allowing-for-the-Start-of-Construction-on-the-Puerto-Del-Aire-Project-in-Mexico/default.aspx)</t>
+          <t>[Louisiana Economic Development](https://www.opportunitylouisiana.gov/news/aclara-invests-277-million-to-build-nations-first-heavy-rare-earth-separation-facility-in-southwest-louisiana)</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>Korea Zinc / Nyrstar Critical Minerals Smelter</t>
+          <t>Archimedes Project (i-80 Gold)</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>Clarksville, Tennessee, EE.UU.</t>
+          <t>Ruby Hill, Eureka County, Nevada, EE.UU.</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>Korea Zinc / U.S. Department of War / U.S. Department of Commerce (participación ~10%)</t>
+          <t>i-80 Gold Corp</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
@@ -7978,12 +7992,12 @@
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>Preparación de sitio en 2026, construcción completa en 2027 (inversión US$7,400 millones, capex US$6,600 millones; producirá zinc, plomo, cobre, oro, plata, antimonio, indio, bismuto, telurio, cadmio, galio, germanio, paladio y ácido sulfúrico; planta altamente intensiva en tubería/piping)</t>
+          <t>Construcción (permisos de Nevada DEP y BLM obtenidos; desarrollo subterráneo en curso; producción esperada 4T2026, objetivo 150,000-200,000 oz Au/año hacia 2028)</t>
         </is>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>[Korea Zinc](https://www.koreazinc.co.kr/en/korea-zinc-partners-with-the-u-s-department-of-war-and-u-s-department-of-commerce-to-build-a-state-of-the-art-critical-minerals-smelter-in-the-united-states-with-6-6-billion-of-capital-expenditures/); [Carbon Credits](https://carboncredits.com/big-bet-bigger-stakes-korea-zincs-7-4-billion-smelter-reshapes-u-s-critical-minerals-supply/)</t>
+          <t>[Resource World](https://resourceworld.com/i-80-gold-obtains-construction-permits-and-begins-underground-development-at-archimedes-project-nevada/)</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -7995,17 +8009,17 @@
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>Aclara Heavy Rare Earth Separation Facility</t>
+          <t>Sweetwater Uranium In-Situ Recovery (ISR) Project</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>Port of Vinton, Calcasieu Parish, Luisiana, EE.UU.</t>
+          <t>Sweetwater County, Wyoming, EE.UU.</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>Aclara Resources Inc.</t>
+          <t>Sweetwater Uranium, Inc.</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
@@ -8015,12 +8029,12 @@
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>Planeación (inversión US$277 millones; groundbreaking previsto 4T2026, construcción hasta 2027; procesará mineral de depósitos propios en Brasil/Chile)</t>
+          <t>Permitting (Plan de Operaciones sometido al BLM nov-2025, periodo de comentarios públicos mar-abr 2026, proyecto designado FAST-41; sería la mayor instalación de producción de uranio de EE.UU. combinando procesamiento convencional e ISR)</t>
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>[Louisiana Economic Development](https://www.opportunitylouisiana.gov/news/aclara-invests-277-million-to-build-nations-first-heavy-rare-earth-separation-facility-in-southwest-louisiana)</t>
+          <t>[BLM](https://www.blm.gov/announcement/sweetwater-uranium-situ-recovery-irs-project-mine-plan-operations)</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -8032,17 +8046,17 @@
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>Archimedes Project (i-80 Gold)</t>
+          <t>Velvet-Wood Uranium-Vanadium Project</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>Ruby Hill, Eureka County, Nevada, EE.UU.</t>
+          <t>San Juan County, Utah, EE.UU.</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>i-80 Gold Corp</t>
+          <t>Anfield Energy Inc.</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
@@ -8052,12 +8066,12 @@
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>Construcción (permisos de Nevada DEP y BLM obtenidos; desarrollo subterráneo en curso; producción esperada 4T2026, objetivo 150,000-200,000 oz Au/año hacia 2028)</t>
+          <t>Construcción (Fase 1 de construcción superficial completada jun-2026; desarrollo subterráneo Fase 2 en curso; regreso a producción previsto fines de 2026)</t>
         </is>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>[Resource World](https://resourceworld.com/i-80-gold-obtains-construction-permits-and-begins-underground-development-at-archimedes-project-nevada/)</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/06/01/3304179/0/en/Anfield-Energy-Inc-Completes-Phase-One-Surface-Construction-at-Velvet-Wood-Project.html)</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -8069,259 +8083,222 @@
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>Sweetwater Uranium In-Situ Recovery (ISR) Project</t>
+          <t>Twin Metals Minnesota</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>Sweetwater County, Wyoming, EE.UU.</t>
+          <t>Ely, Minnesota, EE.UU. (cerca de Boundary Waters)</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>Sweetwater Uranium, Inc.</t>
+          <t>Antofagasta plc (Twin Metals Minnesota LLC)</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>No definido</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>Permitting (Plan de Operaciones sometido al BLM nov-2025, periodo de comentarios públicos mar-abr 2026, proyecto designado FAST-41; sería la mayor instalación de producción de uranio de EE.UU. combinando procesamiento convencional e ISR)</t>
+          <t>Permitting/Pre-EIS (plan de mina formal —concentradora de flotación de 20,000 tpd, cobre-níquel-EGP— presentado ante BLM y Minnesota DNR; el gobernador Walz frenó el trámite estatal en ago-2026, pero el proceso federal continúa activo; construcción aún a años de distancia)</t>
         </is>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>[BLM](https://www.blm.gov/announcement/sweetwater-uranium-situ-recovery-irs-project-mine-plan-operations)</t>
+          <t>[MinnPost](http://www.minnpost.com/state-government/2026/08/walz-halts-state-action-on-mine-near-boundary-waters-but-federal-process-stays-on-track/); [Star Tribune](https://www.startribune.com/twin-metals-submits-formal-mine-plan-to-minnesota-federal-officials/566311242)</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>Velvet-Wood Uranium-Vanadium Project</t>
+          <t>Falcon Copper — Fundición y Refinería de Cobre (greenfield)</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>San Juan County, Utah, EE.UU.</t>
+          <t>Arizona (fundición) / Costa del Golfo (refinería), EE.UU. (sitios por definir)</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>Anfield Energy Inc.</t>
+          <t>Falcon Copper Corp. (MOU con Glencore)</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>No definido</t>
         </is>
       </c>
       <c r="E105" s="2" t="inlineStr">
         <is>
-          <t>Construcción (Fase 1 de construcción superficial completada jun-2026; desarrollo subterráneo Fase 2 en curso; regreso a producción previsto fines de 2026)</t>
+          <t>Evaluación/pre-FEED (proyecto greenfield de ~US$2,000 millones para fundición primaria de cobre más refinería electrolítica; sin sitio definitivo ni FID)</t>
         </is>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/06/01/3304179/0/en/Anfield-Energy-Inc-Completes-Phase-One-Surface-Construction-at-Velvet-Wood-Project.html)</t>
+          <t>[Fastmarkets](https://www.fastmarkets.com/insights/us-copper-smelting-equation-gap-or-glut-hotter-commodities-articles/); [Falcon Copper](https://www.falconcopper.com/projects/works)</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>Twin Metals Minnesota</t>
+          <t>Del Sol Refinery (antimonio/tungsteno) + White Spar Antimony Mine</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>Ely, Minnesota, EE.UU. (cerca de Boundary Waters)</t>
+          <t>Amargosa Valley, Nevada (refinería) / Arizona (mina), EE.UU.</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>Antofagasta plc (Twin Metals Minnesota LLC)</t>
+          <t>American Tungsten &amp; Antimony Corp (ATALF)</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>No definido</t>
+          <t>Metso Finland Oy (estudio de alcance)</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
         <is>
-          <t>Permitting/Pre-EIS (plan de mina formal —concentradora de flotación de 20,000 tpd, cobre-níquel-EGP— presentado ante BLM y Minnesota DNR; el gobernador Walz frenó el trámite estatal en ago-2026, pero el proceso federal continúa activo; construcción aún a años de distancia)</t>
+          <t>Ingeniería/estudio (adquirió el 28-jul-2026 la refinería hidrometalúrgica permisada de antimonio Del Sol —18,500 t/año de capacidad de alimentación— y la mina White Spar (AZ) como fuente de mineral; 1-sep-2026 contrató a Metso para estudio de alcance de un circuito de producción de paratungstato de amonio —APT—, Fase 1: 2,500 t/año, posible Fase 2 a 5,000 t/año; la refinería también recibirá mineral del proyecto Antimony Canyon, Utah)</t>
         </is>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>[MinnPost](http://www.minnpost.com/state-government/2026/08/walz-halts-state-action-on-mine-near-boundary-waters-but-federal-process-stays-on-track/); [Star Tribune](https://www.startribune.com/twin-metals-submits-formal-mine-plan-to-minnesota-federal-officials/566311242)</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/american-tungsten-and-antimony-announces-study-for-tungsten-production-at-del-sol-refinery-in-nevada-302866335.html); [PR Newswire](https://www.prnewswire.com/news-releases/american-tungsten-and-antimony-to-acquire-permitted-critical-metals-refinery-in-nevada-and-white-spar-antimony-mine-in-arizona-302836579.html)</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-02</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>Falcon Copper — Fundición y Refinería de Cobre (greenfield)</t>
+          <t>Spring Valley Gold Mine</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>Arizona (fundición) / Costa del Golfo (refinería), EE.UU. (sitios por definir)</t>
+          <t>Condado de Pershing, Nevada, EE.UU.</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>Falcon Copper Corp. (MOU con Glencore)</t>
+          <t>Solidus Resources LLC (subsidiaria de Waterton Gold)</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>No definido</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E107" s="2" t="inlineStr">
         <is>
-          <t>Evaluación/pre-FEED (proyecto greenfield de ~US$2,000 millones para fundición primaria de cobre más refinería electrolítica; sin sitio definitivo ni FID)</t>
+          <t>Construcción (todos los permisos federales en mano —BLM aprobó el plan de operaciones—; proyecto totalmente financiado, ~US$1,300 millones de capital comprometido incl. stream de oro de US$670M de Wheaton Precious Metals; trabajos de sitio tempranos en curso, construcción completa inicia en 2026; primera producción de oro proyectada 1S2028; reservas probadas/probables de 3.8 Moz Au)</t>
         </is>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>[Fastmarkets](https://www.fastmarkets.com/insights/us-copper-smelting-equation-gap-or-glut-hotter-commodities-articles/); [Falcon Copper](https://www.falconcopper.com/projects/works)</t>
+          <t>[BLM](https://www.blm.gov/announcement/blm-approves-spring-valley-gold-mine-pershing-county); [Wheaton Precious Metals](https://www.wheatonpm.com/portfolio/development-projects/spring-valley/default.aspx); [The Pershing Post](https://www.thepershingpost.com/article/496,spring-valley-mine-project-moves-into-construction-phase-hiring-to-begin-in-2026)</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-03</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>Del Sol Refinery (antimonio/tungsteno) + White Spar Antimony Mine</t>
+          <t>Pitarrilla Project (plata-plomo-zinc)</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>Amargosa Valley, Nevada (refinería) / Arizona (mina), EE.UU.</t>
+          <t>160 km al norte de la ciudad de Durango, Durango, México</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>American Tungsten &amp; Antimony Corp (ATALF)</t>
+          <t>Endeavour Silver Corp.</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>Metso Finland Oy (estudio de alcance)</t>
+          <t>SGS Canada / SGS Bateman / JDS Energy &amp; Mining / T Engineering / Stantec / SRK Consulting (estudio de factibilidad)</t>
         </is>
       </c>
       <c r="E108" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/estudio (adquirió el 28-jul-2026 la refinería hidrometalúrgica permisada de antimonio Del Sol —18,500 t/año de capacidad de alimentación— y la mina White Spar (AZ) como fuente de mineral; 1-sep-2026 contrató a Metso para estudio de alcance de un circuito de producción de paratungstato de amonio —APT—, Fase 1: 2,500 t/año, posible Fase 2 a 5,000 t/año; la refinería también recibirá mineral del proyecto Antimony Canyon, Utah)</t>
+          <t>Ingeniería/estudio de factibilidad (inversión 2026 de US$65.8 millones: US$15M para estudio de factibilidad, US$48M en capex de preparación minera y 1,300 m de desarrollo subterráneo; aún sin decisión de construcción)</t>
         </is>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>[PR Newswire](https://www.prnewswire.com/news-releases/american-tungsten-and-antimony-announces-study-for-tungsten-production-at-del-sol-refinery-in-nevada-302866335.html); [PR Newswire](https://www.prnewswire.com/news-releases/american-tungsten-and-antimony-to-acquire-permitted-critical-metals-refinery-in-nevada-and-white-spar-antimony-mine-in-arizona-302836579.html)</t>
+          <t>[Mexico Business News](https://mexicobusiness.news/mining/news/endeavour-silver-forecasts-89moz-silver-2026); [Endeavour Silver](https://edrsilver.com/portfolio/development/pitarrilla/)</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>Spring Valley Gold Mine</t>
+          <t>Red Dog Mine Life Extension Project</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>Condado de Pershing, Nevada, EE.UU.</t>
+          <t>Distrito Minero de NANA, noroeste de Alaska, EE.UU.</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>Solidus Resources LLC (subsidiaria de Waterton Gold)</t>
+          <t>Teck American Incorporated (Teck Resources), en tierras de NANA Regional Corporation</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>U.S. Army Corps of Engineers (agencia líder de permisos)</t>
         </is>
       </c>
       <c r="E109" s="2" t="inlineStr">
         <is>
-          <t>Construcción (todos los permisos federales en mano —BLM aprobó el plan de operaciones—; proyecto totalmente financiado, ~US$1,300 millones de capital comprometido incl. stream de oro de US$670M de Wheaton Precious Metals; trabajos de sitio tempranos en curso, construcción completa inicia en 2026; primera producción de oro proyectada 1S2028; reservas probadas/probables de 3.8 Moz Au)</t>
+          <t>Prefactibilidad (estudio en curso; Teck destina US$200-250 millones en 2026 a obras tempranas —camino de acceso todo-el-año, perforación— y avance del estudio de prefactibilidad; minado subterráneo por realces largos (long-hole stoping) propuesto para los yacimientos Aktigiruq y Anarraaq, alimentando el molino existente de Red Dog; minerales: zinc, plomo, plata, germanio; proyecto obtuvo cobertura FAST-41 en sep-2026)</t>
         </is>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>[BLM](https://www.blm.gov/announcement/blm-approves-spring-valley-gold-mine-pershing-county); [Wheaton Precious Metals](https://www.wheatonpm.com/portfolio/development-projects/spring-valley/default.aspx); [The Pershing Post](https://www.thepershingpost.com/article/496,spring-valley-mine-project-moves-into-construction-phase-hiring-to-begin-in-2026)</t>
+          <t>[Permitting.gov](https://www.permitting.gov/newsroom/press-releases/red-dog-mine-life-extension-project-gains-fast-41-coverage); [Mining News North](https://www.miningnewsnorth.com/story/2026/09/04/news/red-dog-extension-gains-fast-41-permitting/9851.html)</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" s="2" t="inlineStr">
-        <is>
-          <t>Pitarrilla Project (plata-plomo-zinc)</t>
-        </is>
-      </c>
-      <c r="B110" s="2" t="inlineStr">
-        <is>
-          <t>160 km al norte de la ciudad de Durango, Durango, México</t>
-        </is>
-      </c>
-      <c r="C110" s="2" t="inlineStr">
-        <is>
-          <t>Endeavour Silver Corp.</t>
-        </is>
-      </c>
-      <c r="D110" s="2" t="inlineStr">
-        <is>
-          <t>SGS Canada / SGS Bateman / JDS Energy &amp; Mining / T Engineering / Stantec / SRK Consulting (estudio de factibilidad)</t>
-        </is>
-      </c>
-      <c r="E110" s="2" t="inlineStr">
-        <is>
-          <t>Ingeniería/estudio de factibilidad (inversión 2026 de US$65.8 millones: US$15M para estudio de factibilidad, US$48M en capex de preparación minera y 1,300 m de desarrollo subterráneo; aún sin decisión de construcción)</t>
-        </is>
-      </c>
-      <c r="F110" s="2" t="inlineStr">
-        <is>
-          <t>[Mexico Business News](https://mexicobusiness.news/mining/news/endeavour-silver-forecasts-89moz-silver-2026); [Endeavour Silver](https://edrsilver.com/portfolio/development/pitarrilla/)</t>
-        </is>
-      </c>
-      <c r="G110" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
     </row>
@@ -8336,16 +8313,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G101"/>
+  <dimension ref="A1:G103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -12085,6 +12062,80 @@
         </is>
       </c>
     </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>Fleet Data Centers — Peru Ridge &amp; South Valley Self-Generation Projects</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>Tahoe Reno Industrial Center, Nevada, EE.UU.</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>Fleet Data Centers (subsidiaria de Tract Capital Management)</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>Solicitud regulatoria (dos plantas de gas natural dedicadas —motores de gas metano— para autogeneración: Peru Ridge Self-Generation Project (218 MW) y South Valley (planta temporal, 144 MW), alimentando dos campus de data centers en el mismo parque industrial; solicitud ante la Public Utility Commission of Nevada (PUCN), decisión final esperada 8-sep-2026)</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>[Nevada Current](https://nevadacurrent.com/2026/09/01/private-gas-plants-to-power-data-centers-would-skirt-states-renewable-energy-law/); [The Nevada Independent](https://thenevadaindependent.com/article/why-a-northern-nevada-data-center-wants-to-build-its-own-temporary-natural-gas-power-plant)</t>
+        </is>
+      </c>
+      <c r="G102" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>Cuasar Data Center Campus (Cuasar Capital / grupo EOSOL)</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>Durango, Durango, México</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>Cuasar Capital (grupo español EOSOL), en alianza comercial con KA URBE IT</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>No especificado</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="inlineStr">
+        <is>
+          <t>Anuncio de campus/comercialización (etapa temprana; dos instalaciones — DC Norte Uno, 300 MW total/250 MW IT, sitio de 20 ha, Tier III; y DC Norte Dos, 7.74 MW, Edge/industrial —; enfocado en cargas de IA de alta densidad; respaldo reportado por proyectos fotovoltaicos de EOSOL, sin confirmar planta de gas dedicada)</t>
+        </is>
+      </c>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
+          <t>[Data Center Dynamics](https://www.datacenterdynamics.com/en/news/quasar-launches-a-300-mw-data-center-campus-in-durango-mexico/); [BeBeez](https://bebeez.eu/2026/09/03/cuasar-capital-plans-300mw-data-center-campus-in-durango-mexico/)</t>
+        </is>
+      </c>
+      <c r="G103" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Monitoreo 2026-09-04: 3 proyectos nuevos + 1 actualización de fase (#37)
- Nuevos: Red Dog Mine Life Extension Project (Alaska, Mining), Fleet
  Data Centers Peru Ridge & South Valley Self-Generation Projects
  (Nevada, Data Centers), Cuasar Data Center Campus (Durango, México,
  Data Centers).
- Actualización de fase: Saguaro Energía LNG (más de nueve amparos
  judiciales activos y suspensión de ingreso de buques metaneros al
  Golfo de California).
- proyectos.xlsx regenerado con el acumulado completo en 4 hojas.


Claude-Session: https://claude.ai/code/session_014D76wwULT3tWpnkg8hSics

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/proyectos.xlsx
+++ b/proyectos.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,15 +29,27 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Arial"/>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+        <bgColor rgb="001F4E78"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -54,8 +66,10 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -426,13 +440,13 @@
   <dimension ref="A1:G55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2484,13 +2498,13 @@
   <dimension ref="A1:G47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2849,17 +2863,17 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Pre-FID PAUSADO (suspensión judicial desde abr-2026 por demanda ambiental sobre ballenas en el Mar de Cortés; presión de activistas contra financiadores JPMorgan/Santander, 17-jul-2026; afiliada de ONEOK solicitó extensión de 3 años del plazo de construcción del Saguaro Connector Pipeline, de feb-2027 a feb-2030, confirmando que la construcción del gasoducto aún no inicia; definición de autorización pendiente para 2026)</t>
+          <t>Pre-FID PAUSADO (suspensión judicial desde abr-2026 por demanda ambiental sobre ballenas en el Mar de Cortés; presión de activistas contra financiadores JPMorgan/Santander, 17-jul-2026; afiliada de ONEOK solicitó extensión de 3 años del plazo de construcción del Saguaro Connector Pipeline, de feb-2027 a feb-2030, confirmando que la construcción del gasoducto aún no inicia; reporte del 1-sep-2026 confirma que más de nueve amparos/suspensiones judiciales distintos mantienen frenado el proyecto, incluyendo una suspensión que impide el ingreso de buques metaneros vinculados al proyecto al Golfo de California; la autorización ambiental original de 2018 —modificada de planta de regasificación a terminal de exportación— sigue sin resolverse en definitiva; litigante activo: Nuestro Futuro A.C.)</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>[Dossier Político](https://dossierpolitico.com/2026/07/17/activistas-entregan-90-mil-firmas-para-frenar-proyecto-saguaro-energia-en-sonora/); [Natural Gas Intel](https://naturalgasintel.com/news/oneok-affiliate-seeks-3-year-extension-for-saguaro-connector-pipeline/)</t>
+          <t>[Dossier Político](https://dossierpolitico.com/2026/07/17/activistas-entregan-90-mil-firmas-para-frenar-proyecto-saguaro-energia-en-sonora/); [Natural Gas Intel](https://naturalgasintel.com/news/oneok-affiliate-seeks-3-year-extension-for-saguaro-connector-pipeline/); [Dossier Político](https://dossierpolitico.com/2026/09/01/suspensiones-judiciales-mantienen-frenados-los-megaproyectos-de-gnl-en-sonora-nuestro-futuro/)</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-09-04</t>
         </is>
       </c>
     </row>
@@ -4243,16 +4257,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G110"/>
+  <dimension ref="A1:G109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6108,17 +6122,17 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>NewRange Copper Nickel (Proyecto NorthMet) — Rediseño Mayor</t>
+          <t>White Mesa Mill — Expansión de Tierras Raras Pesadas</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Babbitt/Hoyt Lakes, Minnesota, EE.UU. (Iron Range)</t>
+          <t>Blanding, Utah, EE.UU.</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>NewRange Copper Nickel (JV PolyMet/Glencore + Teck)</t>
+          <t>Energy Fuels Inc.</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -6128,86 +6142,86 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Permitting (rediseño mayor elimina la represa de jales propuesta —roca estéril se almacenaría en tajos de mineral de hierro existentes—; solicitud de permiso de humedales Sección 404/Clean Water Act presentada ante USACE; revisión ambiental suplementaria (SEIS) solicitada a Minnesota DNR)</t>
+          <t>Construcción (planta comercial de tierras raras pesadas —disprosio/terbio— iniciada 29-jul-2026; capex ~US$104 millones, para uso en imanes/defensa/vehículos eléctricos)</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>[MPR News](https://www.mprnews.org/story/2026/07/30/newrange-copper-nickel-proposes-major-changes-to-copper-mine-plan)</t>
+          <t>[Energy Fuels](https://investors.energyfuels.com/2026-07-29-Commercial-Scale-Heavy-Rare-Earth-Plant-Now-Under-Construction-in-Utah); [PR Newswire](https://www.prnewswire.com/news-releases/commercial-scale-heavy-rare-earth-plant-now-under-construction-in-utah-302837314.html)</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-07-30</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>White Mesa Mill — Expansión de Tierras Raras Pesadas</t>
+          <t>Black Butte Copper Project</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Blanding, Utah, EE.UU.</t>
+          <t>Meagher County, Montana, EE.UU.</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Energy Fuels Inc.</t>
+          <t>Sandfire Resources America Inc. (Sandfire Resources)</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>No especificado</t>
+          <t>Por definir (PFS elaborado por DM Consulting)</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Construcción (planta comercial de tierras raras pesadas —disprosio/terbio— iniciada 29-jul-2026; capex ~US$104 millones, para uso en imanes/defensa/vehículos eléctricos)</t>
+          <t>Feasibility (PFS actualizado presentado 28-jul-2026 con nuevas reservas Lowry, vida de mina de 12 años; mina subterránea de cobre de alta ley)</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>[Energy Fuels](https://investors.energyfuels.com/2026-07-29-Commercial-Scale-Heavy-Rare-Earth-Plant-Now-Under-Construction-in-Utah); [PR Newswire](https://www.prnewswire.com/news-releases/commercial-scale-heavy-rare-earth-plant-now-under-construction-in-utah-302837314.html)</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/29/3334925/0/en/sandfire-resources-america-files-black-butte-copper-project-preliminary-feasibility-study.html)</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-03</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Black Butte Copper Project</t>
+          <t>Planta de Procesamiento de Litio Red River (US Army)</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Meagher County, Montana, EE.UU.</t>
+          <t>Bowie County, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Sandfire Resources America Inc. (Sandfire Resources)</t>
+          <t>Pentágono / Departamento del Ejército de EE.UU.</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Por definir (PFS elaborado por DM Consulting)</t>
+          <t>EnergyX (desarrollador-operador)</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>Feasibility (PFS actualizado presentado 28-jul-2026 con nuevas reservas Lowry, vida de mina de 12 años; mina subterránea de cobre de alta ley)</t>
+          <t>Acuerdo de arrendamiento condicional otorgado (confirmado 25-jun-2026; 5to sitio del programa de minerales críticos en bases del Ejército, junto con Tooele, Pine Bluff/Anniston; construcción prevista desde 2027)</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/07/29/3334925/0/en/sandfire-resources-america-files-black-butte-copper-project-preliminary-feasibility-study.html)</t>
+          <t>[Texarkana Gazette](https://www.texarkanagazette.com/news/2026/jun/30/army-awards-lithium-company-energyx-conditional/)</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -6219,54 +6233,54 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Planta de Procesamiento de Litio Red River (US Army)</t>
+          <t>Cerro Caliche Gold Project</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Bowie County, Texas, EE.UU.</t>
+          <t>Sonora, México</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Pentágono / Departamento del Ejército de EE.UU.</t>
+          <t>Sonoro Gold Corp.</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>EnergyX (desarrollador-operador)</t>
+          <t>EPC por definir (en negociación con múltiples empresas EPC de China)</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Acuerdo de arrendamiento condicional otorgado (confirmado 25-jun-2026; 5to sitio del programa de minerales críticos en bases del Ejército, junto con Tooele, Pine Bluff/Anniston; construcción prevista desde 2027)</t>
+          <t>Permisos/estructuración de financiamiento EPC (plataforma consolidada de 3,924 hectáreas en 25 concesiones; finalización de permisos esperada 1T2026; 4 empresas EPC chinas evaluando financiamiento de deuda y desarrollo)</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>[Texarkana Gazette](https://www.texarkanagazette.com/news/2026/jun/30/army-awards-lithium-company-energyx-conditional/)</t>
+          <t>[Sonoro Gold Corp.](https://sonorogold.com/wp-content/uploads/2026/03/2026.03.01_Sonoro-Gold-Corporate-Presentation.pdf); [Mexico Mining Center](https://www.mexicominingcenter.com/sonoro-continues-discussions-with-china-based-epc-companies-and-potential-equity-investors/)</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Camino Rojo — Proyecto Subterráneo (extensión)</t>
+          <t>Pilot Mountain Tungsten Project</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Zacatecas, México</t>
+          <t>Mineral County, Nevada, EE.UU.</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Orla Mining Ltd.</t>
+          <t>Guardian Metal Resources PLC (vía Golden Metal Resources USA LLC)</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
@@ -6276,71 +6290,71 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Permisos completos/inicio de desarrollo subterráneo (SEMARNAT aprobó MIA 18-mar-2026, habilitando minado del resto del tajo de óxidos y construcción de rampa de exploración subterránea; inicio de obras de acceso subterráneo previsto 2S2026; PEA de proyecto subterráneo indica VPN de US$1,300 millones)</t>
+          <t>Ingeniería/Feasibility (PFS positivo completado jun-2026, respaldado por USD 6.2 millones del Departamento de Guerra/DPA Title III; presentación del Mine Plan of Operations federal prevista ago-2026; producción 4T2028)</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>[Mining.com](https://www.mining.com/orla-secures-final-permit-to-advance-underground-mining-at-camino-rojo/); [Orla Mining](https://orlamining.com/news/orla-mining-receives-permits-to-extend-operations-in-mexico-supporting-companys-long-term-commitment-to-camino-rojo/)</t>
+          <t>[Mining Weekly](https://www.miningweekly.com/article/guardian-metals-outlines-viable-tungsten-trioxide-operation-in-nevada-2026-06-30); [StockTitan](https://www.stocktitan.net/news/GMTL/guardian-metal-resources-plc-announces-pilot-mountain-pre-tftnlr9fu3if.html)</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-06</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Cerro Caliche Gold Project</t>
+          <t>Gabbs Project</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Sonora, México</t>
+          <t>Walker-Lane Trend, Nevada, EE.UU.</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Sonoro Gold Corp.</t>
+          <t>P2 Gold Inc.</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>EPC por definir (en negociación con múltiples empresas EPC de China)</t>
+          <t>No especificado</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Permisos/estructuración de financiamiento EPC (plataforma consolidada de 3,924 hectáreas en 25 concesiones; finalización de permisos esperada 1T2026; 4 empresas EPC chinas evaluando financiamiento de deuda y desarrollo)</t>
+          <t>Ingeniería/Feasibility (proyecto oro-cobre; feasibility study en curso, meta 4T2026)</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>[Sonoro Gold Corp.](https://sonorogold.com/wp-content/uploads/2026/03/2026.03.01_Sonoro-Gold-Corporate-Presentation.pdf); [Mexico Mining Center](https://www.mexicominingcenter.com/sonoro-continues-discussions-with-china-based-epc-companies-and-potential-equity-investors/)</t>
+          <t>[Newswire](https://www.newswire.ca/news-releases/p2-gold-gabbs-project-update-feasibility-study-on-track-840759204.html)</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-06</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Pilot Mountain Tungsten Project</t>
+          <t>Treasure Canyon Gold Mine</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Mineral County, Nevada, EE.UU.</t>
+          <t>Plumas National Forest, cerca de Taylorsville, California, EE.UU.</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Guardian Metal Resources PLC (vía Golden Metal Resources USA LLC)</t>
+          <t>Buscar Company (CGLD)</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
@@ -6350,12 +6364,12 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/Feasibility (PFS positivo completado jun-2026, respaldado por USD 6.2 millones del Departamento de Guerra/DPA Title III; presentación del Mine Plan of Operations federal prevista ago-2026; producción 4T2028)</t>
+          <t>Permitting (Plan de Operaciones sometido a US Forest Service feb-2026; en revisión por agencias federales/estatales)</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>[Mining Weekly](https://www.miningweekly.com/article/guardian-metals-outlines-viable-tungsten-trioxide-operation-in-nevada-2026-06-30); [StockTitan](https://www.stocktitan.net/news/GMTL/guardian-metal-resources-plc-announces-pilot-mountain-pre-tftnlr9fu3if.html)</t>
+          <t>[PR Newswire](https://www.prnewswire.com/news-releases/buscar-company-announces-major-advancement-in-the-permitting-process-for-the-treasure-canyon-gold-mine-project-in-california-302772744.html)</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -6367,17 +6381,17 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Gabbs Project</t>
+          <t>Grassy Mountain Gold Project</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Walker-Lane Trend, Nevada, EE.UU.</t>
+          <t>Malheur County, Oregon, EE.UU.</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>P2 Gold Inc.</t>
+          <t>Paramount Gold Nevada Corp. (vía Calico Resources)</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
@@ -6387,12 +6401,12 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Ingeniería/Feasibility (proyecto oro-cobre; feasibility study en curso, meta 4T2026)</t>
+          <t>Permitting (Record of Decision federal firmado 29-ene-2026 bajo NEPA; permisos estatales pendientes, esperados 2S2026; Feasibility Study ya completo con VPN de USD 375 millones)</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>[Newswire](https://www.newswire.ca/news-releases/p2-gold-gabbs-project-update-feasibility-study-on-track-840759204.html)</t>
+          <t>[GlobeNewswire](https://www.globenewswire.com/news-release/2026/01/29/3229150/0/en/Paramount-Gold-Receives-Federal-Approval-for-the-Grassy-Mountain-Gold-Project.html); [OPB](https://www.opb.org/article/2026/01/29/oregon-gold-mine-grassy-mountain/)</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -6404,17 +6418,17 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Treasure Canyon Gold Mine</t>
+          <t>MP Materials 10X Magnet Manufacturing Facility</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Plumas National Forest, cerca de Taylorsville, California, EE.UU.</t>
+          <t>Northlake, Texas, EE.UU.</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Buscar Company (CGLD)</t>
+          <t>MP Materials</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -6424,12 +6438,12 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Permitting (Plan de Operaciones sometido a US Forest Service feb-2026; en revisión por agencias federales/estatales)</t>
+          <t>Construcción (rompimiento de tierra 1T2026; planta de imanes de tierras raras de USD 1,250 millones; ~7,000 t/año de capacidad adicional)</t>
         </is>
       </c>
       <c r="F59" s="2